<commit_message>
Atualização automática: rac (14/09/2026 13:56)
</commit_message>
<xml_diff>
--- a/Coordenadoria/02_Dados_Tratados/base_rac_tratada.xlsx
+++ b/Coordenadoria/02_Dados_Tratados/base_rac_tratada.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1083" uniqueCount="395">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1087" uniqueCount="397">
   <si>
     <t>matricula</t>
   </si>
@@ -713,6 +713,9 @@
     <t>3122678-04</t>
   </si>
   <si>
+    <t>060-0017-00</t>
+  </si>
+  <si>
     <t>D210507</t>
   </si>
   <si>
@@ -1197,6 +1200,9 @@
   </si>
   <si>
     <t>FUEL CONTROL UNIT</t>
+  </si>
+  <si>
+    <t>FLIGHT DIR HOR</t>
   </si>
   <si>
     <t>GOVERNOR,OVERSPEED</t>
@@ -1568,10 +1574,10 @@
         <v>53</v>
       </c>
       <c r="E2">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="F2">
-        <v>5</v>
+        <v>6</v>
       </c>
     </row>
     <row r="3" spans="1:6">
@@ -2161,7 +2167,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E239"/>
+  <dimension ref="A1:E240"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:5">
@@ -2192,7 +2198,7 @@
         <v>58</v>
       </c>
       <c r="D2" t="s">
-        <v>233</v>
+        <v>234</v>
       </c>
       <c r="E2">
         <v>1</v>
@@ -2209,7 +2215,7 @@
         <v>59</v>
       </c>
       <c r="D3" t="s">
-        <v>234</v>
+        <v>235</v>
       </c>
       <c r="E3">
         <v>1</v>
@@ -2226,7 +2232,7 @@
         <v>60</v>
       </c>
       <c r="D4" t="s">
-        <v>235</v>
+        <v>236</v>
       </c>
       <c r="E4">
         <v>1</v>
@@ -2243,7 +2249,7 @@
         <v>61</v>
       </c>
       <c r="D5" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
       <c r="E5">
         <v>1</v>
@@ -2260,7 +2266,7 @@
         <v>62</v>
       </c>
       <c r="D6" t="s">
-        <v>237</v>
+        <v>238</v>
       </c>
       <c r="E6">
         <v>1</v>
@@ -2277,7 +2283,7 @@
         <v>63</v>
       </c>
       <c r="D7" t="s">
-        <v>238</v>
+        <v>239</v>
       </c>
       <c r="E7">
         <v>1</v>
@@ -2294,7 +2300,7 @@
         <v>63</v>
       </c>
       <c r="D8" t="s">
-        <v>238</v>
+        <v>239</v>
       </c>
       <c r="E8">
         <v>1</v>
@@ -2311,7 +2317,7 @@
         <v>63</v>
       </c>
       <c r="D9" t="s">
-        <v>238</v>
+        <v>239</v>
       </c>
       <c r="E9">
         <v>1</v>
@@ -2328,7 +2334,7 @@
         <v>63</v>
       </c>
       <c r="D10" t="s">
-        <v>238</v>
+        <v>239</v>
       </c>
       <c r="E10">
         <v>1</v>
@@ -2345,7 +2351,7 @@
         <v>63</v>
       </c>
       <c r="D11" t="s">
-        <v>238</v>
+        <v>239</v>
       </c>
       <c r="E11">
         <v>1</v>
@@ -2362,7 +2368,7 @@
         <v>63</v>
       </c>
       <c r="D12" t="s">
-        <v>238</v>
+        <v>239</v>
       </c>
       <c r="E12">
         <v>1</v>
@@ -2379,7 +2385,7 @@
         <v>63</v>
       </c>
       <c r="D13" t="s">
-        <v>238</v>
+        <v>239</v>
       </c>
       <c r="E13">
         <v>1</v>
@@ -2396,7 +2402,7 @@
         <v>63</v>
       </c>
       <c r="D14" t="s">
-        <v>238</v>
+        <v>239</v>
       </c>
       <c r="E14">
         <v>1</v>
@@ -2413,7 +2419,7 @@
         <v>63</v>
       </c>
       <c r="D15" t="s">
-        <v>238</v>
+        <v>239</v>
       </c>
       <c r="E15">
         <v>1</v>
@@ -2430,7 +2436,7 @@
         <v>64</v>
       </c>
       <c r="D16" t="s">
-        <v>239</v>
+        <v>240</v>
       </c>
       <c r="E16">
         <v>1</v>
@@ -2447,7 +2453,7 @@
         <v>64</v>
       </c>
       <c r="D17" t="s">
-        <v>239</v>
+        <v>240</v>
       </c>
       <c r="E17">
         <v>2</v>
@@ -2464,7 +2470,7 @@
         <v>65</v>
       </c>
       <c r="D18" t="s">
-        <v>240</v>
+        <v>241</v>
       </c>
       <c r="E18">
         <v>1</v>
@@ -2481,7 +2487,7 @@
         <v>65</v>
       </c>
       <c r="D19" t="s">
-        <v>240</v>
+        <v>241</v>
       </c>
       <c r="E19">
         <v>1</v>
@@ -2498,7 +2504,7 @@
         <v>65</v>
       </c>
       <c r="D20" t="s">
-        <v>240</v>
+        <v>241</v>
       </c>
       <c r="E20">
         <v>1</v>
@@ -2515,7 +2521,7 @@
         <v>65</v>
       </c>
       <c r="D21" t="s">
-        <v>240</v>
+        <v>241</v>
       </c>
       <c r="E21">
         <v>1</v>
@@ -2532,7 +2538,7 @@
         <v>65</v>
       </c>
       <c r="D22" t="s">
-        <v>240</v>
+        <v>241</v>
       </c>
       <c r="E22">
         <v>1</v>
@@ -2549,7 +2555,7 @@
         <v>65</v>
       </c>
       <c r="D23" t="s">
-        <v>240</v>
+        <v>241</v>
       </c>
       <c r="E23">
         <v>1</v>
@@ -2566,7 +2572,7 @@
         <v>66</v>
       </c>
       <c r="D24" t="s">
-        <v>241</v>
+        <v>242</v>
       </c>
       <c r="E24">
         <v>1</v>
@@ -2583,7 +2589,7 @@
         <v>67</v>
       </c>
       <c r="D25" t="s">
-        <v>242</v>
+        <v>243</v>
       </c>
       <c r="E25">
         <v>1</v>
@@ -2600,7 +2606,7 @@
         <v>67</v>
       </c>
       <c r="D26" t="s">
-        <v>242</v>
+        <v>243</v>
       </c>
       <c r="E26">
         <v>1</v>
@@ -2617,7 +2623,7 @@
         <v>67</v>
       </c>
       <c r="D27" t="s">
-        <v>242</v>
+        <v>243</v>
       </c>
       <c r="E27">
         <v>1</v>
@@ -2634,7 +2640,7 @@
         <v>68</v>
       </c>
       <c r="D28" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
       <c r="E28">
         <v>1</v>
@@ -2651,7 +2657,7 @@
         <v>68</v>
       </c>
       <c r="D29" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
       <c r="E29">
         <v>1</v>
@@ -2668,7 +2674,7 @@
         <v>68</v>
       </c>
       <c r="D30" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
       <c r="E30">
         <v>1</v>
@@ -2685,7 +2691,7 @@
         <v>69</v>
       </c>
       <c r="D31" t="s">
-        <v>244</v>
+        <v>245</v>
       </c>
       <c r="E31">
         <v>1</v>
@@ -2702,7 +2708,7 @@
         <v>70</v>
       </c>
       <c r="D32" t="s">
-        <v>245</v>
+        <v>246</v>
       </c>
       <c r="E32">
         <v>1</v>
@@ -2719,7 +2725,7 @@
         <v>70</v>
       </c>
       <c r="D33" t="s">
-        <v>245</v>
+        <v>246</v>
       </c>
       <c r="E33">
         <v>1</v>
@@ -2736,7 +2742,7 @@
         <v>71</v>
       </c>
       <c r="D34" t="s">
-        <v>246</v>
+        <v>247</v>
       </c>
       <c r="E34">
         <v>2</v>
@@ -2753,7 +2759,7 @@
         <v>71</v>
       </c>
       <c r="D35" t="s">
-        <v>246</v>
+        <v>247</v>
       </c>
       <c r="E35">
         <v>2</v>
@@ -2770,7 +2776,7 @@
         <v>71</v>
       </c>
       <c r="D36" t="s">
-        <v>246</v>
+        <v>247</v>
       </c>
       <c r="E36">
         <v>2</v>
@@ -2787,7 +2793,7 @@
         <v>72</v>
       </c>
       <c r="D37" t="s">
-        <v>247</v>
+        <v>248</v>
       </c>
       <c r="E37">
         <v>1</v>
@@ -2804,7 +2810,7 @@
         <v>72</v>
       </c>
       <c r="D38" t="s">
-        <v>247</v>
+        <v>248</v>
       </c>
       <c r="E38">
         <v>1</v>
@@ -2821,7 +2827,7 @@
         <v>72</v>
       </c>
       <c r="D39" t="s">
-        <v>247</v>
+        <v>248</v>
       </c>
       <c r="E39">
         <v>1</v>
@@ -2838,7 +2844,7 @@
         <v>73</v>
       </c>
       <c r="D40" t="s">
-        <v>248</v>
+        <v>249</v>
       </c>
       <c r="E40">
         <v>1</v>
@@ -2855,7 +2861,7 @@
         <v>73</v>
       </c>
       <c r="D41" t="s">
-        <v>248</v>
+        <v>249</v>
       </c>
       <c r="E41">
         <v>1</v>
@@ -2872,7 +2878,7 @@
         <v>73</v>
       </c>
       <c r="D42" t="s">
-        <v>248</v>
+        <v>249</v>
       </c>
       <c r="E42">
         <v>1</v>
@@ -2889,7 +2895,7 @@
         <v>74</v>
       </c>
       <c r="D43" t="s">
-        <v>249</v>
+        <v>250</v>
       </c>
       <c r="E43">
         <v>1</v>
@@ -2906,7 +2912,7 @@
         <v>74</v>
       </c>
       <c r="D44" t="s">
-        <v>249</v>
+        <v>250</v>
       </c>
       <c r="E44">
         <v>1</v>
@@ -2923,7 +2929,7 @@
         <v>75</v>
       </c>
       <c r="D45" t="s">
-        <v>250</v>
+        <v>251</v>
       </c>
       <c r="E45">
         <v>1</v>
@@ -2940,7 +2946,7 @@
         <v>75</v>
       </c>
       <c r="D46" t="s">
-        <v>250</v>
+        <v>251</v>
       </c>
       <c r="E46">
         <v>1</v>
@@ -2957,7 +2963,7 @@
         <v>75</v>
       </c>
       <c r="D47" t="s">
-        <v>250</v>
+        <v>251</v>
       </c>
       <c r="E47">
         <v>1</v>
@@ -2974,7 +2980,7 @@
         <v>76</v>
       </c>
       <c r="D48" t="s">
-        <v>251</v>
+        <v>252</v>
       </c>
       <c r="E48">
         <v>1</v>
@@ -2991,7 +2997,7 @@
         <v>77</v>
       </c>
       <c r="D49" t="s">
-        <v>252</v>
+        <v>253</v>
       </c>
       <c r="E49">
         <v>1</v>
@@ -3008,7 +3014,7 @@
         <v>78</v>
       </c>
       <c r="D50" t="s">
-        <v>253</v>
+        <v>254</v>
       </c>
       <c r="E50">
         <v>1</v>
@@ -3025,7 +3031,7 @@
         <v>79</v>
       </c>
       <c r="D51" t="s">
-        <v>254</v>
+        <v>255</v>
       </c>
       <c r="E51">
         <v>1</v>
@@ -3042,7 +3048,7 @@
         <v>80</v>
       </c>
       <c r="D52" t="s">
-        <v>255</v>
+        <v>256</v>
       </c>
       <c r="E52">
         <v>1</v>
@@ -3059,7 +3065,7 @@
         <v>81</v>
       </c>
       <c r="D53" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
       <c r="E53">
         <v>1</v>
@@ -3076,7 +3082,7 @@
         <v>82</v>
       </c>
       <c r="D54" t="s">
-        <v>257</v>
+        <v>258</v>
       </c>
       <c r="E54">
         <v>1</v>
@@ -3093,7 +3099,7 @@
         <v>83</v>
       </c>
       <c r="D55" t="s">
-        <v>258</v>
+        <v>259</v>
       </c>
       <c r="E55">
         <v>1</v>
@@ -3110,7 +3116,7 @@
         <v>84</v>
       </c>
       <c r="D56" t="s">
-        <v>259</v>
+        <v>260</v>
       </c>
       <c r="E56">
         <v>2</v>
@@ -3127,7 +3133,7 @@
         <v>84</v>
       </c>
       <c r="D57" t="s">
-        <v>259</v>
+        <v>260</v>
       </c>
       <c r="E57">
         <v>3</v>
@@ -3144,7 +3150,7 @@
         <v>84</v>
       </c>
       <c r="D58" t="s">
-        <v>259</v>
+        <v>260</v>
       </c>
       <c r="E58">
         <v>2</v>
@@ -3161,7 +3167,7 @@
         <v>84</v>
       </c>
       <c r="D59" t="s">
-        <v>259</v>
+        <v>260</v>
       </c>
       <c r="E59">
         <v>2</v>
@@ -3178,7 +3184,7 @@
         <v>85</v>
       </c>
       <c r="D60" t="s">
-        <v>260</v>
+        <v>261</v>
       </c>
       <c r="E60">
         <v>2</v>
@@ -3195,7 +3201,7 @@
         <v>85</v>
       </c>
       <c r="D61" t="s">
-        <v>260</v>
+        <v>261</v>
       </c>
       <c r="E61">
         <v>2</v>
@@ -3212,7 +3218,7 @@
         <v>85</v>
       </c>
       <c r="D62" t="s">
-        <v>260</v>
+        <v>261</v>
       </c>
       <c r="E62">
         <v>1</v>
@@ -3229,7 +3235,7 @@
         <v>86</v>
       </c>
       <c r="D63" t="s">
-        <v>261</v>
+        <v>262</v>
       </c>
       <c r="E63">
         <v>2</v>
@@ -3246,7 +3252,7 @@
         <v>86</v>
       </c>
       <c r="D64" t="s">
-        <v>261</v>
+        <v>262</v>
       </c>
       <c r="E64">
         <v>4</v>
@@ -3263,7 +3269,7 @@
         <v>86</v>
       </c>
       <c r="D65" t="s">
-        <v>261</v>
+        <v>262</v>
       </c>
       <c r="E65">
         <v>2</v>
@@ -3280,7 +3286,7 @@
         <v>87</v>
       </c>
       <c r="D66" t="s">
-        <v>262</v>
+        <v>263</v>
       </c>
       <c r="E66">
         <v>2</v>
@@ -3297,7 +3303,7 @@
         <v>87</v>
       </c>
       <c r="D67" t="s">
-        <v>262</v>
+        <v>263</v>
       </c>
       <c r="E67">
         <v>1</v>
@@ -3314,7 +3320,7 @@
         <v>88</v>
       </c>
       <c r="D68" t="s">
-        <v>263</v>
+        <v>264</v>
       </c>
       <c r="E68">
         <v>2</v>
@@ -3331,7 +3337,7 @@
         <v>89</v>
       </c>
       <c r="D69" t="s">
-        <v>264</v>
+        <v>265</v>
       </c>
       <c r="E69">
         <v>2</v>
@@ -3348,7 +3354,7 @@
         <v>90</v>
       </c>
       <c r="D70" t="s">
-        <v>265</v>
+        <v>266</v>
       </c>
       <c r="E70">
         <v>2</v>
@@ -3365,7 +3371,7 @@
         <v>91</v>
       </c>
       <c r="D71" t="s">
-        <v>266</v>
+        <v>267</v>
       </c>
       <c r="E71">
         <v>2</v>
@@ -3382,7 +3388,7 @@
         <v>92</v>
       </c>
       <c r="D72" t="s">
-        <v>267</v>
+        <v>268</v>
       </c>
       <c r="E72">
         <v>2</v>
@@ -3399,7 +3405,7 @@
         <v>93</v>
       </c>
       <c r="D73" t="s">
-        <v>268</v>
+        <v>269</v>
       </c>
       <c r="E73">
         <v>2</v>
@@ -3416,7 +3422,7 @@
         <v>94</v>
       </c>
       <c r="D74" t="s">
-        <v>269</v>
+        <v>270</v>
       </c>
       <c r="E74">
         <v>2</v>
@@ -3433,7 +3439,7 @@
         <v>95</v>
       </c>
       <c r="D75" t="s">
-        <v>259</v>
+        <v>260</v>
       </c>
       <c r="E75">
         <v>2</v>
@@ -3450,7 +3456,7 @@
         <v>96</v>
       </c>
       <c r="D76" t="s">
-        <v>258</v>
+        <v>259</v>
       </c>
       <c r="E76">
         <v>4</v>
@@ -3467,7 +3473,7 @@
         <v>96</v>
       </c>
       <c r="D77" t="s">
-        <v>258</v>
+        <v>259</v>
       </c>
       <c r="E77">
         <v>4</v>
@@ -3484,7 +3490,7 @@
         <v>97</v>
       </c>
       <c r="D78" t="s">
-        <v>270</v>
+        <v>271</v>
       </c>
       <c r="E78">
         <v>4</v>
@@ -3501,7 +3507,7 @@
         <v>98</v>
       </c>
       <c r="D79" t="s">
-        <v>271</v>
+        <v>272</v>
       </c>
       <c r="E79">
         <v>4</v>
@@ -3518,7 +3524,7 @@
         <v>99</v>
       </c>
       <c r="D80" t="s">
-        <v>272</v>
+        <v>273</v>
       </c>
       <c r="E80">
         <v>1</v>
@@ -3535,7 +3541,7 @@
         <v>99</v>
       </c>
       <c r="D81" t="s">
-        <v>272</v>
+        <v>273</v>
       </c>
       <c r="E81">
         <v>1</v>
@@ -3552,7 +3558,7 @@
         <v>99</v>
       </c>
       <c r="D82" t="s">
-        <v>272</v>
+        <v>273</v>
       </c>
       <c r="E82">
         <v>1</v>
@@ -3569,7 +3575,7 @@
         <v>100</v>
       </c>
       <c r="D83" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
       <c r="E83">
         <v>1</v>
@@ -3586,7 +3592,7 @@
         <v>100</v>
       </c>
       <c r="D84" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
       <c r="E84">
         <v>1</v>
@@ -3603,7 +3609,7 @@
         <v>100</v>
       </c>
       <c r="D85" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
       <c r="E85">
         <v>2</v>
@@ -3620,7 +3626,7 @@
         <v>101</v>
       </c>
       <c r="D86" t="s">
-        <v>274</v>
+        <v>275</v>
       </c>
       <c r="E86">
         <v>1</v>
@@ -3637,7 +3643,7 @@
         <v>101</v>
       </c>
       <c r="D87" t="s">
-        <v>274</v>
+        <v>275</v>
       </c>
       <c r="E87">
         <v>1</v>
@@ -3654,7 +3660,7 @@
         <v>102</v>
       </c>
       <c r="D88" t="s">
-        <v>275</v>
+        <v>276</v>
       </c>
       <c r="E88">
         <v>1</v>
@@ -3671,7 +3677,7 @@
         <v>102</v>
       </c>
       <c r="D89" t="s">
-        <v>275</v>
+        <v>276</v>
       </c>
       <c r="E89">
         <v>1</v>
@@ -3688,7 +3694,7 @@
         <v>103</v>
       </c>
       <c r="D90" t="s">
-        <v>276</v>
+        <v>277</v>
       </c>
       <c r="E90">
         <v>1</v>
@@ -3705,7 +3711,7 @@
         <v>103</v>
       </c>
       <c r="D91" t="s">
-        <v>276</v>
+        <v>277</v>
       </c>
       <c r="E91">
         <v>1</v>
@@ -3722,7 +3728,7 @@
         <v>104</v>
       </c>
       <c r="D92" t="s">
-        <v>277</v>
+        <v>278</v>
       </c>
       <c r="E92">
         <v>1</v>
@@ -3739,7 +3745,7 @@
         <v>104</v>
       </c>
       <c r="D93" t="s">
-        <v>277</v>
+        <v>278</v>
       </c>
       <c r="E93">
         <v>1</v>
@@ -3756,7 +3762,7 @@
         <v>105</v>
       </c>
       <c r="D94" t="s">
-        <v>278</v>
+        <v>279</v>
       </c>
       <c r="E94">
         <v>1</v>
@@ -3773,7 +3779,7 @@
         <v>105</v>
       </c>
       <c r="D95" t="s">
-        <v>278</v>
+        <v>279</v>
       </c>
       <c r="E95">
         <v>1</v>
@@ -3790,7 +3796,7 @@
         <v>106</v>
       </c>
       <c r="D96" t="s">
-        <v>279</v>
+        <v>280</v>
       </c>
       <c r="E96">
         <v>1</v>
@@ -3807,7 +3813,7 @@
         <v>106</v>
       </c>
       <c r="D97" t="s">
-        <v>279</v>
+        <v>280</v>
       </c>
       <c r="E97">
         <v>1</v>
@@ -3824,7 +3830,7 @@
         <v>107</v>
       </c>
       <c r="D98" t="s">
-        <v>280</v>
+        <v>281</v>
       </c>
       <c r="E98">
         <v>1</v>
@@ -3841,7 +3847,7 @@
         <v>107</v>
       </c>
       <c r="D99" t="s">
-        <v>280</v>
+        <v>281</v>
       </c>
       <c r="E99">
         <v>1</v>
@@ -3858,7 +3864,7 @@
         <v>108</v>
       </c>
       <c r="D100" t="s">
-        <v>281</v>
+        <v>282</v>
       </c>
       <c r="E100">
         <v>1</v>
@@ -3875,7 +3881,7 @@
         <v>108</v>
       </c>
       <c r="D101" t="s">
-        <v>281</v>
+        <v>282</v>
       </c>
       <c r="E101">
         <v>1</v>
@@ -3892,7 +3898,7 @@
         <v>109</v>
       </c>
       <c r="D102" t="s">
-        <v>282</v>
+        <v>283</v>
       </c>
       <c r="E102">
         <v>1</v>
@@ -3909,7 +3915,7 @@
         <v>110</v>
       </c>
       <c r="D103" t="s">
-        <v>283</v>
+        <v>284</v>
       </c>
       <c r="E103">
         <v>1</v>
@@ -3926,7 +3932,7 @@
         <v>111</v>
       </c>
       <c r="D104" t="s">
-        <v>284</v>
+        <v>285</v>
       </c>
       <c r="E104">
         <v>1</v>
@@ -3943,7 +3949,7 @@
         <v>112</v>
       </c>
       <c r="D105" t="s">
-        <v>285</v>
+        <v>286</v>
       </c>
       <c r="E105">
         <v>1</v>
@@ -3960,7 +3966,7 @@
         <v>113</v>
       </c>
       <c r="D106" t="s">
-        <v>286</v>
+        <v>287</v>
       </c>
       <c r="E106">
         <v>1</v>
@@ -3977,7 +3983,7 @@
         <v>114</v>
       </c>
       <c r="D107" t="s">
-        <v>287</v>
+        <v>288</v>
       </c>
       <c r="E107">
         <v>1</v>
@@ -3994,7 +4000,7 @@
         <v>115</v>
       </c>
       <c r="D108" t="s">
-        <v>288</v>
+        <v>289</v>
       </c>
       <c r="E108">
         <v>2</v>
@@ -4011,7 +4017,7 @@
         <v>115</v>
       </c>
       <c r="D109" t="s">
-        <v>288</v>
+        <v>289</v>
       </c>
       <c r="E109">
         <v>1</v>
@@ -4028,7 +4034,7 @@
         <v>116</v>
       </c>
       <c r="D110" t="s">
-        <v>289</v>
+        <v>290</v>
       </c>
       <c r="E110">
         <v>2</v>
@@ -4045,7 +4051,7 @@
         <v>116</v>
       </c>
       <c r="D111" t="s">
-        <v>289</v>
+        <v>290</v>
       </c>
       <c r="E111">
         <v>2</v>
@@ -4062,7 +4068,7 @@
         <v>116</v>
       </c>
       <c r="D112" t="s">
-        <v>289</v>
+        <v>290</v>
       </c>
       <c r="E112">
         <v>2</v>
@@ -4079,7 +4085,7 @@
         <v>117</v>
       </c>
       <c r="D113" t="s">
-        <v>290</v>
+        <v>291</v>
       </c>
       <c r="E113">
         <v>2</v>
@@ -4096,7 +4102,7 @@
         <v>117</v>
       </c>
       <c r="D114" t="s">
-        <v>290</v>
+        <v>291</v>
       </c>
       <c r="E114">
         <v>2</v>
@@ -4113,7 +4119,7 @@
         <v>117</v>
       </c>
       <c r="D115" t="s">
-        <v>290</v>
+        <v>291</v>
       </c>
       <c r="E115">
         <v>2</v>
@@ -4130,7 +4136,7 @@
         <v>118</v>
       </c>
       <c r="D116" t="s">
-        <v>291</v>
+        <v>292</v>
       </c>
       <c r="E116">
         <v>2</v>
@@ -4147,7 +4153,7 @@
         <v>118</v>
       </c>
       <c r="D117" t="s">
-        <v>291</v>
+        <v>292</v>
       </c>
       <c r="E117">
         <v>2</v>
@@ -4164,7 +4170,7 @@
         <v>119</v>
       </c>
       <c r="D118" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
       <c r="E118">
         <v>2</v>
@@ -4181,7 +4187,7 @@
         <v>119</v>
       </c>
       <c r="D119" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
       <c r="E119">
         <v>4</v>
@@ -4198,7 +4204,7 @@
         <v>119</v>
       </c>
       <c r="D120" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
       <c r="E120">
         <v>4</v>
@@ -4215,7 +4221,7 @@
         <v>120</v>
       </c>
       <c r="D121" t="s">
-        <v>292</v>
+        <v>293</v>
       </c>
       <c r="E121">
         <v>2</v>
@@ -4232,7 +4238,7 @@
         <v>120</v>
       </c>
       <c r="D122" t="s">
-        <v>292</v>
+        <v>293</v>
       </c>
       <c r="E122">
         <v>4</v>
@@ -4249,7 +4255,7 @@
         <v>121</v>
       </c>
       <c r="D123" t="s">
-        <v>277</v>
+        <v>278</v>
       </c>
       <c r="E123">
         <v>2</v>
@@ -4266,7 +4272,7 @@
         <v>122</v>
       </c>
       <c r="D124" t="s">
-        <v>293</v>
+        <v>294</v>
       </c>
       <c r="E124">
         <v>2</v>
@@ -4283,7 +4289,7 @@
         <v>123</v>
       </c>
       <c r="D125" t="s">
-        <v>294</v>
+        <v>295</v>
       </c>
       <c r="E125">
         <v>2</v>
@@ -4300,7 +4306,7 @@
         <v>124</v>
       </c>
       <c r="D126" t="s">
-        <v>295</v>
+        <v>296</v>
       </c>
       <c r="E126">
         <v>5</v>
@@ -4317,7 +4323,7 @@
         <v>124</v>
       </c>
       <c r="D127" t="s">
-        <v>295</v>
+        <v>296</v>
       </c>
       <c r="E127">
         <v>5</v>
@@ -4334,7 +4340,7 @@
         <v>125</v>
       </c>
       <c r="D128" t="s">
-        <v>296</v>
+        <v>297</v>
       </c>
       <c r="E128">
         <v>7</v>
@@ -4351,7 +4357,7 @@
         <v>126</v>
       </c>
       <c r="D129" t="s">
-        <v>297</v>
+        <v>298</v>
       </c>
       <c r="E129">
         <v>8</v>
@@ -4368,7 +4374,7 @@
         <v>127</v>
       </c>
       <c r="D130" t="s">
-        <v>298</v>
+        <v>299</v>
       </c>
       <c r="E130">
         <v>10</v>
@@ -4385,7 +4391,7 @@
         <v>128</v>
       </c>
       <c r="D131" t="s">
-        <v>299</v>
+        <v>300</v>
       </c>
       <c r="E131">
         <v>30</v>
@@ -4402,7 +4408,7 @@
         <v>128</v>
       </c>
       <c r="D132" t="s">
-        <v>299</v>
+        <v>300</v>
       </c>
       <c r="E132">
         <v>30</v>
@@ -4419,7 +4425,7 @@
         <v>129</v>
       </c>
       <c r="D133" t="s">
-        <v>300</v>
+        <v>301</v>
       </c>
       <c r="E133">
         <v>1</v>
@@ -4436,7 +4442,7 @@
         <v>129</v>
       </c>
       <c r="D134" t="s">
-        <v>300</v>
+        <v>301</v>
       </c>
       <c r="E134">
         <v>1</v>
@@ -4453,7 +4459,7 @@
         <v>130</v>
       </c>
       <c r="D135" t="s">
-        <v>301</v>
+        <v>302</v>
       </c>
       <c r="E135">
         <v>1</v>
@@ -4470,7 +4476,7 @@
         <v>131</v>
       </c>
       <c r="D136" t="s">
-        <v>302</v>
+        <v>303</v>
       </c>
       <c r="E136">
         <v>1</v>
@@ -4487,7 +4493,7 @@
         <v>132</v>
       </c>
       <c r="D137" t="s">
-        <v>303</v>
+        <v>304</v>
       </c>
       <c r="E137">
         <v>1</v>
@@ -4504,7 +4510,7 @@
         <v>133</v>
       </c>
       <c r="D138" t="s">
-        <v>304</v>
+        <v>305</v>
       </c>
       <c r="E138">
         <v>1</v>
@@ -4521,7 +4527,7 @@
         <v>134</v>
       </c>
       <c r="D139" t="s">
-        <v>305</v>
+        <v>306</v>
       </c>
       <c r="E139">
         <v>1</v>
@@ -4538,7 +4544,7 @@
         <v>135</v>
       </c>
       <c r="D140" t="s">
-        <v>306</v>
+        <v>307</v>
       </c>
       <c r="E140">
         <v>1</v>
@@ -4555,7 +4561,7 @@
         <v>136</v>
       </c>
       <c r="D141" t="s">
-        <v>307</v>
+        <v>308</v>
       </c>
       <c r="E141">
         <v>1</v>
@@ -4572,7 +4578,7 @@
         <v>137</v>
       </c>
       <c r="D142" t="s">
-        <v>308</v>
+        <v>309</v>
       </c>
       <c r="E142">
         <v>1</v>
@@ -4589,7 +4595,7 @@
         <v>138</v>
       </c>
       <c r="D143" t="s">
-        <v>309</v>
+        <v>310</v>
       </c>
       <c r="E143">
         <v>1</v>
@@ -4606,7 +4612,7 @@
         <v>138</v>
       </c>
       <c r="D144" t="s">
-        <v>309</v>
+        <v>310</v>
       </c>
       <c r="E144">
         <v>1</v>
@@ -4623,7 +4629,7 @@
         <v>139</v>
       </c>
       <c r="D145" t="s">
-        <v>310</v>
+        <v>311</v>
       </c>
       <c r="E145">
         <v>1</v>
@@ -4640,7 +4646,7 @@
         <v>139</v>
       </c>
       <c r="D146" t="s">
-        <v>310</v>
+        <v>311</v>
       </c>
       <c r="E146">
         <v>1</v>
@@ -4657,7 +4663,7 @@
         <v>140</v>
       </c>
       <c r="D147" t="s">
-        <v>311</v>
+        <v>312</v>
       </c>
       <c r="E147">
         <v>1</v>
@@ -4674,7 +4680,7 @@
         <v>141</v>
       </c>
       <c r="D148" t="s">
-        <v>312</v>
+        <v>313</v>
       </c>
       <c r="E148">
         <v>1</v>
@@ -4691,7 +4697,7 @@
         <v>142</v>
       </c>
       <c r="D149" t="s">
-        <v>313</v>
+        <v>314</v>
       </c>
       <c r="E149">
         <v>1</v>
@@ -4708,7 +4714,7 @@
         <v>143</v>
       </c>
       <c r="D150" t="s">
-        <v>314</v>
+        <v>315</v>
       </c>
       <c r="E150">
         <v>1</v>
@@ -4725,7 +4731,7 @@
         <v>144</v>
       </c>
       <c r="D151" t="s">
-        <v>315</v>
+        <v>316</v>
       </c>
       <c r="E151">
         <v>1</v>
@@ -4742,7 +4748,7 @@
         <v>145</v>
       </c>
       <c r="D152" t="s">
-        <v>316</v>
+        <v>317</v>
       </c>
       <c r="E152">
         <v>1</v>
@@ -4759,7 +4765,7 @@
         <v>146</v>
       </c>
       <c r="D153" t="s">
-        <v>317</v>
+        <v>318</v>
       </c>
       <c r="E153">
         <v>1</v>
@@ -4776,7 +4782,7 @@
         <v>147</v>
       </c>
       <c r="D154" t="s">
-        <v>318</v>
+        <v>319</v>
       </c>
       <c r="E154">
         <v>1</v>
@@ -4793,7 +4799,7 @@
         <v>148</v>
       </c>
       <c r="D155" t="s">
-        <v>319</v>
+        <v>320</v>
       </c>
       <c r="E155">
         <v>1</v>
@@ -4810,7 +4816,7 @@
         <v>149</v>
       </c>
       <c r="D156" t="s">
-        <v>320</v>
+        <v>321</v>
       </c>
       <c r="E156">
         <v>1</v>
@@ -4827,7 +4833,7 @@
         <v>150</v>
       </c>
       <c r="D157" t="s">
-        <v>321</v>
+        <v>322</v>
       </c>
       <c r="E157">
         <v>1</v>
@@ -4844,7 +4850,7 @@
         <v>151</v>
       </c>
       <c r="D158" t="s">
-        <v>322</v>
+        <v>323</v>
       </c>
       <c r="E158">
         <v>1</v>
@@ -4861,7 +4867,7 @@
         <v>152</v>
       </c>
       <c r="D159" t="s">
-        <v>323</v>
+        <v>324</v>
       </c>
       <c r="E159">
         <v>1</v>
@@ -4878,7 +4884,7 @@
         <v>153</v>
       </c>
       <c r="D160" t="s">
-        <v>324</v>
+        <v>325</v>
       </c>
       <c r="E160">
         <v>1</v>
@@ -4895,7 +4901,7 @@
         <v>154</v>
       </c>
       <c r="D161" t="s">
-        <v>325</v>
+        <v>326</v>
       </c>
       <c r="E161">
         <v>1</v>
@@ -4912,7 +4918,7 @@
         <v>155</v>
       </c>
       <c r="D162" t="s">
-        <v>326</v>
+        <v>327</v>
       </c>
       <c r="E162">
         <v>1</v>
@@ -4929,7 +4935,7 @@
         <v>156</v>
       </c>
       <c r="D163" t="s">
-        <v>327</v>
+        <v>328</v>
       </c>
       <c r="E163">
         <v>1</v>
@@ -4946,7 +4952,7 @@
         <v>157</v>
       </c>
       <c r="D164" t="s">
-        <v>328</v>
+        <v>329</v>
       </c>
       <c r="E164">
         <v>1</v>
@@ -4963,7 +4969,7 @@
         <v>158</v>
       </c>
       <c r="D165" t="s">
-        <v>329</v>
+        <v>330</v>
       </c>
       <c r="E165">
         <v>1</v>
@@ -4980,7 +4986,7 @@
         <v>159</v>
       </c>
       <c r="D166" t="s">
-        <v>314</v>
+        <v>315</v>
       </c>
       <c r="E166">
         <v>2</v>
@@ -4997,7 +5003,7 @@
         <v>160</v>
       </c>
       <c r="D167" t="s">
-        <v>330</v>
+        <v>331</v>
       </c>
       <c r="E167">
         <v>2</v>
@@ -5014,7 +5020,7 @@
         <v>161</v>
       </c>
       <c r="D168" t="s">
-        <v>331</v>
+        <v>332</v>
       </c>
       <c r="E168">
         <v>2</v>
@@ -5031,7 +5037,7 @@
         <v>162</v>
       </c>
       <c r="D169" t="s">
-        <v>332</v>
+        <v>333</v>
       </c>
       <c r="E169">
         <v>2</v>
@@ -5048,7 +5054,7 @@
         <v>163</v>
       </c>
       <c r="D170" t="s">
-        <v>333</v>
+        <v>334</v>
       </c>
       <c r="E170">
         <v>2</v>
@@ -5065,7 +5071,7 @@
         <v>164</v>
       </c>
       <c r="D171" t="s">
-        <v>334</v>
+        <v>335</v>
       </c>
       <c r="E171">
         <v>3</v>
@@ -5082,7 +5088,7 @@
         <v>165</v>
       </c>
       <c r="D172" t="s">
-        <v>299</v>
+        <v>300</v>
       </c>
       <c r="E172">
         <v>5</v>
@@ -5099,7 +5105,7 @@
         <v>166</v>
       </c>
       <c r="D173" t="s">
-        <v>335</v>
+        <v>336</v>
       </c>
       <c r="E173">
         <v>8</v>
@@ -5116,7 +5122,7 @@
         <v>167</v>
       </c>
       <c r="D174" t="s">
-        <v>255</v>
+        <v>256</v>
       </c>
       <c r="E174">
         <v>8</v>
@@ -5133,7 +5139,7 @@
         <v>168</v>
       </c>
       <c r="D175" t="s">
-        <v>336</v>
+        <v>337</v>
       </c>
       <c r="E175">
         <v>10</v>
@@ -5150,7 +5156,7 @@
         <v>169</v>
       </c>
       <c r="D176" t="s">
-        <v>324</v>
+        <v>325</v>
       </c>
       <c r="E176">
         <v>1</v>
@@ -5167,7 +5173,7 @@
         <v>170</v>
       </c>
       <c r="D177" t="s">
-        <v>337</v>
+        <v>338</v>
       </c>
       <c r="E177">
         <v>1</v>
@@ -5184,7 +5190,7 @@
         <v>171</v>
       </c>
       <c r="D178" t="s">
-        <v>338</v>
+        <v>339</v>
       </c>
       <c r="E178">
         <v>1</v>
@@ -5201,7 +5207,7 @@
         <v>172</v>
       </c>
       <c r="D179" t="s">
-        <v>339</v>
+        <v>340</v>
       </c>
       <c r="E179">
         <v>1</v>
@@ -5218,7 +5224,7 @@
         <v>173</v>
       </c>
       <c r="D180" t="s">
-        <v>340</v>
+        <v>341</v>
       </c>
       <c r="E180">
         <v>1</v>
@@ -5235,7 +5241,7 @@
         <v>174</v>
       </c>
       <c r="D181" t="s">
-        <v>341</v>
+        <v>342</v>
       </c>
       <c r="E181">
         <v>1</v>
@@ -5252,7 +5258,7 @@
         <v>175</v>
       </c>
       <c r="D182" t="s">
-        <v>265</v>
+        <v>266</v>
       </c>
       <c r="E182">
         <v>1</v>
@@ -5269,7 +5275,7 @@
         <v>176</v>
       </c>
       <c r="D183" t="s">
-        <v>342</v>
+        <v>343</v>
       </c>
       <c r="E183">
         <v>1</v>
@@ -5286,7 +5292,7 @@
         <v>177</v>
       </c>
       <c r="D184" t="s">
-        <v>343</v>
+        <v>344</v>
       </c>
       <c r="E184">
         <v>1</v>
@@ -5303,7 +5309,7 @@
         <v>178</v>
       </c>
       <c r="D185" t="s">
-        <v>344</v>
+        <v>345</v>
       </c>
       <c r="E185">
         <v>1</v>
@@ -5320,7 +5326,7 @@
         <v>179</v>
       </c>
       <c r="D186" t="s">
-        <v>345</v>
+        <v>346</v>
       </c>
       <c r="E186">
         <v>1</v>
@@ -5337,7 +5343,7 @@
         <v>180</v>
       </c>
       <c r="D187" t="s">
-        <v>346</v>
+        <v>347</v>
       </c>
       <c r="E187">
         <v>1</v>
@@ -5354,7 +5360,7 @@
         <v>181</v>
       </c>
       <c r="D188" t="s">
-        <v>347</v>
+        <v>348</v>
       </c>
       <c r="E188">
         <v>1</v>
@@ -5371,7 +5377,7 @@
         <v>182</v>
       </c>
       <c r="D189" t="s">
-        <v>348</v>
+        <v>349</v>
       </c>
       <c r="E189">
         <v>1</v>
@@ -5388,7 +5394,7 @@
         <v>183</v>
       </c>
       <c r="D190" t="s">
-        <v>349</v>
+        <v>350</v>
       </c>
       <c r="E190">
         <v>1</v>
@@ -5405,7 +5411,7 @@
         <v>184</v>
       </c>
       <c r="D191" t="s">
-        <v>350</v>
+        <v>351</v>
       </c>
       <c r="E191">
         <v>1</v>
@@ -5422,7 +5428,7 @@
         <v>185</v>
       </c>
       <c r="D192" t="s">
-        <v>351</v>
+        <v>352</v>
       </c>
       <c r="E192">
         <v>1</v>
@@ -5439,7 +5445,7 @@
         <v>186</v>
       </c>
       <c r="D193" t="s">
-        <v>352</v>
+        <v>353</v>
       </c>
       <c r="E193">
         <v>1</v>
@@ -5456,7 +5462,7 @@
         <v>187</v>
       </c>
       <c r="D194" t="s">
-        <v>353</v>
+        <v>354</v>
       </c>
       <c r="E194">
         <v>1</v>
@@ -5473,7 +5479,7 @@
         <v>188</v>
       </c>
       <c r="D195" t="s">
-        <v>354</v>
+        <v>355</v>
       </c>
       <c r="E195">
         <v>1</v>
@@ -5490,7 +5496,7 @@
         <v>189</v>
       </c>
       <c r="D196" t="s">
-        <v>355</v>
+        <v>356</v>
       </c>
       <c r="E196">
         <v>1</v>
@@ -5507,7 +5513,7 @@
         <v>190</v>
       </c>
       <c r="D197" t="s">
-        <v>356</v>
+        <v>357</v>
       </c>
       <c r="E197">
         <v>1</v>
@@ -5524,7 +5530,7 @@
         <v>191</v>
       </c>
       <c r="D198" t="s">
-        <v>357</v>
+        <v>358</v>
       </c>
       <c r="E198">
         <v>1</v>
@@ -5541,7 +5547,7 @@
         <v>192</v>
       </c>
       <c r="D199" t="s">
-        <v>358</v>
+        <v>359</v>
       </c>
       <c r="E199">
         <v>1</v>
@@ -5558,7 +5564,7 @@
         <v>193</v>
       </c>
       <c r="D200" t="s">
-        <v>359</v>
+        <v>360</v>
       </c>
       <c r="E200">
         <v>1</v>
@@ -5575,7 +5581,7 @@
         <v>194</v>
       </c>
       <c r="D201" t="s">
-        <v>360</v>
+        <v>361</v>
       </c>
       <c r="E201">
         <v>1</v>
@@ -5592,7 +5598,7 @@
         <v>195</v>
       </c>
       <c r="D202" t="s">
-        <v>361</v>
+        <v>362</v>
       </c>
       <c r="E202">
         <v>1</v>
@@ -5609,7 +5615,7 @@
         <v>196</v>
       </c>
       <c r="D203" t="s">
-        <v>362</v>
+        <v>363</v>
       </c>
       <c r="E203">
         <v>1</v>
@@ -5626,7 +5632,7 @@
         <v>197</v>
       </c>
       <c r="D204" t="s">
-        <v>363</v>
+        <v>364</v>
       </c>
       <c r="E204">
         <v>1</v>
@@ -5643,7 +5649,7 @@
         <v>198</v>
       </c>
       <c r="D205" t="s">
-        <v>364</v>
+        <v>365</v>
       </c>
       <c r="E205">
         <v>1</v>
@@ -5660,7 +5666,7 @@
         <v>199</v>
       </c>
       <c r="D206" t="s">
-        <v>365</v>
+        <v>366</v>
       </c>
       <c r="E206">
         <v>1</v>
@@ -5677,7 +5683,7 @@
         <v>200</v>
       </c>
       <c r="D207" t="s">
-        <v>366</v>
+        <v>367</v>
       </c>
       <c r="E207">
         <v>1</v>
@@ -5694,7 +5700,7 @@
         <v>201</v>
       </c>
       <c r="D208" t="s">
-        <v>367</v>
+        <v>368</v>
       </c>
       <c r="E208">
         <v>2</v>
@@ -5711,7 +5717,7 @@
         <v>202</v>
       </c>
       <c r="D209" t="s">
-        <v>368</v>
+        <v>369</v>
       </c>
       <c r="E209">
         <v>2</v>
@@ -5728,7 +5734,7 @@
         <v>203</v>
       </c>
       <c r="D210" t="s">
-        <v>369</v>
+        <v>370</v>
       </c>
       <c r="E210">
         <v>2</v>
@@ -5745,7 +5751,7 @@
         <v>204</v>
       </c>
       <c r="D211" t="s">
-        <v>370</v>
+        <v>371</v>
       </c>
       <c r="E211">
         <v>2</v>
@@ -5762,7 +5768,7 @@
         <v>205</v>
       </c>
       <c r="D212" t="s">
-        <v>371</v>
+        <v>372</v>
       </c>
       <c r="E212">
         <v>2</v>
@@ -5779,7 +5785,7 @@
         <v>206</v>
       </c>
       <c r="D213" t="s">
-        <v>372</v>
+        <v>373</v>
       </c>
       <c r="E213">
         <v>2</v>
@@ -5796,7 +5802,7 @@
         <v>207</v>
       </c>
       <c r="D214" t="s">
-        <v>373</v>
+        <v>374</v>
       </c>
       <c r="E214">
         <v>2</v>
@@ -5813,7 +5819,7 @@
         <v>208</v>
       </c>
       <c r="D215" t="s">
-        <v>374</v>
+        <v>375</v>
       </c>
       <c r="E215">
         <v>2</v>
@@ -5830,7 +5836,7 @@
         <v>209</v>
       </c>
       <c r="D216" t="s">
-        <v>374</v>
+        <v>375</v>
       </c>
       <c r="E216">
         <v>2</v>
@@ -5847,7 +5853,7 @@
         <v>210</v>
       </c>
       <c r="D217" t="s">
-        <v>375</v>
+        <v>376</v>
       </c>
       <c r="E217">
         <v>2</v>
@@ -5864,7 +5870,7 @@
         <v>211</v>
       </c>
       <c r="D218" t="s">
-        <v>376</v>
+        <v>377</v>
       </c>
       <c r="E218">
         <v>2</v>
@@ -5881,7 +5887,7 @@
         <v>212</v>
       </c>
       <c r="D219" t="s">
-        <v>377</v>
+        <v>378</v>
       </c>
       <c r="E219">
         <v>2</v>
@@ -5898,7 +5904,7 @@
         <v>213</v>
       </c>
       <c r="D220" t="s">
-        <v>378</v>
+        <v>379</v>
       </c>
       <c r="E220">
         <v>3</v>
@@ -5915,7 +5921,7 @@
         <v>214</v>
       </c>
       <c r="D221" t="s">
-        <v>265</v>
+        <v>266</v>
       </c>
       <c r="E221">
         <v>3</v>
@@ -5932,7 +5938,7 @@
         <v>215</v>
       </c>
       <c r="D222" t="s">
-        <v>379</v>
+        <v>380</v>
       </c>
       <c r="E222">
         <v>4</v>
@@ -5949,7 +5955,7 @@
         <v>216</v>
       </c>
       <c r="D223" t="s">
-        <v>380</v>
+        <v>381</v>
       </c>
       <c r="E223">
         <v>4</v>
@@ -5966,7 +5972,7 @@
         <v>217</v>
       </c>
       <c r="D224" t="s">
-        <v>381</v>
+        <v>382</v>
       </c>
       <c r="E224">
         <v>4</v>
@@ -5983,7 +5989,7 @@
         <v>218</v>
       </c>
       <c r="D225" t="s">
-        <v>382</v>
+        <v>383</v>
       </c>
       <c r="E225">
         <v>4</v>
@@ -6000,7 +6006,7 @@
         <v>219</v>
       </c>
       <c r="D226" t="s">
-        <v>383</v>
+        <v>384</v>
       </c>
       <c r="E226">
         <v>4</v>
@@ -6017,7 +6023,7 @@
         <v>220</v>
       </c>
       <c r="D227" t="s">
-        <v>384</v>
+        <v>385</v>
       </c>
       <c r="E227">
         <v>5</v>
@@ -6034,7 +6040,7 @@
         <v>221</v>
       </c>
       <c r="D228" t="s">
-        <v>385</v>
+        <v>386</v>
       </c>
       <c r="E228">
         <v>5</v>
@@ -6051,7 +6057,7 @@
         <v>222</v>
       </c>
       <c r="D229" t="s">
-        <v>386</v>
+        <v>387</v>
       </c>
       <c r="E229">
         <v>6</v>
@@ -6068,7 +6074,7 @@
         <v>223</v>
       </c>
       <c r="D230" t="s">
-        <v>387</v>
+        <v>388</v>
       </c>
       <c r="E230">
         <v>8</v>
@@ -6085,7 +6091,7 @@
         <v>224</v>
       </c>
       <c r="D231" t="s">
-        <v>388</v>
+        <v>389</v>
       </c>
       <c r="E231">
         <v>10</v>
@@ -6102,7 +6108,7 @@
         <v>225</v>
       </c>
       <c r="D232" t="s">
-        <v>388</v>
+        <v>389</v>
       </c>
       <c r="E232">
         <v>10</v>
@@ -6119,7 +6125,7 @@
         <v>226</v>
       </c>
       <c r="D233" t="s">
-        <v>267</v>
+        <v>268</v>
       </c>
       <c r="E233">
         <v>12</v>
@@ -6136,7 +6142,7 @@
         <v>227</v>
       </c>
       <c r="D234" t="s">
-        <v>389</v>
+        <v>390</v>
       </c>
       <c r="E234">
         <v>12</v>
@@ -6153,7 +6159,7 @@
         <v>228</v>
       </c>
       <c r="D235" t="s">
-        <v>390</v>
+        <v>391</v>
       </c>
       <c r="E235">
         <v>14</v>
@@ -6170,7 +6176,7 @@
         <v>229</v>
       </c>
       <c r="D236" t="s">
-        <v>391</v>
+        <v>392</v>
       </c>
       <c r="E236">
         <v>15</v>
@@ -6187,7 +6193,7 @@
         <v>230</v>
       </c>
       <c r="D237" t="s">
-        <v>392</v>
+        <v>393</v>
       </c>
       <c r="E237">
         <v>20</v>
@@ -6204,7 +6210,7 @@
         <v>231</v>
       </c>
       <c r="D238" t="s">
-        <v>393</v>
+        <v>394</v>
       </c>
       <c r="E238">
         <v>1</v>
@@ -6212,18 +6218,35 @@
     </row>
     <row r="239" spans="1:5">
       <c r="A239" t="s">
-        <v>13</v>
+        <v>6</v>
       </c>
       <c r="B239" t="s">
-        <v>40</v>
+        <v>36</v>
       </c>
       <c r="C239" t="s">
         <v>232</v>
       </c>
       <c r="D239" t="s">
-        <v>394</v>
+        <v>395</v>
       </c>
       <c r="E239">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="240" spans="1:5">
+      <c r="A240" t="s">
+        <v>13</v>
+      </c>
+      <c r="B240" t="s">
+        <v>40</v>
+      </c>
+      <c r="C240" t="s">
+        <v>233</v>
+      </c>
+      <c r="D240" t="s">
+        <v>396</v>
+      </c>
+      <c r="E240">
         <v>1</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualização automática: rac (15/09/2026 08:54)
</commit_message>
<xml_diff>
--- a/Coordenadoria/02_Dados_Tratados/base_rac_tratada.xlsx
+++ b/Coordenadoria/02_Dados_Tratados/base_rac_tratada.xlsx
@@ -1212,8 +1212,16 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <fonts count="1">
+  <fonts count="2">
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -1229,7 +1237,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -1237,12 +1245,30 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1541,22 +1567,22 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:6">
-      <c r="A1" t="s">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" t="s">
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" t="s">
+      <c r="F1" s="1" t="s">
         <v>5</v>
       </c>
     </row>
@@ -2171,19 +2197,19 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:5">
-      <c r="A1" t="s">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" t="s">
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
         <v>55</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>56</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="1" t="s">
         <v>57</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualização automática: rac (15/09/2026 12:32)
</commit_message>
<xml_diff>
--- a/Coordenadoria/02_Dados_Tratados/base_rac_tratada.xlsx
+++ b/Coordenadoria/02_Dados_Tratados/base_rac_tratada.xlsx
@@ -1212,16 +1212,8 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <fonts count="2">
+  <fonts count="1">
     <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -1237,7 +1229,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -1245,30 +1237,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color auto="1"/>
-      </left>
-      <right style="thin">
-        <color auto="1"/>
-      </right>
-      <top style="thin">
-        <color auto="1"/>
-      </top>
-      <bottom style="thin">
-        <color auto="1"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1567,22 +1541,22 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:6">
-      <c r="A1" s="1" t="s">
+      <c r="A1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" s="1" t="s">
+      <c r="B1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" t="s">
         <v>5</v>
       </c>
     </row>
@@ -2197,19 +2171,19 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:5">
-      <c r="A1" s="1" t="s">
+      <c r="A1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" s="1" t="s">
+      <c r="B1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" t="s">
         <v>55</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" t="s">
         <v>56</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" t="s">
         <v>57</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualização automática: rac (15/09/2026 13:43)
</commit_message>
<xml_diff>
--- a/Coordenadoria/02_Dados_Tratados/base_rac_tratada.xlsx
+++ b/Coordenadoria/02_Dados_Tratados/base_rac_tratada.xlsx
@@ -1212,8 +1212,16 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <fonts count="1">
+  <fonts count="2">
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -1229,7 +1237,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -1237,12 +1245,30 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1541,22 +1567,22 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:6">
-      <c r="A1" t="s">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" t="s">
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" t="s">
+      <c r="F1" s="1" t="s">
         <v>5</v>
       </c>
     </row>
@@ -2171,19 +2197,19 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:5">
-      <c r="A1" t="s">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" t="s">
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
         <v>55</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>56</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="1" t="s">
         <v>57</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualização automática: rac (16/09/2026 12:24)
</commit_message>
<xml_diff>
--- a/Coordenadoria/02_Dados_Tratados/base_rac_tratada.xlsx
+++ b/Coordenadoria/02_Dados_Tratados/base_rac_tratada.xlsx
@@ -215,9 +215,6 @@
     <t>3044000</t>
   </si>
   <si>
-    <t>C662504-0101</t>
-  </si>
-  <si>
     <t>2600100-7</t>
   </si>
   <si>
@@ -716,7 +713,10 @@
     <t>060-0017-00</t>
   </si>
   <si>
-    <t>D210507</t>
+    <t>S3309A0160-000D</t>
+  </si>
+  <si>
+    <t>3034792</t>
   </si>
   <si>
     <t>HOUSING</t>
@@ -743,9 +743,6 @@
     <t>ENGINE PT6A-114A</t>
   </si>
   <si>
-    <t>GAGE VOLT AMME</t>
-  </si>
-  <si>
     <t>LINE ASSY-PROP</t>
   </si>
   <si>
@@ -1205,23 +1202,18 @@
     <t>FLIGHT DIR HOR</t>
   </si>
   <si>
-    <t>GOVERNOR,OVERSPEED</t>
+    <t>HOSE AY</t>
+  </si>
+  <si>
+    <t>FUEL PUMP</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <fonts count="2">
+  <fonts count="1">
     <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -1237,7 +1229,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -1245,30 +1237,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color auto="1"/>
-      </left>
-      <right style="thin">
-        <color auto="1"/>
-      </right>
-      <top style="thin">
-        <color auto="1"/>
-      </top>
-      <bottom style="thin">
-        <color auto="1"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1567,22 +1541,22 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:6">
-      <c r="A1" s="1" t="s">
+      <c r="A1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" s="1" t="s">
+      <c r="B1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" t="s">
         <v>5</v>
       </c>
     </row>
@@ -1614,16 +1588,16 @@
         <v>37</v>
       </c>
       <c r="C3" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="D3" t="s">
         <v>53</v>
       </c>
       <c r="E3">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F3">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="4" spans="1:6">
@@ -1660,10 +1634,10 @@
         <v>53</v>
       </c>
       <c r="E5">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F5">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="6" spans="1:6">
@@ -1680,10 +1654,10 @@
         <v>53</v>
       </c>
       <c r="E6">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F6">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="7" spans="1:6">
@@ -1700,10 +1674,10 @@
         <v>54</v>
       </c>
       <c r="E7">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="F7">
-        <v>7</v>
+        <v>9</v>
       </c>
     </row>
     <row r="8" spans="1:6">
@@ -1740,10 +1714,10 @@
         <v>54</v>
       </c>
       <c r="E9">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="F9">
-        <v>107</v>
+        <v>106</v>
       </c>
     </row>
     <row r="10" spans="1:6">
@@ -1800,10 +1774,10 @@
         <v>53</v>
       </c>
       <c r="E12">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="F12">
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
     <row r="13" spans="1:6">
@@ -2197,19 +2171,19 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:5">
-      <c r="A1" s="1" t="s">
+      <c r="A1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" s="1" t="s">
+      <c r="B1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" t="s">
         <v>55</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" t="s">
         <v>56</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" t="s">
         <v>57</v>
       </c>
     </row>
@@ -2300,10 +2274,10 @@
     </row>
     <row r="7" spans="1:5">
       <c r="A7" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="B7" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="C7" t="s">
         <v>63</v>
@@ -2317,10 +2291,10 @@
     </row>
     <row r="8" spans="1:5">
       <c r="A8" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="B8" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="C8" t="s">
         <v>63</v>
@@ -2334,7 +2308,7 @@
     </row>
     <row r="9" spans="1:5">
       <c r="A9" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="B9" t="s">
         <v>39</v>
@@ -2351,10 +2325,10 @@
     </row>
     <row r="10" spans="1:5">
       <c r="A10" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="B10" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="C10" t="s">
         <v>63</v>
@@ -2368,10 +2342,10 @@
     </row>
     <row r="11" spans="1:5">
       <c r="A11" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B11" t="s">
-        <v>40</v>
+        <v>36</v>
       </c>
       <c r="C11" t="s">
         <v>63</v>
@@ -2385,10 +2359,10 @@
     </row>
     <row r="12" spans="1:5">
       <c r="A12" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="B12" t="s">
-        <v>36</v>
+        <v>40</v>
       </c>
       <c r="C12" t="s">
         <v>63</v>
@@ -2402,7 +2376,7 @@
     </row>
     <row r="13" spans="1:5">
       <c r="A13" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="B13" t="s">
         <v>40</v>
@@ -2419,10 +2393,10 @@
     </row>
     <row r="14" spans="1:5">
       <c r="A14" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="B14" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="C14" t="s">
         <v>63</v>
@@ -2436,16 +2410,16 @@
     </row>
     <row r="15" spans="1:5">
       <c r="A15" t="s">
-        <v>15</v>
+        <v>12</v>
       </c>
       <c r="B15" t="s">
-        <v>41</v>
+        <v>36</v>
       </c>
       <c r="C15" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="D15" t="s">
-        <v>239</v>
+        <v>240</v>
       </c>
       <c r="E15">
         <v>1</v>
@@ -2453,10 +2427,10 @@
     </row>
     <row r="16" spans="1:5">
       <c r="A16" t="s">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="B16" t="s">
-        <v>36</v>
+        <v>41</v>
       </c>
       <c r="C16" t="s">
         <v>64</v>
@@ -2465,32 +2439,32 @@
         <v>240</v>
       </c>
       <c r="E16">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="17" spans="1:5">
       <c r="A17" t="s">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="B17" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="C17" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="D17" t="s">
-        <v>240</v>
+        <v>241</v>
       </c>
       <c r="E17">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="18" spans="1:5">
       <c r="A18" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="B18" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="C18" t="s">
         <v>65</v>
@@ -2504,10 +2478,10 @@
     </row>
     <row r="19" spans="1:5">
       <c r="A19" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B19" t="s">
-        <v>40</v>
+        <v>36</v>
       </c>
       <c r="C19" t="s">
         <v>65</v>
@@ -2521,10 +2495,10 @@
     </row>
     <row r="20" spans="1:5">
       <c r="A20" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="B20" t="s">
-        <v>36</v>
+        <v>40</v>
       </c>
       <c r="C20" t="s">
         <v>65</v>
@@ -2538,7 +2512,7 @@
     </row>
     <row r="21" spans="1:5">
       <c r="A21" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="B21" t="s">
         <v>40</v>
@@ -2555,10 +2529,10 @@
     </row>
     <row r="22" spans="1:5">
       <c r="A22" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="B22" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="C22" t="s">
         <v>65</v>
@@ -2572,16 +2546,16 @@
     </row>
     <row r="23" spans="1:5">
       <c r="A23" t="s">
-        <v>15</v>
+        <v>11</v>
       </c>
       <c r="B23" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C23" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="D23" t="s">
-        <v>241</v>
+        <v>242</v>
       </c>
       <c r="E23">
         <v>1</v>
@@ -2589,10 +2563,10 @@
     </row>
     <row r="24" spans="1:5">
       <c r="A24" t="s">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="B24" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="C24" t="s">
         <v>66</v>
@@ -2606,16 +2580,16 @@
     </row>
     <row r="25" spans="1:5">
       <c r="A25" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="B25" t="s">
         <v>40</v>
       </c>
       <c r="C25" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="D25" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
       <c r="E25">
         <v>1</v>
@@ -2623,7 +2597,7 @@
     </row>
     <row r="26" spans="1:5">
       <c r="A26" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="B26" t="s">
         <v>40</v>
@@ -2640,7 +2614,7 @@
     </row>
     <row r="27" spans="1:5">
       <c r="A27" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B27" t="s">
         <v>40</v>
@@ -2657,16 +2631,16 @@
     </row>
     <row r="28" spans="1:5">
       <c r="A28" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="B28" t="s">
         <v>40</v>
       </c>
       <c r="C28" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="D28" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="E28">
         <v>1</v>
@@ -2674,7 +2648,7 @@
     </row>
     <row r="29" spans="1:5">
       <c r="A29" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="B29" t="s">
         <v>40</v>
@@ -2691,16 +2665,16 @@
     </row>
     <row r="30" spans="1:5">
       <c r="A30" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="B30" t="s">
         <v>40</v>
       </c>
       <c r="C30" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="D30" t="s">
-        <v>244</v>
+        <v>245</v>
       </c>
       <c r="E30">
         <v>1</v>
@@ -2737,12 +2711,12 @@
         <v>246</v>
       </c>
       <c r="E32">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="33" spans="1:5">
       <c r="A33" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B33" t="s">
         <v>40</v>
@@ -2754,21 +2728,21 @@
         <v>246</v>
       </c>
       <c r="E33">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="34" spans="1:5">
       <c r="A34" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="B34" t="s">
         <v>40</v>
       </c>
       <c r="C34" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="D34" t="s">
-        <v>247</v>
+        <v>246</v>
       </c>
       <c r="E34">
         <v>2</v>
@@ -2776,10 +2750,10 @@
     </row>
     <row r="35" spans="1:5">
       <c r="A35" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B35" t="s">
-        <v>40</v>
+        <v>36</v>
       </c>
       <c r="C35" t="s">
         <v>71</v>
@@ -2788,12 +2762,12 @@
         <v>247</v>
       </c>
       <c r="E35">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="36" spans="1:5">
       <c r="A36" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B36" t="s">
         <v>40</v>
@@ -2805,21 +2779,21 @@
         <v>247</v>
       </c>
       <c r="E36">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="37" spans="1:5">
       <c r="A37" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="B37" t="s">
-        <v>36</v>
+        <v>40</v>
       </c>
       <c r="C37" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="D37" t="s">
-        <v>248</v>
+        <v>247</v>
       </c>
       <c r="E37">
         <v>1</v>
@@ -2827,10 +2801,10 @@
     </row>
     <row r="38" spans="1:5">
       <c r="A38" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B38" t="s">
-        <v>40</v>
+        <v>36</v>
       </c>
       <c r="C38" t="s">
         <v>72</v>
@@ -2844,7 +2818,7 @@
     </row>
     <row r="39" spans="1:5">
       <c r="A39" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B39" t="s">
         <v>40</v>
@@ -2861,16 +2835,16 @@
     </row>
     <row r="40" spans="1:5">
       <c r="A40" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="B40" t="s">
-        <v>36</v>
+        <v>40</v>
       </c>
       <c r="C40" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="D40" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
       <c r="E40">
         <v>1</v>
@@ -2878,10 +2852,10 @@
     </row>
     <row r="41" spans="1:5">
       <c r="A41" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B41" t="s">
-        <v>40</v>
+        <v>36</v>
       </c>
       <c r="C41" t="s">
         <v>73</v>
@@ -2895,7 +2869,7 @@
     </row>
     <row r="42" spans="1:5">
       <c r="A42" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B42" t="s">
         <v>40</v>
@@ -2929,7 +2903,7 @@
     </row>
     <row r="44" spans="1:5">
       <c r="A44" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="B44" t="s">
         <v>40</v>
@@ -2946,16 +2920,16 @@
     </row>
     <row r="45" spans="1:5">
       <c r="A45" t="s">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="B45" t="s">
-        <v>36</v>
+        <v>41</v>
       </c>
       <c r="C45" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="D45" t="s">
-        <v>251</v>
+        <v>250</v>
       </c>
       <c r="E45">
         <v>1</v>
@@ -2963,10 +2937,10 @@
     </row>
     <row r="46" spans="1:5">
       <c r="A46" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="B46" t="s">
-        <v>40</v>
+        <v>36</v>
       </c>
       <c r="C46" t="s">
         <v>75</v>
@@ -2980,16 +2954,16 @@
     </row>
     <row r="47" spans="1:5">
       <c r="A47" t="s">
-        <v>15</v>
+        <v>12</v>
       </c>
       <c r="B47" t="s">
-        <v>41</v>
+        <v>36</v>
       </c>
       <c r="C47" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="D47" t="s">
-        <v>251</v>
+        <v>252</v>
       </c>
       <c r="E47">
         <v>1</v>
@@ -3003,10 +2977,10 @@
         <v>36</v>
       </c>
       <c r="C48" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="D48" t="s">
-        <v>252</v>
+        <v>253</v>
       </c>
       <c r="E48">
         <v>1</v>
@@ -3020,10 +2994,10 @@
         <v>36</v>
       </c>
       <c r="C49" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="D49" t="s">
-        <v>253</v>
+        <v>254</v>
       </c>
       <c r="E49">
         <v>1</v>
@@ -3037,10 +3011,10 @@
         <v>36</v>
       </c>
       <c r="C50" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="D50" t="s">
-        <v>254</v>
+        <v>255</v>
       </c>
       <c r="E50">
         <v>1</v>
@@ -3054,10 +3028,10 @@
         <v>36</v>
       </c>
       <c r="C51" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="D51" t="s">
-        <v>255</v>
+        <v>256</v>
       </c>
       <c r="E51">
         <v>1</v>
@@ -3071,10 +3045,10 @@
         <v>36</v>
       </c>
       <c r="C52" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="D52" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
       <c r="E52">
         <v>1</v>
@@ -3088,10 +3062,10 @@
         <v>36</v>
       </c>
       <c r="C53" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="D53" t="s">
-        <v>257</v>
+        <v>258</v>
       </c>
       <c r="E53">
         <v>1</v>
@@ -3105,21 +3079,21 @@
         <v>36</v>
       </c>
       <c r="C54" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="D54" t="s">
-        <v>258</v>
+        <v>259</v>
       </c>
       <c r="E54">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="55" spans="1:5">
       <c r="A55" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="B55" t="s">
-        <v>36</v>
+        <v>40</v>
       </c>
       <c r="C55" t="s">
         <v>83</v>
@@ -3128,21 +3102,21 @@
         <v>259</v>
       </c>
       <c r="E55">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="56" spans="1:5">
       <c r="A56" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="B56" t="s">
-        <v>36</v>
+        <v>40</v>
       </c>
       <c r="C56" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="D56" t="s">
-        <v>260</v>
+        <v>259</v>
       </c>
       <c r="E56">
         <v>2</v>
@@ -3150,27 +3124,27 @@
     </row>
     <row r="57" spans="1:5">
       <c r="A57" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="B57" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="C57" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="D57" t="s">
-        <v>260</v>
+        <v>259</v>
       </c>
       <c r="E57">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="58" spans="1:5">
       <c r="A58" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="B58" t="s">
-        <v>40</v>
+        <v>36</v>
       </c>
       <c r="C58" t="s">
         <v>84</v>
@@ -3184,10 +3158,10 @@
     </row>
     <row r="59" spans="1:5">
       <c r="A59" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B59" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C59" t="s">
         <v>84</v>
@@ -3201,27 +3175,27 @@
     </row>
     <row r="60" spans="1:5">
       <c r="A60" t="s">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="B60" t="s">
-        <v>36</v>
+        <v>41</v>
       </c>
       <c r="C60" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="D60" t="s">
-        <v>261</v>
+        <v>260</v>
       </c>
       <c r="E60">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="61" spans="1:5">
       <c r="A61" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="B61" t="s">
-        <v>40</v>
+        <v>36</v>
       </c>
       <c r="C61" t="s">
         <v>85</v>
@@ -3235,10 +3209,10 @@
     </row>
     <row r="62" spans="1:5">
       <c r="A62" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B62" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C62" t="s">
         <v>85</v>
@@ -3247,21 +3221,21 @@
         <v>261</v>
       </c>
       <c r="E62">
-        <v>1</v>
+        <v>4</v>
       </c>
     </row>
     <row r="63" spans="1:5">
       <c r="A63" t="s">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="B63" t="s">
-        <v>36</v>
+        <v>41</v>
       </c>
       <c r="C63" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="D63" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
       <c r="E63">
         <v>2</v>
@@ -3269,10 +3243,10 @@
     </row>
     <row r="64" spans="1:5">
       <c r="A64" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="B64" t="s">
-        <v>40</v>
+        <v>36</v>
       </c>
       <c r="C64" t="s">
         <v>86</v>
@@ -3281,7 +3255,7 @@
         <v>262</v>
       </c>
       <c r="E64">
-        <v>4</v>
+        <v>2</v>
       </c>
     </row>
     <row r="65" spans="1:5">
@@ -3298,7 +3272,7 @@
         <v>262</v>
       </c>
       <c r="E65">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="66" spans="1:5">
@@ -3320,19 +3294,19 @@
     </row>
     <row r="67" spans="1:5">
       <c r="A67" t="s">
-        <v>15</v>
+        <v>12</v>
       </c>
       <c r="B67" t="s">
-        <v>41</v>
+        <v>36</v>
       </c>
       <c r="C67" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="D67" t="s">
-        <v>263</v>
+        <v>264</v>
       </c>
       <c r="E67">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="68" spans="1:5">
@@ -3343,10 +3317,10 @@
         <v>36</v>
       </c>
       <c r="C68" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="D68" t="s">
-        <v>264</v>
+        <v>265</v>
       </c>
       <c r="E68">
         <v>2</v>
@@ -3360,10 +3334,10 @@
         <v>36</v>
       </c>
       <c r="C69" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="D69" t="s">
-        <v>265</v>
+        <v>266</v>
       </c>
       <c r="E69">
         <v>2</v>
@@ -3377,10 +3351,10 @@
         <v>36</v>
       </c>
       <c r="C70" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="D70" t="s">
-        <v>266</v>
+        <v>267</v>
       </c>
       <c r="E70">
         <v>2</v>
@@ -3394,10 +3368,10 @@
         <v>36</v>
       </c>
       <c r="C71" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="D71" t="s">
-        <v>267</v>
+        <v>268</v>
       </c>
       <c r="E71">
         <v>2</v>
@@ -3411,10 +3385,10 @@
         <v>36</v>
       </c>
       <c r="C72" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="D72" t="s">
-        <v>268</v>
+        <v>269</v>
       </c>
       <c r="E72">
         <v>2</v>
@@ -3428,10 +3402,10 @@
         <v>36</v>
       </c>
       <c r="C73" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="D73" t="s">
-        <v>269</v>
+        <v>259</v>
       </c>
       <c r="E73">
         <v>2</v>
@@ -3445,30 +3419,30 @@
         <v>36</v>
       </c>
       <c r="C74" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="D74" t="s">
-        <v>270</v>
+        <v>258</v>
       </c>
       <c r="E74">
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
     <row r="75" spans="1:5">
       <c r="A75" t="s">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="B75" t="s">
-        <v>36</v>
+        <v>41</v>
       </c>
       <c r="C75" t="s">
         <v>95</v>
       </c>
       <c r="D75" t="s">
-        <v>260</v>
+        <v>258</v>
       </c>
       <c r="E75">
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
     <row r="76" spans="1:5">
@@ -3482,7 +3456,7 @@
         <v>96</v>
       </c>
       <c r="D76" t="s">
-        <v>259</v>
+        <v>270</v>
       </c>
       <c r="E76">
         <v>4</v>
@@ -3490,16 +3464,16 @@
     </row>
     <row r="77" spans="1:5">
       <c r="A77" t="s">
-        <v>15</v>
+        <v>12</v>
       </c>
       <c r="B77" t="s">
-        <v>41</v>
+        <v>36</v>
       </c>
       <c r="C77" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="D77" t="s">
-        <v>259</v>
+        <v>271</v>
       </c>
       <c r="E77">
         <v>4</v>
@@ -3507,27 +3481,27 @@
     </row>
     <row r="78" spans="1:5">
       <c r="A78" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="B78" t="s">
-        <v>36</v>
+        <v>40</v>
       </c>
       <c r="C78" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="D78" t="s">
-        <v>271</v>
+        <v>272</v>
       </c>
       <c r="E78">
-        <v>4</v>
+        <v>1</v>
       </c>
     </row>
     <row r="79" spans="1:5">
       <c r="A79" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="B79" t="s">
-        <v>36</v>
+        <v>40</v>
       </c>
       <c r="C79" t="s">
         <v>98</v>
@@ -3536,21 +3510,21 @@
         <v>272</v>
       </c>
       <c r="E79">
-        <v>4</v>
+        <v>1</v>
       </c>
     </row>
     <row r="80" spans="1:5">
       <c r="A80" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="B80" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="C80" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="D80" t="s">
-        <v>273</v>
+        <v>272</v>
       </c>
       <c r="E80">
         <v>1</v>
@@ -3558,7 +3532,7 @@
     </row>
     <row r="81" spans="1:5">
       <c r="A81" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B81" t="s">
         <v>40</v>
@@ -3575,10 +3549,10 @@
     </row>
     <row r="82" spans="1:5">
       <c r="A82" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B82" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C82" t="s">
         <v>99</v>
@@ -3592,24 +3566,24 @@
     </row>
     <row r="83" spans="1:5">
       <c r="A83" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="B83" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="C83" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="D83" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
       <c r="E83">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="84" spans="1:5">
       <c r="A84" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B84" t="s">
         <v>40</v>
@@ -3626,10 +3600,10 @@
     </row>
     <row r="85" spans="1:5">
       <c r="A85" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B85" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C85" t="s">
         <v>100</v>
@@ -3638,7 +3612,7 @@
         <v>274</v>
       </c>
       <c r="E85">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="86" spans="1:5">
@@ -3796,10 +3770,10 @@
     </row>
     <row r="95" spans="1:5">
       <c r="A95" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="B95" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="C95" t="s">
         <v>105</v>
@@ -3898,16 +3872,16 @@
     </row>
     <row r="101" spans="1:5">
       <c r="A101" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="B101" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C101" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="D101" t="s">
-        <v>282</v>
+        <v>283</v>
       </c>
       <c r="E101">
         <v>1</v>
@@ -3921,10 +3895,10 @@
         <v>40</v>
       </c>
       <c r="C102" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="D102" t="s">
-        <v>283</v>
+        <v>284</v>
       </c>
       <c r="E102">
         <v>1</v>
@@ -3938,10 +3912,10 @@
         <v>40</v>
       </c>
       <c r="C103" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="D103" t="s">
-        <v>284</v>
+        <v>285</v>
       </c>
       <c r="E103">
         <v>1</v>
@@ -3955,10 +3929,10 @@
         <v>40</v>
       </c>
       <c r="C104" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="D104" t="s">
-        <v>285</v>
+        <v>286</v>
       </c>
       <c r="E104">
         <v>1</v>
@@ -3972,10 +3946,10 @@
         <v>40</v>
       </c>
       <c r="C105" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="D105" t="s">
-        <v>286</v>
+        <v>287</v>
       </c>
       <c r="E105">
         <v>1</v>
@@ -3989,18 +3963,18 @@
         <v>40</v>
       </c>
       <c r="C106" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="D106" t="s">
-        <v>287</v>
+        <v>288</v>
       </c>
       <c r="E106">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="107" spans="1:5">
       <c r="A107" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="B107" t="s">
         <v>40</v>
@@ -4046,21 +4020,21 @@
         <v>289</v>
       </c>
       <c r="E109">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="110" spans="1:5">
       <c r="A110" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="B110" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="C110" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="D110" t="s">
-        <v>290</v>
+        <v>289</v>
       </c>
       <c r="E110">
         <v>2</v>
@@ -4068,7 +4042,7 @@
     </row>
     <row r="111" spans="1:5">
       <c r="A111" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B111" t="s">
         <v>40</v>
@@ -4085,10 +4059,10 @@
     </row>
     <row r="112" spans="1:5">
       <c r="A112" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B112" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C112" t="s">
         <v>116</v>
@@ -4102,16 +4076,16 @@
     </row>
     <row r="113" spans="1:5">
       <c r="A113" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="B113" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="C113" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="D113" t="s">
-        <v>291</v>
+        <v>290</v>
       </c>
       <c r="E113">
         <v>2</v>
@@ -4119,7 +4093,7 @@
     </row>
     <row r="114" spans="1:5">
       <c r="A114" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B114" t="s">
         <v>40</v>
@@ -4136,10 +4110,10 @@
     </row>
     <row r="115" spans="1:5">
       <c r="A115" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B115" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C115" t="s">
         <v>117</v>
@@ -4162,7 +4136,7 @@
         <v>118</v>
       </c>
       <c r="D116" t="s">
-        <v>292</v>
+        <v>273</v>
       </c>
       <c r="E116">
         <v>2</v>
@@ -4179,32 +4153,32 @@
         <v>118</v>
       </c>
       <c r="D117" t="s">
-        <v>292</v>
+        <v>273</v>
       </c>
       <c r="E117">
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
     <row r="118" spans="1:5">
       <c r="A118" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="B118" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="C118" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="D118" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
       <c r="E118">
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
     <row r="119" spans="1:5">
       <c r="A119" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B119" t="s">
         <v>40</v>
@@ -4213,24 +4187,24 @@
         <v>119</v>
       </c>
       <c r="D119" t="s">
-        <v>274</v>
+        <v>292</v>
       </c>
       <c r="E119">
-        <v>4</v>
+        <v>2</v>
       </c>
     </row>
     <row r="120" spans="1:5">
       <c r="A120" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B120" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C120" t="s">
         <v>119</v>
       </c>
       <c r="D120" t="s">
-        <v>274</v>
+        <v>292</v>
       </c>
       <c r="E120">
         <v>4</v>
@@ -4247,7 +4221,7 @@
         <v>120</v>
       </c>
       <c r="D121" t="s">
-        <v>293</v>
+        <v>277</v>
       </c>
       <c r="E121">
         <v>2</v>
@@ -4255,19 +4229,19 @@
     </row>
     <row r="122" spans="1:5">
       <c r="A122" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B122" t="s">
         <v>40</v>
       </c>
       <c r="C122" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="D122" t="s">
         <v>293</v>
       </c>
       <c r="E122">
-        <v>4</v>
+        <v>2</v>
       </c>
     </row>
     <row r="123" spans="1:5">
@@ -4278,10 +4252,10 @@
         <v>40</v>
       </c>
       <c r="C123" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="D123" t="s">
-        <v>278</v>
+        <v>294</v>
       </c>
       <c r="E123">
         <v>2</v>
@@ -4295,18 +4269,18 @@
         <v>40</v>
       </c>
       <c r="C124" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="D124" t="s">
-        <v>294</v>
+        <v>295</v>
       </c>
       <c r="E124">
-        <v>2</v>
+        <v>5</v>
       </c>
     </row>
     <row r="125" spans="1:5">
       <c r="A125" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="B125" t="s">
         <v>40</v>
@@ -4318,7 +4292,7 @@
         <v>295</v>
       </c>
       <c r="E125">
-        <v>2</v>
+        <v>5</v>
       </c>
     </row>
     <row r="126" spans="1:5">
@@ -4335,24 +4309,24 @@
         <v>296</v>
       </c>
       <c r="E126">
-        <v>5</v>
+        <v>7</v>
       </c>
     </row>
     <row r="127" spans="1:5">
       <c r="A127" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B127" t="s">
         <v>40</v>
       </c>
       <c r="C127" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="D127" t="s">
-        <v>296</v>
+        <v>297</v>
       </c>
       <c r="E127">
-        <v>5</v>
+        <v>8</v>
       </c>
     </row>
     <row r="128" spans="1:5">
@@ -4363,13 +4337,13 @@
         <v>40</v>
       </c>
       <c r="C128" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="D128" t="s">
-        <v>297</v>
+        <v>298</v>
       </c>
       <c r="E128">
-        <v>7</v>
+        <v>10</v>
       </c>
     </row>
     <row r="129" spans="1:5">
@@ -4380,18 +4354,18 @@
         <v>40</v>
       </c>
       <c r="C129" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="D129" t="s">
-        <v>298</v>
+        <v>299</v>
       </c>
       <c r="E129">
-        <v>8</v>
+        <v>30</v>
       </c>
     </row>
     <row r="130" spans="1:5">
       <c r="A130" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="B130" t="s">
         <v>40</v>
@@ -4403,12 +4377,12 @@
         <v>299</v>
       </c>
       <c r="E130">
-        <v>10</v>
+        <v>30</v>
       </c>
     </row>
     <row r="131" spans="1:5">
       <c r="A131" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="B131" t="s">
         <v>40</v>
@@ -4420,15 +4394,15 @@
         <v>300</v>
       </c>
       <c r="E131">
-        <v>30</v>
+        <v>1</v>
       </c>
     </row>
     <row r="132" spans="1:5">
       <c r="A132" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="B132" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="C132" t="s">
         <v>128</v>
@@ -4437,7 +4411,7 @@
         <v>300</v>
       </c>
       <c r="E132">
-        <v>30</v>
+        <v>1</v>
       </c>
     </row>
     <row r="133" spans="1:5">
@@ -4459,16 +4433,16 @@
     </row>
     <row r="134" spans="1:5">
       <c r="A134" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B134" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C134" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="D134" t="s">
-        <v>301</v>
+        <v>302</v>
       </c>
       <c r="E134">
         <v>1</v>
@@ -4482,10 +4456,10 @@
         <v>40</v>
       </c>
       <c r="C135" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="D135" t="s">
-        <v>302</v>
+        <v>303</v>
       </c>
       <c r="E135">
         <v>1</v>
@@ -4499,10 +4473,10 @@
         <v>40</v>
       </c>
       <c r="C136" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="D136" t="s">
-        <v>303</v>
+        <v>304</v>
       </c>
       <c r="E136">
         <v>1</v>
@@ -4516,10 +4490,10 @@
         <v>40</v>
       </c>
       <c r="C137" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="D137" t="s">
-        <v>304</v>
+        <v>305</v>
       </c>
       <c r="E137">
         <v>1</v>
@@ -4533,10 +4507,10 @@
         <v>40</v>
       </c>
       <c r="C138" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="D138" t="s">
-        <v>305</v>
+        <v>306</v>
       </c>
       <c r="E138">
         <v>1</v>
@@ -4550,10 +4524,10 @@
         <v>40</v>
       </c>
       <c r="C139" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="D139" t="s">
-        <v>306</v>
+        <v>307</v>
       </c>
       <c r="E139">
         <v>1</v>
@@ -4567,10 +4541,10 @@
         <v>40</v>
       </c>
       <c r="C140" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="D140" t="s">
-        <v>307</v>
+        <v>308</v>
       </c>
       <c r="E140">
         <v>1</v>
@@ -4584,10 +4558,10 @@
         <v>40</v>
       </c>
       <c r="C141" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="D141" t="s">
-        <v>308</v>
+        <v>309</v>
       </c>
       <c r="E141">
         <v>1</v>
@@ -4595,10 +4569,10 @@
     </row>
     <row r="142" spans="1:5">
       <c r="A142" t="s">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="B142" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="C142" t="s">
         <v>137</v>
@@ -4663,16 +4637,16 @@
     </row>
     <row r="146" spans="1:5">
       <c r="A146" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="B146" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="C146" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="D146" t="s">
-        <v>311</v>
+        <v>312</v>
       </c>
       <c r="E146">
         <v>1</v>
@@ -4686,10 +4660,10 @@
         <v>40</v>
       </c>
       <c r="C147" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="D147" t="s">
-        <v>312</v>
+        <v>313</v>
       </c>
       <c r="E147">
         <v>1</v>
@@ -4703,10 +4677,10 @@
         <v>40</v>
       </c>
       <c r="C148" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="D148" t="s">
-        <v>313</v>
+        <v>314</v>
       </c>
       <c r="E148">
         <v>1</v>
@@ -4720,10 +4694,10 @@
         <v>40</v>
       </c>
       <c r="C149" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="D149" t="s">
-        <v>314</v>
+        <v>315</v>
       </c>
       <c r="E149">
         <v>1</v>
@@ -4737,10 +4711,10 @@
         <v>40</v>
       </c>
       <c r="C150" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="D150" t="s">
-        <v>315</v>
+        <v>316</v>
       </c>
       <c r="E150">
         <v>1</v>
@@ -4754,10 +4728,10 @@
         <v>40</v>
       </c>
       <c r="C151" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="D151" t="s">
-        <v>316</v>
+        <v>317</v>
       </c>
       <c r="E151">
         <v>1</v>
@@ -4771,10 +4745,10 @@
         <v>40</v>
       </c>
       <c r="C152" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="D152" t="s">
-        <v>317</v>
+        <v>318</v>
       </c>
       <c r="E152">
         <v>1</v>
@@ -4788,10 +4762,10 @@
         <v>40</v>
       </c>
       <c r="C153" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="D153" t="s">
-        <v>318</v>
+        <v>319</v>
       </c>
       <c r="E153">
         <v>1</v>
@@ -4805,10 +4779,10 @@
         <v>40</v>
       </c>
       <c r="C154" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="D154" t="s">
-        <v>319</v>
+        <v>320</v>
       </c>
       <c r="E154">
         <v>1</v>
@@ -4822,10 +4796,10 @@
         <v>40</v>
       </c>
       <c r="C155" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="D155" t="s">
-        <v>320</v>
+        <v>321</v>
       </c>
       <c r="E155">
         <v>1</v>
@@ -4839,10 +4813,10 @@
         <v>40</v>
       </c>
       <c r="C156" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="D156" t="s">
-        <v>321</v>
+        <v>322</v>
       </c>
       <c r="E156">
         <v>1</v>
@@ -4856,10 +4830,10 @@
         <v>40</v>
       </c>
       <c r="C157" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="D157" t="s">
-        <v>322</v>
+        <v>323</v>
       </c>
       <c r="E157">
         <v>1</v>
@@ -4873,10 +4847,10 @@
         <v>40</v>
       </c>
       <c r="C158" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="D158" t="s">
-        <v>323</v>
+        <v>324</v>
       </c>
       <c r="E158">
         <v>1</v>
@@ -4890,10 +4864,10 @@
         <v>40</v>
       </c>
       <c r="C159" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="D159" t="s">
-        <v>324</v>
+        <v>325</v>
       </c>
       <c r="E159">
         <v>1</v>
@@ -4907,10 +4881,10 @@
         <v>40</v>
       </c>
       <c r="C160" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="D160" t="s">
-        <v>325</v>
+        <v>326</v>
       </c>
       <c r="E160">
         <v>1</v>
@@ -4924,10 +4898,10 @@
         <v>40</v>
       </c>
       <c r="C161" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="D161" t="s">
-        <v>326</v>
+        <v>327</v>
       </c>
       <c r="E161">
         <v>1</v>
@@ -4941,10 +4915,10 @@
         <v>40</v>
       </c>
       <c r="C162" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="D162" t="s">
-        <v>327</v>
+        <v>328</v>
       </c>
       <c r="E162">
         <v>1</v>
@@ -4958,10 +4932,10 @@
         <v>40</v>
       </c>
       <c r="C163" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="D163" t="s">
-        <v>328</v>
+        <v>329</v>
       </c>
       <c r="E163">
         <v>1</v>
@@ -4975,13 +4949,13 @@
         <v>40</v>
       </c>
       <c r="C164" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="D164" t="s">
-        <v>329</v>
+        <v>314</v>
       </c>
       <c r="E164">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="165" spans="1:5">
@@ -4992,13 +4966,13 @@
         <v>40</v>
       </c>
       <c r="C165" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="D165" t="s">
         <v>330</v>
       </c>
       <c r="E165">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="166" spans="1:5">
@@ -5009,10 +4983,10 @@
         <v>40</v>
       </c>
       <c r="C166" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="D166" t="s">
-        <v>315</v>
+        <v>331</v>
       </c>
       <c r="E166">
         <v>2</v>
@@ -5026,10 +5000,10 @@
         <v>40</v>
       </c>
       <c r="C167" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="D167" t="s">
-        <v>331</v>
+        <v>332</v>
       </c>
       <c r="E167">
         <v>2</v>
@@ -5043,10 +5017,10 @@
         <v>40</v>
       </c>
       <c r="C168" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="D168" t="s">
-        <v>332</v>
+        <v>333</v>
       </c>
       <c r="E168">
         <v>2</v>
@@ -5060,13 +5034,13 @@
         <v>40</v>
       </c>
       <c r="C169" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="D169" t="s">
-        <v>333</v>
+        <v>334</v>
       </c>
       <c r="E169">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="170" spans="1:5">
@@ -5077,13 +5051,13 @@
         <v>40</v>
       </c>
       <c r="C170" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="D170" t="s">
-        <v>334</v>
+        <v>299</v>
       </c>
       <c r="E170">
-        <v>2</v>
+        <v>5</v>
       </c>
     </row>
     <row r="171" spans="1:5">
@@ -5094,13 +5068,13 @@
         <v>40</v>
       </c>
       <c r="C171" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="D171" t="s">
         <v>335</v>
       </c>
       <c r="E171">
-        <v>3</v>
+        <v>8</v>
       </c>
     </row>
     <row r="172" spans="1:5">
@@ -5111,13 +5085,13 @@
         <v>40</v>
       </c>
       <c r="C172" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="D172" t="s">
-        <v>300</v>
+        <v>255</v>
       </c>
       <c r="E172">
-        <v>5</v>
+        <v>8</v>
       </c>
     </row>
     <row r="173" spans="1:5">
@@ -5128,47 +5102,47 @@
         <v>40</v>
       </c>
       <c r="C173" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="D173" t="s">
         <v>336</v>
       </c>
       <c r="E173">
-        <v>8</v>
+        <v>10</v>
       </c>
     </row>
     <row r="174" spans="1:5">
       <c r="A174" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="B174" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="C174" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="D174" t="s">
-        <v>256</v>
+        <v>324</v>
       </c>
       <c r="E174">
-        <v>8</v>
+        <v>1</v>
       </c>
     </row>
     <row r="175" spans="1:5">
       <c r="A175" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="B175" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="C175" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="D175" t="s">
         <v>337</v>
       </c>
       <c r="E175">
-        <v>10</v>
+        <v>1</v>
       </c>
     </row>
     <row r="176" spans="1:5">
@@ -5179,10 +5153,10 @@
         <v>41</v>
       </c>
       <c r="C176" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="D176" t="s">
-        <v>325</v>
+        <v>338</v>
       </c>
       <c r="E176">
         <v>1</v>
@@ -5196,10 +5170,10 @@
         <v>41</v>
       </c>
       <c r="C177" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="D177" t="s">
-        <v>338</v>
+        <v>339</v>
       </c>
       <c r="E177">
         <v>1</v>
@@ -5207,10 +5181,10 @@
     </row>
     <row r="178" spans="1:5">
       <c r="A178" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="B178" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="C178" t="s">
         <v>171</v>
@@ -5267,7 +5241,7 @@
         <v>174</v>
       </c>
       <c r="D181" t="s">
-        <v>342</v>
+        <v>265</v>
       </c>
       <c r="E181">
         <v>1</v>
@@ -5284,7 +5258,7 @@
         <v>175</v>
       </c>
       <c r="D182" t="s">
-        <v>266</v>
+        <v>342</v>
       </c>
       <c r="E182">
         <v>1</v>
@@ -5712,7 +5686,7 @@
         <v>367</v>
       </c>
       <c r="E207">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="208" spans="1:5">
@@ -5845,7 +5819,7 @@
         <v>208</v>
       </c>
       <c r="D215" t="s">
-        <v>375</v>
+        <v>374</v>
       </c>
       <c r="E215">
         <v>2</v>
@@ -5916,7 +5890,7 @@
         <v>378</v>
       </c>
       <c r="E219">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="220" spans="1:5">
@@ -5930,7 +5904,7 @@
         <v>213</v>
       </c>
       <c r="D220" t="s">
-        <v>379</v>
+        <v>265</v>
       </c>
       <c r="E220">
         <v>3</v>
@@ -5947,10 +5921,10 @@
         <v>214</v>
       </c>
       <c r="D221" t="s">
-        <v>266</v>
+        <v>379</v>
       </c>
       <c r="E221">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="222" spans="1:5">
@@ -6035,7 +6009,7 @@
         <v>384</v>
       </c>
       <c r="E226">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="227" spans="1:5">
@@ -6069,7 +6043,7 @@
         <v>386</v>
       </c>
       <c r="E228">
-        <v>5</v>
+        <v>6</v>
       </c>
     </row>
     <row r="229" spans="1:5">
@@ -6086,7 +6060,7 @@
         <v>387</v>
       </c>
       <c r="E229">
-        <v>6</v>
+        <v>8</v>
       </c>
     </row>
     <row r="230" spans="1:5">
@@ -6103,7 +6077,7 @@
         <v>388</v>
       </c>
       <c r="E230">
-        <v>8</v>
+        <v>10</v>
       </c>
     </row>
     <row r="231" spans="1:5">
@@ -6117,7 +6091,7 @@
         <v>224</v>
       </c>
       <c r="D231" t="s">
-        <v>389</v>
+        <v>388</v>
       </c>
       <c r="E231">
         <v>10</v>
@@ -6134,10 +6108,10 @@
         <v>225</v>
       </c>
       <c r="D232" t="s">
-        <v>389</v>
+        <v>267</v>
       </c>
       <c r="E232">
-        <v>10</v>
+        <v>12</v>
       </c>
     </row>
     <row r="233" spans="1:5">
@@ -6151,7 +6125,7 @@
         <v>226</v>
       </c>
       <c r="D233" t="s">
-        <v>268</v>
+        <v>389</v>
       </c>
       <c r="E233">
         <v>12</v>
@@ -6171,7 +6145,7 @@
         <v>390</v>
       </c>
       <c r="E234">
-        <v>12</v>
+        <v>14</v>
       </c>
     </row>
     <row r="235" spans="1:5">
@@ -6188,7 +6162,7 @@
         <v>391</v>
       </c>
       <c r="E235">
-        <v>14</v>
+        <v>15</v>
       </c>
     </row>
     <row r="236" spans="1:5">
@@ -6205,15 +6179,15 @@
         <v>392</v>
       </c>
       <c r="E236">
-        <v>15</v>
+        <v>20</v>
       </c>
     </row>
     <row r="237" spans="1:5">
       <c r="A237" t="s">
-        <v>15</v>
+        <v>11</v>
       </c>
       <c r="B237" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C237" t="s">
         <v>230</v>
@@ -6222,15 +6196,15 @@
         <v>393</v>
       </c>
       <c r="E237">
-        <v>20</v>
+        <v>1</v>
       </c>
     </row>
     <row r="238" spans="1:5">
       <c r="A238" t="s">
-        <v>9</v>
+        <v>6</v>
       </c>
       <c r="B238" t="s">
-        <v>39</v>
+        <v>36</v>
       </c>
       <c r="C238" t="s">
         <v>231</v>
@@ -6244,10 +6218,10 @@
     </row>
     <row r="239" spans="1:5">
       <c r="A239" t="s">
-        <v>6</v>
+        <v>16</v>
       </c>
       <c r="B239" t="s">
-        <v>36</v>
+        <v>42</v>
       </c>
       <c r="C239" t="s">
         <v>232</v>
@@ -6261,7 +6235,7 @@
     </row>
     <row r="240" spans="1:5">
       <c r="A240" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="B240" t="s">
         <v>40</v>

</xml_diff>

<commit_message>
Atualização automática: rac (16/09/2026 12:39)
</commit_message>
<xml_diff>
--- a/Coordenadoria/02_Dados_Tratados/base_rac_tratada.xlsx
+++ b/Coordenadoria/02_Dados_Tratados/base_rac_tratada.xlsx
@@ -1212,8 +1212,16 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <fonts count="1">
+  <fonts count="2">
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -1229,7 +1237,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -1237,12 +1245,30 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1541,22 +1567,22 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:6">
-      <c r="A1" t="s">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" t="s">
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" t="s">
+      <c r="F1" s="1" t="s">
         <v>5</v>
       </c>
     </row>
@@ -2171,19 +2197,19 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:5">
-      <c r="A1" t="s">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" t="s">
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
         <v>55</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>56</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="1" t="s">
         <v>57</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualização automática: rac (17/09/2026 12:31)
</commit_message>
<xml_diff>
--- a/Coordenadoria/02_Dados_Tratados/base_rac_tratada.xlsx
+++ b/Coordenadoria/02_Dados_Tratados/base_rac_tratada.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1087" uniqueCount="397">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1091" uniqueCount="397">
   <si>
     <t>matricula</t>
   </si>
@@ -38,54 +38,54 @@
     <t>2729</t>
   </si>
   <si>
+    <t>2731</t>
+  </si>
+  <si>
+    <t>2709</t>
+  </si>
+  <si>
+    <t>2721</t>
+  </si>
+  <si>
+    <t>2732</t>
+  </si>
+  <si>
+    <t>2728</t>
+  </si>
+  <si>
+    <t>2730</t>
+  </si>
+  <si>
+    <t>2734</t>
+  </si>
+  <si>
+    <t>2726</t>
+  </si>
+  <si>
+    <t>2702</t>
+  </si>
+  <si>
+    <t>2703</t>
+  </si>
+  <si>
+    <t>2704</t>
+  </si>
+  <si>
+    <t>2708</t>
+  </si>
+  <si>
+    <t>2719</t>
+  </si>
+  <si>
+    <t>2720</t>
+  </si>
+  <si>
+    <t>2722</t>
+  </si>
+  <si>
     <t>2723</t>
   </si>
   <si>
-    <t>2731</t>
-  </si>
-  <si>
-    <t>2709</t>
-  </si>
-  <si>
-    <t>2721</t>
-  </si>
-  <si>
-    <t>2732</t>
-  </si>
-  <si>
-    <t>2728</t>
-  </si>
-  <si>
-    <t>2730</t>
-  </si>
-  <si>
-    <t>2734</t>
-  </si>
-  <si>
-    <t>2726</t>
-  </si>
-  <si>
-    <t>2702</t>
-  </si>
-  <si>
-    <t>2703</t>
-  </si>
-  <si>
-    <t>2704</t>
-  </si>
-  <si>
-    <t>2708</t>
-  </si>
-  <si>
-    <t>2719</t>
-  </si>
-  <si>
-    <t>2720</t>
-  </si>
-  <si>
-    <t>2722</t>
-  </si>
-  <si>
     <t>2733</t>
   </si>
   <si>
@@ -128,28 +128,28 @@
     <t>1º/5º GAV</t>
   </si>
   <si>
+    <t>1ª ETA</t>
+  </si>
+  <si>
+    <t>6º ETA</t>
+  </si>
+  <si>
+    <t>7º ETA</t>
+  </si>
+  <si>
+    <t>1º ETA</t>
+  </si>
+  <si>
+    <t>EPCAR</t>
+  </si>
+  <si>
+    <t>PAMALS</t>
+  </si>
+  <si>
+    <t>2ª ETA</t>
+  </si>
+  <si>
     <t>CLA</t>
-  </si>
-  <si>
-    <t>1ª ETA</t>
-  </si>
-  <si>
-    <t>6º ETA</t>
-  </si>
-  <si>
-    <t>7º ETA</t>
-  </si>
-  <si>
-    <t>1º ETA</t>
-  </si>
-  <si>
-    <t>EPCAR</t>
-  </si>
-  <si>
-    <t>PAMALS</t>
-  </si>
-  <si>
-    <t>2ª ETA</t>
   </si>
   <si>
     <t>1/15 GAV</t>
@@ -1212,16 +1212,8 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <fonts count="2">
+  <fonts count="1">
     <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -1237,7 +1229,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -1245,30 +1237,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color auto="1"/>
-      </left>
-      <right style="thin">
-        <color auto="1"/>
-      </right>
-      <top style="thin">
-        <color auto="1"/>
-      </top>
-      <bottom style="thin">
-        <color auto="1"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1567,22 +1541,22 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:6">
-      <c r="A1" s="1" t="s">
+      <c r="A1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" s="1" t="s">
+      <c r="B1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" t="s">
         <v>5</v>
       </c>
     </row>
@@ -1614,16 +1588,16 @@
         <v>37</v>
       </c>
       <c r="C3" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="D3" t="s">
         <v>53</v>
       </c>
       <c r="E3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F3">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="4" spans="1:6">
@@ -1651,7 +1625,7 @@
         <v>9</v>
       </c>
       <c r="B5" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="C5" t="s">
         <v>50</v>
@@ -1660,10 +1634,10 @@
         <v>53</v>
       </c>
       <c r="E5">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F5">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="6" spans="1:6">
@@ -1677,13 +1651,13 @@
         <v>50</v>
       </c>
       <c r="D6" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="E6">
-        <v>2</v>
+        <v>9</v>
       </c>
       <c r="F6">
-        <v>2</v>
+        <v>10</v>
       </c>
     </row>
     <row r="7" spans="1:6">
@@ -1691,19 +1665,19 @@
         <v>11</v>
       </c>
       <c r="B7" t="s">
-        <v>40</v>
+        <v>36</v>
       </c>
       <c r="C7" t="s">
         <v>50</v>
       </c>
       <c r="D7" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="E7">
-        <v>8</v>
+        <v>30</v>
       </c>
       <c r="F7">
-        <v>9</v>
+        <v>51</v>
       </c>
     </row>
     <row r="8" spans="1:6">
@@ -1711,19 +1685,19 @@
         <v>12</v>
       </c>
       <c r="B8" t="s">
-        <v>36</v>
+        <v>39</v>
       </c>
       <c r="C8" t="s">
         <v>50</v>
       </c>
       <c r="D8" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="E8">
-        <v>30</v>
+        <v>39</v>
       </c>
       <c r="F8">
-        <v>51</v>
+        <v>106</v>
       </c>
     </row>
     <row r="9" spans="1:6">
@@ -1731,7 +1705,7 @@
         <v>13</v>
       </c>
       <c r="B9" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="C9" t="s">
         <v>50</v>
@@ -1740,10 +1714,10 @@
         <v>54</v>
       </c>
       <c r="E9">
-        <v>39</v>
+        <v>68</v>
       </c>
       <c r="F9">
-        <v>106</v>
+        <v>150</v>
       </c>
     </row>
     <row r="10" spans="1:6">
@@ -1760,10 +1734,10 @@
         <v>54</v>
       </c>
       <c r="E10">
-        <v>68</v>
+        <v>80</v>
       </c>
       <c r="F10">
-        <v>150</v>
+        <v>229</v>
       </c>
     </row>
     <row r="11" spans="1:6">
@@ -1777,13 +1751,13 @@
         <v>50</v>
       </c>
       <c r="D11" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="E11">
-        <v>80</v>
+        <v>4</v>
       </c>
       <c r="F11">
-        <v>229</v>
+        <v>4</v>
       </c>
     </row>
     <row r="12" spans="1:6">
@@ -1791,19 +1765,19 @@
         <v>16</v>
       </c>
       <c r="B12" t="s">
-        <v>42</v>
+        <v>36</v>
       </c>
       <c r="C12" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="D12" t="s">
         <v>53</v>
       </c>
       <c r="E12">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="F12">
-        <v>4</v>
+        <v>0</v>
       </c>
     </row>
     <row r="13" spans="1:6">
@@ -1811,7 +1785,7 @@
         <v>17</v>
       </c>
       <c r="B13" t="s">
-        <v>36</v>
+        <v>42</v>
       </c>
       <c r="C13" t="s">
         <v>51</v>
@@ -1831,7 +1805,7 @@
         <v>18</v>
       </c>
       <c r="B14" t="s">
-        <v>43</v>
+        <v>36</v>
       </c>
       <c r="C14" t="s">
         <v>51</v>
@@ -1851,7 +1825,7 @@
         <v>19</v>
       </c>
       <c r="B15" t="s">
-        <v>36</v>
+        <v>43</v>
       </c>
       <c r="C15" t="s">
         <v>51</v>
@@ -1871,7 +1845,7 @@
         <v>20</v>
       </c>
       <c r="B16" t="s">
-        <v>44</v>
+        <v>38</v>
       </c>
       <c r="C16" t="s">
         <v>51</v>
@@ -1891,7 +1865,7 @@
         <v>21</v>
       </c>
       <c r="B17" t="s">
-        <v>39</v>
+        <v>43</v>
       </c>
       <c r="C17" t="s">
         <v>51</v>
@@ -1931,7 +1905,7 @@
         <v>23</v>
       </c>
       <c r="B19" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C19" t="s">
         <v>51</v>
@@ -1971,7 +1945,7 @@
         <v>25</v>
       </c>
       <c r="B21" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="C21" t="s">
         <v>51</v>
@@ -1991,7 +1965,7 @@
         <v>26</v>
       </c>
       <c r="B22" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="C22" t="s">
         <v>51</v>
@@ -2031,7 +2005,7 @@
         <v>28</v>
       </c>
       <c r="B24" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C24" t="s">
         <v>51</v>
@@ -2051,7 +2025,7 @@
         <v>29</v>
       </c>
       <c r="B25" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="C25" t="s">
         <v>51</v>
@@ -2131,7 +2105,7 @@
         <v>33</v>
       </c>
       <c r="B29" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="C29" t="s">
         <v>52</v>
@@ -2151,7 +2125,7 @@
         <v>34</v>
       </c>
       <c r="B30" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="C30" t="s">
         <v>52</v>
@@ -2193,23 +2167,23 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E240"/>
+  <dimension ref="A1:E241"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:5">
-      <c r="A1" s="1" t="s">
+      <c r="A1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" s="1" t="s">
+      <c r="B1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" t="s">
         <v>55</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" t="s">
         <v>56</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" t="s">
         <v>57</v>
       </c>
     </row>
@@ -2300,10 +2274,10 @@
     </row>
     <row r="7" spans="1:5">
       <c r="A7" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="B7" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="C7" t="s">
         <v>63</v>
@@ -2317,10 +2291,10 @@
     </row>
     <row r="8" spans="1:5">
       <c r="A8" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B8" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="C8" t="s">
         <v>63</v>
@@ -2334,10 +2308,10 @@
     </row>
     <row r="9" spans="1:5">
       <c r="A9" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="B9" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="C9" t="s">
         <v>63</v>
@@ -2351,10 +2325,10 @@
     </row>
     <row r="10" spans="1:5">
       <c r="A10" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B10" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="C10" t="s">
         <v>63</v>
@@ -2368,7 +2342,7 @@
     </row>
     <row r="11" spans="1:5">
       <c r="A11" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B11" t="s">
         <v>36</v>
@@ -2385,10 +2359,10 @@
     </row>
     <row r="12" spans="1:5">
       <c r="A12" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B12" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="C12" t="s">
         <v>63</v>
@@ -2402,10 +2376,10 @@
     </row>
     <row r="13" spans="1:5">
       <c r="A13" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B13" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="C13" t="s">
         <v>63</v>
@@ -2419,10 +2393,10 @@
     </row>
     <row r="14" spans="1:5">
       <c r="A14" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B14" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C14" t="s">
         <v>63</v>
@@ -2436,7 +2410,7 @@
     </row>
     <row r="15" spans="1:5">
       <c r="A15" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B15" t="s">
         <v>36</v>
@@ -2453,10 +2427,10 @@
     </row>
     <row r="16" spans="1:5">
       <c r="A16" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B16" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C16" t="s">
         <v>64</v>
@@ -2470,10 +2444,10 @@
     </row>
     <row r="17" spans="1:5">
       <c r="A17" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="B17" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="C17" t="s">
         <v>65</v>
@@ -2487,10 +2461,10 @@
     </row>
     <row r="18" spans="1:5">
       <c r="A18" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B18" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="C18" t="s">
         <v>65</v>
@@ -2504,7 +2478,7 @@
     </row>
     <row r="19" spans="1:5">
       <c r="A19" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B19" t="s">
         <v>36</v>
@@ -2521,10 +2495,10 @@
     </row>
     <row r="20" spans="1:5">
       <c r="A20" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B20" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="C20" t="s">
         <v>65</v>
@@ -2538,10 +2512,10 @@
     </row>
     <row r="21" spans="1:5">
       <c r="A21" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B21" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="C21" t="s">
         <v>65</v>
@@ -2555,10 +2529,10 @@
     </row>
     <row r="22" spans="1:5">
       <c r="A22" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B22" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C22" t="s">
         <v>65</v>
@@ -2572,10 +2546,10 @@
     </row>
     <row r="23" spans="1:5">
       <c r="A23" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B23" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="C23" t="s">
         <v>66</v>
@@ -2589,10 +2563,10 @@
     </row>
     <row r="24" spans="1:5">
       <c r="A24" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B24" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="C24" t="s">
         <v>66</v>
@@ -2606,10 +2580,10 @@
     </row>
     <row r="25" spans="1:5">
       <c r="A25" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B25" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="C25" t="s">
         <v>66</v>
@@ -2623,10 +2597,10 @@
     </row>
     <row r="26" spans="1:5">
       <c r="A26" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B26" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="C26" t="s">
         <v>67</v>
@@ -2640,10 +2614,10 @@
     </row>
     <row r="27" spans="1:5">
       <c r="A27" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B27" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="C27" t="s">
         <v>67</v>
@@ -2657,10 +2631,10 @@
     </row>
     <row r="28" spans="1:5">
       <c r="A28" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B28" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="C28" t="s">
         <v>67</v>
@@ -2674,10 +2648,10 @@
     </row>
     <row r="29" spans="1:5">
       <c r="A29" t="s">
-        <v>14</v>
+        <v>10</v>
       </c>
       <c r="B29" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="C29" t="s">
         <v>68</v>
@@ -2691,16 +2665,16 @@
     </row>
     <row r="30" spans="1:5">
       <c r="A30" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="B30" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="C30" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="D30" t="s">
-        <v>245</v>
+        <v>244</v>
       </c>
       <c r="E30">
         <v>1</v>
@@ -2708,10 +2682,10 @@
     </row>
     <row r="31" spans="1:5">
       <c r="A31" t="s">
-        <v>14</v>
+        <v>10</v>
       </c>
       <c r="B31" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="C31" t="s">
         <v>69</v>
@@ -2725,27 +2699,27 @@
     </row>
     <row r="32" spans="1:5">
       <c r="A32" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="B32" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="C32" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="D32" t="s">
-        <v>246</v>
+        <v>245</v>
       </c>
       <c r="E32">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="33" spans="1:5">
       <c r="A33" t="s">
-        <v>13</v>
+        <v>10</v>
       </c>
       <c r="B33" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="C33" t="s">
         <v>70</v>
@@ -2759,10 +2733,10 @@
     </row>
     <row r="34" spans="1:5">
       <c r="A34" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="B34" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="C34" t="s">
         <v>70</v>
@@ -2776,27 +2750,27 @@
     </row>
     <row r="35" spans="1:5">
       <c r="A35" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="B35" t="s">
-        <v>36</v>
+        <v>39</v>
       </c>
       <c r="C35" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="D35" t="s">
-        <v>247</v>
+        <v>246</v>
       </c>
       <c r="E35">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="36" spans="1:5">
       <c r="A36" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="B36" t="s">
-        <v>40</v>
+        <v>36</v>
       </c>
       <c r="C36" t="s">
         <v>71</v>
@@ -2810,10 +2784,10 @@
     </row>
     <row r="37" spans="1:5">
       <c r="A37" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="B37" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="C37" t="s">
         <v>71</v>
@@ -2827,16 +2801,16 @@
     </row>
     <row r="38" spans="1:5">
       <c r="A38" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="B38" t="s">
-        <v>36</v>
+        <v>39</v>
       </c>
       <c r="C38" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="D38" t="s">
-        <v>248</v>
+        <v>247</v>
       </c>
       <c r="E38">
         <v>1</v>
@@ -2844,10 +2818,10 @@
     </row>
     <row r="39" spans="1:5">
       <c r="A39" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="B39" t="s">
-        <v>40</v>
+        <v>36</v>
       </c>
       <c r="C39" t="s">
         <v>72</v>
@@ -2861,10 +2835,10 @@
     </row>
     <row r="40" spans="1:5">
       <c r="A40" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="B40" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="C40" t="s">
         <v>72</v>
@@ -2878,16 +2852,16 @@
     </row>
     <row r="41" spans="1:5">
       <c r="A41" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="B41" t="s">
-        <v>36</v>
+        <v>39</v>
       </c>
       <c r="C41" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="D41" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
       <c r="E41">
         <v>1</v>
@@ -2895,10 +2869,10 @@
     </row>
     <row r="42" spans="1:5">
       <c r="A42" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="B42" t="s">
-        <v>40</v>
+        <v>36</v>
       </c>
       <c r="C42" t="s">
         <v>73</v>
@@ -2915,13 +2889,13 @@
         <v>12</v>
       </c>
       <c r="B43" t="s">
-        <v>36</v>
+        <v>39</v>
       </c>
       <c r="C43" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="D43" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
       <c r="E43">
         <v>1</v>
@@ -2929,10 +2903,10 @@
     </row>
     <row r="44" spans="1:5">
       <c r="A44" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="B44" t="s">
-        <v>40</v>
+        <v>36</v>
       </c>
       <c r="C44" t="s">
         <v>74</v>
@@ -2946,10 +2920,10 @@
     </row>
     <row r="45" spans="1:5">
       <c r="A45" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="B45" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="C45" t="s">
         <v>74</v>
@@ -2963,16 +2937,16 @@
     </row>
     <row r="46" spans="1:5">
       <c r="A46" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="B46" t="s">
-        <v>36</v>
+        <v>40</v>
       </c>
       <c r="C46" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="D46" t="s">
-        <v>251</v>
+        <v>250</v>
       </c>
       <c r="E46">
         <v>1</v>
@@ -2980,16 +2954,16 @@
     </row>
     <row r="47" spans="1:5">
       <c r="A47" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B47" t="s">
         <v>36</v>
       </c>
       <c r="C47" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="D47" t="s">
-        <v>252</v>
+        <v>251</v>
       </c>
       <c r="E47">
         <v>1</v>
@@ -2997,16 +2971,16 @@
     </row>
     <row r="48" spans="1:5">
       <c r="A48" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B48" t="s">
         <v>36</v>
       </c>
       <c r="C48" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="D48" t="s">
-        <v>253</v>
+        <v>252</v>
       </c>
       <c r="E48">
         <v>1</v>
@@ -3014,16 +2988,16 @@
     </row>
     <row r="49" spans="1:5">
       <c r="A49" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B49" t="s">
         <v>36</v>
       </c>
       <c r="C49" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="D49" t="s">
-        <v>254</v>
+        <v>253</v>
       </c>
       <c r="E49">
         <v>1</v>
@@ -3031,16 +3005,16 @@
     </row>
     <row r="50" spans="1:5">
       <c r="A50" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B50" t="s">
         <v>36</v>
       </c>
       <c r="C50" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="D50" t="s">
-        <v>255</v>
+        <v>254</v>
       </c>
       <c r="E50">
         <v>1</v>
@@ -3048,16 +3022,16 @@
     </row>
     <row r="51" spans="1:5">
       <c r="A51" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B51" t="s">
         <v>36</v>
       </c>
       <c r="C51" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="D51" t="s">
-        <v>256</v>
+        <v>255</v>
       </c>
       <c r="E51">
         <v>1</v>
@@ -3065,16 +3039,16 @@
     </row>
     <row r="52" spans="1:5">
       <c r="A52" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B52" t="s">
         <v>36</v>
       </c>
       <c r="C52" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="D52" t="s">
-        <v>257</v>
+        <v>256</v>
       </c>
       <c r="E52">
         <v>1</v>
@@ -3082,16 +3056,16 @@
     </row>
     <row r="53" spans="1:5">
       <c r="A53" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B53" t="s">
         <v>36</v>
       </c>
       <c r="C53" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="D53" t="s">
-        <v>258</v>
+        <v>257</v>
       </c>
       <c r="E53">
         <v>1</v>
@@ -3099,27 +3073,27 @@
     </row>
     <row r="54" spans="1:5">
       <c r="A54" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B54" t="s">
         <v>36</v>
       </c>
       <c r="C54" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="D54" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="E54">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="55" spans="1:5">
       <c r="A55" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="B55" t="s">
-        <v>40</v>
+        <v>36</v>
       </c>
       <c r="C55" t="s">
         <v>83</v>
@@ -3128,15 +3102,15 @@
         <v>259</v>
       </c>
       <c r="E55">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="56" spans="1:5">
       <c r="A56" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="B56" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="C56" t="s">
         <v>83</v>
@@ -3145,15 +3119,15 @@
         <v>259</v>
       </c>
       <c r="E56">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="57" spans="1:5">
       <c r="A57" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="B57" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="C57" t="s">
         <v>83</v>
@@ -3167,16 +3141,16 @@
     </row>
     <row r="58" spans="1:5">
       <c r="A58" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="B58" t="s">
-        <v>36</v>
+        <v>40</v>
       </c>
       <c r="C58" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="D58" t="s">
-        <v>260</v>
+        <v>259</v>
       </c>
       <c r="E58">
         <v>2</v>
@@ -3184,10 +3158,10 @@
     </row>
     <row r="59" spans="1:5">
       <c r="A59" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="B59" t="s">
-        <v>40</v>
+        <v>36</v>
       </c>
       <c r="C59" t="s">
         <v>84</v>
@@ -3201,10 +3175,10 @@
     </row>
     <row r="60" spans="1:5">
       <c r="A60" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="B60" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="C60" t="s">
         <v>84</v>
@@ -3213,32 +3187,32 @@
         <v>260</v>
       </c>
       <c r="E60">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="61" spans="1:5">
       <c r="A61" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="B61" t="s">
-        <v>36</v>
+        <v>40</v>
       </c>
       <c r="C61" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="D61" t="s">
-        <v>261</v>
+        <v>260</v>
       </c>
       <c r="E61">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="62" spans="1:5">
       <c r="A62" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="B62" t="s">
-        <v>40</v>
+        <v>36</v>
       </c>
       <c r="C62" t="s">
         <v>85</v>
@@ -3247,15 +3221,15 @@
         <v>261</v>
       </c>
       <c r="E62">
-        <v>4</v>
+        <v>2</v>
       </c>
     </row>
     <row r="63" spans="1:5">
       <c r="A63" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="B63" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="C63" t="s">
         <v>85</v>
@@ -3264,21 +3238,21 @@
         <v>261</v>
       </c>
       <c r="E63">
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
     <row r="64" spans="1:5">
       <c r="A64" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="B64" t="s">
-        <v>36</v>
+        <v>40</v>
       </c>
       <c r="C64" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="D64" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
       <c r="E64">
         <v>2</v>
@@ -3286,10 +3260,10 @@
     </row>
     <row r="65" spans="1:5">
       <c r="A65" t="s">
-        <v>15</v>
+        <v>11</v>
       </c>
       <c r="B65" t="s">
-        <v>41</v>
+        <v>36</v>
       </c>
       <c r="C65" t="s">
         <v>86</v>
@@ -3298,38 +3272,38 @@
         <v>262</v>
       </c>
       <c r="E65">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="66" spans="1:5">
       <c r="A66" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="B66" t="s">
-        <v>36</v>
+        <v>40</v>
       </c>
       <c r="C66" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="D66" t="s">
-        <v>263</v>
+        <v>262</v>
       </c>
       <c r="E66">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="67" spans="1:5">
       <c r="A67" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B67" t="s">
         <v>36</v>
       </c>
       <c r="C67" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="D67" t="s">
-        <v>264</v>
+        <v>263</v>
       </c>
       <c r="E67">
         <v>2</v>
@@ -3337,16 +3311,16 @@
     </row>
     <row r="68" spans="1:5">
       <c r="A68" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B68" t="s">
         <v>36</v>
       </c>
       <c r="C68" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="D68" t="s">
-        <v>265</v>
+        <v>264</v>
       </c>
       <c r="E68">
         <v>2</v>
@@ -3354,16 +3328,16 @@
     </row>
     <row r="69" spans="1:5">
       <c r="A69" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B69" t="s">
         <v>36</v>
       </c>
       <c r="C69" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="D69" t="s">
-        <v>266</v>
+        <v>265</v>
       </c>
       <c r="E69">
         <v>2</v>
@@ -3371,16 +3345,16 @@
     </row>
     <row r="70" spans="1:5">
       <c r="A70" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B70" t="s">
         <v>36</v>
       </c>
       <c r="C70" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="D70" t="s">
-        <v>267</v>
+        <v>266</v>
       </c>
       <c r="E70">
         <v>2</v>
@@ -3388,16 +3362,16 @@
     </row>
     <row r="71" spans="1:5">
       <c r="A71" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B71" t="s">
         <v>36</v>
       </c>
       <c r="C71" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="D71" t="s">
-        <v>268</v>
+        <v>267</v>
       </c>
       <c r="E71">
         <v>2</v>
@@ -3405,16 +3379,16 @@
     </row>
     <row r="72" spans="1:5">
       <c r="A72" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B72" t="s">
         <v>36</v>
       </c>
       <c r="C72" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="D72" t="s">
-        <v>269</v>
+        <v>268</v>
       </c>
       <c r="E72">
         <v>2</v>
@@ -3422,16 +3396,16 @@
     </row>
     <row r="73" spans="1:5">
       <c r="A73" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B73" t="s">
         <v>36</v>
       </c>
       <c r="C73" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="D73" t="s">
-        <v>259</v>
+        <v>269</v>
       </c>
       <c r="E73">
         <v>2</v>
@@ -3439,27 +3413,27 @@
     </row>
     <row r="74" spans="1:5">
       <c r="A74" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B74" t="s">
         <v>36</v>
       </c>
       <c r="C74" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="D74" t="s">
-        <v>258</v>
+        <v>259</v>
       </c>
       <c r="E74">
-        <v>4</v>
+        <v>2</v>
       </c>
     </row>
     <row r="75" spans="1:5">
       <c r="A75" t="s">
-        <v>15</v>
+        <v>11</v>
       </c>
       <c r="B75" t="s">
-        <v>41</v>
+        <v>36</v>
       </c>
       <c r="C75" t="s">
         <v>95</v>
@@ -3473,16 +3447,16 @@
     </row>
     <row r="76" spans="1:5">
       <c r="A76" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="B76" t="s">
-        <v>36</v>
+        <v>40</v>
       </c>
       <c r="C76" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="D76" t="s">
-        <v>270</v>
+        <v>258</v>
       </c>
       <c r="E76">
         <v>4</v>
@@ -3490,16 +3464,16 @@
     </row>
     <row r="77" spans="1:5">
       <c r="A77" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B77" t="s">
         <v>36</v>
       </c>
       <c r="C77" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="D77" t="s">
-        <v>271</v>
+        <v>270</v>
       </c>
       <c r="E77">
         <v>4</v>
@@ -3507,27 +3481,27 @@
     </row>
     <row r="78" spans="1:5">
       <c r="A78" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="B78" t="s">
-        <v>40</v>
+        <v>36</v>
       </c>
       <c r="C78" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="D78" t="s">
-        <v>272</v>
+        <v>271</v>
       </c>
       <c r="E78">
-        <v>1</v>
+        <v>4</v>
       </c>
     </row>
     <row r="79" spans="1:5">
       <c r="A79" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="B79" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="C79" t="s">
         <v>98</v>
@@ -3541,10 +3515,10 @@
     </row>
     <row r="80" spans="1:5">
       <c r="A80" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="B80" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="C80" t="s">
         <v>98</v>
@@ -3558,16 +3532,16 @@
     </row>
     <row r="81" spans="1:5">
       <c r="A81" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="B81" t="s">
         <v>40</v>
       </c>
       <c r="C81" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="D81" t="s">
-        <v>273</v>
+        <v>272</v>
       </c>
       <c r="E81">
         <v>1</v>
@@ -3575,10 +3549,10 @@
     </row>
     <row r="82" spans="1:5">
       <c r="A82" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="B82" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="C82" t="s">
         <v>99</v>
@@ -3592,10 +3566,10 @@
     </row>
     <row r="83" spans="1:5">
       <c r="A83" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="B83" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="C83" t="s">
         <v>99</v>
@@ -3604,32 +3578,32 @@
         <v>273</v>
       </c>
       <c r="E83">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="84" spans="1:5">
       <c r="A84" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="B84" t="s">
         <v>40</v>
       </c>
       <c r="C84" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="D84" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
       <c r="E84">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="85" spans="1:5">
       <c r="A85" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="B85" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="C85" t="s">
         <v>100</v>
@@ -3646,13 +3620,13 @@
         <v>13</v>
       </c>
       <c r="B86" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="C86" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="D86" t="s">
-        <v>275</v>
+        <v>274</v>
       </c>
       <c r="E86">
         <v>1</v>
@@ -3660,10 +3634,10 @@
     </row>
     <row r="87" spans="1:5">
       <c r="A87" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="B87" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="C87" t="s">
         <v>101</v>
@@ -3680,13 +3654,13 @@
         <v>13</v>
       </c>
       <c r="B88" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="C88" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="D88" t="s">
-        <v>276</v>
+        <v>275</v>
       </c>
       <c r="E88">
         <v>1</v>
@@ -3694,10 +3668,10 @@
     </row>
     <row r="89" spans="1:5">
       <c r="A89" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="B89" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="C89" t="s">
         <v>102</v>
@@ -3714,13 +3688,13 @@
         <v>13</v>
       </c>
       <c r="B90" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="C90" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="D90" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
       <c r="E90">
         <v>1</v>
@@ -3728,10 +3702,10 @@
     </row>
     <row r="91" spans="1:5">
       <c r="A91" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="B91" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="C91" t="s">
         <v>103</v>
@@ -3748,13 +3722,13 @@
         <v>13</v>
       </c>
       <c r="B92" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="C92" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="D92" t="s">
-        <v>278</v>
+        <v>277</v>
       </c>
       <c r="E92">
         <v>1</v>
@@ -3762,10 +3736,10 @@
     </row>
     <row r="93" spans="1:5">
       <c r="A93" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="B93" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="C93" t="s">
         <v>104</v>
@@ -3782,13 +3756,13 @@
         <v>13</v>
       </c>
       <c r="B94" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="C94" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="D94" t="s">
-        <v>279</v>
+        <v>278</v>
       </c>
       <c r="E94">
         <v>1</v>
@@ -3796,10 +3770,10 @@
     </row>
     <row r="95" spans="1:5">
       <c r="A95" t="s">
-        <v>15</v>
+        <v>12</v>
       </c>
       <c r="B95" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="C95" t="s">
         <v>105</v>
@@ -3813,16 +3787,16 @@
     </row>
     <row r="96" spans="1:5">
       <c r="A96" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="B96" t="s">
         <v>40</v>
       </c>
       <c r="C96" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="D96" t="s">
-        <v>280</v>
+        <v>279</v>
       </c>
       <c r="E96">
         <v>1</v>
@@ -3830,10 +3804,10 @@
     </row>
     <row r="97" spans="1:5">
       <c r="A97" t="s">
-        <v>15</v>
+        <v>12</v>
       </c>
       <c r="B97" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="C97" t="s">
         <v>106</v>
@@ -3847,16 +3821,16 @@
     </row>
     <row r="98" spans="1:5">
       <c r="A98" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="B98" t="s">
         <v>40</v>
       </c>
       <c r="C98" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="D98" t="s">
-        <v>281</v>
+        <v>280</v>
       </c>
       <c r="E98">
         <v>1</v>
@@ -3864,10 +3838,10 @@
     </row>
     <row r="99" spans="1:5">
       <c r="A99" t="s">
-        <v>15</v>
+        <v>12</v>
       </c>
       <c r="B99" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="C99" t="s">
         <v>107</v>
@@ -3881,16 +3855,16 @@
     </row>
     <row r="100" spans="1:5">
       <c r="A100" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="B100" t="s">
         <v>40</v>
       </c>
       <c r="C100" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="D100" t="s">
-        <v>282</v>
+        <v>281</v>
       </c>
       <c r="E100">
         <v>1</v>
@@ -3898,16 +3872,16 @@
     </row>
     <row r="101" spans="1:5">
       <c r="A101" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B101" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="C101" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="D101" t="s">
-        <v>283</v>
+        <v>282</v>
       </c>
       <c r="E101">
         <v>1</v>
@@ -3915,16 +3889,16 @@
     </row>
     <row r="102" spans="1:5">
       <c r="A102" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B102" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="C102" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="D102" t="s">
-        <v>284</v>
+        <v>283</v>
       </c>
       <c r="E102">
         <v>1</v>
@@ -3932,16 +3906,16 @@
     </row>
     <row r="103" spans="1:5">
       <c r="A103" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B103" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="C103" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="D103" t="s">
-        <v>285</v>
+        <v>284</v>
       </c>
       <c r="E103">
         <v>1</v>
@@ -3949,16 +3923,16 @@
     </row>
     <row r="104" spans="1:5">
       <c r="A104" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B104" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="C104" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="D104" t="s">
-        <v>286</v>
+        <v>285</v>
       </c>
       <c r="E104">
         <v>1</v>
@@ -3966,16 +3940,16 @@
     </row>
     <row r="105" spans="1:5">
       <c r="A105" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B105" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="C105" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="D105" t="s">
-        <v>287</v>
+        <v>286</v>
       </c>
       <c r="E105">
         <v>1</v>
@@ -3983,27 +3957,27 @@
     </row>
     <row r="106" spans="1:5">
       <c r="A106" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B106" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="C106" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="D106" t="s">
-        <v>288</v>
+        <v>287</v>
       </c>
       <c r="E106">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="107" spans="1:5">
       <c r="A107" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="B107" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="C107" t="s">
         <v>114</v>
@@ -4012,7 +3986,7 @@
         <v>288</v>
       </c>
       <c r="E107">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="108" spans="1:5">
@@ -4020,24 +3994,24 @@
         <v>13</v>
       </c>
       <c r="B108" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="C108" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="D108" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
       <c r="E108">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="109" spans="1:5">
       <c r="A109" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="B109" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="C109" t="s">
         <v>115</v>
@@ -4051,10 +4025,10 @@
     </row>
     <row r="110" spans="1:5">
       <c r="A110" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="B110" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="C110" t="s">
         <v>115</v>
@@ -4068,16 +4042,16 @@
     </row>
     <row r="111" spans="1:5">
       <c r="A111" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="B111" t="s">
         <v>40</v>
       </c>
       <c r="C111" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="D111" t="s">
-        <v>290</v>
+        <v>289</v>
       </c>
       <c r="E111">
         <v>2</v>
@@ -4085,10 +4059,10 @@
     </row>
     <row r="112" spans="1:5">
       <c r="A112" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="B112" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="C112" t="s">
         <v>116</v>
@@ -4102,10 +4076,10 @@
     </row>
     <row r="113" spans="1:5">
       <c r="A113" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="B113" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="C113" t="s">
         <v>116</v>
@@ -4119,16 +4093,16 @@
     </row>
     <row r="114" spans="1:5">
       <c r="A114" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="B114" t="s">
         <v>40</v>
       </c>
       <c r="C114" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="D114" t="s">
-        <v>291</v>
+        <v>290</v>
       </c>
       <c r="E114">
         <v>2</v>
@@ -4136,10 +4110,10 @@
     </row>
     <row r="115" spans="1:5">
       <c r="A115" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="B115" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="C115" t="s">
         <v>117</v>
@@ -4156,13 +4130,13 @@
         <v>13</v>
       </c>
       <c r="B116" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="C116" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="D116" t="s">
-        <v>273</v>
+        <v>291</v>
       </c>
       <c r="E116">
         <v>2</v>
@@ -4170,10 +4144,10 @@
     </row>
     <row r="117" spans="1:5">
       <c r="A117" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="B117" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="C117" t="s">
         <v>118</v>
@@ -4182,15 +4156,15 @@
         <v>273</v>
       </c>
       <c r="E117">
-        <v>4</v>
+        <v>2</v>
       </c>
     </row>
     <row r="118" spans="1:5">
       <c r="A118" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="B118" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="C118" t="s">
         <v>118</v>
@@ -4204,27 +4178,27 @@
     </row>
     <row r="119" spans="1:5">
       <c r="A119" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="B119" t="s">
         <v>40</v>
       </c>
       <c r="C119" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="D119" t="s">
-        <v>292</v>
+        <v>273</v>
       </c>
       <c r="E119">
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
     <row r="120" spans="1:5">
       <c r="A120" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="B120" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="C120" t="s">
         <v>119</v>
@@ -4233,7 +4207,7 @@
         <v>292</v>
       </c>
       <c r="E120">
-        <v>4</v>
+        <v>2</v>
       </c>
     </row>
     <row r="121" spans="1:5">
@@ -4241,30 +4215,30 @@
         <v>13</v>
       </c>
       <c r="B121" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="C121" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="D121" t="s">
-        <v>277</v>
+        <v>292</v>
       </c>
       <c r="E121">
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
     <row r="122" spans="1:5">
       <c r="A122" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B122" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="C122" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="D122" t="s">
-        <v>293</v>
+        <v>277</v>
       </c>
       <c r="E122">
         <v>2</v>
@@ -4272,16 +4246,16 @@
     </row>
     <row r="123" spans="1:5">
       <c r="A123" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B123" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="C123" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="D123" t="s">
-        <v>294</v>
+        <v>293</v>
       </c>
       <c r="E123">
         <v>2</v>
@@ -4289,27 +4263,27 @@
     </row>
     <row r="124" spans="1:5">
       <c r="A124" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B124" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="C124" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="D124" t="s">
-        <v>295</v>
+        <v>294</v>
       </c>
       <c r="E124">
-        <v>5</v>
+        <v>2</v>
       </c>
     </row>
     <row r="125" spans="1:5">
       <c r="A125" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="B125" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="C125" t="s">
         <v>123</v>
@@ -4326,75 +4300,75 @@
         <v>13</v>
       </c>
       <c r="B126" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="C126" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="D126" t="s">
-        <v>296</v>
+        <v>295</v>
       </c>
       <c r="E126">
-        <v>7</v>
+        <v>5</v>
       </c>
     </row>
     <row r="127" spans="1:5">
       <c r="A127" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B127" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="C127" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="D127" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="E127">
-        <v>8</v>
+        <v>7</v>
       </c>
     </row>
     <row r="128" spans="1:5">
       <c r="A128" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B128" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="C128" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="D128" t="s">
-        <v>298</v>
+        <v>297</v>
       </c>
       <c r="E128">
-        <v>10</v>
+        <v>8</v>
       </c>
     </row>
     <row r="129" spans="1:5">
       <c r="A129" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B129" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="C129" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="D129" t="s">
-        <v>299</v>
+        <v>298</v>
       </c>
       <c r="E129">
-        <v>30</v>
+        <v>10</v>
       </c>
     </row>
     <row r="130" spans="1:5">
       <c r="A130" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="B130" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="C130" t="s">
         <v>127</v>
@@ -4408,27 +4382,27 @@
     </row>
     <row r="131" spans="1:5">
       <c r="A131" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B131" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="C131" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="D131" t="s">
-        <v>300</v>
+        <v>299</v>
       </c>
       <c r="E131">
-        <v>1</v>
+        <v>30</v>
       </c>
     </row>
     <row r="132" spans="1:5">
       <c r="A132" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="B132" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="C132" t="s">
         <v>128</v>
@@ -4448,10 +4422,10 @@
         <v>40</v>
       </c>
       <c r="C133" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="D133" t="s">
-        <v>301</v>
+        <v>300</v>
       </c>
       <c r="E133">
         <v>1</v>
@@ -4459,16 +4433,16 @@
     </row>
     <row r="134" spans="1:5">
       <c r="A134" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B134" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="C134" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="D134" t="s">
-        <v>302</v>
+        <v>301</v>
       </c>
       <c r="E134">
         <v>1</v>
@@ -4476,16 +4450,16 @@
     </row>
     <row r="135" spans="1:5">
       <c r="A135" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B135" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="C135" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="D135" t="s">
-        <v>303</v>
+        <v>302</v>
       </c>
       <c r="E135">
         <v>1</v>
@@ -4493,16 +4467,16 @@
     </row>
     <row r="136" spans="1:5">
       <c r="A136" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B136" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="C136" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="D136" t="s">
-        <v>304</v>
+        <v>303</v>
       </c>
       <c r="E136">
         <v>1</v>
@@ -4510,16 +4484,16 @@
     </row>
     <row r="137" spans="1:5">
       <c r="A137" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B137" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="C137" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="D137" t="s">
-        <v>305</v>
+        <v>304</v>
       </c>
       <c r="E137">
         <v>1</v>
@@ -4527,16 +4501,16 @@
     </row>
     <row r="138" spans="1:5">
       <c r="A138" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B138" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="C138" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="D138" t="s">
-        <v>306</v>
+        <v>305</v>
       </c>
       <c r="E138">
         <v>1</v>
@@ -4544,16 +4518,16 @@
     </row>
     <row r="139" spans="1:5">
       <c r="A139" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B139" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="C139" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="D139" t="s">
-        <v>307</v>
+        <v>306</v>
       </c>
       <c r="E139">
         <v>1</v>
@@ -4561,16 +4535,16 @@
     </row>
     <row r="140" spans="1:5">
       <c r="A140" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B140" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="C140" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="D140" t="s">
-        <v>308</v>
+        <v>307</v>
       </c>
       <c r="E140">
         <v>1</v>
@@ -4578,16 +4552,16 @@
     </row>
     <row r="141" spans="1:5">
       <c r="A141" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B141" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="C141" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="D141" t="s">
-        <v>309</v>
+        <v>308</v>
       </c>
       <c r="E141">
         <v>1</v>
@@ -4595,10 +4569,10 @@
     </row>
     <row r="142" spans="1:5">
       <c r="A142" t="s">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="B142" t="s">
-        <v>42</v>
+        <v>39</v>
       </c>
       <c r="C142" t="s">
         <v>137</v>
@@ -4612,16 +4586,16 @@
     </row>
     <row r="143" spans="1:5">
       <c r="A143" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="B143" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="C143" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="D143" t="s">
-        <v>310</v>
+        <v>309</v>
       </c>
       <c r="E143">
         <v>1</v>
@@ -4629,10 +4603,10 @@
     </row>
     <row r="144" spans="1:5">
       <c r="A144" t="s">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="B144" t="s">
-        <v>42</v>
+        <v>39</v>
       </c>
       <c r="C144" t="s">
         <v>138</v>
@@ -4646,16 +4620,16 @@
     </row>
     <row r="145" spans="1:5">
       <c r="A145" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="B145" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="C145" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="D145" t="s">
-        <v>311</v>
+        <v>310</v>
       </c>
       <c r="E145">
         <v>1</v>
@@ -4663,16 +4637,16 @@
     </row>
     <row r="146" spans="1:5">
       <c r="A146" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B146" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="C146" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="D146" t="s">
-        <v>312</v>
+        <v>311</v>
       </c>
       <c r="E146">
         <v>1</v>
@@ -4680,16 +4654,16 @@
     </row>
     <row r="147" spans="1:5">
       <c r="A147" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B147" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="C147" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="D147" t="s">
-        <v>313</v>
+        <v>312</v>
       </c>
       <c r="E147">
         <v>1</v>
@@ -4697,16 +4671,16 @@
     </row>
     <row r="148" spans="1:5">
       <c r="A148" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B148" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="C148" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="D148" t="s">
-        <v>314</v>
+        <v>313</v>
       </c>
       <c r="E148">
         <v>1</v>
@@ -4714,16 +4688,16 @@
     </row>
     <row r="149" spans="1:5">
       <c r="A149" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B149" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="C149" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="D149" t="s">
-        <v>315</v>
+        <v>314</v>
       </c>
       <c r="E149">
         <v>1</v>
@@ -4731,16 +4705,16 @@
     </row>
     <row r="150" spans="1:5">
       <c r="A150" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B150" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="C150" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="D150" t="s">
-        <v>316</v>
+        <v>315</v>
       </c>
       <c r="E150">
         <v>1</v>
@@ -4748,16 +4722,16 @@
     </row>
     <row r="151" spans="1:5">
       <c r="A151" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B151" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="C151" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="D151" t="s">
-        <v>317</v>
+        <v>316</v>
       </c>
       <c r="E151">
         <v>1</v>
@@ -4765,16 +4739,16 @@
     </row>
     <row r="152" spans="1:5">
       <c r="A152" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B152" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="C152" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="D152" t="s">
-        <v>318</v>
+        <v>317</v>
       </c>
       <c r="E152">
         <v>1</v>
@@ -4782,16 +4756,16 @@
     </row>
     <row r="153" spans="1:5">
       <c r="A153" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B153" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="C153" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="D153" t="s">
-        <v>319</v>
+        <v>318</v>
       </c>
       <c r="E153">
         <v>1</v>
@@ -4799,16 +4773,16 @@
     </row>
     <row r="154" spans="1:5">
       <c r="A154" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B154" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="C154" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="D154" t="s">
-        <v>320</v>
+        <v>319</v>
       </c>
       <c r="E154">
         <v>1</v>
@@ -4816,16 +4790,16 @@
     </row>
     <row r="155" spans="1:5">
       <c r="A155" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B155" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="C155" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="D155" t="s">
-        <v>321</v>
+        <v>320</v>
       </c>
       <c r="E155">
         <v>1</v>
@@ -4833,16 +4807,16 @@
     </row>
     <row r="156" spans="1:5">
       <c r="A156" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B156" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="C156" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="D156" t="s">
-        <v>322</v>
+        <v>321</v>
       </c>
       <c r="E156">
         <v>1</v>
@@ -4850,16 +4824,16 @@
     </row>
     <row r="157" spans="1:5">
       <c r="A157" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B157" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="C157" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="D157" t="s">
-        <v>323</v>
+        <v>322</v>
       </c>
       <c r="E157">
         <v>1</v>
@@ -4867,16 +4841,16 @@
     </row>
     <row r="158" spans="1:5">
       <c r="A158" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B158" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="C158" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="D158" t="s">
-        <v>324</v>
+        <v>323</v>
       </c>
       <c r="E158">
         <v>1</v>
@@ -4884,16 +4858,16 @@
     </row>
     <row r="159" spans="1:5">
       <c r="A159" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B159" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="C159" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="D159" t="s">
-        <v>325</v>
+        <v>324</v>
       </c>
       <c r="E159">
         <v>1</v>
@@ -4901,16 +4875,16 @@
     </row>
     <row r="160" spans="1:5">
       <c r="A160" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B160" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="C160" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="D160" t="s">
-        <v>326</v>
+        <v>325</v>
       </c>
       <c r="E160">
         <v>1</v>
@@ -4918,16 +4892,16 @@
     </row>
     <row r="161" spans="1:5">
       <c r="A161" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B161" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="C161" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="D161" t="s">
-        <v>327</v>
+        <v>326</v>
       </c>
       <c r="E161">
         <v>1</v>
@@ -4935,16 +4909,16 @@
     </row>
     <row r="162" spans="1:5">
       <c r="A162" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B162" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="C162" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="D162" t="s">
-        <v>328</v>
+        <v>327</v>
       </c>
       <c r="E162">
         <v>1</v>
@@ -4952,16 +4926,16 @@
     </row>
     <row r="163" spans="1:5">
       <c r="A163" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B163" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="C163" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="D163" t="s">
-        <v>329</v>
+        <v>328</v>
       </c>
       <c r="E163">
         <v>1</v>
@@ -4969,33 +4943,33 @@
     </row>
     <row r="164" spans="1:5">
       <c r="A164" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B164" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="C164" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="D164" t="s">
-        <v>314</v>
+        <v>329</v>
       </c>
       <c r="E164">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="165" spans="1:5">
       <c r="A165" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B165" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="C165" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="D165" t="s">
-        <v>330</v>
+        <v>314</v>
       </c>
       <c r="E165">
         <v>2</v>
@@ -5003,16 +4977,16 @@
     </row>
     <row r="166" spans="1:5">
       <c r="A166" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B166" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="C166" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="D166" t="s">
-        <v>331</v>
+        <v>330</v>
       </c>
       <c r="E166">
         <v>2</v>
@@ -5020,16 +4994,16 @@
     </row>
     <row r="167" spans="1:5">
       <c r="A167" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B167" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="C167" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="D167" t="s">
-        <v>332</v>
+        <v>331</v>
       </c>
       <c r="E167">
         <v>2</v>
@@ -5037,16 +5011,16 @@
     </row>
     <row r="168" spans="1:5">
       <c r="A168" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B168" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="C168" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="D168" t="s">
-        <v>333</v>
+        <v>332</v>
       </c>
       <c r="E168">
         <v>2</v>
@@ -5054,67 +5028,67 @@
     </row>
     <row r="169" spans="1:5">
       <c r="A169" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B169" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="C169" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="D169" t="s">
-        <v>334</v>
+        <v>333</v>
       </c>
       <c r="E169">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="170" spans="1:5">
       <c r="A170" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B170" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="C170" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="D170" t="s">
-        <v>299</v>
+        <v>334</v>
       </c>
       <c r="E170">
-        <v>5</v>
+        <v>3</v>
       </c>
     </row>
     <row r="171" spans="1:5">
       <c r="A171" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B171" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="C171" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="D171" t="s">
-        <v>335</v>
+        <v>299</v>
       </c>
       <c r="E171">
-        <v>8</v>
+        <v>5</v>
       </c>
     </row>
     <row r="172" spans="1:5">
       <c r="A172" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B172" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="C172" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="D172" t="s">
-        <v>255</v>
+        <v>335</v>
       </c>
       <c r="E172">
         <v>8</v>
@@ -5122,50 +5096,50 @@
     </row>
     <row r="173" spans="1:5">
       <c r="A173" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B173" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="C173" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="D173" t="s">
-        <v>336</v>
+        <v>255</v>
       </c>
       <c r="E173">
-        <v>10</v>
+        <v>8</v>
       </c>
     </row>
     <row r="174" spans="1:5">
       <c r="A174" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="B174" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="C174" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="D174" t="s">
-        <v>324</v>
+        <v>336</v>
       </c>
       <c r="E174">
-        <v>1</v>
+        <v>10</v>
       </c>
     </row>
     <row r="175" spans="1:5">
       <c r="A175" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B175" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C175" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="D175" t="s">
-        <v>337</v>
+        <v>324</v>
       </c>
       <c r="E175">
         <v>1</v>
@@ -5173,16 +5147,16 @@
     </row>
     <row r="176" spans="1:5">
       <c r="A176" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B176" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C176" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="D176" t="s">
-        <v>338</v>
+        <v>337</v>
       </c>
       <c r="E176">
         <v>1</v>
@@ -5190,16 +5164,16 @@
     </row>
     <row r="177" spans="1:5">
       <c r="A177" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B177" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C177" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="D177" t="s">
-        <v>339</v>
+        <v>338</v>
       </c>
       <c r="E177">
         <v>1</v>
@@ -5207,10 +5181,10 @@
     </row>
     <row r="178" spans="1:5">
       <c r="A178" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="B178" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="C178" t="s">
         <v>171</v>
@@ -5230,10 +5204,10 @@
         <v>41</v>
       </c>
       <c r="C179" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="D179" t="s">
-        <v>340</v>
+        <v>339</v>
       </c>
       <c r="E179">
         <v>1</v>
@@ -5241,16 +5215,16 @@
     </row>
     <row r="180" spans="1:5">
       <c r="A180" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B180" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C180" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="D180" t="s">
-        <v>341</v>
+        <v>340</v>
       </c>
       <c r="E180">
         <v>1</v>
@@ -5258,16 +5232,16 @@
     </row>
     <row r="181" spans="1:5">
       <c r="A181" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B181" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C181" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="D181" t="s">
-        <v>265</v>
+        <v>341</v>
       </c>
       <c r="E181">
         <v>1</v>
@@ -5275,16 +5249,16 @@
     </row>
     <row r="182" spans="1:5">
       <c r="A182" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B182" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C182" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="D182" t="s">
-        <v>342</v>
+        <v>265</v>
       </c>
       <c r="E182">
         <v>1</v>
@@ -5292,16 +5266,16 @@
     </row>
     <row r="183" spans="1:5">
       <c r="A183" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B183" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C183" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="D183" t="s">
-        <v>343</v>
+        <v>342</v>
       </c>
       <c r="E183">
         <v>1</v>
@@ -5309,16 +5283,16 @@
     </row>
     <row r="184" spans="1:5">
       <c r="A184" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B184" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C184" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="D184" t="s">
-        <v>344</v>
+        <v>343</v>
       </c>
       <c r="E184">
         <v>1</v>
@@ -5326,16 +5300,16 @@
     </row>
     <row r="185" spans="1:5">
       <c r="A185" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B185" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C185" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="D185" t="s">
-        <v>345</v>
+        <v>344</v>
       </c>
       <c r="E185">
         <v>1</v>
@@ -5343,16 +5317,16 @@
     </row>
     <row r="186" spans="1:5">
       <c r="A186" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B186" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C186" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="D186" t="s">
-        <v>346</v>
+        <v>345</v>
       </c>
       <c r="E186">
         <v>1</v>
@@ -5360,16 +5334,16 @@
     </row>
     <row r="187" spans="1:5">
       <c r="A187" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B187" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C187" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="D187" t="s">
-        <v>347</v>
+        <v>346</v>
       </c>
       <c r="E187">
         <v>1</v>
@@ -5377,16 +5351,16 @@
     </row>
     <row r="188" spans="1:5">
       <c r="A188" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B188" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C188" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="D188" t="s">
-        <v>348</v>
+        <v>347</v>
       </c>
       <c r="E188">
         <v>1</v>
@@ -5394,16 +5368,16 @@
     </row>
     <row r="189" spans="1:5">
       <c r="A189" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B189" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C189" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="D189" t="s">
-        <v>349</v>
+        <v>348</v>
       </c>
       <c r="E189">
         <v>1</v>
@@ -5411,16 +5385,16 @@
     </row>
     <row r="190" spans="1:5">
       <c r="A190" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B190" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C190" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="D190" t="s">
-        <v>350</v>
+        <v>349</v>
       </c>
       <c r="E190">
         <v>1</v>
@@ -5428,16 +5402,16 @@
     </row>
     <row r="191" spans="1:5">
       <c r="A191" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B191" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C191" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="D191" t="s">
-        <v>351</v>
+        <v>350</v>
       </c>
       <c r="E191">
         <v>1</v>
@@ -5445,16 +5419,16 @@
     </row>
     <row r="192" spans="1:5">
       <c r="A192" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B192" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C192" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="D192" t="s">
-        <v>352</v>
+        <v>351</v>
       </c>
       <c r="E192">
         <v>1</v>
@@ -5462,16 +5436,16 @@
     </row>
     <row r="193" spans="1:5">
       <c r="A193" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B193" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C193" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="D193" t="s">
-        <v>353</v>
+        <v>352</v>
       </c>
       <c r="E193">
         <v>1</v>
@@ -5479,16 +5453,16 @@
     </row>
     <row r="194" spans="1:5">
       <c r="A194" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B194" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C194" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="D194" t="s">
-        <v>354</v>
+        <v>353</v>
       </c>
       <c r="E194">
         <v>1</v>
@@ -5496,16 +5470,16 @@
     </row>
     <row r="195" spans="1:5">
       <c r="A195" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B195" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C195" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="D195" t="s">
-        <v>355</v>
+        <v>354</v>
       </c>
       <c r="E195">
         <v>1</v>
@@ -5513,16 +5487,16 @@
     </row>
     <row r="196" spans="1:5">
       <c r="A196" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B196" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C196" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
       <c r="D196" t="s">
-        <v>356</v>
+        <v>355</v>
       </c>
       <c r="E196">
         <v>1</v>
@@ -5530,16 +5504,16 @@
     </row>
     <row r="197" spans="1:5">
       <c r="A197" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B197" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C197" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="D197" t="s">
-        <v>357</v>
+        <v>356</v>
       </c>
       <c r="E197">
         <v>1</v>
@@ -5547,16 +5521,16 @@
     </row>
     <row r="198" spans="1:5">
       <c r="A198" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B198" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C198" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="D198" t="s">
-        <v>358</v>
+        <v>357</v>
       </c>
       <c r="E198">
         <v>1</v>
@@ -5564,16 +5538,16 @@
     </row>
     <row r="199" spans="1:5">
       <c r="A199" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B199" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C199" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
       <c r="D199" t="s">
-        <v>359</v>
+        <v>358</v>
       </c>
       <c r="E199">
         <v>1</v>
@@ -5581,16 +5555,16 @@
     </row>
     <row r="200" spans="1:5">
       <c r="A200" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B200" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C200" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="D200" t="s">
-        <v>360</v>
+        <v>359</v>
       </c>
       <c r="E200">
         <v>1</v>
@@ -5598,16 +5572,16 @@
     </row>
     <row r="201" spans="1:5">
       <c r="A201" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B201" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C201" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="D201" t="s">
-        <v>361</v>
+        <v>360</v>
       </c>
       <c r="E201">
         <v>1</v>
@@ -5615,16 +5589,16 @@
     </row>
     <row r="202" spans="1:5">
       <c r="A202" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B202" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C202" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="D202" t="s">
-        <v>362</v>
+        <v>361</v>
       </c>
       <c r="E202">
         <v>1</v>
@@ -5632,16 +5606,16 @@
     </row>
     <row r="203" spans="1:5">
       <c r="A203" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B203" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C203" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="D203" t="s">
-        <v>363</v>
+        <v>362</v>
       </c>
       <c r="E203">
         <v>1</v>
@@ -5649,16 +5623,16 @@
     </row>
     <row r="204" spans="1:5">
       <c r="A204" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B204" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C204" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="D204" t="s">
-        <v>364</v>
+        <v>363</v>
       </c>
       <c r="E204">
         <v>1</v>
@@ -5666,16 +5640,16 @@
     </row>
     <row r="205" spans="1:5">
       <c r="A205" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B205" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C205" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="D205" t="s">
-        <v>365</v>
+        <v>364</v>
       </c>
       <c r="E205">
         <v>1</v>
@@ -5683,16 +5657,16 @@
     </row>
     <row r="206" spans="1:5">
       <c r="A206" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B206" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C206" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="D206" t="s">
-        <v>366</v>
+        <v>365</v>
       </c>
       <c r="E206">
         <v>1</v>
@@ -5700,33 +5674,33 @@
     </row>
     <row r="207" spans="1:5">
       <c r="A207" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B207" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C207" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="D207" t="s">
-        <v>367</v>
+        <v>366</v>
       </c>
       <c r="E207">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="208" spans="1:5">
       <c r="A208" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B208" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C208" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="D208" t="s">
-        <v>368</v>
+        <v>367</v>
       </c>
       <c r="E208">
         <v>2</v>
@@ -5734,16 +5708,16 @@
     </row>
     <row r="209" spans="1:5">
       <c r="A209" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B209" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C209" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
       <c r="D209" t="s">
-        <v>369</v>
+        <v>368</v>
       </c>
       <c r="E209">
         <v>2</v>
@@ -5751,16 +5725,16 @@
     </row>
     <row r="210" spans="1:5">
       <c r="A210" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B210" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C210" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
       <c r="D210" t="s">
-        <v>370</v>
+        <v>369</v>
       </c>
       <c r="E210">
         <v>2</v>
@@ -5768,16 +5742,16 @@
     </row>
     <row r="211" spans="1:5">
       <c r="A211" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B211" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C211" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="D211" t="s">
-        <v>371</v>
+        <v>370</v>
       </c>
       <c r="E211">
         <v>2</v>
@@ -5785,16 +5759,16 @@
     </row>
     <row r="212" spans="1:5">
       <c r="A212" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B212" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C212" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
       <c r="D212" t="s">
-        <v>372</v>
+        <v>371</v>
       </c>
       <c r="E212">
         <v>2</v>
@@ -5802,16 +5776,16 @@
     </row>
     <row r="213" spans="1:5">
       <c r="A213" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B213" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C213" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
       <c r="D213" t="s">
-        <v>373</v>
+        <v>372</v>
       </c>
       <c r="E213">
         <v>2</v>
@@ -5819,16 +5793,16 @@
     </row>
     <row r="214" spans="1:5">
       <c r="A214" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B214" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C214" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
       <c r="D214" t="s">
-        <v>374</v>
+        <v>373</v>
       </c>
       <c r="E214">
         <v>2</v>
@@ -5836,13 +5810,13 @@
     </row>
     <row r="215" spans="1:5">
       <c r="A215" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B215" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C215" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="D215" t="s">
         <v>374</v>
@@ -5853,16 +5827,16 @@
     </row>
     <row r="216" spans="1:5">
       <c r="A216" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B216" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C216" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="D216" t="s">
-        <v>375</v>
+        <v>374</v>
       </c>
       <c r="E216">
         <v>2</v>
@@ -5870,16 +5844,16 @@
     </row>
     <row r="217" spans="1:5">
       <c r="A217" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B217" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C217" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="D217" t="s">
-        <v>376</v>
+        <v>375</v>
       </c>
       <c r="E217">
         <v>2</v>
@@ -5887,16 +5861,16 @@
     </row>
     <row r="218" spans="1:5">
       <c r="A218" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B218" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C218" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
       <c r="D218" t="s">
-        <v>377</v>
+        <v>376</v>
       </c>
       <c r="E218">
         <v>2</v>
@@ -5904,33 +5878,33 @@
     </row>
     <row r="219" spans="1:5">
       <c r="A219" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B219" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C219" t="s">
-        <v>212</v>
+        <v>211</v>
       </c>
       <c r="D219" t="s">
-        <v>378</v>
+        <v>377</v>
       </c>
       <c r="E219">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="220" spans="1:5">
       <c r="A220" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B220" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C220" t="s">
-        <v>213</v>
+        <v>212</v>
       </c>
       <c r="D220" t="s">
-        <v>265</v>
+        <v>378</v>
       </c>
       <c r="E220">
         <v>3</v>
@@ -5938,33 +5912,33 @@
     </row>
     <row r="221" spans="1:5">
       <c r="A221" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B221" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C221" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
       <c r="D221" t="s">
-        <v>379</v>
+        <v>265</v>
       </c>
       <c r="E221">
-        <v>4</v>
+        <v>3</v>
       </c>
     </row>
     <row r="222" spans="1:5">
       <c r="A222" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B222" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C222" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
       <c r="D222" t="s">
-        <v>380</v>
+        <v>379</v>
       </c>
       <c r="E222">
         <v>4</v>
@@ -5972,16 +5946,16 @@
     </row>
     <row r="223" spans="1:5">
       <c r="A223" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B223" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C223" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
       <c r="D223" t="s">
-        <v>381</v>
+        <v>380</v>
       </c>
       <c r="E223">
         <v>4</v>
@@ -5989,16 +5963,16 @@
     </row>
     <row r="224" spans="1:5">
       <c r="A224" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B224" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C224" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
       <c r="D224" t="s">
-        <v>382</v>
+        <v>381</v>
       </c>
       <c r="E224">
         <v>4</v>
@@ -6006,16 +5980,16 @@
     </row>
     <row r="225" spans="1:5">
       <c r="A225" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B225" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C225" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
       <c r="D225" t="s">
-        <v>383</v>
+        <v>382</v>
       </c>
       <c r="E225">
         <v>4</v>
@@ -6023,33 +5997,33 @@
     </row>
     <row r="226" spans="1:5">
       <c r="A226" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B226" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C226" t="s">
-        <v>219</v>
+        <v>218</v>
       </c>
       <c r="D226" t="s">
-        <v>384</v>
+        <v>383</v>
       </c>
       <c r="E226">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="227" spans="1:5">
       <c r="A227" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B227" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C227" t="s">
-        <v>220</v>
+        <v>219</v>
       </c>
       <c r="D227" t="s">
-        <v>385</v>
+        <v>384</v>
       </c>
       <c r="E227">
         <v>5</v>
@@ -6057,64 +6031,64 @@
     </row>
     <row r="228" spans="1:5">
       <c r="A228" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B228" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C228" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
       <c r="D228" t="s">
-        <v>386</v>
+        <v>385</v>
       </c>
       <c r="E228">
-        <v>6</v>
+        <v>5</v>
       </c>
     </row>
     <row r="229" spans="1:5">
       <c r="A229" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B229" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C229" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
       <c r="D229" t="s">
-        <v>387</v>
+        <v>386</v>
       </c>
       <c r="E229">
-        <v>8</v>
+        <v>6</v>
       </c>
     </row>
     <row r="230" spans="1:5">
       <c r="A230" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B230" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C230" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
       <c r="D230" t="s">
-        <v>388</v>
+        <v>387</v>
       </c>
       <c r="E230">
-        <v>10</v>
+        <v>8</v>
       </c>
     </row>
     <row r="231" spans="1:5">
       <c r="A231" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B231" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C231" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="D231" t="s">
         <v>388</v>
@@ -6125,33 +6099,33 @@
     </row>
     <row r="232" spans="1:5">
       <c r="A232" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B232" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C232" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
       <c r="D232" t="s">
-        <v>267</v>
+        <v>388</v>
       </c>
       <c r="E232">
-        <v>12</v>
+        <v>10</v>
       </c>
     </row>
     <row r="233" spans="1:5">
       <c r="A233" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B233" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C233" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
       <c r="D233" t="s">
-        <v>389</v>
+        <v>267</v>
       </c>
       <c r="E233">
         <v>12</v>
@@ -6159,84 +6133,84 @@
     </row>
     <row r="234" spans="1:5">
       <c r="A234" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B234" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C234" t="s">
-        <v>227</v>
+        <v>226</v>
       </c>
       <c r="D234" t="s">
-        <v>390</v>
+        <v>389</v>
       </c>
       <c r="E234">
-        <v>14</v>
+        <v>12</v>
       </c>
     </row>
     <row r="235" spans="1:5">
       <c r="A235" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B235" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C235" t="s">
-        <v>228</v>
+        <v>227</v>
       </c>
       <c r="D235" t="s">
-        <v>391</v>
+        <v>390</v>
       </c>
       <c r="E235">
-        <v>15</v>
+        <v>14</v>
       </c>
     </row>
     <row r="236" spans="1:5">
       <c r="A236" t="s">
+        <v>14</v>
+      </c>
+      <c r="B236" t="s">
+        <v>40</v>
+      </c>
+      <c r="C236" t="s">
+        <v>228</v>
+      </c>
+      <c r="D236" t="s">
+        <v>391</v>
+      </c>
+      <c r="E236">
         <v>15</v>
-      </c>
-      <c r="B236" t="s">
-        <v>41</v>
-      </c>
-      <c r="C236" t="s">
-        <v>229</v>
-      </c>
-      <c r="D236" t="s">
-        <v>392</v>
-      </c>
-      <c r="E236">
-        <v>20</v>
       </c>
     </row>
     <row r="237" spans="1:5">
       <c r="A237" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="B237" t="s">
         <v>40</v>
       </c>
       <c r="C237" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="D237" t="s">
-        <v>393</v>
+        <v>392</v>
       </c>
       <c r="E237">
-        <v>1</v>
+        <v>20</v>
       </c>
     </row>
     <row r="238" spans="1:5">
       <c r="A238" t="s">
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="B238" t="s">
-        <v>36</v>
+        <v>39</v>
       </c>
       <c r="C238" t="s">
-        <v>231</v>
+        <v>230</v>
       </c>
       <c r="D238" t="s">
-        <v>394</v>
+        <v>393</v>
       </c>
       <c r="E238">
         <v>1</v>
@@ -6244,16 +6218,16 @@
     </row>
     <row r="239" spans="1:5">
       <c r="A239" t="s">
-        <v>16</v>
+        <v>6</v>
       </c>
       <c r="B239" t="s">
-        <v>42</v>
+        <v>36</v>
       </c>
       <c r="C239" t="s">
-        <v>232</v>
+        <v>231</v>
       </c>
       <c r="D239" t="s">
-        <v>395</v>
+        <v>394</v>
       </c>
       <c r="E239">
         <v>1</v>
@@ -6261,18 +6235,35 @@
     </row>
     <row r="240" spans="1:5">
       <c r="A240" t="s">
-        <v>11</v>
+        <v>15</v>
       </c>
       <c r="B240" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="C240" t="s">
+        <v>232</v>
+      </c>
+      <c r="D240" t="s">
+        <v>395</v>
+      </c>
+      <c r="E240">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="241" spans="1:5">
+      <c r="A241" t="s">
+        <v>10</v>
+      </c>
+      <c r="B241" t="s">
+        <v>39</v>
+      </c>
+      <c r="C241" t="s">
         <v>233</v>
       </c>
-      <c r="D240" t="s">
+      <c r="D241" t="s">
         <v>396</v>
       </c>
-      <c r="E240">
+      <c r="E241">
         <v>1</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualização automática: rac (17/09/2026 12:57)
</commit_message>
<xml_diff>
--- a/Coordenadoria/02_Dados_Tratados/base_rac_tratada.xlsx
+++ b/Coordenadoria/02_Dados_Tratados/base_rac_tratada.xlsx
@@ -1212,8 +1212,16 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <fonts count="1">
+  <fonts count="2">
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -1229,7 +1237,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -1237,12 +1245,30 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1541,22 +1567,22 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:6">
-      <c r="A1" t="s">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" t="s">
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" t="s">
+      <c r="F1" s="1" t="s">
         <v>5</v>
       </c>
     </row>
@@ -2171,19 +2197,19 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:5">
-      <c r="A1" t="s">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" t="s">
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
         <v>55</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>56</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="1" t="s">
         <v>57</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualização automática: rac (18/09/2026 11:55)
</commit_message>
<xml_diff>
--- a/Coordenadoria/02_Dados_Tratados/base_rac_tratada.xlsx
+++ b/Coordenadoria/02_Dados_Tratados/base_rac_tratada.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1091" uniqueCount="397">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1079" uniqueCount="395">
   <si>
     <t>matricula</t>
   </si>
@@ -65,6 +65,9 @@
     <t>2702</t>
   </si>
   <si>
+    <t>2741</t>
+  </si>
+  <si>
     <t>2703</t>
   </si>
   <si>
@@ -107,9 +110,6 @@
     <t>2740</t>
   </si>
   <si>
-    <t>2741</t>
-  </si>
-  <si>
     <t>2742</t>
   </si>
   <si>
@@ -143,6 +143,9 @@
     <t>EPCAR</t>
   </si>
   <si>
+    <t>BABV</t>
+  </si>
+  <si>
     <t>PAMALS</t>
   </si>
   <si>
@@ -158,9 +161,6 @@
     <t>BAPV</t>
   </si>
   <si>
-    <t>BABV</t>
-  </si>
-  <si>
     <t>DACTA2</t>
   </si>
   <si>
@@ -713,9 +713,6 @@
     <t>060-0017-00</t>
   </si>
   <si>
-    <t>S3309A0160-000D</t>
-  </si>
-  <si>
     <t>3034792</t>
   </si>
   <si>
@@ -1200,9 +1197,6 @@
   </si>
   <si>
     <t>FLIGHT DIR HOR</t>
-  </si>
-  <si>
-    <t>HOSE AY</t>
   </si>
   <si>
     <t>FUEL PUMP</t>
@@ -1212,16 +1206,8 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <fonts count="2">
+  <fonts count="1">
     <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -1237,7 +1223,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -1245,30 +1231,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color auto="1"/>
-      </left>
-      <right style="thin">
-        <color auto="1"/>
-      </right>
-      <top style="thin">
-        <color auto="1"/>
-      </top>
-      <bottom style="thin">
-        <color auto="1"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1567,22 +1535,22 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:6">
-      <c r="A1" s="1" t="s">
+      <c r="A1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" s="1" t="s">
+      <c r="B1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" t="s">
         <v>5</v>
       </c>
     </row>
@@ -1680,10 +1648,10 @@
         <v>54</v>
       </c>
       <c r="E6">
-        <v>9</v>
+        <v>6</v>
       </c>
       <c r="F6">
-        <v>10</v>
+        <v>7</v>
       </c>
     </row>
     <row r="7" spans="1:6">
@@ -1780,10 +1748,10 @@
         <v>53</v>
       </c>
       <c r="E11">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F11">
-        <v>4</v>
+        <v>3</v>
       </c>
     </row>
     <row r="12" spans="1:6">
@@ -1791,19 +1759,19 @@
         <v>16</v>
       </c>
       <c r="B12" t="s">
-        <v>36</v>
+        <v>42</v>
       </c>
       <c r="C12" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="D12" t="s">
         <v>53</v>
       </c>
       <c r="E12">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F12">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="13" spans="1:6">
@@ -1811,7 +1779,7 @@
         <v>17</v>
       </c>
       <c r="B13" t="s">
-        <v>42</v>
+        <v>36</v>
       </c>
       <c r="C13" t="s">
         <v>51</v>
@@ -1831,7 +1799,7 @@
         <v>18</v>
       </c>
       <c r="B14" t="s">
-        <v>36</v>
+        <v>43</v>
       </c>
       <c r="C14" t="s">
         <v>51</v>
@@ -1851,7 +1819,7 @@
         <v>19</v>
       </c>
       <c r="B15" t="s">
-        <v>43</v>
+        <v>36</v>
       </c>
       <c r="C15" t="s">
         <v>51</v>
@@ -1871,7 +1839,7 @@
         <v>20</v>
       </c>
       <c r="B16" t="s">
-        <v>38</v>
+        <v>44</v>
       </c>
       <c r="C16" t="s">
         <v>51</v>
@@ -1891,7 +1859,7 @@
         <v>21</v>
       </c>
       <c r="B17" t="s">
-        <v>43</v>
+        <v>38</v>
       </c>
       <c r="C17" t="s">
         <v>51</v>
@@ -1931,7 +1899,7 @@
         <v>23</v>
       </c>
       <c r="B19" t="s">
-        <v>40</v>
+        <v>45</v>
       </c>
       <c r="C19" t="s">
         <v>51</v>
@@ -1951,7 +1919,7 @@
         <v>24</v>
       </c>
       <c r="B20" t="s">
-        <v>45</v>
+        <v>40</v>
       </c>
       <c r="C20" t="s">
         <v>51</v>
@@ -1971,7 +1939,7 @@
         <v>25</v>
       </c>
       <c r="B21" t="s">
-        <v>39</v>
+        <v>46</v>
       </c>
       <c r="C21" t="s">
         <v>51</v>
@@ -2011,7 +1979,7 @@
         <v>27</v>
       </c>
       <c r="B23" t="s">
-        <v>46</v>
+        <v>39</v>
       </c>
       <c r="C23" t="s">
         <v>51</v>
@@ -2031,7 +1999,7 @@
         <v>28</v>
       </c>
       <c r="B24" t="s">
-        <v>40</v>
+        <v>47</v>
       </c>
       <c r="C24" t="s">
         <v>51</v>
@@ -2051,7 +2019,7 @@
         <v>29</v>
       </c>
       <c r="B25" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="C25" t="s">
         <v>51</v>
@@ -2071,7 +2039,7 @@
         <v>30</v>
       </c>
       <c r="B26" t="s">
-        <v>47</v>
+        <v>39</v>
       </c>
       <c r="C26" t="s">
         <v>51</v>
@@ -2131,7 +2099,7 @@
         <v>33</v>
       </c>
       <c r="B29" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="C29" t="s">
         <v>52</v>
@@ -2151,7 +2119,7 @@
         <v>34</v>
       </c>
       <c r="B30" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="C30" t="s">
         <v>52</v>
@@ -2171,7 +2139,7 @@
         <v>35</v>
       </c>
       <c r="B31" t="s">
-        <v>47</v>
+        <v>42</v>
       </c>
       <c r="C31" t="s">
         <v>52</v>
@@ -2193,23 +2161,23 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E241"/>
+  <dimension ref="A1:E238"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:5">
-      <c r="A1" s="1" t="s">
+      <c r="A1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" s="1" t="s">
+      <c r="B1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" t="s">
         <v>55</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" t="s">
         <v>56</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" t="s">
         <v>57</v>
       </c>
     </row>
@@ -2224,7 +2192,7 @@
         <v>58</v>
       </c>
       <c r="D2" t="s">
-        <v>234</v>
+        <v>233</v>
       </c>
       <c r="E2">
         <v>1</v>
@@ -2241,7 +2209,7 @@
         <v>59</v>
       </c>
       <c r="D3" t="s">
-        <v>235</v>
+        <v>234</v>
       </c>
       <c r="E3">
         <v>1</v>
@@ -2258,7 +2226,7 @@
         <v>60</v>
       </c>
       <c r="D4" t="s">
-        <v>236</v>
+        <v>235</v>
       </c>
       <c r="E4">
         <v>1</v>
@@ -2275,7 +2243,7 @@
         <v>61</v>
       </c>
       <c r="D5" t="s">
-        <v>237</v>
+        <v>236</v>
       </c>
       <c r="E5">
         <v>1</v>
@@ -2292,7 +2260,7 @@
         <v>62</v>
       </c>
       <c r="D6" t="s">
-        <v>238</v>
+        <v>237</v>
       </c>
       <c r="E6">
         <v>1</v>
@@ -2309,7 +2277,7 @@
         <v>63</v>
       </c>
       <c r="D7" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
       <c r="E7">
         <v>1</v>
@@ -2326,7 +2294,7 @@
         <v>63</v>
       </c>
       <c r="D8" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
       <c r="E8">
         <v>1</v>
@@ -2343,7 +2311,7 @@
         <v>63</v>
       </c>
       <c r="D9" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
       <c r="E9">
         <v>1</v>
@@ -2360,7 +2328,7 @@
         <v>63</v>
       </c>
       <c r="D10" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
       <c r="E10">
         <v>1</v>
@@ -2377,7 +2345,7 @@
         <v>63</v>
       </c>
       <c r="D11" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
       <c r="E11">
         <v>1</v>
@@ -2394,7 +2362,7 @@
         <v>63</v>
       </c>
       <c r="D12" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
       <c r="E12">
         <v>1</v>
@@ -2411,7 +2379,7 @@
         <v>63</v>
       </c>
       <c r="D13" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
       <c r="E13">
         <v>1</v>
@@ -2428,7 +2396,7 @@
         <v>63</v>
       </c>
       <c r="D14" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
       <c r="E14">
         <v>1</v>
@@ -2445,7 +2413,7 @@
         <v>64</v>
       </c>
       <c r="D15" t="s">
-        <v>240</v>
+        <v>239</v>
       </c>
       <c r="E15">
         <v>1</v>
@@ -2462,7 +2430,7 @@
         <v>64</v>
       </c>
       <c r="D16" t="s">
-        <v>240</v>
+        <v>239</v>
       </c>
       <c r="E16">
         <v>2</v>
@@ -2479,7 +2447,7 @@
         <v>65</v>
       </c>
       <c r="D17" t="s">
-        <v>241</v>
+        <v>240</v>
       </c>
       <c r="E17">
         <v>1</v>
@@ -2496,7 +2464,7 @@
         <v>65</v>
       </c>
       <c r="D18" t="s">
-        <v>241</v>
+        <v>240</v>
       </c>
       <c r="E18">
         <v>1</v>
@@ -2513,7 +2481,7 @@
         <v>65</v>
       </c>
       <c r="D19" t="s">
-        <v>241</v>
+        <v>240</v>
       </c>
       <c r="E19">
         <v>1</v>
@@ -2530,7 +2498,7 @@
         <v>65</v>
       </c>
       <c r="D20" t="s">
-        <v>241</v>
+        <v>240</v>
       </c>
       <c r="E20">
         <v>1</v>
@@ -2547,7 +2515,7 @@
         <v>65</v>
       </c>
       <c r="D21" t="s">
-        <v>241</v>
+        <v>240</v>
       </c>
       <c r="E21">
         <v>1</v>
@@ -2564,7 +2532,7 @@
         <v>65</v>
       </c>
       <c r="D22" t="s">
-        <v>241</v>
+        <v>240</v>
       </c>
       <c r="E22">
         <v>1</v>
@@ -2572,7 +2540,7 @@
     </row>
     <row r="23" spans="1:5">
       <c r="A23" t="s">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="B23" t="s">
         <v>39</v>
@@ -2581,7 +2549,7 @@
         <v>66</v>
       </c>
       <c r="D23" t="s">
-        <v>242</v>
+        <v>241</v>
       </c>
       <c r="E23">
         <v>1</v>
@@ -2589,7 +2557,7 @@
     </row>
     <row r="24" spans="1:5">
       <c r="A24" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="B24" t="s">
         <v>39</v>
@@ -2598,7 +2566,7 @@
         <v>66</v>
       </c>
       <c r="D24" t="s">
-        <v>242</v>
+        <v>241</v>
       </c>
       <c r="E24">
         <v>1</v>
@@ -2606,13 +2574,13 @@
     </row>
     <row r="25" spans="1:5">
       <c r="A25" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B25" t="s">
         <v>39</v>
       </c>
       <c r="C25" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="D25" t="s">
         <v>242</v>
@@ -2623,7 +2591,7 @@
     </row>
     <row r="26" spans="1:5">
       <c r="A26" t="s">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="B26" t="s">
         <v>39</v>
@@ -2632,7 +2600,7 @@
         <v>67</v>
       </c>
       <c r="D26" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
       <c r="E26">
         <v>1</v>
@@ -2640,13 +2608,13 @@
     </row>
     <row r="27" spans="1:5">
       <c r="A27" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="B27" t="s">
         <v>39</v>
       </c>
       <c r="C27" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="D27" t="s">
         <v>243</v>
@@ -2663,7 +2631,7 @@
         <v>39</v>
       </c>
       <c r="C28" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="D28" t="s">
         <v>243</v>
@@ -2674,16 +2642,16 @@
     </row>
     <row r="29" spans="1:5">
       <c r="A29" t="s">
-        <v>10</v>
+        <v>16</v>
       </c>
       <c r="B29" t="s">
-        <v>39</v>
+        <v>42</v>
       </c>
       <c r="C29" t="s">
         <v>68</v>
       </c>
       <c r="D29" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="E29">
         <v>1</v>
@@ -2697,7 +2665,7 @@
         <v>39</v>
       </c>
       <c r="C30" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="D30" t="s">
         <v>244</v>
@@ -2714,35 +2682,35 @@
         <v>39</v>
       </c>
       <c r="C31" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="D31" t="s">
         <v>245</v>
       </c>
       <c r="E31">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="32" spans="1:5">
       <c r="A32" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B32" t="s">
         <v>39</v>
       </c>
       <c r="C32" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="D32" t="s">
         <v>245</v>
       </c>
       <c r="E32">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="33" spans="1:5">
       <c r="A33" t="s">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="B33" t="s">
         <v>39</v>
@@ -2751,7 +2719,7 @@
         <v>70</v>
       </c>
       <c r="D33" t="s">
-        <v>246</v>
+        <v>245</v>
       </c>
       <c r="E33">
         <v>2</v>
@@ -2759,50 +2727,50 @@
     </row>
     <row r="34" spans="1:5">
       <c r="A34" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B34" t="s">
-        <v>39</v>
+        <v>36</v>
       </c>
       <c r="C34" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="D34" t="s">
         <v>246</v>
       </c>
       <c r="E34">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="35" spans="1:5">
       <c r="A35" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B35" t="s">
         <v>39</v>
       </c>
       <c r="C35" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="D35" t="s">
         <v>246</v>
       </c>
       <c r="E35">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="36" spans="1:5">
       <c r="A36" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="B36" t="s">
-        <v>36</v>
+        <v>39</v>
       </c>
       <c r="C36" t="s">
         <v>71</v>
       </c>
       <c r="D36" t="s">
-        <v>247</v>
+        <v>246</v>
       </c>
       <c r="E36">
         <v>1</v>
@@ -2810,13 +2778,13 @@
     </row>
     <row r="37" spans="1:5">
       <c r="A37" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B37" t="s">
-        <v>39</v>
+        <v>36</v>
       </c>
       <c r="C37" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="D37" t="s">
         <v>247</v>
@@ -2827,13 +2795,13 @@
     </row>
     <row r="38" spans="1:5">
       <c r="A38" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B38" t="s">
         <v>39</v>
       </c>
       <c r="C38" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="D38" t="s">
         <v>247</v>
@@ -2844,16 +2812,16 @@
     </row>
     <row r="39" spans="1:5">
       <c r="A39" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="B39" t="s">
-        <v>36</v>
+        <v>39</v>
       </c>
       <c r="C39" t="s">
         <v>72</v>
       </c>
       <c r="D39" t="s">
-        <v>248</v>
+        <v>247</v>
       </c>
       <c r="E39">
         <v>1</v>
@@ -2861,13 +2829,13 @@
     </row>
     <row r="40" spans="1:5">
       <c r="A40" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B40" t="s">
-        <v>39</v>
+        <v>36</v>
       </c>
       <c r="C40" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="D40" t="s">
         <v>248</v>
@@ -2878,13 +2846,13 @@
     </row>
     <row r="41" spans="1:5">
       <c r="A41" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B41" t="s">
         <v>39</v>
       </c>
       <c r="C41" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="D41" t="s">
         <v>248</v>
@@ -2901,7 +2869,7 @@
         <v>36</v>
       </c>
       <c r="C42" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="D42" t="s">
         <v>249</v>
@@ -2912,13 +2880,13 @@
     </row>
     <row r="43" spans="1:5">
       <c r="A43" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="B43" t="s">
         <v>39</v>
       </c>
       <c r="C43" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="D43" t="s">
         <v>249</v>
@@ -2929,16 +2897,16 @@
     </row>
     <row r="44" spans="1:5">
       <c r="A44" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="B44" t="s">
-        <v>36</v>
+        <v>40</v>
       </c>
       <c r="C44" t="s">
         <v>74</v>
       </c>
       <c r="D44" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
       <c r="E44">
         <v>1</v>
@@ -2946,13 +2914,13 @@
     </row>
     <row r="45" spans="1:5">
       <c r="A45" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="B45" t="s">
-        <v>39</v>
+        <v>36</v>
       </c>
       <c r="C45" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="D45" t="s">
         <v>250</v>
@@ -2963,16 +2931,16 @@
     </row>
     <row r="46" spans="1:5">
       <c r="A46" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="B46" t="s">
-        <v>40</v>
+        <v>36</v>
       </c>
       <c r="C46" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="D46" t="s">
-        <v>250</v>
+        <v>251</v>
       </c>
       <c r="E46">
         <v>1</v>
@@ -2986,10 +2954,10 @@
         <v>36</v>
       </c>
       <c r="C47" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="D47" t="s">
-        <v>251</v>
+        <v>252</v>
       </c>
       <c r="E47">
         <v>1</v>
@@ -3003,10 +2971,10 @@
         <v>36</v>
       </c>
       <c r="C48" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="D48" t="s">
-        <v>252</v>
+        <v>253</v>
       </c>
       <c r="E48">
         <v>1</v>
@@ -3020,10 +2988,10 @@
         <v>36</v>
       </c>
       <c r="C49" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="D49" t="s">
-        <v>253</v>
+        <v>254</v>
       </c>
       <c r="E49">
         <v>1</v>
@@ -3037,10 +3005,10 @@
         <v>36</v>
       </c>
       <c r="C50" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="D50" t="s">
-        <v>254</v>
+        <v>255</v>
       </c>
       <c r="E50">
         <v>1</v>
@@ -3054,10 +3022,10 @@
         <v>36</v>
       </c>
       <c r="C51" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="D51" t="s">
-        <v>255</v>
+        <v>256</v>
       </c>
       <c r="E51">
         <v>1</v>
@@ -3071,10 +3039,10 @@
         <v>36</v>
       </c>
       <c r="C52" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="D52" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
       <c r="E52">
         <v>1</v>
@@ -3088,44 +3056,44 @@
         <v>36</v>
       </c>
       <c r="C53" t="s">
-        <v>81</v>
+        <v>83</v>
       </c>
       <c r="D53" t="s">
-        <v>257</v>
+        <v>258</v>
       </c>
       <c r="E53">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="54" spans="1:5">
       <c r="A54" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B54" t="s">
-        <v>36</v>
+        <v>39</v>
       </c>
       <c r="C54" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="D54" t="s">
         <v>258</v>
       </c>
       <c r="E54">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="55" spans="1:5">
       <c r="A55" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="B55" t="s">
-        <v>36</v>
+        <v>39</v>
       </c>
       <c r="C55" t="s">
         <v>83</v>
       </c>
       <c r="D55" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="E55">
         <v>2</v>
@@ -3133,30 +3101,30 @@
     </row>
     <row r="56" spans="1:5">
       <c r="A56" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="B56" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="C56" t="s">
         <v>83</v>
       </c>
       <c r="D56" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="E56">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="57" spans="1:5">
       <c r="A57" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="B57" t="s">
-        <v>39</v>
+        <v>36</v>
       </c>
       <c r="C57" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="D57" t="s">
         <v>259</v>
@@ -3167,13 +3135,13 @@
     </row>
     <row r="58" spans="1:5">
       <c r="A58" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B58" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="C58" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="D58" t="s">
         <v>259</v>
@@ -3184,30 +3152,30 @@
     </row>
     <row r="59" spans="1:5">
       <c r="A59" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="B59" t="s">
-        <v>36</v>
+        <v>40</v>
       </c>
       <c r="C59" t="s">
         <v>84</v>
       </c>
       <c r="D59" t="s">
-        <v>260</v>
+        <v>259</v>
       </c>
       <c r="E59">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="60" spans="1:5">
       <c r="A60" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="B60" t="s">
-        <v>39</v>
+        <v>36</v>
       </c>
       <c r="C60" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="D60" t="s">
         <v>260</v>
@@ -3218,33 +3186,33 @@
     </row>
     <row r="61" spans="1:5">
       <c r="A61" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B61" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="C61" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="D61" t="s">
         <v>260</v>
       </c>
       <c r="E61">
-        <v>1</v>
+        <v>4</v>
       </c>
     </row>
     <row r="62" spans="1:5">
       <c r="A62" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="B62" t="s">
-        <v>36</v>
+        <v>40</v>
       </c>
       <c r="C62" t="s">
         <v>85</v>
       </c>
       <c r="D62" t="s">
-        <v>261</v>
+        <v>260</v>
       </c>
       <c r="E62">
         <v>2</v>
@@ -3252,19 +3220,19 @@
     </row>
     <row r="63" spans="1:5">
       <c r="A63" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="B63" t="s">
-        <v>39</v>
+        <v>36</v>
       </c>
       <c r="C63" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="D63" t="s">
         <v>261</v>
       </c>
       <c r="E63">
-        <v>4</v>
+        <v>2</v>
       </c>
     </row>
     <row r="64" spans="1:5">
@@ -3275,13 +3243,13 @@
         <v>40</v>
       </c>
       <c r="C64" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="D64" t="s">
         <v>261</v>
       </c>
       <c r="E64">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="65" spans="1:5">
@@ -3292,7 +3260,7 @@
         <v>36</v>
       </c>
       <c r="C65" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="D65" t="s">
         <v>262</v>
@@ -3303,19 +3271,19 @@
     </row>
     <row r="66" spans="1:5">
       <c r="A66" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="B66" t="s">
-        <v>40</v>
+        <v>36</v>
       </c>
       <c r="C66" t="s">
-        <v>86</v>
+        <v>88</v>
       </c>
       <c r="D66" t="s">
-        <v>262</v>
+        <v>263</v>
       </c>
       <c r="E66">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="67" spans="1:5">
@@ -3326,10 +3294,10 @@
         <v>36</v>
       </c>
       <c r="C67" t="s">
-        <v>87</v>
+        <v>89</v>
       </c>
       <c r="D67" t="s">
-        <v>263</v>
+        <v>264</v>
       </c>
       <c r="E67">
         <v>2</v>
@@ -3343,10 +3311,10 @@
         <v>36</v>
       </c>
       <c r="C68" t="s">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="D68" t="s">
-        <v>264</v>
+        <v>265</v>
       </c>
       <c r="E68">
         <v>2</v>
@@ -3360,10 +3328,10 @@
         <v>36</v>
       </c>
       <c r="C69" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="D69" t="s">
-        <v>265</v>
+        <v>266</v>
       </c>
       <c r="E69">
         <v>2</v>
@@ -3377,10 +3345,10 @@
         <v>36</v>
       </c>
       <c r="C70" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="D70" t="s">
-        <v>266</v>
+        <v>267</v>
       </c>
       <c r="E70">
         <v>2</v>
@@ -3394,10 +3362,10 @@
         <v>36</v>
       </c>
       <c r="C71" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="D71" t="s">
-        <v>267</v>
+        <v>268</v>
       </c>
       <c r="E71">
         <v>2</v>
@@ -3411,10 +3379,10 @@
         <v>36</v>
       </c>
       <c r="C72" t="s">
-        <v>92</v>
+        <v>94</v>
       </c>
       <c r="D72" t="s">
-        <v>268</v>
+        <v>258</v>
       </c>
       <c r="E72">
         <v>2</v>
@@ -3428,30 +3396,30 @@
         <v>36</v>
       </c>
       <c r="C73" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="D73" t="s">
-        <v>269</v>
+        <v>257</v>
       </c>
       <c r="E73">
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
     <row r="74" spans="1:5">
       <c r="A74" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="B74" t="s">
-        <v>36</v>
+        <v>40</v>
       </c>
       <c r="C74" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="D74" t="s">
-        <v>259</v>
+        <v>257</v>
       </c>
       <c r="E74">
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
     <row r="75" spans="1:5">
@@ -3462,10 +3430,10 @@
         <v>36</v>
       </c>
       <c r="C75" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="D75" t="s">
-        <v>258</v>
+        <v>269</v>
       </c>
       <c r="E75">
         <v>4</v>
@@ -3473,16 +3441,16 @@
     </row>
     <row r="76" spans="1:5">
       <c r="A76" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="B76" t="s">
-        <v>40</v>
+        <v>36</v>
       </c>
       <c r="C76" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="D76" t="s">
-        <v>258</v>
+        <v>270</v>
       </c>
       <c r="E76">
         <v>4</v>
@@ -3490,50 +3458,50 @@
     </row>
     <row r="77" spans="1:5">
       <c r="A77" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B77" t="s">
-        <v>36</v>
+        <v>39</v>
       </c>
       <c r="C77" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="D77" t="s">
-        <v>270</v>
+        <v>271</v>
       </c>
       <c r="E77">
-        <v>4</v>
+        <v>1</v>
       </c>
     </row>
     <row r="78" spans="1:5">
       <c r="A78" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="B78" t="s">
-        <v>36</v>
+        <v>39</v>
       </c>
       <c r="C78" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="D78" t="s">
         <v>271</v>
       </c>
       <c r="E78">
-        <v>4</v>
+        <v>1</v>
       </c>
     </row>
     <row r="79" spans="1:5">
       <c r="A79" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="B79" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="C79" t="s">
         <v>98</v>
       </c>
       <c r="D79" t="s">
-        <v>272</v>
+        <v>271</v>
       </c>
       <c r="E79">
         <v>1</v>
@@ -3541,13 +3509,13 @@
     </row>
     <row r="80" spans="1:5">
       <c r="A80" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B80" t="s">
         <v>39</v>
       </c>
       <c r="C80" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="D80" t="s">
         <v>272</v>
@@ -3558,13 +3526,13 @@
     </row>
     <row r="81" spans="1:5">
       <c r="A81" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B81" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="C81" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="D81" t="s">
         <v>272</v>
@@ -3575,30 +3543,30 @@
     </row>
     <row r="82" spans="1:5">
       <c r="A82" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="B82" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="C82" t="s">
         <v>99</v>
       </c>
       <c r="D82" t="s">
-        <v>273</v>
+        <v>272</v>
       </c>
       <c r="E82">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="83" spans="1:5">
       <c r="A83" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B83" t="s">
         <v>39</v>
       </c>
       <c r="C83" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="D83" t="s">
         <v>273</v>
@@ -3609,19 +3577,19 @@
     </row>
     <row r="84" spans="1:5">
       <c r="A84" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B84" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="C84" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="D84" t="s">
         <v>273</v>
       </c>
       <c r="E84">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="85" spans="1:5">
@@ -3632,7 +3600,7 @@
         <v>39</v>
       </c>
       <c r="C85" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="D85" t="s">
         <v>274</v>
@@ -3649,7 +3617,7 @@
         <v>39</v>
       </c>
       <c r="C86" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="D86" t="s">
         <v>274</v>
@@ -3666,7 +3634,7 @@
         <v>39</v>
       </c>
       <c r="C87" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="D87" t="s">
         <v>275</v>
@@ -3683,7 +3651,7 @@
         <v>39</v>
       </c>
       <c r="C88" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="D88" t="s">
         <v>275</v>
@@ -3700,7 +3668,7 @@
         <v>39</v>
       </c>
       <c r="C89" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="D89" t="s">
         <v>276</v>
@@ -3717,7 +3685,7 @@
         <v>39</v>
       </c>
       <c r="C90" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="D90" t="s">
         <v>276</v>
@@ -3734,7 +3702,7 @@
         <v>39</v>
       </c>
       <c r="C91" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="D91" t="s">
         <v>277</v>
@@ -3751,7 +3719,7 @@
         <v>39</v>
       </c>
       <c r="C92" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="D92" t="s">
         <v>277</v>
@@ -3768,7 +3736,7 @@
         <v>39</v>
       </c>
       <c r="C93" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="D93" t="s">
         <v>278</v>
@@ -3779,13 +3747,13 @@
     </row>
     <row r="94" spans="1:5">
       <c r="A94" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="B94" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="C94" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="D94" t="s">
         <v>278</v>
@@ -3802,7 +3770,7 @@
         <v>39</v>
       </c>
       <c r="C95" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="D95" t="s">
         <v>279</v>
@@ -3819,7 +3787,7 @@
         <v>40</v>
       </c>
       <c r="C96" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="D96" t="s">
         <v>279</v>
@@ -3836,7 +3804,7 @@
         <v>39</v>
       </c>
       <c r="C97" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="D97" t="s">
         <v>280</v>
@@ -3853,7 +3821,7 @@
         <v>40</v>
       </c>
       <c r="C98" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="D98" t="s">
         <v>280</v>
@@ -3870,7 +3838,7 @@
         <v>39</v>
       </c>
       <c r="C99" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="D99" t="s">
         <v>281</v>
@@ -3881,16 +3849,16 @@
     </row>
     <row r="100" spans="1:5">
       <c r="A100" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="B100" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="C100" t="s">
-        <v>107</v>
+        <v>109</v>
       </c>
       <c r="D100" t="s">
-        <v>281</v>
+        <v>282</v>
       </c>
       <c r="E100">
         <v>1</v>
@@ -3904,10 +3872,10 @@
         <v>39</v>
       </c>
       <c r="C101" t="s">
-        <v>108</v>
+        <v>110</v>
       </c>
       <c r="D101" t="s">
-        <v>282</v>
+        <v>283</v>
       </c>
       <c r="E101">
         <v>1</v>
@@ -3921,10 +3889,10 @@
         <v>39</v>
       </c>
       <c r="C102" t="s">
-        <v>109</v>
+        <v>111</v>
       </c>
       <c r="D102" t="s">
-        <v>283</v>
+        <v>284</v>
       </c>
       <c r="E102">
         <v>1</v>
@@ -3938,10 +3906,10 @@
         <v>39</v>
       </c>
       <c r="C103" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="D103" t="s">
-        <v>284</v>
+        <v>285</v>
       </c>
       <c r="E103">
         <v>1</v>
@@ -3955,10 +3923,10 @@
         <v>39</v>
       </c>
       <c r="C104" t="s">
-        <v>111</v>
+        <v>113</v>
       </c>
       <c r="D104" t="s">
-        <v>285</v>
+        <v>286</v>
       </c>
       <c r="E104">
         <v>1</v>
@@ -3972,24 +3940,24 @@
         <v>39</v>
       </c>
       <c r="C105" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
       <c r="D105" t="s">
-        <v>286</v>
+        <v>287</v>
       </c>
       <c r="E105">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="106" spans="1:5">
       <c r="A106" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="B106" t="s">
         <v>39</v>
       </c>
       <c r="C106" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="D106" t="s">
         <v>287</v>
@@ -4006,7 +3974,7 @@
         <v>39</v>
       </c>
       <c r="C107" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="D107" t="s">
         <v>288</v>
@@ -4023,27 +3991,27 @@
         <v>39</v>
       </c>
       <c r="C108" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="D108" t="s">
         <v>288</v>
       </c>
       <c r="E108">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="109" spans="1:5">
       <c r="A109" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="B109" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="C109" t="s">
         <v>115</v>
       </c>
       <c r="D109" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
       <c r="E109">
         <v>2</v>
@@ -4051,13 +4019,13 @@
     </row>
     <row r="110" spans="1:5">
       <c r="A110" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B110" t="s">
         <v>39</v>
       </c>
       <c r="C110" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="D110" t="s">
         <v>289</v>
@@ -4068,13 +4036,13 @@
     </row>
     <row r="111" spans="1:5">
       <c r="A111" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B111" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="C111" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="D111" t="s">
         <v>289</v>
@@ -4085,16 +4053,16 @@
     </row>
     <row r="112" spans="1:5">
       <c r="A112" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="B112" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="C112" t="s">
         <v>116</v>
       </c>
       <c r="D112" t="s">
-        <v>290</v>
+        <v>289</v>
       </c>
       <c r="E112">
         <v>2</v>
@@ -4102,13 +4070,13 @@
     </row>
     <row r="113" spans="1:5">
       <c r="A113" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B113" t="s">
         <v>39</v>
       </c>
       <c r="C113" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="D113" t="s">
         <v>290</v>
@@ -4119,13 +4087,13 @@
     </row>
     <row r="114" spans="1:5">
       <c r="A114" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B114" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="C114" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="D114" t="s">
         <v>290</v>
@@ -4142,10 +4110,10 @@
         <v>39</v>
       </c>
       <c r="C115" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="D115" t="s">
-        <v>291</v>
+        <v>272</v>
       </c>
       <c r="E115">
         <v>2</v>
@@ -4159,61 +4127,61 @@
         <v>39</v>
       </c>
       <c r="C116" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="D116" t="s">
-        <v>291</v>
+        <v>272</v>
       </c>
       <c r="E116">
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
     <row r="117" spans="1:5">
       <c r="A117" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="B117" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="C117" t="s">
         <v>118</v>
       </c>
       <c r="D117" t="s">
-        <v>273</v>
+        <v>272</v>
       </c>
       <c r="E117">
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
     <row r="118" spans="1:5">
       <c r="A118" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B118" t="s">
         <v>39</v>
       </c>
       <c r="C118" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="D118" t="s">
-        <v>273</v>
+        <v>291</v>
       </c>
       <c r="E118">
-        <v>4</v>
+        <v>2</v>
       </c>
     </row>
     <row r="119" spans="1:5">
       <c r="A119" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B119" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="C119" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="D119" t="s">
-        <v>273</v>
+        <v>291</v>
       </c>
       <c r="E119">
         <v>4</v>
@@ -4227,10 +4195,10 @@
         <v>39</v>
       </c>
       <c r="C120" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="D120" t="s">
-        <v>292</v>
+        <v>276</v>
       </c>
       <c r="E120">
         <v>2</v>
@@ -4238,19 +4206,19 @@
     </row>
     <row r="121" spans="1:5">
       <c r="A121" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B121" t="s">
         <v>39</v>
       </c>
       <c r="C121" t="s">
-        <v>119</v>
+        <v>121</v>
       </c>
       <c r="D121" t="s">
         <v>292</v>
       </c>
       <c r="E121">
-        <v>4</v>
+        <v>2</v>
       </c>
     </row>
     <row r="122" spans="1:5">
@@ -4261,10 +4229,10 @@
         <v>39</v>
       </c>
       <c r="C122" t="s">
-        <v>120</v>
+        <v>122</v>
       </c>
       <c r="D122" t="s">
-        <v>277</v>
+        <v>293</v>
       </c>
       <c r="E122">
         <v>2</v>
@@ -4278,30 +4246,30 @@
         <v>39</v>
       </c>
       <c r="C123" t="s">
-        <v>121</v>
+        <v>123</v>
       </c>
       <c r="D123" t="s">
-        <v>293</v>
+        <v>294</v>
       </c>
       <c r="E123">
-        <v>2</v>
+        <v>5</v>
       </c>
     </row>
     <row r="124" spans="1:5">
       <c r="A124" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="B124" t="s">
         <v>39</v>
       </c>
       <c r="C124" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="D124" t="s">
         <v>294</v>
       </c>
       <c r="E124">
-        <v>2</v>
+        <v>5</v>
       </c>
     </row>
     <row r="125" spans="1:5">
@@ -4312,30 +4280,30 @@
         <v>39</v>
       </c>
       <c r="C125" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="D125" t="s">
         <v>295</v>
       </c>
       <c r="E125">
-        <v>5</v>
+        <v>7</v>
       </c>
     </row>
     <row r="126" spans="1:5">
       <c r="A126" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B126" t="s">
         <v>39</v>
       </c>
       <c r="C126" t="s">
-        <v>123</v>
+        <v>125</v>
       </c>
       <c r="D126" t="s">
-        <v>295</v>
+        <v>296</v>
       </c>
       <c r="E126">
-        <v>5</v>
+        <v>8</v>
       </c>
     </row>
     <row r="127" spans="1:5">
@@ -4346,13 +4314,13 @@
         <v>39</v>
       </c>
       <c r="C127" t="s">
-        <v>124</v>
+        <v>126</v>
       </c>
       <c r="D127" t="s">
-        <v>296</v>
+        <v>297</v>
       </c>
       <c r="E127">
-        <v>7</v>
+        <v>10</v>
       </c>
     </row>
     <row r="128" spans="1:5">
@@ -4363,64 +4331,64 @@
         <v>39</v>
       </c>
       <c r="C128" t="s">
-        <v>125</v>
+        <v>127</v>
       </c>
       <c r="D128" t="s">
-        <v>297</v>
+        <v>298</v>
       </c>
       <c r="E128">
-        <v>8</v>
+        <v>30</v>
       </c>
     </row>
     <row r="129" spans="1:5">
       <c r="A129" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="B129" t="s">
         <v>39</v>
       </c>
       <c r="C129" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="D129" t="s">
         <v>298</v>
       </c>
       <c r="E129">
-        <v>10</v>
+        <v>30</v>
       </c>
     </row>
     <row r="130" spans="1:5">
       <c r="A130" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="B130" t="s">
         <v>39</v>
       </c>
       <c r="C130" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="D130" t="s">
         <v>299</v>
       </c>
       <c r="E130">
-        <v>30</v>
+        <v>1</v>
       </c>
     </row>
     <row r="131" spans="1:5">
       <c r="A131" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="B131" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="C131" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="D131" t="s">
         <v>299</v>
       </c>
       <c r="E131">
-        <v>30</v>
+        <v>1</v>
       </c>
     </row>
     <row r="132" spans="1:5">
@@ -4431,7 +4399,7 @@
         <v>39</v>
       </c>
       <c r="C132" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="D132" t="s">
         <v>300</v>
@@ -4442,16 +4410,16 @@
     </row>
     <row r="133" spans="1:5">
       <c r="A133" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B133" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="C133" t="s">
-        <v>128</v>
+        <v>130</v>
       </c>
       <c r="D133" t="s">
-        <v>300</v>
+        <v>301</v>
       </c>
       <c r="E133">
         <v>1</v>
@@ -4465,10 +4433,10 @@
         <v>39</v>
       </c>
       <c r="C134" t="s">
-        <v>129</v>
+        <v>131</v>
       </c>
       <c r="D134" t="s">
-        <v>301</v>
+        <v>302</v>
       </c>
       <c r="E134">
         <v>1</v>
@@ -4482,10 +4450,10 @@
         <v>39</v>
       </c>
       <c r="C135" t="s">
-        <v>130</v>
+        <v>132</v>
       </c>
       <c r="D135" t="s">
-        <v>302</v>
+        <v>303</v>
       </c>
       <c r="E135">
         <v>1</v>
@@ -4499,10 +4467,10 @@
         <v>39</v>
       </c>
       <c r="C136" t="s">
-        <v>131</v>
+        <v>133</v>
       </c>
       <c r="D136" t="s">
-        <v>303</v>
+        <v>304</v>
       </c>
       <c r="E136">
         <v>1</v>
@@ -4516,10 +4484,10 @@
         <v>39</v>
       </c>
       <c r="C137" t="s">
-        <v>132</v>
+        <v>134</v>
       </c>
       <c r="D137" t="s">
-        <v>304</v>
+        <v>305</v>
       </c>
       <c r="E137">
         <v>1</v>
@@ -4533,10 +4501,10 @@
         <v>39</v>
       </c>
       <c r="C138" t="s">
-        <v>133</v>
+        <v>135</v>
       </c>
       <c r="D138" t="s">
-        <v>305</v>
+        <v>306</v>
       </c>
       <c r="E138">
         <v>1</v>
@@ -4550,10 +4518,10 @@
         <v>39</v>
       </c>
       <c r="C139" t="s">
-        <v>134</v>
+        <v>136</v>
       </c>
       <c r="D139" t="s">
-        <v>306</v>
+        <v>307</v>
       </c>
       <c r="E139">
         <v>1</v>
@@ -4567,10 +4535,10 @@
         <v>39</v>
       </c>
       <c r="C140" t="s">
-        <v>135</v>
+        <v>137</v>
       </c>
       <c r="D140" t="s">
-        <v>307</v>
+        <v>308</v>
       </c>
       <c r="E140">
         <v>1</v>
@@ -4578,13 +4546,13 @@
     </row>
     <row r="141" spans="1:5">
       <c r="A141" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="B141" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="C141" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="D141" t="s">
         <v>308</v>
@@ -4601,7 +4569,7 @@
         <v>39</v>
       </c>
       <c r="C142" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="D142" t="s">
         <v>309</v>
@@ -4618,7 +4586,7 @@
         <v>41</v>
       </c>
       <c r="C143" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="D143" t="s">
         <v>309</v>
@@ -4635,7 +4603,7 @@
         <v>39</v>
       </c>
       <c r="C144" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="D144" t="s">
         <v>310</v>
@@ -4646,16 +4614,16 @@
     </row>
     <row r="145" spans="1:5">
       <c r="A145" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="B145" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="C145" t="s">
-        <v>138</v>
+        <v>140</v>
       </c>
       <c r="D145" t="s">
-        <v>310</v>
+        <v>311</v>
       </c>
       <c r="E145">
         <v>1</v>
@@ -4669,10 +4637,10 @@
         <v>39</v>
       </c>
       <c r="C146" t="s">
-        <v>139</v>
+        <v>141</v>
       </c>
       <c r="D146" t="s">
-        <v>311</v>
+        <v>312</v>
       </c>
       <c r="E146">
         <v>1</v>
@@ -4686,10 +4654,10 @@
         <v>39</v>
       </c>
       <c r="C147" t="s">
-        <v>140</v>
+        <v>142</v>
       </c>
       <c r="D147" t="s">
-        <v>312</v>
+        <v>313</v>
       </c>
       <c r="E147">
         <v>1</v>
@@ -4703,10 +4671,10 @@
         <v>39</v>
       </c>
       <c r="C148" t="s">
-        <v>141</v>
+        <v>143</v>
       </c>
       <c r="D148" t="s">
-        <v>313</v>
+        <v>314</v>
       </c>
       <c r="E148">
         <v>1</v>
@@ -4720,10 +4688,10 @@
         <v>39</v>
       </c>
       <c r="C149" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="D149" t="s">
-        <v>314</v>
+        <v>315</v>
       </c>
       <c r="E149">
         <v>1</v>
@@ -4737,10 +4705,10 @@
         <v>39</v>
       </c>
       <c r="C150" t="s">
-        <v>143</v>
+        <v>145</v>
       </c>
       <c r="D150" t="s">
-        <v>315</v>
+        <v>316</v>
       </c>
       <c r="E150">
         <v>1</v>
@@ -4754,10 +4722,10 @@
         <v>39</v>
       </c>
       <c r="C151" t="s">
-        <v>144</v>
+        <v>146</v>
       </c>
       <c r="D151" t="s">
-        <v>316</v>
+        <v>317</v>
       </c>
       <c r="E151">
         <v>1</v>
@@ -4771,10 +4739,10 @@
         <v>39</v>
       </c>
       <c r="C152" t="s">
-        <v>145</v>
+        <v>147</v>
       </c>
       <c r="D152" t="s">
-        <v>317</v>
+        <v>318</v>
       </c>
       <c r="E152">
         <v>1</v>
@@ -4788,10 +4756,10 @@
         <v>39</v>
       </c>
       <c r="C153" t="s">
-        <v>146</v>
+        <v>148</v>
       </c>
       <c r="D153" t="s">
-        <v>318</v>
+        <v>319</v>
       </c>
       <c r="E153">
         <v>1</v>
@@ -4805,10 +4773,10 @@
         <v>39</v>
       </c>
       <c r="C154" t="s">
-        <v>147</v>
+        <v>149</v>
       </c>
       <c r="D154" t="s">
-        <v>319</v>
+        <v>320</v>
       </c>
       <c r="E154">
         <v>1</v>
@@ -4822,10 +4790,10 @@
         <v>39</v>
       </c>
       <c r="C155" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
       <c r="D155" t="s">
-        <v>320</v>
+        <v>321</v>
       </c>
       <c r="E155">
         <v>1</v>
@@ -4839,10 +4807,10 @@
         <v>39</v>
       </c>
       <c r="C156" t="s">
-        <v>149</v>
+        <v>151</v>
       </c>
       <c r="D156" t="s">
-        <v>321</v>
+        <v>322</v>
       </c>
       <c r="E156">
         <v>1</v>
@@ -4856,10 +4824,10 @@
         <v>39</v>
       </c>
       <c r="C157" t="s">
-        <v>150</v>
+        <v>152</v>
       </c>
       <c r="D157" t="s">
-        <v>322</v>
+        <v>323</v>
       </c>
       <c r="E157">
         <v>1</v>
@@ -4873,10 +4841,10 @@
         <v>39</v>
       </c>
       <c r="C158" t="s">
-        <v>151</v>
+        <v>153</v>
       </c>
       <c r="D158" t="s">
-        <v>323</v>
+        <v>324</v>
       </c>
       <c r="E158">
         <v>1</v>
@@ -4890,10 +4858,10 @@
         <v>39</v>
       </c>
       <c r="C159" t="s">
-        <v>152</v>
+        <v>154</v>
       </c>
       <c r="D159" t="s">
-        <v>324</v>
+        <v>325</v>
       </c>
       <c r="E159">
         <v>1</v>
@@ -4907,10 +4875,10 @@
         <v>39</v>
       </c>
       <c r="C160" t="s">
-        <v>153</v>
+        <v>155</v>
       </c>
       <c r="D160" t="s">
-        <v>325</v>
+        <v>326</v>
       </c>
       <c r="E160">
         <v>1</v>
@@ -4924,10 +4892,10 @@
         <v>39</v>
       </c>
       <c r="C161" t="s">
-        <v>154</v>
+        <v>156</v>
       </c>
       <c r="D161" t="s">
-        <v>326</v>
+        <v>327</v>
       </c>
       <c r="E161">
         <v>1</v>
@@ -4941,10 +4909,10 @@
         <v>39</v>
       </c>
       <c r="C162" t="s">
-        <v>155</v>
+        <v>157</v>
       </c>
       <c r="D162" t="s">
-        <v>327</v>
+        <v>328</v>
       </c>
       <c r="E162">
         <v>1</v>
@@ -4958,13 +4926,13 @@
         <v>39</v>
       </c>
       <c r="C163" t="s">
-        <v>156</v>
+        <v>158</v>
       </c>
       <c r="D163" t="s">
-        <v>328</v>
+        <v>313</v>
       </c>
       <c r="E163">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="164" spans="1:5">
@@ -4975,13 +4943,13 @@
         <v>39</v>
       </c>
       <c r="C164" t="s">
-        <v>157</v>
+        <v>159</v>
       </c>
       <c r="D164" t="s">
         <v>329</v>
       </c>
       <c r="E164">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="165" spans="1:5">
@@ -4992,10 +4960,10 @@
         <v>39</v>
       </c>
       <c r="C165" t="s">
-        <v>158</v>
+        <v>160</v>
       </c>
       <c r="D165" t="s">
-        <v>314</v>
+        <v>330</v>
       </c>
       <c r="E165">
         <v>2</v>
@@ -5009,10 +4977,10 @@
         <v>39</v>
       </c>
       <c r="C166" t="s">
-        <v>159</v>
+        <v>161</v>
       </c>
       <c r="D166" t="s">
-        <v>330</v>
+        <v>331</v>
       </c>
       <c r="E166">
         <v>2</v>
@@ -5026,10 +4994,10 @@
         <v>39</v>
       </c>
       <c r="C167" t="s">
-        <v>160</v>
+        <v>162</v>
       </c>
       <c r="D167" t="s">
-        <v>331</v>
+        <v>332</v>
       </c>
       <c r="E167">
         <v>2</v>
@@ -5043,13 +5011,13 @@
         <v>39</v>
       </c>
       <c r="C168" t="s">
-        <v>161</v>
+        <v>163</v>
       </c>
       <c r="D168" t="s">
-        <v>332</v>
+        <v>333</v>
       </c>
       <c r="E168">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="169" spans="1:5">
@@ -5060,13 +5028,13 @@
         <v>39</v>
       </c>
       <c r="C169" t="s">
-        <v>162</v>
+        <v>164</v>
       </c>
       <c r="D169" t="s">
-        <v>333</v>
+        <v>298</v>
       </c>
       <c r="E169">
-        <v>2</v>
+        <v>5</v>
       </c>
     </row>
     <row r="170" spans="1:5">
@@ -5077,13 +5045,13 @@
         <v>39</v>
       </c>
       <c r="C170" t="s">
-        <v>163</v>
+        <v>165</v>
       </c>
       <c r="D170" t="s">
         <v>334</v>
       </c>
       <c r="E170">
-        <v>3</v>
+        <v>8</v>
       </c>
     </row>
     <row r="171" spans="1:5">
@@ -5094,13 +5062,13 @@
         <v>39</v>
       </c>
       <c r="C171" t="s">
-        <v>164</v>
+        <v>166</v>
       </c>
       <c r="D171" t="s">
-        <v>299</v>
+        <v>254</v>
       </c>
       <c r="E171">
-        <v>5</v>
+        <v>8</v>
       </c>
     </row>
     <row r="172" spans="1:5">
@@ -5111,47 +5079,47 @@
         <v>39</v>
       </c>
       <c r="C172" t="s">
-        <v>165</v>
+        <v>167</v>
       </c>
       <c r="D172" t="s">
         <v>335</v>
       </c>
       <c r="E172">
-        <v>8</v>
+        <v>10</v>
       </c>
     </row>
     <row r="173" spans="1:5">
       <c r="A173" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="B173" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="C173" t="s">
-        <v>166</v>
+        <v>168</v>
       </c>
       <c r="D173" t="s">
-        <v>255</v>
+        <v>323</v>
       </c>
       <c r="E173">
-        <v>8</v>
+        <v>1</v>
       </c>
     </row>
     <row r="174" spans="1:5">
       <c r="A174" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="B174" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="C174" t="s">
-        <v>167</v>
+        <v>169</v>
       </c>
       <c r="D174" t="s">
         <v>336</v>
       </c>
       <c r="E174">
-        <v>10</v>
+        <v>1</v>
       </c>
     </row>
     <row r="175" spans="1:5">
@@ -5162,10 +5130,10 @@
         <v>40</v>
       </c>
       <c r="C175" t="s">
-        <v>168</v>
+        <v>170</v>
       </c>
       <c r="D175" t="s">
-        <v>324</v>
+        <v>337</v>
       </c>
       <c r="E175">
         <v>1</v>
@@ -5179,10 +5147,10 @@
         <v>40</v>
       </c>
       <c r="C176" t="s">
-        <v>169</v>
+        <v>171</v>
       </c>
       <c r="D176" t="s">
-        <v>337</v>
+        <v>338</v>
       </c>
       <c r="E176">
         <v>1</v>
@@ -5190,13 +5158,13 @@
     </row>
     <row r="177" spans="1:5">
       <c r="A177" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="B177" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="C177" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="D177" t="s">
         <v>338</v>
@@ -5213,7 +5181,7 @@
         <v>40</v>
       </c>
       <c r="C178" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="D178" t="s">
         <v>339</v>
@@ -5224,16 +5192,16 @@
     </row>
     <row r="179" spans="1:5">
       <c r="A179" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B179" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C179" t="s">
-        <v>171</v>
+        <v>173</v>
       </c>
       <c r="D179" t="s">
-        <v>339</v>
+        <v>340</v>
       </c>
       <c r="E179">
         <v>1</v>
@@ -5247,10 +5215,10 @@
         <v>40</v>
       </c>
       <c r="C180" t="s">
-        <v>172</v>
+        <v>174</v>
       </c>
       <c r="D180" t="s">
-        <v>340</v>
+        <v>264</v>
       </c>
       <c r="E180">
         <v>1</v>
@@ -5264,7 +5232,7 @@
         <v>40</v>
       </c>
       <c r="C181" t="s">
-        <v>173</v>
+        <v>175</v>
       </c>
       <c r="D181" t="s">
         <v>341</v>
@@ -5281,10 +5249,10 @@
         <v>40</v>
       </c>
       <c r="C182" t="s">
-        <v>174</v>
+        <v>176</v>
       </c>
       <c r="D182" t="s">
-        <v>265</v>
+        <v>342</v>
       </c>
       <c r="E182">
         <v>1</v>
@@ -5298,10 +5266,10 @@
         <v>40</v>
       </c>
       <c r="C183" t="s">
-        <v>175</v>
+        <v>177</v>
       </c>
       <c r="D183" t="s">
-        <v>342</v>
+        <v>343</v>
       </c>
       <c r="E183">
         <v>1</v>
@@ -5315,10 +5283,10 @@
         <v>40</v>
       </c>
       <c r="C184" t="s">
-        <v>176</v>
+        <v>178</v>
       </c>
       <c r="D184" t="s">
-        <v>343</v>
+        <v>344</v>
       </c>
       <c r="E184">
         <v>1</v>
@@ -5332,10 +5300,10 @@
         <v>40</v>
       </c>
       <c r="C185" t="s">
-        <v>177</v>
+        <v>179</v>
       </c>
       <c r="D185" t="s">
-        <v>344</v>
+        <v>345</v>
       </c>
       <c r="E185">
         <v>1</v>
@@ -5349,10 +5317,10 @@
         <v>40</v>
       </c>
       <c r="C186" t="s">
-        <v>178</v>
+        <v>180</v>
       </c>
       <c r="D186" t="s">
-        <v>345</v>
+        <v>346</v>
       </c>
       <c r="E186">
         <v>1</v>
@@ -5366,10 +5334,10 @@
         <v>40</v>
       </c>
       <c r="C187" t="s">
-        <v>179</v>
+        <v>181</v>
       </c>
       <c r="D187" t="s">
-        <v>346</v>
+        <v>347</v>
       </c>
       <c r="E187">
         <v>1</v>
@@ -5383,10 +5351,10 @@
         <v>40</v>
       </c>
       <c r="C188" t="s">
-        <v>180</v>
+        <v>182</v>
       </c>
       <c r="D188" t="s">
-        <v>347</v>
+        <v>348</v>
       </c>
       <c r="E188">
         <v>1</v>
@@ -5400,10 +5368,10 @@
         <v>40</v>
       </c>
       <c r="C189" t="s">
-        <v>181</v>
+        <v>183</v>
       </c>
       <c r="D189" t="s">
-        <v>348</v>
+        <v>349</v>
       </c>
       <c r="E189">
         <v>1</v>
@@ -5417,10 +5385,10 @@
         <v>40</v>
       </c>
       <c r="C190" t="s">
-        <v>182</v>
+        <v>184</v>
       </c>
       <c r="D190" t="s">
-        <v>349</v>
+        <v>350</v>
       </c>
       <c r="E190">
         <v>1</v>
@@ -5434,10 +5402,10 @@
         <v>40</v>
       </c>
       <c r="C191" t="s">
-        <v>183</v>
+        <v>185</v>
       </c>
       <c r="D191" t="s">
-        <v>350</v>
+        <v>351</v>
       </c>
       <c r="E191">
         <v>1</v>
@@ -5451,10 +5419,10 @@
         <v>40</v>
       </c>
       <c r="C192" t="s">
-        <v>184</v>
+        <v>186</v>
       </c>
       <c r="D192" t="s">
-        <v>351</v>
+        <v>352</v>
       </c>
       <c r="E192">
         <v>1</v>
@@ -5468,10 +5436,10 @@
         <v>40</v>
       </c>
       <c r="C193" t="s">
-        <v>185</v>
+        <v>187</v>
       </c>
       <c r="D193" t="s">
-        <v>352</v>
+        <v>353</v>
       </c>
       <c r="E193">
         <v>1</v>
@@ -5485,10 +5453,10 @@
         <v>40</v>
       </c>
       <c r="C194" t="s">
-        <v>186</v>
+        <v>188</v>
       </c>
       <c r="D194" t="s">
-        <v>353</v>
+        <v>354</v>
       </c>
       <c r="E194">
         <v>1</v>
@@ -5502,10 +5470,10 @@
         <v>40</v>
       </c>
       <c r="C195" t="s">
-        <v>187</v>
+        <v>189</v>
       </c>
       <c r="D195" t="s">
-        <v>354</v>
+        <v>355</v>
       </c>
       <c r="E195">
         <v>1</v>
@@ -5519,10 +5487,10 @@
         <v>40</v>
       </c>
       <c r="C196" t="s">
-        <v>188</v>
+        <v>190</v>
       </c>
       <c r="D196" t="s">
-        <v>355</v>
+        <v>356</v>
       </c>
       <c r="E196">
         <v>1</v>
@@ -5536,10 +5504,10 @@
         <v>40</v>
       </c>
       <c r="C197" t="s">
-        <v>189</v>
+        <v>191</v>
       </c>
       <c r="D197" t="s">
-        <v>356</v>
+        <v>357</v>
       </c>
       <c r="E197">
         <v>1</v>
@@ -5553,10 +5521,10 @@
         <v>40</v>
       </c>
       <c r="C198" t="s">
-        <v>190</v>
+        <v>192</v>
       </c>
       <c r="D198" t="s">
-        <v>357</v>
+        <v>358</v>
       </c>
       <c r="E198">
         <v>1</v>
@@ -5570,10 +5538,10 @@
         <v>40</v>
       </c>
       <c r="C199" t="s">
-        <v>191</v>
+        <v>193</v>
       </c>
       <c r="D199" t="s">
-        <v>358</v>
+        <v>359</v>
       </c>
       <c r="E199">
         <v>1</v>
@@ -5587,10 +5555,10 @@
         <v>40</v>
       </c>
       <c r="C200" t="s">
-        <v>192</v>
+        <v>194</v>
       </c>
       <c r="D200" t="s">
-        <v>359</v>
+        <v>360</v>
       </c>
       <c r="E200">
         <v>1</v>
@@ -5604,10 +5572,10 @@
         <v>40</v>
       </c>
       <c r="C201" t="s">
-        <v>193</v>
+        <v>195</v>
       </c>
       <c r="D201" t="s">
-        <v>360</v>
+        <v>361</v>
       </c>
       <c r="E201">
         <v>1</v>
@@ -5621,10 +5589,10 @@
         <v>40</v>
       </c>
       <c r="C202" t="s">
-        <v>194</v>
+        <v>196</v>
       </c>
       <c r="D202" t="s">
-        <v>361</v>
+        <v>362</v>
       </c>
       <c r="E202">
         <v>1</v>
@@ -5638,10 +5606,10 @@
         <v>40</v>
       </c>
       <c r="C203" t="s">
-        <v>195</v>
+        <v>197</v>
       </c>
       <c r="D203" t="s">
-        <v>362</v>
+        <v>363</v>
       </c>
       <c r="E203">
         <v>1</v>
@@ -5655,10 +5623,10 @@
         <v>40</v>
       </c>
       <c r="C204" t="s">
-        <v>196</v>
+        <v>198</v>
       </c>
       <c r="D204" t="s">
-        <v>363</v>
+        <v>364</v>
       </c>
       <c r="E204">
         <v>1</v>
@@ -5672,10 +5640,10 @@
         <v>40</v>
       </c>
       <c r="C205" t="s">
-        <v>197</v>
+        <v>199</v>
       </c>
       <c r="D205" t="s">
-        <v>364</v>
+        <v>365</v>
       </c>
       <c r="E205">
         <v>1</v>
@@ -5689,13 +5657,13 @@
         <v>40</v>
       </c>
       <c r="C206" t="s">
-        <v>198</v>
+        <v>200</v>
       </c>
       <c r="D206" t="s">
-        <v>365</v>
+        <v>366</v>
       </c>
       <c r="E206">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="207" spans="1:5">
@@ -5706,13 +5674,13 @@
         <v>40</v>
       </c>
       <c r="C207" t="s">
-        <v>199</v>
+        <v>201</v>
       </c>
       <c r="D207" t="s">
-        <v>366</v>
+        <v>367</v>
       </c>
       <c r="E207">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="208" spans="1:5">
@@ -5723,10 +5691,10 @@
         <v>40</v>
       </c>
       <c r="C208" t="s">
-        <v>200</v>
+        <v>202</v>
       </c>
       <c r="D208" t="s">
-        <v>367</v>
+        <v>368</v>
       </c>
       <c r="E208">
         <v>2</v>
@@ -5740,10 +5708,10 @@
         <v>40</v>
       </c>
       <c r="C209" t="s">
-        <v>201</v>
+        <v>203</v>
       </c>
       <c r="D209" t="s">
-        <v>368</v>
+        <v>369</v>
       </c>
       <c r="E209">
         <v>2</v>
@@ -5757,10 +5725,10 @@
         <v>40</v>
       </c>
       <c r="C210" t="s">
-        <v>202</v>
+        <v>204</v>
       </c>
       <c r="D210" t="s">
-        <v>369</v>
+        <v>370</v>
       </c>
       <c r="E210">
         <v>2</v>
@@ -5774,10 +5742,10 @@
         <v>40</v>
       </c>
       <c r="C211" t="s">
-        <v>203</v>
+        <v>205</v>
       </c>
       <c r="D211" t="s">
-        <v>370</v>
+        <v>371</v>
       </c>
       <c r="E211">
         <v>2</v>
@@ -5791,10 +5759,10 @@
         <v>40</v>
       </c>
       <c r="C212" t="s">
-        <v>204</v>
+        <v>206</v>
       </c>
       <c r="D212" t="s">
-        <v>371</v>
+        <v>372</v>
       </c>
       <c r="E212">
         <v>2</v>
@@ -5808,10 +5776,10 @@
         <v>40</v>
       </c>
       <c r="C213" t="s">
-        <v>205</v>
+        <v>207</v>
       </c>
       <c r="D213" t="s">
-        <v>372</v>
+        <v>373</v>
       </c>
       <c r="E213">
         <v>2</v>
@@ -5825,7 +5793,7 @@
         <v>40</v>
       </c>
       <c r="C214" t="s">
-        <v>206</v>
+        <v>208</v>
       </c>
       <c r="D214" t="s">
         <v>373</v>
@@ -5842,7 +5810,7 @@
         <v>40</v>
       </c>
       <c r="C215" t="s">
-        <v>207</v>
+        <v>209</v>
       </c>
       <c r="D215" t="s">
         <v>374</v>
@@ -5859,10 +5827,10 @@
         <v>40</v>
       </c>
       <c r="C216" t="s">
-        <v>208</v>
+        <v>210</v>
       </c>
       <c r="D216" t="s">
-        <v>374</v>
+        <v>375</v>
       </c>
       <c r="E216">
         <v>2</v>
@@ -5876,10 +5844,10 @@
         <v>40</v>
       </c>
       <c r="C217" t="s">
-        <v>209</v>
+        <v>211</v>
       </c>
       <c r="D217" t="s">
-        <v>375</v>
+        <v>376</v>
       </c>
       <c r="E217">
         <v>2</v>
@@ -5893,13 +5861,13 @@
         <v>40</v>
       </c>
       <c r="C218" t="s">
-        <v>210</v>
+        <v>212</v>
       </c>
       <c r="D218" t="s">
-        <v>376</v>
+        <v>377</v>
       </c>
       <c r="E218">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="219" spans="1:5">
@@ -5910,13 +5878,13 @@
         <v>40</v>
       </c>
       <c r="C219" t="s">
-        <v>211</v>
+        <v>213</v>
       </c>
       <c r="D219" t="s">
-        <v>377</v>
+        <v>264</v>
       </c>
       <c r="E219">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="220" spans="1:5">
@@ -5927,13 +5895,13 @@
         <v>40</v>
       </c>
       <c r="C220" t="s">
-        <v>212</v>
+        <v>214</v>
       </c>
       <c r="D220" t="s">
         <v>378</v>
       </c>
       <c r="E220">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="221" spans="1:5">
@@ -5944,13 +5912,13 @@
         <v>40</v>
       </c>
       <c r="C221" t="s">
-        <v>213</v>
+        <v>215</v>
       </c>
       <c r="D221" t="s">
-        <v>265</v>
+        <v>379</v>
       </c>
       <c r="E221">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="222" spans="1:5">
@@ -5961,10 +5929,10 @@
         <v>40</v>
       </c>
       <c r="C222" t="s">
-        <v>214</v>
+        <v>216</v>
       </c>
       <c r="D222" t="s">
-        <v>379</v>
+        <v>380</v>
       </c>
       <c r="E222">
         <v>4</v>
@@ -5978,10 +5946,10 @@
         <v>40</v>
       </c>
       <c r="C223" t="s">
-        <v>215</v>
+        <v>217</v>
       </c>
       <c r="D223" t="s">
-        <v>380</v>
+        <v>381</v>
       </c>
       <c r="E223">
         <v>4</v>
@@ -5995,10 +5963,10 @@
         <v>40</v>
       </c>
       <c r="C224" t="s">
-        <v>216</v>
+        <v>218</v>
       </c>
       <c r="D224" t="s">
-        <v>381</v>
+        <v>382</v>
       </c>
       <c r="E224">
         <v>4</v>
@@ -6012,13 +5980,13 @@
         <v>40</v>
       </c>
       <c r="C225" t="s">
-        <v>217</v>
+        <v>219</v>
       </c>
       <c r="D225" t="s">
-        <v>382</v>
+        <v>383</v>
       </c>
       <c r="E225">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="226" spans="1:5">
@@ -6029,13 +5997,13 @@
         <v>40</v>
       </c>
       <c r="C226" t="s">
-        <v>218</v>
+        <v>220</v>
       </c>
       <c r="D226" t="s">
-        <v>383</v>
+        <v>384</v>
       </c>
       <c r="E226">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="227" spans="1:5">
@@ -6046,13 +6014,13 @@
         <v>40</v>
       </c>
       <c r="C227" t="s">
-        <v>219</v>
+        <v>221</v>
       </c>
       <c r="D227" t="s">
-        <v>384</v>
+        <v>385</v>
       </c>
       <c r="E227">
-        <v>5</v>
+        <v>6</v>
       </c>
     </row>
     <row r="228" spans="1:5">
@@ -6063,13 +6031,13 @@
         <v>40</v>
       </c>
       <c r="C228" t="s">
-        <v>220</v>
+        <v>222</v>
       </c>
       <c r="D228" t="s">
-        <v>385</v>
+        <v>386</v>
       </c>
       <c r="E228">
-        <v>5</v>
+        <v>8</v>
       </c>
     </row>
     <row r="229" spans="1:5">
@@ -6080,13 +6048,13 @@
         <v>40</v>
       </c>
       <c r="C229" t="s">
-        <v>221</v>
+        <v>223</v>
       </c>
       <c r="D229" t="s">
-        <v>386</v>
+        <v>387</v>
       </c>
       <c r="E229">
-        <v>6</v>
+        <v>10</v>
       </c>
     </row>
     <row r="230" spans="1:5">
@@ -6097,13 +6065,13 @@
         <v>40</v>
       </c>
       <c r="C230" t="s">
-        <v>222</v>
+        <v>224</v>
       </c>
       <c r="D230" t="s">
         <v>387</v>
       </c>
       <c r="E230">
-        <v>8</v>
+        <v>10</v>
       </c>
     </row>
     <row r="231" spans="1:5">
@@ -6114,13 +6082,13 @@
         <v>40</v>
       </c>
       <c r="C231" t="s">
-        <v>223</v>
+        <v>225</v>
       </c>
       <c r="D231" t="s">
-        <v>388</v>
+        <v>266</v>
       </c>
       <c r="E231">
-        <v>10</v>
+        <v>12</v>
       </c>
     </row>
     <row r="232" spans="1:5">
@@ -6131,13 +6099,13 @@
         <v>40</v>
       </c>
       <c r="C232" t="s">
-        <v>224</v>
+        <v>226</v>
       </c>
       <c r="D232" t="s">
         <v>388</v>
       </c>
       <c r="E232">
-        <v>10</v>
+        <v>12</v>
       </c>
     </row>
     <row r="233" spans="1:5">
@@ -6148,13 +6116,13 @@
         <v>40</v>
       </c>
       <c r="C233" t="s">
-        <v>225</v>
+        <v>227</v>
       </c>
       <c r="D233" t="s">
-        <v>267</v>
+        <v>389</v>
       </c>
       <c r="E233">
-        <v>12</v>
+        <v>14</v>
       </c>
     </row>
     <row r="234" spans="1:5">
@@ -6165,13 +6133,13 @@
         <v>40</v>
       </c>
       <c r="C234" t="s">
-        <v>226</v>
+        <v>228</v>
       </c>
       <c r="D234" t="s">
-        <v>389</v>
+        <v>390</v>
       </c>
       <c r="E234">
-        <v>12</v>
+        <v>15</v>
       </c>
     </row>
     <row r="235" spans="1:5">
@@ -6182,47 +6150,47 @@
         <v>40</v>
       </c>
       <c r="C235" t="s">
-        <v>227</v>
+        <v>229</v>
       </c>
       <c r="D235" t="s">
-        <v>390</v>
+        <v>391</v>
       </c>
       <c r="E235">
-        <v>14</v>
+        <v>20</v>
       </c>
     </row>
     <row r="236" spans="1:5">
       <c r="A236" t="s">
-        <v>14</v>
+        <v>10</v>
       </c>
       <c r="B236" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="C236" t="s">
-        <v>228</v>
+        <v>230</v>
       </c>
       <c r="D236" t="s">
-        <v>391</v>
+        <v>392</v>
       </c>
       <c r="E236">
-        <v>15</v>
+        <v>1</v>
       </c>
     </row>
     <row r="237" spans="1:5">
       <c r="A237" t="s">
-        <v>14</v>
+        <v>6</v>
       </c>
       <c r="B237" t="s">
-        <v>40</v>
+        <v>36</v>
       </c>
       <c r="C237" t="s">
-        <v>229</v>
+        <v>231</v>
       </c>
       <c r="D237" t="s">
-        <v>392</v>
+        <v>393</v>
       </c>
       <c r="E237">
-        <v>20</v>
+        <v>1</v>
       </c>
     </row>
     <row r="238" spans="1:5">
@@ -6233,63 +6201,12 @@
         <v>39</v>
       </c>
       <c r="C238" t="s">
-        <v>230</v>
+        <v>232</v>
       </c>
       <c r="D238" t="s">
-        <v>393</v>
+        <v>394</v>
       </c>
       <c r="E238">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="239" spans="1:5">
-      <c r="A239" t="s">
-        <v>6</v>
-      </c>
-      <c r="B239" t="s">
-        <v>36</v>
-      </c>
-      <c r="C239" t="s">
-        <v>231</v>
-      </c>
-      <c r="D239" t="s">
-        <v>394</v>
-      </c>
-      <c r="E239">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="240" spans="1:5">
-      <c r="A240" t="s">
-        <v>15</v>
-      </c>
-      <c r="B240" t="s">
-        <v>41</v>
-      </c>
-      <c r="C240" t="s">
-        <v>232</v>
-      </c>
-      <c r="D240" t="s">
-        <v>395</v>
-      </c>
-      <c r="E240">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="241" spans="1:5">
-      <c r="A241" t="s">
-        <v>10</v>
-      </c>
-      <c r="B241" t="s">
-        <v>39</v>
-      </c>
-      <c r="C241" t="s">
-        <v>233</v>
-      </c>
-      <c r="D241" t="s">
-        <v>396</v>
-      </c>
-      <c r="E241">
         <v>1</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualização automática: rac (18/09/2026 16:36)
</commit_message>
<xml_diff>
--- a/Coordenadoria/02_Dados_Tratados/base_rac_tratada.xlsx
+++ b/Coordenadoria/02_Dados_Tratados/base_rac_tratada.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1079" uniqueCount="395">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1071" uniqueCount="395">
   <si>
     <t>matricula</t>
   </si>
@@ -62,12 +62,12 @@
     <t>2726</t>
   </si>
   <si>
+    <t>2741</t>
+  </si>
+  <si>
     <t>2702</t>
   </si>
   <si>
-    <t>2741</t>
-  </si>
-  <si>
     <t>2703</t>
   </si>
   <si>
@@ -140,10 +140,10 @@
     <t>1º ETA</t>
   </si>
   <si>
+    <t>BABV</t>
+  </si>
+  <si>
     <t>EPCAR</t>
-  </si>
-  <si>
-    <t>BABV</t>
   </si>
   <si>
     <t>PAMALS</t>
@@ -1206,8 +1206,16 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <fonts count="1">
+  <fonts count="2">
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -1223,7 +1231,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -1231,12 +1239,30 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1535,22 +1561,22 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:6">
-      <c r="A1" t="s">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" t="s">
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" t="s">
+      <c r="F1" s="1" t="s">
         <v>5</v>
       </c>
     </row>
@@ -1748,10 +1774,10 @@
         <v>53</v>
       </c>
       <c r="E11">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F11">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="12" spans="1:6">
@@ -1762,16 +1788,16 @@
         <v>42</v>
       </c>
       <c r="C12" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="D12" t="s">
         <v>53</v>
       </c>
       <c r="E12">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F12">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="13" spans="1:6">
@@ -2139,7 +2165,7 @@
         <v>35</v>
       </c>
       <c r="B31" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="C31" t="s">
         <v>52</v>
@@ -2161,23 +2187,23 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E238"/>
+  <dimension ref="A1:E236"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:5">
-      <c r="A1" t="s">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" t="s">
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
         <v>55</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>56</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="1" t="s">
         <v>57</v>
       </c>
     </row>
@@ -2642,10 +2668,10 @@
     </row>
     <row r="29" spans="1:5">
       <c r="A29" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="B29" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="C29" t="s">
         <v>68</v>
@@ -4546,16 +4572,16 @@
     </row>
     <row r="141" spans="1:5">
       <c r="A141" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="B141" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="C141" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="D141" t="s">
-        <v>308</v>
+        <v>309</v>
       </c>
       <c r="E141">
         <v>1</v>
@@ -4569,10 +4595,10 @@
         <v>39</v>
       </c>
       <c r="C142" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="D142" t="s">
-        <v>309</v>
+        <v>310</v>
       </c>
       <c r="E142">
         <v>1</v>
@@ -4580,16 +4606,16 @@
     </row>
     <row r="143" spans="1:5">
       <c r="A143" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="B143" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="C143" t="s">
-        <v>138</v>
+        <v>140</v>
       </c>
       <c r="D143" t="s">
-        <v>309</v>
+        <v>311</v>
       </c>
       <c r="E143">
         <v>1</v>
@@ -4603,10 +4629,10 @@
         <v>39</v>
       </c>
       <c r="C144" t="s">
-        <v>139</v>
+        <v>141</v>
       </c>
       <c r="D144" t="s">
-        <v>310</v>
+        <v>312</v>
       </c>
       <c r="E144">
         <v>1</v>
@@ -4620,10 +4646,10 @@
         <v>39</v>
       </c>
       <c r="C145" t="s">
-        <v>140</v>
+        <v>142</v>
       </c>
       <c r="D145" t="s">
-        <v>311</v>
+        <v>313</v>
       </c>
       <c r="E145">
         <v>1</v>
@@ -4637,10 +4663,10 @@
         <v>39</v>
       </c>
       <c r="C146" t="s">
-        <v>141</v>
+        <v>143</v>
       </c>
       <c r="D146" t="s">
-        <v>312</v>
+        <v>314</v>
       </c>
       <c r="E146">
         <v>1</v>
@@ -4654,10 +4680,10 @@
         <v>39</v>
       </c>
       <c r="C147" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="D147" t="s">
-        <v>313</v>
+        <v>315</v>
       </c>
       <c r="E147">
         <v>1</v>
@@ -4671,10 +4697,10 @@
         <v>39</v>
       </c>
       <c r="C148" t="s">
-        <v>143</v>
+        <v>145</v>
       </c>
       <c r="D148" t="s">
-        <v>314</v>
+        <v>316</v>
       </c>
       <c r="E148">
         <v>1</v>
@@ -4688,10 +4714,10 @@
         <v>39</v>
       </c>
       <c r="C149" t="s">
-        <v>144</v>
+        <v>146</v>
       </c>
       <c r="D149" t="s">
-        <v>315</v>
+        <v>317</v>
       </c>
       <c r="E149">
         <v>1</v>
@@ -4705,10 +4731,10 @@
         <v>39</v>
       </c>
       <c r="C150" t="s">
-        <v>145</v>
+        <v>147</v>
       </c>
       <c r="D150" t="s">
-        <v>316</v>
+        <v>318</v>
       </c>
       <c r="E150">
         <v>1</v>
@@ -4722,10 +4748,10 @@
         <v>39</v>
       </c>
       <c r="C151" t="s">
-        <v>146</v>
+        <v>148</v>
       </c>
       <c r="D151" t="s">
-        <v>317</v>
+        <v>319</v>
       </c>
       <c r="E151">
         <v>1</v>
@@ -4739,10 +4765,10 @@
         <v>39</v>
       </c>
       <c r="C152" t="s">
-        <v>147</v>
+        <v>149</v>
       </c>
       <c r="D152" t="s">
-        <v>318</v>
+        <v>320</v>
       </c>
       <c r="E152">
         <v>1</v>
@@ -4756,10 +4782,10 @@
         <v>39</v>
       </c>
       <c r="C153" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
       <c r="D153" t="s">
-        <v>319</v>
+        <v>321</v>
       </c>
       <c r="E153">
         <v>1</v>
@@ -4773,10 +4799,10 @@
         <v>39</v>
       </c>
       <c r="C154" t="s">
-        <v>149</v>
+        <v>151</v>
       </c>
       <c r="D154" t="s">
-        <v>320</v>
+        <v>322</v>
       </c>
       <c r="E154">
         <v>1</v>
@@ -4790,10 +4816,10 @@
         <v>39</v>
       </c>
       <c r="C155" t="s">
-        <v>150</v>
+        <v>152</v>
       </c>
       <c r="D155" t="s">
-        <v>321</v>
+        <v>323</v>
       </c>
       <c r="E155">
         <v>1</v>
@@ -4807,10 +4833,10 @@
         <v>39</v>
       </c>
       <c r="C156" t="s">
-        <v>151</v>
+        <v>153</v>
       </c>
       <c r="D156" t="s">
-        <v>322</v>
+        <v>324</v>
       </c>
       <c r="E156">
         <v>1</v>
@@ -4824,10 +4850,10 @@
         <v>39</v>
       </c>
       <c r="C157" t="s">
-        <v>152</v>
+        <v>154</v>
       </c>
       <c r="D157" t="s">
-        <v>323</v>
+        <v>325</v>
       </c>
       <c r="E157">
         <v>1</v>
@@ -4841,10 +4867,10 @@
         <v>39</v>
       </c>
       <c r="C158" t="s">
-        <v>153</v>
+        <v>155</v>
       </c>
       <c r="D158" t="s">
-        <v>324</v>
+        <v>326</v>
       </c>
       <c r="E158">
         <v>1</v>
@@ -4858,10 +4884,10 @@
         <v>39</v>
       </c>
       <c r="C159" t="s">
-        <v>154</v>
+        <v>156</v>
       </c>
       <c r="D159" t="s">
-        <v>325</v>
+        <v>327</v>
       </c>
       <c r="E159">
         <v>1</v>
@@ -4875,10 +4901,10 @@
         <v>39</v>
       </c>
       <c r="C160" t="s">
-        <v>155</v>
+        <v>157</v>
       </c>
       <c r="D160" t="s">
-        <v>326</v>
+        <v>328</v>
       </c>
       <c r="E160">
         <v>1</v>
@@ -4892,13 +4918,13 @@
         <v>39</v>
       </c>
       <c r="C161" t="s">
-        <v>156</v>
+        <v>158</v>
       </c>
       <c r="D161" t="s">
-        <v>327</v>
+        <v>313</v>
       </c>
       <c r="E161">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="162" spans="1:5">
@@ -4909,13 +4935,13 @@
         <v>39</v>
       </c>
       <c r="C162" t="s">
-        <v>157</v>
+        <v>159</v>
       </c>
       <c r="D162" t="s">
-        <v>328</v>
+        <v>329</v>
       </c>
       <c r="E162">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="163" spans="1:5">
@@ -4926,10 +4952,10 @@
         <v>39</v>
       </c>
       <c r="C163" t="s">
-        <v>158</v>
+        <v>160</v>
       </c>
       <c r="D163" t="s">
-        <v>313</v>
+        <v>330</v>
       </c>
       <c r="E163">
         <v>2</v>
@@ -4943,10 +4969,10 @@
         <v>39</v>
       </c>
       <c r="C164" t="s">
-        <v>159</v>
+        <v>161</v>
       </c>
       <c r="D164" t="s">
-        <v>329</v>
+        <v>331</v>
       </c>
       <c r="E164">
         <v>2</v>
@@ -4960,10 +4986,10 @@
         <v>39</v>
       </c>
       <c r="C165" t="s">
-        <v>160</v>
+        <v>162</v>
       </c>
       <c r="D165" t="s">
-        <v>330</v>
+        <v>332</v>
       </c>
       <c r="E165">
         <v>2</v>
@@ -4977,13 +5003,13 @@
         <v>39</v>
       </c>
       <c r="C166" t="s">
-        <v>161</v>
+        <v>163</v>
       </c>
       <c r="D166" t="s">
-        <v>331</v>
+        <v>333</v>
       </c>
       <c r="E166">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="167" spans="1:5">
@@ -4994,13 +5020,13 @@
         <v>39</v>
       </c>
       <c r="C167" t="s">
-        <v>162</v>
+        <v>164</v>
       </c>
       <c r="D167" t="s">
-        <v>332</v>
+        <v>298</v>
       </c>
       <c r="E167">
-        <v>2</v>
+        <v>5</v>
       </c>
     </row>
     <row r="168" spans="1:5">
@@ -5011,13 +5037,13 @@
         <v>39</v>
       </c>
       <c r="C168" t="s">
-        <v>163</v>
+        <v>165</v>
       </c>
       <c r="D168" t="s">
-        <v>333</v>
+        <v>334</v>
       </c>
       <c r="E168">
-        <v>3</v>
+        <v>8</v>
       </c>
     </row>
     <row r="169" spans="1:5">
@@ -5028,13 +5054,13 @@
         <v>39</v>
       </c>
       <c r="C169" t="s">
-        <v>164</v>
+        <v>166</v>
       </c>
       <c r="D169" t="s">
-        <v>298</v>
+        <v>254</v>
       </c>
       <c r="E169">
-        <v>5</v>
+        <v>8</v>
       </c>
     </row>
     <row r="170" spans="1:5">
@@ -5045,47 +5071,47 @@
         <v>39</v>
       </c>
       <c r="C170" t="s">
-        <v>165</v>
+        <v>167</v>
       </c>
       <c r="D170" t="s">
-        <v>334</v>
+        <v>335</v>
       </c>
       <c r="E170">
-        <v>8</v>
+        <v>10</v>
       </c>
     </row>
     <row r="171" spans="1:5">
       <c r="A171" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="B171" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="C171" t="s">
-        <v>166</v>
+        <v>168</v>
       </c>
       <c r="D171" t="s">
-        <v>254</v>
+        <v>323</v>
       </c>
       <c r="E171">
-        <v>8</v>
+        <v>1</v>
       </c>
     </row>
     <row r="172" spans="1:5">
       <c r="A172" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="B172" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="C172" t="s">
-        <v>167</v>
+        <v>169</v>
       </c>
       <c r="D172" t="s">
-        <v>335</v>
+        <v>336</v>
       </c>
       <c r="E172">
-        <v>10</v>
+        <v>1</v>
       </c>
     </row>
     <row r="173" spans="1:5">
@@ -5096,10 +5122,10 @@
         <v>40</v>
       </c>
       <c r="C173" t="s">
-        <v>168</v>
+        <v>170</v>
       </c>
       <c r="D173" t="s">
-        <v>323</v>
+        <v>337</v>
       </c>
       <c r="E173">
         <v>1</v>
@@ -5113,10 +5139,10 @@
         <v>40</v>
       </c>
       <c r="C174" t="s">
-        <v>169</v>
+        <v>171</v>
       </c>
       <c r="D174" t="s">
-        <v>336</v>
+        <v>338</v>
       </c>
       <c r="E174">
         <v>1</v>
@@ -5130,10 +5156,10 @@
         <v>40</v>
       </c>
       <c r="C175" t="s">
-        <v>170</v>
+        <v>172</v>
       </c>
       <c r="D175" t="s">
-        <v>337</v>
+        <v>339</v>
       </c>
       <c r="E175">
         <v>1</v>
@@ -5147,10 +5173,10 @@
         <v>40</v>
       </c>
       <c r="C176" t="s">
-        <v>171</v>
+        <v>173</v>
       </c>
       <c r="D176" t="s">
-        <v>338</v>
+        <v>340</v>
       </c>
       <c r="E176">
         <v>1</v>
@@ -5158,16 +5184,16 @@
     </row>
     <row r="177" spans="1:5">
       <c r="A177" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B177" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C177" t="s">
-        <v>171</v>
+        <v>174</v>
       </c>
       <c r="D177" t="s">
-        <v>338</v>
+        <v>264</v>
       </c>
       <c r="E177">
         <v>1</v>
@@ -5181,10 +5207,10 @@
         <v>40</v>
       </c>
       <c r="C178" t="s">
-        <v>172</v>
+        <v>175</v>
       </c>
       <c r="D178" t="s">
-        <v>339</v>
+        <v>341</v>
       </c>
       <c r="E178">
         <v>1</v>
@@ -5198,10 +5224,10 @@
         <v>40</v>
       </c>
       <c r="C179" t="s">
-        <v>173</v>
+        <v>176</v>
       </c>
       <c r="D179" t="s">
-        <v>340</v>
+        <v>342</v>
       </c>
       <c r="E179">
         <v>1</v>
@@ -5215,10 +5241,10 @@
         <v>40</v>
       </c>
       <c r="C180" t="s">
-        <v>174</v>
+        <v>177</v>
       </c>
       <c r="D180" t="s">
-        <v>264</v>
+        <v>343</v>
       </c>
       <c r="E180">
         <v>1</v>
@@ -5232,10 +5258,10 @@
         <v>40</v>
       </c>
       <c r="C181" t="s">
-        <v>175</v>
+        <v>178</v>
       </c>
       <c r="D181" t="s">
-        <v>341</v>
+        <v>344</v>
       </c>
       <c r="E181">
         <v>1</v>
@@ -5249,10 +5275,10 @@
         <v>40</v>
       </c>
       <c r="C182" t="s">
-        <v>176</v>
+        <v>179</v>
       </c>
       <c r="D182" t="s">
-        <v>342</v>
+        <v>345</v>
       </c>
       <c r="E182">
         <v>1</v>
@@ -5266,10 +5292,10 @@
         <v>40</v>
       </c>
       <c r="C183" t="s">
-        <v>177</v>
+        <v>180</v>
       </c>
       <c r="D183" t="s">
-        <v>343</v>
+        <v>346</v>
       </c>
       <c r="E183">
         <v>1</v>
@@ -5283,10 +5309,10 @@
         <v>40</v>
       </c>
       <c r="C184" t="s">
-        <v>178</v>
+        <v>181</v>
       </c>
       <c r="D184" t="s">
-        <v>344</v>
+        <v>347</v>
       </c>
       <c r="E184">
         <v>1</v>
@@ -5300,10 +5326,10 @@
         <v>40</v>
       </c>
       <c r="C185" t="s">
-        <v>179</v>
+        <v>182</v>
       </c>
       <c r="D185" t="s">
-        <v>345</v>
+        <v>348</v>
       </c>
       <c r="E185">
         <v>1</v>
@@ -5317,10 +5343,10 @@
         <v>40</v>
       </c>
       <c r="C186" t="s">
-        <v>180</v>
+        <v>183</v>
       </c>
       <c r="D186" t="s">
-        <v>346</v>
+        <v>349</v>
       </c>
       <c r="E186">
         <v>1</v>
@@ -5334,10 +5360,10 @@
         <v>40</v>
       </c>
       <c r="C187" t="s">
-        <v>181</v>
+        <v>184</v>
       </c>
       <c r="D187" t="s">
-        <v>347</v>
+        <v>350</v>
       </c>
       <c r="E187">
         <v>1</v>
@@ -5351,10 +5377,10 @@
         <v>40</v>
       </c>
       <c r="C188" t="s">
-        <v>182</v>
+        <v>185</v>
       </c>
       <c r="D188" t="s">
-        <v>348</v>
+        <v>351</v>
       </c>
       <c r="E188">
         <v>1</v>
@@ -5368,10 +5394,10 @@
         <v>40</v>
       </c>
       <c r="C189" t="s">
-        <v>183</v>
+        <v>186</v>
       </c>
       <c r="D189" t="s">
-        <v>349</v>
+        <v>352</v>
       </c>
       <c r="E189">
         <v>1</v>
@@ -5385,10 +5411,10 @@
         <v>40</v>
       </c>
       <c r="C190" t="s">
-        <v>184</v>
+        <v>187</v>
       </c>
       <c r="D190" t="s">
-        <v>350</v>
+        <v>353</v>
       </c>
       <c r="E190">
         <v>1</v>
@@ -5402,10 +5428,10 @@
         <v>40</v>
       </c>
       <c r="C191" t="s">
-        <v>185</v>
+        <v>188</v>
       </c>
       <c r="D191" t="s">
-        <v>351</v>
+        <v>354</v>
       </c>
       <c r="E191">
         <v>1</v>
@@ -5419,10 +5445,10 @@
         <v>40</v>
       </c>
       <c r="C192" t="s">
-        <v>186</v>
+        <v>189</v>
       </c>
       <c r="D192" t="s">
-        <v>352</v>
+        <v>355</v>
       </c>
       <c r="E192">
         <v>1</v>
@@ -5436,10 +5462,10 @@
         <v>40</v>
       </c>
       <c r="C193" t="s">
-        <v>187</v>
+        <v>190</v>
       </c>
       <c r="D193" t="s">
-        <v>353</v>
+        <v>356</v>
       </c>
       <c r="E193">
         <v>1</v>
@@ -5453,10 +5479,10 @@
         <v>40</v>
       </c>
       <c r="C194" t="s">
-        <v>188</v>
+        <v>191</v>
       </c>
       <c r="D194" t="s">
-        <v>354</v>
+        <v>357</v>
       </c>
       <c r="E194">
         <v>1</v>
@@ -5470,10 +5496,10 @@
         <v>40</v>
       </c>
       <c r="C195" t="s">
-        <v>189</v>
+        <v>192</v>
       </c>
       <c r="D195" t="s">
-        <v>355</v>
+        <v>358</v>
       </c>
       <c r="E195">
         <v>1</v>
@@ -5487,10 +5513,10 @@
         <v>40</v>
       </c>
       <c r="C196" t="s">
-        <v>190</v>
+        <v>193</v>
       </c>
       <c r="D196" t="s">
-        <v>356</v>
+        <v>359</v>
       </c>
       <c r="E196">
         <v>1</v>
@@ -5504,10 +5530,10 @@
         <v>40</v>
       </c>
       <c r="C197" t="s">
-        <v>191</v>
+        <v>194</v>
       </c>
       <c r="D197" t="s">
-        <v>357</v>
+        <v>360</v>
       </c>
       <c r="E197">
         <v>1</v>
@@ -5521,10 +5547,10 @@
         <v>40</v>
       </c>
       <c r="C198" t="s">
-        <v>192</v>
+        <v>195</v>
       </c>
       <c r="D198" t="s">
-        <v>358</v>
+        <v>361</v>
       </c>
       <c r="E198">
         <v>1</v>
@@ -5538,10 +5564,10 @@
         <v>40</v>
       </c>
       <c r="C199" t="s">
-        <v>193</v>
+        <v>196</v>
       </c>
       <c r="D199" t="s">
-        <v>359</v>
+        <v>362</v>
       </c>
       <c r="E199">
         <v>1</v>
@@ -5555,10 +5581,10 @@
         <v>40</v>
       </c>
       <c r="C200" t="s">
-        <v>194</v>
+        <v>197</v>
       </c>
       <c r="D200" t="s">
-        <v>360</v>
+        <v>363</v>
       </c>
       <c r="E200">
         <v>1</v>
@@ -5572,10 +5598,10 @@
         <v>40</v>
       </c>
       <c r="C201" t="s">
-        <v>195</v>
+        <v>198</v>
       </c>
       <c r="D201" t="s">
-        <v>361</v>
+        <v>364</v>
       </c>
       <c r="E201">
         <v>1</v>
@@ -5589,10 +5615,10 @@
         <v>40</v>
       </c>
       <c r="C202" t="s">
-        <v>196</v>
+        <v>199</v>
       </c>
       <c r="D202" t="s">
-        <v>362</v>
+        <v>365</v>
       </c>
       <c r="E202">
         <v>1</v>
@@ -5606,13 +5632,13 @@
         <v>40</v>
       </c>
       <c r="C203" t="s">
-        <v>197</v>
+        <v>200</v>
       </c>
       <c r="D203" t="s">
-        <v>363</v>
+        <v>366</v>
       </c>
       <c r="E203">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="204" spans="1:5">
@@ -5623,13 +5649,13 @@
         <v>40</v>
       </c>
       <c r="C204" t="s">
-        <v>198</v>
+        <v>201</v>
       </c>
       <c r="D204" t="s">
-        <v>364</v>
+        <v>367</v>
       </c>
       <c r="E204">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="205" spans="1:5">
@@ -5640,13 +5666,13 @@
         <v>40</v>
       </c>
       <c r="C205" t="s">
-        <v>199</v>
+        <v>202</v>
       </c>
       <c r="D205" t="s">
-        <v>365</v>
+        <v>368</v>
       </c>
       <c r="E205">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="206" spans="1:5">
@@ -5657,10 +5683,10 @@
         <v>40</v>
       </c>
       <c r="C206" t="s">
-        <v>200</v>
+        <v>203</v>
       </c>
       <c r="D206" t="s">
-        <v>366</v>
+        <v>369</v>
       </c>
       <c r="E206">
         <v>2</v>
@@ -5674,10 +5700,10 @@
         <v>40</v>
       </c>
       <c r="C207" t="s">
-        <v>201</v>
+        <v>204</v>
       </c>
       <c r="D207" t="s">
-        <v>367</v>
+        <v>370</v>
       </c>
       <c r="E207">
         <v>2</v>
@@ -5691,10 +5717,10 @@
         <v>40</v>
       </c>
       <c r="C208" t="s">
-        <v>202</v>
+        <v>205</v>
       </c>
       <c r="D208" t="s">
-        <v>368</v>
+        <v>371</v>
       </c>
       <c r="E208">
         <v>2</v>
@@ -5708,10 +5734,10 @@
         <v>40</v>
       </c>
       <c r="C209" t="s">
-        <v>203</v>
+        <v>206</v>
       </c>
       <c r="D209" t="s">
-        <v>369</v>
+        <v>372</v>
       </c>
       <c r="E209">
         <v>2</v>
@@ -5725,10 +5751,10 @@
         <v>40</v>
       </c>
       <c r="C210" t="s">
-        <v>204</v>
+        <v>207</v>
       </c>
       <c r="D210" t="s">
-        <v>370</v>
+        <v>373</v>
       </c>
       <c r="E210">
         <v>2</v>
@@ -5742,10 +5768,10 @@
         <v>40</v>
       </c>
       <c r="C211" t="s">
-        <v>205</v>
+        <v>208</v>
       </c>
       <c r="D211" t="s">
-        <v>371</v>
+        <v>373</v>
       </c>
       <c r="E211">
         <v>2</v>
@@ -5759,10 +5785,10 @@
         <v>40</v>
       </c>
       <c r="C212" t="s">
-        <v>206</v>
+        <v>209</v>
       </c>
       <c r="D212" t="s">
-        <v>372</v>
+        <v>374</v>
       </c>
       <c r="E212">
         <v>2</v>
@@ -5776,10 +5802,10 @@
         <v>40</v>
       </c>
       <c r="C213" t="s">
-        <v>207</v>
+        <v>210</v>
       </c>
       <c r="D213" t="s">
-        <v>373</v>
+        <v>375</v>
       </c>
       <c r="E213">
         <v>2</v>
@@ -5793,10 +5819,10 @@
         <v>40</v>
       </c>
       <c r="C214" t="s">
-        <v>208</v>
+        <v>211</v>
       </c>
       <c r="D214" t="s">
-        <v>373</v>
+        <v>376</v>
       </c>
       <c r="E214">
         <v>2</v>
@@ -5810,13 +5836,13 @@
         <v>40</v>
       </c>
       <c r="C215" t="s">
-        <v>209</v>
+        <v>212</v>
       </c>
       <c r="D215" t="s">
-        <v>374</v>
+        <v>377</v>
       </c>
       <c r="E215">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="216" spans="1:5">
@@ -5827,13 +5853,13 @@
         <v>40</v>
       </c>
       <c r="C216" t="s">
-        <v>210</v>
+        <v>213</v>
       </c>
       <c r="D216" t="s">
-        <v>375</v>
+        <v>264</v>
       </c>
       <c r="E216">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="217" spans="1:5">
@@ -5844,13 +5870,13 @@
         <v>40</v>
       </c>
       <c r="C217" t="s">
-        <v>211</v>
+        <v>214</v>
       </c>
       <c r="D217" t="s">
-        <v>376</v>
+        <v>378</v>
       </c>
       <c r="E217">
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
     <row r="218" spans="1:5">
@@ -5861,13 +5887,13 @@
         <v>40</v>
       </c>
       <c r="C218" t="s">
-        <v>212</v>
+        <v>215</v>
       </c>
       <c r="D218" t="s">
-        <v>377</v>
+        <v>379</v>
       </c>
       <c r="E218">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="219" spans="1:5">
@@ -5878,13 +5904,13 @@
         <v>40</v>
       </c>
       <c r="C219" t="s">
-        <v>213</v>
+        <v>216</v>
       </c>
       <c r="D219" t="s">
-        <v>264</v>
+        <v>380</v>
       </c>
       <c r="E219">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="220" spans="1:5">
@@ -5895,10 +5921,10 @@
         <v>40</v>
       </c>
       <c r="C220" t="s">
-        <v>214</v>
+        <v>217</v>
       </c>
       <c r="D220" t="s">
-        <v>378</v>
+        <v>381</v>
       </c>
       <c r="E220">
         <v>4</v>
@@ -5912,10 +5938,10 @@
         <v>40</v>
       </c>
       <c r="C221" t="s">
-        <v>215</v>
+        <v>218</v>
       </c>
       <c r="D221" t="s">
-        <v>379</v>
+        <v>382</v>
       </c>
       <c r="E221">
         <v>4</v>
@@ -5929,13 +5955,13 @@
         <v>40</v>
       </c>
       <c r="C222" t="s">
-        <v>216</v>
+        <v>219</v>
       </c>
       <c r="D222" t="s">
-        <v>380</v>
+        <v>383</v>
       </c>
       <c r="E222">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="223" spans="1:5">
@@ -5946,13 +5972,13 @@
         <v>40</v>
       </c>
       <c r="C223" t="s">
-        <v>217</v>
+        <v>220</v>
       </c>
       <c r="D223" t="s">
-        <v>381</v>
+        <v>384</v>
       </c>
       <c r="E223">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="224" spans="1:5">
@@ -5963,13 +5989,13 @@
         <v>40</v>
       </c>
       <c r="C224" t="s">
-        <v>218</v>
+        <v>221</v>
       </c>
       <c r="D224" t="s">
-        <v>382</v>
+        <v>385</v>
       </c>
       <c r="E224">
-        <v>4</v>
+        <v>6</v>
       </c>
     </row>
     <row r="225" spans="1:5">
@@ -5980,13 +6006,13 @@
         <v>40</v>
       </c>
       <c r="C225" t="s">
-        <v>219</v>
+        <v>222</v>
       </c>
       <c r="D225" t="s">
-        <v>383</v>
+        <v>386</v>
       </c>
       <c r="E225">
-        <v>5</v>
+        <v>8</v>
       </c>
     </row>
     <row r="226" spans="1:5">
@@ -5997,13 +6023,13 @@
         <v>40</v>
       </c>
       <c r="C226" t="s">
-        <v>220</v>
+        <v>223</v>
       </c>
       <c r="D226" t="s">
-        <v>384</v>
+        <v>387</v>
       </c>
       <c r="E226">
-        <v>5</v>
+        <v>10</v>
       </c>
     </row>
     <row r="227" spans="1:5">
@@ -6014,13 +6040,13 @@
         <v>40</v>
       </c>
       <c r="C227" t="s">
-        <v>221</v>
+        <v>224</v>
       </c>
       <c r="D227" t="s">
-        <v>385</v>
+        <v>387</v>
       </c>
       <c r="E227">
-        <v>6</v>
+        <v>10</v>
       </c>
     </row>
     <row r="228" spans="1:5">
@@ -6031,13 +6057,13 @@
         <v>40</v>
       </c>
       <c r="C228" t="s">
-        <v>222</v>
+        <v>225</v>
       </c>
       <c r="D228" t="s">
-        <v>386</v>
+        <v>266</v>
       </c>
       <c r="E228">
-        <v>8</v>
+        <v>12</v>
       </c>
     </row>
     <row r="229" spans="1:5">
@@ -6048,13 +6074,13 @@
         <v>40</v>
       </c>
       <c r="C229" t="s">
-        <v>223</v>
+        <v>226</v>
       </c>
       <c r="D229" t="s">
-        <v>387</v>
+        <v>388</v>
       </c>
       <c r="E229">
-        <v>10</v>
+        <v>12</v>
       </c>
     </row>
     <row r="230" spans="1:5">
@@ -6065,13 +6091,13 @@
         <v>40</v>
       </c>
       <c r="C230" t="s">
-        <v>224</v>
+        <v>227</v>
       </c>
       <c r="D230" t="s">
-        <v>387</v>
+        <v>389</v>
       </c>
       <c r="E230">
-        <v>10</v>
+        <v>14</v>
       </c>
     </row>
     <row r="231" spans="1:5">
@@ -6082,13 +6108,13 @@
         <v>40</v>
       </c>
       <c r="C231" t="s">
-        <v>225</v>
+        <v>228</v>
       </c>
       <c r="D231" t="s">
-        <v>266</v>
+        <v>390</v>
       </c>
       <c r="E231">
-        <v>12</v>
+        <v>15</v>
       </c>
     </row>
     <row r="232" spans="1:5">
@@ -6099,114 +6125,80 @@
         <v>40</v>
       </c>
       <c r="C232" t="s">
-        <v>226</v>
+        <v>229</v>
       </c>
       <c r="D232" t="s">
-        <v>388</v>
+        <v>391</v>
       </c>
       <c r="E232">
-        <v>12</v>
+        <v>20</v>
       </c>
     </row>
     <row r="233" spans="1:5">
       <c r="A233" t="s">
-        <v>14</v>
+        <v>10</v>
       </c>
       <c r="B233" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="C233" t="s">
-        <v>227</v>
+        <v>230</v>
       </c>
       <c r="D233" t="s">
-        <v>389</v>
+        <v>392</v>
       </c>
       <c r="E233">
-        <v>14</v>
+        <v>1</v>
       </c>
     </row>
     <row r="234" spans="1:5">
       <c r="A234" t="s">
-        <v>14</v>
+        <v>6</v>
       </c>
       <c r="B234" t="s">
-        <v>40</v>
+        <v>36</v>
       </c>
       <c r="C234" t="s">
-        <v>228</v>
+        <v>231</v>
       </c>
       <c r="D234" t="s">
-        <v>390</v>
+        <v>393</v>
       </c>
       <c r="E234">
-        <v>15</v>
+        <v>1</v>
       </c>
     </row>
     <row r="235" spans="1:5">
       <c r="A235" t="s">
-        <v>14</v>
+        <v>10</v>
       </c>
       <c r="B235" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="C235" t="s">
-        <v>229</v>
+        <v>232</v>
       </c>
       <c r="D235" t="s">
-        <v>391</v>
+        <v>394</v>
       </c>
       <c r="E235">
-        <v>20</v>
+        <v>1</v>
       </c>
     </row>
     <row r="236" spans="1:5">
       <c r="A236" t="s">
-        <v>10</v>
+        <v>15</v>
       </c>
       <c r="B236" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="C236" t="s">
-        <v>230</v>
+        <v>232</v>
       </c>
       <c r="D236" t="s">
-        <v>392</v>
+        <v>394</v>
       </c>
       <c r="E236">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="237" spans="1:5">
-      <c r="A237" t="s">
-        <v>6</v>
-      </c>
-      <c r="B237" t="s">
-        <v>36</v>
-      </c>
-      <c r="C237" t="s">
-        <v>231</v>
-      </c>
-      <c r="D237" t="s">
-        <v>393</v>
-      </c>
-      <c r="E237">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="238" spans="1:5">
-      <c r="A238" t="s">
-        <v>10</v>
-      </c>
-      <c r="B238" t="s">
-        <v>39</v>
-      </c>
-      <c r="C238" t="s">
-        <v>232</v>
-      </c>
-      <c r="D238" t="s">
-        <v>394</v>
-      </c>
-      <c r="E238">
         <v>1</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualização automática: rac (21/09/2026 13:59)
</commit_message>
<xml_diff>
--- a/Coordenadoria/02_Dados_Tratados/base_rac_tratada.xlsx
+++ b/Coordenadoria/02_Dados_Tratados/base_rac_tratada.xlsx
@@ -1206,16 +1206,8 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <fonts count="2">
+  <fonts count="1">
     <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -1231,7 +1223,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -1239,30 +1231,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color auto="1"/>
-      </left>
-      <right style="thin">
-        <color auto="1"/>
-      </right>
-      <top style="thin">
-        <color auto="1"/>
-      </top>
-      <bottom style="thin">
-        <color auto="1"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1561,22 +1535,22 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:6">
-      <c r="A1" s="1" t="s">
+      <c r="A1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" s="1" t="s">
+      <c r="B1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" t="s">
         <v>5</v>
       </c>
     </row>
@@ -2191,19 +2165,19 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:5">
-      <c r="A1" s="1" t="s">
+      <c r="A1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" s="1" t="s">
+      <c r="B1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" t="s">
         <v>55</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" t="s">
         <v>56</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" t="s">
         <v>57</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualização automática: rac (21/09/2026 14:29)
</commit_message>
<xml_diff>
--- a/Coordenadoria/02_Dados_Tratados/base_rac_tratada.xlsx
+++ b/Coordenadoria/02_Dados_Tratados/base_rac_tratada.xlsx
@@ -1206,8 +1206,16 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <fonts count="1">
+  <fonts count="2">
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -1223,7 +1231,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -1231,12 +1239,30 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1535,22 +1561,22 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:6">
-      <c r="A1" t="s">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" t="s">
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" t="s">
+      <c r="F1" s="1" t="s">
         <v>5</v>
       </c>
     </row>
@@ -2165,19 +2191,19 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:5">
-      <c r="A1" t="s">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" t="s">
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
         <v>55</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>56</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="1" t="s">
         <v>57</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualização automática: rac (22/09/2026 12:29)
</commit_message>
<xml_diff>
--- a/Coordenadoria/02_Dados_Tratados/base_rac_tratada.xlsx
+++ b/Coordenadoria/02_Dados_Tratados/base_rac_tratada.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1071" uniqueCount="395">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1059" uniqueCount="393">
   <si>
     <t>matricula</t>
   </si>
@@ -707,15 +707,12 @@
     <t>2670067-1</t>
   </si>
   <si>
-    <t>3122678-04</t>
-  </si>
-  <si>
-    <t>060-0017-00</t>
-  </si>
-  <si>
     <t>3034792</t>
   </si>
   <si>
+    <t>CM2022-1</t>
+  </si>
+  <si>
     <t>HOUSING</t>
   </si>
   <si>
@@ -1193,29 +1190,18 @@
     <t>POST LIGHT ASS</t>
   </si>
   <si>
-    <t>FUEL CONTROL UNIT</t>
-  </si>
-  <si>
-    <t>FLIGHT DIR HOR</t>
-  </si>
-  <si>
     <t>FUEL PUMP</t>
+  </si>
+  <si>
+    <t>SEAL</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <fonts count="2">
+  <fonts count="1">
     <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -1231,7 +1217,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -1239,30 +1225,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color auto="1"/>
-      </left>
-      <right style="thin">
-        <color auto="1"/>
-      </right>
-      <top style="thin">
-        <color auto="1"/>
-      </top>
-      <bottom style="thin">
-        <color auto="1"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1561,22 +1529,22 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:6">
-      <c r="A1" s="1" t="s">
+      <c r="A1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" s="1" t="s">
+      <c r="B1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" t="s">
         <v>5</v>
       </c>
     </row>
@@ -1594,10 +1562,10 @@
         <v>53</v>
       </c>
       <c r="E2">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F2">
-        <v>6</v>
+        <v>5</v>
       </c>
     </row>
     <row r="3" spans="1:6">
@@ -1674,10 +1642,10 @@
         <v>54</v>
       </c>
       <c r="E6">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="F6">
-        <v>7</v>
+        <v>4</v>
       </c>
     </row>
     <row r="7" spans="1:6">
@@ -1694,10 +1662,10 @@
         <v>53</v>
       </c>
       <c r="E7">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="F7">
-        <v>51</v>
+        <v>55</v>
       </c>
     </row>
     <row r="8" spans="1:6">
@@ -1774,10 +1742,10 @@
         <v>53</v>
       </c>
       <c r="E11">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F11">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="12" spans="1:6">
@@ -2187,23 +2155,23 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E236"/>
+  <dimension ref="A1:E233"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:5">
-      <c r="A1" s="1" t="s">
+      <c r="A1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" s="1" t="s">
+      <c r="B1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" t="s">
         <v>55</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" t="s">
         <v>56</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" t="s">
         <v>57</v>
       </c>
     </row>
@@ -2218,7 +2186,7 @@
         <v>58</v>
       </c>
       <c r="D2" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
       <c r="E2">
         <v>1</v>
@@ -2235,7 +2203,7 @@
         <v>59</v>
       </c>
       <c r="D3" t="s">
-        <v>234</v>
+        <v>233</v>
       </c>
       <c r="E3">
         <v>1</v>
@@ -2252,7 +2220,7 @@
         <v>60</v>
       </c>
       <c r="D4" t="s">
-        <v>235</v>
+        <v>234</v>
       </c>
       <c r="E4">
         <v>1</v>
@@ -2269,7 +2237,7 @@
         <v>61</v>
       </c>
       <c r="D5" t="s">
-        <v>236</v>
+        <v>235</v>
       </c>
       <c r="E5">
         <v>1</v>
@@ -2286,7 +2254,7 @@
         <v>62</v>
       </c>
       <c r="D6" t="s">
-        <v>237</v>
+        <v>236</v>
       </c>
       <c r="E6">
         <v>1</v>
@@ -2303,7 +2271,7 @@
         <v>63</v>
       </c>
       <c r="D7" t="s">
-        <v>238</v>
+        <v>237</v>
       </c>
       <c r="E7">
         <v>1</v>
@@ -2320,7 +2288,7 @@
         <v>63</v>
       </c>
       <c r="D8" t="s">
-        <v>238</v>
+        <v>237</v>
       </c>
       <c r="E8">
         <v>1</v>
@@ -2337,7 +2305,7 @@
         <v>63</v>
       </c>
       <c r="D9" t="s">
-        <v>238</v>
+        <v>237</v>
       </c>
       <c r="E9">
         <v>1</v>
@@ -2354,7 +2322,7 @@
         <v>63</v>
       </c>
       <c r="D10" t="s">
-        <v>238</v>
+        <v>237</v>
       </c>
       <c r="E10">
         <v>1</v>
@@ -2371,7 +2339,7 @@
         <v>63</v>
       </c>
       <c r="D11" t="s">
-        <v>238</v>
+        <v>237</v>
       </c>
       <c r="E11">
         <v>1</v>
@@ -2388,7 +2356,7 @@
         <v>63</v>
       </c>
       <c r="D12" t="s">
-        <v>238</v>
+        <v>237</v>
       </c>
       <c r="E12">
         <v>1</v>
@@ -2405,7 +2373,7 @@
         <v>63</v>
       </c>
       <c r="D13" t="s">
-        <v>238</v>
+        <v>237</v>
       </c>
       <c r="E13">
         <v>1</v>
@@ -2422,7 +2390,7 @@
         <v>63</v>
       </c>
       <c r="D14" t="s">
-        <v>238</v>
+        <v>237</v>
       </c>
       <c r="E14">
         <v>1</v>
@@ -2439,7 +2407,7 @@
         <v>64</v>
       </c>
       <c r="D15" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
       <c r="E15">
         <v>1</v>
@@ -2456,7 +2424,7 @@
         <v>64</v>
       </c>
       <c r="D16" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
       <c r="E16">
         <v>2</v>
@@ -2473,7 +2441,7 @@
         <v>65</v>
       </c>
       <c r="D17" t="s">
-        <v>240</v>
+        <v>239</v>
       </c>
       <c r="E17">
         <v>1</v>
@@ -2490,7 +2458,7 @@
         <v>65</v>
       </c>
       <c r="D18" t="s">
-        <v>240</v>
+        <v>239</v>
       </c>
       <c r="E18">
         <v>1</v>
@@ -2507,7 +2475,7 @@
         <v>65</v>
       </c>
       <c r="D19" t="s">
-        <v>240</v>
+        <v>239</v>
       </c>
       <c r="E19">
         <v>1</v>
@@ -2524,7 +2492,7 @@
         <v>65</v>
       </c>
       <c r="D20" t="s">
-        <v>240</v>
+        <v>239</v>
       </c>
       <c r="E20">
         <v>1</v>
@@ -2541,7 +2509,7 @@
         <v>65</v>
       </c>
       <c r="D21" t="s">
-        <v>240</v>
+        <v>239</v>
       </c>
       <c r="E21">
         <v>1</v>
@@ -2558,7 +2526,7 @@
         <v>65</v>
       </c>
       <c r="D22" t="s">
-        <v>240</v>
+        <v>239</v>
       </c>
       <c r="E22">
         <v>1</v>
@@ -2575,7 +2543,7 @@
         <v>66</v>
       </c>
       <c r="D23" t="s">
-        <v>241</v>
+        <v>240</v>
       </c>
       <c r="E23">
         <v>1</v>
@@ -2592,7 +2560,7 @@
         <v>66</v>
       </c>
       <c r="D24" t="s">
-        <v>241</v>
+        <v>240</v>
       </c>
       <c r="E24">
         <v>1</v>
@@ -2609,7 +2577,7 @@
         <v>67</v>
       </c>
       <c r="D25" t="s">
-        <v>242</v>
+        <v>241</v>
       </c>
       <c r="E25">
         <v>1</v>
@@ -2626,7 +2594,7 @@
         <v>67</v>
       </c>
       <c r="D26" t="s">
-        <v>242</v>
+        <v>241</v>
       </c>
       <c r="E26">
         <v>1</v>
@@ -2643,7 +2611,7 @@
         <v>68</v>
       </c>
       <c r="D27" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
       <c r="E27">
         <v>1</v>
@@ -2660,7 +2628,7 @@
         <v>68</v>
       </c>
       <c r="D28" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
       <c r="E28">
         <v>1</v>
@@ -2668,13 +2636,13 @@
     </row>
     <row r="29" spans="1:5">
       <c r="A29" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="B29" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="C29" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="D29" t="s">
         <v>243</v>
@@ -2685,24 +2653,24 @@
     </row>
     <row r="30" spans="1:5">
       <c r="A30" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B30" t="s">
         <v>39</v>
       </c>
       <c r="C30" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="D30" t="s">
         <v>244</v>
       </c>
       <c r="E30">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="31" spans="1:5">
       <c r="A31" t="s">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="B31" t="s">
         <v>39</v>
@@ -2711,7 +2679,7 @@
         <v>70</v>
       </c>
       <c r="D31" t="s">
-        <v>245</v>
+        <v>244</v>
       </c>
       <c r="E31">
         <v>2</v>
@@ -2719,50 +2687,50 @@
     </row>
     <row r="32" spans="1:5">
       <c r="A32" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B32" t="s">
-        <v>39</v>
+        <v>36</v>
       </c>
       <c r="C32" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="D32" t="s">
         <v>245</v>
       </c>
       <c r="E32">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="33" spans="1:5">
       <c r="A33" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B33" t="s">
         <v>39</v>
       </c>
       <c r="C33" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="D33" t="s">
         <v>245</v>
       </c>
       <c r="E33">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="34" spans="1:5">
       <c r="A34" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="B34" t="s">
-        <v>36</v>
+        <v>39</v>
       </c>
       <c r="C34" t="s">
         <v>71</v>
       </c>
       <c r="D34" t="s">
-        <v>246</v>
+        <v>245</v>
       </c>
       <c r="E34">
         <v>1</v>
@@ -2770,13 +2738,13 @@
     </row>
     <row r="35" spans="1:5">
       <c r="A35" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B35" t="s">
-        <v>39</v>
+        <v>36</v>
       </c>
       <c r="C35" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="D35" t="s">
         <v>246</v>
@@ -2787,13 +2755,13 @@
     </row>
     <row r="36" spans="1:5">
       <c r="A36" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B36" t="s">
         <v>39</v>
       </c>
       <c r="C36" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="D36" t="s">
         <v>246</v>
@@ -2804,16 +2772,16 @@
     </row>
     <row r="37" spans="1:5">
       <c r="A37" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="B37" t="s">
-        <v>36</v>
+        <v>39</v>
       </c>
       <c r="C37" t="s">
         <v>72</v>
       </c>
       <c r="D37" t="s">
-        <v>247</v>
+        <v>246</v>
       </c>
       <c r="E37">
         <v>1</v>
@@ -2821,13 +2789,13 @@
     </row>
     <row r="38" spans="1:5">
       <c r="A38" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B38" t="s">
-        <v>39</v>
+        <v>36</v>
       </c>
       <c r="C38" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="D38" t="s">
         <v>247</v>
@@ -2838,13 +2806,13 @@
     </row>
     <row r="39" spans="1:5">
       <c r="A39" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B39" t="s">
         <v>39</v>
       </c>
       <c r="C39" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="D39" t="s">
         <v>247</v>
@@ -2861,7 +2829,7 @@
         <v>36</v>
       </c>
       <c r="C40" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="D40" t="s">
         <v>248</v>
@@ -2872,13 +2840,13 @@
     </row>
     <row r="41" spans="1:5">
       <c r="A41" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="B41" t="s">
         <v>39</v>
       </c>
       <c r="C41" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="D41" t="s">
         <v>248</v>
@@ -2889,16 +2857,16 @@
     </row>
     <row r="42" spans="1:5">
       <c r="A42" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="B42" t="s">
-        <v>36</v>
+        <v>40</v>
       </c>
       <c r="C42" t="s">
         <v>74</v>
       </c>
       <c r="D42" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
       <c r="E42">
         <v>1</v>
@@ -2906,13 +2874,13 @@
     </row>
     <row r="43" spans="1:5">
       <c r="A43" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="B43" t="s">
-        <v>39</v>
+        <v>36</v>
       </c>
       <c r="C43" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="D43" t="s">
         <v>249</v>
@@ -2923,16 +2891,16 @@
     </row>
     <row r="44" spans="1:5">
       <c r="A44" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="B44" t="s">
-        <v>40</v>
+        <v>36</v>
       </c>
       <c r="C44" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="D44" t="s">
-        <v>249</v>
+        <v>250</v>
       </c>
       <c r="E44">
         <v>1</v>
@@ -2946,10 +2914,10 @@
         <v>36</v>
       </c>
       <c r="C45" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="D45" t="s">
-        <v>250</v>
+        <v>251</v>
       </c>
       <c r="E45">
         <v>1</v>
@@ -2963,10 +2931,10 @@
         <v>36</v>
       </c>
       <c r="C46" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="D46" t="s">
-        <v>251</v>
+        <v>252</v>
       </c>
       <c r="E46">
         <v>1</v>
@@ -2980,10 +2948,10 @@
         <v>36</v>
       </c>
       <c r="C47" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="D47" t="s">
-        <v>252</v>
+        <v>253</v>
       </c>
       <c r="E47">
         <v>1</v>
@@ -2997,10 +2965,10 @@
         <v>36</v>
       </c>
       <c r="C48" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="D48" t="s">
-        <v>253</v>
+        <v>254</v>
       </c>
       <c r="E48">
         <v>1</v>
@@ -3014,10 +2982,10 @@
         <v>36</v>
       </c>
       <c r="C49" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="D49" t="s">
-        <v>254</v>
+        <v>255</v>
       </c>
       <c r="E49">
         <v>1</v>
@@ -3031,10 +2999,10 @@
         <v>36</v>
       </c>
       <c r="C50" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="D50" t="s">
-        <v>255</v>
+        <v>256</v>
       </c>
       <c r="E50">
         <v>1</v>
@@ -3048,44 +3016,44 @@
         <v>36</v>
       </c>
       <c r="C51" t="s">
-        <v>81</v>
+        <v>83</v>
       </c>
       <c r="D51" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
       <c r="E51">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="52" spans="1:5">
       <c r="A52" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B52" t="s">
-        <v>36</v>
+        <v>39</v>
       </c>
       <c r="C52" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="D52" t="s">
         <v>257</v>
       </c>
       <c r="E52">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="53" spans="1:5">
       <c r="A53" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="B53" t="s">
-        <v>36</v>
+        <v>39</v>
       </c>
       <c r="C53" t="s">
         <v>83</v>
       </c>
       <c r="D53" t="s">
-        <v>258</v>
+        <v>257</v>
       </c>
       <c r="E53">
         <v>2</v>
@@ -3093,30 +3061,30 @@
     </row>
     <row r="54" spans="1:5">
       <c r="A54" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="B54" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="C54" t="s">
         <v>83</v>
       </c>
       <c r="D54" t="s">
-        <v>258</v>
+        <v>257</v>
       </c>
       <c r="E54">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="55" spans="1:5">
       <c r="A55" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="B55" t="s">
-        <v>39</v>
+        <v>36</v>
       </c>
       <c r="C55" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="D55" t="s">
         <v>258</v>
@@ -3127,13 +3095,13 @@
     </row>
     <row r="56" spans="1:5">
       <c r="A56" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B56" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="C56" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="D56" t="s">
         <v>258</v>
@@ -3144,30 +3112,30 @@
     </row>
     <row r="57" spans="1:5">
       <c r="A57" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="B57" t="s">
-        <v>36</v>
+        <v>40</v>
       </c>
       <c r="C57" t="s">
         <v>84</v>
       </c>
       <c r="D57" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="E57">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="58" spans="1:5">
       <c r="A58" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="B58" t="s">
-        <v>39</v>
+        <v>36</v>
       </c>
       <c r="C58" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="D58" t="s">
         <v>259</v>
@@ -3178,33 +3146,33 @@
     </row>
     <row r="59" spans="1:5">
       <c r="A59" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B59" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="C59" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="D59" t="s">
         <v>259</v>
       </c>
       <c r="E59">
-        <v>1</v>
+        <v>4</v>
       </c>
     </row>
     <row r="60" spans="1:5">
       <c r="A60" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="B60" t="s">
-        <v>36</v>
+        <v>40</v>
       </c>
       <c r="C60" t="s">
         <v>85</v>
       </c>
       <c r="D60" t="s">
-        <v>260</v>
+        <v>259</v>
       </c>
       <c r="E60">
         <v>2</v>
@@ -3212,19 +3180,19 @@
     </row>
     <row r="61" spans="1:5">
       <c r="A61" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="B61" t="s">
-        <v>39</v>
+        <v>36</v>
       </c>
       <c r="C61" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="D61" t="s">
         <v>260</v>
       </c>
       <c r="E61">
-        <v>4</v>
+        <v>2</v>
       </c>
     </row>
     <row r="62" spans="1:5">
@@ -3235,13 +3203,13 @@
         <v>40</v>
       </c>
       <c r="C62" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="D62" t="s">
         <v>260</v>
       </c>
       <c r="E62">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="63" spans="1:5">
@@ -3252,7 +3220,7 @@
         <v>36</v>
       </c>
       <c r="C63" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="D63" t="s">
         <v>261</v>
@@ -3263,19 +3231,19 @@
     </row>
     <row r="64" spans="1:5">
       <c r="A64" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="B64" t="s">
-        <v>40</v>
+        <v>36</v>
       </c>
       <c r="C64" t="s">
-        <v>86</v>
+        <v>88</v>
       </c>
       <c r="D64" t="s">
-        <v>261</v>
+        <v>262</v>
       </c>
       <c r="E64">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="65" spans="1:5">
@@ -3286,10 +3254,10 @@
         <v>36</v>
       </c>
       <c r="C65" t="s">
-        <v>87</v>
+        <v>89</v>
       </c>
       <c r="D65" t="s">
-        <v>262</v>
+        <v>263</v>
       </c>
       <c r="E65">
         <v>2</v>
@@ -3303,10 +3271,10 @@
         <v>36</v>
       </c>
       <c r="C66" t="s">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="D66" t="s">
-        <v>263</v>
+        <v>264</v>
       </c>
       <c r="E66">
         <v>2</v>
@@ -3320,10 +3288,10 @@
         <v>36</v>
       </c>
       <c r="C67" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="D67" t="s">
-        <v>264</v>
+        <v>265</v>
       </c>
       <c r="E67">
         <v>2</v>
@@ -3337,10 +3305,10 @@
         <v>36</v>
       </c>
       <c r="C68" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="D68" t="s">
-        <v>265</v>
+        <v>266</v>
       </c>
       <c r="E68">
         <v>2</v>
@@ -3354,10 +3322,10 @@
         <v>36</v>
       </c>
       <c r="C69" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="D69" t="s">
-        <v>266</v>
+        <v>267</v>
       </c>
       <c r="E69">
         <v>2</v>
@@ -3371,10 +3339,10 @@
         <v>36</v>
       </c>
       <c r="C70" t="s">
-        <v>92</v>
+        <v>94</v>
       </c>
       <c r="D70" t="s">
-        <v>267</v>
+        <v>257</v>
       </c>
       <c r="E70">
         <v>2</v>
@@ -3388,30 +3356,30 @@
         <v>36</v>
       </c>
       <c r="C71" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="D71" t="s">
-        <v>268</v>
+        <v>256</v>
       </c>
       <c r="E71">
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
     <row r="72" spans="1:5">
       <c r="A72" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="B72" t="s">
-        <v>36</v>
+        <v>40</v>
       </c>
       <c r="C72" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="D72" t="s">
-        <v>258</v>
+        <v>256</v>
       </c>
       <c r="E72">
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
     <row r="73" spans="1:5">
@@ -3422,10 +3390,10 @@
         <v>36</v>
       </c>
       <c r="C73" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="D73" t="s">
-        <v>257</v>
+        <v>268</v>
       </c>
       <c r="E73">
         <v>4</v>
@@ -3433,16 +3401,16 @@
     </row>
     <row r="74" spans="1:5">
       <c r="A74" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="B74" t="s">
-        <v>40</v>
+        <v>36</v>
       </c>
       <c r="C74" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="D74" t="s">
-        <v>257</v>
+        <v>269</v>
       </c>
       <c r="E74">
         <v>4</v>
@@ -3450,50 +3418,50 @@
     </row>
     <row r="75" spans="1:5">
       <c r="A75" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B75" t="s">
-        <v>36</v>
+        <v>39</v>
       </c>
       <c r="C75" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="D75" t="s">
-        <v>269</v>
+        <v>270</v>
       </c>
       <c r="E75">
-        <v>4</v>
+        <v>1</v>
       </c>
     </row>
     <row r="76" spans="1:5">
       <c r="A76" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="B76" t="s">
-        <v>36</v>
+        <v>39</v>
       </c>
       <c r="C76" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="D76" t="s">
         <v>270</v>
       </c>
       <c r="E76">
-        <v>4</v>
+        <v>1</v>
       </c>
     </row>
     <row r="77" spans="1:5">
       <c r="A77" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="B77" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="C77" t="s">
         <v>98</v>
       </c>
       <c r="D77" t="s">
-        <v>271</v>
+        <v>270</v>
       </c>
       <c r="E77">
         <v>1</v>
@@ -3501,13 +3469,13 @@
     </row>
     <row r="78" spans="1:5">
       <c r="A78" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B78" t="s">
         <v>39</v>
       </c>
       <c r="C78" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="D78" t="s">
         <v>271</v>
@@ -3518,13 +3486,13 @@
     </row>
     <row r="79" spans="1:5">
       <c r="A79" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B79" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="C79" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="D79" t="s">
         <v>271</v>
@@ -3535,30 +3503,30 @@
     </row>
     <row r="80" spans="1:5">
       <c r="A80" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="B80" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="C80" t="s">
         <v>99</v>
       </c>
       <c r="D80" t="s">
-        <v>272</v>
+        <v>271</v>
       </c>
       <c r="E80">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="81" spans="1:5">
       <c r="A81" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B81" t="s">
         <v>39</v>
       </c>
       <c r="C81" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="D81" t="s">
         <v>272</v>
@@ -3569,19 +3537,19 @@
     </row>
     <row r="82" spans="1:5">
       <c r="A82" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B82" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="C82" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="D82" t="s">
         <v>272</v>
       </c>
       <c r="E82">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="83" spans="1:5">
@@ -3592,7 +3560,7 @@
         <v>39</v>
       </c>
       <c r="C83" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="D83" t="s">
         <v>273</v>
@@ -3609,7 +3577,7 @@
         <v>39</v>
       </c>
       <c r="C84" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="D84" t="s">
         <v>273</v>
@@ -3626,7 +3594,7 @@
         <v>39</v>
       </c>
       <c r="C85" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="D85" t="s">
         <v>274</v>
@@ -3643,7 +3611,7 @@
         <v>39</v>
       </c>
       <c r="C86" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="D86" t="s">
         <v>274</v>
@@ -3660,7 +3628,7 @@
         <v>39</v>
       </c>
       <c r="C87" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="D87" t="s">
         <v>275</v>
@@ -3677,7 +3645,7 @@
         <v>39</v>
       </c>
       <c r="C88" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="D88" t="s">
         <v>275</v>
@@ -3694,7 +3662,7 @@
         <v>39</v>
       </c>
       <c r="C89" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="D89" t="s">
         <v>276</v>
@@ -3711,7 +3679,7 @@
         <v>39</v>
       </c>
       <c r="C90" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="D90" t="s">
         <v>276</v>
@@ -3728,7 +3696,7 @@
         <v>39</v>
       </c>
       <c r="C91" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="D91" t="s">
         <v>277</v>
@@ -3739,13 +3707,13 @@
     </row>
     <row r="92" spans="1:5">
       <c r="A92" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="B92" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="C92" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="D92" t="s">
         <v>277</v>
@@ -3762,7 +3730,7 @@
         <v>39</v>
       </c>
       <c r="C93" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="D93" t="s">
         <v>278</v>
@@ -3779,7 +3747,7 @@
         <v>40</v>
       </c>
       <c r="C94" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="D94" t="s">
         <v>278</v>
@@ -3796,7 +3764,7 @@
         <v>39</v>
       </c>
       <c r="C95" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="D95" t="s">
         <v>279</v>
@@ -3813,7 +3781,7 @@
         <v>40</v>
       </c>
       <c r="C96" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="D96" t="s">
         <v>279</v>
@@ -3830,7 +3798,7 @@
         <v>39</v>
       </c>
       <c r="C97" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="D97" t="s">
         <v>280</v>
@@ -3841,16 +3809,16 @@
     </row>
     <row r="98" spans="1:5">
       <c r="A98" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="B98" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="C98" t="s">
-        <v>107</v>
+        <v>109</v>
       </c>
       <c r="D98" t="s">
-        <v>280</v>
+        <v>281</v>
       </c>
       <c r="E98">
         <v>1</v>
@@ -3864,10 +3832,10 @@
         <v>39</v>
       </c>
       <c r="C99" t="s">
-        <v>108</v>
+        <v>110</v>
       </c>
       <c r="D99" t="s">
-        <v>281</v>
+        <v>282</v>
       </c>
       <c r="E99">
         <v>1</v>
@@ -3881,10 +3849,10 @@
         <v>39</v>
       </c>
       <c r="C100" t="s">
-        <v>109</v>
+        <v>111</v>
       </c>
       <c r="D100" t="s">
-        <v>282</v>
+        <v>283</v>
       </c>
       <c r="E100">
         <v>1</v>
@@ -3898,10 +3866,10 @@
         <v>39</v>
       </c>
       <c r="C101" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="D101" t="s">
-        <v>283</v>
+        <v>284</v>
       </c>
       <c r="E101">
         <v>1</v>
@@ -3915,10 +3883,10 @@
         <v>39</v>
       </c>
       <c r="C102" t="s">
-        <v>111</v>
+        <v>113</v>
       </c>
       <c r="D102" t="s">
-        <v>284</v>
+        <v>285</v>
       </c>
       <c r="E102">
         <v>1</v>
@@ -3932,24 +3900,24 @@
         <v>39</v>
       </c>
       <c r="C103" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
       <c r="D103" t="s">
-        <v>285</v>
+        <v>286</v>
       </c>
       <c r="E103">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="104" spans="1:5">
       <c r="A104" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="B104" t="s">
         <v>39</v>
       </c>
       <c r="C104" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="D104" t="s">
         <v>286</v>
@@ -3966,7 +3934,7 @@
         <v>39</v>
       </c>
       <c r="C105" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="D105" t="s">
         <v>287</v>
@@ -3983,27 +3951,27 @@
         <v>39</v>
       </c>
       <c r="C106" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="D106" t="s">
         <v>287</v>
       </c>
       <c r="E106">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="107" spans="1:5">
       <c r="A107" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="B107" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="C107" t="s">
         <v>115</v>
       </c>
       <c r="D107" t="s">
-        <v>288</v>
+        <v>287</v>
       </c>
       <c r="E107">
         <v>2</v>
@@ -4011,13 +3979,13 @@
     </row>
     <row r="108" spans="1:5">
       <c r="A108" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B108" t="s">
         <v>39</v>
       </c>
       <c r="C108" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="D108" t="s">
         <v>288</v>
@@ -4028,13 +3996,13 @@
     </row>
     <row r="109" spans="1:5">
       <c r="A109" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B109" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="C109" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="D109" t="s">
         <v>288</v>
@@ -4045,16 +4013,16 @@
     </row>
     <row r="110" spans="1:5">
       <c r="A110" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="B110" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="C110" t="s">
         <v>116</v>
       </c>
       <c r="D110" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
       <c r="E110">
         <v>2</v>
@@ -4062,13 +4030,13 @@
     </row>
     <row r="111" spans="1:5">
       <c r="A111" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B111" t="s">
         <v>39</v>
       </c>
       <c r="C111" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="D111" t="s">
         <v>289</v>
@@ -4079,13 +4047,13 @@
     </row>
     <row r="112" spans="1:5">
       <c r="A112" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B112" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="C112" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="D112" t="s">
         <v>289</v>
@@ -4102,10 +4070,10 @@
         <v>39</v>
       </c>
       <c r="C113" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="D113" t="s">
-        <v>290</v>
+        <v>271</v>
       </c>
       <c r="E113">
         <v>2</v>
@@ -4119,61 +4087,61 @@
         <v>39</v>
       </c>
       <c r="C114" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="D114" t="s">
-        <v>290</v>
+        <v>271</v>
       </c>
       <c r="E114">
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
     <row r="115" spans="1:5">
       <c r="A115" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="B115" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="C115" t="s">
         <v>118</v>
       </c>
       <c r="D115" t="s">
-        <v>272</v>
+        <v>271</v>
       </c>
       <c r="E115">
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
     <row r="116" spans="1:5">
       <c r="A116" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B116" t="s">
         <v>39</v>
       </c>
       <c r="C116" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="D116" t="s">
-        <v>272</v>
+        <v>290</v>
       </c>
       <c r="E116">
-        <v>4</v>
+        <v>2</v>
       </c>
     </row>
     <row r="117" spans="1:5">
       <c r="A117" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B117" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="C117" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="D117" t="s">
-        <v>272</v>
+        <v>290</v>
       </c>
       <c r="E117">
         <v>4</v>
@@ -4187,10 +4155,10 @@
         <v>39</v>
       </c>
       <c r="C118" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="D118" t="s">
-        <v>291</v>
+        <v>275</v>
       </c>
       <c r="E118">
         <v>2</v>
@@ -4198,19 +4166,19 @@
     </row>
     <row r="119" spans="1:5">
       <c r="A119" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B119" t="s">
         <v>39</v>
       </c>
       <c r="C119" t="s">
-        <v>119</v>
+        <v>121</v>
       </c>
       <c r="D119" t="s">
         <v>291</v>
       </c>
       <c r="E119">
-        <v>4</v>
+        <v>2</v>
       </c>
     </row>
     <row r="120" spans="1:5">
@@ -4221,10 +4189,10 @@
         <v>39</v>
       </c>
       <c r="C120" t="s">
-        <v>120</v>
+        <v>122</v>
       </c>
       <c r="D120" t="s">
-        <v>276</v>
+        <v>292</v>
       </c>
       <c r="E120">
         <v>2</v>
@@ -4238,30 +4206,30 @@
         <v>39</v>
       </c>
       <c r="C121" t="s">
-        <v>121</v>
+        <v>123</v>
       </c>
       <c r="D121" t="s">
-        <v>292</v>
+        <v>293</v>
       </c>
       <c r="E121">
-        <v>2</v>
+        <v>5</v>
       </c>
     </row>
     <row r="122" spans="1:5">
       <c r="A122" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="B122" t="s">
         <v>39</v>
       </c>
       <c r="C122" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="D122" t="s">
         <v>293</v>
       </c>
       <c r="E122">
-        <v>2</v>
+        <v>5</v>
       </c>
     </row>
     <row r="123" spans="1:5">
@@ -4272,30 +4240,30 @@
         <v>39</v>
       </c>
       <c r="C123" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="D123" t="s">
         <v>294</v>
       </c>
       <c r="E123">
-        <v>5</v>
+        <v>7</v>
       </c>
     </row>
     <row r="124" spans="1:5">
       <c r="A124" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B124" t="s">
         <v>39</v>
       </c>
       <c r="C124" t="s">
-        <v>123</v>
+        <v>125</v>
       </c>
       <c r="D124" t="s">
-        <v>294</v>
+        <v>295</v>
       </c>
       <c r="E124">
-        <v>5</v>
+        <v>8</v>
       </c>
     </row>
     <row r="125" spans="1:5">
@@ -4306,13 +4274,13 @@
         <v>39</v>
       </c>
       <c r="C125" t="s">
-        <v>124</v>
+        <v>126</v>
       </c>
       <c r="D125" t="s">
-        <v>295</v>
+        <v>296</v>
       </c>
       <c r="E125">
-        <v>7</v>
+        <v>10</v>
       </c>
     </row>
     <row r="126" spans="1:5">
@@ -4323,64 +4291,64 @@
         <v>39</v>
       </c>
       <c r="C126" t="s">
-        <v>125</v>
+        <v>127</v>
       </c>
       <c r="D126" t="s">
-        <v>296</v>
+        <v>297</v>
       </c>
       <c r="E126">
-        <v>8</v>
+        <v>30</v>
       </c>
     </row>
     <row r="127" spans="1:5">
       <c r="A127" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="B127" t="s">
         <v>39</v>
       </c>
       <c r="C127" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="D127" t="s">
         <v>297</v>
       </c>
       <c r="E127">
-        <v>10</v>
+        <v>30</v>
       </c>
     </row>
     <row r="128" spans="1:5">
       <c r="A128" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="B128" t="s">
         <v>39</v>
       </c>
       <c r="C128" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="D128" t="s">
         <v>298</v>
       </c>
       <c r="E128">
-        <v>30</v>
+        <v>1</v>
       </c>
     </row>
     <row r="129" spans="1:5">
       <c r="A129" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="B129" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="C129" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="D129" t="s">
         <v>298</v>
       </c>
       <c r="E129">
-        <v>30</v>
+        <v>1</v>
       </c>
     </row>
     <row r="130" spans="1:5">
@@ -4391,7 +4359,7 @@
         <v>39</v>
       </c>
       <c r="C130" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="D130" t="s">
         <v>299</v>
@@ -4402,16 +4370,16 @@
     </row>
     <row r="131" spans="1:5">
       <c r="A131" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B131" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="C131" t="s">
-        <v>128</v>
+        <v>130</v>
       </c>
       <c r="D131" t="s">
-        <v>299</v>
+        <v>300</v>
       </c>
       <c r="E131">
         <v>1</v>
@@ -4425,10 +4393,10 @@
         <v>39</v>
       </c>
       <c r="C132" t="s">
-        <v>129</v>
+        <v>131</v>
       </c>
       <c r="D132" t="s">
-        <v>300</v>
+        <v>301</v>
       </c>
       <c r="E132">
         <v>1</v>
@@ -4442,10 +4410,10 @@
         <v>39</v>
       </c>
       <c r="C133" t="s">
-        <v>130</v>
+        <v>132</v>
       </c>
       <c r="D133" t="s">
-        <v>301</v>
+        <v>302</v>
       </c>
       <c r="E133">
         <v>1</v>
@@ -4459,10 +4427,10 @@
         <v>39</v>
       </c>
       <c r="C134" t="s">
-        <v>131</v>
+        <v>133</v>
       </c>
       <c r="D134" t="s">
-        <v>302</v>
+        <v>303</v>
       </c>
       <c r="E134">
         <v>1</v>
@@ -4476,10 +4444,10 @@
         <v>39</v>
       </c>
       <c r="C135" t="s">
-        <v>132</v>
+        <v>134</v>
       </c>
       <c r="D135" t="s">
-        <v>303</v>
+        <v>304</v>
       </c>
       <c r="E135">
         <v>1</v>
@@ -4493,10 +4461,10 @@
         <v>39</v>
       </c>
       <c r="C136" t="s">
-        <v>133</v>
+        <v>135</v>
       </c>
       <c r="D136" t="s">
-        <v>304</v>
+        <v>305</v>
       </c>
       <c r="E136">
         <v>1</v>
@@ -4510,10 +4478,10 @@
         <v>39</v>
       </c>
       <c r="C137" t="s">
-        <v>134</v>
+        <v>136</v>
       </c>
       <c r="D137" t="s">
-        <v>305</v>
+        <v>306</v>
       </c>
       <c r="E137">
         <v>1</v>
@@ -4527,10 +4495,10 @@
         <v>39</v>
       </c>
       <c r="C138" t="s">
-        <v>135</v>
+        <v>137</v>
       </c>
       <c r="D138" t="s">
-        <v>306</v>
+        <v>307</v>
       </c>
       <c r="E138">
         <v>1</v>
@@ -4544,10 +4512,10 @@
         <v>39</v>
       </c>
       <c r="C139" t="s">
-        <v>136</v>
+        <v>138</v>
       </c>
       <c r="D139" t="s">
-        <v>307</v>
+        <v>308</v>
       </c>
       <c r="E139">
         <v>1</v>
@@ -4561,10 +4529,10 @@
         <v>39</v>
       </c>
       <c r="C140" t="s">
-        <v>137</v>
+        <v>139</v>
       </c>
       <c r="D140" t="s">
-        <v>308</v>
+        <v>309</v>
       </c>
       <c r="E140">
         <v>1</v>
@@ -4578,10 +4546,10 @@
         <v>39</v>
       </c>
       <c r="C141" t="s">
-        <v>138</v>
+        <v>140</v>
       </c>
       <c r="D141" t="s">
-        <v>309</v>
+        <v>310</v>
       </c>
       <c r="E141">
         <v>1</v>
@@ -4595,10 +4563,10 @@
         <v>39</v>
       </c>
       <c r="C142" t="s">
-        <v>139</v>
+        <v>141</v>
       </c>
       <c r="D142" t="s">
-        <v>310</v>
+        <v>311</v>
       </c>
       <c r="E142">
         <v>1</v>
@@ -4612,10 +4580,10 @@
         <v>39</v>
       </c>
       <c r="C143" t="s">
-        <v>140</v>
+        <v>142</v>
       </c>
       <c r="D143" t="s">
-        <v>311</v>
+        <v>312</v>
       </c>
       <c r="E143">
         <v>1</v>
@@ -4629,10 +4597,10 @@
         <v>39</v>
       </c>
       <c r="C144" t="s">
-        <v>141</v>
+        <v>143</v>
       </c>
       <c r="D144" t="s">
-        <v>312</v>
+        <v>313</v>
       </c>
       <c r="E144">
         <v>1</v>
@@ -4646,10 +4614,10 @@
         <v>39</v>
       </c>
       <c r="C145" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="D145" t="s">
-        <v>313</v>
+        <v>314</v>
       </c>
       <c r="E145">
         <v>1</v>
@@ -4663,10 +4631,10 @@
         <v>39</v>
       </c>
       <c r="C146" t="s">
-        <v>143</v>
+        <v>145</v>
       </c>
       <c r="D146" t="s">
-        <v>314</v>
+        <v>315</v>
       </c>
       <c r="E146">
         <v>1</v>
@@ -4680,10 +4648,10 @@
         <v>39</v>
       </c>
       <c r="C147" t="s">
-        <v>144</v>
+        <v>146</v>
       </c>
       <c r="D147" t="s">
-        <v>315</v>
+        <v>316</v>
       </c>
       <c r="E147">
         <v>1</v>
@@ -4697,10 +4665,10 @@
         <v>39</v>
       </c>
       <c r="C148" t="s">
-        <v>145</v>
+        <v>147</v>
       </c>
       <c r="D148" t="s">
-        <v>316</v>
+        <v>317</v>
       </c>
       <c r="E148">
         <v>1</v>
@@ -4714,10 +4682,10 @@
         <v>39</v>
       </c>
       <c r="C149" t="s">
-        <v>146</v>
+        <v>148</v>
       </c>
       <c r="D149" t="s">
-        <v>317</v>
+        <v>318</v>
       </c>
       <c r="E149">
         <v>1</v>
@@ -4731,10 +4699,10 @@
         <v>39</v>
       </c>
       <c r="C150" t="s">
-        <v>147</v>
+        <v>149</v>
       </c>
       <c r="D150" t="s">
-        <v>318</v>
+        <v>319</v>
       </c>
       <c r="E150">
         <v>1</v>
@@ -4748,10 +4716,10 @@
         <v>39</v>
       </c>
       <c r="C151" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
       <c r="D151" t="s">
-        <v>319</v>
+        <v>320</v>
       </c>
       <c r="E151">
         <v>1</v>
@@ -4765,10 +4733,10 @@
         <v>39</v>
       </c>
       <c r="C152" t="s">
-        <v>149</v>
+        <v>151</v>
       </c>
       <c r="D152" t="s">
-        <v>320</v>
+        <v>321</v>
       </c>
       <c r="E152">
         <v>1</v>
@@ -4782,10 +4750,10 @@
         <v>39</v>
       </c>
       <c r="C153" t="s">
-        <v>150</v>
+        <v>152</v>
       </c>
       <c r="D153" t="s">
-        <v>321</v>
+        <v>322</v>
       </c>
       <c r="E153">
         <v>1</v>
@@ -4799,10 +4767,10 @@
         <v>39</v>
       </c>
       <c r="C154" t="s">
-        <v>151</v>
+        <v>153</v>
       </c>
       <c r="D154" t="s">
-        <v>322</v>
+        <v>323</v>
       </c>
       <c r="E154">
         <v>1</v>
@@ -4816,10 +4784,10 @@
         <v>39</v>
       </c>
       <c r="C155" t="s">
-        <v>152</v>
+        <v>154</v>
       </c>
       <c r="D155" t="s">
-        <v>323</v>
+        <v>324</v>
       </c>
       <c r="E155">
         <v>1</v>
@@ -4833,10 +4801,10 @@
         <v>39</v>
       </c>
       <c r="C156" t="s">
-        <v>153</v>
+        <v>155</v>
       </c>
       <c r="D156" t="s">
-        <v>324</v>
+        <v>325</v>
       </c>
       <c r="E156">
         <v>1</v>
@@ -4850,10 +4818,10 @@
         <v>39</v>
       </c>
       <c r="C157" t="s">
-        <v>154</v>
+        <v>156</v>
       </c>
       <c r="D157" t="s">
-        <v>325</v>
+        <v>326</v>
       </c>
       <c r="E157">
         <v>1</v>
@@ -4867,10 +4835,10 @@
         <v>39</v>
       </c>
       <c r="C158" t="s">
-        <v>155</v>
+        <v>157</v>
       </c>
       <c r="D158" t="s">
-        <v>326</v>
+        <v>327</v>
       </c>
       <c r="E158">
         <v>1</v>
@@ -4884,13 +4852,13 @@
         <v>39</v>
       </c>
       <c r="C159" t="s">
-        <v>156</v>
+        <v>158</v>
       </c>
       <c r="D159" t="s">
-        <v>327</v>
+        <v>312</v>
       </c>
       <c r="E159">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="160" spans="1:5">
@@ -4901,13 +4869,13 @@
         <v>39</v>
       </c>
       <c r="C160" t="s">
-        <v>157</v>
+        <v>159</v>
       </c>
       <c r="D160" t="s">
         <v>328</v>
       </c>
       <c r="E160">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="161" spans="1:5">
@@ -4918,10 +4886,10 @@
         <v>39</v>
       </c>
       <c r="C161" t="s">
-        <v>158</v>
+        <v>160</v>
       </c>
       <c r="D161" t="s">
-        <v>313</v>
+        <v>329</v>
       </c>
       <c r="E161">
         <v>2</v>
@@ -4935,10 +4903,10 @@
         <v>39</v>
       </c>
       <c r="C162" t="s">
-        <v>159</v>
+        <v>161</v>
       </c>
       <c r="D162" t="s">
-        <v>329</v>
+        <v>330</v>
       </c>
       <c r="E162">
         <v>2</v>
@@ -4952,10 +4920,10 @@
         <v>39</v>
       </c>
       <c r="C163" t="s">
-        <v>160</v>
+        <v>162</v>
       </c>
       <c r="D163" t="s">
-        <v>330</v>
+        <v>331</v>
       </c>
       <c r="E163">
         <v>2</v>
@@ -4969,13 +4937,13 @@
         <v>39</v>
       </c>
       <c r="C164" t="s">
-        <v>161</v>
+        <v>163</v>
       </c>
       <c r="D164" t="s">
-        <v>331</v>
+        <v>332</v>
       </c>
       <c r="E164">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="165" spans="1:5">
@@ -4986,13 +4954,13 @@
         <v>39</v>
       </c>
       <c r="C165" t="s">
-        <v>162</v>
+        <v>164</v>
       </c>
       <c r="D165" t="s">
-        <v>332</v>
+        <v>297</v>
       </c>
       <c r="E165">
-        <v>2</v>
+        <v>5</v>
       </c>
     </row>
     <row r="166" spans="1:5">
@@ -5003,13 +4971,13 @@
         <v>39</v>
       </c>
       <c r="C166" t="s">
-        <v>163</v>
+        <v>165</v>
       </c>
       <c r="D166" t="s">
         <v>333</v>
       </c>
       <c r="E166">
-        <v>3</v>
+        <v>8</v>
       </c>
     </row>
     <row r="167" spans="1:5">
@@ -5020,13 +4988,13 @@
         <v>39</v>
       </c>
       <c r="C167" t="s">
-        <v>164</v>
+        <v>166</v>
       </c>
       <c r="D167" t="s">
-        <v>298</v>
+        <v>253</v>
       </c>
       <c r="E167">
-        <v>5</v>
+        <v>8</v>
       </c>
     </row>
     <row r="168" spans="1:5">
@@ -5037,47 +5005,47 @@
         <v>39</v>
       </c>
       <c r="C168" t="s">
-        <v>165</v>
+        <v>167</v>
       </c>
       <c r="D168" t="s">
         <v>334</v>
       </c>
       <c r="E168">
-        <v>8</v>
+        <v>10</v>
       </c>
     </row>
     <row r="169" spans="1:5">
       <c r="A169" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="B169" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="C169" t="s">
-        <v>166</v>
+        <v>168</v>
       </c>
       <c r="D169" t="s">
-        <v>254</v>
+        <v>322</v>
       </c>
       <c r="E169">
-        <v>8</v>
+        <v>1</v>
       </c>
     </row>
     <row r="170" spans="1:5">
       <c r="A170" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="B170" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="C170" t="s">
-        <v>167</v>
+        <v>169</v>
       </c>
       <c r="D170" t="s">
         <v>335</v>
       </c>
       <c r="E170">
-        <v>10</v>
+        <v>1</v>
       </c>
     </row>
     <row r="171" spans="1:5">
@@ -5088,10 +5056,10 @@
         <v>40</v>
       </c>
       <c r="C171" t="s">
-        <v>168</v>
+        <v>170</v>
       </c>
       <c r="D171" t="s">
-        <v>323</v>
+        <v>336</v>
       </c>
       <c r="E171">
         <v>1</v>
@@ -5105,10 +5073,10 @@
         <v>40</v>
       </c>
       <c r="C172" t="s">
-        <v>169</v>
+        <v>171</v>
       </c>
       <c r="D172" t="s">
-        <v>336</v>
+        <v>337</v>
       </c>
       <c r="E172">
         <v>1</v>
@@ -5122,10 +5090,10 @@
         <v>40</v>
       </c>
       <c r="C173" t="s">
-        <v>170</v>
+        <v>172</v>
       </c>
       <c r="D173" t="s">
-        <v>337</v>
+        <v>338</v>
       </c>
       <c r="E173">
         <v>1</v>
@@ -5139,10 +5107,10 @@
         <v>40</v>
       </c>
       <c r="C174" t="s">
-        <v>171</v>
+        <v>173</v>
       </c>
       <c r="D174" t="s">
-        <v>338</v>
+        <v>339</v>
       </c>
       <c r="E174">
         <v>1</v>
@@ -5156,10 +5124,10 @@
         <v>40</v>
       </c>
       <c r="C175" t="s">
-        <v>172</v>
+        <v>174</v>
       </c>
       <c r="D175" t="s">
-        <v>339</v>
+        <v>263</v>
       </c>
       <c r="E175">
         <v>1</v>
@@ -5173,7 +5141,7 @@
         <v>40</v>
       </c>
       <c r="C176" t="s">
-        <v>173</v>
+        <v>175</v>
       </c>
       <c r="D176" t="s">
         <v>340</v>
@@ -5190,10 +5158,10 @@
         <v>40</v>
       </c>
       <c r="C177" t="s">
-        <v>174</v>
+        <v>176</v>
       </c>
       <c r="D177" t="s">
-        <v>264</v>
+        <v>341</v>
       </c>
       <c r="E177">
         <v>1</v>
@@ -5207,10 +5175,10 @@
         <v>40</v>
       </c>
       <c r="C178" t="s">
-        <v>175</v>
+        <v>177</v>
       </c>
       <c r="D178" t="s">
-        <v>341</v>
+        <v>342</v>
       </c>
       <c r="E178">
         <v>1</v>
@@ -5224,10 +5192,10 @@
         <v>40</v>
       </c>
       <c r="C179" t="s">
-        <v>176</v>
+        <v>178</v>
       </c>
       <c r="D179" t="s">
-        <v>342</v>
+        <v>343</v>
       </c>
       <c r="E179">
         <v>1</v>
@@ -5241,10 +5209,10 @@
         <v>40</v>
       </c>
       <c r="C180" t="s">
-        <v>177</v>
+        <v>179</v>
       </c>
       <c r="D180" t="s">
-        <v>343</v>
+        <v>344</v>
       </c>
       <c r="E180">
         <v>1</v>
@@ -5258,10 +5226,10 @@
         <v>40</v>
       </c>
       <c r="C181" t="s">
-        <v>178</v>
+        <v>180</v>
       </c>
       <c r="D181" t="s">
-        <v>344</v>
+        <v>345</v>
       </c>
       <c r="E181">
         <v>1</v>
@@ -5275,10 +5243,10 @@
         <v>40</v>
       </c>
       <c r="C182" t="s">
-        <v>179</v>
+        <v>181</v>
       </c>
       <c r="D182" t="s">
-        <v>345</v>
+        <v>346</v>
       </c>
       <c r="E182">
         <v>1</v>
@@ -5292,10 +5260,10 @@
         <v>40</v>
       </c>
       <c r="C183" t="s">
-        <v>180</v>
+        <v>182</v>
       </c>
       <c r="D183" t="s">
-        <v>346</v>
+        <v>347</v>
       </c>
       <c r="E183">
         <v>1</v>
@@ -5309,10 +5277,10 @@
         <v>40</v>
       </c>
       <c r="C184" t="s">
-        <v>181</v>
+        <v>183</v>
       </c>
       <c r="D184" t="s">
-        <v>347</v>
+        <v>348</v>
       </c>
       <c r="E184">
         <v>1</v>
@@ -5326,10 +5294,10 @@
         <v>40</v>
       </c>
       <c r="C185" t="s">
-        <v>182</v>
+        <v>184</v>
       </c>
       <c r="D185" t="s">
-        <v>348</v>
+        <v>349</v>
       </c>
       <c r="E185">
         <v>1</v>
@@ -5343,10 +5311,10 @@
         <v>40</v>
       </c>
       <c r="C186" t="s">
-        <v>183</v>
+        <v>185</v>
       </c>
       <c r="D186" t="s">
-        <v>349</v>
+        <v>350</v>
       </c>
       <c r="E186">
         <v>1</v>
@@ -5360,10 +5328,10 @@
         <v>40</v>
       </c>
       <c r="C187" t="s">
-        <v>184</v>
+        <v>186</v>
       </c>
       <c r="D187" t="s">
-        <v>350</v>
+        <v>351</v>
       </c>
       <c r="E187">
         <v>1</v>
@@ -5377,10 +5345,10 @@
         <v>40</v>
       </c>
       <c r="C188" t="s">
-        <v>185</v>
+        <v>187</v>
       </c>
       <c r="D188" t="s">
-        <v>351</v>
+        <v>352</v>
       </c>
       <c r="E188">
         <v>1</v>
@@ -5394,10 +5362,10 @@
         <v>40</v>
       </c>
       <c r="C189" t="s">
-        <v>186</v>
+        <v>188</v>
       </c>
       <c r="D189" t="s">
-        <v>352</v>
+        <v>353</v>
       </c>
       <c r="E189">
         <v>1</v>
@@ -5411,10 +5379,10 @@
         <v>40</v>
       </c>
       <c r="C190" t="s">
-        <v>187</v>
+        <v>189</v>
       </c>
       <c r="D190" t="s">
-        <v>353</v>
+        <v>354</v>
       </c>
       <c r="E190">
         <v>1</v>
@@ -5428,10 +5396,10 @@
         <v>40</v>
       </c>
       <c r="C191" t="s">
-        <v>188</v>
+        <v>190</v>
       </c>
       <c r="D191" t="s">
-        <v>354</v>
+        <v>355</v>
       </c>
       <c r="E191">
         <v>1</v>
@@ -5445,10 +5413,10 @@
         <v>40</v>
       </c>
       <c r="C192" t="s">
-        <v>189</v>
+        <v>191</v>
       </c>
       <c r="D192" t="s">
-        <v>355</v>
+        <v>356</v>
       </c>
       <c r="E192">
         <v>1</v>
@@ -5462,10 +5430,10 @@
         <v>40</v>
       </c>
       <c r="C193" t="s">
-        <v>190</v>
+        <v>192</v>
       </c>
       <c r="D193" t="s">
-        <v>356</v>
+        <v>357</v>
       </c>
       <c r="E193">
         <v>1</v>
@@ -5479,10 +5447,10 @@
         <v>40</v>
       </c>
       <c r="C194" t="s">
-        <v>191</v>
+        <v>193</v>
       </c>
       <c r="D194" t="s">
-        <v>357</v>
+        <v>358</v>
       </c>
       <c r="E194">
         <v>1</v>
@@ -5496,10 +5464,10 @@
         <v>40</v>
       </c>
       <c r="C195" t="s">
-        <v>192</v>
+        <v>194</v>
       </c>
       <c r="D195" t="s">
-        <v>358</v>
+        <v>359</v>
       </c>
       <c r="E195">
         <v>1</v>
@@ -5513,10 +5481,10 @@
         <v>40</v>
       </c>
       <c r="C196" t="s">
-        <v>193</v>
+        <v>195</v>
       </c>
       <c r="D196" t="s">
-        <v>359</v>
+        <v>360</v>
       </c>
       <c r="E196">
         <v>1</v>
@@ -5530,10 +5498,10 @@
         <v>40</v>
       </c>
       <c r="C197" t="s">
-        <v>194</v>
+        <v>196</v>
       </c>
       <c r="D197" t="s">
-        <v>360</v>
+        <v>361</v>
       </c>
       <c r="E197">
         <v>1</v>
@@ -5547,10 +5515,10 @@
         <v>40</v>
       </c>
       <c r="C198" t="s">
-        <v>195</v>
+        <v>197</v>
       </c>
       <c r="D198" t="s">
-        <v>361</v>
+        <v>362</v>
       </c>
       <c r="E198">
         <v>1</v>
@@ -5564,10 +5532,10 @@
         <v>40</v>
       </c>
       <c r="C199" t="s">
-        <v>196</v>
+        <v>198</v>
       </c>
       <c r="D199" t="s">
-        <v>362</v>
+        <v>363</v>
       </c>
       <c r="E199">
         <v>1</v>
@@ -5581,10 +5549,10 @@
         <v>40</v>
       </c>
       <c r="C200" t="s">
-        <v>197</v>
+        <v>199</v>
       </c>
       <c r="D200" t="s">
-        <v>363</v>
+        <v>364</v>
       </c>
       <c r="E200">
         <v>1</v>
@@ -5598,13 +5566,13 @@
         <v>40</v>
       </c>
       <c r="C201" t="s">
-        <v>198</v>
+        <v>200</v>
       </c>
       <c r="D201" t="s">
-        <v>364</v>
+        <v>365</v>
       </c>
       <c r="E201">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="202" spans="1:5">
@@ -5615,13 +5583,13 @@
         <v>40</v>
       </c>
       <c r="C202" t="s">
-        <v>199</v>
+        <v>201</v>
       </c>
       <c r="D202" t="s">
-        <v>365</v>
+        <v>366</v>
       </c>
       <c r="E202">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="203" spans="1:5">
@@ -5632,10 +5600,10 @@
         <v>40</v>
       </c>
       <c r="C203" t="s">
-        <v>200</v>
+        <v>202</v>
       </c>
       <c r="D203" t="s">
-        <v>366</v>
+        <v>367</v>
       </c>
       <c r="E203">
         <v>2</v>
@@ -5649,10 +5617,10 @@
         <v>40</v>
       </c>
       <c r="C204" t="s">
-        <v>201</v>
+        <v>203</v>
       </c>
       <c r="D204" t="s">
-        <v>367</v>
+        <v>368</v>
       </c>
       <c r="E204">
         <v>2</v>
@@ -5666,10 +5634,10 @@
         <v>40</v>
       </c>
       <c r="C205" t="s">
-        <v>202</v>
+        <v>204</v>
       </c>
       <c r="D205" t="s">
-        <v>368</v>
+        <v>369</v>
       </c>
       <c r="E205">
         <v>2</v>
@@ -5683,10 +5651,10 @@
         <v>40</v>
       </c>
       <c r="C206" t="s">
-        <v>203</v>
+        <v>205</v>
       </c>
       <c r="D206" t="s">
-        <v>369</v>
+        <v>370</v>
       </c>
       <c r="E206">
         <v>2</v>
@@ -5700,10 +5668,10 @@
         <v>40</v>
       </c>
       <c r="C207" t="s">
-        <v>204</v>
+        <v>206</v>
       </c>
       <c r="D207" t="s">
-        <v>370</v>
+        <v>371</v>
       </c>
       <c r="E207">
         <v>2</v>
@@ -5717,10 +5685,10 @@
         <v>40</v>
       </c>
       <c r="C208" t="s">
-        <v>205</v>
+        <v>207</v>
       </c>
       <c r="D208" t="s">
-        <v>371</v>
+        <v>372</v>
       </c>
       <c r="E208">
         <v>2</v>
@@ -5734,7 +5702,7 @@
         <v>40</v>
       </c>
       <c r="C209" t="s">
-        <v>206</v>
+        <v>208</v>
       </c>
       <c r="D209" t="s">
         <v>372</v>
@@ -5751,7 +5719,7 @@
         <v>40</v>
       </c>
       <c r="C210" t="s">
-        <v>207</v>
+        <v>209</v>
       </c>
       <c r="D210" t="s">
         <v>373</v>
@@ -5768,10 +5736,10 @@
         <v>40</v>
       </c>
       <c r="C211" t="s">
-        <v>208</v>
+        <v>210</v>
       </c>
       <c r="D211" t="s">
-        <v>373</v>
+        <v>374</v>
       </c>
       <c r="E211">
         <v>2</v>
@@ -5785,10 +5753,10 @@
         <v>40</v>
       </c>
       <c r="C212" t="s">
-        <v>209</v>
+        <v>211</v>
       </c>
       <c r="D212" t="s">
-        <v>374</v>
+        <v>375</v>
       </c>
       <c r="E212">
         <v>2</v>
@@ -5802,13 +5770,13 @@
         <v>40</v>
       </c>
       <c r="C213" t="s">
-        <v>210</v>
+        <v>212</v>
       </c>
       <c r="D213" t="s">
-        <v>375</v>
+        <v>376</v>
       </c>
       <c r="E213">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="214" spans="1:5">
@@ -5819,13 +5787,13 @@
         <v>40</v>
       </c>
       <c r="C214" t="s">
-        <v>211</v>
+        <v>213</v>
       </c>
       <c r="D214" t="s">
-        <v>376</v>
+        <v>263</v>
       </c>
       <c r="E214">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="215" spans="1:5">
@@ -5836,13 +5804,13 @@
         <v>40</v>
       </c>
       <c r="C215" t="s">
-        <v>212</v>
+        <v>214</v>
       </c>
       <c r="D215" t="s">
         <v>377</v>
       </c>
       <c r="E215">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="216" spans="1:5">
@@ -5853,13 +5821,13 @@
         <v>40</v>
       </c>
       <c r="C216" t="s">
-        <v>213</v>
+        <v>215</v>
       </c>
       <c r="D216" t="s">
-        <v>264</v>
+        <v>378</v>
       </c>
       <c r="E216">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="217" spans="1:5">
@@ -5870,10 +5838,10 @@
         <v>40</v>
       </c>
       <c r="C217" t="s">
-        <v>214</v>
+        <v>216</v>
       </c>
       <c r="D217" t="s">
-        <v>378</v>
+        <v>379</v>
       </c>
       <c r="E217">
         <v>4</v>
@@ -5887,10 +5855,10 @@
         <v>40</v>
       </c>
       <c r="C218" t="s">
-        <v>215</v>
+        <v>217</v>
       </c>
       <c r="D218" t="s">
-        <v>379</v>
+        <v>380</v>
       </c>
       <c r="E218">
         <v>4</v>
@@ -5904,10 +5872,10 @@
         <v>40</v>
       </c>
       <c r="C219" t="s">
-        <v>216</v>
+        <v>218</v>
       </c>
       <c r="D219" t="s">
-        <v>380</v>
+        <v>381</v>
       </c>
       <c r="E219">
         <v>4</v>
@@ -5921,13 +5889,13 @@
         <v>40</v>
       </c>
       <c r="C220" t="s">
-        <v>217</v>
+        <v>219</v>
       </c>
       <c r="D220" t="s">
-        <v>381</v>
+        <v>382</v>
       </c>
       <c r="E220">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="221" spans="1:5">
@@ -5938,13 +5906,13 @@
         <v>40</v>
       </c>
       <c r="C221" t="s">
-        <v>218</v>
+        <v>220</v>
       </c>
       <c r="D221" t="s">
-        <v>382</v>
+        <v>383</v>
       </c>
       <c r="E221">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="222" spans="1:5">
@@ -5955,13 +5923,13 @@
         <v>40</v>
       </c>
       <c r="C222" t="s">
-        <v>219</v>
+        <v>221</v>
       </c>
       <c r="D222" t="s">
-        <v>383</v>
+        <v>384</v>
       </c>
       <c r="E222">
-        <v>5</v>
+        <v>6</v>
       </c>
     </row>
     <row r="223" spans="1:5">
@@ -5972,13 +5940,13 @@
         <v>40</v>
       </c>
       <c r="C223" t="s">
-        <v>220</v>
+        <v>222</v>
       </c>
       <c r="D223" t="s">
-        <v>384</v>
+        <v>385</v>
       </c>
       <c r="E223">
-        <v>5</v>
+        <v>8</v>
       </c>
     </row>
     <row r="224" spans="1:5">
@@ -5989,13 +5957,13 @@
         <v>40</v>
       </c>
       <c r="C224" t="s">
-        <v>221</v>
+        <v>223</v>
       </c>
       <c r="D224" t="s">
-        <v>385</v>
+        <v>386</v>
       </c>
       <c r="E224">
-        <v>6</v>
+        <v>10</v>
       </c>
     </row>
     <row r="225" spans="1:5">
@@ -6006,13 +5974,13 @@
         <v>40</v>
       </c>
       <c r="C225" t="s">
-        <v>222</v>
+        <v>224</v>
       </c>
       <c r="D225" t="s">
         <v>386</v>
       </c>
       <c r="E225">
-        <v>8</v>
+        <v>10</v>
       </c>
     </row>
     <row r="226" spans="1:5">
@@ -6023,13 +5991,13 @@
         <v>40</v>
       </c>
       <c r="C226" t="s">
-        <v>223</v>
+        <v>225</v>
       </c>
       <c r="D226" t="s">
-        <v>387</v>
+        <v>265</v>
       </c>
       <c r="E226">
-        <v>10</v>
+        <v>12</v>
       </c>
     </row>
     <row r="227" spans="1:5">
@@ -6040,13 +6008,13 @@
         <v>40</v>
       </c>
       <c r="C227" t="s">
-        <v>224</v>
+        <v>226</v>
       </c>
       <c r="D227" t="s">
         <v>387</v>
       </c>
       <c r="E227">
-        <v>10</v>
+        <v>12</v>
       </c>
     </row>
     <row r="228" spans="1:5">
@@ -6057,13 +6025,13 @@
         <v>40</v>
       </c>
       <c r="C228" t="s">
-        <v>225</v>
+        <v>227</v>
       </c>
       <c r="D228" t="s">
-        <v>266</v>
+        <v>388</v>
       </c>
       <c r="E228">
-        <v>12</v>
+        <v>14</v>
       </c>
     </row>
     <row r="229" spans="1:5">
@@ -6074,13 +6042,13 @@
         <v>40</v>
       </c>
       <c r="C229" t="s">
-        <v>226</v>
+        <v>228</v>
       </c>
       <c r="D229" t="s">
-        <v>388</v>
+        <v>389</v>
       </c>
       <c r="E229">
-        <v>12</v>
+        <v>15</v>
       </c>
     </row>
     <row r="230" spans="1:5">
@@ -6091,115 +6059,64 @@
         <v>40</v>
       </c>
       <c r="C230" t="s">
-        <v>227</v>
+        <v>229</v>
       </c>
       <c r="D230" t="s">
-        <v>389</v>
+        <v>390</v>
       </c>
       <c r="E230">
-        <v>14</v>
+        <v>20</v>
       </c>
     </row>
     <row r="231" spans="1:5">
       <c r="A231" t="s">
-        <v>14</v>
+        <v>10</v>
       </c>
       <c r="B231" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="C231" t="s">
-        <v>228</v>
+        <v>230</v>
       </c>
       <c r="D231" t="s">
-        <v>390</v>
+        <v>391</v>
       </c>
       <c r="E231">
-        <v>15</v>
+        <v>1</v>
       </c>
     </row>
     <row r="232" spans="1:5">
       <c r="A232" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="B232" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="C232" t="s">
-        <v>229</v>
+        <v>230</v>
       </c>
       <c r="D232" t="s">
         <v>391</v>
       </c>
       <c r="E232">
-        <v>20</v>
+        <v>1</v>
       </c>
     </row>
     <row r="233" spans="1:5">
       <c r="A233" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="B233" t="s">
-        <v>39</v>
+        <v>36</v>
       </c>
       <c r="C233" t="s">
-        <v>230</v>
+        <v>231</v>
       </c>
       <c r="D233" t="s">
         <v>392</v>
       </c>
       <c r="E233">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="234" spans="1:5">
-      <c r="A234" t="s">
-        <v>6</v>
-      </c>
-      <c r="B234" t="s">
-        <v>36</v>
-      </c>
-      <c r="C234" t="s">
-        <v>231</v>
-      </c>
-      <c r="D234" t="s">
-        <v>393</v>
-      </c>
-      <c r="E234">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="235" spans="1:5">
-      <c r="A235" t="s">
-        <v>10</v>
-      </c>
-      <c r="B235" t="s">
-        <v>39</v>
-      </c>
-      <c r="C235" t="s">
-        <v>232</v>
-      </c>
-      <c r="D235" t="s">
-        <v>394</v>
-      </c>
-      <c r="E235">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="236" spans="1:5">
-      <c r="A236" t="s">
-        <v>15</v>
-      </c>
-      <c r="B236" t="s">
-        <v>41</v>
-      </c>
-      <c r="C236" t="s">
-        <v>232</v>
-      </c>
-      <c r="D236" t="s">
-        <v>394</v>
-      </c>
-      <c r="E236">
-        <v>1</v>
+        <v>4</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Atualização automática: rac (23/09/2026 10:00)
</commit_message>
<xml_diff>
--- a/Coordenadoria/02_Dados_Tratados/base_rac_tratada.xlsx
+++ b/Coordenadoria/02_Dados_Tratados/base_rac_tratada.xlsx
@@ -1200,8 +1200,16 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <fonts count="1">
+  <fonts count="2">
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -1217,7 +1225,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -1225,12 +1233,30 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1529,22 +1555,22 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:6">
-      <c r="A1" t="s">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" t="s">
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" t="s">
+      <c r="F1" s="1" t="s">
         <v>5</v>
       </c>
     </row>
@@ -2159,19 +2185,19 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:5">
-      <c r="A1" t="s">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" t="s">
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
         <v>55</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>56</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="1" t="s">
         <v>57</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualização automática: rac (23/09/2026 12:25)
</commit_message>
<xml_diff>
--- a/Coordenadoria/02_Dados_Tratados/base_rac_tratada.xlsx
+++ b/Coordenadoria/02_Dados_Tratados/base_rac_tratada.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1059" uniqueCount="393">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1063" uniqueCount="393">
   <si>
     <t>matricula</t>
   </si>
@@ -1200,16 +1200,8 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <fonts count="2">
+  <fonts count="1">
     <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -1225,7 +1217,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -1233,30 +1225,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color auto="1"/>
-      </left>
-      <right style="thin">
-        <color auto="1"/>
-      </right>
-      <top style="thin">
-        <color auto="1"/>
-      </top>
-      <bottom style="thin">
-        <color auto="1"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1555,22 +1529,22 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:6">
-      <c r="A1" s="1" t="s">
+      <c r="A1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" s="1" t="s">
+      <c r="B1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" t="s">
         <v>5</v>
       </c>
     </row>
@@ -1768,10 +1742,10 @@
         <v>53</v>
       </c>
       <c r="E11">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F11">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="12" spans="1:6">
@@ -2181,23 +2155,23 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E233"/>
+  <dimension ref="A1:E234"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:5">
-      <c r="A1" s="1" t="s">
+      <c r="A1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" s="1" t="s">
+      <c r="B1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" t="s">
         <v>55</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" t="s">
         <v>56</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" t="s">
         <v>57</v>
       </c>
     </row>
@@ -2662,16 +2636,16 @@
     </row>
     <row r="29" spans="1:5">
       <c r="A29" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="B29" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="C29" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="D29" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
       <c r="E29">
         <v>1</v>
@@ -2679,24 +2653,24 @@
     </row>
     <row r="30" spans="1:5">
       <c r="A30" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="B30" t="s">
         <v>39</v>
       </c>
       <c r="C30" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="D30" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="E30">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="31" spans="1:5">
       <c r="A31" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B31" t="s">
         <v>39</v>
@@ -2713,27 +2687,27 @@
     </row>
     <row r="32" spans="1:5">
       <c r="A32" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="B32" t="s">
-        <v>36</v>
+        <v>39</v>
       </c>
       <c r="C32" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="D32" t="s">
-        <v>245</v>
+        <v>244</v>
       </c>
       <c r="E32">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="33" spans="1:5">
       <c r="A33" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B33" t="s">
-        <v>39</v>
+        <v>36</v>
       </c>
       <c r="C33" t="s">
         <v>71</v>
@@ -2747,7 +2721,7 @@
     </row>
     <row r="34" spans="1:5">
       <c r="A34" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B34" t="s">
         <v>39</v>
@@ -2764,16 +2738,16 @@
     </row>
     <row r="35" spans="1:5">
       <c r="A35" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="B35" t="s">
-        <v>36</v>
+        <v>39</v>
       </c>
       <c r="C35" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="D35" t="s">
-        <v>246</v>
+        <v>245</v>
       </c>
       <c r="E35">
         <v>1</v>
@@ -2781,10 +2755,10 @@
     </row>
     <row r="36" spans="1:5">
       <c r="A36" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B36" t="s">
-        <v>39</v>
+        <v>36</v>
       </c>
       <c r="C36" t="s">
         <v>72</v>
@@ -2798,7 +2772,7 @@
     </row>
     <row r="37" spans="1:5">
       <c r="A37" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B37" t="s">
         <v>39</v>
@@ -2815,16 +2789,16 @@
     </row>
     <row r="38" spans="1:5">
       <c r="A38" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="B38" t="s">
-        <v>36</v>
+        <v>39</v>
       </c>
       <c r="C38" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="D38" t="s">
-        <v>247</v>
+        <v>246</v>
       </c>
       <c r="E38">
         <v>1</v>
@@ -2832,10 +2806,10 @@
     </row>
     <row r="39" spans="1:5">
       <c r="A39" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B39" t="s">
-        <v>39</v>
+        <v>36</v>
       </c>
       <c r="C39" t="s">
         <v>73</v>
@@ -2849,16 +2823,16 @@
     </row>
     <row r="40" spans="1:5">
       <c r="A40" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B40" t="s">
-        <v>36</v>
+        <v>39</v>
       </c>
       <c r="C40" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="D40" t="s">
-        <v>248</v>
+        <v>247</v>
       </c>
       <c r="E40">
         <v>1</v>
@@ -2866,10 +2840,10 @@
     </row>
     <row r="41" spans="1:5">
       <c r="A41" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="B41" t="s">
-        <v>39</v>
+        <v>36</v>
       </c>
       <c r="C41" t="s">
         <v>74</v>
@@ -2883,10 +2857,10 @@
     </row>
     <row r="42" spans="1:5">
       <c r="A42" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B42" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="C42" t="s">
         <v>74</v>
@@ -2900,16 +2874,16 @@
     </row>
     <row r="43" spans="1:5">
       <c r="A43" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="B43" t="s">
-        <v>36</v>
+        <v>40</v>
       </c>
       <c r="C43" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="D43" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
       <c r="E43">
         <v>1</v>
@@ -2923,10 +2897,10 @@
         <v>36</v>
       </c>
       <c r="C44" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="D44" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
       <c r="E44">
         <v>1</v>
@@ -2940,10 +2914,10 @@
         <v>36</v>
       </c>
       <c r="C45" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="D45" t="s">
-        <v>251</v>
+        <v>250</v>
       </c>
       <c r="E45">
         <v>1</v>
@@ -2957,10 +2931,10 @@
         <v>36</v>
       </c>
       <c r="C46" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="D46" t="s">
-        <v>252</v>
+        <v>251</v>
       </c>
       <c r="E46">
         <v>1</v>
@@ -2974,10 +2948,10 @@
         <v>36</v>
       </c>
       <c r="C47" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="D47" t="s">
-        <v>253</v>
+        <v>252</v>
       </c>
       <c r="E47">
         <v>1</v>
@@ -2991,10 +2965,10 @@
         <v>36</v>
       </c>
       <c r="C48" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="D48" t="s">
-        <v>254</v>
+        <v>253</v>
       </c>
       <c r="E48">
         <v>1</v>
@@ -3008,10 +2982,10 @@
         <v>36</v>
       </c>
       <c r="C49" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="D49" t="s">
-        <v>255</v>
+        <v>254</v>
       </c>
       <c r="E49">
         <v>1</v>
@@ -3025,10 +2999,10 @@
         <v>36</v>
       </c>
       <c r="C50" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="D50" t="s">
-        <v>256</v>
+        <v>255</v>
       </c>
       <c r="E50">
         <v>1</v>
@@ -3042,21 +3016,21 @@
         <v>36</v>
       </c>
       <c r="C51" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="D51" t="s">
-        <v>257</v>
+        <v>256</v>
       </c>
       <c r="E51">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="52" spans="1:5">
       <c r="A52" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B52" t="s">
-        <v>39</v>
+        <v>36</v>
       </c>
       <c r="C52" t="s">
         <v>83</v>
@@ -3065,12 +3039,12 @@
         <v>257</v>
       </c>
       <c r="E52">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="53" spans="1:5">
       <c r="A53" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B53" t="s">
         <v>39</v>
@@ -3082,15 +3056,15 @@
         <v>257</v>
       </c>
       <c r="E53">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="54" spans="1:5">
       <c r="A54" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B54" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="C54" t="s">
         <v>83</v>
@@ -3104,16 +3078,16 @@
     </row>
     <row r="55" spans="1:5">
       <c r="A55" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="B55" t="s">
-        <v>36</v>
+        <v>40</v>
       </c>
       <c r="C55" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="D55" t="s">
-        <v>258</v>
+        <v>257</v>
       </c>
       <c r="E55">
         <v>2</v>
@@ -3121,10 +3095,10 @@
     </row>
     <row r="56" spans="1:5">
       <c r="A56" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="B56" t="s">
-        <v>39</v>
+        <v>36</v>
       </c>
       <c r="C56" t="s">
         <v>84</v>
@@ -3138,10 +3112,10 @@
     </row>
     <row r="57" spans="1:5">
       <c r="A57" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B57" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="C57" t="s">
         <v>84</v>
@@ -3150,32 +3124,32 @@
         <v>258</v>
       </c>
       <c r="E57">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="58" spans="1:5">
       <c r="A58" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="B58" t="s">
-        <v>36</v>
+        <v>40</v>
       </c>
       <c r="C58" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="D58" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="E58">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="59" spans="1:5">
       <c r="A59" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="B59" t="s">
-        <v>39</v>
+        <v>36</v>
       </c>
       <c r="C59" t="s">
         <v>85</v>
@@ -3184,15 +3158,15 @@
         <v>259</v>
       </c>
       <c r="E59">
-        <v>4</v>
+        <v>2</v>
       </c>
     </row>
     <row r="60" spans="1:5">
       <c r="A60" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B60" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="C60" t="s">
         <v>85</v>
@@ -3201,21 +3175,21 @@
         <v>259</v>
       </c>
       <c r="E60">
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
     <row r="61" spans="1:5">
       <c r="A61" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="B61" t="s">
-        <v>36</v>
+        <v>40</v>
       </c>
       <c r="C61" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="D61" t="s">
-        <v>260</v>
+        <v>259</v>
       </c>
       <c r="E61">
         <v>2</v>
@@ -3223,10 +3197,10 @@
     </row>
     <row r="62" spans="1:5">
       <c r="A62" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="B62" t="s">
-        <v>40</v>
+        <v>36</v>
       </c>
       <c r="C62" t="s">
         <v>86</v>
@@ -3235,24 +3209,24 @@
         <v>260</v>
       </c>
       <c r="E62">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="63" spans="1:5">
       <c r="A63" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="B63" t="s">
-        <v>36</v>
+        <v>40</v>
       </c>
       <c r="C63" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="D63" t="s">
-        <v>261</v>
+        <v>260</v>
       </c>
       <c r="E63">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="64" spans="1:5">
@@ -3263,10 +3237,10 @@
         <v>36</v>
       </c>
       <c r="C64" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="D64" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
       <c r="E64">
         <v>2</v>
@@ -3280,10 +3254,10 @@
         <v>36</v>
       </c>
       <c r="C65" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="D65" t="s">
-        <v>263</v>
+        <v>262</v>
       </c>
       <c r="E65">
         <v>2</v>
@@ -3297,10 +3271,10 @@
         <v>36</v>
       </c>
       <c r="C66" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="D66" t="s">
-        <v>264</v>
+        <v>263</v>
       </c>
       <c r="E66">
         <v>2</v>
@@ -3314,10 +3288,10 @@
         <v>36</v>
       </c>
       <c r="C67" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="D67" t="s">
-        <v>265</v>
+        <v>264</v>
       </c>
       <c r="E67">
         <v>2</v>
@@ -3331,10 +3305,10 @@
         <v>36</v>
       </c>
       <c r="C68" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="D68" t="s">
-        <v>266</v>
+        <v>265</v>
       </c>
       <c r="E68">
         <v>2</v>
@@ -3348,10 +3322,10 @@
         <v>36</v>
       </c>
       <c r="C69" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="D69" t="s">
-        <v>267</v>
+        <v>266</v>
       </c>
       <c r="E69">
         <v>2</v>
@@ -3365,10 +3339,10 @@
         <v>36</v>
       </c>
       <c r="C70" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="D70" t="s">
-        <v>257</v>
+        <v>267</v>
       </c>
       <c r="E70">
         <v>2</v>
@@ -3382,21 +3356,21 @@
         <v>36</v>
       </c>
       <c r="C71" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="D71" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
       <c r="E71">
-        <v>4</v>
+        <v>2</v>
       </c>
     </row>
     <row r="72" spans="1:5">
       <c r="A72" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="B72" t="s">
-        <v>40</v>
+        <v>36</v>
       </c>
       <c r="C72" t="s">
         <v>95</v>
@@ -3410,16 +3384,16 @@
     </row>
     <row r="73" spans="1:5">
       <c r="A73" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="B73" t="s">
-        <v>36</v>
+        <v>40</v>
       </c>
       <c r="C73" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="D73" t="s">
-        <v>268</v>
+        <v>256</v>
       </c>
       <c r="E73">
         <v>4</v>
@@ -3433,10 +3407,10 @@
         <v>36</v>
       </c>
       <c r="C74" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="D74" t="s">
-        <v>269</v>
+        <v>268</v>
       </c>
       <c r="E74">
         <v>4</v>
@@ -3444,24 +3418,24 @@
     </row>
     <row r="75" spans="1:5">
       <c r="A75" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B75" t="s">
-        <v>39</v>
+        <v>36</v>
       </c>
       <c r="C75" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="D75" t="s">
-        <v>270</v>
+        <v>269</v>
       </c>
       <c r="E75">
-        <v>1</v>
+        <v>4</v>
       </c>
     </row>
     <row r="76" spans="1:5">
       <c r="A76" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B76" t="s">
         <v>39</v>
@@ -3478,10 +3452,10 @@
     </row>
     <row r="77" spans="1:5">
       <c r="A77" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B77" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="C77" t="s">
         <v>98</v>
@@ -3495,16 +3469,16 @@
     </row>
     <row r="78" spans="1:5">
       <c r="A78" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="B78" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="C78" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="D78" t="s">
-        <v>271</v>
+        <v>270</v>
       </c>
       <c r="E78">
         <v>1</v>
@@ -3512,7 +3486,7 @@
     </row>
     <row r="79" spans="1:5">
       <c r="A79" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B79" t="s">
         <v>39</v>
@@ -3529,10 +3503,10 @@
     </row>
     <row r="80" spans="1:5">
       <c r="A80" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B80" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="C80" t="s">
         <v>99</v>
@@ -3541,29 +3515,29 @@
         <v>271</v>
       </c>
       <c r="E80">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="81" spans="1:5">
       <c r="A81" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="B81" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="C81" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="D81" t="s">
-        <v>272</v>
+        <v>271</v>
       </c>
       <c r="E81">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="82" spans="1:5">
       <c r="A82" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B82" t="s">
         <v>39</v>
@@ -3580,16 +3554,16 @@
     </row>
     <row r="83" spans="1:5">
       <c r="A83" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="B83" t="s">
         <v>39</v>
       </c>
       <c r="C83" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="D83" t="s">
-        <v>273</v>
+        <v>272</v>
       </c>
       <c r="E83">
         <v>1</v>
@@ -3597,7 +3571,7 @@
     </row>
     <row r="84" spans="1:5">
       <c r="A84" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B84" t="s">
         <v>39</v>
@@ -3614,16 +3588,16 @@
     </row>
     <row r="85" spans="1:5">
       <c r="A85" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="B85" t="s">
         <v>39</v>
       </c>
       <c r="C85" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="D85" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
       <c r="E85">
         <v>1</v>
@@ -3631,7 +3605,7 @@
     </row>
     <row r="86" spans="1:5">
       <c r="A86" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B86" t="s">
         <v>39</v>
@@ -3648,16 +3622,16 @@
     </row>
     <row r="87" spans="1:5">
       <c r="A87" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="B87" t="s">
         <v>39</v>
       </c>
       <c r="C87" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="D87" t="s">
-        <v>275</v>
+        <v>274</v>
       </c>
       <c r="E87">
         <v>1</v>
@@ -3665,7 +3639,7 @@
     </row>
     <row r="88" spans="1:5">
       <c r="A88" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B88" t="s">
         <v>39</v>
@@ -3682,16 +3656,16 @@
     </row>
     <row r="89" spans="1:5">
       <c r="A89" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="B89" t="s">
         <v>39</v>
       </c>
       <c r="C89" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="D89" t="s">
-        <v>276</v>
+        <v>275</v>
       </c>
       <c r="E89">
         <v>1</v>
@@ -3699,7 +3673,7 @@
     </row>
     <row r="90" spans="1:5">
       <c r="A90" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B90" t="s">
         <v>39</v>
@@ -3716,16 +3690,16 @@
     </row>
     <row r="91" spans="1:5">
       <c r="A91" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="B91" t="s">
         <v>39</v>
       </c>
       <c r="C91" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="D91" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
       <c r="E91">
         <v>1</v>
@@ -3733,10 +3707,10 @@
     </row>
     <row r="92" spans="1:5">
       <c r="A92" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="B92" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="C92" t="s">
         <v>105</v>
@@ -3750,16 +3724,16 @@
     </row>
     <row r="93" spans="1:5">
       <c r="A93" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="B93" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="C93" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="D93" t="s">
-        <v>278</v>
+        <v>277</v>
       </c>
       <c r="E93">
         <v>1</v>
@@ -3767,10 +3741,10 @@
     </row>
     <row r="94" spans="1:5">
       <c r="A94" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="B94" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="C94" t="s">
         <v>106</v>
@@ -3784,16 +3758,16 @@
     </row>
     <row r="95" spans="1:5">
       <c r="A95" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="B95" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="C95" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="D95" t="s">
-        <v>279</v>
+        <v>278</v>
       </c>
       <c r="E95">
         <v>1</v>
@@ -3801,10 +3775,10 @@
     </row>
     <row r="96" spans="1:5">
       <c r="A96" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="B96" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="C96" t="s">
         <v>107</v>
@@ -3818,16 +3792,16 @@
     </row>
     <row r="97" spans="1:5">
       <c r="A97" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="B97" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="C97" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="D97" t="s">
-        <v>280</v>
+        <v>279</v>
       </c>
       <c r="E97">
         <v>1</v>
@@ -3841,10 +3815,10 @@
         <v>39</v>
       </c>
       <c r="C98" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="D98" t="s">
-        <v>281</v>
+        <v>280</v>
       </c>
       <c r="E98">
         <v>1</v>
@@ -3858,10 +3832,10 @@
         <v>39</v>
       </c>
       <c r="C99" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="D99" t="s">
-        <v>282</v>
+        <v>281</v>
       </c>
       <c r="E99">
         <v>1</v>
@@ -3875,10 +3849,10 @@
         <v>39</v>
       </c>
       <c r="C100" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="D100" t="s">
-        <v>283</v>
+        <v>282</v>
       </c>
       <c r="E100">
         <v>1</v>
@@ -3892,10 +3866,10 @@
         <v>39</v>
       </c>
       <c r="C101" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="D101" t="s">
-        <v>284</v>
+        <v>283</v>
       </c>
       <c r="E101">
         <v>1</v>
@@ -3909,10 +3883,10 @@
         <v>39</v>
       </c>
       <c r="C102" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="D102" t="s">
-        <v>285</v>
+        <v>284</v>
       </c>
       <c r="E102">
         <v>1</v>
@@ -3926,18 +3900,18 @@
         <v>39</v>
       </c>
       <c r="C103" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="D103" t="s">
-        <v>286</v>
+        <v>285</v>
       </c>
       <c r="E103">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="104" spans="1:5">
       <c r="A104" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B104" t="s">
         <v>39</v>
@@ -3949,29 +3923,29 @@
         <v>286</v>
       </c>
       <c r="E104">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="105" spans="1:5">
       <c r="A105" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="B105" t="s">
         <v>39</v>
       </c>
       <c r="C105" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="D105" t="s">
-        <v>287</v>
+        <v>286</v>
       </c>
       <c r="E105">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="106" spans="1:5">
       <c r="A106" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B106" t="s">
         <v>39</v>
@@ -3988,10 +3962,10 @@
     </row>
     <row r="107" spans="1:5">
       <c r="A107" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B107" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="C107" t="s">
         <v>115</v>
@@ -4005,16 +3979,16 @@
     </row>
     <row r="108" spans="1:5">
       <c r="A108" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="B108" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="C108" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="D108" t="s">
-        <v>288</v>
+        <v>287</v>
       </c>
       <c r="E108">
         <v>2</v>
@@ -4022,7 +3996,7 @@
     </row>
     <row r="109" spans="1:5">
       <c r="A109" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B109" t="s">
         <v>39</v>
@@ -4039,10 +4013,10 @@
     </row>
     <row r="110" spans="1:5">
       <c r="A110" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B110" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="C110" t="s">
         <v>116</v>
@@ -4056,16 +4030,16 @@
     </row>
     <row r="111" spans="1:5">
       <c r="A111" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="B111" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="C111" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="D111" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
       <c r="E111">
         <v>2</v>
@@ -4073,7 +4047,7 @@
     </row>
     <row r="112" spans="1:5">
       <c r="A112" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B112" t="s">
         <v>39</v>
@@ -4090,16 +4064,16 @@
     </row>
     <row r="113" spans="1:5">
       <c r="A113" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="B113" t="s">
         <v>39</v>
       </c>
       <c r="C113" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="D113" t="s">
-        <v>271</v>
+        <v>289</v>
       </c>
       <c r="E113">
         <v>2</v>
@@ -4107,7 +4081,7 @@
     </row>
     <row r="114" spans="1:5">
       <c r="A114" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B114" t="s">
         <v>39</v>
@@ -4119,15 +4093,15 @@
         <v>271</v>
       </c>
       <c r="E114">
-        <v>4</v>
+        <v>2</v>
       </c>
     </row>
     <row r="115" spans="1:5">
       <c r="A115" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B115" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="C115" t="s">
         <v>118</v>
@@ -4141,24 +4115,24 @@
     </row>
     <row r="116" spans="1:5">
       <c r="A116" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="B116" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="C116" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="D116" t="s">
-        <v>290</v>
+        <v>271</v>
       </c>
       <c r="E116">
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
     <row r="117" spans="1:5">
       <c r="A117" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B117" t="s">
         <v>39</v>
@@ -4170,24 +4144,24 @@
         <v>290</v>
       </c>
       <c r="E117">
-        <v>4</v>
+        <v>2</v>
       </c>
     </row>
     <row r="118" spans="1:5">
       <c r="A118" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="B118" t="s">
         <v>39</v>
       </c>
       <c r="C118" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="D118" t="s">
-        <v>275</v>
+        <v>290</v>
       </c>
       <c r="E118">
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
     <row r="119" spans="1:5">
@@ -4198,10 +4172,10 @@
         <v>39</v>
       </c>
       <c r="C119" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="D119" t="s">
-        <v>291</v>
+        <v>275</v>
       </c>
       <c r="E119">
         <v>2</v>
@@ -4215,10 +4189,10 @@
         <v>39</v>
       </c>
       <c r="C120" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="D120" t="s">
-        <v>292</v>
+        <v>291</v>
       </c>
       <c r="E120">
         <v>2</v>
@@ -4232,18 +4206,18 @@
         <v>39</v>
       </c>
       <c r="C121" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="D121" t="s">
-        <v>293</v>
+        <v>292</v>
       </c>
       <c r="E121">
-        <v>5</v>
+        <v>2</v>
       </c>
     </row>
     <row r="122" spans="1:5">
       <c r="A122" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B122" t="s">
         <v>39</v>
@@ -4260,19 +4234,19 @@
     </row>
     <row r="123" spans="1:5">
       <c r="A123" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="B123" t="s">
         <v>39</v>
       </c>
       <c r="C123" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="D123" t="s">
-        <v>294</v>
+        <v>293</v>
       </c>
       <c r="E123">
-        <v>7</v>
+        <v>5</v>
       </c>
     </row>
     <row r="124" spans="1:5">
@@ -4283,13 +4257,13 @@
         <v>39</v>
       </c>
       <c r="C124" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="D124" t="s">
-        <v>295</v>
+        <v>294</v>
       </c>
       <c r="E124">
-        <v>8</v>
+        <v>7</v>
       </c>
     </row>
     <row r="125" spans="1:5">
@@ -4300,13 +4274,13 @@
         <v>39</v>
       </c>
       <c r="C125" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="D125" t="s">
-        <v>296</v>
+        <v>295</v>
       </c>
       <c r="E125">
-        <v>10</v>
+        <v>8</v>
       </c>
     </row>
     <row r="126" spans="1:5">
@@ -4317,18 +4291,18 @@
         <v>39</v>
       </c>
       <c r="C126" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="D126" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="E126">
-        <v>30</v>
+        <v>10</v>
       </c>
     </row>
     <row r="127" spans="1:5">
       <c r="A127" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B127" t="s">
         <v>39</v>
@@ -4351,21 +4325,21 @@
         <v>39</v>
       </c>
       <c r="C128" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="D128" t="s">
-        <v>298</v>
+        <v>297</v>
       </c>
       <c r="E128">
-        <v>1</v>
+        <v>30</v>
       </c>
     </row>
     <row r="129" spans="1:5">
       <c r="A129" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B129" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="C129" t="s">
         <v>128</v>
@@ -4379,16 +4353,16 @@
     </row>
     <row r="130" spans="1:5">
       <c r="A130" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="B130" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="C130" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="D130" t="s">
-        <v>299</v>
+        <v>298</v>
       </c>
       <c r="E130">
         <v>1</v>
@@ -4402,10 +4376,10 @@
         <v>39</v>
       </c>
       <c r="C131" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="D131" t="s">
-        <v>300</v>
+        <v>299</v>
       </c>
       <c r="E131">
         <v>1</v>
@@ -4419,10 +4393,10 @@
         <v>39</v>
       </c>
       <c r="C132" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="D132" t="s">
-        <v>301</v>
+        <v>300</v>
       </c>
       <c r="E132">
         <v>1</v>
@@ -4436,10 +4410,10 @@
         <v>39</v>
       </c>
       <c r="C133" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="D133" t="s">
-        <v>302</v>
+        <v>301</v>
       </c>
       <c r="E133">
         <v>1</v>
@@ -4453,10 +4427,10 @@
         <v>39</v>
       </c>
       <c r="C134" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="D134" t="s">
-        <v>303</v>
+        <v>302</v>
       </c>
       <c r="E134">
         <v>1</v>
@@ -4470,10 +4444,10 @@
         <v>39</v>
       </c>
       <c r="C135" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="D135" t="s">
-        <v>304</v>
+        <v>303</v>
       </c>
       <c r="E135">
         <v>1</v>
@@ -4487,10 +4461,10 @@
         <v>39</v>
       </c>
       <c r="C136" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="D136" t="s">
-        <v>305</v>
+        <v>304</v>
       </c>
       <c r="E136">
         <v>1</v>
@@ -4504,10 +4478,10 @@
         <v>39</v>
       </c>
       <c r="C137" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="D137" t="s">
-        <v>306</v>
+        <v>305</v>
       </c>
       <c r="E137">
         <v>1</v>
@@ -4521,10 +4495,10 @@
         <v>39</v>
       </c>
       <c r="C138" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="D138" t="s">
-        <v>307</v>
+        <v>306</v>
       </c>
       <c r="E138">
         <v>1</v>
@@ -4538,10 +4512,10 @@
         <v>39</v>
       </c>
       <c r="C139" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="D139" t="s">
-        <v>308</v>
+        <v>307</v>
       </c>
       <c r="E139">
         <v>1</v>
@@ -4555,10 +4529,10 @@
         <v>39</v>
       </c>
       <c r="C140" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="D140" t="s">
-        <v>309</v>
+        <v>308</v>
       </c>
       <c r="E140">
         <v>1</v>
@@ -4572,10 +4546,10 @@
         <v>39</v>
       </c>
       <c r="C141" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="D141" t="s">
-        <v>310</v>
+        <v>309</v>
       </c>
       <c r="E141">
         <v>1</v>
@@ -4589,10 +4563,10 @@
         <v>39</v>
       </c>
       <c r="C142" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="D142" t="s">
-        <v>311</v>
+        <v>310</v>
       </c>
       <c r="E142">
         <v>1</v>
@@ -4606,10 +4580,10 @@
         <v>39</v>
       </c>
       <c r="C143" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="D143" t="s">
-        <v>312</v>
+        <v>311</v>
       </c>
       <c r="E143">
         <v>1</v>
@@ -4623,10 +4597,10 @@
         <v>39</v>
       </c>
       <c r="C144" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="D144" t="s">
-        <v>313</v>
+        <v>312</v>
       </c>
       <c r="E144">
         <v>1</v>
@@ -4640,10 +4614,10 @@
         <v>39</v>
       </c>
       <c r="C145" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="D145" t="s">
-        <v>314</v>
+        <v>313</v>
       </c>
       <c r="E145">
         <v>1</v>
@@ -4657,10 +4631,10 @@
         <v>39</v>
       </c>
       <c r="C146" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="D146" t="s">
-        <v>315</v>
+        <v>314</v>
       </c>
       <c r="E146">
         <v>1</v>
@@ -4674,10 +4648,10 @@
         <v>39</v>
       </c>
       <c r="C147" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="D147" t="s">
-        <v>316</v>
+        <v>315</v>
       </c>
       <c r="E147">
         <v>1</v>
@@ -4691,10 +4665,10 @@
         <v>39</v>
       </c>
       <c r="C148" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="D148" t="s">
-        <v>317</v>
+        <v>316</v>
       </c>
       <c r="E148">
         <v>1</v>
@@ -4708,10 +4682,10 @@
         <v>39</v>
       </c>
       <c r="C149" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="D149" t="s">
-        <v>318</v>
+        <v>317</v>
       </c>
       <c r="E149">
         <v>1</v>
@@ -4725,10 +4699,10 @@
         <v>39</v>
       </c>
       <c r="C150" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="D150" t="s">
-        <v>319</v>
+        <v>318</v>
       </c>
       <c r="E150">
         <v>1</v>
@@ -4742,10 +4716,10 @@
         <v>39</v>
       </c>
       <c r="C151" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="D151" t="s">
-        <v>320</v>
+        <v>319</v>
       </c>
       <c r="E151">
         <v>1</v>
@@ -4759,10 +4733,10 @@
         <v>39</v>
       </c>
       <c r="C152" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="D152" t="s">
-        <v>321</v>
+        <v>320</v>
       </c>
       <c r="E152">
         <v>1</v>
@@ -4776,10 +4750,10 @@
         <v>39</v>
       </c>
       <c r="C153" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="D153" t="s">
-        <v>322</v>
+        <v>321</v>
       </c>
       <c r="E153">
         <v>1</v>
@@ -4793,10 +4767,10 @@
         <v>39</v>
       </c>
       <c r="C154" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="D154" t="s">
-        <v>323</v>
+        <v>322</v>
       </c>
       <c r="E154">
         <v>1</v>
@@ -4810,10 +4784,10 @@
         <v>39</v>
       </c>
       <c r="C155" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="D155" t="s">
-        <v>324</v>
+        <v>323</v>
       </c>
       <c r="E155">
         <v>1</v>
@@ -4827,10 +4801,10 @@
         <v>39</v>
       </c>
       <c r="C156" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="D156" t="s">
-        <v>325</v>
+        <v>324</v>
       </c>
       <c r="E156">
         <v>1</v>
@@ -4844,10 +4818,10 @@
         <v>39</v>
       </c>
       <c r="C157" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="D157" t="s">
-        <v>326</v>
+        <v>325</v>
       </c>
       <c r="E157">
         <v>1</v>
@@ -4861,10 +4835,10 @@
         <v>39</v>
       </c>
       <c r="C158" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="D158" t="s">
-        <v>327</v>
+        <v>326</v>
       </c>
       <c r="E158">
         <v>1</v>
@@ -4878,13 +4852,13 @@
         <v>39</v>
       </c>
       <c r="C159" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="D159" t="s">
-        <v>312</v>
+        <v>327</v>
       </c>
       <c r="E159">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="160" spans="1:5">
@@ -4895,10 +4869,10 @@
         <v>39</v>
       </c>
       <c r="C160" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="D160" t="s">
-        <v>328</v>
+        <v>312</v>
       </c>
       <c r="E160">
         <v>2</v>
@@ -4912,10 +4886,10 @@
         <v>39</v>
       </c>
       <c r="C161" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="D161" t="s">
-        <v>329</v>
+        <v>328</v>
       </c>
       <c r="E161">
         <v>2</v>
@@ -4929,10 +4903,10 @@
         <v>39</v>
       </c>
       <c r="C162" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="D162" t="s">
-        <v>330</v>
+        <v>329</v>
       </c>
       <c r="E162">
         <v>2</v>
@@ -4946,10 +4920,10 @@
         <v>39</v>
       </c>
       <c r="C163" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="D163" t="s">
-        <v>331</v>
+        <v>330</v>
       </c>
       <c r="E163">
         <v>2</v>
@@ -4963,13 +4937,13 @@
         <v>39</v>
       </c>
       <c r="C164" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="D164" t="s">
-        <v>332</v>
+        <v>331</v>
       </c>
       <c r="E164">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="165" spans="1:5">
@@ -4980,13 +4954,13 @@
         <v>39</v>
       </c>
       <c r="C165" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="D165" t="s">
-        <v>297</v>
+        <v>332</v>
       </c>
       <c r="E165">
-        <v>5</v>
+        <v>3</v>
       </c>
     </row>
     <row r="166" spans="1:5">
@@ -4997,13 +4971,13 @@
         <v>39</v>
       </c>
       <c r="C166" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="D166" t="s">
-        <v>333</v>
+        <v>297</v>
       </c>
       <c r="E166">
-        <v>8</v>
+        <v>5</v>
       </c>
     </row>
     <row r="167" spans="1:5">
@@ -5014,10 +4988,10 @@
         <v>39</v>
       </c>
       <c r="C167" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="D167" t="s">
-        <v>253</v>
+        <v>333</v>
       </c>
       <c r="E167">
         <v>8</v>
@@ -5031,30 +5005,30 @@
         <v>39</v>
       </c>
       <c r="C168" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="D168" t="s">
-        <v>334</v>
+        <v>253</v>
       </c>
       <c r="E168">
-        <v>10</v>
+        <v>8</v>
       </c>
     </row>
     <row r="169" spans="1:5">
       <c r="A169" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B169" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="C169" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="D169" t="s">
-        <v>322</v>
+        <v>334</v>
       </c>
       <c r="E169">
-        <v>1</v>
+        <v>10</v>
       </c>
     </row>
     <row r="170" spans="1:5">
@@ -5065,10 +5039,10 @@
         <v>40</v>
       </c>
       <c r="C170" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="D170" t="s">
-        <v>335</v>
+        <v>322</v>
       </c>
       <c r="E170">
         <v>1</v>
@@ -5082,10 +5056,10 @@
         <v>40</v>
       </c>
       <c r="C171" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="D171" t="s">
-        <v>336</v>
+        <v>335</v>
       </c>
       <c r="E171">
         <v>1</v>
@@ -5099,10 +5073,10 @@
         <v>40</v>
       </c>
       <c r="C172" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="D172" t="s">
-        <v>337</v>
+        <v>336</v>
       </c>
       <c r="E172">
         <v>1</v>
@@ -5116,10 +5090,10 @@
         <v>40</v>
       </c>
       <c r="C173" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="D173" t="s">
-        <v>338</v>
+        <v>337</v>
       </c>
       <c r="E173">
         <v>1</v>
@@ -5133,10 +5107,10 @@
         <v>40</v>
       </c>
       <c r="C174" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="D174" t="s">
-        <v>339</v>
+        <v>338</v>
       </c>
       <c r="E174">
         <v>1</v>
@@ -5150,10 +5124,10 @@
         <v>40</v>
       </c>
       <c r="C175" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="D175" t="s">
-        <v>263</v>
+        <v>339</v>
       </c>
       <c r="E175">
         <v>1</v>
@@ -5167,10 +5141,10 @@
         <v>40</v>
       </c>
       <c r="C176" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="D176" t="s">
-        <v>340</v>
+        <v>263</v>
       </c>
       <c r="E176">
         <v>1</v>
@@ -5184,10 +5158,10 @@
         <v>40</v>
       </c>
       <c r="C177" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="D177" t="s">
-        <v>341</v>
+        <v>340</v>
       </c>
       <c r="E177">
         <v>1</v>
@@ -5201,10 +5175,10 @@
         <v>40</v>
       </c>
       <c r="C178" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="D178" t="s">
-        <v>342</v>
+        <v>341</v>
       </c>
       <c r="E178">
         <v>1</v>
@@ -5218,10 +5192,10 @@
         <v>40</v>
       </c>
       <c r="C179" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="D179" t="s">
-        <v>343</v>
+        <v>342</v>
       </c>
       <c r="E179">
         <v>1</v>
@@ -5235,10 +5209,10 @@
         <v>40</v>
       </c>
       <c r="C180" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="D180" t="s">
-        <v>344</v>
+        <v>343</v>
       </c>
       <c r="E180">
         <v>1</v>
@@ -5252,10 +5226,10 @@
         <v>40</v>
       </c>
       <c r="C181" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="D181" t="s">
-        <v>345</v>
+        <v>344</v>
       </c>
       <c r="E181">
         <v>1</v>
@@ -5269,10 +5243,10 @@
         <v>40</v>
       </c>
       <c r="C182" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="D182" t="s">
-        <v>346</v>
+        <v>345</v>
       </c>
       <c r="E182">
         <v>1</v>
@@ -5286,10 +5260,10 @@
         <v>40</v>
       </c>
       <c r="C183" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="D183" t="s">
-        <v>347</v>
+        <v>346</v>
       </c>
       <c r="E183">
         <v>1</v>
@@ -5303,10 +5277,10 @@
         <v>40</v>
       </c>
       <c r="C184" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="D184" t="s">
-        <v>348</v>
+        <v>347</v>
       </c>
       <c r="E184">
         <v>1</v>
@@ -5320,10 +5294,10 @@
         <v>40</v>
       </c>
       <c r="C185" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="D185" t="s">
-        <v>349</v>
+        <v>348</v>
       </c>
       <c r="E185">
         <v>1</v>
@@ -5337,10 +5311,10 @@
         <v>40</v>
       </c>
       <c r="C186" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="D186" t="s">
-        <v>350</v>
+        <v>349</v>
       </c>
       <c r="E186">
         <v>1</v>
@@ -5354,10 +5328,10 @@
         <v>40</v>
       </c>
       <c r="C187" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="D187" t="s">
-        <v>351</v>
+        <v>350</v>
       </c>
       <c r="E187">
         <v>1</v>
@@ -5371,10 +5345,10 @@
         <v>40</v>
       </c>
       <c r="C188" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="D188" t="s">
-        <v>352</v>
+        <v>351</v>
       </c>
       <c r="E188">
         <v>1</v>
@@ -5388,10 +5362,10 @@
         <v>40</v>
       </c>
       <c r="C189" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="D189" t="s">
-        <v>353</v>
+        <v>352</v>
       </c>
       <c r="E189">
         <v>1</v>
@@ -5405,10 +5379,10 @@
         <v>40</v>
       </c>
       <c r="C190" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
       <c r="D190" t="s">
-        <v>354</v>
+        <v>353</v>
       </c>
       <c r="E190">
         <v>1</v>
@@ -5422,10 +5396,10 @@
         <v>40</v>
       </c>
       <c r="C191" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="D191" t="s">
-        <v>355</v>
+        <v>354</v>
       </c>
       <c r="E191">
         <v>1</v>
@@ -5439,10 +5413,10 @@
         <v>40</v>
       </c>
       <c r="C192" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="D192" t="s">
-        <v>356</v>
+        <v>355</v>
       </c>
       <c r="E192">
         <v>1</v>
@@ -5456,10 +5430,10 @@
         <v>40</v>
       </c>
       <c r="C193" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
       <c r="D193" t="s">
-        <v>357</v>
+        <v>356</v>
       </c>
       <c r="E193">
         <v>1</v>
@@ -5473,10 +5447,10 @@
         <v>40</v>
       </c>
       <c r="C194" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="D194" t="s">
-        <v>358</v>
+        <v>357</v>
       </c>
       <c r="E194">
         <v>1</v>
@@ -5490,10 +5464,10 @@
         <v>40</v>
       </c>
       <c r="C195" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="D195" t="s">
-        <v>359</v>
+        <v>358</v>
       </c>
       <c r="E195">
         <v>1</v>
@@ -5507,10 +5481,10 @@
         <v>40</v>
       </c>
       <c r="C196" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="D196" t="s">
-        <v>360</v>
+        <v>359</v>
       </c>
       <c r="E196">
         <v>1</v>
@@ -5524,10 +5498,10 @@
         <v>40</v>
       </c>
       <c r="C197" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="D197" t="s">
-        <v>361</v>
+        <v>360</v>
       </c>
       <c r="E197">
         <v>1</v>
@@ -5541,10 +5515,10 @@
         <v>40</v>
       </c>
       <c r="C198" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="D198" t="s">
-        <v>362</v>
+        <v>361</v>
       </c>
       <c r="E198">
         <v>1</v>
@@ -5558,10 +5532,10 @@
         <v>40</v>
       </c>
       <c r="C199" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="D199" t="s">
-        <v>363</v>
+        <v>362</v>
       </c>
       <c r="E199">
         <v>1</v>
@@ -5575,10 +5549,10 @@
         <v>40</v>
       </c>
       <c r="C200" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="D200" t="s">
-        <v>364</v>
+        <v>363</v>
       </c>
       <c r="E200">
         <v>1</v>
@@ -5592,13 +5566,13 @@
         <v>40</v>
       </c>
       <c r="C201" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="D201" t="s">
-        <v>365</v>
+        <v>364</v>
       </c>
       <c r="E201">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="202" spans="1:5">
@@ -5609,10 +5583,10 @@
         <v>40</v>
       </c>
       <c r="C202" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="D202" t="s">
-        <v>366</v>
+        <v>365</v>
       </c>
       <c r="E202">
         <v>2</v>
@@ -5626,10 +5600,10 @@
         <v>40</v>
       </c>
       <c r="C203" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
       <c r="D203" t="s">
-        <v>367</v>
+        <v>366</v>
       </c>
       <c r="E203">
         <v>2</v>
@@ -5643,10 +5617,10 @@
         <v>40</v>
       </c>
       <c r="C204" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
       <c r="D204" t="s">
-        <v>368</v>
+        <v>367</v>
       </c>
       <c r="E204">
         <v>2</v>
@@ -5660,10 +5634,10 @@
         <v>40</v>
       </c>
       <c r="C205" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="D205" t="s">
-        <v>369</v>
+        <v>368</v>
       </c>
       <c r="E205">
         <v>2</v>
@@ -5677,10 +5651,10 @@
         <v>40</v>
       </c>
       <c r="C206" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
       <c r="D206" t="s">
-        <v>370</v>
+        <v>369</v>
       </c>
       <c r="E206">
         <v>2</v>
@@ -5694,10 +5668,10 @@
         <v>40</v>
       </c>
       <c r="C207" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
       <c r="D207" t="s">
-        <v>371</v>
+        <v>370</v>
       </c>
       <c r="E207">
         <v>2</v>
@@ -5711,10 +5685,10 @@
         <v>40</v>
       </c>
       <c r="C208" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
       <c r="D208" t="s">
-        <v>372</v>
+        <v>371</v>
       </c>
       <c r="E208">
         <v>2</v>
@@ -5728,7 +5702,7 @@
         <v>40</v>
       </c>
       <c r="C209" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="D209" t="s">
         <v>372</v>
@@ -5745,10 +5719,10 @@
         <v>40</v>
       </c>
       <c r="C210" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="D210" t="s">
-        <v>373</v>
+        <v>372</v>
       </c>
       <c r="E210">
         <v>2</v>
@@ -5762,10 +5736,10 @@
         <v>40</v>
       </c>
       <c r="C211" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="D211" t="s">
-        <v>374</v>
+        <v>373</v>
       </c>
       <c r="E211">
         <v>2</v>
@@ -5779,10 +5753,10 @@
         <v>40</v>
       </c>
       <c r="C212" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
       <c r="D212" t="s">
-        <v>375</v>
+        <v>374</v>
       </c>
       <c r="E212">
         <v>2</v>
@@ -5796,13 +5770,13 @@
         <v>40</v>
       </c>
       <c r="C213" t="s">
-        <v>212</v>
+        <v>211</v>
       </c>
       <c r="D213" t="s">
-        <v>376</v>
+        <v>375</v>
       </c>
       <c r="E213">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="214" spans="1:5">
@@ -5813,10 +5787,10 @@
         <v>40</v>
       </c>
       <c r="C214" t="s">
-        <v>213</v>
+        <v>212</v>
       </c>
       <c r="D214" t="s">
-        <v>263</v>
+        <v>376</v>
       </c>
       <c r="E214">
         <v>3</v>
@@ -5830,13 +5804,13 @@
         <v>40</v>
       </c>
       <c r="C215" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
       <c r="D215" t="s">
-        <v>377</v>
+        <v>263</v>
       </c>
       <c r="E215">
-        <v>4</v>
+        <v>3</v>
       </c>
     </row>
     <row r="216" spans="1:5">
@@ -5847,10 +5821,10 @@
         <v>40</v>
       </c>
       <c r="C216" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
       <c r="D216" t="s">
-        <v>378</v>
+        <v>377</v>
       </c>
       <c r="E216">
         <v>4</v>
@@ -5864,10 +5838,10 @@
         <v>40</v>
       </c>
       <c r="C217" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
       <c r="D217" t="s">
-        <v>379</v>
+        <v>378</v>
       </c>
       <c r="E217">
         <v>4</v>
@@ -5881,10 +5855,10 @@
         <v>40</v>
       </c>
       <c r="C218" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
       <c r="D218" t="s">
-        <v>380</v>
+        <v>379</v>
       </c>
       <c r="E218">
         <v>4</v>
@@ -5898,10 +5872,10 @@
         <v>40</v>
       </c>
       <c r="C219" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
       <c r="D219" t="s">
-        <v>381</v>
+        <v>380</v>
       </c>
       <c r="E219">
         <v>4</v>
@@ -5915,13 +5889,13 @@
         <v>40</v>
       </c>
       <c r="C220" t="s">
-        <v>219</v>
+        <v>218</v>
       </c>
       <c r="D220" t="s">
-        <v>382</v>
+        <v>381</v>
       </c>
       <c r="E220">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="221" spans="1:5">
@@ -5932,10 +5906,10 @@
         <v>40</v>
       </c>
       <c r="C221" t="s">
-        <v>220</v>
+        <v>219</v>
       </c>
       <c r="D221" t="s">
-        <v>383</v>
+        <v>382</v>
       </c>
       <c r="E221">
         <v>5</v>
@@ -5949,13 +5923,13 @@
         <v>40</v>
       </c>
       <c r="C222" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
       <c r="D222" t="s">
-        <v>384</v>
+        <v>383</v>
       </c>
       <c r="E222">
-        <v>6</v>
+        <v>5</v>
       </c>
     </row>
     <row r="223" spans="1:5">
@@ -5966,13 +5940,13 @@
         <v>40</v>
       </c>
       <c r="C223" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
       <c r="D223" t="s">
-        <v>385</v>
+        <v>384</v>
       </c>
       <c r="E223">
-        <v>8</v>
+        <v>6</v>
       </c>
     </row>
     <row r="224" spans="1:5">
@@ -5983,13 +5957,13 @@
         <v>40</v>
       </c>
       <c r="C224" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
       <c r="D224" t="s">
-        <v>386</v>
+        <v>385</v>
       </c>
       <c r="E224">
-        <v>10</v>
+        <v>8</v>
       </c>
     </row>
     <row r="225" spans="1:5">
@@ -6000,7 +5974,7 @@
         <v>40</v>
       </c>
       <c r="C225" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="D225" t="s">
         <v>386</v>
@@ -6017,13 +5991,13 @@
         <v>40</v>
       </c>
       <c r="C226" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
       <c r="D226" t="s">
-        <v>265</v>
+        <v>386</v>
       </c>
       <c r="E226">
-        <v>12</v>
+        <v>10</v>
       </c>
     </row>
     <row r="227" spans="1:5">
@@ -6034,10 +6008,10 @@
         <v>40</v>
       </c>
       <c r="C227" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
       <c r="D227" t="s">
-        <v>387</v>
+        <v>265</v>
       </c>
       <c r="E227">
         <v>12</v>
@@ -6051,13 +6025,13 @@
         <v>40</v>
       </c>
       <c r="C228" t="s">
-        <v>227</v>
+        <v>226</v>
       </c>
       <c r="D228" t="s">
-        <v>388</v>
+        <v>387</v>
       </c>
       <c r="E228">
-        <v>14</v>
+        <v>12</v>
       </c>
     </row>
     <row r="229" spans="1:5">
@@ -6068,13 +6042,13 @@
         <v>40</v>
       </c>
       <c r="C229" t="s">
-        <v>228</v>
+        <v>227</v>
       </c>
       <c r="D229" t="s">
-        <v>389</v>
+        <v>388</v>
       </c>
       <c r="E229">
-        <v>15</v>
+        <v>14</v>
       </c>
     </row>
     <row r="230" spans="1:5">
@@ -6085,38 +6059,38 @@
         <v>40</v>
       </c>
       <c r="C230" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
       <c r="D230" t="s">
-        <v>390</v>
+        <v>389</v>
       </c>
       <c r="E230">
-        <v>20</v>
+        <v>15</v>
       </c>
     </row>
     <row r="231" spans="1:5">
       <c r="A231" t="s">
-        <v>10</v>
+        <v>14</v>
       </c>
       <c r="B231" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="C231" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="D231" t="s">
-        <v>391</v>
+        <v>390</v>
       </c>
       <c r="E231">
-        <v>1</v>
+        <v>20</v>
       </c>
     </row>
     <row r="232" spans="1:5">
       <c r="A232" t="s">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="B232" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="C232" t="s">
         <v>230</v>
@@ -6130,18 +6104,35 @@
     </row>
     <row r="233" spans="1:5">
       <c r="A233" t="s">
+        <v>15</v>
+      </c>
+      <c r="B233" t="s">
+        <v>41</v>
+      </c>
+      <c r="C233" t="s">
+        <v>230</v>
+      </c>
+      <c r="D233" t="s">
+        <v>391</v>
+      </c>
+      <c r="E233">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="234" spans="1:5">
+      <c r="A234" t="s">
         <v>11</v>
       </c>
-      <c r="B233" t="s">
+      <c r="B234" t="s">
         <v>36</v>
       </c>
-      <c r="C233" t="s">
+      <c r="C234" t="s">
         <v>231</v>
       </c>
-      <c r="D233" t="s">
+      <c r="D234" t="s">
         <v>392</v>
       </c>
-      <c r="E233">
+      <c r="E234">
         <v>4</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualização automática: rac (28/09/2026 13:05)
</commit_message>
<xml_diff>
--- a/Coordenadoria/02_Dados_Tratados/base_rac_tratada.xlsx
+++ b/Coordenadoria/02_Dados_Tratados/base_rac_tratada.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1059" uniqueCount="395">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1071" uniqueCount="401">
   <si>
     <t>matricula</t>
   </si>
@@ -200,12 +200,12 @@
     <t>3034792</t>
   </si>
   <si>
+    <t>3044000</t>
+  </si>
+  <si>
     <t>P7036368-01</t>
   </si>
   <si>
-    <t>3044000</t>
-  </si>
-  <si>
     <t>3107453-01</t>
   </si>
   <si>
@@ -530,6 +530,12 @@
     <t>S2319-64</t>
   </si>
   <si>
+    <t>2652022-18</t>
+  </si>
+  <si>
+    <t>2651031-1</t>
+  </si>
+  <si>
     <t>2650113-5</t>
   </si>
   <si>
@@ -716,6 +722,9 @@
     <t>2670067-1</t>
   </si>
   <si>
+    <t>2643031-7</t>
+  </si>
+  <si>
     <t>PIN-MAIN GEAR ATTACH</t>
   </si>
   <si>
@@ -725,12 +734,12 @@
     <t>FUEL PUMP</t>
   </si>
   <si>
+    <t>ENGINE PT6A-114A</t>
+  </si>
+  <si>
     <t>PROPELLER ASSEMBLY</t>
   </si>
   <si>
-    <t>ENGINE PT6A-114A</t>
-  </si>
-  <si>
     <t>HOUSING</t>
   </si>
   <si>
@@ -1034,6 +1043,12 @@
     <t>GROMMET</t>
   </si>
   <si>
+    <t>TUBE ASSY</t>
+  </si>
+  <si>
+    <t>LEVER FUEL CON</t>
+  </si>
+  <si>
     <t>TRUNNION ASSY-RH-MAI</t>
   </si>
   <si>
@@ -1200,14 +1215,25 @@
   </si>
   <si>
     <t>POST LIGHT ASS</t>
+  </si>
+  <si>
+    <t>FORK ASSY,NOSE GEAR SPRING</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <fonts count="1">
+  <fonts count="2">
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -1223,7 +1249,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -1231,12 +1257,30 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1535,22 +1579,22 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:6">
-      <c r="A1" t="s">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" t="s">
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" t="s">
+      <c r="F1" s="1" t="s">
         <v>5</v>
       </c>
     </row>
@@ -1568,10 +1612,10 @@
         <v>53</v>
       </c>
       <c r="E2">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F2">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="3" spans="1:6">
@@ -1728,10 +1772,10 @@
         <v>54</v>
       </c>
       <c r="E10">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="F10">
-        <v>150</v>
+        <v>152</v>
       </c>
     </row>
     <row r="11" spans="1:6">
@@ -2161,23 +2205,23 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E233"/>
+  <dimension ref="A1:E236"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:5">
-      <c r="A1" t="s">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" t="s">
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
         <v>55</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>56</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="1" t="s">
         <v>57</v>
       </c>
     </row>
@@ -2192,7 +2236,7 @@
         <v>58</v>
       </c>
       <c r="D2" t="s">
-        <v>233</v>
+        <v>236</v>
       </c>
       <c r="E2">
         <v>1</v>
@@ -2209,7 +2253,7 @@
         <v>59</v>
       </c>
       <c r="D3" t="s">
-        <v>234</v>
+        <v>237</v>
       </c>
       <c r="E3">
         <v>1</v>
@@ -2226,7 +2270,7 @@
         <v>59</v>
       </c>
       <c r="D4" t="s">
-        <v>234</v>
+        <v>237</v>
       </c>
       <c r="E4">
         <v>1</v>
@@ -2243,7 +2287,7 @@
         <v>59</v>
       </c>
       <c r="D5" t="s">
-        <v>234</v>
+        <v>237</v>
       </c>
       <c r="E5">
         <v>1</v>
@@ -2260,7 +2304,7 @@
         <v>60</v>
       </c>
       <c r="D6" t="s">
-        <v>235</v>
+        <v>238</v>
       </c>
       <c r="E6">
         <v>1</v>
@@ -2277,7 +2321,7 @@
         <v>61</v>
       </c>
       <c r="D7" t="s">
-        <v>236</v>
+        <v>239</v>
       </c>
       <c r="E7">
         <v>1</v>
@@ -2285,16 +2329,16 @@
     </row>
     <row r="8" spans="1:5">
       <c r="A8" t="s">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="B8" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="C8" t="s">
         <v>61</v>
       </c>
       <c r="D8" t="s">
-        <v>236</v>
+        <v>239</v>
       </c>
       <c r="E8">
         <v>1</v>
@@ -2302,16 +2346,16 @@
     </row>
     <row r="9" spans="1:5">
       <c r="A9" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B9" t="s">
-        <v>40</v>
+        <v>36</v>
       </c>
       <c r="C9" t="s">
         <v>61</v>
       </c>
       <c r="D9" t="s">
-        <v>236</v>
+        <v>239</v>
       </c>
       <c r="E9">
         <v>1</v>
@@ -2319,16 +2363,16 @@
     </row>
     <row r="10" spans="1:5">
       <c r="A10" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="B10" t="s">
-        <v>36</v>
+        <v>40</v>
       </c>
       <c r="C10" t="s">
         <v>61</v>
       </c>
       <c r="D10" t="s">
-        <v>236</v>
+        <v>239</v>
       </c>
       <c r="E10">
         <v>1</v>
@@ -2336,7 +2380,7 @@
     </row>
     <row r="11" spans="1:5">
       <c r="A11" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="B11" t="s">
         <v>40</v>
@@ -2345,7 +2389,7 @@
         <v>61</v>
       </c>
       <c r="D11" t="s">
-        <v>236</v>
+        <v>239</v>
       </c>
       <c r="E11">
         <v>1</v>
@@ -2353,16 +2397,16 @@
     </row>
     <row r="12" spans="1:5">
       <c r="A12" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="B12" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="C12" t="s">
         <v>61</v>
       </c>
       <c r="D12" t="s">
-        <v>236</v>
+        <v>239</v>
       </c>
       <c r="E12">
         <v>1</v>
@@ -2370,16 +2414,16 @@
     </row>
     <row r="13" spans="1:5">
       <c r="A13" t="s">
-        <v>15</v>
+        <v>8</v>
       </c>
       <c r="B13" t="s">
-        <v>41</v>
+        <v>38</v>
       </c>
       <c r="C13" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="D13" t="s">
-        <v>236</v>
+        <v>240</v>
       </c>
       <c r="E13">
         <v>1</v>
@@ -2387,16 +2431,16 @@
     </row>
     <row r="14" spans="1:5">
       <c r="A14" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="B14" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="C14" t="s">
         <v>62</v>
       </c>
       <c r="D14" t="s">
-        <v>237</v>
+        <v>240</v>
       </c>
       <c r="E14">
         <v>1</v>
@@ -2413,7 +2457,7 @@
         <v>62</v>
       </c>
       <c r="D15" t="s">
-        <v>237</v>
+        <v>240</v>
       </c>
       <c r="E15">
         <v>1</v>
@@ -2430,7 +2474,7 @@
         <v>62</v>
       </c>
       <c r="D16" t="s">
-        <v>237</v>
+        <v>240</v>
       </c>
       <c r="E16">
         <v>1</v>
@@ -2447,7 +2491,7 @@
         <v>62</v>
       </c>
       <c r="D17" t="s">
-        <v>237</v>
+        <v>240</v>
       </c>
       <c r="E17">
         <v>1</v>
@@ -2464,7 +2508,7 @@
         <v>62</v>
       </c>
       <c r="D18" t="s">
-        <v>237</v>
+        <v>240</v>
       </c>
       <c r="E18">
         <v>1</v>
@@ -2481,7 +2525,7 @@
         <v>62</v>
       </c>
       <c r="D19" t="s">
-        <v>237</v>
+        <v>240</v>
       </c>
       <c r="E19">
         <v>1</v>
@@ -2498,7 +2542,7 @@
         <v>63</v>
       </c>
       <c r="D20" t="s">
-        <v>238</v>
+        <v>241</v>
       </c>
       <c r="E20">
         <v>1</v>
@@ -2515,7 +2559,7 @@
         <v>64</v>
       </c>
       <c r="D21" t="s">
-        <v>239</v>
+        <v>242</v>
       </c>
       <c r="E21">
         <v>1</v>
@@ -2532,7 +2576,7 @@
         <v>65</v>
       </c>
       <c r="D22" t="s">
-        <v>240</v>
+        <v>243</v>
       </c>
       <c r="E22">
         <v>1</v>
@@ -2549,7 +2593,7 @@
         <v>66</v>
       </c>
       <c r="D23" t="s">
-        <v>241</v>
+        <v>244</v>
       </c>
       <c r="E23">
         <v>1</v>
@@ -2566,7 +2610,7 @@
         <v>67</v>
       </c>
       <c r="D24" t="s">
-        <v>242</v>
+        <v>245</v>
       </c>
       <c r="E24">
         <v>1</v>
@@ -2583,7 +2627,7 @@
         <v>68</v>
       </c>
       <c r="D25" t="s">
-        <v>243</v>
+        <v>246</v>
       </c>
       <c r="E25">
         <v>1</v>
@@ -2600,7 +2644,7 @@
         <v>68</v>
       </c>
       <c r="D26" t="s">
-        <v>243</v>
+        <v>246</v>
       </c>
       <c r="E26">
         <v>1</v>
@@ -2617,7 +2661,7 @@
         <v>68</v>
       </c>
       <c r="D27" t="s">
-        <v>243</v>
+        <v>246</v>
       </c>
       <c r="E27">
         <v>1</v>
@@ -2634,7 +2678,7 @@
         <v>69</v>
       </c>
       <c r="D28" t="s">
-        <v>244</v>
+        <v>247</v>
       </c>
       <c r="E28">
         <v>1</v>
@@ -2651,7 +2695,7 @@
         <v>69</v>
       </c>
       <c r="D29" t="s">
-        <v>244</v>
+        <v>247</v>
       </c>
       <c r="E29">
         <v>1</v>
@@ -2668,7 +2712,7 @@
         <v>69</v>
       </c>
       <c r="D30" t="s">
-        <v>244</v>
+        <v>247</v>
       </c>
       <c r="E30">
         <v>1</v>
@@ -2685,7 +2729,7 @@
         <v>70</v>
       </c>
       <c r="D31" t="s">
-        <v>245</v>
+        <v>248</v>
       </c>
       <c r="E31">
         <v>1</v>
@@ -2702,7 +2746,7 @@
         <v>70</v>
       </c>
       <c r="D32" t="s">
-        <v>245</v>
+        <v>248</v>
       </c>
       <c r="E32">
         <v>1</v>
@@ -2719,7 +2763,7 @@
         <v>71</v>
       </c>
       <c r="D33" t="s">
-        <v>246</v>
+        <v>249</v>
       </c>
       <c r="E33">
         <v>1</v>
@@ -2736,7 +2780,7 @@
         <v>71</v>
       </c>
       <c r="D34" t="s">
-        <v>246</v>
+        <v>249</v>
       </c>
       <c r="E34">
         <v>1</v>
@@ -2753,7 +2797,7 @@
         <v>71</v>
       </c>
       <c r="D35" t="s">
-        <v>246</v>
+        <v>249</v>
       </c>
       <c r="E35">
         <v>1</v>
@@ -2770,7 +2814,7 @@
         <v>72</v>
       </c>
       <c r="D36" t="s">
-        <v>247</v>
+        <v>250</v>
       </c>
       <c r="E36">
         <v>1</v>
@@ -2787,7 +2831,7 @@
         <v>72</v>
       </c>
       <c r="D37" t="s">
-        <v>247</v>
+        <v>250</v>
       </c>
       <c r="E37">
         <v>2</v>
@@ -2804,7 +2848,7 @@
         <v>73</v>
       </c>
       <c r="D38" t="s">
-        <v>248</v>
+        <v>251</v>
       </c>
       <c r="E38">
         <v>1</v>
@@ -2821,7 +2865,7 @@
         <v>74</v>
       </c>
       <c r="D39" t="s">
-        <v>249</v>
+        <v>252</v>
       </c>
       <c r="E39">
         <v>1</v>
@@ -2838,7 +2882,7 @@
         <v>75</v>
       </c>
       <c r="D40" t="s">
-        <v>250</v>
+        <v>253</v>
       </c>
       <c r="E40">
         <v>1</v>
@@ -2855,7 +2899,7 @@
         <v>76</v>
       </c>
       <c r="D41" t="s">
-        <v>251</v>
+        <v>254</v>
       </c>
       <c r="E41">
         <v>1</v>
@@ -2872,7 +2916,7 @@
         <v>77</v>
       </c>
       <c r="D42" t="s">
-        <v>252</v>
+        <v>255</v>
       </c>
       <c r="E42">
         <v>1</v>
@@ -2889,7 +2933,7 @@
         <v>78</v>
       </c>
       <c r="D43" t="s">
-        <v>253</v>
+        <v>256</v>
       </c>
       <c r="E43">
         <v>1</v>
@@ -2906,7 +2950,7 @@
         <v>79</v>
       </c>
       <c r="D44" t="s">
-        <v>254</v>
+        <v>257</v>
       </c>
       <c r="E44">
         <v>1</v>
@@ -2923,7 +2967,7 @@
         <v>80</v>
       </c>
       <c r="D45" t="s">
-        <v>255</v>
+        <v>258</v>
       </c>
       <c r="E45">
         <v>1</v>
@@ -2940,7 +2984,7 @@
         <v>81</v>
       </c>
       <c r="D46" t="s">
-        <v>256</v>
+        <v>259</v>
       </c>
       <c r="E46">
         <v>2</v>
@@ -2957,7 +3001,7 @@
         <v>81</v>
       </c>
       <c r="D47" t="s">
-        <v>256</v>
+        <v>259</v>
       </c>
       <c r="E47">
         <v>3</v>
@@ -2974,7 +3018,7 @@
         <v>81</v>
       </c>
       <c r="D48" t="s">
-        <v>256</v>
+        <v>259</v>
       </c>
       <c r="E48">
         <v>2</v>
@@ -2991,7 +3035,7 @@
         <v>81</v>
       </c>
       <c r="D49" t="s">
-        <v>256</v>
+        <v>259</v>
       </c>
       <c r="E49">
         <v>2</v>
@@ -3008,7 +3052,7 @@
         <v>82</v>
       </c>
       <c r="D50" t="s">
-        <v>257</v>
+        <v>260</v>
       </c>
       <c r="E50">
         <v>2</v>
@@ -3025,7 +3069,7 @@
         <v>82</v>
       </c>
       <c r="D51" t="s">
-        <v>257</v>
+        <v>260</v>
       </c>
       <c r="E51">
         <v>2</v>
@@ -3042,7 +3086,7 @@
         <v>82</v>
       </c>
       <c r="D52" t="s">
-        <v>257</v>
+        <v>260</v>
       </c>
       <c r="E52">
         <v>1</v>
@@ -3059,7 +3103,7 @@
         <v>83</v>
       </c>
       <c r="D53" t="s">
-        <v>258</v>
+        <v>261</v>
       </c>
       <c r="E53">
         <v>2</v>
@@ -3076,7 +3120,7 @@
         <v>83</v>
       </c>
       <c r="D54" t="s">
-        <v>258</v>
+        <v>261</v>
       </c>
       <c r="E54">
         <v>4</v>
@@ -3093,7 +3137,7 @@
         <v>83</v>
       </c>
       <c r="D55" t="s">
-        <v>258</v>
+        <v>261</v>
       </c>
       <c r="E55">
         <v>2</v>
@@ -3110,7 +3154,7 @@
         <v>84</v>
       </c>
       <c r="D56" t="s">
-        <v>259</v>
+        <v>262</v>
       </c>
       <c r="E56">
         <v>2</v>
@@ -3127,7 +3171,7 @@
         <v>84</v>
       </c>
       <c r="D57" t="s">
-        <v>259</v>
+        <v>262</v>
       </c>
       <c r="E57">
         <v>1</v>
@@ -3144,7 +3188,7 @@
         <v>85</v>
       </c>
       <c r="D58" t="s">
-        <v>260</v>
+        <v>263</v>
       </c>
       <c r="E58">
         <v>2</v>
@@ -3161,7 +3205,7 @@
         <v>86</v>
       </c>
       <c r="D59" t="s">
-        <v>261</v>
+        <v>264</v>
       </c>
       <c r="E59">
         <v>2</v>
@@ -3178,7 +3222,7 @@
         <v>87</v>
       </c>
       <c r="D60" t="s">
-        <v>262</v>
+        <v>265</v>
       </c>
       <c r="E60">
         <v>2</v>
@@ -3195,7 +3239,7 @@
         <v>88</v>
       </c>
       <c r="D61" t="s">
-        <v>263</v>
+        <v>266</v>
       </c>
       <c r="E61">
         <v>2</v>
@@ -3212,7 +3256,7 @@
         <v>89</v>
       </c>
       <c r="D62" t="s">
-        <v>264</v>
+        <v>267</v>
       </c>
       <c r="E62">
         <v>2</v>
@@ -3229,7 +3273,7 @@
         <v>90</v>
       </c>
       <c r="D63" t="s">
-        <v>265</v>
+        <v>268</v>
       </c>
       <c r="E63">
         <v>2</v>
@@ -3246,7 +3290,7 @@
         <v>91</v>
       </c>
       <c r="D64" t="s">
-        <v>266</v>
+        <v>269</v>
       </c>
       <c r="E64">
         <v>2</v>
@@ -3263,7 +3307,7 @@
         <v>92</v>
       </c>
       <c r="D65" t="s">
-        <v>256</v>
+        <v>259</v>
       </c>
       <c r="E65">
         <v>2</v>
@@ -3280,7 +3324,7 @@
         <v>93</v>
       </c>
       <c r="D66" t="s">
-        <v>255</v>
+        <v>258</v>
       </c>
       <c r="E66">
         <v>4</v>
@@ -3297,7 +3341,7 @@
         <v>93</v>
       </c>
       <c r="D67" t="s">
-        <v>255</v>
+        <v>258</v>
       </c>
       <c r="E67">
         <v>4</v>
@@ -3314,7 +3358,7 @@
         <v>94</v>
       </c>
       <c r="D68" t="s">
-        <v>267</v>
+        <v>270</v>
       </c>
       <c r="E68">
         <v>4</v>
@@ -3331,7 +3375,7 @@
         <v>95</v>
       </c>
       <c r="D69" t="s">
-        <v>268</v>
+        <v>271</v>
       </c>
       <c r="E69">
         <v>4</v>
@@ -3348,7 +3392,7 @@
         <v>96</v>
       </c>
       <c r="D70" t="s">
-        <v>269</v>
+        <v>272</v>
       </c>
       <c r="E70">
         <v>4</v>
@@ -3365,7 +3409,7 @@
         <v>97</v>
       </c>
       <c r="D71" t="s">
-        <v>270</v>
+        <v>273</v>
       </c>
       <c r="E71">
         <v>1</v>
@@ -3382,7 +3426,7 @@
         <v>97</v>
       </c>
       <c r="D72" t="s">
-        <v>270</v>
+        <v>273</v>
       </c>
       <c r="E72">
         <v>1</v>
@@ -3399,7 +3443,7 @@
         <v>97</v>
       </c>
       <c r="D73" t="s">
-        <v>270</v>
+        <v>273</v>
       </c>
       <c r="E73">
         <v>1</v>
@@ -3416,7 +3460,7 @@
         <v>98</v>
       </c>
       <c r="D74" t="s">
-        <v>271</v>
+        <v>274</v>
       </c>
       <c r="E74">
         <v>1</v>
@@ -3433,7 +3477,7 @@
         <v>98</v>
       </c>
       <c r="D75" t="s">
-        <v>271</v>
+        <v>274</v>
       </c>
       <c r="E75">
         <v>1</v>
@@ -3450,7 +3494,7 @@
         <v>98</v>
       </c>
       <c r="D76" t="s">
-        <v>271</v>
+        <v>274</v>
       </c>
       <c r="E76">
         <v>2</v>
@@ -3467,7 +3511,7 @@
         <v>99</v>
       </c>
       <c r="D77" t="s">
-        <v>272</v>
+        <v>275</v>
       </c>
       <c r="E77">
         <v>1</v>
@@ -3484,7 +3528,7 @@
         <v>99</v>
       </c>
       <c r="D78" t="s">
-        <v>272</v>
+        <v>275</v>
       </c>
       <c r="E78">
         <v>1</v>
@@ -3501,7 +3545,7 @@
         <v>100</v>
       </c>
       <c r="D79" t="s">
-        <v>273</v>
+        <v>276</v>
       </c>
       <c r="E79">
         <v>1</v>
@@ -3518,7 +3562,7 @@
         <v>100</v>
       </c>
       <c r="D80" t="s">
-        <v>273</v>
+        <v>276</v>
       </c>
       <c r="E80">
         <v>1</v>
@@ -3535,7 +3579,7 @@
         <v>101</v>
       </c>
       <c r="D81" t="s">
-        <v>274</v>
+        <v>277</v>
       </c>
       <c r="E81">
         <v>1</v>
@@ -3552,7 +3596,7 @@
         <v>101</v>
       </c>
       <c r="D82" t="s">
-        <v>274</v>
+        <v>277</v>
       </c>
       <c r="E82">
         <v>1</v>
@@ -3569,7 +3613,7 @@
         <v>102</v>
       </c>
       <c r="D83" t="s">
-        <v>275</v>
+        <v>278</v>
       </c>
       <c r="E83">
         <v>1</v>
@@ -3586,7 +3630,7 @@
         <v>102</v>
       </c>
       <c r="D84" t="s">
-        <v>275</v>
+        <v>278</v>
       </c>
       <c r="E84">
         <v>1</v>
@@ -3603,7 +3647,7 @@
         <v>103</v>
       </c>
       <c r="D85" t="s">
-        <v>276</v>
+        <v>279</v>
       </c>
       <c r="E85">
         <v>1</v>
@@ -3620,7 +3664,7 @@
         <v>103</v>
       </c>
       <c r="D86" t="s">
-        <v>276</v>
+        <v>279</v>
       </c>
       <c r="E86">
         <v>1</v>
@@ -3637,7 +3681,7 @@
         <v>104</v>
       </c>
       <c r="D87" t="s">
-        <v>277</v>
+        <v>280</v>
       </c>
       <c r="E87">
         <v>1</v>
@@ -3654,7 +3698,7 @@
         <v>104</v>
       </c>
       <c r="D88" t="s">
-        <v>277</v>
+        <v>280</v>
       </c>
       <c r="E88">
         <v>1</v>
@@ -3671,7 +3715,7 @@
         <v>105</v>
       </c>
       <c r="D89" t="s">
-        <v>278</v>
+        <v>281</v>
       </c>
       <c r="E89">
         <v>1</v>
@@ -3688,7 +3732,7 @@
         <v>105</v>
       </c>
       <c r="D90" t="s">
-        <v>278</v>
+        <v>281</v>
       </c>
       <c r="E90">
         <v>1</v>
@@ -3705,7 +3749,7 @@
         <v>106</v>
       </c>
       <c r="D91" t="s">
-        <v>279</v>
+        <v>282</v>
       </c>
       <c r="E91">
         <v>1</v>
@@ -3722,7 +3766,7 @@
         <v>106</v>
       </c>
       <c r="D92" t="s">
-        <v>279</v>
+        <v>282</v>
       </c>
       <c r="E92">
         <v>1</v>
@@ -3739,7 +3783,7 @@
         <v>107</v>
       </c>
       <c r="D93" t="s">
-        <v>280</v>
+        <v>283</v>
       </c>
       <c r="E93">
         <v>1</v>
@@ -3756,7 +3800,7 @@
         <v>107</v>
       </c>
       <c r="D94" t="s">
-        <v>280</v>
+        <v>283</v>
       </c>
       <c r="E94">
         <v>1</v>
@@ -3773,7 +3817,7 @@
         <v>108</v>
       </c>
       <c r="D95" t="s">
-        <v>281</v>
+        <v>284</v>
       </c>
       <c r="E95">
         <v>1</v>
@@ -3790,7 +3834,7 @@
         <v>108</v>
       </c>
       <c r="D96" t="s">
-        <v>281</v>
+        <v>284</v>
       </c>
       <c r="E96">
         <v>1</v>
@@ -3807,7 +3851,7 @@
         <v>109</v>
       </c>
       <c r="D97" t="s">
-        <v>282</v>
+        <v>285</v>
       </c>
       <c r="E97">
         <v>1</v>
@@ -3824,7 +3868,7 @@
         <v>110</v>
       </c>
       <c r="D98" t="s">
-        <v>283</v>
+        <v>286</v>
       </c>
       <c r="E98">
         <v>1</v>
@@ -3841,7 +3885,7 @@
         <v>111</v>
       </c>
       <c r="D99" t="s">
-        <v>284</v>
+        <v>287</v>
       </c>
       <c r="E99">
         <v>1</v>
@@ -3858,7 +3902,7 @@
         <v>112</v>
       </c>
       <c r="D100" t="s">
-        <v>285</v>
+        <v>288</v>
       </c>
       <c r="E100">
         <v>1</v>
@@ -3875,7 +3919,7 @@
         <v>113</v>
       </c>
       <c r="D101" t="s">
-        <v>286</v>
+        <v>289</v>
       </c>
       <c r="E101">
         <v>1</v>
@@ -3892,7 +3936,7 @@
         <v>114</v>
       </c>
       <c r="D102" t="s">
-        <v>287</v>
+        <v>290</v>
       </c>
       <c r="E102">
         <v>1</v>
@@ -3909,7 +3953,7 @@
         <v>115</v>
       </c>
       <c r="D103" t="s">
-        <v>288</v>
+        <v>291</v>
       </c>
       <c r="E103">
         <v>2</v>
@@ -3926,7 +3970,7 @@
         <v>115</v>
       </c>
       <c r="D104" t="s">
-        <v>288</v>
+        <v>291</v>
       </c>
       <c r="E104">
         <v>1</v>
@@ -3943,7 +3987,7 @@
         <v>116</v>
       </c>
       <c r="D105" t="s">
-        <v>289</v>
+        <v>292</v>
       </c>
       <c r="E105">
         <v>2</v>
@@ -3960,7 +4004,7 @@
         <v>116</v>
       </c>
       <c r="D106" t="s">
-        <v>289</v>
+        <v>292</v>
       </c>
       <c r="E106">
         <v>2</v>
@@ -3977,7 +4021,7 @@
         <v>116</v>
       </c>
       <c r="D107" t="s">
-        <v>289</v>
+        <v>292</v>
       </c>
       <c r="E107">
         <v>2</v>
@@ -3994,7 +4038,7 @@
         <v>117</v>
       </c>
       <c r="D108" t="s">
-        <v>290</v>
+        <v>293</v>
       </c>
       <c r="E108">
         <v>2</v>
@@ -4011,7 +4055,7 @@
         <v>117</v>
       </c>
       <c r="D109" t="s">
-        <v>290</v>
+        <v>293</v>
       </c>
       <c r="E109">
         <v>2</v>
@@ -4028,7 +4072,7 @@
         <v>117</v>
       </c>
       <c r="D110" t="s">
-        <v>290</v>
+        <v>293</v>
       </c>
       <c r="E110">
         <v>2</v>
@@ -4045,7 +4089,7 @@
         <v>118</v>
       </c>
       <c r="D111" t="s">
-        <v>291</v>
+        <v>294</v>
       </c>
       <c r="E111">
         <v>2</v>
@@ -4062,7 +4106,7 @@
         <v>118</v>
       </c>
       <c r="D112" t="s">
-        <v>291</v>
+        <v>294</v>
       </c>
       <c r="E112">
         <v>2</v>
@@ -4079,7 +4123,7 @@
         <v>119</v>
       </c>
       <c r="D113" t="s">
-        <v>292</v>
+        <v>295</v>
       </c>
       <c r="E113">
         <v>2</v>
@@ -4096,7 +4140,7 @@
         <v>119</v>
       </c>
       <c r="D114" t="s">
-        <v>292</v>
+        <v>295</v>
       </c>
       <c r="E114">
         <v>2</v>
@@ -4113,7 +4157,7 @@
         <v>120</v>
       </c>
       <c r="D115" t="s">
-        <v>271</v>
+        <v>274</v>
       </c>
       <c r="E115">
         <v>2</v>
@@ -4130,7 +4174,7 @@
         <v>120</v>
       </c>
       <c r="D116" t="s">
-        <v>271</v>
+        <v>274</v>
       </c>
       <c r="E116">
         <v>4</v>
@@ -4147,7 +4191,7 @@
         <v>120</v>
       </c>
       <c r="D117" t="s">
-        <v>271</v>
+        <v>274</v>
       </c>
       <c r="E117">
         <v>4</v>
@@ -4164,7 +4208,7 @@
         <v>121</v>
       </c>
       <c r="D118" t="s">
-        <v>293</v>
+        <v>296</v>
       </c>
       <c r="E118">
         <v>2</v>
@@ -4181,7 +4225,7 @@
         <v>121</v>
       </c>
       <c r="D119" t="s">
-        <v>293</v>
+        <v>296</v>
       </c>
       <c r="E119">
         <v>4</v>
@@ -4198,7 +4242,7 @@
         <v>122</v>
       </c>
       <c r="D120" t="s">
-        <v>277</v>
+        <v>280</v>
       </c>
       <c r="E120">
         <v>2</v>
@@ -4215,7 +4259,7 @@
         <v>123</v>
       </c>
       <c r="D121" t="s">
-        <v>294</v>
+        <v>297</v>
       </c>
       <c r="E121">
         <v>2</v>
@@ -4232,7 +4276,7 @@
         <v>124</v>
       </c>
       <c r="D122" t="s">
-        <v>295</v>
+        <v>298</v>
       </c>
       <c r="E122">
         <v>2</v>
@@ -4249,7 +4293,7 @@
         <v>125</v>
       </c>
       <c r="D123" t="s">
-        <v>296</v>
+        <v>299</v>
       </c>
       <c r="E123">
         <v>5</v>
@@ -4266,7 +4310,7 @@
         <v>125</v>
       </c>
       <c r="D124" t="s">
-        <v>296</v>
+        <v>299</v>
       </c>
       <c r="E124">
         <v>5</v>
@@ -4283,7 +4327,7 @@
         <v>126</v>
       </c>
       <c r="D125" t="s">
-        <v>297</v>
+        <v>300</v>
       </c>
       <c r="E125">
         <v>7</v>
@@ -4300,7 +4344,7 @@
         <v>127</v>
       </c>
       <c r="D126" t="s">
-        <v>298</v>
+        <v>301</v>
       </c>
       <c r="E126">
         <v>8</v>
@@ -4317,7 +4361,7 @@
         <v>128</v>
       </c>
       <c r="D127" t="s">
-        <v>299</v>
+        <v>302</v>
       </c>
       <c r="E127">
         <v>10</v>
@@ -4334,7 +4378,7 @@
         <v>129</v>
       </c>
       <c r="D128" t="s">
-        <v>300</v>
+        <v>303</v>
       </c>
       <c r="E128">
         <v>30</v>
@@ -4351,7 +4395,7 @@
         <v>129</v>
       </c>
       <c r="D129" t="s">
-        <v>300</v>
+        <v>303</v>
       </c>
       <c r="E129">
         <v>30</v>
@@ -4368,7 +4412,7 @@
         <v>130</v>
       </c>
       <c r="D130" t="s">
-        <v>301</v>
+        <v>304</v>
       </c>
       <c r="E130">
         <v>1</v>
@@ -4385,7 +4429,7 @@
         <v>130</v>
       </c>
       <c r="D131" t="s">
-        <v>301</v>
+        <v>304</v>
       </c>
       <c r="E131">
         <v>1</v>
@@ -4402,7 +4446,7 @@
         <v>131</v>
       </c>
       <c r="D132" t="s">
-        <v>302</v>
+        <v>305</v>
       </c>
       <c r="E132">
         <v>1</v>
@@ -4419,7 +4463,7 @@
         <v>132</v>
       </c>
       <c r="D133" t="s">
-        <v>303</v>
+        <v>306</v>
       </c>
       <c r="E133">
         <v>1</v>
@@ -4436,7 +4480,7 @@
         <v>133</v>
       </c>
       <c r="D134" t="s">
-        <v>304</v>
+        <v>307</v>
       </c>
       <c r="E134">
         <v>1</v>
@@ -4453,7 +4497,7 @@
         <v>134</v>
       </c>
       <c r="D135" t="s">
-        <v>305</v>
+        <v>308</v>
       </c>
       <c r="E135">
         <v>1</v>
@@ -4470,7 +4514,7 @@
         <v>135</v>
       </c>
       <c r="D136" t="s">
-        <v>306</v>
+        <v>309</v>
       </c>
       <c r="E136">
         <v>1</v>
@@ -4487,7 +4531,7 @@
         <v>136</v>
       </c>
       <c r="D137" t="s">
-        <v>307</v>
+        <v>310</v>
       </c>
       <c r="E137">
         <v>1</v>
@@ -4504,7 +4548,7 @@
         <v>137</v>
       </c>
       <c r="D138" t="s">
-        <v>308</v>
+        <v>311</v>
       </c>
       <c r="E138">
         <v>1</v>
@@ -4521,7 +4565,7 @@
         <v>138</v>
       </c>
       <c r="D139" t="s">
-        <v>309</v>
+        <v>312</v>
       </c>
       <c r="E139">
         <v>1</v>
@@ -4538,7 +4582,7 @@
         <v>139</v>
       </c>
       <c r="D140" t="s">
-        <v>310</v>
+        <v>313</v>
       </c>
       <c r="E140">
         <v>1</v>
@@ -4555,7 +4599,7 @@
         <v>140</v>
       </c>
       <c r="D141" t="s">
-        <v>311</v>
+        <v>314</v>
       </c>
       <c r="E141">
         <v>1</v>
@@ -4572,7 +4616,7 @@
         <v>141</v>
       </c>
       <c r="D142" t="s">
-        <v>312</v>
+        <v>315</v>
       </c>
       <c r="E142">
         <v>1</v>
@@ -4589,7 +4633,7 @@
         <v>142</v>
       </c>
       <c r="D143" t="s">
-        <v>313</v>
+        <v>316</v>
       </c>
       <c r="E143">
         <v>1</v>
@@ -4606,7 +4650,7 @@
         <v>143</v>
       </c>
       <c r="D144" t="s">
-        <v>314</v>
+        <v>317</v>
       </c>
       <c r="E144">
         <v>1</v>
@@ -4623,7 +4667,7 @@
         <v>144</v>
       </c>
       <c r="D145" t="s">
-        <v>315</v>
+        <v>318</v>
       </c>
       <c r="E145">
         <v>1</v>
@@ -4640,7 +4684,7 @@
         <v>145</v>
       </c>
       <c r="D146" t="s">
-        <v>316</v>
+        <v>319</v>
       </c>
       <c r="E146">
         <v>1</v>
@@ -4657,7 +4701,7 @@
         <v>146</v>
       </c>
       <c r="D147" t="s">
-        <v>317</v>
+        <v>320</v>
       </c>
       <c r="E147">
         <v>1</v>
@@ -4674,7 +4718,7 @@
         <v>147</v>
       </c>
       <c r="D148" t="s">
-        <v>318</v>
+        <v>321</v>
       </c>
       <c r="E148">
         <v>1</v>
@@ -4691,7 +4735,7 @@
         <v>148</v>
       </c>
       <c r="D149" t="s">
-        <v>319</v>
+        <v>322</v>
       </c>
       <c r="E149">
         <v>1</v>
@@ -4708,7 +4752,7 @@
         <v>149</v>
       </c>
       <c r="D150" t="s">
-        <v>320</v>
+        <v>323</v>
       </c>
       <c r="E150">
         <v>1</v>
@@ -4725,7 +4769,7 @@
         <v>150</v>
       </c>
       <c r="D151" t="s">
-        <v>321</v>
+        <v>324</v>
       </c>
       <c r="E151">
         <v>1</v>
@@ -4742,7 +4786,7 @@
         <v>151</v>
       </c>
       <c r="D152" t="s">
-        <v>322</v>
+        <v>325</v>
       </c>
       <c r="E152">
         <v>1</v>
@@ -4759,7 +4803,7 @@
         <v>152</v>
       </c>
       <c r="D153" t="s">
-        <v>323</v>
+        <v>326</v>
       </c>
       <c r="E153">
         <v>1</v>
@@ -4776,7 +4820,7 @@
         <v>153</v>
       </c>
       <c r="D154" t="s">
-        <v>324</v>
+        <v>327</v>
       </c>
       <c r="E154">
         <v>1</v>
@@ -4793,7 +4837,7 @@
         <v>154</v>
       </c>
       <c r="D155" t="s">
-        <v>325</v>
+        <v>328</v>
       </c>
       <c r="E155">
         <v>1</v>
@@ -4810,7 +4854,7 @@
         <v>155</v>
       </c>
       <c r="D156" t="s">
-        <v>326</v>
+        <v>329</v>
       </c>
       <c r="E156">
         <v>1</v>
@@ -4827,7 +4871,7 @@
         <v>156</v>
       </c>
       <c r="D157" t="s">
-        <v>327</v>
+        <v>330</v>
       </c>
       <c r="E157">
         <v>1</v>
@@ -4844,7 +4888,7 @@
         <v>157</v>
       </c>
       <c r="D158" t="s">
-        <v>328</v>
+        <v>331</v>
       </c>
       <c r="E158">
         <v>1</v>
@@ -4861,7 +4905,7 @@
         <v>158</v>
       </c>
       <c r="D159" t="s">
-        <v>329</v>
+        <v>332</v>
       </c>
       <c r="E159">
         <v>1</v>
@@ -4878,7 +4922,7 @@
         <v>159</v>
       </c>
       <c r="D160" t="s">
-        <v>330</v>
+        <v>333</v>
       </c>
       <c r="E160">
         <v>1</v>
@@ -4895,7 +4939,7 @@
         <v>160</v>
       </c>
       <c r="D161" t="s">
-        <v>331</v>
+        <v>334</v>
       </c>
       <c r="E161">
         <v>1</v>
@@ -4912,7 +4956,7 @@
         <v>161</v>
       </c>
       <c r="D162" t="s">
-        <v>316</v>
+        <v>319</v>
       </c>
       <c r="E162">
         <v>2</v>
@@ -4929,7 +4973,7 @@
         <v>162</v>
       </c>
       <c r="D163" t="s">
-        <v>332</v>
+        <v>335</v>
       </c>
       <c r="E163">
         <v>2</v>
@@ -4946,7 +4990,7 @@
         <v>163</v>
       </c>
       <c r="D164" t="s">
-        <v>333</v>
+        <v>336</v>
       </c>
       <c r="E164">
         <v>2</v>
@@ -4963,7 +5007,7 @@
         <v>164</v>
       </c>
       <c r="D165" t="s">
-        <v>334</v>
+        <v>337</v>
       </c>
       <c r="E165">
         <v>2</v>
@@ -4980,7 +5024,7 @@
         <v>165</v>
       </c>
       <c r="D166" t="s">
-        <v>335</v>
+        <v>338</v>
       </c>
       <c r="E166">
         <v>2</v>
@@ -4997,7 +5041,7 @@
         <v>166</v>
       </c>
       <c r="D167" t="s">
-        <v>336</v>
+        <v>339</v>
       </c>
       <c r="E167">
         <v>3</v>
@@ -5014,7 +5058,7 @@
         <v>167</v>
       </c>
       <c r="D168" t="s">
-        <v>300</v>
+        <v>303</v>
       </c>
       <c r="E168">
         <v>5</v>
@@ -5031,7 +5075,7 @@
         <v>168</v>
       </c>
       <c r="D169" t="s">
-        <v>337</v>
+        <v>340</v>
       </c>
       <c r="E169">
         <v>8</v>
@@ -5048,7 +5092,7 @@
         <v>169</v>
       </c>
       <c r="D170" t="s">
-        <v>252</v>
+        <v>255</v>
       </c>
       <c r="E170">
         <v>8</v>
@@ -5065,7 +5109,7 @@
         <v>170</v>
       </c>
       <c r="D171" t="s">
-        <v>338</v>
+        <v>341</v>
       </c>
       <c r="E171">
         <v>10</v>
@@ -5073,16 +5117,16 @@
     </row>
     <row r="172" spans="1:5">
       <c r="A172" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B172" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C172" t="s">
         <v>171</v>
       </c>
       <c r="D172" t="s">
-        <v>326</v>
+        <v>342</v>
       </c>
       <c r="E172">
         <v>1</v>
@@ -5090,16 +5134,16 @@
     </row>
     <row r="173" spans="1:5">
       <c r="A173" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B173" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C173" t="s">
         <v>172</v>
       </c>
       <c r="D173" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="E173">
         <v>1</v>
@@ -5116,7 +5160,7 @@
         <v>173</v>
       </c>
       <c r="D174" t="s">
-        <v>340</v>
+        <v>329</v>
       </c>
       <c r="E174">
         <v>1</v>
@@ -5133,7 +5177,7 @@
         <v>174</v>
       </c>
       <c r="D175" t="s">
-        <v>341</v>
+        <v>344</v>
       </c>
       <c r="E175">
         <v>1</v>
@@ -5150,7 +5194,7 @@
         <v>175</v>
       </c>
       <c r="D176" t="s">
-        <v>342</v>
+        <v>345</v>
       </c>
       <c r="E176">
         <v>1</v>
@@ -5167,7 +5211,7 @@
         <v>176</v>
       </c>
       <c r="D177" t="s">
-        <v>343</v>
+        <v>346</v>
       </c>
       <c r="E177">
         <v>1</v>
@@ -5184,7 +5228,7 @@
         <v>177</v>
       </c>
       <c r="D178" t="s">
-        <v>262</v>
+        <v>347</v>
       </c>
       <c r="E178">
         <v>1</v>
@@ -5201,7 +5245,7 @@
         <v>178</v>
       </c>
       <c r="D179" t="s">
-        <v>344</v>
+        <v>348</v>
       </c>
       <c r="E179">
         <v>1</v>
@@ -5218,7 +5262,7 @@
         <v>179</v>
       </c>
       <c r="D180" t="s">
-        <v>345</v>
+        <v>265</v>
       </c>
       <c r="E180">
         <v>1</v>
@@ -5235,7 +5279,7 @@
         <v>180</v>
       </c>
       <c r="D181" t="s">
-        <v>346</v>
+        <v>349</v>
       </c>
       <c r="E181">
         <v>1</v>
@@ -5252,7 +5296,7 @@
         <v>181</v>
       </c>
       <c r="D182" t="s">
-        <v>347</v>
+        <v>350</v>
       </c>
       <c r="E182">
         <v>1</v>
@@ -5269,7 +5313,7 @@
         <v>182</v>
       </c>
       <c r="D183" t="s">
-        <v>348</v>
+        <v>351</v>
       </c>
       <c r="E183">
         <v>1</v>
@@ -5286,7 +5330,7 @@
         <v>183</v>
       </c>
       <c r="D184" t="s">
-        <v>349</v>
+        <v>352</v>
       </c>
       <c r="E184">
         <v>1</v>
@@ -5303,7 +5347,7 @@
         <v>184</v>
       </c>
       <c r="D185" t="s">
-        <v>350</v>
+        <v>353</v>
       </c>
       <c r="E185">
         <v>1</v>
@@ -5320,7 +5364,7 @@
         <v>185</v>
       </c>
       <c r="D186" t="s">
-        <v>351</v>
+        <v>354</v>
       </c>
       <c r="E186">
         <v>1</v>
@@ -5337,7 +5381,7 @@
         <v>186</v>
       </c>
       <c r="D187" t="s">
-        <v>352</v>
+        <v>355</v>
       </c>
       <c r="E187">
         <v>1</v>
@@ -5354,7 +5398,7 @@
         <v>187</v>
       </c>
       <c r="D188" t="s">
-        <v>353</v>
+        <v>356</v>
       </c>
       <c r="E188">
         <v>1</v>
@@ -5371,7 +5415,7 @@
         <v>188</v>
       </c>
       <c r="D189" t="s">
-        <v>354</v>
+        <v>357</v>
       </c>
       <c r="E189">
         <v>1</v>
@@ -5388,7 +5432,7 @@
         <v>189</v>
       </c>
       <c r="D190" t="s">
-        <v>355</v>
+        <v>358</v>
       </c>
       <c r="E190">
         <v>1</v>
@@ -5405,7 +5449,7 @@
         <v>190</v>
       </c>
       <c r="D191" t="s">
-        <v>356</v>
+        <v>359</v>
       </c>
       <c r="E191">
         <v>1</v>
@@ -5422,7 +5466,7 @@
         <v>191</v>
       </c>
       <c r="D192" t="s">
-        <v>357</v>
+        <v>360</v>
       </c>
       <c r="E192">
         <v>1</v>
@@ -5439,7 +5483,7 @@
         <v>192</v>
       </c>
       <c r="D193" t="s">
-        <v>358</v>
+        <v>361</v>
       </c>
       <c r="E193">
         <v>1</v>
@@ -5456,7 +5500,7 @@
         <v>193</v>
       </c>
       <c r="D194" t="s">
-        <v>359</v>
+        <v>362</v>
       </c>
       <c r="E194">
         <v>1</v>
@@ -5473,7 +5517,7 @@
         <v>194</v>
       </c>
       <c r="D195" t="s">
-        <v>360</v>
+        <v>363</v>
       </c>
       <c r="E195">
         <v>1</v>
@@ -5490,7 +5534,7 @@
         <v>195</v>
       </c>
       <c r="D196" t="s">
-        <v>361</v>
+        <v>364</v>
       </c>
       <c r="E196">
         <v>1</v>
@@ -5507,7 +5551,7 @@
         <v>196</v>
       </c>
       <c r="D197" t="s">
-        <v>362</v>
+        <v>365</v>
       </c>
       <c r="E197">
         <v>1</v>
@@ -5524,7 +5568,7 @@
         <v>197</v>
       </c>
       <c r="D198" t="s">
-        <v>363</v>
+        <v>366</v>
       </c>
       <c r="E198">
         <v>1</v>
@@ -5541,7 +5585,7 @@
         <v>198</v>
       </c>
       <c r="D199" t="s">
-        <v>364</v>
+        <v>367</v>
       </c>
       <c r="E199">
         <v>1</v>
@@ -5558,7 +5602,7 @@
         <v>199</v>
       </c>
       <c r="D200" t="s">
-        <v>365</v>
+        <v>368</v>
       </c>
       <c r="E200">
         <v>1</v>
@@ -5575,7 +5619,7 @@
         <v>200</v>
       </c>
       <c r="D201" t="s">
-        <v>366</v>
+        <v>369</v>
       </c>
       <c r="E201">
         <v>1</v>
@@ -5592,7 +5636,7 @@
         <v>201</v>
       </c>
       <c r="D202" t="s">
-        <v>367</v>
+        <v>370</v>
       </c>
       <c r="E202">
         <v>1</v>
@@ -5609,7 +5653,7 @@
         <v>202</v>
       </c>
       <c r="D203" t="s">
-        <v>368</v>
+        <v>371</v>
       </c>
       <c r="E203">
         <v>1</v>
@@ -5626,10 +5670,10 @@
         <v>203</v>
       </c>
       <c r="D204" t="s">
-        <v>369</v>
+        <v>372</v>
       </c>
       <c r="E204">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="205" spans="1:5">
@@ -5643,10 +5687,10 @@
         <v>204</v>
       </c>
       <c r="D205" t="s">
-        <v>370</v>
+        <v>373</v>
       </c>
       <c r="E205">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="206" spans="1:5">
@@ -5660,7 +5704,7 @@
         <v>205</v>
       </c>
       <c r="D206" t="s">
-        <v>371</v>
+        <v>374</v>
       </c>
       <c r="E206">
         <v>2</v>
@@ -5677,7 +5721,7 @@
         <v>206</v>
       </c>
       <c r="D207" t="s">
-        <v>372</v>
+        <v>375</v>
       </c>
       <c r="E207">
         <v>2</v>
@@ -5694,7 +5738,7 @@
         <v>207</v>
       </c>
       <c r="D208" t="s">
-        <v>373</v>
+        <v>376</v>
       </c>
       <c r="E208">
         <v>2</v>
@@ -5711,7 +5755,7 @@
         <v>208</v>
       </c>
       <c r="D209" t="s">
-        <v>374</v>
+        <v>377</v>
       </c>
       <c r="E209">
         <v>2</v>
@@ -5728,7 +5772,7 @@
         <v>209</v>
       </c>
       <c r="D210" t="s">
-        <v>375</v>
+        <v>378</v>
       </c>
       <c r="E210">
         <v>2</v>
@@ -5745,7 +5789,7 @@
         <v>210</v>
       </c>
       <c r="D211" t="s">
-        <v>376</v>
+        <v>379</v>
       </c>
       <c r="E211">
         <v>2</v>
@@ -5762,7 +5806,7 @@
         <v>211</v>
       </c>
       <c r="D212" t="s">
-        <v>376</v>
+        <v>380</v>
       </c>
       <c r="E212">
         <v>2</v>
@@ -5779,7 +5823,7 @@
         <v>212</v>
       </c>
       <c r="D213" t="s">
-        <v>377</v>
+        <v>381</v>
       </c>
       <c r="E213">
         <v>2</v>
@@ -5796,7 +5840,7 @@
         <v>213</v>
       </c>
       <c r="D214" t="s">
-        <v>378</v>
+        <v>381</v>
       </c>
       <c r="E214">
         <v>2</v>
@@ -5813,7 +5857,7 @@
         <v>214</v>
       </c>
       <c r="D215" t="s">
-        <v>379</v>
+        <v>382</v>
       </c>
       <c r="E215">
         <v>2</v>
@@ -5830,10 +5874,10 @@
         <v>215</v>
       </c>
       <c r="D216" t="s">
-        <v>380</v>
+        <v>383</v>
       </c>
       <c r="E216">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="217" spans="1:5">
@@ -5847,10 +5891,10 @@
         <v>216</v>
       </c>
       <c r="D217" t="s">
-        <v>262</v>
+        <v>384</v>
       </c>
       <c r="E217">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="218" spans="1:5">
@@ -5864,10 +5908,10 @@
         <v>217</v>
       </c>
       <c r="D218" t="s">
-        <v>381</v>
+        <v>385</v>
       </c>
       <c r="E218">
-        <v>4</v>
+        <v>3</v>
       </c>
     </row>
     <row r="219" spans="1:5">
@@ -5881,10 +5925,10 @@
         <v>218</v>
       </c>
       <c r="D219" t="s">
-        <v>382</v>
+        <v>265</v>
       </c>
       <c r="E219">
-        <v>4</v>
+        <v>3</v>
       </c>
     </row>
     <row r="220" spans="1:5">
@@ -5898,7 +5942,7 @@
         <v>219</v>
       </c>
       <c r="D220" t="s">
-        <v>383</v>
+        <v>386</v>
       </c>
       <c r="E220">
         <v>4</v>
@@ -5915,7 +5959,7 @@
         <v>220</v>
       </c>
       <c r="D221" t="s">
-        <v>384</v>
+        <v>387</v>
       </c>
       <c r="E221">
         <v>4</v>
@@ -5932,7 +5976,7 @@
         <v>221</v>
       </c>
       <c r="D222" t="s">
-        <v>385</v>
+        <v>388</v>
       </c>
       <c r="E222">
         <v>4</v>
@@ -5949,10 +5993,10 @@
         <v>222</v>
       </c>
       <c r="D223" t="s">
-        <v>386</v>
+        <v>389</v>
       </c>
       <c r="E223">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="224" spans="1:5">
@@ -5966,10 +6010,10 @@
         <v>223</v>
       </c>
       <c r="D224" t="s">
-        <v>387</v>
+        <v>390</v>
       </c>
       <c r="E224">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="225" spans="1:5">
@@ -5983,10 +6027,10 @@
         <v>224</v>
       </c>
       <c r="D225" t="s">
-        <v>388</v>
+        <v>391</v>
       </c>
       <c r="E225">
-        <v>6</v>
+        <v>5</v>
       </c>
     </row>
     <row r="226" spans="1:5">
@@ -6000,10 +6044,10 @@
         <v>225</v>
       </c>
       <c r="D226" t="s">
-        <v>389</v>
+        <v>392</v>
       </c>
       <c r="E226">
-        <v>8</v>
+        <v>5</v>
       </c>
     </row>
     <row r="227" spans="1:5">
@@ -6017,10 +6061,10 @@
         <v>226</v>
       </c>
       <c r="D227" t="s">
-        <v>390</v>
+        <v>393</v>
       </c>
       <c r="E227">
-        <v>10</v>
+        <v>6</v>
       </c>
     </row>
     <row r="228" spans="1:5">
@@ -6034,10 +6078,10 @@
         <v>227</v>
       </c>
       <c r="D228" t="s">
-        <v>390</v>
+        <v>394</v>
       </c>
       <c r="E228">
-        <v>10</v>
+        <v>8</v>
       </c>
     </row>
     <row r="229" spans="1:5">
@@ -6051,10 +6095,10 @@
         <v>228</v>
       </c>
       <c r="D229" t="s">
-        <v>264</v>
+        <v>395</v>
       </c>
       <c r="E229">
-        <v>12</v>
+        <v>10</v>
       </c>
     </row>
     <row r="230" spans="1:5">
@@ -6068,10 +6112,10 @@
         <v>229</v>
       </c>
       <c r="D230" t="s">
-        <v>391</v>
+        <v>395</v>
       </c>
       <c r="E230">
-        <v>12</v>
+        <v>10</v>
       </c>
     </row>
     <row r="231" spans="1:5">
@@ -6085,10 +6129,10 @@
         <v>230</v>
       </c>
       <c r="D231" t="s">
-        <v>392</v>
+        <v>267</v>
       </c>
       <c r="E231">
-        <v>14</v>
+        <v>12</v>
       </c>
     </row>
     <row r="232" spans="1:5">
@@ -6102,10 +6146,10 @@
         <v>231</v>
       </c>
       <c r="D232" t="s">
-        <v>393</v>
+        <v>396</v>
       </c>
       <c r="E232">
-        <v>15</v>
+        <v>12</v>
       </c>
     </row>
     <row r="233" spans="1:5">
@@ -6119,10 +6163,61 @@
         <v>232</v>
       </c>
       <c r="D233" t="s">
-        <v>394</v>
+        <v>397</v>
       </c>
       <c r="E233">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="234" spans="1:5">
+      <c r="A234" t="s">
+        <v>15</v>
+      </c>
+      <c r="B234" t="s">
+        <v>41</v>
+      </c>
+      <c r="C234" t="s">
+        <v>233</v>
+      </c>
+      <c r="D234" t="s">
+        <v>398</v>
+      </c>
+      <c r="E234">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="235" spans="1:5">
+      <c r="A235" t="s">
+        <v>15</v>
+      </c>
+      <c r="B235" t="s">
+        <v>41</v>
+      </c>
+      <c r="C235" t="s">
+        <v>234</v>
+      </c>
+      <c r="D235" t="s">
+        <v>399</v>
+      </c>
+      <c r="E235">
         <v>20</v>
+      </c>
+    </row>
+    <row r="236" spans="1:5">
+      <c r="A236" t="s">
+        <v>6</v>
+      </c>
+      <c r="B236" t="s">
+        <v>36</v>
+      </c>
+      <c r="C236" t="s">
+        <v>235</v>
+      </c>
+      <c r="D236" t="s">
+        <v>400</v>
+      </c>
+      <c r="E236">
+        <v>1</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Atualização automática: rac (28/09/2026 15:34)
</commit_message>
<xml_diff>
--- a/Coordenadoria/02_Dados_Tratados/base_rac_tratada.xlsx
+++ b/Coordenadoria/02_Dados_Tratados/base_rac_tratada.xlsx
@@ -1224,16 +1224,8 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <fonts count="2">
+  <fonts count="1">
     <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -1249,7 +1241,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -1257,30 +1249,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color auto="1"/>
-      </left>
-      <right style="thin">
-        <color auto="1"/>
-      </right>
-      <top style="thin">
-        <color auto="1"/>
-      </top>
-      <bottom style="thin">
-        <color auto="1"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1579,22 +1553,22 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:6">
-      <c r="A1" s="1" t="s">
+      <c r="A1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" s="1" t="s">
+      <c r="B1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" t="s">
         <v>5</v>
       </c>
     </row>
@@ -2209,19 +2183,19 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:5">
-      <c r="A1" s="1" t="s">
+      <c r="A1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" s="1" t="s">
+      <c r="B1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" t="s">
         <v>55</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" t="s">
         <v>56</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" t="s">
         <v>57</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualização automática: rac (29/09/2026 13:52)
</commit_message>
<xml_diff>
--- a/Coordenadoria/02_Dados_Tratados/base_rac_tratada.xlsx
+++ b/Coordenadoria/02_Dados_Tratados/base_rac_tratada.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1071" uniqueCount="401">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1071" uniqueCount="399">
   <si>
     <t>matricula</t>
   </si>
@@ -197,9 +197,6 @@
     <t>2698010-7</t>
   </si>
   <si>
-    <t>3034792</t>
-  </si>
-  <si>
     <t>3044000</t>
   </si>
   <si>
@@ -729,9 +726,6 @@
   </si>
   <si>
     <t>PASSENGER DOOR - LOW</t>
-  </si>
-  <si>
-    <t>FUEL PUMP</t>
   </si>
   <si>
     <t>ENGINE PT6A-114A</t>
@@ -1586,10 +1580,10 @@
         <v>53</v>
       </c>
       <c r="E2">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F2">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="3" spans="1:6">
@@ -1606,10 +1600,10 @@
         <v>53</v>
       </c>
       <c r="E3">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F3">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="4" spans="1:6">
@@ -2210,7 +2204,7 @@
         <v>58</v>
       </c>
       <c r="D2" t="s">
-        <v>236</v>
+        <v>235</v>
       </c>
       <c r="E2">
         <v>1</v>
@@ -2227,7 +2221,7 @@
         <v>59</v>
       </c>
       <c r="D3" t="s">
-        <v>237</v>
+        <v>236</v>
       </c>
       <c r="E3">
         <v>1</v>
@@ -2244,7 +2238,7 @@
         <v>59</v>
       </c>
       <c r="D4" t="s">
-        <v>237</v>
+        <v>236</v>
       </c>
       <c r="E4">
         <v>1</v>
@@ -2261,7 +2255,7 @@
         <v>59</v>
       </c>
       <c r="D5" t="s">
-        <v>237</v>
+        <v>236</v>
       </c>
       <c r="E5">
         <v>1</v>
@@ -2269,16 +2263,16 @@
     </row>
     <row r="6" spans="1:5">
       <c r="A6" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="B6" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="C6" t="s">
         <v>60</v>
       </c>
       <c r="D6" t="s">
-        <v>238</v>
+        <v>237</v>
       </c>
       <c r="E6">
         <v>1</v>
@@ -2286,16 +2280,16 @@
     </row>
     <row r="7" spans="1:5">
       <c r="A7" t="s">
-        <v>8</v>
+        <v>11</v>
       </c>
       <c r="B7" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="C7" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="D7" t="s">
-        <v>239</v>
+        <v>237</v>
       </c>
       <c r="E7">
         <v>1</v>
@@ -2303,16 +2297,16 @@
     </row>
     <row r="8" spans="1:5">
       <c r="A8" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B8" t="s">
-        <v>40</v>
+        <v>36</v>
       </c>
       <c r="C8" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="D8" t="s">
-        <v>239</v>
+        <v>237</v>
       </c>
       <c r="E8">
         <v>1</v>
@@ -2320,16 +2314,16 @@
     </row>
     <row r="9" spans="1:5">
       <c r="A9" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="B9" t="s">
-        <v>36</v>
+        <v>40</v>
       </c>
       <c r="C9" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="D9" t="s">
-        <v>239</v>
+        <v>237</v>
       </c>
       <c r="E9">
         <v>1</v>
@@ -2337,16 +2331,16 @@
     </row>
     <row r="10" spans="1:5">
       <c r="A10" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="B10" t="s">
         <v>40</v>
       </c>
       <c r="C10" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="D10" t="s">
-        <v>239</v>
+        <v>237</v>
       </c>
       <c r="E10">
         <v>1</v>
@@ -2354,16 +2348,16 @@
     </row>
     <row r="11" spans="1:5">
       <c r="A11" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="B11" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="C11" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="D11" t="s">
-        <v>239</v>
+        <v>237</v>
       </c>
       <c r="E11">
         <v>1</v>
@@ -2371,16 +2365,16 @@
     </row>
     <row r="12" spans="1:5">
       <c r="A12" t="s">
-        <v>15</v>
+        <v>8</v>
       </c>
       <c r="B12" t="s">
-        <v>41</v>
+        <v>38</v>
       </c>
       <c r="C12" t="s">
         <v>61</v>
       </c>
       <c r="D12" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
       <c r="E12">
         <v>1</v>
@@ -2388,16 +2382,16 @@
     </row>
     <row r="13" spans="1:5">
       <c r="A13" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="B13" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="C13" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="D13" t="s">
-        <v>240</v>
+        <v>238</v>
       </c>
       <c r="E13">
         <v>1</v>
@@ -2405,16 +2399,16 @@
     </row>
     <row r="14" spans="1:5">
       <c r="A14" t="s">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="B14" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="C14" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="D14" t="s">
-        <v>240</v>
+        <v>238</v>
       </c>
       <c r="E14">
         <v>1</v>
@@ -2422,16 +2416,16 @@
     </row>
     <row r="15" spans="1:5">
       <c r="A15" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B15" t="s">
-        <v>40</v>
+        <v>36</v>
       </c>
       <c r="C15" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="D15" t="s">
-        <v>240</v>
+        <v>238</v>
       </c>
       <c r="E15">
         <v>1</v>
@@ -2439,16 +2433,16 @@
     </row>
     <row r="16" spans="1:5">
       <c r="A16" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="B16" t="s">
-        <v>36</v>
+        <v>40</v>
       </c>
       <c r="C16" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="D16" t="s">
-        <v>240</v>
+        <v>238</v>
       </c>
       <c r="E16">
         <v>1</v>
@@ -2456,16 +2450,16 @@
     </row>
     <row r="17" spans="1:5">
       <c r="A17" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="B17" t="s">
         <v>40</v>
       </c>
       <c r="C17" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="D17" t="s">
-        <v>240</v>
+        <v>238</v>
       </c>
       <c r="E17">
         <v>1</v>
@@ -2473,16 +2467,16 @@
     </row>
     <row r="18" spans="1:5">
       <c r="A18" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="B18" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="C18" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="D18" t="s">
-        <v>240</v>
+        <v>238</v>
       </c>
       <c r="E18">
         <v>1</v>
@@ -2490,16 +2484,16 @@
     </row>
     <row r="19" spans="1:5">
       <c r="A19" t="s">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="B19" t="s">
-        <v>41</v>
+        <v>36</v>
       </c>
       <c r="C19" t="s">
         <v>62</v>
       </c>
       <c r="D19" t="s">
-        <v>240</v>
+        <v>239</v>
       </c>
       <c r="E19">
         <v>1</v>
@@ -2516,7 +2510,7 @@
         <v>63</v>
       </c>
       <c r="D20" t="s">
-        <v>241</v>
+        <v>240</v>
       </c>
       <c r="E20">
         <v>1</v>
@@ -2533,7 +2527,7 @@
         <v>64</v>
       </c>
       <c r="D21" t="s">
-        <v>242</v>
+        <v>241</v>
       </c>
       <c r="E21">
         <v>1</v>
@@ -2550,7 +2544,7 @@
         <v>65</v>
       </c>
       <c r="D22" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
       <c r="E22">
         <v>1</v>
@@ -2567,7 +2561,7 @@
         <v>66</v>
       </c>
       <c r="D23" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="E23">
         <v>1</v>
@@ -2575,7 +2569,7 @@
     </row>
     <row r="24" spans="1:5">
       <c r="A24" t="s">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="B24" t="s">
         <v>36</v>
@@ -2584,7 +2578,7 @@
         <v>67</v>
       </c>
       <c r="D24" t="s">
-        <v>245</v>
+        <v>244</v>
       </c>
       <c r="E24">
         <v>1</v>
@@ -2592,16 +2586,16 @@
     </row>
     <row r="25" spans="1:5">
       <c r="A25" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="B25" t="s">
-        <v>36</v>
+        <v>40</v>
       </c>
       <c r="C25" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="D25" t="s">
-        <v>246</v>
+        <v>244</v>
       </c>
       <c r="E25">
         <v>1</v>
@@ -2609,16 +2603,16 @@
     </row>
     <row r="26" spans="1:5">
       <c r="A26" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="B26" t="s">
         <v>40</v>
       </c>
       <c r="C26" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="D26" t="s">
-        <v>246</v>
+        <v>244</v>
       </c>
       <c r="E26">
         <v>1</v>
@@ -2626,16 +2620,16 @@
     </row>
     <row r="27" spans="1:5">
       <c r="A27" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="B27" t="s">
-        <v>40</v>
+        <v>36</v>
       </c>
       <c r="C27" t="s">
         <v>68</v>
       </c>
       <c r="D27" t="s">
-        <v>246</v>
+        <v>245</v>
       </c>
       <c r="E27">
         <v>1</v>
@@ -2643,16 +2637,16 @@
     </row>
     <row r="28" spans="1:5">
       <c r="A28" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="B28" t="s">
-        <v>36</v>
+        <v>40</v>
       </c>
       <c r="C28" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="D28" t="s">
-        <v>247</v>
+        <v>245</v>
       </c>
       <c r="E28">
         <v>1</v>
@@ -2660,16 +2654,16 @@
     </row>
     <row r="29" spans="1:5">
       <c r="A29" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="B29" t="s">
         <v>40</v>
       </c>
       <c r="C29" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="D29" t="s">
-        <v>247</v>
+        <v>245</v>
       </c>
       <c r="E29">
         <v>1</v>
@@ -2677,16 +2671,16 @@
     </row>
     <row r="30" spans="1:5">
       <c r="A30" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="B30" t="s">
-        <v>40</v>
+        <v>36</v>
       </c>
       <c r="C30" t="s">
         <v>69</v>
       </c>
       <c r="D30" t="s">
-        <v>247</v>
+        <v>246</v>
       </c>
       <c r="E30">
         <v>1</v>
@@ -2694,16 +2688,16 @@
     </row>
     <row r="31" spans="1:5">
       <c r="A31" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="B31" t="s">
-        <v>36</v>
+        <v>40</v>
       </c>
       <c r="C31" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="D31" t="s">
-        <v>248</v>
+        <v>246</v>
       </c>
       <c r="E31">
         <v>1</v>
@@ -2711,16 +2705,16 @@
     </row>
     <row r="32" spans="1:5">
       <c r="A32" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B32" t="s">
-        <v>40</v>
+        <v>36</v>
       </c>
       <c r="C32" t="s">
         <v>70</v>
       </c>
       <c r="D32" t="s">
-        <v>248</v>
+        <v>247</v>
       </c>
       <c r="E32">
         <v>1</v>
@@ -2728,16 +2722,16 @@
     </row>
     <row r="33" spans="1:5">
       <c r="A33" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="B33" t="s">
-        <v>36</v>
+        <v>40</v>
       </c>
       <c r="C33" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="D33" t="s">
-        <v>249</v>
+        <v>247</v>
       </c>
       <c r="E33">
         <v>1</v>
@@ -2745,16 +2739,16 @@
     </row>
     <row r="34" spans="1:5">
       <c r="A34" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="B34" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="C34" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="D34" t="s">
-        <v>249</v>
+        <v>247</v>
       </c>
       <c r="E34">
         <v>1</v>
@@ -2762,16 +2756,16 @@
     </row>
     <row r="35" spans="1:5">
       <c r="A35" t="s">
-        <v>15</v>
+        <v>12</v>
       </c>
       <c r="B35" t="s">
-        <v>41</v>
+        <v>36</v>
       </c>
       <c r="C35" t="s">
         <v>71</v>
       </c>
       <c r="D35" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
       <c r="E35">
         <v>1</v>
@@ -2779,36 +2773,36 @@
     </row>
     <row r="36" spans="1:5">
       <c r="A36" t="s">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="B36" t="s">
-        <v>36</v>
+        <v>41</v>
       </c>
       <c r="C36" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="D36" t="s">
-        <v>250</v>
+        <v>248</v>
       </c>
       <c r="E36">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="37" spans="1:5">
       <c r="A37" t="s">
-        <v>15</v>
+        <v>12</v>
       </c>
       <c r="B37" t="s">
-        <v>41</v>
+        <v>36</v>
       </c>
       <c r="C37" t="s">
         <v>72</v>
       </c>
       <c r="D37" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
       <c r="E37">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="38" spans="1:5">
@@ -2822,7 +2816,7 @@
         <v>73</v>
       </c>
       <c r="D38" t="s">
-        <v>251</v>
+        <v>250</v>
       </c>
       <c r="E38">
         <v>1</v>
@@ -2839,7 +2833,7 @@
         <v>74</v>
       </c>
       <c r="D39" t="s">
-        <v>252</v>
+        <v>251</v>
       </c>
       <c r="E39">
         <v>1</v>
@@ -2856,7 +2850,7 @@
         <v>75</v>
       </c>
       <c r="D40" t="s">
-        <v>253</v>
+        <v>252</v>
       </c>
       <c r="E40">
         <v>1</v>
@@ -2873,7 +2867,7 @@
         <v>76</v>
       </c>
       <c r="D41" t="s">
-        <v>254</v>
+        <v>253</v>
       </c>
       <c r="E41">
         <v>1</v>
@@ -2890,7 +2884,7 @@
         <v>77</v>
       </c>
       <c r="D42" t="s">
-        <v>255</v>
+        <v>254</v>
       </c>
       <c r="E42">
         <v>1</v>
@@ -2907,7 +2901,7 @@
         <v>78</v>
       </c>
       <c r="D43" t="s">
-        <v>256</v>
+        <v>255</v>
       </c>
       <c r="E43">
         <v>1</v>
@@ -2924,7 +2918,7 @@
         <v>79</v>
       </c>
       <c r="D44" t="s">
-        <v>257</v>
+        <v>256</v>
       </c>
       <c r="E44">
         <v>1</v>
@@ -2941,58 +2935,58 @@
         <v>80</v>
       </c>
       <c r="D45" t="s">
-        <v>258</v>
+        <v>257</v>
       </c>
       <c r="E45">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="46" spans="1:5">
       <c r="A46" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="B46" t="s">
-        <v>36</v>
+        <v>40</v>
       </c>
       <c r="C46" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="D46" t="s">
-        <v>259</v>
+        <v>257</v>
       </c>
       <c r="E46">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="47" spans="1:5">
       <c r="A47" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="B47" t="s">
         <v>40</v>
       </c>
       <c r="C47" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="D47" t="s">
-        <v>259</v>
+        <v>257</v>
       </c>
       <c r="E47">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="48" spans="1:5">
       <c r="A48" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="B48" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="C48" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="D48" t="s">
-        <v>259</v>
+        <v>257</v>
       </c>
       <c r="E48">
         <v>2</v>
@@ -3000,16 +2994,16 @@
     </row>
     <row r="49" spans="1:5">
       <c r="A49" t="s">
-        <v>15</v>
+        <v>12</v>
       </c>
       <c r="B49" t="s">
-        <v>41</v>
+        <v>36</v>
       </c>
       <c r="C49" t="s">
         <v>81</v>
       </c>
       <c r="D49" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="E49">
         <v>2</v>
@@ -3017,16 +3011,16 @@
     </row>
     <row r="50" spans="1:5">
       <c r="A50" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="B50" t="s">
-        <v>36</v>
+        <v>40</v>
       </c>
       <c r="C50" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="D50" t="s">
-        <v>260</v>
+        <v>258</v>
       </c>
       <c r="E50">
         <v>2</v>
@@ -3034,84 +3028,84 @@
     </row>
     <row r="51" spans="1:5">
       <c r="A51" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="B51" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="C51" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="D51" t="s">
-        <v>260</v>
+        <v>258</v>
       </c>
       <c r="E51">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="52" spans="1:5">
       <c r="A52" t="s">
-        <v>15</v>
+        <v>12</v>
       </c>
       <c r="B52" t="s">
-        <v>41</v>
+        <v>36</v>
       </c>
       <c r="C52" t="s">
         <v>82</v>
       </c>
       <c r="D52" t="s">
-        <v>260</v>
+        <v>259</v>
       </c>
       <c r="E52">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="53" spans="1:5">
       <c r="A53" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="B53" t="s">
-        <v>36</v>
+        <v>40</v>
       </c>
       <c r="C53" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="D53" t="s">
-        <v>261</v>
+        <v>259</v>
       </c>
       <c r="E53">
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
     <row r="54" spans="1:5">
       <c r="A54" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="B54" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="C54" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="D54" t="s">
-        <v>261</v>
+        <v>259</v>
       </c>
       <c r="E54">
-        <v>4</v>
+        <v>2</v>
       </c>
     </row>
     <row r="55" spans="1:5">
       <c r="A55" t="s">
-        <v>15</v>
+        <v>12</v>
       </c>
       <c r="B55" t="s">
-        <v>41</v>
+        <v>36</v>
       </c>
       <c r="C55" t="s">
         <v>83</v>
       </c>
       <c r="D55" t="s">
-        <v>261</v>
+        <v>260</v>
       </c>
       <c r="E55">
         <v>2</v>
@@ -3119,36 +3113,36 @@
     </row>
     <row r="56" spans="1:5">
       <c r="A56" t="s">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="B56" t="s">
-        <v>36</v>
+        <v>41</v>
       </c>
       <c r="C56" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="D56" t="s">
-        <v>262</v>
+        <v>260</v>
       </c>
       <c r="E56">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="57" spans="1:5">
       <c r="A57" t="s">
-        <v>15</v>
+        <v>12</v>
       </c>
       <c r="B57" t="s">
-        <v>41</v>
+        <v>36</v>
       </c>
       <c r="C57" t="s">
         <v>84</v>
       </c>
       <c r="D57" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
       <c r="E57">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="58" spans="1:5">
@@ -3162,7 +3156,7 @@
         <v>85</v>
       </c>
       <c r="D58" t="s">
-        <v>263</v>
+        <v>262</v>
       </c>
       <c r="E58">
         <v>2</v>
@@ -3179,7 +3173,7 @@
         <v>86</v>
       </c>
       <c r="D59" t="s">
-        <v>264</v>
+        <v>263</v>
       </c>
       <c r="E59">
         <v>2</v>
@@ -3196,7 +3190,7 @@
         <v>87</v>
       </c>
       <c r="D60" t="s">
-        <v>265</v>
+        <v>264</v>
       </c>
       <c r="E60">
         <v>2</v>
@@ -3213,7 +3207,7 @@
         <v>88</v>
       </c>
       <c r="D61" t="s">
-        <v>266</v>
+        <v>265</v>
       </c>
       <c r="E61">
         <v>2</v>
@@ -3230,7 +3224,7 @@
         <v>89</v>
       </c>
       <c r="D62" t="s">
-        <v>267</v>
+        <v>266</v>
       </c>
       <c r="E62">
         <v>2</v>
@@ -3247,7 +3241,7 @@
         <v>90</v>
       </c>
       <c r="D63" t="s">
-        <v>268</v>
+        <v>267</v>
       </c>
       <c r="E63">
         <v>2</v>
@@ -3264,7 +3258,7 @@
         <v>91</v>
       </c>
       <c r="D64" t="s">
-        <v>269</v>
+        <v>257</v>
       </c>
       <c r="E64">
         <v>2</v>
@@ -3281,24 +3275,24 @@
         <v>92</v>
       </c>
       <c r="D65" t="s">
-        <v>259</v>
+        <v>256</v>
       </c>
       <c r="E65">
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
     <row r="66" spans="1:5">
       <c r="A66" t="s">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="B66" t="s">
-        <v>36</v>
+        <v>41</v>
       </c>
       <c r="C66" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="D66" t="s">
-        <v>258</v>
+        <v>256</v>
       </c>
       <c r="E66">
         <v>4</v>
@@ -3306,16 +3300,16 @@
     </row>
     <row r="67" spans="1:5">
       <c r="A67" t="s">
-        <v>15</v>
+        <v>12</v>
       </c>
       <c r="B67" t="s">
-        <v>41</v>
+        <v>36</v>
       </c>
       <c r="C67" t="s">
         <v>93</v>
       </c>
       <c r="D67" t="s">
-        <v>258</v>
+        <v>268</v>
       </c>
       <c r="E67">
         <v>4</v>
@@ -3332,7 +3326,7 @@
         <v>94</v>
       </c>
       <c r="D68" t="s">
-        <v>270</v>
+        <v>269</v>
       </c>
       <c r="E68">
         <v>4</v>
@@ -3349,7 +3343,7 @@
         <v>95</v>
       </c>
       <c r="D69" t="s">
-        <v>271</v>
+        <v>270</v>
       </c>
       <c r="E69">
         <v>4</v>
@@ -3357,33 +3351,33 @@
     </row>
     <row r="70" spans="1:5">
       <c r="A70" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="B70" t="s">
-        <v>36</v>
+        <v>40</v>
       </c>
       <c r="C70" t="s">
         <v>96</v>
       </c>
       <c r="D70" t="s">
-        <v>272</v>
+        <v>271</v>
       </c>
       <c r="E70">
-        <v>4</v>
+        <v>1</v>
       </c>
     </row>
     <row r="71" spans="1:5">
       <c r="A71" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="B71" t="s">
         <v>40</v>
       </c>
       <c r="C71" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="D71" t="s">
-        <v>273</v>
+        <v>271</v>
       </c>
       <c r="E71">
         <v>1</v>
@@ -3391,16 +3385,16 @@
     </row>
     <row r="72" spans="1:5">
       <c r="A72" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="B72" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="C72" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="D72" t="s">
-        <v>273</v>
+        <v>271</v>
       </c>
       <c r="E72">
         <v>1</v>
@@ -3408,16 +3402,16 @@
     </row>
     <row r="73" spans="1:5">
       <c r="A73" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="B73" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C73" t="s">
         <v>97</v>
       </c>
       <c r="D73" t="s">
-        <v>273</v>
+        <v>272</v>
       </c>
       <c r="E73">
         <v>1</v>
@@ -3425,16 +3419,16 @@
     </row>
     <row r="74" spans="1:5">
       <c r="A74" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="B74" t="s">
         <v>40</v>
       </c>
       <c r="C74" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="D74" t="s">
-        <v>274</v>
+        <v>272</v>
       </c>
       <c r="E74">
         <v>1</v>
@@ -3442,50 +3436,50 @@
     </row>
     <row r="75" spans="1:5">
       <c r="A75" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="B75" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="C75" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="D75" t="s">
-        <v>274</v>
+        <v>272</v>
       </c>
       <c r="E75">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="76" spans="1:5">
       <c r="A76" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="B76" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C76" t="s">
         <v>98</v>
       </c>
       <c r="D76" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
       <c r="E76">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="77" spans="1:5">
       <c r="A77" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="B77" t="s">
         <v>40</v>
       </c>
       <c r="C77" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="D77" t="s">
-        <v>275</v>
+        <v>273</v>
       </c>
       <c r="E77">
         <v>1</v>
@@ -3493,7 +3487,7 @@
     </row>
     <row r="78" spans="1:5">
       <c r="A78" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B78" t="s">
         <v>40</v>
@@ -3502,7 +3496,7 @@
         <v>99</v>
       </c>
       <c r="D78" t="s">
-        <v>275</v>
+        <v>274</v>
       </c>
       <c r="E78">
         <v>1</v>
@@ -3510,16 +3504,16 @@
     </row>
     <row r="79" spans="1:5">
       <c r="A79" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="B79" t="s">
         <v>40</v>
       </c>
       <c r="C79" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="D79" t="s">
-        <v>276</v>
+        <v>274</v>
       </c>
       <c r="E79">
         <v>1</v>
@@ -3527,7 +3521,7 @@
     </row>
     <row r="80" spans="1:5">
       <c r="A80" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B80" t="s">
         <v>40</v>
@@ -3536,7 +3530,7 @@
         <v>100</v>
       </c>
       <c r="D80" t="s">
-        <v>276</v>
+        <v>275</v>
       </c>
       <c r="E80">
         <v>1</v>
@@ -3544,16 +3538,16 @@
     </row>
     <row r="81" spans="1:5">
       <c r="A81" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="B81" t="s">
         <v>40</v>
       </c>
       <c r="C81" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="D81" t="s">
-        <v>277</v>
+        <v>275</v>
       </c>
       <c r="E81">
         <v>1</v>
@@ -3561,7 +3555,7 @@
     </row>
     <row r="82" spans="1:5">
       <c r="A82" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B82" t="s">
         <v>40</v>
@@ -3570,7 +3564,7 @@
         <v>101</v>
       </c>
       <c r="D82" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
       <c r="E82">
         <v>1</v>
@@ -3578,16 +3572,16 @@
     </row>
     <row r="83" spans="1:5">
       <c r="A83" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="B83" t="s">
         <v>40</v>
       </c>
       <c r="C83" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="D83" t="s">
-        <v>278</v>
+        <v>276</v>
       </c>
       <c r="E83">
         <v>1</v>
@@ -3595,7 +3589,7 @@
     </row>
     <row r="84" spans="1:5">
       <c r="A84" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B84" t="s">
         <v>40</v>
@@ -3604,7 +3598,7 @@
         <v>102</v>
       </c>
       <c r="D84" t="s">
-        <v>278</v>
+        <v>277</v>
       </c>
       <c r="E84">
         <v>1</v>
@@ -3612,16 +3606,16 @@
     </row>
     <row r="85" spans="1:5">
       <c r="A85" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="B85" t="s">
         <v>40</v>
       </c>
       <c r="C85" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="D85" t="s">
-        <v>279</v>
+        <v>277</v>
       </c>
       <c r="E85">
         <v>1</v>
@@ -3629,7 +3623,7 @@
     </row>
     <row r="86" spans="1:5">
       <c r="A86" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B86" t="s">
         <v>40</v>
@@ -3638,7 +3632,7 @@
         <v>103</v>
       </c>
       <c r="D86" t="s">
-        <v>279</v>
+        <v>278</v>
       </c>
       <c r="E86">
         <v>1</v>
@@ -3646,16 +3640,16 @@
     </row>
     <row r="87" spans="1:5">
       <c r="A87" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="B87" t="s">
         <v>40</v>
       </c>
       <c r="C87" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="D87" t="s">
-        <v>280</v>
+        <v>278</v>
       </c>
       <c r="E87">
         <v>1</v>
@@ -3663,7 +3657,7 @@
     </row>
     <row r="88" spans="1:5">
       <c r="A88" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B88" t="s">
         <v>40</v>
@@ -3672,7 +3666,7 @@
         <v>104</v>
       </c>
       <c r="D88" t="s">
-        <v>280</v>
+        <v>279</v>
       </c>
       <c r="E88">
         <v>1</v>
@@ -3680,16 +3674,16 @@
     </row>
     <row r="89" spans="1:5">
       <c r="A89" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="B89" t="s">
         <v>40</v>
       </c>
       <c r="C89" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="D89" t="s">
-        <v>281</v>
+        <v>279</v>
       </c>
       <c r="E89">
         <v>1</v>
@@ -3697,7 +3691,7 @@
     </row>
     <row r="90" spans="1:5">
       <c r="A90" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B90" t="s">
         <v>40</v>
@@ -3706,7 +3700,7 @@
         <v>105</v>
       </c>
       <c r="D90" t="s">
-        <v>281</v>
+        <v>280</v>
       </c>
       <c r="E90">
         <v>1</v>
@@ -3714,16 +3708,16 @@
     </row>
     <row r="91" spans="1:5">
       <c r="A91" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="B91" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="C91" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="D91" t="s">
-        <v>282</v>
+        <v>280</v>
       </c>
       <c r="E91">
         <v>1</v>
@@ -3731,16 +3725,16 @@
     </row>
     <row r="92" spans="1:5">
       <c r="A92" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="B92" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C92" t="s">
         <v>106</v>
       </c>
       <c r="D92" t="s">
-        <v>282</v>
+        <v>281</v>
       </c>
       <c r="E92">
         <v>1</v>
@@ -3748,16 +3742,16 @@
     </row>
     <row r="93" spans="1:5">
       <c r="A93" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="B93" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="C93" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="D93" t="s">
-        <v>283</v>
+        <v>281</v>
       </c>
       <c r="E93">
         <v>1</v>
@@ -3765,16 +3759,16 @@
     </row>
     <row r="94" spans="1:5">
       <c r="A94" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="B94" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C94" t="s">
         <v>107</v>
       </c>
       <c r="D94" t="s">
-        <v>283</v>
+        <v>282</v>
       </c>
       <c r="E94">
         <v>1</v>
@@ -3782,16 +3776,16 @@
     </row>
     <row r="95" spans="1:5">
       <c r="A95" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="B95" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="C95" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="D95" t="s">
-        <v>284</v>
+        <v>282</v>
       </c>
       <c r="E95">
         <v>1</v>
@@ -3799,16 +3793,16 @@
     </row>
     <row r="96" spans="1:5">
       <c r="A96" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="B96" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C96" t="s">
         <v>108</v>
       </c>
       <c r="D96" t="s">
-        <v>284</v>
+        <v>283</v>
       </c>
       <c r="E96">
         <v>1</v>
@@ -3825,7 +3819,7 @@
         <v>109</v>
       </c>
       <c r="D97" t="s">
-        <v>285</v>
+        <v>284</v>
       </c>
       <c r="E97">
         <v>1</v>
@@ -3842,7 +3836,7 @@
         <v>110</v>
       </c>
       <c r="D98" t="s">
-        <v>286</v>
+        <v>285</v>
       </c>
       <c r="E98">
         <v>1</v>
@@ -3859,7 +3853,7 @@
         <v>111</v>
       </c>
       <c r="D99" t="s">
-        <v>287</v>
+        <v>286</v>
       </c>
       <c r="E99">
         <v>1</v>
@@ -3876,7 +3870,7 @@
         <v>112</v>
       </c>
       <c r="D100" t="s">
-        <v>288</v>
+        <v>287</v>
       </c>
       <c r="E100">
         <v>1</v>
@@ -3893,7 +3887,7 @@
         <v>113</v>
       </c>
       <c r="D101" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
       <c r="E101">
         <v>1</v>
@@ -3910,32 +3904,32 @@
         <v>114</v>
       </c>
       <c r="D102" t="s">
-        <v>290</v>
+        <v>289</v>
       </c>
       <c r="E102">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="103" spans="1:5">
       <c r="A103" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="B103" t="s">
         <v>40</v>
       </c>
       <c r="C103" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="D103" t="s">
-        <v>291</v>
+        <v>289</v>
       </c>
       <c r="E103">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="104" spans="1:5">
       <c r="A104" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B104" t="s">
         <v>40</v>
@@ -3944,24 +3938,24 @@
         <v>115</v>
       </c>
       <c r="D104" t="s">
-        <v>291</v>
+        <v>290</v>
       </c>
       <c r="E104">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="105" spans="1:5">
       <c r="A105" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="B105" t="s">
         <v>40</v>
       </c>
       <c r="C105" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="D105" t="s">
-        <v>292</v>
+        <v>290</v>
       </c>
       <c r="E105">
         <v>2</v>
@@ -3969,16 +3963,16 @@
     </row>
     <row r="106" spans="1:5">
       <c r="A106" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="B106" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="C106" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="D106" t="s">
-        <v>292</v>
+        <v>290</v>
       </c>
       <c r="E106">
         <v>2</v>
@@ -3986,16 +3980,16 @@
     </row>
     <row r="107" spans="1:5">
       <c r="A107" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="B107" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C107" t="s">
         <v>116</v>
       </c>
       <c r="D107" t="s">
-        <v>292</v>
+        <v>291</v>
       </c>
       <c r="E107">
         <v>2</v>
@@ -4003,16 +3997,16 @@
     </row>
     <row r="108" spans="1:5">
       <c r="A108" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="B108" t="s">
         <v>40</v>
       </c>
       <c r="C108" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="D108" t="s">
-        <v>293</v>
+        <v>291</v>
       </c>
       <c r="E108">
         <v>2</v>
@@ -4020,16 +4014,16 @@
     </row>
     <row r="109" spans="1:5">
       <c r="A109" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="B109" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="C109" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="D109" t="s">
-        <v>293</v>
+        <v>291</v>
       </c>
       <c r="E109">
         <v>2</v>
@@ -4037,16 +4031,16 @@
     </row>
     <row r="110" spans="1:5">
       <c r="A110" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="B110" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C110" t="s">
         <v>117</v>
       </c>
       <c r="D110" t="s">
-        <v>293</v>
+        <v>292</v>
       </c>
       <c r="E110">
         <v>2</v>
@@ -4054,16 +4048,16 @@
     </row>
     <row r="111" spans="1:5">
       <c r="A111" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="B111" t="s">
         <v>40</v>
       </c>
       <c r="C111" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="D111" t="s">
-        <v>294</v>
+        <v>292</v>
       </c>
       <c r="E111">
         <v>2</v>
@@ -4071,7 +4065,7 @@
     </row>
     <row r="112" spans="1:5">
       <c r="A112" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B112" t="s">
         <v>40</v>
@@ -4080,7 +4074,7 @@
         <v>118</v>
       </c>
       <c r="D112" t="s">
-        <v>294</v>
+        <v>293</v>
       </c>
       <c r="E112">
         <v>2</v>
@@ -4088,16 +4082,16 @@
     </row>
     <row r="113" spans="1:5">
       <c r="A113" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="B113" t="s">
         <v>40</v>
       </c>
       <c r="C113" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="D113" t="s">
-        <v>295</v>
+        <v>293</v>
       </c>
       <c r="E113">
         <v>2</v>
@@ -4105,7 +4099,7 @@
     </row>
     <row r="114" spans="1:5">
       <c r="A114" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B114" t="s">
         <v>40</v>
@@ -4114,7 +4108,7 @@
         <v>119</v>
       </c>
       <c r="D114" t="s">
-        <v>295</v>
+        <v>272</v>
       </c>
       <c r="E114">
         <v>2</v>
@@ -4122,33 +4116,33 @@
     </row>
     <row r="115" spans="1:5">
       <c r="A115" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="B115" t="s">
         <v>40</v>
       </c>
       <c r="C115" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="D115" t="s">
-        <v>274</v>
+        <v>272</v>
       </c>
       <c r="E115">
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
     <row r="116" spans="1:5">
       <c r="A116" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="B116" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="C116" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="D116" t="s">
-        <v>274</v>
+        <v>272</v>
       </c>
       <c r="E116">
         <v>4</v>
@@ -4156,41 +4150,41 @@
     </row>
     <row r="117" spans="1:5">
       <c r="A117" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="B117" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C117" t="s">
         <v>120</v>
       </c>
       <c r="D117" t="s">
-        <v>274</v>
+        <v>294</v>
       </c>
       <c r="E117">
-        <v>4</v>
+        <v>2</v>
       </c>
     </row>
     <row r="118" spans="1:5">
       <c r="A118" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="B118" t="s">
         <v>40</v>
       </c>
       <c r="C118" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="D118" t="s">
-        <v>296</v>
+        <v>294</v>
       </c>
       <c r="E118">
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
     <row r="119" spans="1:5">
       <c r="A119" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B119" t="s">
         <v>40</v>
@@ -4199,10 +4193,10 @@
         <v>121</v>
       </c>
       <c r="D119" t="s">
-        <v>296</v>
+        <v>278</v>
       </c>
       <c r="E119">
-        <v>4</v>
+        <v>2</v>
       </c>
     </row>
     <row r="120" spans="1:5">
@@ -4216,7 +4210,7 @@
         <v>122</v>
       </c>
       <c r="D120" t="s">
-        <v>280</v>
+        <v>295</v>
       </c>
       <c r="E120">
         <v>2</v>
@@ -4233,7 +4227,7 @@
         <v>123</v>
       </c>
       <c r="D121" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="E121">
         <v>2</v>
@@ -4250,24 +4244,24 @@
         <v>124</v>
       </c>
       <c r="D122" t="s">
-        <v>298</v>
+        <v>297</v>
       </c>
       <c r="E122">
-        <v>2</v>
+        <v>5</v>
       </c>
     </row>
     <row r="123" spans="1:5">
       <c r="A123" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="B123" t="s">
         <v>40</v>
       </c>
       <c r="C123" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="D123" t="s">
-        <v>299</v>
+        <v>297</v>
       </c>
       <c r="E123">
         <v>5</v>
@@ -4275,7 +4269,7 @@
     </row>
     <row r="124" spans="1:5">
       <c r="A124" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B124" t="s">
         <v>40</v>
@@ -4284,10 +4278,10 @@
         <v>125</v>
       </c>
       <c r="D124" t="s">
-        <v>299</v>
+        <v>298</v>
       </c>
       <c r="E124">
-        <v>5</v>
+        <v>7</v>
       </c>
     </row>
     <row r="125" spans="1:5">
@@ -4301,10 +4295,10 @@
         <v>126</v>
       </c>
       <c r="D125" t="s">
-        <v>300</v>
+        <v>299</v>
       </c>
       <c r="E125">
-        <v>7</v>
+        <v>8</v>
       </c>
     </row>
     <row r="126" spans="1:5">
@@ -4318,10 +4312,10 @@
         <v>127</v>
       </c>
       <c r="D126" t="s">
-        <v>301</v>
+        <v>300</v>
       </c>
       <c r="E126">
-        <v>8</v>
+        <v>10</v>
       </c>
     </row>
     <row r="127" spans="1:5">
@@ -4335,24 +4329,24 @@
         <v>128</v>
       </c>
       <c r="D127" t="s">
-        <v>302</v>
+        <v>301</v>
       </c>
       <c r="E127">
-        <v>10</v>
+        <v>30</v>
       </c>
     </row>
     <row r="128" spans="1:5">
       <c r="A128" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="B128" t="s">
         <v>40</v>
       </c>
       <c r="C128" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="D128" t="s">
-        <v>303</v>
+        <v>301</v>
       </c>
       <c r="E128">
         <v>30</v>
@@ -4369,24 +4363,24 @@
         <v>129</v>
       </c>
       <c r="D129" t="s">
-        <v>303</v>
+        <v>302</v>
       </c>
       <c r="E129">
-        <v>30</v>
+        <v>1</v>
       </c>
     </row>
     <row r="130" spans="1:5">
       <c r="A130" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="B130" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="C130" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="D130" t="s">
-        <v>304</v>
+        <v>302</v>
       </c>
       <c r="E130">
         <v>1</v>
@@ -4394,16 +4388,16 @@
     </row>
     <row r="131" spans="1:5">
       <c r="A131" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B131" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C131" t="s">
         <v>130</v>
       </c>
       <c r="D131" t="s">
-        <v>304</v>
+        <v>303</v>
       </c>
       <c r="E131">
         <v>1</v>
@@ -4420,7 +4414,7 @@
         <v>131</v>
       </c>
       <c r="D132" t="s">
-        <v>305</v>
+        <v>304</v>
       </c>
       <c r="E132">
         <v>1</v>
@@ -4437,7 +4431,7 @@
         <v>132</v>
       </c>
       <c r="D133" t="s">
-        <v>306</v>
+        <v>305</v>
       </c>
       <c r="E133">
         <v>1</v>
@@ -4454,7 +4448,7 @@
         <v>133</v>
       </c>
       <c r="D134" t="s">
-        <v>307</v>
+        <v>306</v>
       </c>
       <c r="E134">
         <v>1</v>
@@ -4471,7 +4465,7 @@
         <v>134</v>
       </c>
       <c r="D135" t="s">
-        <v>308</v>
+        <v>307</v>
       </c>
       <c r="E135">
         <v>1</v>
@@ -4488,7 +4482,7 @@
         <v>135</v>
       </c>
       <c r="D136" t="s">
-        <v>309</v>
+        <v>308</v>
       </c>
       <c r="E136">
         <v>1</v>
@@ -4505,7 +4499,7 @@
         <v>136</v>
       </c>
       <c r="D137" t="s">
-        <v>310</v>
+        <v>309</v>
       </c>
       <c r="E137">
         <v>1</v>
@@ -4522,7 +4516,7 @@
         <v>137</v>
       </c>
       <c r="D138" t="s">
-        <v>311</v>
+        <v>310</v>
       </c>
       <c r="E138">
         <v>1</v>
@@ -4539,7 +4533,7 @@
         <v>138</v>
       </c>
       <c r="D139" t="s">
-        <v>312</v>
+        <v>311</v>
       </c>
       <c r="E139">
         <v>1</v>
@@ -4556,7 +4550,7 @@
         <v>139</v>
       </c>
       <c r="D140" t="s">
-        <v>313</v>
+        <v>312</v>
       </c>
       <c r="E140">
         <v>1</v>
@@ -4573,7 +4567,7 @@
         <v>140</v>
       </c>
       <c r="D141" t="s">
-        <v>314</v>
+        <v>313</v>
       </c>
       <c r="E141">
         <v>1</v>
@@ -4590,7 +4584,7 @@
         <v>141</v>
       </c>
       <c r="D142" t="s">
-        <v>315</v>
+        <v>314</v>
       </c>
       <c r="E142">
         <v>1</v>
@@ -4607,7 +4601,7 @@
         <v>142</v>
       </c>
       <c r="D143" t="s">
-        <v>316</v>
+        <v>315</v>
       </c>
       <c r="E143">
         <v>1</v>
@@ -4624,7 +4618,7 @@
         <v>143</v>
       </c>
       <c r="D144" t="s">
-        <v>317</v>
+        <v>316</v>
       </c>
       <c r="E144">
         <v>1</v>
@@ -4641,7 +4635,7 @@
         <v>144</v>
       </c>
       <c r="D145" t="s">
-        <v>318</v>
+        <v>317</v>
       </c>
       <c r="E145">
         <v>1</v>
@@ -4658,7 +4652,7 @@
         <v>145</v>
       </c>
       <c r="D146" t="s">
-        <v>319</v>
+        <v>318</v>
       </c>
       <c r="E146">
         <v>1</v>
@@ -4675,7 +4669,7 @@
         <v>146</v>
       </c>
       <c r="D147" t="s">
-        <v>320</v>
+        <v>319</v>
       </c>
       <c r="E147">
         <v>1</v>
@@ -4692,7 +4686,7 @@
         <v>147</v>
       </c>
       <c r="D148" t="s">
-        <v>321</v>
+        <v>320</v>
       </c>
       <c r="E148">
         <v>1</v>
@@ -4709,7 +4703,7 @@
         <v>148</v>
       </c>
       <c r="D149" t="s">
-        <v>322</v>
+        <v>321</v>
       </c>
       <c r="E149">
         <v>1</v>
@@ -4726,7 +4720,7 @@
         <v>149</v>
       </c>
       <c r="D150" t="s">
-        <v>323</v>
+        <v>322</v>
       </c>
       <c r="E150">
         <v>1</v>
@@ -4743,7 +4737,7 @@
         <v>150</v>
       </c>
       <c r="D151" t="s">
-        <v>324</v>
+        <v>323</v>
       </c>
       <c r="E151">
         <v>1</v>
@@ -4760,7 +4754,7 @@
         <v>151</v>
       </c>
       <c r="D152" t="s">
-        <v>325</v>
+        <v>324</v>
       </c>
       <c r="E152">
         <v>1</v>
@@ -4777,7 +4771,7 @@
         <v>152</v>
       </c>
       <c r="D153" t="s">
-        <v>326</v>
+        <v>325</v>
       </c>
       <c r="E153">
         <v>1</v>
@@ -4794,7 +4788,7 @@
         <v>153</v>
       </c>
       <c r="D154" t="s">
-        <v>327</v>
+        <v>326</v>
       </c>
       <c r="E154">
         <v>1</v>
@@ -4811,7 +4805,7 @@
         <v>154</v>
       </c>
       <c r="D155" t="s">
-        <v>328</v>
+        <v>327</v>
       </c>
       <c r="E155">
         <v>1</v>
@@ -4828,7 +4822,7 @@
         <v>155</v>
       </c>
       <c r="D156" t="s">
-        <v>329</v>
+        <v>328</v>
       </c>
       <c r="E156">
         <v>1</v>
@@ -4845,7 +4839,7 @@
         <v>156</v>
       </c>
       <c r="D157" t="s">
-        <v>330</v>
+        <v>329</v>
       </c>
       <c r="E157">
         <v>1</v>
@@ -4862,7 +4856,7 @@
         <v>157</v>
       </c>
       <c r="D158" t="s">
-        <v>331</v>
+        <v>330</v>
       </c>
       <c r="E158">
         <v>1</v>
@@ -4879,7 +4873,7 @@
         <v>158</v>
       </c>
       <c r="D159" t="s">
-        <v>332</v>
+        <v>331</v>
       </c>
       <c r="E159">
         <v>1</v>
@@ -4896,7 +4890,7 @@
         <v>159</v>
       </c>
       <c r="D160" t="s">
-        <v>333</v>
+        <v>332</v>
       </c>
       <c r="E160">
         <v>1</v>
@@ -4913,10 +4907,10 @@
         <v>160</v>
       </c>
       <c r="D161" t="s">
-        <v>334</v>
+        <v>317</v>
       </c>
       <c r="E161">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="162" spans="1:5">
@@ -4930,7 +4924,7 @@
         <v>161</v>
       </c>
       <c r="D162" t="s">
-        <v>319</v>
+        <v>333</v>
       </c>
       <c r="E162">
         <v>2</v>
@@ -4947,7 +4941,7 @@
         <v>162</v>
       </c>
       <c r="D163" t="s">
-        <v>335</v>
+        <v>334</v>
       </c>
       <c r="E163">
         <v>2</v>
@@ -4964,7 +4958,7 @@
         <v>163</v>
       </c>
       <c r="D164" t="s">
-        <v>336</v>
+        <v>335</v>
       </c>
       <c r="E164">
         <v>2</v>
@@ -4981,7 +4975,7 @@
         <v>164</v>
       </c>
       <c r="D165" t="s">
-        <v>337</v>
+        <v>336</v>
       </c>
       <c r="E165">
         <v>2</v>
@@ -4998,10 +4992,10 @@
         <v>165</v>
       </c>
       <c r="D166" t="s">
-        <v>338</v>
+        <v>337</v>
       </c>
       <c r="E166">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="167" spans="1:5">
@@ -5015,10 +5009,10 @@
         <v>166</v>
       </c>
       <c r="D167" t="s">
-        <v>339</v>
+        <v>301</v>
       </c>
       <c r="E167">
-        <v>3</v>
+        <v>5</v>
       </c>
     </row>
     <row r="168" spans="1:5">
@@ -5032,10 +5026,10 @@
         <v>167</v>
       </c>
       <c r="D168" t="s">
-        <v>303</v>
+        <v>338</v>
       </c>
       <c r="E168">
-        <v>5</v>
+        <v>8</v>
       </c>
     </row>
     <row r="169" spans="1:5">
@@ -5049,7 +5043,7 @@
         <v>168</v>
       </c>
       <c r="D169" t="s">
-        <v>340</v>
+        <v>253</v>
       </c>
       <c r="E169">
         <v>8</v>
@@ -5066,10 +5060,10 @@
         <v>169</v>
       </c>
       <c r="D170" t="s">
-        <v>255</v>
+        <v>339</v>
       </c>
       <c r="E170">
-        <v>8</v>
+        <v>10</v>
       </c>
     </row>
     <row r="171" spans="1:5">
@@ -5083,10 +5077,10 @@
         <v>170</v>
       </c>
       <c r="D171" t="s">
-        <v>341</v>
+        <v>340</v>
       </c>
       <c r="E171">
-        <v>10</v>
+        <v>1</v>
       </c>
     </row>
     <row r="172" spans="1:5">
@@ -5100,7 +5094,7 @@
         <v>171</v>
       </c>
       <c r="D172" t="s">
-        <v>342</v>
+        <v>341</v>
       </c>
       <c r="E172">
         <v>1</v>
@@ -5108,16 +5102,16 @@
     </row>
     <row r="173" spans="1:5">
       <c r="A173" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="B173" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="C173" t="s">
         <v>172</v>
       </c>
       <c r="D173" t="s">
-        <v>343</v>
+        <v>327</v>
       </c>
       <c r="E173">
         <v>1</v>
@@ -5134,7 +5128,7 @@
         <v>173</v>
       </c>
       <c r="D174" t="s">
-        <v>329</v>
+        <v>342</v>
       </c>
       <c r="E174">
         <v>1</v>
@@ -5151,7 +5145,7 @@
         <v>174</v>
       </c>
       <c r="D175" t="s">
-        <v>344</v>
+        <v>343</v>
       </c>
       <c r="E175">
         <v>1</v>
@@ -5168,7 +5162,7 @@
         <v>175</v>
       </c>
       <c r="D176" t="s">
-        <v>345</v>
+        <v>344</v>
       </c>
       <c r="E176">
         <v>1</v>
@@ -5185,7 +5179,7 @@
         <v>176</v>
       </c>
       <c r="D177" t="s">
-        <v>346</v>
+        <v>345</v>
       </c>
       <c r="E177">
         <v>1</v>
@@ -5202,7 +5196,7 @@
         <v>177</v>
       </c>
       <c r="D178" t="s">
-        <v>347</v>
+        <v>346</v>
       </c>
       <c r="E178">
         <v>1</v>
@@ -5219,7 +5213,7 @@
         <v>178</v>
       </c>
       <c r="D179" t="s">
-        <v>348</v>
+        <v>263</v>
       </c>
       <c r="E179">
         <v>1</v>
@@ -5236,7 +5230,7 @@
         <v>179</v>
       </c>
       <c r="D180" t="s">
-        <v>265</v>
+        <v>347</v>
       </c>
       <c r="E180">
         <v>1</v>
@@ -5253,7 +5247,7 @@
         <v>180</v>
       </c>
       <c r="D181" t="s">
-        <v>349</v>
+        <v>348</v>
       </c>
       <c r="E181">
         <v>1</v>
@@ -5270,7 +5264,7 @@
         <v>181</v>
       </c>
       <c r="D182" t="s">
-        <v>350</v>
+        <v>349</v>
       </c>
       <c r="E182">
         <v>1</v>
@@ -5287,7 +5281,7 @@
         <v>182</v>
       </c>
       <c r="D183" t="s">
-        <v>351</v>
+        <v>350</v>
       </c>
       <c r="E183">
         <v>1</v>
@@ -5304,7 +5298,7 @@
         <v>183</v>
       </c>
       <c r="D184" t="s">
-        <v>352</v>
+        <v>351</v>
       </c>
       <c r="E184">
         <v>1</v>
@@ -5321,7 +5315,7 @@
         <v>184</v>
       </c>
       <c r="D185" t="s">
-        <v>353</v>
+        <v>352</v>
       </c>
       <c r="E185">
         <v>1</v>
@@ -5338,7 +5332,7 @@
         <v>185</v>
       </c>
       <c r="D186" t="s">
-        <v>354</v>
+        <v>353</v>
       </c>
       <c r="E186">
         <v>1</v>
@@ -5355,7 +5349,7 @@
         <v>186</v>
       </c>
       <c r="D187" t="s">
-        <v>355</v>
+        <v>354</v>
       </c>
       <c r="E187">
         <v>1</v>
@@ -5372,7 +5366,7 @@
         <v>187</v>
       </c>
       <c r="D188" t="s">
-        <v>356</v>
+        <v>355</v>
       </c>
       <c r="E188">
         <v>1</v>
@@ -5389,7 +5383,7 @@
         <v>188</v>
       </c>
       <c r="D189" t="s">
-        <v>357</v>
+        <v>356</v>
       </c>
       <c r="E189">
         <v>1</v>
@@ -5406,7 +5400,7 @@
         <v>189</v>
       </c>
       <c r="D190" t="s">
-        <v>358</v>
+        <v>357</v>
       </c>
       <c r="E190">
         <v>1</v>
@@ -5423,7 +5417,7 @@
         <v>190</v>
       </c>
       <c r="D191" t="s">
-        <v>359</v>
+        <v>358</v>
       </c>
       <c r="E191">
         <v>1</v>
@@ -5440,7 +5434,7 @@
         <v>191</v>
       </c>
       <c r="D192" t="s">
-        <v>360</v>
+        <v>359</v>
       </c>
       <c r="E192">
         <v>1</v>
@@ -5457,7 +5451,7 @@
         <v>192</v>
       </c>
       <c r="D193" t="s">
-        <v>361</v>
+        <v>360</v>
       </c>
       <c r="E193">
         <v>1</v>
@@ -5474,7 +5468,7 @@
         <v>193</v>
       </c>
       <c r="D194" t="s">
-        <v>362</v>
+        <v>361</v>
       </c>
       <c r="E194">
         <v>1</v>
@@ -5491,7 +5485,7 @@
         <v>194</v>
       </c>
       <c r="D195" t="s">
-        <v>363</v>
+        <v>362</v>
       </c>
       <c r="E195">
         <v>1</v>
@@ -5508,7 +5502,7 @@
         <v>195</v>
       </c>
       <c r="D196" t="s">
-        <v>364</v>
+        <v>363</v>
       </c>
       <c r="E196">
         <v>1</v>
@@ -5525,7 +5519,7 @@
         <v>196</v>
       </c>
       <c r="D197" t="s">
-        <v>365</v>
+        <v>364</v>
       </c>
       <c r="E197">
         <v>1</v>
@@ -5542,7 +5536,7 @@
         <v>197</v>
       </c>
       <c r="D198" t="s">
-        <v>366</v>
+        <v>365</v>
       </c>
       <c r="E198">
         <v>1</v>
@@ -5559,7 +5553,7 @@
         <v>198</v>
       </c>
       <c r="D199" t="s">
-        <v>367</v>
+        <v>366</v>
       </c>
       <c r="E199">
         <v>1</v>
@@ -5576,7 +5570,7 @@
         <v>199</v>
       </c>
       <c r="D200" t="s">
-        <v>368</v>
+        <v>367</v>
       </c>
       <c r="E200">
         <v>1</v>
@@ -5593,7 +5587,7 @@
         <v>200</v>
       </c>
       <c r="D201" t="s">
-        <v>369</v>
+        <v>368</v>
       </c>
       <c r="E201">
         <v>1</v>
@@ -5610,7 +5604,7 @@
         <v>201</v>
       </c>
       <c r="D202" t="s">
-        <v>370</v>
+        <v>369</v>
       </c>
       <c r="E202">
         <v>1</v>
@@ -5627,7 +5621,7 @@
         <v>202</v>
       </c>
       <c r="D203" t="s">
-        <v>371</v>
+        <v>370</v>
       </c>
       <c r="E203">
         <v>1</v>
@@ -5644,7 +5638,7 @@
         <v>203</v>
       </c>
       <c r="D204" t="s">
-        <v>372</v>
+        <v>371</v>
       </c>
       <c r="E204">
         <v>1</v>
@@ -5661,10 +5655,10 @@
         <v>204</v>
       </c>
       <c r="D205" t="s">
-        <v>373</v>
+        <v>372</v>
       </c>
       <c r="E205">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="206" spans="1:5">
@@ -5678,7 +5672,7 @@
         <v>205</v>
       </c>
       <c r="D206" t="s">
-        <v>374</v>
+        <v>373</v>
       </c>
       <c r="E206">
         <v>2</v>
@@ -5695,7 +5689,7 @@
         <v>206</v>
       </c>
       <c r="D207" t="s">
-        <v>375</v>
+        <v>374</v>
       </c>
       <c r="E207">
         <v>2</v>
@@ -5712,7 +5706,7 @@
         <v>207</v>
       </c>
       <c r="D208" t="s">
-        <v>376</v>
+        <v>375</v>
       </c>
       <c r="E208">
         <v>2</v>
@@ -5729,7 +5723,7 @@
         <v>208</v>
       </c>
       <c r="D209" t="s">
-        <v>377</v>
+        <v>376</v>
       </c>
       <c r="E209">
         <v>2</v>
@@ -5746,7 +5740,7 @@
         <v>209</v>
       </c>
       <c r="D210" t="s">
-        <v>378</v>
+        <v>377</v>
       </c>
       <c r="E210">
         <v>2</v>
@@ -5763,7 +5757,7 @@
         <v>210</v>
       </c>
       <c r="D211" t="s">
-        <v>379</v>
+        <v>378</v>
       </c>
       <c r="E211">
         <v>2</v>
@@ -5780,7 +5774,7 @@
         <v>211</v>
       </c>
       <c r="D212" t="s">
-        <v>380</v>
+        <v>379</v>
       </c>
       <c r="E212">
         <v>2</v>
@@ -5797,7 +5791,7 @@
         <v>212</v>
       </c>
       <c r="D213" t="s">
-        <v>381</v>
+        <v>379</v>
       </c>
       <c r="E213">
         <v>2</v>
@@ -5805,19 +5799,19 @@
     </row>
     <row r="214" spans="1:5">
       <c r="A214" t="s">
-        <v>15</v>
+        <v>6</v>
       </c>
       <c r="B214" t="s">
-        <v>41</v>
+        <v>36</v>
       </c>
       <c r="C214" t="s">
         <v>213</v>
       </c>
       <c r="D214" t="s">
-        <v>381</v>
+        <v>380</v>
       </c>
       <c r="E214">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="215" spans="1:5">
@@ -5828,10 +5822,10 @@
         <v>41</v>
       </c>
       <c r="C215" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
       <c r="D215" t="s">
-        <v>382</v>
+        <v>380</v>
       </c>
       <c r="E215">
         <v>2</v>
@@ -5845,10 +5839,10 @@
         <v>41</v>
       </c>
       <c r="C216" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
       <c r="D216" t="s">
-        <v>383</v>
+        <v>381</v>
       </c>
       <c r="E216">
         <v>2</v>
@@ -5862,10 +5856,10 @@
         <v>41</v>
       </c>
       <c r="C217" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
       <c r="D217" t="s">
-        <v>384</v>
+        <v>382</v>
       </c>
       <c r="E217">
         <v>2</v>
@@ -5879,10 +5873,10 @@
         <v>41</v>
       </c>
       <c r="C218" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
       <c r="D218" t="s">
-        <v>385</v>
+        <v>383</v>
       </c>
       <c r="E218">
         <v>3</v>
@@ -5896,10 +5890,10 @@
         <v>41</v>
       </c>
       <c r="C219" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
       <c r="D219" t="s">
-        <v>265</v>
+        <v>263</v>
       </c>
       <c r="E219">
         <v>3</v>
@@ -5913,10 +5907,10 @@
         <v>41</v>
       </c>
       <c r="C220" t="s">
-        <v>219</v>
+        <v>218</v>
       </c>
       <c r="D220" t="s">
-        <v>386</v>
+        <v>384</v>
       </c>
       <c r="E220">
         <v>4</v>
@@ -5930,10 +5924,10 @@
         <v>41</v>
       </c>
       <c r="C221" t="s">
-        <v>220</v>
+        <v>219</v>
       </c>
       <c r="D221" t="s">
-        <v>387</v>
+        <v>385</v>
       </c>
       <c r="E221">
         <v>4</v>
@@ -5947,10 +5941,10 @@
         <v>41</v>
       </c>
       <c r="C222" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
       <c r="D222" t="s">
-        <v>388</v>
+        <v>386</v>
       </c>
       <c r="E222">
         <v>4</v>
@@ -5964,10 +5958,10 @@
         <v>41</v>
       </c>
       <c r="C223" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
       <c r="D223" t="s">
-        <v>389</v>
+        <v>387</v>
       </c>
       <c r="E223">
         <v>4</v>
@@ -5981,10 +5975,10 @@
         <v>41</v>
       </c>
       <c r="C224" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
       <c r="D224" t="s">
-        <v>390</v>
+        <v>388</v>
       </c>
       <c r="E224">
         <v>4</v>
@@ -5998,10 +5992,10 @@
         <v>41</v>
       </c>
       <c r="C225" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="D225" t="s">
-        <v>391</v>
+        <v>389</v>
       </c>
       <c r="E225">
         <v>5</v>
@@ -6015,10 +6009,10 @@
         <v>41</v>
       </c>
       <c r="C226" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
       <c r="D226" t="s">
-        <v>392</v>
+        <v>390</v>
       </c>
       <c r="E226">
         <v>5</v>
@@ -6032,10 +6026,10 @@
         <v>41</v>
       </c>
       <c r="C227" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
       <c r="D227" t="s">
-        <v>393</v>
+        <v>391</v>
       </c>
       <c r="E227">
         <v>6</v>
@@ -6049,10 +6043,10 @@
         <v>41</v>
       </c>
       <c r="C228" t="s">
-        <v>227</v>
+        <v>226</v>
       </c>
       <c r="D228" t="s">
-        <v>394</v>
+        <v>392</v>
       </c>
       <c r="E228">
         <v>8</v>
@@ -6066,10 +6060,10 @@
         <v>41</v>
       </c>
       <c r="C229" t="s">
-        <v>228</v>
+        <v>227</v>
       </c>
       <c r="D229" t="s">
-        <v>395</v>
+        <v>393</v>
       </c>
       <c r="E229">
         <v>10</v>
@@ -6083,10 +6077,10 @@
         <v>41</v>
       </c>
       <c r="C230" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
       <c r="D230" t="s">
-        <v>395</v>
+        <v>393</v>
       </c>
       <c r="E230">
         <v>10</v>
@@ -6100,10 +6094,10 @@
         <v>41</v>
       </c>
       <c r="C231" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="D231" t="s">
-        <v>267</v>
+        <v>265</v>
       </c>
       <c r="E231">
         <v>12</v>
@@ -6117,10 +6111,10 @@
         <v>41</v>
       </c>
       <c r="C232" t="s">
-        <v>231</v>
+        <v>230</v>
       </c>
       <c r="D232" t="s">
-        <v>396</v>
+        <v>394</v>
       </c>
       <c r="E232">
         <v>12</v>
@@ -6134,10 +6128,10 @@
         <v>41</v>
       </c>
       <c r="C233" t="s">
-        <v>232</v>
+        <v>231</v>
       </c>
       <c r="D233" t="s">
-        <v>397</v>
+        <v>395</v>
       </c>
       <c r="E233">
         <v>14</v>
@@ -6151,10 +6145,10 @@
         <v>41</v>
       </c>
       <c r="C234" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
       <c r="D234" t="s">
-        <v>398</v>
+        <v>396</v>
       </c>
       <c r="E234">
         <v>15</v>
@@ -6168,10 +6162,10 @@
         <v>41</v>
       </c>
       <c r="C235" t="s">
-        <v>234</v>
+        <v>233</v>
       </c>
       <c r="D235" t="s">
-        <v>399</v>
+        <v>397</v>
       </c>
       <c r="E235">
         <v>20</v>
@@ -6185,10 +6179,10 @@
         <v>36</v>
       </c>
       <c r="C236" t="s">
-        <v>235</v>
+        <v>234</v>
       </c>
       <c r="D236" t="s">
-        <v>400</v>
+        <v>398</v>
       </c>
       <c r="E236">
         <v>1</v>

</xml_diff>

<commit_message>
Atualização automática: rac (29/09/2026 19:53)
</commit_message>
<xml_diff>
--- a/Coordenadoria/02_Dados_Tratados/base_rac_tratada.xlsx
+++ b/Coordenadoria/02_Dados_Tratados/base_rac_tratada.xlsx
@@ -1218,8 +1218,16 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <fonts count="1">
+  <fonts count="2">
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -1235,7 +1243,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -1243,12 +1251,30 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1547,22 +1573,22 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:6">
-      <c r="A1" t="s">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" t="s">
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" t="s">
+      <c r="F1" s="1" t="s">
         <v>5</v>
       </c>
     </row>
@@ -2177,19 +2203,19 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:5">
-      <c r="A1" t="s">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" t="s">
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
         <v>55</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>56</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="1" t="s">
         <v>57</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualização automática: rac (02/10/2026 09:56)
</commit_message>
<xml_diff>
--- a/Coordenadoria/02_Dados_Tratados/base_rac_tratada.xlsx
+++ b/Coordenadoria/02_Dados_Tratados/base_rac_tratada.xlsx
@@ -1242,8 +1242,16 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <fonts count="1">
+  <fonts count="2">
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -1259,7 +1267,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -1267,12 +1275,30 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1571,22 +1597,22 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:6">
-      <c r="A1" t="s">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" t="s">
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" t="s">
+      <c r="F1" s="1" t="s">
         <v>5</v>
       </c>
     </row>
@@ -2201,19 +2227,19 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:5">
-      <c r="A1" t="s">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" t="s">
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
         <v>55</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>56</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="1" t="s">
         <v>57</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualização automática: rac (05/10/2026 08:39)
</commit_message>
<xml_diff>
--- a/Coordenadoria/02_Dados_Tratados/base_rac_tratada.xlsx
+++ b/Coordenadoria/02_Dados_Tratados/base_rac_tratada.xlsx
@@ -194,45 +194,57 @@
     <t>2641008-200</t>
   </si>
   <si>
+    <t>2643031-7</t>
+  </si>
+  <si>
+    <t>P7036368-01</t>
+  </si>
+  <si>
+    <t>066-3046-07</t>
+  </si>
+  <si>
+    <t>200SGL153Q</t>
+  </si>
+  <si>
+    <t>AN921-3D</t>
+  </si>
+  <si>
+    <t>MS28778-3</t>
+  </si>
+  <si>
+    <t>2643084-1</t>
+  </si>
+  <si>
+    <t>431-0101-01</t>
+  </si>
+  <si>
+    <t>2643100-206</t>
+  </si>
+  <si>
+    <t>3107453-01</t>
+  </si>
+  <si>
+    <t>3026812</t>
+  </si>
+  <si>
+    <t>3013411</t>
+  </si>
+  <si>
+    <t>3043672CL03</t>
+  </si>
+  <si>
+    <t>25536-4</t>
+  </si>
+  <si>
     <t>MS24462-5</t>
   </si>
   <si>
-    <t>2643031-7</t>
-  </si>
-  <si>
     <t>2698010-7</t>
   </si>
   <si>
     <t>3044000</t>
   </si>
   <si>
-    <t>P7036368-01</t>
-  </si>
-  <si>
-    <t>066-3046-07</t>
-  </si>
-  <si>
-    <t>2643084-1</t>
-  </si>
-  <si>
-    <t>431-0101-01</t>
-  </si>
-  <si>
-    <t>3107453-01</t>
-  </si>
-  <si>
-    <t>3026812</t>
-  </si>
-  <si>
-    <t>3013411</t>
-  </si>
-  <si>
-    <t>3043672CL03</t>
-  </si>
-  <si>
-    <t>25536-4</t>
-  </si>
-  <si>
     <t>C611505-0201</t>
   </si>
   <si>
@@ -251,9 +263,6 @@
     <t>162-10700</t>
   </si>
   <si>
-    <t>2643100-206</t>
-  </si>
-  <si>
     <t>400454</t>
   </si>
   <si>
@@ -728,57 +737,60 @@
     <t>2670067-1</t>
   </si>
   <si>
-    <t>200SGL153Q</t>
-  </si>
-  <si>
-    <t>AN921-3D</t>
-  </si>
-  <si>
-    <t>MS28778-3</t>
-  </si>
-  <si>
     <t>PIN-MAIN GEAR ATTACH</t>
   </si>
   <si>
+    <t>FORK ASSY,NOSE GEAR SPRING</t>
+  </si>
+  <si>
+    <t>PROPELLER ASSEMBLY</t>
+  </si>
+  <si>
+    <t>CONTROL,INDICATOR</t>
+  </si>
+  <si>
+    <t>STARTER GENERATOR</t>
+  </si>
+  <si>
+    <t>ELBOW</t>
+  </si>
+  <si>
+    <t>O-RING</t>
+  </si>
+  <si>
+    <t>TORQUE LINK ASSY-UPP</t>
+  </si>
+  <si>
+    <t>SWITCH,PROXIMITY</t>
+  </si>
+  <si>
+    <t>NOSE GEAR STRUT ASSY - TALL FORK</t>
+  </si>
+  <si>
+    <t>HOUSING</t>
+  </si>
+  <si>
+    <t>DISK AND HUB,TURBIN</t>
+  </si>
+  <si>
+    <t>DISK AND HUB,COMPRE</t>
+  </si>
+  <si>
+    <t>STATOR ASSY-POWER TU</t>
+  </si>
+  <si>
+    <t>FLOW DIVIDER</t>
+  </si>
+  <si>
     <t>BEARING ROLLER</t>
   </si>
   <si>
-    <t>FORK ASSY,NOSE GEAR SPRING</t>
-  </si>
-  <si>
     <t>PASSENGER DOOR - LOW</t>
   </si>
   <si>
     <t>ENGINE PT6A-114A</t>
   </si>
   <si>
-    <t>PROPELLER ASSEMBLY</t>
-  </si>
-  <si>
-    <t>CONTROL,INDICATOR</t>
-  </si>
-  <si>
-    <t>TORQUE LINK ASSY-UPP</t>
-  </si>
-  <si>
-    <t>SWITCH,PROXIMITY</t>
-  </si>
-  <si>
-    <t>HOUSING</t>
-  </si>
-  <si>
-    <t>DISK AND HUB,TURBIN</t>
-  </si>
-  <si>
-    <t>DISK AND HUB,COMPRE</t>
-  </si>
-  <si>
-    <t>STATOR ASSY-POWER TU</t>
-  </si>
-  <si>
-    <t>FLOW DIVIDER</t>
-  </si>
-  <si>
     <t>ALTERNATOR</t>
   </si>
   <si>
@@ -797,9 +809,6 @@
     <t>OUTER WHEEL HALF ASSY</t>
   </si>
   <si>
-    <t>NOSE GEAR STRUT ASSY - TALL FORK</t>
-  </si>
-  <si>
     <t>SEAL,PLAIN ENCASED</t>
   </si>
   <si>
@@ -1233,23 +1242,22 @@
   </si>
   <si>
     <t>POST LIGHT ASS</t>
-  </si>
-  <si>
-    <t>STARTER GENERATOR</t>
-  </si>
-  <si>
-    <t>ELBOW</t>
-  </si>
-  <si>
-    <t>O-RING</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <fonts count="1">
+  <fonts count="2">
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -1265,7 +1273,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -1273,12 +1281,30 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1577,22 +1603,22 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:6">
-      <c r="A1" t="s">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" t="s">
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" t="s">
+      <c r="F1" s="1" t="s">
         <v>5</v>
       </c>
     </row>
@@ -2207,19 +2233,19 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:5">
-      <c r="A1" t="s">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" t="s">
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
         <v>55</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>56</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="1" t="s">
         <v>57</v>
       </c>
     </row>
@@ -2242,10 +2268,10 @@
     </row>
     <row r="3" spans="1:5">
       <c r="A3" t="s">
-        <v>14</v>
+        <v>6</v>
       </c>
       <c r="B3" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
       <c r="C3" t="s">
         <v>59</v>
@@ -2254,15 +2280,15 @@
         <v>241</v>
       </c>
       <c r="E3">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="4" spans="1:5">
       <c r="A4" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="B4" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="C4" t="s">
         <v>60</v>
@@ -2276,16 +2302,16 @@
     </row>
     <row r="5" spans="1:5">
       <c r="A5" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="B5" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="C5" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="D5" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
       <c r="E5">
         <v>1</v>
@@ -2293,16 +2319,16 @@
     </row>
     <row r="6" spans="1:5">
       <c r="A6" t="s">
-        <v>13</v>
+        <v>10</v>
       </c>
       <c r="B6" t="s">
         <v>39</v>
       </c>
       <c r="C6" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="D6" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
       <c r="E6">
         <v>1</v>
@@ -2310,16 +2336,16 @@
     </row>
     <row r="7" spans="1:5">
       <c r="A7" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="B7" t="s">
-        <v>39</v>
+        <v>36</v>
       </c>
       <c r="C7" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="D7" t="s">
-        <v>244</v>
+        <v>242</v>
       </c>
       <c r="E7">
         <v>1</v>
@@ -2327,16 +2353,16 @@
     </row>
     <row r="8" spans="1:5">
       <c r="A8" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B8" t="s">
-        <v>36</v>
+        <v>39</v>
       </c>
       <c r="C8" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="D8" t="s">
-        <v>244</v>
+        <v>242</v>
       </c>
       <c r="E8">
         <v>1</v>
@@ -2344,16 +2370,16 @@
     </row>
     <row r="9" spans="1:5">
       <c r="A9" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="B9" t="s">
         <v>39</v>
       </c>
       <c r="C9" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="D9" t="s">
-        <v>244</v>
+        <v>242</v>
       </c>
       <c r="E9">
         <v>1</v>
@@ -2361,16 +2387,16 @@
     </row>
     <row r="10" spans="1:5">
       <c r="A10" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="B10" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="C10" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="D10" t="s">
-        <v>244</v>
+        <v>242</v>
       </c>
       <c r="E10">
         <v>1</v>
@@ -2378,16 +2404,16 @@
     </row>
     <row r="11" spans="1:5">
       <c r="A11" t="s">
-        <v>14</v>
+        <v>7</v>
       </c>
       <c r="B11" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="C11" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="D11" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="E11">
         <v>1</v>
@@ -2401,10 +2427,10 @@
         <v>37</v>
       </c>
       <c r="C12" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="D12" t="s">
-        <v>245</v>
+        <v>244</v>
       </c>
       <c r="E12">
         <v>1</v>
@@ -2412,10 +2438,10 @@
     </row>
     <row r="13" spans="1:5">
       <c r="A13" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="B13" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="C13" t="s">
         <v>63</v>
@@ -2424,38 +2450,38 @@
         <v>245</v>
       </c>
       <c r="E13">
-        <v>1</v>
+        <v>4</v>
       </c>
     </row>
     <row r="14" spans="1:5">
       <c r="A14" t="s">
-        <v>10</v>
+        <v>7</v>
       </c>
       <c r="B14" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="C14" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="D14" t="s">
-        <v>245</v>
+        <v>246</v>
       </c>
       <c r="E14">
-        <v>1</v>
+        <v>4</v>
       </c>
     </row>
     <row r="15" spans="1:5">
       <c r="A15" t="s">
-        <v>11</v>
+        <v>8</v>
       </c>
       <c r="B15" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="C15" t="s">
-        <v>63</v>
+        <v>65</v>
       </c>
       <c r="D15" t="s">
-        <v>245</v>
+        <v>247</v>
       </c>
       <c r="E15">
         <v>1</v>
@@ -2463,16 +2489,16 @@
     </row>
     <row r="16" spans="1:5">
       <c r="A16" t="s">
-        <v>12</v>
+        <v>8</v>
       </c>
       <c r="B16" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="C16" t="s">
-        <v>63</v>
+        <v>66</v>
       </c>
       <c r="D16" t="s">
-        <v>245</v>
+        <v>248</v>
       </c>
       <c r="E16">
         <v>1</v>
@@ -2480,16 +2506,16 @@
     </row>
     <row r="17" spans="1:5">
       <c r="A17" t="s">
-        <v>13</v>
+        <v>8</v>
       </c>
       <c r="B17" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="C17" t="s">
-        <v>63</v>
+        <v>67</v>
       </c>
       <c r="D17" t="s">
-        <v>245</v>
+        <v>249</v>
       </c>
       <c r="E17">
         <v>1</v>
@@ -2497,16 +2523,16 @@
     </row>
     <row r="18" spans="1:5">
       <c r="A18" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="B18" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
       <c r="C18" t="s">
-        <v>63</v>
+        <v>67</v>
       </c>
       <c r="D18" t="s">
-        <v>245</v>
+        <v>249</v>
       </c>
       <c r="E18">
         <v>1</v>
@@ -2514,16 +2540,16 @@
     </row>
     <row r="19" spans="1:5">
       <c r="A19" t="s">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="B19" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="C19" t="s">
-        <v>64</v>
+        <v>68</v>
       </c>
       <c r="D19" t="s">
-        <v>246</v>
+        <v>250</v>
       </c>
       <c r="E19">
         <v>1</v>
@@ -2531,16 +2557,16 @@
     </row>
     <row r="20" spans="1:5">
       <c r="A20" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="B20" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
       <c r="C20" t="s">
-        <v>65</v>
+        <v>69</v>
       </c>
       <c r="D20" t="s">
-        <v>247</v>
+        <v>251</v>
       </c>
       <c r="E20">
         <v>1</v>
@@ -2548,16 +2574,16 @@
     </row>
     <row r="21" spans="1:5">
       <c r="A21" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="B21" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
       <c r="C21" t="s">
-        <v>66</v>
+        <v>70</v>
       </c>
       <c r="D21" t="s">
-        <v>248</v>
+        <v>252</v>
       </c>
       <c r="E21">
         <v>1</v>
@@ -2571,10 +2597,10 @@
         <v>36</v>
       </c>
       <c r="C22" t="s">
-        <v>67</v>
+        <v>71</v>
       </c>
       <c r="D22" t="s">
-        <v>249</v>
+        <v>253</v>
       </c>
       <c r="E22">
         <v>1</v>
@@ -2588,10 +2614,10 @@
         <v>36</v>
       </c>
       <c r="C23" t="s">
-        <v>68</v>
+        <v>72</v>
       </c>
       <c r="D23" t="s">
-        <v>250</v>
+        <v>254</v>
       </c>
       <c r="E23">
         <v>1</v>
@@ -2599,33 +2625,33 @@
     </row>
     <row r="24" spans="1:5">
       <c r="A24" t="s">
-        <v>9</v>
+        <v>14</v>
       </c>
       <c r="B24" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="C24" t="s">
-        <v>69</v>
+        <v>73</v>
       </c>
       <c r="D24" t="s">
-        <v>251</v>
+        <v>255</v>
       </c>
       <c r="E24">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="25" spans="1:5">
       <c r="A25" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="B25" t="s">
-        <v>36</v>
+        <v>39</v>
       </c>
       <c r="C25" t="s">
-        <v>70</v>
+        <v>74</v>
       </c>
       <c r="D25" t="s">
-        <v>252</v>
+        <v>256</v>
       </c>
       <c r="E25">
         <v>1</v>
@@ -2633,16 +2659,16 @@
     </row>
     <row r="26" spans="1:5">
       <c r="A26" t="s">
-        <v>9</v>
+        <v>13</v>
       </c>
       <c r="B26" t="s">
-        <v>36</v>
+        <v>39</v>
       </c>
       <c r="C26" t="s">
-        <v>71</v>
+        <v>74</v>
       </c>
       <c r="D26" t="s">
-        <v>253</v>
+        <v>256</v>
       </c>
       <c r="E26">
         <v>1</v>
@@ -2650,16 +2676,16 @@
     </row>
     <row r="27" spans="1:5">
       <c r="A27" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B27" t="s">
-        <v>36</v>
+        <v>39</v>
       </c>
       <c r="C27" t="s">
-        <v>72</v>
+        <v>75</v>
       </c>
       <c r="D27" t="s">
-        <v>254</v>
+        <v>257</v>
       </c>
       <c r="E27">
         <v>1</v>
@@ -2667,16 +2693,16 @@
     </row>
     <row r="28" spans="1:5">
       <c r="A28" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B28" t="s">
-        <v>39</v>
+        <v>36</v>
       </c>
       <c r="C28" t="s">
-        <v>72</v>
+        <v>75</v>
       </c>
       <c r="D28" t="s">
-        <v>254</v>
+        <v>257</v>
       </c>
       <c r="E28">
         <v>1</v>
@@ -2684,16 +2710,16 @@
     </row>
     <row r="29" spans="1:5">
       <c r="A29" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B29" t="s">
         <v>39</v>
       </c>
       <c r="C29" t="s">
-        <v>72</v>
+        <v>75</v>
       </c>
       <c r="D29" t="s">
-        <v>254</v>
+        <v>257</v>
       </c>
       <c r="E29">
         <v>1</v>
@@ -2701,16 +2727,16 @@
     </row>
     <row r="30" spans="1:5">
       <c r="A30" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="B30" t="s">
-        <v>36</v>
+        <v>39</v>
       </c>
       <c r="C30" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="D30" t="s">
-        <v>255</v>
+        <v>257</v>
       </c>
       <c r="E30">
         <v>1</v>
@@ -2718,16 +2744,16 @@
     </row>
     <row r="31" spans="1:5">
       <c r="A31" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="B31" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="C31" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="D31" t="s">
-        <v>255</v>
+        <v>257</v>
       </c>
       <c r="E31">
         <v>1</v>
@@ -2735,16 +2761,16 @@
     </row>
     <row r="32" spans="1:5">
       <c r="A32" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="B32" t="s">
-        <v>39</v>
+        <v>36</v>
       </c>
       <c r="C32" t="s">
-        <v>73</v>
+        <v>76</v>
       </c>
       <c r="D32" t="s">
-        <v>255</v>
+        <v>258</v>
       </c>
       <c r="E32">
         <v>1</v>
@@ -2752,16 +2778,16 @@
     </row>
     <row r="33" spans="1:5">
       <c r="A33" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B33" t="s">
-        <v>36</v>
+        <v>39</v>
       </c>
       <c r="C33" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="D33" t="s">
-        <v>256</v>
+        <v>258</v>
       </c>
       <c r="E33">
         <v>1</v>
@@ -2769,16 +2795,16 @@
     </row>
     <row r="34" spans="1:5">
       <c r="A34" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="B34" t="s">
         <v>39</v>
       </c>
       <c r="C34" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="D34" t="s">
-        <v>256</v>
+        <v>258</v>
       </c>
       <c r="E34">
         <v>1</v>
@@ -2792,10 +2818,10 @@
         <v>36</v>
       </c>
       <c r="C35" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="D35" t="s">
-        <v>257</v>
+        <v>259</v>
       </c>
       <c r="E35">
         <v>1</v>
@@ -2803,16 +2829,16 @@
     </row>
     <row r="36" spans="1:5">
       <c r="A36" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B36" t="s">
         <v>39</v>
       </c>
       <c r="C36" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="D36" t="s">
-        <v>257</v>
+        <v>259</v>
       </c>
       <c r="E36">
         <v>1</v>
@@ -2820,16 +2846,16 @@
     </row>
     <row r="37" spans="1:5">
       <c r="A37" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B37" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="C37" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="D37" t="s">
-        <v>257</v>
+        <v>259</v>
       </c>
       <c r="E37">
         <v>1</v>
@@ -2843,10 +2869,10 @@
         <v>36</v>
       </c>
       <c r="C38" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="D38" t="s">
-        <v>258</v>
+        <v>260</v>
       </c>
       <c r="E38">
         <v>1</v>
@@ -2854,19 +2880,19 @@
     </row>
     <row r="39" spans="1:5">
       <c r="A39" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="B39" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="C39" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="D39" t="s">
-        <v>258</v>
+        <v>260</v>
       </c>
       <c r="E39">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="40" spans="1:5">
@@ -2877,10 +2903,10 @@
         <v>36</v>
       </c>
       <c r="C40" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="D40" t="s">
-        <v>259</v>
+        <v>261</v>
       </c>
       <c r="E40">
         <v>1</v>
@@ -2888,16 +2914,16 @@
     </row>
     <row r="41" spans="1:5">
       <c r="A41" t="s">
-        <v>8</v>
+        <v>13</v>
       </c>
       <c r="B41" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="C41" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="D41" t="s">
-        <v>260</v>
+        <v>261</v>
       </c>
       <c r="E41">
         <v>1</v>
@@ -2905,16 +2931,16 @@
     </row>
     <row r="42" spans="1:5">
       <c r="A42" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="B42" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="C42" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="D42" t="s">
-        <v>260</v>
+        <v>261</v>
       </c>
       <c r="E42">
         <v>1</v>
@@ -2928,10 +2954,10 @@
         <v>36</v>
       </c>
       <c r="C43" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="D43" t="s">
-        <v>261</v>
+        <v>262</v>
       </c>
       <c r="E43">
         <v>1</v>
@@ -2939,10 +2965,10 @@
     </row>
     <row r="44" spans="1:5">
       <c r="A44" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="B44" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="C44" t="s">
         <v>80</v>
@@ -2951,7 +2977,7 @@
         <v>262</v>
       </c>
       <c r="E44">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="45" spans="1:5">
@@ -3036,55 +3062,55 @@
         <v>267</v>
       </c>
       <c r="E49">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="50" spans="1:5">
       <c r="A50" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B50" t="s">
-        <v>39</v>
+        <v>36</v>
       </c>
       <c r="C50" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="D50" t="s">
-        <v>267</v>
+        <v>268</v>
       </c>
       <c r="E50">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="51" spans="1:5">
       <c r="A51" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="B51" t="s">
-        <v>39</v>
+        <v>36</v>
       </c>
       <c r="C51" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="D51" t="s">
-        <v>267</v>
+        <v>269</v>
       </c>
       <c r="E51">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="52" spans="1:5">
       <c r="A52" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="B52" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
       <c r="C52" t="s">
-        <v>85</v>
+        <v>88</v>
       </c>
       <c r="D52" t="s">
-        <v>267</v>
+        <v>270</v>
       </c>
       <c r="E52">
         <v>2</v>
@@ -3092,19 +3118,19 @@
     </row>
     <row r="53" spans="1:5">
       <c r="A53" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B53" t="s">
-        <v>36</v>
+        <v>39</v>
       </c>
       <c r="C53" t="s">
-        <v>86</v>
+        <v>88</v>
       </c>
       <c r="D53" t="s">
-        <v>268</v>
+        <v>270</v>
       </c>
       <c r="E53">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="54" spans="1:5">
@@ -3115,10 +3141,10 @@
         <v>39</v>
       </c>
       <c r="C54" t="s">
-        <v>86</v>
+        <v>88</v>
       </c>
       <c r="D54" t="s">
-        <v>268</v>
+        <v>270</v>
       </c>
       <c r="E54">
         <v>2</v>
@@ -3132,13 +3158,13 @@
         <v>38</v>
       </c>
       <c r="C55" t="s">
-        <v>86</v>
+        <v>88</v>
       </c>
       <c r="D55" t="s">
-        <v>268</v>
+        <v>270</v>
       </c>
       <c r="E55">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="56" spans="1:5">
@@ -3149,10 +3175,10 @@
         <v>36</v>
       </c>
       <c r="C56" t="s">
-        <v>87</v>
+        <v>89</v>
       </c>
       <c r="D56" t="s">
-        <v>269</v>
+        <v>271</v>
       </c>
       <c r="E56">
         <v>2</v>
@@ -3166,13 +3192,13 @@
         <v>39</v>
       </c>
       <c r="C57" t="s">
-        <v>87</v>
+        <v>89</v>
       </c>
       <c r="D57" t="s">
-        <v>269</v>
+        <v>271</v>
       </c>
       <c r="E57">
-        <v>4</v>
+        <v>2</v>
       </c>
     </row>
     <row r="58" spans="1:5">
@@ -3183,13 +3209,13 @@
         <v>38</v>
       </c>
       <c r="C58" t="s">
-        <v>87</v>
+        <v>89</v>
       </c>
       <c r="D58" t="s">
-        <v>269</v>
+        <v>271</v>
       </c>
       <c r="E58">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="59" spans="1:5">
@@ -3200,10 +3226,10 @@
         <v>36</v>
       </c>
       <c r="C59" t="s">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="D59" t="s">
-        <v>270</v>
+        <v>272</v>
       </c>
       <c r="E59">
         <v>2</v>
@@ -3211,33 +3237,33 @@
     </row>
     <row r="60" spans="1:5">
       <c r="A60" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B60" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="C60" t="s">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="D60" t="s">
-        <v>270</v>
+        <v>272</v>
       </c>
       <c r="E60">
-        <v>1</v>
+        <v>4</v>
       </c>
     </row>
     <row r="61" spans="1:5">
       <c r="A61" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="B61" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="C61" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="D61" t="s">
-        <v>271</v>
+        <v>272</v>
       </c>
       <c r="E61">
         <v>2</v>
@@ -3251,10 +3277,10 @@
         <v>36</v>
       </c>
       <c r="C62" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="D62" t="s">
-        <v>272</v>
+        <v>273</v>
       </c>
       <c r="E62">
         <v>2</v>
@@ -3262,10 +3288,10 @@
     </row>
     <row r="63" spans="1:5">
       <c r="A63" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="B63" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="C63" t="s">
         <v>91</v>
@@ -3274,7 +3300,7 @@
         <v>273</v>
       </c>
       <c r="E63">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="64" spans="1:5">
@@ -3356,7 +3382,7 @@
         <v>96</v>
       </c>
       <c r="D68" t="s">
-        <v>267</v>
+        <v>278</v>
       </c>
       <c r="E68">
         <v>2</v>
@@ -3373,27 +3399,27 @@
         <v>97</v>
       </c>
       <c r="D69" t="s">
-        <v>266</v>
+        <v>279</v>
       </c>
       <c r="E69">
-        <v>4</v>
+        <v>2</v>
       </c>
     </row>
     <row r="70" spans="1:5">
       <c r="A70" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="B70" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
       <c r="C70" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="D70" t="s">
-        <v>266</v>
+        <v>280</v>
       </c>
       <c r="E70">
-        <v>4</v>
+        <v>2</v>
       </c>
     </row>
     <row r="71" spans="1:5">
@@ -3404,13 +3430,13 @@
         <v>36</v>
       </c>
       <c r="C71" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="D71" t="s">
-        <v>278</v>
+        <v>270</v>
       </c>
       <c r="E71">
-        <v>4</v>
+        <v>2</v>
       </c>
     </row>
     <row r="72" spans="1:5">
@@ -3421,10 +3447,10 @@
         <v>36</v>
       </c>
       <c r="C72" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="D72" t="s">
-        <v>279</v>
+        <v>269</v>
       </c>
       <c r="E72">
         <v>4</v>
@@ -3432,16 +3458,16 @@
     </row>
     <row r="73" spans="1:5">
       <c r="A73" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="B73" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="C73" t="s">
         <v>100</v>
       </c>
       <c r="D73" t="s">
-        <v>280</v>
+        <v>269</v>
       </c>
       <c r="E73">
         <v>4</v>
@@ -3449,10 +3475,10 @@
     </row>
     <row r="74" spans="1:5">
       <c r="A74" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B74" t="s">
-        <v>39</v>
+        <v>36</v>
       </c>
       <c r="C74" t="s">
         <v>101</v>
@@ -3461,41 +3487,41 @@
         <v>281</v>
       </c>
       <c r="E74">
-        <v>1</v>
+        <v>4</v>
       </c>
     </row>
     <row r="75" spans="1:5">
       <c r="A75" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="B75" t="s">
-        <v>39</v>
+        <v>36</v>
       </c>
       <c r="C75" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="D75" t="s">
-        <v>281</v>
+        <v>282</v>
       </c>
       <c r="E75">
-        <v>1</v>
+        <v>4</v>
       </c>
     </row>
     <row r="76" spans="1:5">
       <c r="A76" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="B76" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
       <c r="C76" t="s">
-        <v>101</v>
+        <v>103</v>
       </c>
       <c r="D76" t="s">
-        <v>281</v>
+        <v>283</v>
       </c>
       <c r="E76">
-        <v>1</v>
+        <v>4</v>
       </c>
     </row>
     <row r="77" spans="1:5">
@@ -3506,10 +3532,10 @@
         <v>39</v>
       </c>
       <c r="C77" t="s">
-        <v>102</v>
+        <v>104</v>
       </c>
       <c r="D77" t="s">
-        <v>282</v>
+        <v>284</v>
       </c>
       <c r="E77">
         <v>1</v>
@@ -3523,10 +3549,10 @@
         <v>39</v>
       </c>
       <c r="C78" t="s">
-        <v>102</v>
+        <v>104</v>
       </c>
       <c r="D78" t="s">
-        <v>282</v>
+        <v>284</v>
       </c>
       <c r="E78">
         <v>1</v>
@@ -3540,13 +3566,13 @@
         <v>38</v>
       </c>
       <c r="C79" t="s">
-        <v>102</v>
+        <v>104</v>
       </c>
       <c r="D79" t="s">
-        <v>282</v>
+        <v>284</v>
       </c>
       <c r="E79">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="80" spans="1:5">
@@ -3557,10 +3583,10 @@
         <v>39</v>
       </c>
       <c r="C80" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="D80" t="s">
-        <v>283</v>
+        <v>285</v>
       </c>
       <c r="E80">
         <v>1</v>
@@ -3574,10 +3600,10 @@
         <v>39</v>
       </c>
       <c r="C81" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="D81" t="s">
-        <v>283</v>
+        <v>285</v>
       </c>
       <c r="E81">
         <v>1</v>
@@ -3585,33 +3611,33 @@
     </row>
     <row r="82" spans="1:5">
       <c r="A82" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="B82" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="C82" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="D82" t="s">
-        <v>284</v>
+        <v>285</v>
       </c>
       <c r="E82">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="83" spans="1:5">
       <c r="A83" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B83" t="s">
         <v>39</v>
       </c>
       <c r="C83" t="s">
-        <v>104</v>
+        <v>106</v>
       </c>
       <c r="D83" t="s">
-        <v>284</v>
+        <v>286</v>
       </c>
       <c r="E83">
         <v>1</v>
@@ -3619,16 +3645,16 @@
     </row>
     <row r="84" spans="1:5">
       <c r="A84" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="B84" t="s">
         <v>39</v>
       </c>
       <c r="C84" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="D84" t="s">
-        <v>285</v>
+        <v>286</v>
       </c>
       <c r="E84">
         <v>1</v>
@@ -3636,16 +3662,16 @@
     </row>
     <row r="85" spans="1:5">
       <c r="A85" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B85" t="s">
         <v>39</v>
       </c>
       <c r="C85" t="s">
-        <v>105</v>
+        <v>107</v>
       </c>
       <c r="D85" t="s">
-        <v>285</v>
+        <v>287</v>
       </c>
       <c r="E85">
         <v>1</v>
@@ -3653,16 +3679,16 @@
     </row>
     <row r="86" spans="1:5">
       <c r="A86" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="B86" t="s">
         <v>39</v>
       </c>
       <c r="C86" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="D86" t="s">
-        <v>286</v>
+        <v>287</v>
       </c>
       <c r="E86">
         <v>1</v>
@@ -3670,16 +3696,16 @@
     </row>
     <row r="87" spans="1:5">
       <c r="A87" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B87" t="s">
         <v>39</v>
       </c>
       <c r="C87" t="s">
-        <v>106</v>
+        <v>108</v>
       </c>
       <c r="D87" t="s">
-        <v>286</v>
+        <v>288</v>
       </c>
       <c r="E87">
         <v>1</v>
@@ -3687,16 +3713,16 @@
     </row>
     <row r="88" spans="1:5">
       <c r="A88" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="B88" t="s">
         <v>39</v>
       </c>
       <c r="C88" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="D88" t="s">
-        <v>287</v>
+        <v>288</v>
       </c>
       <c r="E88">
         <v>1</v>
@@ -3704,16 +3730,16 @@
     </row>
     <row r="89" spans="1:5">
       <c r="A89" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B89" t="s">
         <v>39</v>
       </c>
       <c r="C89" t="s">
-        <v>107</v>
+        <v>109</v>
       </c>
       <c r="D89" t="s">
-        <v>287</v>
+        <v>289</v>
       </c>
       <c r="E89">
         <v>1</v>
@@ -3721,16 +3747,16 @@
     </row>
     <row r="90" spans="1:5">
       <c r="A90" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="B90" t="s">
         <v>39</v>
       </c>
       <c r="C90" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="D90" t="s">
-        <v>288</v>
+        <v>289</v>
       </c>
       <c r="E90">
         <v>1</v>
@@ -3738,16 +3764,16 @@
     </row>
     <row r="91" spans="1:5">
       <c r="A91" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B91" t="s">
         <v>39</v>
       </c>
       <c r="C91" t="s">
-        <v>108</v>
+        <v>110</v>
       </c>
       <c r="D91" t="s">
-        <v>288</v>
+        <v>290</v>
       </c>
       <c r="E91">
         <v>1</v>
@@ -3755,16 +3781,16 @@
     </row>
     <row r="92" spans="1:5">
       <c r="A92" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="B92" t="s">
         <v>39</v>
       </c>
       <c r="C92" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="D92" t="s">
-        <v>289</v>
+        <v>290</v>
       </c>
       <c r="E92">
         <v>1</v>
@@ -3772,16 +3798,16 @@
     </row>
     <row r="93" spans="1:5">
       <c r="A93" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B93" t="s">
         <v>39</v>
       </c>
       <c r="C93" t="s">
-        <v>109</v>
+        <v>111</v>
       </c>
       <c r="D93" t="s">
-        <v>289</v>
+        <v>291</v>
       </c>
       <c r="E93">
         <v>1</v>
@@ -3789,16 +3815,16 @@
     </row>
     <row r="94" spans="1:5">
       <c r="A94" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="B94" t="s">
         <v>39</v>
       </c>
       <c r="C94" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="D94" t="s">
-        <v>290</v>
+        <v>291</v>
       </c>
       <c r="E94">
         <v>1</v>
@@ -3806,16 +3832,16 @@
     </row>
     <row r="95" spans="1:5">
       <c r="A95" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="B95" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="C95" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="D95" t="s">
-        <v>290</v>
+        <v>292</v>
       </c>
       <c r="E95">
         <v>1</v>
@@ -3823,16 +3849,16 @@
     </row>
     <row r="96" spans="1:5">
       <c r="A96" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="B96" t="s">
         <v>39</v>
       </c>
       <c r="C96" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="D96" t="s">
-        <v>291</v>
+        <v>292</v>
       </c>
       <c r="E96">
         <v>1</v>
@@ -3840,16 +3866,16 @@
     </row>
     <row r="97" spans="1:5">
       <c r="A97" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="B97" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="C97" t="s">
-        <v>111</v>
+        <v>113</v>
       </c>
       <c r="D97" t="s">
-        <v>291</v>
+        <v>293</v>
       </c>
       <c r="E97">
         <v>1</v>
@@ -3857,16 +3883,16 @@
     </row>
     <row r="98" spans="1:5">
       <c r="A98" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="B98" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="C98" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="D98" t="s">
-        <v>292</v>
+        <v>293</v>
       </c>
       <c r="E98">
         <v>1</v>
@@ -3874,16 +3900,16 @@
     </row>
     <row r="99" spans="1:5">
       <c r="A99" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="B99" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="C99" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
       <c r="D99" t="s">
-        <v>292</v>
+        <v>294</v>
       </c>
       <c r="E99">
         <v>1</v>
@@ -3891,16 +3917,16 @@
     </row>
     <row r="100" spans="1:5">
       <c r="A100" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="B100" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="C100" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="D100" t="s">
-        <v>293</v>
+        <v>294</v>
       </c>
       <c r="E100">
         <v>1</v>
@@ -3914,10 +3940,10 @@
         <v>39</v>
       </c>
       <c r="C101" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="D101" t="s">
-        <v>294</v>
+        <v>295</v>
       </c>
       <c r="E101">
         <v>1</v>
@@ -3925,10 +3951,10 @@
     </row>
     <row r="102" spans="1:5">
       <c r="A102" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="B102" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="C102" t="s">
         <v>115</v>
@@ -4005,21 +4031,21 @@
         <v>299</v>
       </c>
       <c r="E106">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="107" spans="1:5">
       <c r="A107" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B107" t="s">
         <v>39</v>
       </c>
       <c r="C107" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="D107" t="s">
-        <v>299</v>
+        <v>300</v>
       </c>
       <c r="E107">
         <v>1</v>
@@ -4033,27 +4059,27 @@
         <v>39</v>
       </c>
       <c r="C108" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="D108" t="s">
-        <v>300</v>
+        <v>301</v>
       </c>
       <c r="E108">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="109" spans="1:5">
       <c r="A109" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B109" t="s">
         <v>39</v>
       </c>
       <c r="C109" t="s">
-        <v>120</v>
+        <v>122</v>
       </c>
       <c r="D109" t="s">
-        <v>300</v>
+        <v>302</v>
       </c>
       <c r="E109">
         <v>2</v>
@@ -4061,19 +4087,19 @@
     </row>
     <row r="110" spans="1:5">
       <c r="A110" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B110" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="C110" t="s">
-        <v>120</v>
+        <v>122</v>
       </c>
       <c r="D110" t="s">
-        <v>300</v>
+        <v>302</v>
       </c>
       <c r="E110">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="111" spans="1:5">
@@ -4084,10 +4110,10 @@
         <v>39</v>
       </c>
       <c r="C111" t="s">
-        <v>121</v>
+        <v>123</v>
       </c>
       <c r="D111" t="s">
-        <v>301</v>
+        <v>303</v>
       </c>
       <c r="E111">
         <v>2</v>
@@ -4101,10 +4127,10 @@
         <v>39</v>
       </c>
       <c r="C112" t="s">
-        <v>121</v>
+        <v>123</v>
       </c>
       <c r="D112" t="s">
-        <v>301</v>
+        <v>303</v>
       </c>
       <c r="E112">
         <v>2</v>
@@ -4118,10 +4144,10 @@
         <v>38</v>
       </c>
       <c r="C113" t="s">
-        <v>121</v>
+        <v>123</v>
       </c>
       <c r="D113" t="s">
-        <v>301</v>
+        <v>303</v>
       </c>
       <c r="E113">
         <v>2</v>
@@ -4135,10 +4161,10 @@
         <v>39</v>
       </c>
       <c r="C114" t="s">
-        <v>122</v>
+        <v>124</v>
       </c>
       <c r="D114" t="s">
-        <v>302</v>
+        <v>304</v>
       </c>
       <c r="E114">
         <v>2</v>
@@ -4152,10 +4178,10 @@
         <v>39</v>
       </c>
       <c r="C115" t="s">
-        <v>122</v>
+        <v>124</v>
       </c>
       <c r="D115" t="s">
-        <v>302</v>
+        <v>304</v>
       </c>
       <c r="E115">
         <v>2</v>
@@ -4163,16 +4189,16 @@
     </row>
     <row r="116" spans="1:5">
       <c r="A116" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="B116" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="C116" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="D116" t="s">
-        <v>303</v>
+        <v>304</v>
       </c>
       <c r="E116">
         <v>2</v>
@@ -4180,16 +4206,16 @@
     </row>
     <row r="117" spans="1:5">
       <c r="A117" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B117" t="s">
         <v>39</v>
       </c>
       <c r="C117" t="s">
-        <v>123</v>
+        <v>125</v>
       </c>
       <c r="D117" t="s">
-        <v>303</v>
+        <v>305</v>
       </c>
       <c r="E117">
         <v>2</v>
@@ -4197,16 +4223,16 @@
     </row>
     <row r="118" spans="1:5">
       <c r="A118" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="B118" t="s">
         <v>39</v>
       </c>
       <c r="C118" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="D118" t="s">
-        <v>282</v>
+        <v>305</v>
       </c>
       <c r="E118">
         <v>2</v>
@@ -4214,36 +4240,36 @@
     </row>
     <row r="119" spans="1:5">
       <c r="A119" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B119" t="s">
         <v>39</v>
       </c>
       <c r="C119" t="s">
-        <v>124</v>
+        <v>126</v>
       </c>
       <c r="D119" t="s">
-        <v>282</v>
+        <v>306</v>
       </c>
       <c r="E119">
-        <v>4</v>
+        <v>2</v>
       </c>
     </row>
     <row r="120" spans="1:5">
       <c r="A120" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B120" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="C120" t="s">
-        <v>124</v>
+        <v>126</v>
       </c>
       <c r="D120" t="s">
-        <v>282</v>
+        <v>306</v>
       </c>
       <c r="E120">
-        <v>4</v>
+        <v>2</v>
       </c>
     </row>
     <row r="121" spans="1:5">
@@ -4254,10 +4280,10 @@
         <v>39</v>
       </c>
       <c r="C121" t="s">
-        <v>125</v>
+        <v>127</v>
       </c>
       <c r="D121" t="s">
-        <v>304</v>
+        <v>285</v>
       </c>
       <c r="E121">
         <v>2</v>
@@ -4271,10 +4297,10 @@
         <v>39</v>
       </c>
       <c r="C122" t="s">
-        <v>125</v>
+        <v>127</v>
       </c>
       <c r="D122" t="s">
-        <v>304</v>
+        <v>285</v>
       </c>
       <c r="E122">
         <v>4</v>
@@ -4282,19 +4308,19 @@
     </row>
     <row r="123" spans="1:5">
       <c r="A123" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="B123" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="C123" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="D123" t="s">
-        <v>288</v>
+        <v>285</v>
       </c>
       <c r="E123">
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
     <row r="124" spans="1:5">
@@ -4305,10 +4331,10 @@
         <v>39</v>
       </c>
       <c r="C124" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="D124" t="s">
-        <v>305</v>
+        <v>307</v>
       </c>
       <c r="E124">
         <v>2</v>
@@ -4316,7 +4342,7 @@
     </row>
     <row r="125" spans="1:5">
       <c r="A125" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="B125" t="s">
         <v>39</v>
@@ -4325,10 +4351,10 @@
         <v>128</v>
       </c>
       <c r="D125" t="s">
-        <v>306</v>
+        <v>307</v>
       </c>
       <c r="E125">
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
     <row r="126" spans="1:5">
@@ -4342,27 +4368,27 @@
         <v>129</v>
       </c>
       <c r="D126" t="s">
-        <v>307</v>
+        <v>291</v>
       </c>
       <c r="E126">
-        <v>5</v>
+        <v>2</v>
       </c>
     </row>
     <row r="127" spans="1:5">
       <c r="A127" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B127" t="s">
         <v>39</v>
       </c>
       <c r="C127" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="D127" t="s">
-        <v>307</v>
+        <v>308</v>
       </c>
       <c r="E127">
-        <v>5</v>
+        <v>2</v>
       </c>
     </row>
     <row r="128" spans="1:5">
@@ -4373,13 +4399,13 @@
         <v>39</v>
       </c>
       <c r="C128" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="D128" t="s">
-        <v>308</v>
+        <v>309</v>
       </c>
       <c r="E128">
-        <v>7</v>
+        <v>2</v>
       </c>
     </row>
     <row r="129" spans="1:5">
@@ -4390,18 +4416,18 @@
         <v>39</v>
       </c>
       <c r="C129" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="D129" t="s">
-        <v>309</v>
+        <v>310</v>
       </c>
       <c r="E129">
-        <v>10</v>
+        <v>5</v>
       </c>
     </row>
     <row r="130" spans="1:5">
       <c r="A130" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="B130" t="s">
         <v>39</v>
@@ -4413,58 +4439,58 @@
         <v>310</v>
       </c>
       <c r="E130">
-        <v>30</v>
+        <v>5</v>
       </c>
     </row>
     <row r="131" spans="1:5">
       <c r="A131" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B131" t="s">
         <v>39</v>
       </c>
       <c r="C131" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="D131" t="s">
-        <v>310</v>
+        <v>311</v>
       </c>
       <c r="E131">
-        <v>30</v>
+        <v>7</v>
       </c>
     </row>
     <row r="132" spans="1:5">
       <c r="A132" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B132" t="s">
         <v>39</v>
       </c>
       <c r="C132" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="D132" t="s">
-        <v>311</v>
+        <v>312</v>
       </c>
       <c r="E132">
-        <v>1</v>
+        <v>10</v>
       </c>
     </row>
     <row r="133" spans="1:5">
       <c r="A133" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="B133" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="C133" t="s">
-        <v>133</v>
+        <v>135</v>
       </c>
       <c r="D133" t="s">
-        <v>311</v>
+        <v>313</v>
       </c>
       <c r="E133">
-        <v>1</v>
+        <v>30</v>
       </c>
     </row>
     <row r="134" spans="1:5">
@@ -4475,13 +4501,13 @@
         <v>39</v>
       </c>
       <c r="C134" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="D134" t="s">
-        <v>312</v>
+        <v>313</v>
       </c>
       <c r="E134">
-        <v>1</v>
+        <v>30</v>
       </c>
     </row>
     <row r="135" spans="1:5">
@@ -4492,10 +4518,10 @@
         <v>39</v>
       </c>
       <c r="C135" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="D135" t="s">
-        <v>313</v>
+        <v>314</v>
       </c>
       <c r="E135">
         <v>1</v>
@@ -4503,10 +4529,10 @@
     </row>
     <row r="136" spans="1:5">
       <c r="A136" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="B136" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="C136" t="s">
         <v>136</v>
@@ -4988,10 +5014,10 @@
         <v>164</v>
       </c>
       <c r="D164" t="s">
-        <v>326</v>
+        <v>342</v>
       </c>
       <c r="E164">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="165" spans="1:5">
@@ -5005,10 +5031,10 @@
         <v>165</v>
       </c>
       <c r="D165" t="s">
-        <v>342</v>
+        <v>343</v>
       </c>
       <c r="E165">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="166" spans="1:5">
@@ -5022,10 +5048,10 @@
         <v>166</v>
       </c>
       <c r="D166" t="s">
-        <v>343</v>
+        <v>344</v>
       </c>
       <c r="E166">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="167" spans="1:5">
@@ -5039,7 +5065,7 @@
         <v>167</v>
       </c>
       <c r="D167" t="s">
-        <v>344</v>
+        <v>329</v>
       </c>
       <c r="E167">
         <v>2</v>
@@ -5076,7 +5102,7 @@
         <v>346</v>
       </c>
       <c r="E169">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="170" spans="1:5">
@@ -5090,10 +5116,10 @@
         <v>170</v>
       </c>
       <c r="D170" t="s">
-        <v>310</v>
+        <v>347</v>
       </c>
       <c r="E170">
-        <v>5</v>
+        <v>2</v>
       </c>
     </row>
     <row r="171" spans="1:5">
@@ -5107,10 +5133,10 @@
         <v>171</v>
       </c>
       <c r="D171" t="s">
-        <v>347</v>
+        <v>348</v>
       </c>
       <c r="E171">
-        <v>8</v>
+        <v>2</v>
       </c>
     </row>
     <row r="172" spans="1:5">
@@ -5124,10 +5150,10 @@
         <v>172</v>
       </c>
       <c r="D172" t="s">
-        <v>263</v>
+        <v>349</v>
       </c>
       <c r="E172">
-        <v>8</v>
+        <v>3</v>
       </c>
     </row>
     <row r="173" spans="1:5">
@@ -5141,10 +5167,10 @@
         <v>173</v>
       </c>
       <c r="D173" t="s">
-        <v>348</v>
+        <v>313</v>
       </c>
       <c r="E173">
-        <v>10</v>
+        <v>5</v>
       </c>
     </row>
     <row r="174" spans="1:5">
@@ -5158,10 +5184,10 @@
         <v>174</v>
       </c>
       <c r="D174" t="s">
-        <v>349</v>
+        <v>350</v>
       </c>
       <c r="E174">
-        <v>1</v>
+        <v>8</v>
       </c>
     </row>
     <row r="175" spans="1:5">
@@ -5175,41 +5201,41 @@
         <v>175</v>
       </c>
       <c r="D175" t="s">
-        <v>350</v>
+        <v>266</v>
       </c>
       <c r="E175">
-        <v>1</v>
+        <v>8</v>
       </c>
     </row>
     <row r="176" spans="1:5">
       <c r="A176" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B176" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="C176" t="s">
         <v>176</v>
       </c>
       <c r="D176" t="s">
-        <v>336</v>
+        <v>351</v>
       </c>
       <c r="E176">
-        <v>1</v>
+        <v>10</v>
       </c>
     </row>
     <row r="177" spans="1:5">
       <c r="A177" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B177" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="C177" t="s">
         <v>177</v>
       </c>
       <c r="D177" t="s">
-        <v>351</v>
+        <v>352</v>
       </c>
       <c r="E177">
         <v>1</v>
@@ -5217,16 +5243,16 @@
     </row>
     <row r="178" spans="1:5">
       <c r="A178" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B178" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="C178" t="s">
         <v>178</v>
       </c>
       <c r="D178" t="s">
-        <v>352</v>
+        <v>353</v>
       </c>
       <c r="E178">
         <v>1</v>
@@ -5243,7 +5269,7 @@
         <v>179</v>
       </c>
       <c r="D179" t="s">
-        <v>353</v>
+        <v>339</v>
       </c>
       <c r="E179">
         <v>1</v>
@@ -5294,7 +5320,7 @@
         <v>182</v>
       </c>
       <c r="D182" t="s">
-        <v>273</v>
+        <v>356</v>
       </c>
       <c r="E182">
         <v>1</v>
@@ -5311,7 +5337,7 @@
         <v>183</v>
       </c>
       <c r="D183" t="s">
-        <v>356</v>
+        <v>357</v>
       </c>
       <c r="E183">
         <v>1</v>
@@ -5328,7 +5354,7 @@
         <v>184</v>
       </c>
       <c r="D184" t="s">
-        <v>357</v>
+        <v>358</v>
       </c>
       <c r="E184">
         <v>1</v>
@@ -5345,7 +5371,7 @@
         <v>185</v>
       </c>
       <c r="D185" t="s">
-        <v>358</v>
+        <v>276</v>
       </c>
       <c r="E185">
         <v>1</v>
@@ -5739,7 +5765,7 @@
         <v>381</v>
       </c>
       <c r="E208">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="209" spans="1:5">
@@ -5756,7 +5782,7 @@
         <v>382</v>
       </c>
       <c r="E209">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="210" spans="1:5">
@@ -5773,7 +5799,7 @@
         <v>383</v>
       </c>
       <c r="E210">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="211" spans="1:5">
@@ -5872,7 +5898,7 @@
         <v>216</v>
       </c>
       <c r="D216" t="s">
-        <v>388</v>
+        <v>389</v>
       </c>
       <c r="E216">
         <v>2</v>
@@ -5889,7 +5915,7 @@
         <v>217</v>
       </c>
       <c r="D217" t="s">
-        <v>389</v>
+        <v>390</v>
       </c>
       <c r="E217">
         <v>2</v>
@@ -5906,7 +5932,7 @@
         <v>218</v>
       </c>
       <c r="D218" t="s">
-        <v>390</v>
+        <v>391</v>
       </c>
       <c r="E218">
         <v>2</v>
@@ -5926,7 +5952,7 @@
         <v>391</v>
       </c>
       <c r="E219">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="220" spans="1:5">
@@ -5940,10 +5966,10 @@
         <v>220</v>
       </c>
       <c r="D220" t="s">
-        <v>273</v>
+        <v>392</v>
       </c>
       <c r="E220">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="221" spans="1:5">
@@ -5957,10 +5983,10 @@
         <v>221</v>
       </c>
       <c r="D221" t="s">
-        <v>392</v>
+        <v>393</v>
       </c>
       <c r="E221">
-        <v>4</v>
+        <v>2</v>
       </c>
     </row>
     <row r="222" spans="1:5">
@@ -5974,10 +6000,10 @@
         <v>222</v>
       </c>
       <c r="D222" t="s">
-        <v>393</v>
+        <v>394</v>
       </c>
       <c r="E222">
-        <v>4</v>
+        <v>3</v>
       </c>
     </row>
     <row r="223" spans="1:5">
@@ -5991,10 +6017,10 @@
         <v>223</v>
       </c>
       <c r="D223" t="s">
-        <v>394</v>
+        <v>276</v>
       </c>
       <c r="E223">
-        <v>4</v>
+        <v>3</v>
       </c>
     </row>
     <row r="224" spans="1:5">
@@ -6045,7 +6071,7 @@
         <v>397</v>
       </c>
       <c r="E226">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="227" spans="1:5">
@@ -6062,7 +6088,7 @@
         <v>398</v>
       </c>
       <c r="E227">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="228" spans="1:5">
@@ -6079,7 +6105,7 @@
         <v>399</v>
       </c>
       <c r="E228">
-        <v>6</v>
+        <v>4</v>
       </c>
     </row>
     <row r="229" spans="1:5">
@@ -6096,7 +6122,7 @@
         <v>400</v>
       </c>
       <c r="E229">
-        <v>8</v>
+        <v>5</v>
       </c>
     </row>
     <row r="230" spans="1:5">
@@ -6113,7 +6139,7 @@
         <v>401</v>
       </c>
       <c r="E230">
-        <v>10</v>
+        <v>5</v>
       </c>
     </row>
     <row r="231" spans="1:5">
@@ -6127,10 +6153,10 @@
         <v>231</v>
       </c>
       <c r="D231" t="s">
-        <v>401</v>
+        <v>402</v>
       </c>
       <c r="E231">
-        <v>10</v>
+        <v>6</v>
       </c>
     </row>
     <row r="232" spans="1:5">
@@ -6144,10 +6170,10 @@
         <v>232</v>
       </c>
       <c r="D232" t="s">
-        <v>275</v>
+        <v>403</v>
       </c>
       <c r="E232">
-        <v>12</v>
+        <v>8</v>
       </c>
     </row>
     <row r="233" spans="1:5">
@@ -6161,10 +6187,10 @@
         <v>233</v>
       </c>
       <c r="D233" t="s">
-        <v>402</v>
+        <v>404</v>
       </c>
       <c r="E233">
-        <v>12</v>
+        <v>10</v>
       </c>
     </row>
     <row r="234" spans="1:5">
@@ -6178,10 +6204,10 @@
         <v>234</v>
       </c>
       <c r="D234" t="s">
-        <v>403</v>
+        <v>404</v>
       </c>
       <c r="E234">
-        <v>14</v>
+        <v>10</v>
       </c>
     </row>
     <row r="235" spans="1:5">
@@ -6195,10 +6221,10 @@
         <v>235</v>
       </c>
       <c r="D235" t="s">
-        <v>404</v>
+        <v>278</v>
       </c>
       <c r="E235">
-        <v>15</v>
+        <v>12</v>
       </c>
     </row>
     <row r="236" spans="1:5">
@@ -6215,15 +6241,15 @@
         <v>405</v>
       </c>
       <c r="E236">
-        <v>20</v>
+        <v>12</v>
       </c>
     </row>
     <row r="237" spans="1:5">
       <c r="A237" t="s">
-        <v>7</v>
+        <v>14</v>
       </c>
       <c r="B237" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="C237" t="s">
         <v>237</v>
@@ -6232,15 +6258,15 @@
         <v>406</v>
       </c>
       <c r="E237">
-        <v>1</v>
+        <v>14</v>
       </c>
     </row>
     <row r="238" spans="1:5">
       <c r="A238" t="s">
-        <v>7</v>
+        <v>14</v>
       </c>
       <c r="B238" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="C238" t="s">
         <v>238</v>
@@ -6249,15 +6275,15 @@
         <v>407</v>
       </c>
       <c r="E238">
-        <v>4</v>
+        <v>15</v>
       </c>
     </row>
     <row r="239" spans="1:5">
       <c r="A239" t="s">
-        <v>7</v>
+        <v>14</v>
       </c>
       <c r="B239" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="C239" t="s">
         <v>239</v>
@@ -6266,7 +6292,7 @@
         <v>408</v>
       </c>
       <c r="E239">
-        <v>4</v>
+        <v>20</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Atualização automática: rac (06/10/2026 14:09)
</commit_message>
<xml_diff>
--- a/Coordenadoria/02_Dados_Tratados/base_rac_tratada.xlsx
+++ b/Coordenadoria/02_Dados_Tratados/base_rac_tratada.xlsx
@@ -1212,16 +1212,8 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <fonts count="2">
+  <fonts count="1">
     <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -1237,7 +1229,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -1245,30 +1237,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color auto="1"/>
-      </left>
-      <right style="thin">
-        <color auto="1"/>
-      </right>
-      <top style="thin">
-        <color auto="1"/>
-      </top>
-      <bottom style="thin">
-        <color auto="1"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1567,22 +1541,22 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:6">
-      <c r="A1" s="1" t="s">
+      <c r="A1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" s="1" t="s">
+      <c r="B1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" t="s">
         <v>5</v>
       </c>
     </row>
@@ -2197,19 +2171,19 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:5">
-      <c r="A1" s="1" t="s">
+      <c r="A1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" s="1" t="s">
+      <c r="B1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" t="s">
         <v>55</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" t="s">
         <v>56</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" t="s">
         <v>57</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualização automática: rac (07/10/2026 14:46)
</commit_message>
<xml_diff>
--- a/Coordenadoria/02_Dados_Tratados/base_rac_tratada.xlsx
+++ b/Coordenadoria/02_Dados_Tratados/base_rac_tratada.xlsx
@@ -1230,16 +1230,8 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <fonts count="2">
+  <fonts count="1">
     <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -1255,7 +1247,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -1263,30 +1255,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color auto="1"/>
-      </left>
-      <right style="thin">
-        <color auto="1"/>
-      </right>
-      <top style="thin">
-        <color auto="1"/>
-      </top>
-      <bottom style="thin">
-        <color auto="1"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1585,22 +1559,22 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:6">
-      <c r="A1" s="1" t="s">
+      <c r="A1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" s="1" t="s">
+      <c r="B1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" t="s">
         <v>5</v>
       </c>
     </row>
@@ -2215,19 +2189,19 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:5">
-      <c r="A1" s="1" t="s">
+      <c r="A1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" s="1" t="s">
+      <c r="B1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" t="s">
         <v>55</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" t="s">
         <v>56</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" t="s">
         <v>57</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualização automática: rac (08/10/2026 14:50)
</commit_message>
<xml_diff>
--- a/Coordenadoria/02_Dados_Tratados/base_rac_tratada.xlsx
+++ b/Coordenadoria/02_Dados_Tratados/base_rac_tratada.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1075" uniqueCount="403">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1071" uniqueCount="401">
   <si>
     <t>matricula</t>
   </si>
@@ -200,9 +200,6 @@
     <t>P7036368-01</t>
   </si>
   <si>
-    <t>066-3046-07</t>
-  </si>
-  <si>
     <t>200SGL153Q</t>
   </si>
   <si>
@@ -735,9 +732,6 @@
   </si>
   <si>
     <t>PROPELLER ASSEMBLY</t>
-  </si>
-  <si>
-    <t>CONTROL,INDICATOR</t>
   </si>
   <si>
     <t>STARTER GENERATOR</t>
@@ -1612,10 +1606,10 @@
         <v>53</v>
       </c>
       <c r="E3">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F3">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="4" spans="1:6">
@@ -2185,7 +2179,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E237"/>
+  <dimension ref="A1:E236"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:5">
@@ -2216,7 +2210,7 @@
         <v>58</v>
       </c>
       <c r="D2" t="s">
-        <v>237</v>
+        <v>236</v>
       </c>
       <c r="E2">
         <v>1</v>
@@ -2233,7 +2227,7 @@
         <v>58</v>
       </c>
       <c r="D3" t="s">
-        <v>237</v>
+        <v>236</v>
       </c>
       <c r="E3">
         <v>1</v>
@@ -2250,7 +2244,7 @@
         <v>59</v>
       </c>
       <c r="D4" t="s">
-        <v>238</v>
+        <v>237</v>
       </c>
       <c r="E4">
         <v>1</v>
@@ -2267,7 +2261,7 @@
         <v>60</v>
       </c>
       <c r="D5" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
       <c r="E5">
         <v>1</v>
@@ -2284,7 +2278,7 @@
         <v>60</v>
       </c>
       <c r="D6" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
       <c r="E6">
         <v>1</v>
@@ -2301,7 +2295,7 @@
         <v>60</v>
       </c>
       <c r="D7" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
       <c r="E7">
         <v>1</v>
@@ -2318,7 +2312,7 @@
         <v>60</v>
       </c>
       <c r="D8" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
       <c r="E8">
         <v>1</v>
@@ -2335,7 +2329,7 @@
         <v>60</v>
       </c>
       <c r="D9" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
       <c r="E9">
         <v>1</v>
@@ -2352,7 +2346,7 @@
         <v>60</v>
       </c>
       <c r="D10" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
       <c r="E10">
         <v>1</v>
@@ -2369,7 +2363,7 @@
         <v>60</v>
       </c>
       <c r="D11" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
       <c r="E11">
         <v>1</v>
@@ -2386,7 +2380,7 @@
         <v>61</v>
       </c>
       <c r="D12" t="s">
-        <v>240</v>
+        <v>239</v>
       </c>
       <c r="E12">
         <v>1</v>
@@ -2394,16 +2388,16 @@
     </row>
     <row r="13" spans="1:5">
       <c r="A13" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="B13" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="C13" t="s">
         <v>62</v>
       </c>
       <c r="D13" t="s">
-        <v>241</v>
+        <v>240</v>
       </c>
       <c r="E13">
         <v>1</v>
@@ -2411,16 +2405,16 @@
     </row>
     <row r="14" spans="1:5">
       <c r="A14" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="B14" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="C14" t="s">
         <v>63</v>
       </c>
       <c r="D14" t="s">
-        <v>242</v>
+        <v>241</v>
       </c>
       <c r="E14">
         <v>1</v>
@@ -2437,7 +2431,7 @@
         <v>64</v>
       </c>
       <c r="D15" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
       <c r="E15">
         <v>1</v>
@@ -2454,7 +2448,7 @@
         <v>65</v>
       </c>
       <c r="D16" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="E16">
         <v>1</v>
@@ -2471,7 +2465,7 @@
         <v>66</v>
       </c>
       <c r="D17" t="s">
-        <v>245</v>
+        <v>244</v>
       </c>
       <c r="E17">
         <v>1</v>
@@ -2488,7 +2482,7 @@
         <v>67</v>
       </c>
       <c r="D18" t="s">
-        <v>246</v>
+        <v>245</v>
       </c>
       <c r="E18">
         <v>1</v>
@@ -2496,16 +2490,16 @@
     </row>
     <row r="19" spans="1:5">
       <c r="A19" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="B19" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="C19" t="s">
         <v>68</v>
       </c>
       <c r="D19" t="s">
-        <v>247</v>
+        <v>246</v>
       </c>
       <c r="E19">
         <v>1</v>
@@ -2513,16 +2507,16 @@
     </row>
     <row r="20" spans="1:5">
       <c r="A20" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="B20" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="C20" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="D20" t="s">
-        <v>248</v>
+        <v>246</v>
       </c>
       <c r="E20">
         <v>1</v>
@@ -2530,16 +2524,16 @@
     </row>
     <row r="21" spans="1:5">
       <c r="A21" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B21" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="C21" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="D21" t="s">
-        <v>248</v>
+        <v>246</v>
       </c>
       <c r="E21">
         <v>1</v>
@@ -2547,16 +2541,16 @@
     </row>
     <row r="22" spans="1:5">
       <c r="A22" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="B22" t="s">
         <v>40</v>
       </c>
       <c r="C22" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="D22" t="s">
-        <v>248</v>
+        <v>246</v>
       </c>
       <c r="E22">
         <v>1</v>
@@ -2564,16 +2558,16 @@
     </row>
     <row r="23" spans="1:5">
       <c r="A23" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="B23" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="C23" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="D23" t="s">
-        <v>248</v>
+        <v>246</v>
       </c>
       <c r="E23">
         <v>1</v>
@@ -2581,16 +2575,16 @@
     </row>
     <row r="24" spans="1:5">
       <c r="A24" t="s">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="B24" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="C24" t="s">
         <v>69</v>
       </c>
       <c r="D24" t="s">
-        <v>248</v>
+        <v>247</v>
       </c>
       <c r="E24">
         <v>1</v>
@@ -2598,16 +2592,16 @@
     </row>
     <row r="25" spans="1:5">
       <c r="A25" t="s">
-        <v>10</v>
+        <v>14</v>
       </c>
       <c r="B25" t="s">
         <v>40</v>
       </c>
       <c r="C25" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="D25" t="s">
-        <v>249</v>
+        <v>247</v>
       </c>
       <c r="E25">
         <v>1</v>
@@ -2615,16 +2609,16 @@
     </row>
     <row r="26" spans="1:5">
       <c r="A26" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="B26" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="C26" t="s">
         <v>70</v>
       </c>
       <c r="D26" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
       <c r="E26">
         <v>1</v>
@@ -2632,16 +2626,16 @@
     </row>
     <row r="27" spans="1:5">
       <c r="A27" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B27" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="C27" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="D27" t="s">
-        <v>250</v>
+        <v>248</v>
       </c>
       <c r="E27">
         <v>1</v>
@@ -2649,16 +2643,16 @@
     </row>
     <row r="28" spans="1:5">
       <c r="A28" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="B28" t="s">
         <v>40</v>
       </c>
       <c r="C28" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="D28" t="s">
-        <v>250</v>
+        <v>248</v>
       </c>
       <c r="E28">
         <v>1</v>
@@ -2666,16 +2660,16 @@
     </row>
     <row r="29" spans="1:5">
       <c r="A29" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="B29" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="C29" t="s">
         <v>71</v>
       </c>
       <c r="D29" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
       <c r="E29">
         <v>1</v>
@@ -2683,16 +2677,16 @@
     </row>
     <row r="30" spans="1:5">
       <c r="A30" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B30" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="C30" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="D30" t="s">
-        <v>251</v>
+        <v>249</v>
       </c>
       <c r="E30">
         <v>1</v>
@@ -2700,16 +2694,16 @@
     </row>
     <row r="31" spans="1:5">
       <c r="A31" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="B31" t="s">
         <v>40</v>
       </c>
       <c r="C31" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="D31" t="s">
-        <v>251</v>
+        <v>249</v>
       </c>
       <c r="E31">
         <v>1</v>
@@ -2717,16 +2711,16 @@
     </row>
     <row r="32" spans="1:5">
       <c r="A32" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="B32" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="C32" t="s">
         <v>72</v>
       </c>
       <c r="D32" t="s">
-        <v>251</v>
+        <v>250</v>
       </c>
       <c r="E32">
         <v>1</v>
@@ -2734,16 +2728,16 @@
     </row>
     <row r="33" spans="1:5">
       <c r="A33" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B33" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="C33" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="D33" t="s">
-        <v>252</v>
+        <v>250</v>
       </c>
       <c r="E33">
         <v>1</v>
@@ -2751,16 +2745,16 @@
     </row>
     <row r="34" spans="1:5">
       <c r="A34" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B34" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="C34" t="s">
         <v>73</v>
       </c>
       <c r="D34" t="s">
-        <v>252</v>
+        <v>251</v>
       </c>
       <c r="E34">
         <v>1</v>
@@ -2768,16 +2762,16 @@
     </row>
     <row r="35" spans="1:5">
       <c r="A35" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="B35" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="C35" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="D35" t="s">
-        <v>253</v>
+        <v>251</v>
       </c>
       <c r="E35">
         <v>1</v>
@@ -2785,16 +2779,16 @@
     </row>
     <row r="36" spans="1:5">
       <c r="A36" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="B36" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="C36" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="D36" t="s">
-        <v>253</v>
+        <v>251</v>
       </c>
       <c r="E36">
         <v>1</v>
@@ -2802,16 +2796,16 @@
     </row>
     <row r="37" spans="1:5">
       <c r="A37" t="s">
-        <v>15</v>
+        <v>11</v>
       </c>
       <c r="B37" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="C37" t="s">
         <v>74</v>
       </c>
       <c r="D37" t="s">
-        <v>253</v>
+        <v>252</v>
       </c>
       <c r="E37">
         <v>1</v>
@@ -2819,36 +2813,36 @@
     </row>
     <row r="38" spans="1:5">
       <c r="A38" t="s">
-        <v>11</v>
+        <v>15</v>
       </c>
       <c r="B38" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="C38" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="D38" t="s">
-        <v>254</v>
+        <v>252</v>
       </c>
       <c r="E38">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="39" spans="1:5">
       <c r="A39" t="s">
-        <v>15</v>
+        <v>11</v>
       </c>
       <c r="B39" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="C39" t="s">
         <v>75</v>
       </c>
       <c r="D39" t="s">
-        <v>254</v>
+        <v>253</v>
       </c>
       <c r="E39">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="40" spans="1:5">
@@ -2862,7 +2856,7 @@
         <v>76</v>
       </c>
       <c r="D40" t="s">
-        <v>255</v>
+        <v>254</v>
       </c>
       <c r="E40">
         <v>1</v>
@@ -2879,7 +2873,7 @@
         <v>77</v>
       </c>
       <c r="D41" t="s">
-        <v>256</v>
+        <v>255</v>
       </c>
       <c r="E41">
         <v>1</v>
@@ -2896,7 +2890,7 @@
         <v>78</v>
       </c>
       <c r="D42" t="s">
-        <v>257</v>
+        <v>256</v>
       </c>
       <c r="E42">
         <v>1</v>
@@ -2913,7 +2907,7 @@
         <v>79</v>
       </c>
       <c r="D43" t="s">
-        <v>258</v>
+        <v>257</v>
       </c>
       <c r="E43">
         <v>1</v>
@@ -2930,7 +2924,7 @@
         <v>80</v>
       </c>
       <c r="D44" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="E44">
         <v>1</v>
@@ -2947,7 +2941,7 @@
         <v>81</v>
       </c>
       <c r="D45" t="s">
-        <v>260</v>
+        <v>259</v>
       </c>
       <c r="E45">
         <v>1</v>
@@ -2964,7 +2958,7 @@
         <v>82</v>
       </c>
       <c r="D46" t="s">
-        <v>261</v>
+        <v>260</v>
       </c>
       <c r="E46">
         <v>1</v>
@@ -2981,58 +2975,58 @@
         <v>83</v>
       </c>
       <c r="D47" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
       <c r="E47">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="48" spans="1:5">
       <c r="A48" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B48" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="C48" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="D48" t="s">
-        <v>263</v>
+        <v>261</v>
       </c>
       <c r="E48">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="49" spans="1:5">
       <c r="A49" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="B49" t="s">
         <v>40</v>
       </c>
       <c r="C49" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="D49" t="s">
-        <v>263</v>
+        <v>261</v>
       </c>
       <c r="E49">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="50" spans="1:5">
       <c r="A50" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="B50" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="C50" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="D50" t="s">
-        <v>263</v>
+        <v>261</v>
       </c>
       <c r="E50">
         <v>2</v>
@@ -3040,16 +3034,16 @@
     </row>
     <row r="51" spans="1:5">
       <c r="A51" t="s">
-        <v>15</v>
+        <v>11</v>
       </c>
       <c r="B51" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="C51" t="s">
         <v>84</v>
       </c>
       <c r="D51" t="s">
-        <v>263</v>
+        <v>262</v>
       </c>
       <c r="E51">
         <v>2</v>
@@ -3057,16 +3051,16 @@
     </row>
     <row r="52" spans="1:5">
       <c r="A52" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="B52" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="C52" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="D52" t="s">
-        <v>264</v>
+        <v>262</v>
       </c>
       <c r="E52">
         <v>2</v>
@@ -3074,84 +3068,84 @@
     </row>
     <row r="53" spans="1:5">
       <c r="A53" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="B53" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="C53" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="D53" t="s">
-        <v>264</v>
+        <v>262</v>
       </c>
       <c r="E53">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="54" spans="1:5">
       <c r="A54" t="s">
-        <v>15</v>
+        <v>11</v>
       </c>
       <c r="B54" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="C54" t="s">
         <v>85</v>
       </c>
       <c r="D54" t="s">
-        <v>264</v>
+        <v>263</v>
       </c>
       <c r="E54">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="55" spans="1:5">
       <c r="A55" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="B55" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="C55" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="D55" t="s">
-        <v>265</v>
+        <v>263</v>
       </c>
       <c r="E55">
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
     <row r="56" spans="1:5">
       <c r="A56" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="B56" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="C56" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="D56" t="s">
-        <v>265</v>
+        <v>263</v>
       </c>
       <c r="E56">
-        <v>4</v>
+        <v>2</v>
       </c>
     </row>
     <row r="57" spans="1:5">
       <c r="A57" t="s">
-        <v>15</v>
+        <v>11</v>
       </c>
       <c r="B57" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="C57" t="s">
         <v>86</v>
       </c>
       <c r="D57" t="s">
-        <v>265</v>
+        <v>264</v>
       </c>
       <c r="E57">
         <v>2</v>
@@ -3159,36 +3153,36 @@
     </row>
     <row r="58" spans="1:5">
       <c r="A58" t="s">
-        <v>11</v>
+        <v>15</v>
       </c>
       <c r="B58" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="C58" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="D58" t="s">
-        <v>266</v>
+        <v>264</v>
       </c>
       <c r="E58">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="59" spans="1:5">
       <c r="A59" t="s">
-        <v>15</v>
+        <v>11</v>
       </c>
       <c r="B59" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="C59" t="s">
         <v>87</v>
       </c>
       <c r="D59" t="s">
-        <v>266</v>
+        <v>265</v>
       </c>
       <c r="E59">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="60" spans="1:5">
@@ -3202,7 +3196,7 @@
         <v>88</v>
       </c>
       <c r="D60" t="s">
-        <v>267</v>
+        <v>266</v>
       </c>
       <c r="E60">
         <v>2</v>
@@ -3219,7 +3213,7 @@
         <v>89</v>
       </c>
       <c r="D61" t="s">
-        <v>268</v>
+        <v>267</v>
       </c>
       <c r="E61">
         <v>2</v>
@@ -3236,7 +3230,7 @@
         <v>90</v>
       </c>
       <c r="D62" t="s">
-        <v>269</v>
+        <v>268</v>
       </c>
       <c r="E62">
         <v>2</v>
@@ -3253,7 +3247,7 @@
         <v>91</v>
       </c>
       <c r="D63" t="s">
-        <v>270</v>
+        <v>269</v>
       </c>
       <c r="E63">
         <v>2</v>
@@ -3270,7 +3264,7 @@
         <v>92</v>
       </c>
       <c r="D64" t="s">
-        <v>271</v>
+        <v>270</v>
       </c>
       <c r="E64">
         <v>2</v>
@@ -3287,7 +3281,7 @@
         <v>93</v>
       </c>
       <c r="D65" t="s">
-        <v>272</v>
+        <v>271</v>
       </c>
       <c r="E65">
         <v>2</v>
@@ -3304,7 +3298,7 @@
         <v>94</v>
       </c>
       <c r="D66" t="s">
-        <v>273</v>
+        <v>261</v>
       </c>
       <c r="E66">
         <v>2</v>
@@ -3321,24 +3315,24 @@
         <v>95</v>
       </c>
       <c r="D67" t="s">
-        <v>263</v>
+        <v>260</v>
       </c>
       <c r="E67">
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
     <row r="68" spans="1:5">
       <c r="A68" t="s">
-        <v>11</v>
+        <v>15</v>
       </c>
       <c r="B68" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="C68" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="D68" t="s">
-        <v>262</v>
+        <v>260</v>
       </c>
       <c r="E68">
         <v>4</v>
@@ -3346,16 +3340,16 @@
     </row>
     <row r="69" spans="1:5">
       <c r="A69" t="s">
-        <v>15</v>
+        <v>11</v>
       </c>
       <c r="B69" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="C69" t="s">
         <v>96</v>
       </c>
       <c r="D69" t="s">
-        <v>262</v>
+        <v>272</v>
       </c>
       <c r="E69">
         <v>4</v>
@@ -3372,7 +3366,7 @@
         <v>97</v>
       </c>
       <c r="D70" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
       <c r="E70">
         <v>4</v>
@@ -3389,7 +3383,7 @@
         <v>98</v>
       </c>
       <c r="D71" t="s">
-        <v>275</v>
+        <v>274</v>
       </c>
       <c r="E71">
         <v>4</v>
@@ -3397,33 +3391,33 @@
     </row>
     <row r="72" spans="1:5">
       <c r="A72" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B72" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="C72" t="s">
         <v>99</v>
       </c>
       <c r="D72" t="s">
-        <v>276</v>
+        <v>275</v>
       </c>
       <c r="E72">
-        <v>4</v>
+        <v>1</v>
       </c>
     </row>
     <row r="73" spans="1:5">
       <c r="A73" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="B73" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="C73" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="D73" t="s">
-        <v>277</v>
+        <v>275</v>
       </c>
       <c r="E73">
         <v>1</v>
@@ -3431,16 +3425,16 @@
     </row>
     <row r="74" spans="1:5">
       <c r="A74" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="B74" t="s">
-        <v>41</v>
+        <v>38</v>
       </c>
       <c r="C74" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="D74" t="s">
-        <v>277</v>
+        <v>275</v>
       </c>
       <c r="E74">
         <v>1</v>
@@ -3448,16 +3442,16 @@
     </row>
     <row r="75" spans="1:5">
       <c r="A75" t="s">
-        <v>15</v>
+        <v>12</v>
       </c>
       <c r="B75" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="C75" t="s">
         <v>100</v>
       </c>
       <c r="D75" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
       <c r="E75">
         <v>1</v>
@@ -3465,16 +3459,16 @@
     </row>
     <row r="76" spans="1:5">
       <c r="A76" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="B76" t="s">
         <v>40</v>
       </c>
       <c r="C76" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="D76" t="s">
-        <v>278</v>
+        <v>276</v>
       </c>
       <c r="E76">
         <v>1</v>
@@ -3482,16 +3476,16 @@
     </row>
     <row r="77" spans="1:5">
       <c r="A77" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="B77" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="C77" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="D77" t="s">
-        <v>278</v>
+        <v>276</v>
       </c>
       <c r="E77">
         <v>1</v>
@@ -3499,16 +3493,16 @@
     </row>
     <row r="78" spans="1:5">
       <c r="A78" t="s">
-        <v>15</v>
+        <v>12</v>
       </c>
       <c r="B78" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="C78" t="s">
         <v>101</v>
       </c>
       <c r="D78" t="s">
-        <v>278</v>
+        <v>277</v>
       </c>
       <c r="E78">
         <v>1</v>
@@ -3516,16 +3510,16 @@
     </row>
     <row r="79" spans="1:5">
       <c r="A79" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="B79" t="s">
         <v>40</v>
       </c>
       <c r="C79" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="D79" t="s">
-        <v>279</v>
+        <v>277</v>
       </c>
       <c r="E79">
         <v>1</v>
@@ -3533,50 +3527,50 @@
     </row>
     <row r="80" spans="1:5">
       <c r="A80" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="B80" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="C80" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="D80" t="s">
-        <v>279</v>
+        <v>277</v>
       </c>
       <c r="E80">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="81" spans="1:5">
       <c r="A81" t="s">
-        <v>15</v>
+        <v>12</v>
       </c>
       <c r="B81" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="C81" t="s">
         <v>102</v>
       </c>
       <c r="D81" t="s">
-        <v>279</v>
+        <v>278</v>
       </c>
       <c r="E81">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="82" spans="1:5">
       <c r="A82" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="B82" t="s">
         <v>40</v>
       </c>
       <c r="C82" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="D82" t="s">
-        <v>280</v>
+        <v>278</v>
       </c>
       <c r="E82">
         <v>1</v>
@@ -3584,7 +3578,7 @@
     </row>
     <row r="83" spans="1:5">
       <c r="A83" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="B83" t="s">
         <v>40</v>
@@ -3593,7 +3587,7 @@
         <v>103</v>
       </c>
       <c r="D83" t="s">
-        <v>280</v>
+        <v>279</v>
       </c>
       <c r="E83">
         <v>1</v>
@@ -3601,16 +3595,16 @@
     </row>
     <row r="84" spans="1:5">
       <c r="A84" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="B84" t="s">
         <v>40</v>
       </c>
       <c r="C84" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="D84" t="s">
-        <v>281</v>
+        <v>279</v>
       </c>
       <c r="E84">
         <v>1</v>
@@ -3618,7 +3612,7 @@
     </row>
     <row r="85" spans="1:5">
       <c r="A85" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="B85" t="s">
         <v>40</v>
@@ -3627,7 +3621,7 @@
         <v>104</v>
       </c>
       <c r="D85" t="s">
-        <v>281</v>
+        <v>280</v>
       </c>
       <c r="E85">
         <v>1</v>
@@ -3635,16 +3629,16 @@
     </row>
     <row r="86" spans="1:5">
       <c r="A86" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="B86" t="s">
         <v>40</v>
       </c>
       <c r="C86" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="D86" t="s">
-        <v>282</v>
+        <v>280</v>
       </c>
       <c r="E86">
         <v>1</v>
@@ -3652,7 +3646,7 @@
     </row>
     <row r="87" spans="1:5">
       <c r="A87" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="B87" t="s">
         <v>40</v>
@@ -3661,7 +3655,7 @@
         <v>105</v>
       </c>
       <c r="D87" t="s">
-        <v>282</v>
+        <v>281</v>
       </c>
       <c r="E87">
         <v>1</v>
@@ -3669,16 +3663,16 @@
     </row>
     <row r="88" spans="1:5">
       <c r="A88" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="B88" t="s">
         <v>40</v>
       </c>
       <c r="C88" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="D88" t="s">
-        <v>283</v>
+        <v>281</v>
       </c>
       <c r="E88">
         <v>1</v>
@@ -3686,7 +3680,7 @@
     </row>
     <row r="89" spans="1:5">
       <c r="A89" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="B89" t="s">
         <v>40</v>
@@ -3695,7 +3689,7 @@
         <v>106</v>
       </c>
       <c r="D89" t="s">
-        <v>283</v>
+        <v>282</v>
       </c>
       <c r="E89">
         <v>1</v>
@@ -3703,16 +3697,16 @@
     </row>
     <row r="90" spans="1:5">
       <c r="A90" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="B90" t="s">
         <v>40</v>
       </c>
       <c r="C90" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="D90" t="s">
-        <v>284</v>
+        <v>282</v>
       </c>
       <c r="E90">
         <v>1</v>
@@ -3720,7 +3714,7 @@
     </row>
     <row r="91" spans="1:5">
       <c r="A91" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="B91" t="s">
         <v>40</v>
@@ -3729,7 +3723,7 @@
         <v>107</v>
       </c>
       <c r="D91" t="s">
-        <v>284</v>
+        <v>283</v>
       </c>
       <c r="E91">
         <v>1</v>
@@ -3737,16 +3731,16 @@
     </row>
     <row r="92" spans="1:5">
       <c r="A92" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="B92" t="s">
         <v>40</v>
       </c>
       <c r="C92" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="D92" t="s">
-        <v>285</v>
+        <v>283</v>
       </c>
       <c r="E92">
         <v>1</v>
@@ -3754,7 +3748,7 @@
     </row>
     <row r="93" spans="1:5">
       <c r="A93" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="B93" t="s">
         <v>40</v>
@@ -3763,7 +3757,7 @@
         <v>108</v>
       </c>
       <c r="D93" t="s">
-        <v>285</v>
+        <v>284</v>
       </c>
       <c r="E93">
         <v>1</v>
@@ -3771,16 +3765,16 @@
     </row>
     <row r="94" spans="1:5">
       <c r="A94" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="B94" t="s">
         <v>40</v>
       </c>
       <c r="C94" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="D94" t="s">
-        <v>286</v>
+        <v>284</v>
       </c>
       <c r="E94">
         <v>1</v>
@@ -3788,7 +3782,7 @@
     </row>
     <row r="95" spans="1:5">
       <c r="A95" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="B95" t="s">
         <v>40</v>
@@ -3797,7 +3791,7 @@
         <v>109</v>
       </c>
       <c r="D95" t="s">
-        <v>286</v>
+        <v>285</v>
       </c>
       <c r="E95">
         <v>1</v>
@@ -3805,16 +3799,16 @@
     </row>
     <row r="96" spans="1:5">
       <c r="A96" t="s">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="B96" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="C96" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="D96" t="s">
-        <v>287</v>
+        <v>285</v>
       </c>
       <c r="E96">
         <v>1</v>
@@ -3822,16 +3816,16 @@
     </row>
     <row r="97" spans="1:5">
       <c r="A97" t="s">
-        <v>15</v>
+        <v>12</v>
       </c>
       <c r="B97" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="C97" t="s">
         <v>110</v>
       </c>
       <c r="D97" t="s">
-        <v>287</v>
+        <v>286</v>
       </c>
       <c r="E97">
         <v>1</v>
@@ -3839,16 +3833,16 @@
     </row>
     <row r="98" spans="1:5">
       <c r="A98" t="s">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="B98" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="C98" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="D98" t="s">
-        <v>288</v>
+        <v>286</v>
       </c>
       <c r="E98">
         <v>1</v>
@@ -3856,16 +3850,16 @@
     </row>
     <row r="99" spans="1:5">
       <c r="A99" t="s">
-        <v>15</v>
+        <v>12</v>
       </c>
       <c r="B99" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="C99" t="s">
         <v>111</v>
       </c>
       <c r="D99" t="s">
-        <v>288</v>
+        <v>287</v>
       </c>
       <c r="E99">
         <v>1</v>
@@ -3882,7 +3876,7 @@
         <v>112</v>
       </c>
       <c r="D100" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
       <c r="E100">
         <v>1</v>
@@ -3899,7 +3893,7 @@
         <v>113</v>
       </c>
       <c r="D101" t="s">
-        <v>290</v>
+        <v>289</v>
       </c>
       <c r="E101">
         <v>1</v>
@@ -3916,7 +3910,7 @@
         <v>114</v>
       </c>
       <c r="D102" t="s">
-        <v>291</v>
+        <v>290</v>
       </c>
       <c r="E102">
         <v>1</v>
@@ -3933,7 +3927,7 @@
         <v>115</v>
       </c>
       <c r="D103" t="s">
-        <v>292</v>
+        <v>291</v>
       </c>
       <c r="E103">
         <v>1</v>
@@ -3950,7 +3944,7 @@
         <v>116</v>
       </c>
       <c r="D104" t="s">
-        <v>293</v>
+        <v>292</v>
       </c>
       <c r="E104">
         <v>1</v>
@@ -3967,32 +3961,32 @@
         <v>117</v>
       </c>
       <c r="D105" t="s">
-        <v>294</v>
+        <v>293</v>
       </c>
       <c r="E105">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="106" spans="1:5">
       <c r="A106" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="B106" t="s">
         <v>40</v>
       </c>
       <c r="C106" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="D106" t="s">
-        <v>295</v>
+        <v>293</v>
       </c>
       <c r="E106">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="107" spans="1:5">
       <c r="A107" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="B107" t="s">
         <v>40</v>
@@ -4001,24 +3995,24 @@
         <v>118</v>
       </c>
       <c r="D107" t="s">
-        <v>295</v>
+        <v>294</v>
       </c>
       <c r="E107">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="108" spans="1:5">
       <c r="A108" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="B108" t="s">
         <v>40</v>
       </c>
       <c r="C108" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="D108" t="s">
-        <v>296</v>
+        <v>294</v>
       </c>
       <c r="E108">
         <v>2</v>
@@ -4026,16 +4020,16 @@
     </row>
     <row r="109" spans="1:5">
       <c r="A109" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="B109" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="C109" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="D109" t="s">
-        <v>296</v>
+        <v>294</v>
       </c>
       <c r="E109">
         <v>2</v>
@@ -4043,16 +4037,16 @@
     </row>
     <row r="110" spans="1:5">
       <c r="A110" t="s">
-        <v>15</v>
+        <v>12</v>
       </c>
       <c r="B110" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="C110" t="s">
         <v>119</v>
       </c>
       <c r="D110" t="s">
-        <v>296</v>
+        <v>295</v>
       </c>
       <c r="E110">
         <v>2</v>
@@ -4060,16 +4054,16 @@
     </row>
     <row r="111" spans="1:5">
       <c r="A111" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="B111" t="s">
         <v>40</v>
       </c>
       <c r="C111" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="D111" t="s">
-        <v>297</v>
+        <v>295</v>
       </c>
       <c r="E111">
         <v>2</v>
@@ -4077,16 +4071,16 @@
     </row>
     <row r="112" spans="1:5">
       <c r="A112" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="B112" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="C112" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="D112" t="s">
-        <v>297</v>
+        <v>295</v>
       </c>
       <c r="E112">
         <v>2</v>
@@ -4094,16 +4088,16 @@
     </row>
     <row r="113" spans="1:5">
       <c r="A113" t="s">
-        <v>15</v>
+        <v>12</v>
       </c>
       <c r="B113" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="C113" t="s">
         <v>120</v>
       </c>
       <c r="D113" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="E113">
         <v>2</v>
@@ -4111,16 +4105,16 @@
     </row>
     <row r="114" spans="1:5">
       <c r="A114" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="B114" t="s">
         <v>40</v>
       </c>
       <c r="C114" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="D114" t="s">
-        <v>298</v>
+        <v>296</v>
       </c>
       <c r="E114">
         <v>2</v>
@@ -4128,7 +4122,7 @@
     </row>
     <row r="115" spans="1:5">
       <c r="A115" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="B115" t="s">
         <v>40</v>
@@ -4137,7 +4131,7 @@
         <v>121</v>
       </c>
       <c r="D115" t="s">
-        <v>298</v>
+        <v>297</v>
       </c>
       <c r="E115">
         <v>2</v>
@@ -4145,16 +4139,16 @@
     </row>
     <row r="116" spans="1:5">
       <c r="A116" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="B116" t="s">
         <v>40</v>
       </c>
       <c r="C116" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="D116" t="s">
-        <v>299</v>
+        <v>297</v>
       </c>
       <c r="E116">
         <v>2</v>
@@ -4162,7 +4156,7 @@
     </row>
     <row r="117" spans="1:5">
       <c r="A117" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="B117" t="s">
         <v>40</v>
@@ -4171,7 +4165,7 @@
         <v>122</v>
       </c>
       <c r="D117" t="s">
-        <v>299</v>
+        <v>277</v>
       </c>
       <c r="E117">
         <v>2</v>
@@ -4179,33 +4173,33 @@
     </row>
     <row r="118" spans="1:5">
       <c r="A118" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="B118" t="s">
         <v>40</v>
       </c>
       <c r="C118" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="D118" t="s">
-        <v>279</v>
+        <v>277</v>
       </c>
       <c r="E118">
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
     <row r="119" spans="1:5">
       <c r="A119" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="B119" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="C119" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="D119" t="s">
-        <v>279</v>
+        <v>277</v>
       </c>
       <c r="E119">
         <v>4</v>
@@ -4213,41 +4207,41 @@
     </row>
     <row r="120" spans="1:5">
       <c r="A120" t="s">
-        <v>15</v>
+        <v>12</v>
       </c>
       <c r="B120" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="C120" t="s">
         <v>123</v>
       </c>
       <c r="D120" t="s">
-        <v>279</v>
+        <v>298</v>
       </c>
       <c r="E120">
-        <v>4</v>
+        <v>2</v>
       </c>
     </row>
     <row r="121" spans="1:5">
       <c r="A121" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="B121" t="s">
         <v>40</v>
       </c>
       <c r="C121" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="D121" t="s">
-        <v>300</v>
+        <v>298</v>
       </c>
       <c r="E121">
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
     <row r="122" spans="1:5">
       <c r="A122" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="B122" t="s">
         <v>40</v>
@@ -4256,10 +4250,10 @@
         <v>124</v>
       </c>
       <c r="D122" t="s">
-        <v>300</v>
+        <v>283</v>
       </c>
       <c r="E122">
-        <v>4</v>
+        <v>2</v>
       </c>
     </row>
     <row r="123" spans="1:5">
@@ -4273,7 +4267,7 @@
         <v>125</v>
       </c>
       <c r="D123" t="s">
-        <v>285</v>
+        <v>299</v>
       </c>
       <c r="E123">
         <v>2</v>
@@ -4290,7 +4284,7 @@
         <v>126</v>
       </c>
       <c r="D124" t="s">
-        <v>301</v>
+        <v>300</v>
       </c>
       <c r="E124">
         <v>2</v>
@@ -4307,24 +4301,24 @@
         <v>127</v>
       </c>
       <c r="D125" t="s">
-        <v>302</v>
+        <v>301</v>
       </c>
       <c r="E125">
-        <v>2</v>
+        <v>5</v>
       </c>
     </row>
     <row r="126" spans="1:5">
       <c r="A126" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="B126" t="s">
         <v>40</v>
       </c>
       <c r="C126" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="D126" t="s">
-        <v>303</v>
+        <v>301</v>
       </c>
       <c r="E126">
         <v>5</v>
@@ -4332,7 +4326,7 @@
     </row>
     <row r="127" spans="1:5">
       <c r="A127" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="B127" t="s">
         <v>40</v>
@@ -4341,10 +4335,10 @@
         <v>128</v>
       </c>
       <c r="D127" t="s">
-        <v>303</v>
+        <v>302</v>
       </c>
       <c r="E127">
-        <v>5</v>
+        <v>7</v>
       </c>
     </row>
     <row r="128" spans="1:5">
@@ -4358,10 +4352,10 @@
         <v>129</v>
       </c>
       <c r="D128" t="s">
-        <v>304</v>
+        <v>303</v>
       </c>
       <c r="E128">
-        <v>7</v>
+        <v>10</v>
       </c>
     </row>
     <row r="129" spans="1:5">
@@ -4375,24 +4369,24 @@
         <v>130</v>
       </c>
       <c r="D129" t="s">
-        <v>305</v>
+        <v>304</v>
       </c>
       <c r="E129">
-        <v>10</v>
+        <v>30</v>
       </c>
     </row>
     <row r="130" spans="1:5">
       <c r="A130" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="B130" t="s">
         <v>40</v>
       </c>
       <c r="C130" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="D130" t="s">
-        <v>306</v>
+        <v>304</v>
       </c>
       <c r="E130">
         <v>30</v>
@@ -4409,24 +4403,24 @@
         <v>131</v>
       </c>
       <c r="D131" t="s">
-        <v>306</v>
+        <v>305</v>
       </c>
       <c r="E131">
-        <v>30</v>
+        <v>1</v>
       </c>
     </row>
     <row r="132" spans="1:5">
       <c r="A132" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="B132" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="C132" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="D132" t="s">
-        <v>307</v>
+        <v>305</v>
       </c>
       <c r="E132">
         <v>1</v>
@@ -4434,16 +4428,16 @@
     </row>
     <row r="133" spans="1:5">
       <c r="A133" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B133" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="C133" t="s">
         <v>132</v>
       </c>
       <c r="D133" t="s">
-        <v>307</v>
+        <v>306</v>
       </c>
       <c r="E133">
         <v>1</v>
@@ -4460,7 +4454,7 @@
         <v>133</v>
       </c>
       <c r="D134" t="s">
-        <v>308</v>
+        <v>307</v>
       </c>
       <c r="E134">
         <v>1</v>
@@ -4477,7 +4471,7 @@
         <v>134</v>
       </c>
       <c r="D135" t="s">
-        <v>309</v>
+        <v>308</v>
       </c>
       <c r="E135">
         <v>1</v>
@@ -4494,7 +4488,7 @@
         <v>135</v>
       </c>
       <c r="D136" t="s">
-        <v>310</v>
+        <v>309</v>
       </c>
       <c r="E136">
         <v>1</v>
@@ -4511,7 +4505,7 @@
         <v>136</v>
       </c>
       <c r="D137" t="s">
-        <v>311</v>
+        <v>310</v>
       </c>
       <c r="E137">
         <v>1</v>
@@ -4528,7 +4522,7 @@
         <v>137</v>
       </c>
       <c r="D138" t="s">
-        <v>312</v>
+        <v>311</v>
       </c>
       <c r="E138">
         <v>1</v>
@@ -4545,7 +4539,7 @@
         <v>138</v>
       </c>
       <c r="D139" t="s">
-        <v>313</v>
+        <v>312</v>
       </c>
       <c r="E139">
         <v>1</v>
@@ -4562,7 +4556,7 @@
         <v>139</v>
       </c>
       <c r="D140" t="s">
-        <v>314</v>
+        <v>313</v>
       </c>
       <c r="E140">
         <v>1</v>
@@ -4579,7 +4573,7 @@
         <v>140</v>
       </c>
       <c r="D141" t="s">
-        <v>315</v>
+        <v>314</v>
       </c>
       <c r="E141">
         <v>1</v>
@@ -4596,7 +4590,7 @@
         <v>141</v>
       </c>
       <c r="D142" t="s">
-        <v>316</v>
+        <v>315</v>
       </c>
       <c r="E142">
         <v>1</v>
@@ -4613,7 +4607,7 @@
         <v>142</v>
       </c>
       <c r="D143" t="s">
-        <v>317</v>
+        <v>316</v>
       </c>
       <c r="E143">
         <v>1</v>
@@ -4630,7 +4624,7 @@
         <v>143</v>
       </c>
       <c r="D144" t="s">
-        <v>318</v>
+        <v>317</v>
       </c>
       <c r="E144">
         <v>1</v>
@@ -4647,7 +4641,7 @@
         <v>144</v>
       </c>
       <c r="D145" t="s">
-        <v>319</v>
+        <v>318</v>
       </c>
       <c r="E145">
         <v>1</v>
@@ -4664,7 +4658,7 @@
         <v>145</v>
       </c>
       <c r="D146" t="s">
-        <v>320</v>
+        <v>319</v>
       </c>
       <c r="E146">
         <v>1</v>
@@ -4681,7 +4675,7 @@
         <v>146</v>
       </c>
       <c r="D147" t="s">
-        <v>321</v>
+        <v>320</v>
       </c>
       <c r="E147">
         <v>1</v>
@@ -4698,7 +4692,7 @@
         <v>147</v>
       </c>
       <c r="D148" t="s">
-        <v>322</v>
+        <v>321</v>
       </c>
       <c r="E148">
         <v>1</v>
@@ -4715,7 +4709,7 @@
         <v>148</v>
       </c>
       <c r="D149" t="s">
-        <v>323</v>
+        <v>322</v>
       </c>
       <c r="E149">
         <v>1</v>
@@ -4732,7 +4726,7 @@
         <v>149</v>
       </c>
       <c r="D150" t="s">
-        <v>324</v>
+        <v>323</v>
       </c>
       <c r="E150">
         <v>1</v>
@@ -4749,7 +4743,7 @@
         <v>150</v>
       </c>
       <c r="D151" t="s">
-        <v>325</v>
+        <v>324</v>
       </c>
       <c r="E151">
         <v>1</v>
@@ -4766,7 +4760,7 @@
         <v>151</v>
       </c>
       <c r="D152" t="s">
-        <v>326</v>
+        <v>325</v>
       </c>
       <c r="E152">
         <v>1</v>
@@ -4783,7 +4777,7 @@
         <v>152</v>
       </c>
       <c r="D153" t="s">
-        <v>327</v>
+        <v>326</v>
       </c>
       <c r="E153">
         <v>1</v>
@@ -4800,7 +4794,7 @@
         <v>153</v>
       </c>
       <c r="D154" t="s">
-        <v>328</v>
+        <v>327</v>
       </c>
       <c r="E154">
         <v>1</v>
@@ -4817,7 +4811,7 @@
         <v>154</v>
       </c>
       <c r="D155" t="s">
-        <v>329</v>
+        <v>328</v>
       </c>
       <c r="E155">
         <v>1</v>
@@ -4834,7 +4828,7 @@
         <v>155</v>
       </c>
       <c r="D156" t="s">
-        <v>330</v>
+        <v>329</v>
       </c>
       <c r="E156">
         <v>1</v>
@@ -4851,7 +4845,7 @@
         <v>156</v>
       </c>
       <c r="D157" t="s">
-        <v>331</v>
+        <v>330</v>
       </c>
       <c r="E157">
         <v>1</v>
@@ -4868,7 +4862,7 @@
         <v>157</v>
       </c>
       <c r="D158" t="s">
-        <v>332</v>
+        <v>331</v>
       </c>
       <c r="E158">
         <v>1</v>
@@ -4885,7 +4879,7 @@
         <v>158</v>
       </c>
       <c r="D159" t="s">
-        <v>333</v>
+        <v>332</v>
       </c>
       <c r="E159">
         <v>1</v>
@@ -4902,7 +4896,7 @@
         <v>159</v>
       </c>
       <c r="D160" t="s">
-        <v>334</v>
+        <v>333</v>
       </c>
       <c r="E160">
         <v>1</v>
@@ -4919,7 +4913,7 @@
         <v>160</v>
       </c>
       <c r="D161" t="s">
-        <v>335</v>
+        <v>334</v>
       </c>
       <c r="E161">
         <v>1</v>
@@ -4936,7 +4930,7 @@
         <v>161</v>
       </c>
       <c r="D162" t="s">
-        <v>336</v>
+        <v>335</v>
       </c>
       <c r="E162">
         <v>1</v>
@@ -4953,7 +4947,7 @@
         <v>162</v>
       </c>
       <c r="D163" t="s">
-        <v>337</v>
+        <v>336</v>
       </c>
       <c r="E163">
         <v>1</v>
@@ -4970,7 +4964,7 @@
         <v>163</v>
       </c>
       <c r="D164" t="s">
-        <v>338</v>
+        <v>337</v>
       </c>
       <c r="E164">
         <v>1</v>
@@ -4987,10 +4981,10 @@
         <v>164</v>
       </c>
       <c r="D165" t="s">
-        <v>339</v>
+        <v>320</v>
       </c>
       <c r="E165">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="166" spans="1:5">
@@ -5004,7 +4998,7 @@
         <v>165</v>
       </c>
       <c r="D166" t="s">
-        <v>322</v>
+        <v>338</v>
       </c>
       <c r="E166">
         <v>2</v>
@@ -5021,7 +5015,7 @@
         <v>166</v>
       </c>
       <c r="D167" t="s">
-        <v>340</v>
+        <v>339</v>
       </c>
       <c r="E167">
         <v>2</v>
@@ -5038,7 +5032,7 @@
         <v>167</v>
       </c>
       <c r="D168" t="s">
-        <v>341</v>
+        <v>340</v>
       </c>
       <c r="E168">
         <v>2</v>
@@ -5055,7 +5049,7 @@
         <v>168</v>
       </c>
       <c r="D169" t="s">
-        <v>342</v>
+        <v>341</v>
       </c>
       <c r="E169">
         <v>2</v>
@@ -5072,10 +5066,10 @@
         <v>169</v>
       </c>
       <c r="D170" t="s">
-        <v>343</v>
+        <v>342</v>
       </c>
       <c r="E170">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="171" spans="1:5">
@@ -5089,10 +5083,10 @@
         <v>170</v>
       </c>
       <c r="D171" t="s">
-        <v>344</v>
+        <v>304</v>
       </c>
       <c r="E171">
-        <v>3</v>
+        <v>5</v>
       </c>
     </row>
     <row r="172" spans="1:5">
@@ -5106,10 +5100,10 @@
         <v>171</v>
       </c>
       <c r="D172" t="s">
-        <v>306</v>
+        <v>343</v>
       </c>
       <c r="E172">
-        <v>5</v>
+        <v>8</v>
       </c>
     </row>
     <row r="173" spans="1:5">
@@ -5123,7 +5117,7 @@
         <v>172</v>
       </c>
       <c r="D173" t="s">
-        <v>345</v>
+        <v>257</v>
       </c>
       <c r="E173">
         <v>8</v>
@@ -5140,27 +5134,27 @@
         <v>173</v>
       </c>
       <c r="D174" t="s">
-        <v>259</v>
+        <v>344</v>
       </c>
       <c r="E174">
-        <v>8</v>
+        <v>10</v>
       </c>
     </row>
     <row r="175" spans="1:5">
       <c r="A175" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="B175" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="C175" t="s">
         <v>174</v>
       </c>
       <c r="D175" t="s">
-        <v>346</v>
+        <v>330</v>
       </c>
       <c r="E175">
-        <v>10</v>
+        <v>1</v>
       </c>
     </row>
     <row r="176" spans="1:5">
@@ -5174,7 +5168,7 @@
         <v>175</v>
       </c>
       <c r="D176" t="s">
-        <v>332</v>
+        <v>345</v>
       </c>
       <c r="E176">
         <v>1</v>
@@ -5191,7 +5185,7 @@
         <v>176</v>
       </c>
       <c r="D177" t="s">
-        <v>347</v>
+        <v>346</v>
       </c>
       <c r="E177">
         <v>1</v>
@@ -5208,7 +5202,7 @@
         <v>177</v>
       </c>
       <c r="D178" t="s">
-        <v>348</v>
+        <v>347</v>
       </c>
       <c r="E178">
         <v>1</v>
@@ -5225,7 +5219,7 @@
         <v>178</v>
       </c>
       <c r="D179" t="s">
-        <v>349</v>
+        <v>348</v>
       </c>
       <c r="E179">
         <v>1</v>
@@ -5242,7 +5236,7 @@
         <v>179</v>
       </c>
       <c r="D180" t="s">
-        <v>350</v>
+        <v>349</v>
       </c>
       <c r="E180">
         <v>1</v>
@@ -5259,7 +5253,7 @@
         <v>180</v>
       </c>
       <c r="D181" t="s">
-        <v>351</v>
+        <v>267</v>
       </c>
       <c r="E181">
         <v>1</v>
@@ -5276,7 +5270,7 @@
         <v>181</v>
       </c>
       <c r="D182" t="s">
-        <v>269</v>
+        <v>350</v>
       </c>
       <c r="E182">
         <v>1</v>
@@ -5293,7 +5287,7 @@
         <v>182</v>
       </c>
       <c r="D183" t="s">
-        <v>352</v>
+        <v>351</v>
       </c>
       <c r="E183">
         <v>1</v>
@@ -5310,7 +5304,7 @@
         <v>183</v>
       </c>
       <c r="D184" t="s">
-        <v>353</v>
+        <v>352</v>
       </c>
       <c r="E184">
         <v>1</v>
@@ -5327,7 +5321,7 @@
         <v>184</v>
       </c>
       <c r="D185" t="s">
-        <v>354</v>
+        <v>353</v>
       </c>
       <c r="E185">
         <v>1</v>
@@ -5344,7 +5338,7 @@
         <v>185</v>
       </c>
       <c r="D186" t="s">
-        <v>355</v>
+        <v>354</v>
       </c>
       <c r="E186">
         <v>1</v>
@@ -5361,7 +5355,7 @@
         <v>186</v>
       </c>
       <c r="D187" t="s">
-        <v>356</v>
+        <v>355</v>
       </c>
       <c r="E187">
         <v>1</v>
@@ -5378,7 +5372,7 @@
         <v>187</v>
       </c>
       <c r="D188" t="s">
-        <v>357</v>
+        <v>356</v>
       </c>
       <c r="E188">
         <v>1</v>
@@ -5395,7 +5389,7 @@
         <v>188</v>
       </c>
       <c r="D189" t="s">
-        <v>358</v>
+        <v>357</v>
       </c>
       <c r="E189">
         <v>1</v>
@@ -5412,7 +5406,7 @@
         <v>189</v>
       </c>
       <c r="D190" t="s">
-        <v>359</v>
+        <v>358</v>
       </c>
       <c r="E190">
         <v>1</v>
@@ -5429,7 +5423,7 @@
         <v>190</v>
       </c>
       <c r="D191" t="s">
-        <v>360</v>
+        <v>359</v>
       </c>
       <c r="E191">
         <v>1</v>
@@ -5446,7 +5440,7 @@
         <v>191</v>
       </c>
       <c r="D192" t="s">
-        <v>361</v>
+        <v>360</v>
       </c>
       <c r="E192">
         <v>1</v>
@@ -5463,7 +5457,7 @@
         <v>192</v>
       </c>
       <c r="D193" t="s">
-        <v>362</v>
+        <v>361</v>
       </c>
       <c r="E193">
         <v>1</v>
@@ -5480,7 +5474,7 @@
         <v>193</v>
       </c>
       <c r="D194" t="s">
-        <v>363</v>
+        <v>362</v>
       </c>
       <c r="E194">
         <v>1</v>
@@ -5497,7 +5491,7 @@
         <v>194</v>
       </c>
       <c r="D195" t="s">
-        <v>364</v>
+        <v>363</v>
       </c>
       <c r="E195">
         <v>1</v>
@@ -5514,7 +5508,7 @@
         <v>195</v>
       </c>
       <c r="D196" t="s">
-        <v>365</v>
+        <v>364</v>
       </c>
       <c r="E196">
         <v>1</v>
@@ -5531,7 +5525,7 @@
         <v>196</v>
       </c>
       <c r="D197" t="s">
-        <v>366</v>
+        <v>365</v>
       </c>
       <c r="E197">
         <v>1</v>
@@ -5548,7 +5542,7 @@
         <v>197</v>
       </c>
       <c r="D198" t="s">
-        <v>367</v>
+        <v>366</v>
       </c>
       <c r="E198">
         <v>1</v>
@@ -5565,7 +5559,7 @@
         <v>198</v>
       </c>
       <c r="D199" t="s">
-        <v>368</v>
+        <v>367</v>
       </c>
       <c r="E199">
         <v>1</v>
@@ -5582,7 +5576,7 @@
         <v>199</v>
       </c>
       <c r="D200" t="s">
-        <v>369</v>
+        <v>368</v>
       </c>
       <c r="E200">
         <v>1</v>
@@ -5599,7 +5593,7 @@
         <v>200</v>
       </c>
       <c r="D201" t="s">
-        <v>370</v>
+        <v>369</v>
       </c>
       <c r="E201">
         <v>1</v>
@@ -5616,7 +5610,7 @@
         <v>201</v>
       </c>
       <c r="D202" t="s">
-        <v>371</v>
+        <v>370</v>
       </c>
       <c r="E202">
         <v>1</v>
@@ -5633,7 +5627,7 @@
         <v>202</v>
       </c>
       <c r="D203" t="s">
-        <v>372</v>
+        <v>371</v>
       </c>
       <c r="E203">
         <v>1</v>
@@ -5650,7 +5644,7 @@
         <v>203</v>
       </c>
       <c r="D204" t="s">
-        <v>373</v>
+        <v>372</v>
       </c>
       <c r="E204">
         <v>1</v>
@@ -5667,7 +5661,7 @@
         <v>204</v>
       </c>
       <c r="D205" t="s">
-        <v>374</v>
+        <v>373</v>
       </c>
       <c r="E205">
         <v>1</v>
@@ -5684,7 +5678,7 @@
         <v>205</v>
       </c>
       <c r="D206" t="s">
-        <v>375</v>
+        <v>374</v>
       </c>
       <c r="E206">
         <v>1</v>
@@ -5701,10 +5695,10 @@
         <v>206</v>
       </c>
       <c r="D207" t="s">
-        <v>376</v>
+        <v>375</v>
       </c>
       <c r="E207">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="208" spans="1:5">
@@ -5718,7 +5712,7 @@
         <v>207</v>
       </c>
       <c r="D208" t="s">
-        <v>377</v>
+        <v>376</v>
       </c>
       <c r="E208">
         <v>2</v>
@@ -5735,7 +5729,7 @@
         <v>208</v>
       </c>
       <c r="D209" t="s">
-        <v>378</v>
+        <v>377</v>
       </c>
       <c r="E209">
         <v>2</v>
@@ -5752,7 +5746,7 @@
         <v>209</v>
       </c>
       <c r="D210" t="s">
-        <v>379</v>
+        <v>378</v>
       </c>
       <c r="E210">
         <v>2</v>
@@ -5769,7 +5763,7 @@
         <v>210</v>
       </c>
       <c r="D211" t="s">
-        <v>380</v>
+        <v>379</v>
       </c>
       <c r="E211">
         <v>2</v>
@@ -5786,7 +5780,7 @@
         <v>211</v>
       </c>
       <c r="D212" t="s">
-        <v>381</v>
+        <v>380</v>
       </c>
       <c r="E212">
         <v>2</v>
@@ -5803,7 +5797,7 @@
         <v>212</v>
       </c>
       <c r="D213" t="s">
-        <v>382</v>
+        <v>381</v>
       </c>
       <c r="E213">
         <v>2</v>
@@ -5820,7 +5814,7 @@
         <v>213</v>
       </c>
       <c r="D214" t="s">
-        <v>383</v>
+        <v>382</v>
       </c>
       <c r="E214">
         <v>2</v>
@@ -5837,7 +5831,7 @@
         <v>214</v>
       </c>
       <c r="D215" t="s">
-        <v>384</v>
+        <v>383</v>
       </c>
       <c r="E215">
         <v>2</v>
@@ -5854,7 +5848,7 @@
         <v>215</v>
       </c>
       <c r="D216" t="s">
-        <v>385</v>
+        <v>383</v>
       </c>
       <c r="E216">
         <v>2</v>
@@ -5871,7 +5865,7 @@
         <v>216</v>
       </c>
       <c r="D217" t="s">
-        <v>385</v>
+        <v>384</v>
       </c>
       <c r="E217">
         <v>2</v>
@@ -5888,7 +5882,7 @@
         <v>217</v>
       </c>
       <c r="D218" t="s">
-        <v>386</v>
+        <v>385</v>
       </c>
       <c r="E218">
         <v>2</v>
@@ -5905,10 +5899,10 @@
         <v>218</v>
       </c>
       <c r="D219" t="s">
-        <v>387</v>
+        <v>386</v>
       </c>
       <c r="E219">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="220" spans="1:5">
@@ -5922,7 +5916,7 @@
         <v>219</v>
       </c>
       <c r="D220" t="s">
-        <v>388</v>
+        <v>267</v>
       </c>
       <c r="E220">
         <v>3</v>
@@ -5939,10 +5933,10 @@
         <v>220</v>
       </c>
       <c r="D221" t="s">
-        <v>269</v>
+        <v>387</v>
       </c>
       <c r="E221">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="222" spans="1:5">
@@ -5956,7 +5950,7 @@
         <v>221</v>
       </c>
       <c r="D222" t="s">
-        <v>389</v>
+        <v>388</v>
       </c>
       <c r="E222">
         <v>4</v>
@@ -5973,7 +5967,7 @@
         <v>222</v>
       </c>
       <c r="D223" t="s">
-        <v>390</v>
+        <v>389</v>
       </c>
       <c r="E223">
         <v>4</v>
@@ -5990,7 +5984,7 @@
         <v>223</v>
       </c>
       <c r="D224" t="s">
-        <v>391</v>
+        <v>390</v>
       </c>
       <c r="E224">
         <v>4</v>
@@ -6007,7 +6001,7 @@
         <v>224</v>
       </c>
       <c r="D225" t="s">
-        <v>392</v>
+        <v>391</v>
       </c>
       <c r="E225">
         <v>4</v>
@@ -6024,10 +6018,10 @@
         <v>225</v>
       </c>
       <c r="D226" t="s">
-        <v>393</v>
+        <v>392</v>
       </c>
       <c r="E226">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="227" spans="1:5">
@@ -6041,7 +6035,7 @@
         <v>226</v>
       </c>
       <c r="D227" t="s">
-        <v>394</v>
+        <v>393</v>
       </c>
       <c r="E227">
         <v>5</v>
@@ -6058,10 +6052,10 @@
         <v>227</v>
       </c>
       <c r="D228" t="s">
-        <v>395</v>
+        <v>394</v>
       </c>
       <c r="E228">
-        <v>5</v>
+        <v>6</v>
       </c>
     </row>
     <row r="229" spans="1:5">
@@ -6075,10 +6069,10 @@
         <v>228</v>
       </c>
       <c r="D229" t="s">
-        <v>396</v>
+        <v>395</v>
       </c>
       <c r="E229">
-        <v>6</v>
+        <v>8</v>
       </c>
     </row>
     <row r="230" spans="1:5">
@@ -6092,10 +6086,10 @@
         <v>229</v>
       </c>
       <c r="D230" t="s">
-        <v>397</v>
+        <v>396</v>
       </c>
       <c r="E230">
-        <v>8</v>
+        <v>10</v>
       </c>
     </row>
     <row r="231" spans="1:5">
@@ -6109,7 +6103,7 @@
         <v>230</v>
       </c>
       <c r="D231" t="s">
-        <v>398</v>
+        <v>396</v>
       </c>
       <c r="E231">
         <v>10</v>
@@ -6126,10 +6120,10 @@
         <v>231</v>
       </c>
       <c r="D232" t="s">
-        <v>398</v>
+        <v>269</v>
       </c>
       <c r="E232">
-        <v>10</v>
+        <v>12</v>
       </c>
     </row>
     <row r="233" spans="1:5">
@@ -6143,7 +6137,7 @@
         <v>232</v>
       </c>
       <c r="D233" t="s">
-        <v>271</v>
+        <v>397</v>
       </c>
       <c r="E233">
         <v>12</v>
@@ -6160,10 +6154,10 @@
         <v>233</v>
       </c>
       <c r="D234" t="s">
-        <v>399</v>
+        <v>398</v>
       </c>
       <c r="E234">
-        <v>12</v>
+        <v>14</v>
       </c>
     </row>
     <row r="235" spans="1:5">
@@ -6177,10 +6171,10 @@
         <v>234</v>
       </c>
       <c r="D235" t="s">
-        <v>400</v>
+        <v>399</v>
       </c>
       <c r="E235">
-        <v>14</v>
+        <v>15</v>
       </c>
     </row>
     <row r="236" spans="1:5">
@@ -6194,26 +6188,9 @@
         <v>235</v>
       </c>
       <c r="D236" t="s">
-        <v>401</v>
+        <v>400</v>
       </c>
       <c r="E236">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="237" spans="1:5">
-      <c r="A237" t="s">
-        <v>15</v>
-      </c>
-      <c r="B237" t="s">
-        <v>38</v>
-      </c>
-      <c r="C237" t="s">
-        <v>236</v>
-      </c>
-      <c r="D237" t="s">
-        <v>402</v>
-      </c>
-      <c r="E237">
         <v>20</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualização automática: rac (09/10/2026 14:25)
</commit_message>
<xml_diff>
--- a/Coordenadoria/02_Dados_Tratados/base_rac_tratada.xlsx
+++ b/Coordenadoria/02_Dados_Tratados/base_rac_tratada.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1071" uniqueCount="401">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1091" uniqueCount="406">
   <si>
     <t>matricula</t>
   </si>
@@ -167,12 +167,12 @@
     <t>5º ETA</t>
   </si>
   <si>
+    <t>Montada</t>
+  </si>
+  <si>
     <t>Desmontada</t>
   </si>
   <si>
-    <t>Montada</t>
-  </si>
-  <si>
     <t>Sem condições</t>
   </si>
   <si>
@@ -194,18 +194,9 @@
     <t>C611008-0101</t>
   </si>
   <si>
-    <t>066-1055-00</t>
-  </si>
-  <si>
     <t>P7036368-01</t>
   </si>
   <si>
-    <t>200SGL153Q</t>
-  </si>
-  <si>
-    <t>3041153</t>
-  </si>
-  <si>
     <t>3107453-01</t>
   </si>
   <si>
@@ -725,21 +716,30 @@
     <t>2670067-1</t>
   </si>
   <si>
+    <t>3034792</t>
+  </si>
+  <si>
+    <t>MS29512-5</t>
+  </si>
+  <si>
+    <t>3122678-04</t>
+  </si>
+  <si>
+    <t>MS28773-05</t>
+  </si>
+  <si>
+    <t>3004085</t>
+  </si>
+  <si>
+    <t>3022375</t>
+  </si>
+  <si>
     <t>ALTERNATOR CONTROL UNIT ASSY</t>
   </si>
   <si>
-    <t>AUDIO CONTROL PANEL</t>
-  </si>
-  <si>
     <t>PROPELLER ASSEMBLY</t>
   </si>
   <si>
-    <t>STARTER GENERATOR</t>
-  </si>
-  <si>
-    <t>PARTS KIT,GAS TURBIN</t>
-  </si>
-  <si>
     <t>HOUSING</t>
   </si>
   <si>
@@ -1218,6 +1218,21 @@
   </si>
   <si>
     <t>POST LIGHT ASS</t>
+  </si>
+  <si>
+    <t>FUEL PUMP</t>
+  </si>
+  <si>
+    <t>O-RING</t>
+  </si>
+  <si>
+    <t>FUEL CONTROL UNIT</t>
+  </si>
+  <si>
+    <t>RETAINER-PACKING BACKUP</t>
+  </si>
+  <si>
+    <t>SEAL,PLAIN</t>
   </si>
 </sst>
 </file>
@@ -1586,10 +1601,10 @@
         <v>53</v>
       </c>
       <c r="E2">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="F2">
-        <v>2</v>
+        <v>0</v>
       </c>
     </row>
     <row r="3" spans="1:6">
@@ -1600,16 +1615,16 @@
         <v>37</v>
       </c>
       <c r="C3" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="D3" t="s">
         <v>53</v>
       </c>
       <c r="E3">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F3">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="4" spans="1:6">
@@ -1620,16 +1635,16 @@
         <v>38</v>
       </c>
       <c r="C4" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="D4" t="s">
         <v>53</v>
       </c>
       <c r="E4">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F4">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="5" spans="1:6">
@@ -1640,7 +1655,7 @@
         <v>39</v>
       </c>
       <c r="C5" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="D5" t="s">
         <v>53</v>
@@ -1660,7 +1675,7 @@
         <v>40</v>
       </c>
       <c r="C6" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="D6" t="s">
         <v>54</v>
@@ -1680,7 +1695,7 @@
         <v>39</v>
       </c>
       <c r="C7" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="D7" t="s">
         <v>53</v>
@@ -1700,7 +1715,7 @@
         <v>40</v>
       </c>
       <c r="C8" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="D8" t="s">
         <v>54</v>
@@ -1720,16 +1735,16 @@
         <v>41</v>
       </c>
       <c r="C9" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="D9" t="s">
         <v>53</v>
       </c>
       <c r="E9">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F9">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="10" spans="1:6">
@@ -1740,7 +1755,7 @@
         <v>40</v>
       </c>
       <c r="C10" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="D10" t="s">
         <v>54</v>
@@ -1760,7 +1775,7 @@
         <v>38</v>
       </c>
       <c r="C11" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="D11" t="s">
         <v>54</v>
@@ -1780,7 +1795,7 @@
         <v>39</v>
       </c>
       <c r="C12" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="D12" t="s">
         <v>53</v>
@@ -1800,7 +1815,7 @@
         <v>42</v>
       </c>
       <c r="C13" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="D13" t="s">
         <v>53</v>
@@ -1820,7 +1835,7 @@
         <v>39</v>
       </c>
       <c r="C14" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="D14" t="s">
         <v>53</v>
@@ -1840,7 +1855,7 @@
         <v>37</v>
       </c>
       <c r="C15" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="D15" t="s">
         <v>53</v>
@@ -1860,7 +1875,7 @@
         <v>43</v>
       </c>
       <c r="C16" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="D16" t="s">
         <v>53</v>
@@ -1880,7 +1895,7 @@
         <v>37</v>
       </c>
       <c r="C17" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="D17" t="s">
         <v>53</v>
@@ -1900,7 +1915,7 @@
         <v>43</v>
       </c>
       <c r="C18" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="D18" t="s">
         <v>53</v>
@@ -1920,7 +1935,7 @@
         <v>44</v>
       </c>
       <c r="C19" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="D19" t="s">
         <v>53</v>
@@ -1940,7 +1955,7 @@
         <v>38</v>
       </c>
       <c r="C20" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="D20" t="s">
         <v>53</v>
@@ -1966,10 +1981,10 @@
         <v>53</v>
       </c>
       <c r="E21">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="F21">
-        <v>0</v>
+        <v>8</v>
       </c>
     </row>
     <row r="22" spans="1:6">
@@ -1980,7 +1995,7 @@
         <v>40</v>
       </c>
       <c r="C22" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="D22" t="s">
         <v>53</v>
@@ -2000,7 +2015,7 @@
         <v>40</v>
       </c>
       <c r="C23" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="D23" t="s">
         <v>53</v>
@@ -2020,7 +2035,7 @@
         <v>46</v>
       </c>
       <c r="C24" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="D24" t="s">
         <v>53</v>
@@ -2040,7 +2055,7 @@
         <v>40</v>
       </c>
       <c r="C25" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="D25" t="s">
         <v>53</v>
@@ -2060,7 +2075,7 @@
         <v>47</v>
       </c>
       <c r="C26" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="D26" t="s">
         <v>53</v>
@@ -2080,7 +2095,7 @@
         <v>48</v>
       </c>
       <c r="C27" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="D27" t="s">
         <v>53</v>
@@ -2100,7 +2115,7 @@
         <v>49</v>
       </c>
       <c r="C28" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="D28" t="s">
         <v>53</v>
@@ -2179,7 +2194,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E236"/>
+  <dimension ref="A1:E241"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:5">
@@ -2201,16 +2216,16 @@
     </row>
     <row r="2" spans="1:5">
       <c r="A2" t="s">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="B2" t="s">
-        <v>36</v>
+        <v>39</v>
       </c>
       <c r="C2" t="s">
         <v>58</v>
       </c>
       <c r="D2" t="s">
-        <v>236</v>
+        <v>239</v>
       </c>
       <c r="E2">
         <v>1</v>
@@ -2218,16 +2233,16 @@
     </row>
     <row r="3" spans="1:5">
       <c r="A3" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="B3" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="C3" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="D3" t="s">
-        <v>236</v>
+        <v>240</v>
       </c>
       <c r="E3">
         <v>1</v>
@@ -2235,16 +2250,16 @@
     </row>
     <row r="4" spans="1:5">
       <c r="A4" t="s">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="B4" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="C4" t="s">
         <v>59</v>
       </c>
       <c r="D4" t="s">
-        <v>237</v>
+        <v>240</v>
       </c>
       <c r="E4">
         <v>1</v>
@@ -2252,16 +2267,16 @@
     </row>
     <row r="5" spans="1:5">
       <c r="A5" t="s">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="B5" t="s">
-        <v>37</v>
+        <v>40</v>
       </c>
       <c r="C5" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="D5" t="s">
-        <v>238</v>
+        <v>240</v>
       </c>
       <c r="E5">
         <v>1</v>
@@ -2269,16 +2284,16 @@
     </row>
     <row r="6" spans="1:5">
       <c r="A6" t="s">
-        <v>8</v>
+        <v>11</v>
       </c>
       <c r="B6" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="C6" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="D6" t="s">
-        <v>238</v>
+        <v>240</v>
       </c>
       <c r="E6">
         <v>1</v>
@@ -2286,16 +2301,16 @@
     </row>
     <row r="7" spans="1:5">
       <c r="A7" t="s">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="B7" t="s">
         <v>40</v>
       </c>
       <c r="C7" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="D7" t="s">
-        <v>238</v>
+        <v>240</v>
       </c>
       <c r="E7">
         <v>1</v>
@@ -2303,16 +2318,16 @@
     </row>
     <row r="8" spans="1:5">
       <c r="A8" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="B8" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="C8" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="D8" t="s">
-        <v>238</v>
+        <v>240</v>
       </c>
       <c r="E8">
         <v>1</v>
@@ -2320,16 +2335,16 @@
     </row>
     <row r="9" spans="1:5">
       <c r="A9" t="s">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="B9" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="C9" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="D9" t="s">
-        <v>238</v>
+        <v>240</v>
       </c>
       <c r="E9">
         <v>1</v>
@@ -2337,16 +2352,16 @@
     </row>
     <row r="10" spans="1:5">
       <c r="A10" t="s">
-        <v>14</v>
+        <v>9</v>
       </c>
       <c r="B10" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="C10" t="s">
         <v>60</v>
       </c>
       <c r="D10" t="s">
-        <v>238</v>
+        <v>241</v>
       </c>
       <c r="E10">
         <v>1</v>
@@ -2354,16 +2369,16 @@
     </row>
     <row r="11" spans="1:5">
       <c r="A11" t="s">
-        <v>15</v>
+        <v>9</v>
       </c>
       <c r="B11" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="C11" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="D11" t="s">
-        <v>238</v>
+        <v>242</v>
       </c>
       <c r="E11">
         <v>1</v>
@@ -2371,16 +2386,16 @@
     </row>
     <row r="12" spans="1:5">
       <c r="A12" t="s">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="B12" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="C12" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="D12" t="s">
-        <v>239</v>
+        <v>243</v>
       </c>
       <c r="E12">
         <v>1</v>
@@ -2388,16 +2403,16 @@
     </row>
     <row r="13" spans="1:5">
       <c r="A13" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="B13" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="C13" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="D13" t="s">
-        <v>240</v>
+        <v>244</v>
       </c>
       <c r="E13">
         <v>1</v>
@@ -2411,10 +2426,10 @@
         <v>39</v>
       </c>
       <c r="C14" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="D14" t="s">
-        <v>241</v>
+        <v>245</v>
       </c>
       <c r="E14">
         <v>1</v>
@@ -2422,16 +2437,16 @@
     </row>
     <row r="15" spans="1:5">
       <c r="A15" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="B15" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="C15" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="D15" t="s">
-        <v>242</v>
+        <v>246</v>
       </c>
       <c r="E15">
         <v>1</v>
@@ -2439,7 +2454,7 @@
     </row>
     <row r="16" spans="1:5">
       <c r="A16" t="s">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="B16" t="s">
         <v>39</v>
@@ -2448,7 +2463,7 @@
         <v>65</v>
       </c>
       <c r="D16" t="s">
-        <v>243</v>
+        <v>246</v>
       </c>
       <c r="E16">
         <v>1</v>
@@ -2456,16 +2471,16 @@
     </row>
     <row r="17" spans="1:5">
       <c r="A17" t="s">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="B17" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="C17" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="D17" t="s">
-        <v>244</v>
+        <v>246</v>
       </c>
       <c r="E17">
         <v>1</v>
@@ -2473,16 +2488,16 @@
     </row>
     <row r="18" spans="1:5">
       <c r="A18" t="s">
-        <v>9</v>
+        <v>14</v>
       </c>
       <c r="B18" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="C18" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="D18" t="s">
-        <v>245</v>
+        <v>246</v>
       </c>
       <c r="E18">
         <v>1</v>
@@ -2490,13 +2505,13 @@
     </row>
     <row r="19" spans="1:5">
       <c r="A19" t="s">
-        <v>10</v>
+        <v>15</v>
       </c>
       <c r="B19" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="C19" t="s">
-        <v>68</v>
+        <v>65</v>
       </c>
       <c r="D19" t="s">
         <v>246</v>
@@ -2507,16 +2522,16 @@
     </row>
     <row r="20" spans="1:5">
       <c r="A20" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B20" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="C20" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
       <c r="D20" t="s">
-        <v>246</v>
+        <v>247</v>
       </c>
       <c r="E20">
         <v>1</v>
@@ -2524,16 +2539,16 @@
     </row>
     <row r="21" spans="1:5">
       <c r="A21" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="B21" t="s">
         <v>40</v>
       </c>
       <c r="C21" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
       <c r="D21" t="s">
-        <v>246</v>
+        <v>247</v>
       </c>
       <c r="E21">
         <v>1</v>
@@ -2541,16 +2556,16 @@
     </row>
     <row r="22" spans="1:5">
       <c r="A22" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="B22" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="C22" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="D22" t="s">
-        <v>246</v>
+        <v>248</v>
       </c>
       <c r="E22">
         <v>1</v>
@@ -2558,16 +2573,16 @@
     </row>
     <row r="23" spans="1:5">
       <c r="A23" t="s">
-        <v>15</v>
+        <v>12</v>
       </c>
       <c r="B23" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="C23" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="D23" t="s">
-        <v>246</v>
+        <v>248</v>
       </c>
       <c r="E23">
         <v>1</v>
@@ -2575,16 +2590,16 @@
     </row>
     <row r="24" spans="1:5">
       <c r="A24" t="s">
-        <v>10</v>
+        <v>14</v>
       </c>
       <c r="B24" t="s">
         <v>40</v>
       </c>
       <c r="C24" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="D24" t="s">
-        <v>247</v>
+        <v>248</v>
       </c>
       <c r="E24">
         <v>1</v>
@@ -2592,16 +2607,16 @@
     </row>
     <row r="25" spans="1:5">
       <c r="A25" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="B25" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="C25" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="D25" t="s">
-        <v>247</v>
+        <v>249</v>
       </c>
       <c r="E25">
         <v>1</v>
@@ -2609,16 +2624,16 @@
     </row>
     <row r="26" spans="1:5">
       <c r="A26" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B26" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="C26" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="D26" t="s">
-        <v>248</v>
+        <v>249</v>
       </c>
       <c r="E26">
         <v>1</v>
@@ -2626,16 +2641,16 @@
     </row>
     <row r="27" spans="1:5">
       <c r="A27" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="B27" t="s">
         <v>40</v>
       </c>
       <c r="C27" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="D27" t="s">
-        <v>248</v>
+        <v>249</v>
       </c>
       <c r="E27">
         <v>1</v>
@@ -2643,16 +2658,16 @@
     </row>
     <row r="28" spans="1:5">
       <c r="A28" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="B28" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="C28" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="D28" t="s">
-        <v>248</v>
+        <v>250</v>
       </c>
       <c r="E28">
         <v>1</v>
@@ -2660,16 +2675,16 @@
     </row>
     <row r="29" spans="1:5">
       <c r="A29" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B29" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="C29" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="D29" t="s">
-        <v>249</v>
+        <v>250</v>
       </c>
       <c r="E29">
         <v>1</v>
@@ -2677,16 +2692,16 @@
     </row>
     <row r="30" spans="1:5">
       <c r="A30" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B30" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="C30" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="D30" t="s">
-        <v>249</v>
+        <v>251</v>
       </c>
       <c r="E30">
         <v>1</v>
@@ -2700,10 +2715,10 @@
         <v>40</v>
       </c>
       <c r="C31" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="D31" t="s">
-        <v>249</v>
+        <v>251</v>
       </c>
       <c r="E31">
         <v>1</v>
@@ -2711,16 +2726,16 @@
     </row>
     <row r="32" spans="1:5">
       <c r="A32" t="s">
-        <v>11</v>
+        <v>15</v>
       </c>
       <c r="B32" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="C32" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
       <c r="D32" t="s">
-        <v>250</v>
+        <v>251</v>
       </c>
       <c r="E32">
         <v>1</v>
@@ -2728,16 +2743,16 @@
     </row>
     <row r="33" spans="1:5">
       <c r="A33" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B33" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="C33" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="D33" t="s">
-        <v>250</v>
+        <v>252</v>
       </c>
       <c r="E33">
         <v>1</v>
@@ -2745,33 +2760,33 @@
     </row>
     <row r="34" spans="1:5">
       <c r="A34" t="s">
-        <v>11</v>
+        <v>15</v>
       </c>
       <c r="B34" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="C34" t="s">
-        <v>73</v>
+        <v>71</v>
       </c>
       <c r="D34" t="s">
-        <v>251</v>
+        <v>252</v>
       </c>
       <c r="E34">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="35" spans="1:5">
       <c r="A35" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="B35" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="C35" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="D35" t="s">
-        <v>251</v>
+        <v>253</v>
       </c>
       <c r="E35">
         <v>1</v>
@@ -2779,16 +2794,16 @@
     </row>
     <row r="36" spans="1:5">
       <c r="A36" t="s">
-        <v>15</v>
+        <v>11</v>
       </c>
       <c r="B36" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="C36" t="s">
         <v>73</v>
       </c>
       <c r="D36" t="s">
-        <v>251</v>
+        <v>254</v>
       </c>
       <c r="E36">
         <v>1</v>
@@ -2805,7 +2820,7 @@
         <v>74</v>
       </c>
       <c r="D37" t="s">
-        <v>252</v>
+        <v>255</v>
       </c>
       <c r="E37">
         <v>1</v>
@@ -2813,19 +2828,19 @@
     </row>
     <row r="38" spans="1:5">
       <c r="A38" t="s">
-        <v>15</v>
+        <v>11</v>
       </c>
       <c r="B38" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="C38" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="D38" t="s">
-        <v>252</v>
+        <v>256</v>
       </c>
       <c r="E38">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="39" spans="1:5">
@@ -2836,10 +2851,10 @@
         <v>39</v>
       </c>
       <c r="C39" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="D39" t="s">
-        <v>253</v>
+        <v>257</v>
       </c>
       <c r="E39">
         <v>1</v>
@@ -2853,10 +2868,10 @@
         <v>39</v>
       </c>
       <c r="C40" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="D40" t="s">
-        <v>254</v>
+        <v>258</v>
       </c>
       <c r="E40">
         <v>1</v>
@@ -2870,10 +2885,10 @@
         <v>39</v>
       </c>
       <c r="C41" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="D41" t="s">
-        <v>255</v>
+        <v>259</v>
       </c>
       <c r="E41">
         <v>1</v>
@@ -2887,10 +2902,10 @@
         <v>39</v>
       </c>
       <c r="C42" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="D42" t="s">
-        <v>256</v>
+        <v>260</v>
       </c>
       <c r="E42">
         <v>1</v>
@@ -2904,64 +2919,64 @@
         <v>39</v>
       </c>
       <c r="C43" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="D43" t="s">
-        <v>257</v>
+        <v>261</v>
       </c>
       <c r="E43">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="44" spans="1:5">
       <c r="A44" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B44" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="C44" t="s">
         <v>80</v>
       </c>
       <c r="D44" t="s">
-        <v>258</v>
+        <v>261</v>
       </c>
       <c r="E44">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="45" spans="1:5">
       <c r="A45" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="B45" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="C45" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="D45" t="s">
-        <v>259</v>
+        <v>261</v>
       </c>
       <c r="E45">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="46" spans="1:5">
       <c r="A46" t="s">
-        <v>11</v>
+        <v>15</v>
       </c>
       <c r="B46" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="C46" t="s">
-        <v>82</v>
+        <v>80</v>
       </c>
       <c r="D46" t="s">
-        <v>260</v>
+        <v>261</v>
       </c>
       <c r="E46">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="47" spans="1:5">
@@ -2972,10 +2987,10 @@
         <v>39</v>
       </c>
       <c r="C47" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="D47" t="s">
-        <v>261</v>
+        <v>262</v>
       </c>
       <c r="E47">
         <v>2</v>
@@ -2983,50 +2998,50 @@
     </row>
     <row r="48" spans="1:5">
       <c r="A48" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="B48" t="s">
         <v>40</v>
       </c>
       <c r="C48" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="D48" t="s">
-        <v>261</v>
+        <v>262</v>
       </c>
       <c r="E48">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="49" spans="1:5">
       <c r="A49" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="B49" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="C49" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="D49" t="s">
-        <v>261</v>
+        <v>262</v>
       </c>
       <c r="E49">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="50" spans="1:5">
       <c r="A50" t="s">
-        <v>15</v>
+        <v>11</v>
       </c>
       <c r="B50" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="C50" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="D50" t="s">
-        <v>261</v>
+        <v>263</v>
       </c>
       <c r="E50">
         <v>2</v>
@@ -3034,33 +3049,33 @@
     </row>
     <row r="51" spans="1:5">
       <c r="A51" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="B51" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="C51" t="s">
-        <v>84</v>
+        <v>82</v>
       </c>
       <c r="D51" t="s">
-        <v>262</v>
+        <v>263</v>
       </c>
       <c r="E51">
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
     <row r="52" spans="1:5">
       <c r="A52" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="B52" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="C52" t="s">
-        <v>84</v>
+        <v>82</v>
       </c>
       <c r="D52" t="s">
-        <v>262</v>
+        <v>263</v>
       </c>
       <c r="E52">
         <v>2</v>
@@ -3068,67 +3083,67 @@
     </row>
     <row r="53" spans="1:5">
       <c r="A53" t="s">
-        <v>15</v>
+        <v>11</v>
       </c>
       <c r="B53" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="C53" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="D53" t="s">
-        <v>262</v>
+        <v>264</v>
       </c>
       <c r="E53">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="54" spans="1:5">
       <c r="A54" t="s">
-        <v>11</v>
+        <v>15</v>
       </c>
       <c r="B54" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="C54" t="s">
-        <v>85</v>
+        <v>83</v>
       </c>
       <c r="D54" t="s">
-        <v>263</v>
+        <v>264</v>
       </c>
       <c r="E54">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="55" spans="1:5">
       <c r="A55" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="B55" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="C55" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="D55" t="s">
-        <v>263</v>
+        <v>265</v>
       </c>
       <c r="E55">
-        <v>4</v>
+        <v>2</v>
       </c>
     </row>
     <row r="56" spans="1:5">
       <c r="A56" t="s">
-        <v>15</v>
+        <v>11</v>
       </c>
       <c r="B56" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="C56" t="s">
         <v>85</v>
       </c>
       <c r="D56" t="s">
-        <v>263</v>
+        <v>266</v>
       </c>
       <c r="E56">
         <v>2</v>
@@ -3145,7 +3160,7 @@
         <v>86</v>
       </c>
       <c r="D57" t="s">
-        <v>264</v>
+        <v>267</v>
       </c>
       <c r="E57">
         <v>2</v>
@@ -3153,19 +3168,19 @@
     </row>
     <row r="58" spans="1:5">
       <c r="A58" t="s">
-        <v>15</v>
+        <v>11</v>
       </c>
       <c r="B58" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="C58" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="D58" t="s">
-        <v>264</v>
+        <v>268</v>
       </c>
       <c r="E58">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="59" spans="1:5">
@@ -3176,10 +3191,10 @@
         <v>39</v>
       </c>
       <c r="C59" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="D59" t="s">
-        <v>265</v>
+        <v>269</v>
       </c>
       <c r="E59">
         <v>2</v>
@@ -3193,10 +3208,10 @@
         <v>39</v>
       </c>
       <c r="C60" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="D60" t="s">
-        <v>266</v>
+        <v>270</v>
       </c>
       <c r="E60">
         <v>2</v>
@@ -3210,10 +3225,10 @@
         <v>39</v>
       </c>
       <c r="C61" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="D61" t="s">
-        <v>267</v>
+        <v>271</v>
       </c>
       <c r="E61">
         <v>2</v>
@@ -3227,10 +3242,10 @@
         <v>39</v>
       </c>
       <c r="C62" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="D62" t="s">
-        <v>268</v>
+        <v>261</v>
       </c>
       <c r="E62">
         <v>2</v>
@@ -3244,30 +3259,30 @@
         <v>39</v>
       </c>
       <c r="C63" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="D63" t="s">
-        <v>269</v>
+        <v>260</v>
       </c>
       <c r="E63">
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
     <row r="64" spans="1:5">
       <c r="A64" t="s">
-        <v>11</v>
+        <v>15</v>
       </c>
       <c r="B64" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="C64" t="s">
         <v>92</v>
       </c>
       <c r="D64" t="s">
-        <v>270</v>
+        <v>260</v>
       </c>
       <c r="E64">
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
     <row r="65" spans="1:5">
@@ -3281,10 +3296,10 @@
         <v>93</v>
       </c>
       <c r="D65" t="s">
-        <v>271</v>
+        <v>272</v>
       </c>
       <c r="E65">
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
     <row r="66" spans="1:5">
@@ -3298,10 +3313,10 @@
         <v>94</v>
       </c>
       <c r="D66" t="s">
-        <v>261</v>
+        <v>273</v>
       </c>
       <c r="E66">
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
     <row r="67" spans="1:5">
@@ -3315,7 +3330,7 @@
         <v>95</v>
       </c>
       <c r="D67" t="s">
-        <v>260</v>
+        <v>274</v>
       </c>
       <c r="E67">
         <v>4</v>
@@ -3323,84 +3338,84 @@
     </row>
     <row r="68" spans="1:5">
       <c r="A68" t="s">
-        <v>15</v>
+        <v>12</v>
       </c>
       <c r="B68" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="C68" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="D68" t="s">
-        <v>260</v>
+        <v>275</v>
       </c>
       <c r="E68">
-        <v>4</v>
+        <v>1</v>
       </c>
     </row>
     <row r="69" spans="1:5">
       <c r="A69" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="B69" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="C69" t="s">
         <v>96</v>
       </c>
       <c r="D69" t="s">
-        <v>272</v>
+        <v>275</v>
       </c>
       <c r="E69">
-        <v>4</v>
+        <v>1</v>
       </c>
     </row>
     <row r="70" spans="1:5">
       <c r="A70" t="s">
-        <v>11</v>
+        <v>15</v>
       </c>
       <c r="B70" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="C70" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="D70" t="s">
-        <v>273</v>
+        <v>275</v>
       </c>
       <c r="E70">
-        <v>4</v>
+        <v>1</v>
       </c>
     </row>
     <row r="71" spans="1:5">
       <c r="A71" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B71" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="C71" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="D71" t="s">
-        <v>274</v>
+        <v>276</v>
       </c>
       <c r="E71">
-        <v>4</v>
+        <v>1</v>
       </c>
     </row>
     <row r="72" spans="1:5">
       <c r="A72" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="B72" t="s">
         <v>40</v>
       </c>
       <c r="C72" t="s">
-        <v>99</v>
+        <v>97</v>
       </c>
       <c r="D72" t="s">
-        <v>275</v>
+        <v>276</v>
       </c>
       <c r="E72">
         <v>1</v>
@@ -3408,16 +3423,16 @@
     </row>
     <row r="73" spans="1:5">
       <c r="A73" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="B73" t="s">
-        <v>41</v>
+        <v>38</v>
       </c>
       <c r="C73" t="s">
-        <v>99</v>
+        <v>97</v>
       </c>
       <c r="D73" t="s">
-        <v>275</v>
+        <v>276</v>
       </c>
       <c r="E73">
         <v>1</v>
@@ -3425,16 +3440,16 @@
     </row>
     <row r="74" spans="1:5">
       <c r="A74" t="s">
-        <v>15</v>
+        <v>12</v>
       </c>
       <c r="B74" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="C74" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="D74" t="s">
-        <v>275</v>
+        <v>277</v>
       </c>
       <c r="E74">
         <v>1</v>
@@ -3442,16 +3457,16 @@
     </row>
     <row r="75" spans="1:5">
       <c r="A75" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="B75" t="s">
         <v>40</v>
       </c>
       <c r="C75" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="D75" t="s">
-        <v>276</v>
+        <v>277</v>
       </c>
       <c r="E75">
         <v>1</v>
@@ -3459,33 +3474,33 @@
     </row>
     <row r="76" spans="1:5">
       <c r="A76" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="B76" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="C76" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="D76" t="s">
-        <v>276</v>
+        <v>277</v>
       </c>
       <c r="E76">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="77" spans="1:5">
       <c r="A77" t="s">
-        <v>15</v>
+        <v>12</v>
       </c>
       <c r="B77" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="C77" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="D77" t="s">
-        <v>276</v>
+        <v>278</v>
       </c>
       <c r="E77">
         <v>1</v>
@@ -3493,16 +3508,16 @@
     </row>
     <row r="78" spans="1:5">
       <c r="A78" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="B78" t="s">
         <v>40</v>
       </c>
       <c r="C78" t="s">
-        <v>101</v>
+        <v>99</v>
       </c>
       <c r="D78" t="s">
-        <v>277</v>
+        <v>278</v>
       </c>
       <c r="E78">
         <v>1</v>
@@ -3510,16 +3525,16 @@
     </row>
     <row r="79" spans="1:5">
       <c r="A79" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="B79" t="s">
         <v>40</v>
       </c>
       <c r="C79" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="D79" t="s">
-        <v>277</v>
+        <v>279</v>
       </c>
       <c r="E79">
         <v>1</v>
@@ -3527,19 +3542,19 @@
     </row>
     <row r="80" spans="1:5">
       <c r="A80" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B80" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="C80" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="D80" t="s">
-        <v>277</v>
+        <v>279</v>
       </c>
       <c r="E80">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="81" spans="1:5">
@@ -3550,10 +3565,10 @@
         <v>40</v>
       </c>
       <c r="C81" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="D81" t="s">
-        <v>278</v>
+        <v>280</v>
       </c>
       <c r="E81">
         <v>1</v>
@@ -3567,10 +3582,10 @@
         <v>40</v>
       </c>
       <c r="C82" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="D82" t="s">
-        <v>278</v>
+        <v>280</v>
       </c>
       <c r="E82">
         <v>1</v>
@@ -3584,10 +3599,10 @@
         <v>40</v>
       </c>
       <c r="C83" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="D83" t="s">
-        <v>279</v>
+        <v>281</v>
       </c>
       <c r="E83">
         <v>1</v>
@@ -3601,10 +3616,10 @@
         <v>40</v>
       </c>
       <c r="C84" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="D84" t="s">
-        <v>279</v>
+        <v>281</v>
       </c>
       <c r="E84">
         <v>1</v>
@@ -3618,10 +3633,10 @@
         <v>40</v>
       </c>
       <c r="C85" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="D85" t="s">
-        <v>280</v>
+        <v>282</v>
       </c>
       <c r="E85">
         <v>1</v>
@@ -3635,10 +3650,10 @@
         <v>40</v>
       </c>
       <c r="C86" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="D86" t="s">
-        <v>280</v>
+        <v>282</v>
       </c>
       <c r="E86">
         <v>1</v>
@@ -3652,10 +3667,10 @@
         <v>40</v>
       </c>
       <c r="C87" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="D87" t="s">
-        <v>281</v>
+        <v>283</v>
       </c>
       <c r="E87">
         <v>1</v>
@@ -3669,10 +3684,10 @@
         <v>40</v>
       </c>
       <c r="C88" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="D88" t="s">
-        <v>281</v>
+        <v>283</v>
       </c>
       <c r="E88">
         <v>1</v>
@@ -3686,10 +3701,10 @@
         <v>40</v>
       </c>
       <c r="C89" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="D89" t="s">
-        <v>282</v>
+        <v>284</v>
       </c>
       <c r="E89">
         <v>1</v>
@@ -3703,10 +3718,10 @@
         <v>40</v>
       </c>
       <c r="C90" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="D90" t="s">
-        <v>282</v>
+        <v>284</v>
       </c>
       <c r="E90">
         <v>1</v>
@@ -3720,10 +3735,10 @@
         <v>40</v>
       </c>
       <c r="C91" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="D91" t="s">
-        <v>283</v>
+        <v>285</v>
       </c>
       <c r="E91">
         <v>1</v>
@@ -3731,16 +3746,16 @@
     </row>
     <row r="92" spans="1:5">
       <c r="A92" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B92" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="C92" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="D92" t="s">
-        <v>283</v>
+        <v>285</v>
       </c>
       <c r="E92">
         <v>1</v>
@@ -3748,16 +3763,16 @@
     </row>
     <row r="93" spans="1:5">
       <c r="A93" t="s">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="B93" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="C93" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
       <c r="D93" t="s">
-        <v>284</v>
+        <v>285</v>
       </c>
       <c r="E93">
         <v>1</v>
@@ -3765,16 +3780,16 @@
     </row>
     <row r="94" spans="1:5">
       <c r="A94" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="B94" t="s">
         <v>40</v>
       </c>
       <c r="C94" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="D94" t="s">
-        <v>284</v>
+        <v>286</v>
       </c>
       <c r="E94">
         <v>1</v>
@@ -3782,16 +3797,16 @@
     </row>
     <row r="95" spans="1:5">
       <c r="A95" t="s">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="B95" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="C95" t="s">
-        <v>109</v>
+        <v>107</v>
       </c>
       <c r="D95" t="s">
-        <v>285</v>
+        <v>286</v>
       </c>
       <c r="E95">
         <v>1</v>
@@ -3799,16 +3814,16 @@
     </row>
     <row r="96" spans="1:5">
       <c r="A96" t="s">
-        <v>15</v>
+        <v>12</v>
       </c>
       <c r="B96" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="C96" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="D96" t="s">
-        <v>285</v>
+        <v>287</v>
       </c>
       <c r="E96">
         <v>1</v>
@@ -3822,10 +3837,10 @@
         <v>40</v>
       </c>
       <c r="C97" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="D97" t="s">
-        <v>286</v>
+        <v>288</v>
       </c>
       <c r="E97">
         <v>1</v>
@@ -3833,16 +3848,16 @@
     </row>
     <row r="98" spans="1:5">
       <c r="A98" t="s">
-        <v>15</v>
+        <v>12</v>
       </c>
       <c r="B98" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="C98" t="s">
         <v>110</v>
       </c>
       <c r="D98" t="s">
-        <v>286</v>
+        <v>289</v>
       </c>
       <c r="E98">
         <v>1</v>
@@ -3859,7 +3874,7 @@
         <v>111</v>
       </c>
       <c r="D99" t="s">
-        <v>287</v>
+        <v>290</v>
       </c>
       <c r="E99">
         <v>1</v>
@@ -3876,7 +3891,7 @@
         <v>112</v>
       </c>
       <c r="D100" t="s">
-        <v>288</v>
+        <v>291</v>
       </c>
       <c r="E100">
         <v>1</v>
@@ -3893,7 +3908,7 @@
         <v>113</v>
       </c>
       <c r="D101" t="s">
-        <v>289</v>
+        <v>292</v>
       </c>
       <c r="E101">
         <v>1</v>
@@ -3910,24 +3925,24 @@
         <v>114</v>
       </c>
       <c r="D102" t="s">
-        <v>290</v>
+        <v>293</v>
       </c>
       <c r="E102">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="103" spans="1:5">
       <c r="A103" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="B103" t="s">
         <v>40</v>
       </c>
       <c r="C103" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="D103" t="s">
-        <v>291</v>
+        <v>293</v>
       </c>
       <c r="E103">
         <v>1</v>
@@ -3941,27 +3956,27 @@
         <v>40</v>
       </c>
       <c r="C104" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="D104" t="s">
-        <v>292</v>
+        <v>294</v>
       </c>
       <c r="E104">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="105" spans="1:5">
       <c r="A105" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="B105" t="s">
         <v>40</v>
       </c>
       <c r="C105" t="s">
-        <v>117</v>
+        <v>115</v>
       </c>
       <c r="D105" t="s">
-        <v>293</v>
+        <v>294</v>
       </c>
       <c r="E105">
         <v>2</v>
@@ -3969,19 +3984,19 @@
     </row>
     <row r="106" spans="1:5">
       <c r="A106" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="B106" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="C106" t="s">
-        <v>117</v>
+        <v>115</v>
       </c>
       <c r="D106" t="s">
-        <v>293</v>
+        <v>294</v>
       </c>
       <c r="E106">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="107" spans="1:5">
@@ -3992,10 +4007,10 @@
         <v>40</v>
       </c>
       <c r="C107" t="s">
-        <v>118</v>
+        <v>116</v>
       </c>
       <c r="D107" t="s">
-        <v>294</v>
+        <v>295</v>
       </c>
       <c r="E107">
         <v>2</v>
@@ -4009,10 +4024,10 @@
         <v>40</v>
       </c>
       <c r="C108" t="s">
-        <v>118</v>
+        <v>116</v>
       </c>
       <c r="D108" t="s">
-        <v>294</v>
+        <v>295</v>
       </c>
       <c r="E108">
         <v>2</v>
@@ -4026,10 +4041,10 @@
         <v>38</v>
       </c>
       <c r="C109" t="s">
-        <v>118</v>
+        <v>116</v>
       </c>
       <c r="D109" t="s">
-        <v>294</v>
+        <v>295</v>
       </c>
       <c r="E109">
         <v>2</v>
@@ -4043,10 +4058,10 @@
         <v>40</v>
       </c>
       <c r="C110" t="s">
-        <v>119</v>
+        <v>117</v>
       </c>
       <c r="D110" t="s">
-        <v>295</v>
+        <v>296</v>
       </c>
       <c r="E110">
         <v>2</v>
@@ -4060,10 +4075,10 @@
         <v>40</v>
       </c>
       <c r="C111" t="s">
-        <v>119</v>
+        <v>117</v>
       </c>
       <c r="D111" t="s">
-        <v>295</v>
+        <v>296</v>
       </c>
       <c r="E111">
         <v>2</v>
@@ -4071,16 +4086,16 @@
     </row>
     <row r="112" spans="1:5">
       <c r="A112" t="s">
-        <v>15</v>
+        <v>12</v>
       </c>
       <c r="B112" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="C112" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="D112" t="s">
-        <v>295</v>
+        <v>297</v>
       </c>
       <c r="E112">
         <v>2</v>
@@ -4088,16 +4103,16 @@
     </row>
     <row r="113" spans="1:5">
       <c r="A113" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="B113" t="s">
         <v>40</v>
       </c>
       <c r="C113" t="s">
-        <v>120</v>
+        <v>118</v>
       </c>
       <c r="D113" t="s">
-        <v>296</v>
+        <v>297</v>
       </c>
       <c r="E113">
         <v>2</v>
@@ -4105,16 +4120,16 @@
     </row>
     <row r="114" spans="1:5">
       <c r="A114" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="B114" t="s">
         <v>40</v>
       </c>
       <c r="C114" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="D114" t="s">
-        <v>296</v>
+        <v>277</v>
       </c>
       <c r="E114">
         <v>2</v>
@@ -4122,36 +4137,36 @@
     </row>
     <row r="115" spans="1:5">
       <c r="A115" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="B115" t="s">
         <v>40</v>
       </c>
       <c r="C115" t="s">
-        <v>121</v>
+        <v>119</v>
       </c>
       <c r="D115" t="s">
-        <v>297</v>
+        <v>277</v>
       </c>
       <c r="E115">
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
     <row r="116" spans="1:5">
       <c r="A116" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="B116" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="C116" t="s">
-        <v>121</v>
+        <v>119</v>
       </c>
       <c r="D116" t="s">
-        <v>297</v>
+        <v>277</v>
       </c>
       <c r="E116">
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
     <row r="117" spans="1:5">
@@ -4162,10 +4177,10 @@
         <v>40</v>
       </c>
       <c r="C117" t="s">
-        <v>122</v>
+        <v>120</v>
       </c>
       <c r="D117" t="s">
-        <v>277</v>
+        <v>298</v>
       </c>
       <c r="E117">
         <v>2</v>
@@ -4179,10 +4194,10 @@
         <v>40</v>
       </c>
       <c r="C118" t="s">
-        <v>122</v>
+        <v>120</v>
       </c>
       <c r="D118" t="s">
-        <v>277</v>
+        <v>298</v>
       </c>
       <c r="E118">
         <v>4</v>
@@ -4190,19 +4205,19 @@
     </row>
     <row r="119" spans="1:5">
       <c r="A119" t="s">
-        <v>15</v>
+        <v>12</v>
       </c>
       <c r="B119" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="C119" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="D119" t="s">
-        <v>277</v>
+        <v>283</v>
       </c>
       <c r="E119">
-        <v>4</v>
+        <v>2</v>
       </c>
     </row>
     <row r="120" spans="1:5">
@@ -4213,10 +4228,10 @@
         <v>40</v>
       </c>
       <c r="C120" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="D120" t="s">
-        <v>298</v>
+        <v>299</v>
       </c>
       <c r="E120">
         <v>2</v>
@@ -4224,7 +4239,7 @@
     </row>
     <row r="121" spans="1:5">
       <c r="A121" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="B121" t="s">
         <v>40</v>
@@ -4233,10 +4248,10 @@
         <v>123</v>
       </c>
       <c r="D121" t="s">
-        <v>298</v>
+        <v>300</v>
       </c>
       <c r="E121">
-        <v>4</v>
+        <v>2</v>
       </c>
     </row>
     <row r="122" spans="1:5">
@@ -4250,27 +4265,27 @@
         <v>124</v>
       </c>
       <c r="D122" t="s">
-        <v>283</v>
+        <v>301</v>
       </c>
       <c r="E122">
-        <v>2</v>
+        <v>5</v>
       </c>
     </row>
     <row r="123" spans="1:5">
       <c r="A123" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="B123" t="s">
         <v>40</v>
       </c>
       <c r="C123" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="D123" t="s">
-        <v>299</v>
+        <v>301</v>
       </c>
       <c r="E123">
-        <v>2</v>
+        <v>5</v>
       </c>
     </row>
     <row r="124" spans="1:5">
@@ -4281,13 +4296,13 @@
         <v>40</v>
       </c>
       <c r="C124" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="D124" t="s">
-        <v>300</v>
+        <v>302</v>
       </c>
       <c r="E124">
-        <v>2</v>
+        <v>7</v>
       </c>
     </row>
     <row r="125" spans="1:5">
@@ -4298,18 +4313,18 @@
         <v>40</v>
       </c>
       <c r="C125" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="D125" t="s">
-        <v>301</v>
+        <v>303</v>
       </c>
       <c r="E125">
-        <v>5</v>
+        <v>10</v>
       </c>
     </row>
     <row r="126" spans="1:5">
       <c r="A126" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="B126" t="s">
         <v>40</v>
@@ -4318,61 +4333,61 @@
         <v>127</v>
       </c>
       <c r="D126" t="s">
-        <v>301</v>
+        <v>304</v>
       </c>
       <c r="E126">
-        <v>5</v>
+        <v>30</v>
       </c>
     </row>
     <row r="127" spans="1:5">
       <c r="A127" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="B127" t="s">
         <v>40</v>
       </c>
       <c r="C127" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="D127" t="s">
-        <v>302</v>
+        <v>304</v>
       </c>
       <c r="E127">
-        <v>7</v>
+        <v>30</v>
       </c>
     </row>
     <row r="128" spans="1:5">
       <c r="A128" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="B128" t="s">
         <v>40</v>
       </c>
       <c r="C128" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="D128" t="s">
-        <v>303</v>
+        <v>305</v>
       </c>
       <c r="E128">
-        <v>10</v>
+        <v>1</v>
       </c>
     </row>
     <row r="129" spans="1:5">
       <c r="A129" t="s">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="B129" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="C129" t="s">
-        <v>130</v>
+        <v>128</v>
       </c>
       <c r="D129" t="s">
-        <v>304</v>
+        <v>305</v>
       </c>
       <c r="E129">
-        <v>30</v>
+        <v>1</v>
       </c>
     </row>
     <row r="130" spans="1:5">
@@ -4383,13 +4398,13 @@
         <v>40</v>
       </c>
       <c r="C130" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="D130" t="s">
-        <v>304</v>
+        <v>306</v>
       </c>
       <c r="E130">
-        <v>30</v>
+        <v>1</v>
       </c>
     </row>
     <row r="131" spans="1:5">
@@ -4400,10 +4415,10 @@
         <v>40</v>
       </c>
       <c r="C131" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="D131" t="s">
-        <v>305</v>
+        <v>307</v>
       </c>
       <c r="E131">
         <v>1</v>
@@ -4411,16 +4426,16 @@
     </row>
     <row r="132" spans="1:5">
       <c r="A132" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B132" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="C132" t="s">
         <v>131</v>
       </c>
       <c r="D132" t="s">
-        <v>305</v>
+        <v>308</v>
       </c>
       <c r="E132">
         <v>1</v>
@@ -4437,7 +4452,7 @@
         <v>132</v>
       </c>
       <c r="D133" t="s">
-        <v>306</v>
+        <v>309</v>
       </c>
       <c r="E133">
         <v>1</v>
@@ -4454,7 +4469,7 @@
         <v>133</v>
       </c>
       <c r="D134" t="s">
-        <v>307</v>
+        <v>310</v>
       </c>
       <c r="E134">
         <v>1</v>
@@ -4471,7 +4486,7 @@
         <v>134</v>
       </c>
       <c r="D135" t="s">
-        <v>308</v>
+        <v>311</v>
       </c>
       <c r="E135">
         <v>1</v>
@@ -4488,7 +4503,7 @@
         <v>135</v>
       </c>
       <c r="D136" t="s">
-        <v>309</v>
+        <v>312</v>
       </c>
       <c r="E136">
         <v>1</v>
@@ -4505,7 +4520,7 @@
         <v>136</v>
       </c>
       <c r="D137" t="s">
-        <v>310</v>
+        <v>313</v>
       </c>
       <c r="E137">
         <v>1</v>
@@ -4522,7 +4537,7 @@
         <v>137</v>
       </c>
       <c r="D138" t="s">
-        <v>311</v>
+        <v>314</v>
       </c>
       <c r="E138">
         <v>1</v>
@@ -4539,7 +4554,7 @@
         <v>138</v>
       </c>
       <c r="D139" t="s">
-        <v>312</v>
+        <v>315</v>
       </c>
       <c r="E139">
         <v>1</v>
@@ -4556,7 +4571,7 @@
         <v>139</v>
       </c>
       <c r="D140" t="s">
-        <v>313</v>
+        <v>316</v>
       </c>
       <c r="E140">
         <v>1</v>
@@ -4573,7 +4588,7 @@
         <v>140</v>
       </c>
       <c r="D141" t="s">
-        <v>314</v>
+        <v>317</v>
       </c>
       <c r="E141">
         <v>1</v>
@@ -4590,7 +4605,7 @@
         <v>141</v>
       </c>
       <c r="D142" t="s">
-        <v>315</v>
+        <v>318</v>
       </c>
       <c r="E142">
         <v>1</v>
@@ -4607,7 +4622,7 @@
         <v>142</v>
       </c>
       <c r="D143" t="s">
-        <v>316</v>
+        <v>319</v>
       </c>
       <c r="E143">
         <v>1</v>
@@ -4624,7 +4639,7 @@
         <v>143</v>
       </c>
       <c r="D144" t="s">
-        <v>317</v>
+        <v>320</v>
       </c>
       <c r="E144">
         <v>1</v>
@@ -4641,7 +4656,7 @@
         <v>144</v>
       </c>
       <c r="D145" t="s">
-        <v>318</v>
+        <v>321</v>
       </c>
       <c r="E145">
         <v>1</v>
@@ -4658,7 +4673,7 @@
         <v>145</v>
       </c>
       <c r="D146" t="s">
-        <v>319</v>
+        <v>322</v>
       </c>
       <c r="E146">
         <v>1</v>
@@ -4675,7 +4690,7 @@
         <v>146</v>
       </c>
       <c r="D147" t="s">
-        <v>320</v>
+        <v>323</v>
       </c>
       <c r="E147">
         <v>1</v>
@@ -4692,7 +4707,7 @@
         <v>147</v>
       </c>
       <c r="D148" t="s">
-        <v>321</v>
+        <v>324</v>
       </c>
       <c r="E148">
         <v>1</v>
@@ -4709,7 +4724,7 @@
         <v>148</v>
       </c>
       <c r="D149" t="s">
-        <v>322</v>
+        <v>325</v>
       </c>
       <c r="E149">
         <v>1</v>
@@ -4726,7 +4741,7 @@
         <v>149</v>
       </c>
       <c r="D150" t="s">
-        <v>323</v>
+        <v>326</v>
       </c>
       <c r="E150">
         <v>1</v>
@@ -4743,7 +4758,7 @@
         <v>150</v>
       </c>
       <c r="D151" t="s">
-        <v>324</v>
+        <v>327</v>
       </c>
       <c r="E151">
         <v>1</v>
@@ -4760,7 +4775,7 @@
         <v>151</v>
       </c>
       <c r="D152" t="s">
-        <v>325</v>
+        <v>328</v>
       </c>
       <c r="E152">
         <v>1</v>
@@ -4777,7 +4792,7 @@
         <v>152</v>
       </c>
       <c r="D153" t="s">
-        <v>326</v>
+        <v>329</v>
       </c>
       <c r="E153">
         <v>1</v>
@@ -4794,7 +4809,7 @@
         <v>153</v>
       </c>
       <c r="D154" t="s">
-        <v>327</v>
+        <v>330</v>
       </c>
       <c r="E154">
         <v>1</v>
@@ -4811,7 +4826,7 @@
         <v>154</v>
       </c>
       <c r="D155" t="s">
-        <v>328</v>
+        <v>331</v>
       </c>
       <c r="E155">
         <v>1</v>
@@ -4828,7 +4843,7 @@
         <v>155</v>
       </c>
       <c r="D156" t="s">
-        <v>329</v>
+        <v>332</v>
       </c>
       <c r="E156">
         <v>1</v>
@@ -4845,7 +4860,7 @@
         <v>156</v>
       </c>
       <c r="D157" t="s">
-        <v>330</v>
+        <v>333</v>
       </c>
       <c r="E157">
         <v>1</v>
@@ -4862,7 +4877,7 @@
         <v>157</v>
       </c>
       <c r="D158" t="s">
-        <v>331</v>
+        <v>334</v>
       </c>
       <c r="E158">
         <v>1</v>
@@ -4879,7 +4894,7 @@
         <v>158</v>
       </c>
       <c r="D159" t="s">
-        <v>332</v>
+        <v>335</v>
       </c>
       <c r="E159">
         <v>1</v>
@@ -4896,7 +4911,7 @@
         <v>159</v>
       </c>
       <c r="D160" t="s">
-        <v>333</v>
+        <v>336</v>
       </c>
       <c r="E160">
         <v>1</v>
@@ -4913,7 +4928,7 @@
         <v>160</v>
       </c>
       <c r="D161" t="s">
-        <v>334</v>
+        <v>337</v>
       </c>
       <c r="E161">
         <v>1</v>
@@ -4930,10 +4945,10 @@
         <v>161</v>
       </c>
       <c r="D162" t="s">
-        <v>335</v>
+        <v>320</v>
       </c>
       <c r="E162">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="163" spans="1:5">
@@ -4947,10 +4962,10 @@
         <v>162</v>
       </c>
       <c r="D163" t="s">
-        <v>336</v>
+        <v>338</v>
       </c>
       <c r="E163">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="164" spans="1:5">
@@ -4964,10 +4979,10 @@
         <v>163</v>
       </c>
       <c r="D164" t="s">
-        <v>337</v>
+        <v>339</v>
       </c>
       <c r="E164">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="165" spans="1:5">
@@ -4981,7 +4996,7 @@
         <v>164</v>
       </c>
       <c r="D165" t="s">
-        <v>320</v>
+        <v>340</v>
       </c>
       <c r="E165">
         <v>2</v>
@@ -4998,7 +5013,7 @@
         <v>165</v>
       </c>
       <c r="D166" t="s">
-        <v>338</v>
+        <v>341</v>
       </c>
       <c r="E166">
         <v>2</v>
@@ -5015,10 +5030,10 @@
         <v>166</v>
       </c>
       <c r="D167" t="s">
-        <v>339</v>
+        <v>342</v>
       </c>
       <c r="E167">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="168" spans="1:5">
@@ -5032,10 +5047,10 @@
         <v>167</v>
       </c>
       <c r="D168" t="s">
-        <v>340</v>
+        <v>304</v>
       </c>
       <c r="E168">
-        <v>2</v>
+        <v>5</v>
       </c>
     </row>
     <row r="169" spans="1:5">
@@ -5049,10 +5064,10 @@
         <v>168</v>
       </c>
       <c r="D169" t="s">
-        <v>341</v>
+        <v>343</v>
       </c>
       <c r="E169">
-        <v>2</v>
+        <v>8</v>
       </c>
     </row>
     <row r="170" spans="1:5">
@@ -5066,10 +5081,10 @@
         <v>169</v>
       </c>
       <c r="D170" t="s">
-        <v>342</v>
+        <v>257</v>
       </c>
       <c r="E170">
-        <v>3</v>
+        <v>8</v>
       </c>
     </row>
     <row r="171" spans="1:5">
@@ -5083,61 +5098,61 @@
         <v>170</v>
       </c>
       <c r="D171" t="s">
-        <v>304</v>
+        <v>344</v>
       </c>
       <c r="E171">
-        <v>5</v>
+        <v>10</v>
       </c>
     </row>
     <row r="172" spans="1:5">
       <c r="A172" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="B172" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="C172" t="s">
         <v>171</v>
       </c>
       <c r="D172" t="s">
-        <v>343</v>
+        <v>330</v>
       </c>
       <c r="E172">
-        <v>8</v>
+        <v>1</v>
       </c>
     </row>
     <row r="173" spans="1:5">
       <c r="A173" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="B173" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="C173" t="s">
         <v>172</v>
       </c>
       <c r="D173" t="s">
-        <v>257</v>
+        <v>345</v>
       </c>
       <c r="E173">
-        <v>8</v>
+        <v>1</v>
       </c>
     </row>
     <row r="174" spans="1:5">
       <c r="A174" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="B174" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="C174" t="s">
         <v>173</v>
       </c>
       <c r="D174" t="s">
-        <v>344</v>
+        <v>346</v>
       </c>
       <c r="E174">
-        <v>10</v>
+        <v>1</v>
       </c>
     </row>
     <row r="175" spans="1:5">
@@ -5151,7 +5166,7 @@
         <v>174</v>
       </c>
       <c r="D175" t="s">
-        <v>330</v>
+        <v>347</v>
       </c>
       <c r="E175">
         <v>1</v>
@@ -5168,7 +5183,7 @@
         <v>175</v>
       </c>
       <c r="D176" t="s">
-        <v>345</v>
+        <v>348</v>
       </c>
       <c r="E176">
         <v>1</v>
@@ -5185,7 +5200,7 @@
         <v>176</v>
       </c>
       <c r="D177" t="s">
-        <v>346</v>
+        <v>349</v>
       </c>
       <c r="E177">
         <v>1</v>
@@ -5202,7 +5217,7 @@
         <v>177</v>
       </c>
       <c r="D178" t="s">
-        <v>347</v>
+        <v>267</v>
       </c>
       <c r="E178">
         <v>1</v>
@@ -5210,16 +5225,16 @@
     </row>
     <row r="179" spans="1:5">
       <c r="A179" t="s">
-        <v>15</v>
+        <v>7</v>
       </c>
       <c r="B179" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="C179" t="s">
         <v>178</v>
       </c>
       <c r="D179" t="s">
-        <v>348</v>
+        <v>350</v>
       </c>
       <c r="E179">
         <v>1</v>
@@ -5233,10 +5248,10 @@
         <v>38</v>
       </c>
       <c r="C180" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="D180" t="s">
-        <v>349</v>
+        <v>350</v>
       </c>
       <c r="E180">
         <v>1</v>
@@ -5250,10 +5265,10 @@
         <v>38</v>
       </c>
       <c r="C181" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="D181" t="s">
-        <v>267</v>
+        <v>351</v>
       </c>
       <c r="E181">
         <v>1</v>
@@ -5267,10 +5282,10 @@
         <v>38</v>
       </c>
       <c r="C182" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="D182" t="s">
-        <v>350</v>
+        <v>352</v>
       </c>
       <c r="E182">
         <v>1</v>
@@ -5284,10 +5299,10 @@
         <v>38</v>
       </c>
       <c r="C183" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="D183" t="s">
-        <v>351</v>
+        <v>353</v>
       </c>
       <c r="E183">
         <v>1</v>
@@ -5301,10 +5316,10 @@
         <v>38</v>
       </c>
       <c r="C184" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="D184" t="s">
-        <v>352</v>
+        <v>354</v>
       </c>
       <c r="E184">
         <v>1</v>
@@ -5318,10 +5333,10 @@
         <v>38</v>
       </c>
       <c r="C185" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="D185" t="s">
-        <v>353</v>
+        <v>355</v>
       </c>
       <c r="E185">
         <v>1</v>
@@ -5335,10 +5350,10 @@
         <v>38</v>
       </c>
       <c r="C186" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="D186" t="s">
-        <v>354</v>
+        <v>356</v>
       </c>
       <c r="E186">
         <v>1</v>
@@ -5352,10 +5367,10 @@
         <v>38</v>
       </c>
       <c r="C187" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="D187" t="s">
-        <v>355</v>
+        <v>357</v>
       </c>
       <c r="E187">
         <v>1</v>
@@ -5369,10 +5384,10 @@
         <v>38</v>
       </c>
       <c r="C188" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="D188" t="s">
-        <v>356</v>
+        <v>358</v>
       </c>
       <c r="E188">
         <v>1</v>
@@ -5386,10 +5401,10 @@
         <v>38</v>
       </c>
       <c r="C189" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="D189" t="s">
-        <v>357</v>
+        <v>359</v>
       </c>
       <c r="E189">
         <v>1</v>
@@ -5403,10 +5418,10 @@
         <v>38</v>
       </c>
       <c r="C190" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
       <c r="D190" t="s">
-        <v>358</v>
+        <v>360</v>
       </c>
       <c r="E190">
         <v>1</v>
@@ -5420,10 +5435,10 @@
         <v>38</v>
       </c>
       <c r="C191" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="D191" t="s">
-        <v>359</v>
+        <v>361</v>
       </c>
       <c r="E191">
         <v>1</v>
@@ -5437,10 +5452,10 @@
         <v>38</v>
       </c>
       <c r="C192" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="D192" t="s">
-        <v>360</v>
+        <v>362</v>
       </c>
       <c r="E192">
         <v>1</v>
@@ -5454,10 +5469,10 @@
         <v>38</v>
       </c>
       <c r="C193" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
       <c r="D193" t="s">
-        <v>361</v>
+        <v>363</v>
       </c>
       <c r="E193">
         <v>1</v>
@@ -5471,10 +5486,10 @@
         <v>38</v>
       </c>
       <c r="C194" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="D194" t="s">
-        <v>362</v>
+        <v>364</v>
       </c>
       <c r="E194">
         <v>1</v>
@@ -5488,10 +5503,10 @@
         <v>38</v>
       </c>
       <c r="C195" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="D195" t="s">
-        <v>363</v>
+        <v>365</v>
       </c>
       <c r="E195">
         <v>1</v>
@@ -5505,10 +5520,10 @@
         <v>38</v>
       </c>
       <c r="C196" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="D196" t="s">
-        <v>364</v>
+        <v>366</v>
       </c>
       <c r="E196">
         <v>1</v>
@@ -5522,10 +5537,10 @@
         <v>38</v>
       </c>
       <c r="C197" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="D197" t="s">
-        <v>365</v>
+        <v>367</v>
       </c>
       <c r="E197">
         <v>1</v>
@@ -5539,10 +5554,10 @@
         <v>38</v>
       </c>
       <c r="C198" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="D198" t="s">
-        <v>366</v>
+        <v>368</v>
       </c>
       <c r="E198">
         <v>1</v>
@@ -5556,10 +5571,10 @@
         <v>38</v>
       </c>
       <c r="C199" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="D199" t="s">
-        <v>367</v>
+        <v>369</v>
       </c>
       <c r="E199">
         <v>1</v>
@@ -5573,10 +5588,10 @@
         <v>38</v>
       </c>
       <c r="C200" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="D200" t="s">
-        <v>368</v>
+        <v>370</v>
       </c>
       <c r="E200">
         <v>1</v>
@@ -5590,10 +5605,10 @@
         <v>38</v>
       </c>
       <c r="C201" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="D201" t="s">
-        <v>369</v>
+        <v>371</v>
       </c>
       <c r="E201">
         <v>1</v>
@@ -5607,10 +5622,10 @@
         <v>38</v>
       </c>
       <c r="C202" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="D202" t="s">
-        <v>370</v>
+        <v>372</v>
       </c>
       <c r="E202">
         <v>1</v>
@@ -5624,10 +5639,10 @@
         <v>38</v>
       </c>
       <c r="C203" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
       <c r="D203" t="s">
-        <v>371</v>
+        <v>373</v>
       </c>
       <c r="E203">
         <v>1</v>
@@ -5641,10 +5656,10 @@
         <v>38</v>
       </c>
       <c r="C204" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
       <c r="D204" t="s">
-        <v>372</v>
+        <v>374</v>
       </c>
       <c r="E204">
         <v>1</v>
@@ -5658,13 +5673,13 @@
         <v>38</v>
       </c>
       <c r="C205" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="D205" t="s">
-        <v>373</v>
+        <v>375</v>
       </c>
       <c r="E205">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="206" spans="1:5">
@@ -5675,13 +5690,13 @@
         <v>38</v>
       </c>
       <c r="C206" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
       <c r="D206" t="s">
-        <v>374</v>
+        <v>376</v>
       </c>
       <c r="E206">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="207" spans="1:5">
@@ -5692,10 +5707,10 @@
         <v>38</v>
       </c>
       <c r="C207" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
       <c r="D207" t="s">
-        <v>375</v>
+        <v>377</v>
       </c>
       <c r="E207">
         <v>2</v>
@@ -5709,10 +5724,10 @@
         <v>38</v>
       </c>
       <c r="C208" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
       <c r="D208" t="s">
-        <v>376</v>
+        <v>378</v>
       </c>
       <c r="E208">
         <v>2</v>
@@ -5726,10 +5741,10 @@
         <v>38</v>
       </c>
       <c r="C209" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="D209" t="s">
-        <v>377</v>
+        <v>379</v>
       </c>
       <c r="E209">
         <v>2</v>
@@ -5743,10 +5758,10 @@
         <v>38</v>
       </c>
       <c r="C210" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="D210" t="s">
-        <v>378</v>
+        <v>380</v>
       </c>
       <c r="E210">
         <v>2</v>
@@ -5760,10 +5775,10 @@
         <v>38</v>
       </c>
       <c r="C211" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="D211" t="s">
-        <v>379</v>
+        <v>381</v>
       </c>
       <c r="E211">
         <v>2</v>
@@ -5777,10 +5792,10 @@
         <v>38</v>
       </c>
       <c r="C212" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
       <c r="D212" t="s">
-        <v>380</v>
+        <v>382</v>
       </c>
       <c r="E212">
         <v>2</v>
@@ -5794,10 +5809,10 @@
         <v>38</v>
       </c>
       <c r="C213" t="s">
-        <v>212</v>
+        <v>211</v>
       </c>
       <c r="D213" t="s">
-        <v>381</v>
+        <v>383</v>
       </c>
       <c r="E213">
         <v>2</v>
@@ -5811,10 +5826,10 @@
         <v>38</v>
       </c>
       <c r="C214" t="s">
-        <v>213</v>
+        <v>212</v>
       </c>
       <c r="D214" t="s">
-        <v>382</v>
+        <v>383</v>
       </c>
       <c r="E214">
         <v>2</v>
@@ -5828,10 +5843,10 @@
         <v>38</v>
       </c>
       <c r="C215" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
       <c r="D215" t="s">
-        <v>383</v>
+        <v>384</v>
       </c>
       <c r="E215">
         <v>2</v>
@@ -5845,10 +5860,10 @@
         <v>38</v>
       </c>
       <c r="C216" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
       <c r="D216" t="s">
-        <v>383</v>
+        <v>385</v>
       </c>
       <c r="E216">
         <v>2</v>
@@ -5862,13 +5877,13 @@
         <v>38</v>
       </c>
       <c r="C217" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
       <c r="D217" t="s">
-        <v>384</v>
+        <v>386</v>
       </c>
       <c r="E217">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="218" spans="1:5">
@@ -5879,13 +5894,13 @@
         <v>38</v>
       </c>
       <c r="C218" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
       <c r="D218" t="s">
-        <v>385</v>
+        <v>267</v>
       </c>
       <c r="E218">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="219" spans="1:5">
@@ -5896,13 +5911,13 @@
         <v>38</v>
       </c>
       <c r="C219" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
       <c r="D219" t="s">
-        <v>386</v>
+        <v>387</v>
       </c>
       <c r="E219">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="220" spans="1:5">
@@ -5913,13 +5928,13 @@
         <v>38</v>
       </c>
       <c r="C220" t="s">
-        <v>219</v>
+        <v>218</v>
       </c>
       <c r="D220" t="s">
-        <v>267</v>
+        <v>388</v>
       </c>
       <c r="E220">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="221" spans="1:5">
@@ -5930,10 +5945,10 @@
         <v>38</v>
       </c>
       <c r="C221" t="s">
-        <v>220</v>
+        <v>219</v>
       </c>
       <c r="D221" t="s">
-        <v>387</v>
+        <v>389</v>
       </c>
       <c r="E221">
         <v>4</v>
@@ -5947,10 +5962,10 @@
         <v>38</v>
       </c>
       <c r="C222" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
       <c r="D222" t="s">
-        <v>388</v>
+        <v>390</v>
       </c>
       <c r="E222">
         <v>4</v>
@@ -5964,10 +5979,10 @@
         <v>38</v>
       </c>
       <c r="C223" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
       <c r="D223" t="s">
-        <v>389</v>
+        <v>391</v>
       </c>
       <c r="E223">
         <v>4</v>
@@ -5981,13 +5996,13 @@
         <v>38</v>
       </c>
       <c r="C224" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
       <c r="D224" t="s">
-        <v>390</v>
+        <v>392</v>
       </c>
       <c r="E224">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="225" spans="1:5">
@@ -5998,13 +6013,13 @@
         <v>38</v>
       </c>
       <c r="C225" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="D225" t="s">
-        <v>391</v>
+        <v>393</v>
       </c>
       <c r="E225">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="226" spans="1:5">
@@ -6015,13 +6030,13 @@
         <v>38</v>
       </c>
       <c r="C226" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
       <c r="D226" t="s">
-        <v>392</v>
+        <v>394</v>
       </c>
       <c r="E226">
-        <v>5</v>
+        <v>6</v>
       </c>
     </row>
     <row r="227" spans="1:5">
@@ -6032,13 +6047,13 @@
         <v>38</v>
       </c>
       <c r="C227" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
       <c r="D227" t="s">
-        <v>393</v>
+        <v>395</v>
       </c>
       <c r="E227">
-        <v>5</v>
+        <v>8</v>
       </c>
     </row>
     <row r="228" spans="1:5">
@@ -6049,13 +6064,13 @@
         <v>38</v>
       </c>
       <c r="C228" t="s">
-        <v>227</v>
+        <v>226</v>
       </c>
       <c r="D228" t="s">
-        <v>394</v>
+        <v>396</v>
       </c>
       <c r="E228">
-        <v>6</v>
+        <v>10</v>
       </c>
     </row>
     <row r="229" spans="1:5">
@@ -6066,13 +6081,13 @@
         <v>38</v>
       </c>
       <c r="C229" t="s">
-        <v>228</v>
+        <v>227</v>
       </c>
       <c r="D229" t="s">
-        <v>395</v>
+        <v>396</v>
       </c>
       <c r="E229">
-        <v>8</v>
+        <v>10</v>
       </c>
     </row>
     <row r="230" spans="1:5">
@@ -6083,13 +6098,13 @@
         <v>38</v>
       </c>
       <c r="C230" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
       <c r="D230" t="s">
-        <v>396</v>
+        <v>269</v>
       </c>
       <c r="E230">
-        <v>10</v>
+        <v>12</v>
       </c>
     </row>
     <row r="231" spans="1:5">
@@ -6100,13 +6115,13 @@
         <v>38</v>
       </c>
       <c r="C231" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="D231" t="s">
-        <v>396</v>
+        <v>397</v>
       </c>
       <c r="E231">
-        <v>10</v>
+        <v>12</v>
       </c>
     </row>
     <row r="232" spans="1:5">
@@ -6117,13 +6132,13 @@
         <v>38</v>
       </c>
       <c r="C232" t="s">
-        <v>231</v>
+        <v>230</v>
       </c>
       <c r="D232" t="s">
-        <v>269</v>
+        <v>398</v>
       </c>
       <c r="E232">
-        <v>12</v>
+        <v>14</v>
       </c>
     </row>
     <row r="233" spans="1:5">
@@ -6134,13 +6149,13 @@
         <v>38</v>
       </c>
       <c r="C233" t="s">
-        <v>232</v>
+        <v>231</v>
       </c>
       <c r="D233" t="s">
-        <v>397</v>
+        <v>399</v>
       </c>
       <c r="E233">
-        <v>12</v>
+        <v>15</v>
       </c>
     </row>
     <row r="234" spans="1:5">
@@ -6151,47 +6166,132 @@
         <v>38</v>
       </c>
       <c r="C234" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
       <c r="D234" t="s">
-        <v>398</v>
+        <v>400</v>
       </c>
       <c r="E234">
-        <v>14</v>
+        <v>20</v>
       </c>
     </row>
     <row r="235" spans="1:5">
       <c r="A235" t="s">
-        <v>15</v>
+        <v>25</v>
       </c>
       <c r="B235" t="s">
-        <v>38</v>
+        <v>45</v>
       </c>
       <c r="C235" t="s">
-        <v>234</v>
+        <v>233</v>
       </c>
       <c r="D235" t="s">
-        <v>399</v>
+        <v>401</v>
       </c>
       <c r="E235">
-        <v>15</v>
+        <v>1</v>
       </c>
     </row>
     <row r="236" spans="1:5">
       <c r="A236" t="s">
-        <v>15</v>
+        <v>25</v>
       </c>
       <c r="B236" t="s">
-        <v>38</v>
+        <v>45</v>
       </c>
       <c r="C236" t="s">
+        <v>234</v>
+      </c>
+      <c r="D236" t="s">
+        <v>402</v>
+      </c>
+      <c r="E236">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="237" spans="1:5">
+      <c r="A237" t="s">
+        <v>25</v>
+      </c>
+      <c r="B237" t="s">
+        <v>45</v>
+      </c>
+      <c r="C237" t="s">
         <v>235</v>
       </c>
-      <c r="D236" t="s">
-        <v>400</v>
-      </c>
-      <c r="E236">
-        <v>20</v>
+      <c r="D237" t="s">
+        <v>403</v>
+      </c>
+      <c r="E237">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="238" spans="1:5">
+      <c r="A238" t="s">
+        <v>7</v>
+      </c>
+      <c r="B238" t="s">
+        <v>37</v>
+      </c>
+      <c r="C238" t="s">
+        <v>236</v>
+      </c>
+      <c r="D238" t="s">
+        <v>404</v>
+      </c>
+      <c r="E238">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="239" spans="1:5">
+      <c r="A239" t="s">
+        <v>25</v>
+      </c>
+      <c r="B239" t="s">
+        <v>45</v>
+      </c>
+      <c r="C239" t="s">
+        <v>236</v>
+      </c>
+      <c r="D239" t="s">
+        <v>404</v>
+      </c>
+      <c r="E239">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="240" spans="1:5">
+      <c r="A240" t="s">
+        <v>25</v>
+      </c>
+      <c r="B240" t="s">
+        <v>45</v>
+      </c>
+      <c r="C240" t="s">
+        <v>237</v>
+      </c>
+      <c r="D240" t="s">
+        <v>274</v>
+      </c>
+      <c r="E240">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="241" spans="1:5">
+      <c r="A241" t="s">
+        <v>25</v>
+      </c>
+      <c r="B241" t="s">
+        <v>45</v>
+      </c>
+      <c r="C241" t="s">
+        <v>238</v>
+      </c>
+      <c r="D241" t="s">
+        <v>405</v>
+      </c>
+      <c r="E241">
+        <v>1</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Atualização automática: rac (13/10/2026 10:13)
</commit_message>
<xml_diff>
--- a/Coordenadoria/02_Dados_Tratados/base_rac_tratada.xlsx
+++ b/Coordenadoria/02_Dados_Tratados/base_rac_tratada.xlsx
@@ -1239,8 +1239,16 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <fonts count="1">
+  <fonts count="2">
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -1256,7 +1264,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -1264,12 +1272,30 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1568,22 +1594,22 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:6">
-      <c r="A1" t="s">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" t="s">
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" t="s">
+      <c r="F1" s="1" t="s">
         <v>5</v>
       </c>
     </row>
@@ -2198,19 +2224,19 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:5">
-      <c r="A1" t="s">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" t="s">
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
         <v>55</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>56</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="1" t="s">
         <v>57</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualização automática: rac (13/10/2026 15:08)
</commit_message>
<xml_diff>
--- a/Coordenadoria/02_Dados_Tratados/base_rac_tratada.xlsx
+++ b/Coordenadoria/02_Dados_Tratados/base_rac_tratada.xlsx
@@ -1239,16 +1239,8 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <fonts count="2">
+  <fonts count="1">
     <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -1264,7 +1256,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -1272,30 +1264,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color auto="1"/>
-      </left>
-      <right style="thin">
-        <color auto="1"/>
-      </right>
-      <top style="thin">
-        <color auto="1"/>
-      </top>
-      <bottom style="thin">
-        <color auto="1"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1594,22 +1568,22 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:6">
-      <c r="A1" s="1" t="s">
+      <c r="A1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" s="1" t="s">
+      <c r="B1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" t="s">
         <v>5</v>
       </c>
     </row>
@@ -2224,19 +2198,19 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:5">
-      <c r="A1" s="1" t="s">
+      <c r="A1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" s="1" t="s">
+      <c r="B1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" t="s">
         <v>55</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" t="s">
         <v>56</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" t="s">
         <v>57</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualização automática: rac (14/10/2026 13:33)
</commit_message>
<xml_diff>
--- a/Coordenadoria/02_Dados_Tratados/base_rac_tratada.xlsx
+++ b/Coordenadoria/02_Dados_Tratados/base_rac_tratada.xlsx
@@ -1230,8 +1230,16 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <fonts count="1">
+  <fonts count="2">
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -1247,7 +1255,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -1255,12 +1263,30 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1559,22 +1585,22 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:6">
-      <c r="A1" t="s">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" t="s">
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" t="s">
+      <c r="F1" s="1" t="s">
         <v>5</v>
       </c>
     </row>
@@ -2189,19 +2215,19 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:5">
-      <c r="A1" t="s">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" t="s">
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
         <v>55</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>56</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="1" t="s">
         <v>57</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualização automática: rac (15/10/2026 12:34)
</commit_message>
<xml_diff>
--- a/Coordenadoria/02_Dados_Tratados/base_rac_tratada.xlsx
+++ b/Coordenadoria/02_Dados_Tratados/base_rac_tratada.xlsx
@@ -1230,16 +1230,8 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <fonts count="2">
+  <fonts count="1">
     <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -1255,7 +1247,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -1263,30 +1255,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color auto="1"/>
-      </left>
-      <right style="thin">
-        <color auto="1"/>
-      </right>
-      <top style="thin">
-        <color auto="1"/>
-      </top>
-      <bottom style="thin">
-        <color auto="1"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1585,22 +1559,22 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:6">
-      <c r="A1" s="1" t="s">
+      <c r="A1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" s="1" t="s">
+      <c r="B1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" t="s">
         <v>5</v>
       </c>
     </row>
@@ -2215,19 +2189,19 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:5">
-      <c r="A1" s="1" t="s">
+      <c r="A1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" s="1" t="s">
+      <c r="B1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" t="s">
         <v>55</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" t="s">
         <v>56</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" t="s">
         <v>57</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualização automática: rac (16/10/2026 12:01)
</commit_message>
<xml_diff>
--- a/Coordenadoria/02_Dados_Tratados/base_rac_tratada.xlsx
+++ b/Coordenadoria/02_Dados_Tratados/base_rac_tratada.xlsx
@@ -1230,8 +1230,16 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <fonts count="1">
+  <fonts count="2">
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -1247,7 +1255,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -1255,12 +1263,30 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1559,22 +1585,22 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:6">
-      <c r="A1" t="s">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" t="s">
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" t="s">
+      <c r="F1" s="1" t="s">
         <v>5</v>
       </c>
     </row>
@@ -2189,19 +2215,19 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:5">
-      <c r="A1" t="s">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" t="s">
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
         <v>55</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>56</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="1" t="s">
         <v>57</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualização automática: rac (16/10/2026 12:20)
</commit_message>
<xml_diff>
--- a/Coordenadoria/02_Dados_Tratados/base_rac_tratada.xlsx
+++ b/Coordenadoria/02_Dados_Tratados/base_rac_tratada.xlsx
@@ -1230,16 +1230,8 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <fonts count="2">
+  <fonts count="1">
     <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -1255,7 +1247,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -1263,30 +1255,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color auto="1"/>
-      </left>
-      <right style="thin">
-        <color auto="1"/>
-      </right>
-      <top style="thin">
-        <color auto="1"/>
-      </top>
-      <bottom style="thin">
-        <color auto="1"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1585,22 +1559,22 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:6">
-      <c r="A1" s="1" t="s">
+      <c r="A1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" s="1" t="s">
+      <c r="B1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" t="s">
         <v>5</v>
       </c>
     </row>
@@ -2215,19 +2189,19 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:5">
-      <c r="A1" s="1" t="s">
+      <c r="A1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" s="1" t="s">
+      <c r="B1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" t="s">
         <v>55</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" t="s">
         <v>56</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" t="s">
         <v>57</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualização automática: rac (19/10/2026 09:34)
</commit_message>
<xml_diff>
--- a/Coordenadoria/02_Dados_Tratados/base_rac_tratada.xlsx
+++ b/Coordenadoria/02_Dados_Tratados/base_rac_tratada.xlsx
@@ -1230,8 +1230,16 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <fonts count="1">
+  <fonts count="2">
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -1247,7 +1255,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -1255,12 +1263,30 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1559,22 +1585,22 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:6">
-      <c r="A1" t="s">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" t="s">
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" t="s">
+      <c r="F1" s="1" t="s">
         <v>5</v>
       </c>
     </row>
@@ -2189,19 +2215,19 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:5">
-      <c r="A1" t="s">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" t="s">
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
         <v>55</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>56</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="1" t="s">
         <v>57</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualização automática: rac (19/10/2026 14:26)
</commit_message>
<xml_diff>
--- a/Coordenadoria/02_Dados_Tratados/base_rac_tratada.xlsx
+++ b/Coordenadoria/02_Dados_Tratados/base_rac_tratada.xlsx
@@ -1230,16 +1230,8 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <fonts count="2">
+  <fonts count="1">
     <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -1255,7 +1247,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -1263,30 +1255,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color auto="1"/>
-      </left>
-      <right style="thin">
-        <color auto="1"/>
-      </right>
-      <top style="thin">
-        <color auto="1"/>
-      </top>
-      <bottom style="thin">
-        <color auto="1"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1585,22 +1559,22 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:6">
-      <c r="A1" s="1" t="s">
+      <c r="A1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" s="1" t="s">
+      <c r="B1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" t="s">
         <v>5</v>
       </c>
     </row>
@@ -2215,19 +2189,19 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:5">
-      <c r="A1" s="1" t="s">
+      <c r="A1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" s="1" t="s">
+      <c r="B1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" t="s">
         <v>55</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" t="s">
         <v>56</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" t="s">
         <v>57</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualização automática: rac (20/10/2026 12:02)
</commit_message>
<xml_diff>
--- a/Coordenadoria/02_Dados_Tratados/base_rac_tratada.xlsx
+++ b/Coordenadoria/02_Dados_Tratados/base_rac_tratada.xlsx
@@ -1230,8 +1230,16 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <fonts count="1">
+  <fonts count="2">
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -1247,7 +1255,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -1255,12 +1263,30 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1559,22 +1585,22 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:6">
-      <c r="A1" t="s">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" t="s">
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" t="s">
+      <c r="F1" s="1" t="s">
         <v>5</v>
       </c>
     </row>
@@ -2189,19 +2215,19 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:5">
-      <c r="A1" t="s">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" t="s">
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
         <v>55</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>56</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="1" t="s">
         <v>57</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualização automática: rac (20/10/2026 12:37)
</commit_message>
<xml_diff>
--- a/Coordenadoria/02_Dados_Tratados/base_rac_tratada.xlsx
+++ b/Coordenadoria/02_Dados_Tratados/base_rac_tratada.xlsx
@@ -1230,16 +1230,8 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <fonts count="2">
+  <fonts count="1">
     <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -1255,7 +1247,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -1263,30 +1255,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color auto="1"/>
-      </left>
-      <right style="thin">
-        <color auto="1"/>
-      </right>
-      <top style="thin">
-        <color auto="1"/>
-      </top>
-      <bottom style="thin">
-        <color auto="1"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1585,22 +1559,22 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:6">
-      <c r="A1" s="1" t="s">
+      <c r="A1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" s="1" t="s">
+      <c r="B1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" t="s">
         <v>5</v>
       </c>
     </row>
@@ -2215,19 +2189,19 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:5">
-      <c r="A1" s="1" t="s">
+      <c r="A1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" s="1" t="s">
+      <c r="B1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" t="s">
         <v>55</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" t="s">
         <v>56</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" t="s">
         <v>57</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualização automática: rac (21/10/2026 14:21)
</commit_message>
<xml_diff>
--- a/Coordenadoria/02_Dados_Tratados/base_rac_tratada.xlsx
+++ b/Coordenadoria/02_Dados_Tratados/base_rac_tratada.xlsx
@@ -1227,8 +1227,16 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <fonts count="1">
+  <fonts count="2">
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -1244,7 +1252,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -1252,12 +1260,30 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1556,22 +1582,22 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:6">
-      <c r="A1" t="s">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" t="s">
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" t="s">
+      <c r="F1" s="1" t="s">
         <v>5</v>
       </c>
     </row>
@@ -2186,19 +2212,19 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:5">
-      <c r="A1" t="s">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" t="s">
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
         <v>55</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>56</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="1" t="s">
         <v>57</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualização automática: rac (22/10/2026 12:51)
</commit_message>
<xml_diff>
--- a/Coordenadoria/02_Dados_Tratados/base_rac_tratada.xlsx
+++ b/Coordenadoria/02_Dados_Tratados/base_rac_tratada.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1099" uniqueCount="402">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1099" uniqueCount="404">
   <si>
     <t>matricula</t>
   </si>
@@ -194,9 +194,6 @@
     <t>C611008-0101</t>
   </si>
   <si>
-    <t>MS28773-05</t>
-  </si>
-  <si>
     <t>C611505-0201</t>
   </si>
   <si>
@@ -236,6 +233,9 @@
     <t>103-20400</t>
   </si>
   <si>
+    <t>030-02178-0000</t>
+  </si>
+  <si>
     <t>P7036368-01</t>
   </si>
   <si>
@@ -731,12 +731,12 @@
     <t>2670067-1</t>
   </si>
   <si>
+    <t>C660501-0103</t>
+  </si>
+  <si>
     <t>ALTERNATOR CONTROL UNIT ASSY</t>
   </si>
   <si>
-    <t>RETAINER-PACKING BACKUP</t>
-  </si>
-  <si>
     <t>ALTERNATOR</t>
   </si>
   <si>
@@ -776,6 +776,9 @@
     <t>BOLT,MACHINE</t>
   </si>
   <si>
+    <t>CONNECTOR,ELECTRICAL</t>
+  </si>
+  <si>
     <t>PROPELLER ASSEMBLY</t>
   </si>
   <si>
@@ -1221,22 +1224,17 @@
   </si>
   <si>
     <t>POST LIGHT ASS</t>
+  </si>
+  <si>
+    <t>COMPASS,SPEC</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <fonts count="2">
+  <fonts count="1">
     <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -1252,7 +1250,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -1260,30 +1258,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color auto="1"/>
-      </left>
-      <right style="thin">
-        <color auto="1"/>
-      </right>
-      <top style="thin">
-        <color auto="1"/>
-      </top>
-      <bottom style="thin">
-        <color auto="1"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1582,22 +1562,22 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:6">
-      <c r="A1" s="1" t="s">
+      <c r="A1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" s="1" t="s">
+      <c r="B1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" t="s">
         <v>5</v>
       </c>
     </row>
@@ -1758,7 +1738,7 @@
         <v>68</v>
       </c>
       <c r="F9">
-        <v>151</v>
+        <v>150</v>
       </c>
     </row>
     <row r="10" spans="1:6">
@@ -1778,7 +1758,7 @@
         <v>81</v>
       </c>
       <c r="F10">
-        <v>240</v>
+        <v>230</v>
       </c>
     </row>
     <row r="11" spans="1:6">
@@ -2212,19 +2192,19 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:5">
-      <c r="A1" s="1" t="s">
+      <c r="A1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" s="1" t="s">
+      <c r="B1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" t="s">
         <v>55</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" t="s">
         <v>56</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" t="s">
         <v>57</v>
       </c>
     </row>
@@ -2239,7 +2219,7 @@
         <v>58</v>
       </c>
       <c r="D2" t="s">
-        <v>238</v>
+        <v>239</v>
       </c>
       <c r="E2">
         <v>1</v>
@@ -2256,7 +2236,7 @@
         <v>58</v>
       </c>
       <c r="D3" t="s">
-        <v>238</v>
+        <v>239</v>
       </c>
       <c r="E3">
         <v>1</v>
@@ -2273,7 +2253,7 @@
         <v>59</v>
       </c>
       <c r="D4" t="s">
-        <v>239</v>
+        <v>240</v>
       </c>
       <c r="E4">
         <v>1</v>
@@ -2281,13 +2261,13 @@
     </row>
     <row r="5" spans="1:5">
       <c r="A5" t="s">
-        <v>6</v>
+        <v>11</v>
       </c>
       <c r="B5" t="s">
-        <v>36</v>
+        <v>39</v>
       </c>
       <c r="C5" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="D5" t="s">
         <v>240</v>
@@ -2298,13 +2278,13 @@
     </row>
     <row r="6" spans="1:5">
       <c r="A6" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B6" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="C6" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="D6" t="s">
         <v>240</v>
@@ -2315,13 +2295,13 @@
     </row>
     <row r="7" spans="1:5">
       <c r="A7" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="B7" t="s">
         <v>40</v>
       </c>
       <c r="C7" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="D7" t="s">
         <v>240</v>
@@ -2332,16 +2312,16 @@
     </row>
     <row r="8" spans="1:5">
       <c r="A8" t="s">
-        <v>13</v>
+        <v>6</v>
       </c>
       <c r="B8" t="s">
-        <v>40</v>
+        <v>36</v>
       </c>
       <c r="C8" t="s">
         <v>60</v>
       </c>
       <c r="D8" t="s">
-        <v>240</v>
+        <v>241</v>
       </c>
       <c r="E8">
         <v>1</v>
@@ -2349,13 +2329,13 @@
     </row>
     <row r="9" spans="1:5">
       <c r="A9" t="s">
-        <v>6</v>
+        <v>14</v>
       </c>
       <c r="B9" t="s">
-        <v>36</v>
+        <v>41</v>
       </c>
       <c r="C9" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="D9" t="s">
         <v>241</v>
@@ -2366,16 +2346,16 @@
     </row>
     <row r="10" spans="1:5">
       <c r="A10" t="s">
-        <v>14</v>
+        <v>7</v>
       </c>
       <c r="B10" t="s">
-        <v>41</v>
+        <v>37</v>
       </c>
       <c r="C10" t="s">
         <v>61</v>
       </c>
       <c r="D10" t="s">
-        <v>241</v>
+        <v>242</v>
       </c>
       <c r="E10">
         <v>1</v>
@@ -2383,13 +2363,13 @@
     </row>
     <row r="11" spans="1:5">
       <c r="A11" t="s">
-        <v>7</v>
+        <v>11</v>
       </c>
       <c r="B11" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="C11" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="D11" t="s">
         <v>242</v>
@@ -2400,13 +2380,13 @@
     </row>
     <row r="12" spans="1:5">
       <c r="A12" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="B12" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="C12" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="D12" t="s">
         <v>242</v>
@@ -2417,13 +2397,13 @@
     </row>
     <row r="13" spans="1:5">
       <c r="A13" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="B13" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="C13" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="D13" t="s">
         <v>242</v>
@@ -2434,19 +2414,19 @@
     </row>
     <row r="14" spans="1:5">
       <c r="A14" t="s">
-        <v>14</v>
+        <v>7</v>
       </c>
       <c r="B14" t="s">
-        <v>41</v>
+        <v>37</v>
       </c>
       <c r="C14" t="s">
         <v>62</v>
       </c>
       <c r="D14" t="s">
-        <v>242</v>
+        <v>243</v>
       </c>
       <c r="E14">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="15" spans="1:5">
@@ -2460,27 +2440,27 @@
         <v>63</v>
       </c>
       <c r="D15" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
       <c r="E15">
-        <v>2</v>
+        <v>12</v>
       </c>
     </row>
     <row r="16" spans="1:5">
       <c r="A16" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="B16" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="C16" t="s">
         <v>64</v>
       </c>
       <c r="D16" t="s">
-        <v>244</v>
+        <v>245</v>
       </c>
       <c r="E16">
-        <v>12</v>
+        <v>1</v>
       </c>
     </row>
     <row r="17" spans="1:5">
@@ -2494,21 +2474,21 @@
         <v>65</v>
       </c>
       <c r="D17" t="s">
-        <v>245</v>
+        <v>246</v>
       </c>
       <c r="E17">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="18" spans="1:5">
       <c r="A18" t="s">
-        <v>8</v>
+        <v>11</v>
       </c>
       <c r="B18" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="C18" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="D18" t="s">
         <v>246</v>
@@ -2519,41 +2499,41 @@
     </row>
     <row r="19" spans="1:5">
       <c r="A19" t="s">
-        <v>11</v>
+        <v>8</v>
       </c>
       <c r="B19" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="C19" t="s">
         <v>66</v>
       </c>
       <c r="D19" t="s">
-        <v>246</v>
+        <v>247</v>
       </c>
       <c r="E19">
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
     <row r="20" spans="1:5">
       <c r="A20" t="s">
-        <v>8</v>
+        <v>11</v>
       </c>
       <c r="B20" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="C20" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="D20" t="s">
         <v>247</v>
       </c>
       <c r="E20">
-        <v>4</v>
+        <v>2</v>
       </c>
     </row>
     <row r="21" spans="1:5">
       <c r="A21" t="s">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="B21" t="s">
         <v>39</v>
@@ -2562,10 +2542,10 @@
         <v>67</v>
       </c>
       <c r="D21" t="s">
-        <v>247</v>
+        <v>248</v>
       </c>
       <c r="E21">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="22" spans="1:5">
@@ -2579,7 +2559,7 @@
         <v>68</v>
       </c>
       <c r="D22" t="s">
-        <v>248</v>
+        <v>249</v>
       </c>
       <c r="E22">
         <v>1</v>
@@ -2596,7 +2576,7 @@
         <v>69</v>
       </c>
       <c r="D23" t="s">
-        <v>249</v>
+        <v>250</v>
       </c>
       <c r="E23">
         <v>1</v>
@@ -2613,7 +2593,7 @@
         <v>70</v>
       </c>
       <c r="D24" t="s">
-        <v>250</v>
+        <v>251</v>
       </c>
       <c r="E24">
         <v>1</v>
@@ -2630,41 +2610,41 @@
         <v>71</v>
       </c>
       <c r="D25" t="s">
-        <v>251</v>
+        <v>252</v>
       </c>
       <c r="E25">
-        <v>1</v>
+        <v>12</v>
       </c>
     </row>
     <row r="26" spans="1:5">
       <c r="A26" t="s">
-        <v>9</v>
+        <v>6</v>
       </c>
       <c r="B26" t="s">
-        <v>39</v>
+        <v>36</v>
       </c>
       <c r="C26" t="s">
         <v>72</v>
       </c>
       <c r="D26" t="s">
-        <v>252</v>
+        <v>253</v>
       </c>
       <c r="E26">
-        <v>12</v>
+        <v>1</v>
       </c>
     </row>
     <row r="27" spans="1:5">
       <c r="A27" t="s">
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="B27" t="s">
-        <v>36</v>
+        <v>40</v>
       </c>
       <c r="C27" t="s">
         <v>73</v>
       </c>
       <c r="D27" t="s">
-        <v>253</v>
+        <v>254</v>
       </c>
       <c r="E27">
         <v>1</v>
@@ -2672,16 +2652,16 @@
     </row>
     <row r="28" spans="1:5">
       <c r="A28" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="B28" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="C28" t="s">
         <v>73</v>
       </c>
       <c r="D28" t="s">
-        <v>253</v>
+        <v>254</v>
       </c>
       <c r="E28">
         <v>1</v>
@@ -2689,16 +2669,16 @@
     </row>
     <row r="29" spans="1:5">
       <c r="A29" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B29" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="C29" t="s">
         <v>73</v>
       </c>
       <c r="D29" t="s">
-        <v>253</v>
+        <v>254</v>
       </c>
       <c r="E29">
         <v>1</v>
@@ -2706,7 +2686,7 @@
     </row>
     <row r="30" spans="1:5">
       <c r="A30" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="B30" t="s">
         <v>40</v>
@@ -2715,7 +2695,7 @@
         <v>73</v>
       </c>
       <c r="D30" t="s">
-        <v>253</v>
+        <v>254</v>
       </c>
       <c r="E30">
         <v>1</v>
@@ -2723,16 +2703,16 @@
     </row>
     <row r="31" spans="1:5">
       <c r="A31" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="B31" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="C31" t="s">
         <v>73</v>
       </c>
       <c r="D31" t="s">
-        <v>253</v>
+        <v>254</v>
       </c>
       <c r="E31">
         <v>1</v>
@@ -2740,16 +2720,16 @@
     </row>
     <row r="32" spans="1:5">
       <c r="A32" t="s">
-        <v>14</v>
+        <v>10</v>
       </c>
       <c r="B32" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C32" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="D32" t="s">
-        <v>253</v>
+        <v>255</v>
       </c>
       <c r="E32">
         <v>1</v>
@@ -2757,16 +2737,16 @@
     </row>
     <row r="33" spans="1:5">
       <c r="A33" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="B33" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="C33" t="s">
         <v>74</v>
       </c>
       <c r="D33" t="s">
-        <v>254</v>
+        <v>255</v>
       </c>
       <c r="E33">
         <v>1</v>
@@ -2774,16 +2754,16 @@
     </row>
     <row r="34" spans="1:5">
       <c r="A34" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B34" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="C34" t="s">
         <v>74</v>
       </c>
       <c r="D34" t="s">
-        <v>254</v>
+        <v>255</v>
       </c>
       <c r="E34">
         <v>1</v>
@@ -2791,7 +2771,7 @@
     </row>
     <row r="35" spans="1:5">
       <c r="A35" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="B35" t="s">
         <v>40</v>
@@ -2800,7 +2780,7 @@
         <v>74</v>
       </c>
       <c r="D35" t="s">
-        <v>254</v>
+        <v>255</v>
       </c>
       <c r="E35">
         <v>1</v>
@@ -2808,16 +2788,16 @@
     </row>
     <row r="36" spans="1:5">
       <c r="A36" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="B36" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="C36" t="s">
         <v>74</v>
       </c>
       <c r="D36" t="s">
-        <v>254</v>
+        <v>255</v>
       </c>
       <c r="E36">
         <v>1</v>
@@ -2825,16 +2805,16 @@
     </row>
     <row r="37" spans="1:5">
       <c r="A37" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="B37" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="C37" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="D37" t="s">
-        <v>254</v>
+        <v>256</v>
       </c>
       <c r="E37">
         <v>1</v>
@@ -2842,16 +2822,16 @@
     </row>
     <row r="38" spans="1:5">
       <c r="A38" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B38" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="C38" t="s">
         <v>75</v>
       </c>
       <c r="D38" t="s">
-        <v>255</v>
+        <v>256</v>
       </c>
       <c r="E38">
         <v>1</v>
@@ -2859,7 +2839,7 @@
     </row>
     <row r="39" spans="1:5">
       <c r="A39" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="B39" t="s">
         <v>40</v>
@@ -2868,7 +2848,7 @@
         <v>75</v>
       </c>
       <c r="D39" t="s">
-        <v>255</v>
+        <v>256</v>
       </c>
       <c r="E39">
         <v>1</v>
@@ -2876,16 +2856,16 @@
     </row>
     <row r="40" spans="1:5">
       <c r="A40" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="B40" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="C40" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="D40" t="s">
-        <v>255</v>
+        <v>257</v>
       </c>
       <c r="E40">
         <v>1</v>
@@ -2893,16 +2873,16 @@
     </row>
     <row r="41" spans="1:5">
       <c r="A41" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B41" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="C41" t="s">
         <v>76</v>
       </c>
       <c r="D41" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
       <c r="E41">
         <v>1</v>
@@ -2910,16 +2890,16 @@
     </row>
     <row r="42" spans="1:5">
       <c r="A42" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B42" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="C42" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="D42" t="s">
-        <v>256</v>
+        <v>258</v>
       </c>
       <c r="E42">
         <v>1</v>
@@ -2927,50 +2907,50 @@
     </row>
     <row r="43" spans="1:5">
       <c r="A43" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="B43" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="C43" t="s">
         <v>77</v>
       </c>
       <c r="D43" t="s">
-        <v>257</v>
+        <v>258</v>
       </c>
       <c r="E43">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="44" spans="1:5">
       <c r="A44" t="s">
-        <v>14</v>
+        <v>8</v>
       </c>
       <c r="B44" t="s">
-        <v>41</v>
+        <v>38</v>
       </c>
       <c r="C44" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="D44" t="s">
-        <v>257</v>
+        <v>259</v>
       </c>
       <c r="E44">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="45" spans="1:5">
       <c r="A45" t="s">
-        <v>8</v>
+        <v>11</v>
       </c>
       <c r="B45" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="C45" t="s">
         <v>78</v>
       </c>
       <c r="D45" t="s">
-        <v>258</v>
+        <v>259</v>
       </c>
       <c r="E45">
         <v>1</v>
@@ -2978,16 +2958,16 @@
     </row>
     <row r="46" spans="1:5">
       <c r="A46" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="B46" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="C46" t="s">
         <v>78</v>
       </c>
       <c r="D46" t="s">
-        <v>258</v>
+        <v>259</v>
       </c>
       <c r="E46">
         <v>1</v>
@@ -2995,16 +2975,16 @@
     </row>
     <row r="47" spans="1:5">
       <c r="A47" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="B47" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="C47" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="D47" t="s">
-        <v>258</v>
+        <v>260</v>
       </c>
       <c r="E47">
         <v>1</v>
@@ -3018,10 +2998,10 @@
         <v>39</v>
       </c>
       <c r="C48" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="D48" t="s">
-        <v>259</v>
+        <v>261</v>
       </c>
       <c r="E48">
         <v>1</v>
@@ -3035,10 +3015,10 @@
         <v>39</v>
       </c>
       <c r="C49" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="D49" t="s">
-        <v>260</v>
+        <v>262</v>
       </c>
       <c r="E49">
         <v>1</v>
@@ -3052,10 +3032,10 @@
         <v>39</v>
       </c>
       <c r="C50" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="D50" t="s">
-        <v>261</v>
+        <v>263</v>
       </c>
       <c r="E50">
         <v>1</v>
@@ -3069,10 +3049,10 @@
         <v>39</v>
       </c>
       <c r="C51" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="D51" t="s">
-        <v>262</v>
+        <v>264</v>
       </c>
       <c r="E51">
         <v>1</v>
@@ -3086,13 +3066,13 @@
         <v>39</v>
       </c>
       <c r="C52" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="D52" t="s">
-        <v>263</v>
+        <v>265</v>
       </c>
       <c r="E52">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="53" spans="1:5">
@@ -3103,10 +3083,10 @@
         <v>39</v>
       </c>
       <c r="C53" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="D53" t="s">
-        <v>264</v>
+        <v>266</v>
       </c>
       <c r="E53">
         <v>2</v>
@@ -3114,24 +3094,24 @@
     </row>
     <row r="54" spans="1:5">
       <c r="A54" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B54" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="C54" t="s">
         <v>85</v>
       </c>
       <c r="D54" t="s">
-        <v>265</v>
+        <v>266</v>
       </c>
       <c r="E54">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="55" spans="1:5">
       <c r="A55" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="B55" t="s">
         <v>40</v>
@@ -3140,24 +3120,24 @@
         <v>85</v>
       </c>
       <c r="D55" t="s">
-        <v>265</v>
+        <v>266</v>
       </c>
       <c r="E55">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="56" spans="1:5">
       <c r="A56" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="B56" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="C56" t="s">
         <v>85</v>
       </c>
       <c r="D56" t="s">
-        <v>265</v>
+        <v>266</v>
       </c>
       <c r="E56">
         <v>2</v>
@@ -3165,16 +3145,16 @@
     </row>
     <row r="57" spans="1:5">
       <c r="A57" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="B57" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="C57" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="D57" t="s">
-        <v>265</v>
+        <v>267</v>
       </c>
       <c r="E57">
         <v>2</v>
@@ -3182,16 +3162,16 @@
     </row>
     <row r="58" spans="1:5">
       <c r="A58" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="B58" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="C58" t="s">
         <v>86</v>
       </c>
       <c r="D58" t="s">
-        <v>266</v>
+        <v>267</v>
       </c>
       <c r="E58">
         <v>2</v>
@@ -3199,84 +3179,84 @@
     </row>
     <row r="59" spans="1:5">
       <c r="A59" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="B59" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="C59" t="s">
         <v>86</v>
       </c>
       <c r="D59" t="s">
-        <v>266</v>
+        <v>267</v>
       </c>
       <c r="E59">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="60" spans="1:5">
       <c r="A60" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="B60" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="C60" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="D60" t="s">
-        <v>266</v>
+        <v>268</v>
       </c>
       <c r="E60">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="61" spans="1:5">
       <c r="A61" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="B61" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="C61" t="s">
         <v>87</v>
       </c>
       <c r="D61" t="s">
-        <v>267</v>
+        <v>268</v>
       </c>
       <c r="E61">
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
     <row r="62" spans="1:5">
       <c r="A62" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="B62" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="C62" t="s">
         <v>87</v>
       </c>
       <c r="D62" t="s">
-        <v>267</v>
+        <v>268</v>
       </c>
       <c r="E62">
-        <v>4</v>
+        <v>2</v>
       </c>
     </row>
     <row r="63" spans="1:5">
       <c r="A63" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="B63" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="C63" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="D63" t="s">
-        <v>267</v>
+        <v>269</v>
       </c>
       <c r="E63">
         <v>2</v>
@@ -3284,36 +3264,36 @@
     </row>
     <row r="64" spans="1:5">
       <c r="A64" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="B64" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="C64" t="s">
         <v>88</v>
       </c>
       <c r="D64" t="s">
-        <v>268</v>
+        <v>269</v>
       </c>
       <c r="E64">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="65" spans="1:5">
       <c r="A65" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="B65" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="C65" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="D65" t="s">
-        <v>268</v>
+        <v>270</v>
       </c>
       <c r="E65">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="66" spans="1:5">
@@ -3324,10 +3304,10 @@
         <v>39</v>
       </c>
       <c r="C66" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="D66" t="s">
-        <v>269</v>
+        <v>271</v>
       </c>
       <c r="E66">
         <v>2</v>
@@ -3341,10 +3321,10 @@
         <v>39</v>
       </c>
       <c r="C67" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="D67" t="s">
-        <v>270</v>
+        <v>272</v>
       </c>
       <c r="E67">
         <v>2</v>
@@ -3358,10 +3338,10 @@
         <v>39</v>
       </c>
       <c r="C68" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="D68" t="s">
-        <v>271</v>
+        <v>265</v>
       </c>
       <c r="E68">
         <v>2</v>
@@ -3375,10 +3355,10 @@
         <v>39</v>
       </c>
       <c r="C69" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="D69" t="s">
-        <v>264</v>
+        <v>273</v>
       </c>
       <c r="E69">
         <v>2</v>
@@ -3392,10 +3372,10 @@
         <v>39</v>
       </c>
       <c r="C70" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="D70" t="s">
-        <v>272</v>
+        <v>266</v>
       </c>
       <c r="E70">
         <v>2</v>
@@ -3409,27 +3389,27 @@
         <v>39</v>
       </c>
       <c r="C71" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="D71" t="s">
-        <v>265</v>
+        <v>264</v>
       </c>
       <c r="E71">
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
     <row r="72" spans="1:5">
       <c r="A72" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="B72" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="C72" t="s">
         <v>95</v>
       </c>
       <c r="D72" t="s">
-        <v>263</v>
+        <v>264</v>
       </c>
       <c r="E72">
         <v>4</v>
@@ -3437,16 +3417,16 @@
     </row>
     <row r="73" spans="1:5">
       <c r="A73" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="B73" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="C73" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="D73" t="s">
-        <v>263</v>
+        <v>274</v>
       </c>
       <c r="E73">
         <v>4</v>
@@ -3460,10 +3440,10 @@
         <v>39</v>
       </c>
       <c r="C74" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="D74" t="s">
-        <v>273</v>
+        <v>275</v>
       </c>
       <c r="E74">
         <v>4</v>
@@ -3477,10 +3457,10 @@
         <v>39</v>
       </c>
       <c r="C75" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="D75" t="s">
-        <v>274</v>
+        <v>252</v>
       </c>
       <c r="E75">
         <v>4</v>
@@ -3494,13 +3474,13 @@
         <v>39</v>
       </c>
       <c r="C76" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="D76" t="s">
-        <v>252</v>
+        <v>276</v>
       </c>
       <c r="E76">
-        <v>4</v>
+        <v>40</v>
       </c>
     </row>
     <row r="77" spans="1:5">
@@ -3511,44 +3491,44 @@
         <v>39</v>
       </c>
       <c r="C77" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="D77" t="s">
-        <v>275</v>
+        <v>277</v>
       </c>
       <c r="E77">
-        <v>40</v>
+        <v>4</v>
       </c>
     </row>
     <row r="78" spans="1:5">
       <c r="A78" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="B78" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="C78" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="D78" t="s">
-        <v>276</v>
+        <v>278</v>
       </c>
       <c r="E78">
-        <v>4</v>
+        <v>1</v>
       </c>
     </row>
     <row r="79" spans="1:5">
       <c r="A79" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="B79" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="C79" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="D79" t="s">
-        <v>277</v>
+        <v>279</v>
       </c>
       <c r="E79">
         <v>1</v>
@@ -3562,10 +3542,10 @@
         <v>39</v>
       </c>
       <c r="C80" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="D80" t="s">
-        <v>278</v>
+        <v>252</v>
       </c>
       <c r="E80">
         <v>1</v>
@@ -3573,16 +3553,16 @@
     </row>
     <row r="81" spans="1:5">
       <c r="A81" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B81" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="C81" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="D81" t="s">
-        <v>252</v>
+        <v>280</v>
       </c>
       <c r="E81">
         <v>1</v>
@@ -3590,16 +3570,16 @@
     </row>
     <row r="82" spans="1:5">
       <c r="A82" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="B82" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="C82" t="s">
         <v>104</v>
       </c>
       <c r="D82" t="s">
-        <v>279</v>
+        <v>280</v>
       </c>
       <c r="E82">
         <v>1</v>
@@ -3607,16 +3587,16 @@
     </row>
     <row r="83" spans="1:5">
       <c r="A83" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="B83" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C83" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="D83" t="s">
-        <v>279</v>
+        <v>281</v>
       </c>
       <c r="E83">
         <v>1</v>
@@ -3624,7 +3604,7 @@
     </row>
     <row r="84" spans="1:5">
       <c r="A84" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="B84" t="s">
         <v>40</v>
@@ -3633,7 +3613,7 @@
         <v>105</v>
       </c>
       <c r="D84" t="s">
-        <v>280</v>
+        <v>281</v>
       </c>
       <c r="E84">
         <v>1</v>
@@ -3641,16 +3621,16 @@
     </row>
     <row r="85" spans="1:5">
       <c r="A85" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="B85" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="C85" t="s">
         <v>105</v>
       </c>
       <c r="D85" t="s">
-        <v>280</v>
+        <v>281</v>
       </c>
       <c r="E85">
         <v>1</v>
@@ -3658,16 +3638,16 @@
     </row>
     <row r="86" spans="1:5">
       <c r="A86" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="B86" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C86" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="D86" t="s">
-        <v>280</v>
+        <v>282</v>
       </c>
       <c r="E86">
         <v>1</v>
@@ -3675,7 +3655,7 @@
     </row>
     <row r="87" spans="1:5">
       <c r="A87" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="B87" t="s">
         <v>40</v>
@@ -3684,7 +3664,7 @@
         <v>106</v>
       </c>
       <c r="D87" t="s">
-        <v>281</v>
+        <v>282</v>
       </c>
       <c r="E87">
         <v>1</v>
@@ -3692,41 +3672,41 @@
     </row>
     <row r="88" spans="1:5">
       <c r="A88" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="B88" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="C88" t="s">
         <v>106</v>
       </c>
       <c r="D88" t="s">
-        <v>281</v>
+        <v>282</v>
       </c>
       <c r="E88">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="89" spans="1:5">
       <c r="A89" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="B89" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C89" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="D89" t="s">
-        <v>281</v>
+        <v>283</v>
       </c>
       <c r="E89">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="90" spans="1:5">
       <c r="A90" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="B90" t="s">
         <v>40</v>
@@ -3735,7 +3715,7 @@
         <v>107</v>
       </c>
       <c r="D90" t="s">
-        <v>282</v>
+        <v>283</v>
       </c>
       <c r="E90">
         <v>1</v>
@@ -3743,16 +3723,16 @@
     </row>
     <row r="91" spans="1:5">
       <c r="A91" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B91" t="s">
         <v>40</v>
       </c>
       <c r="C91" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="D91" t="s">
-        <v>282</v>
+        <v>284</v>
       </c>
       <c r="E91">
         <v>1</v>
@@ -3760,7 +3740,7 @@
     </row>
     <row r="92" spans="1:5">
       <c r="A92" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="B92" t="s">
         <v>40</v>
@@ -3769,7 +3749,7 @@
         <v>108</v>
       </c>
       <c r="D92" t="s">
-        <v>283</v>
+        <v>284</v>
       </c>
       <c r="E92">
         <v>1</v>
@@ -3777,16 +3757,16 @@
     </row>
     <row r="93" spans="1:5">
       <c r="A93" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B93" t="s">
         <v>40</v>
       </c>
       <c r="C93" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="D93" t="s">
-        <v>283</v>
+        <v>285</v>
       </c>
       <c r="E93">
         <v>1</v>
@@ -3794,7 +3774,7 @@
     </row>
     <row r="94" spans="1:5">
       <c r="A94" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="B94" t="s">
         <v>40</v>
@@ -3803,7 +3783,7 @@
         <v>109</v>
       </c>
       <c r="D94" t="s">
-        <v>284</v>
+        <v>285</v>
       </c>
       <c r="E94">
         <v>1</v>
@@ -3811,16 +3791,16 @@
     </row>
     <row r="95" spans="1:5">
       <c r="A95" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B95" t="s">
         <v>40</v>
       </c>
       <c r="C95" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="D95" t="s">
-        <v>284</v>
+        <v>286</v>
       </c>
       <c r="E95">
         <v>1</v>
@@ -3828,7 +3808,7 @@
     </row>
     <row r="96" spans="1:5">
       <c r="A96" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="B96" t="s">
         <v>40</v>
@@ -3837,7 +3817,7 @@
         <v>110</v>
       </c>
       <c r="D96" t="s">
-        <v>285</v>
+        <v>286</v>
       </c>
       <c r="E96">
         <v>1</v>
@@ -3845,16 +3825,16 @@
     </row>
     <row r="97" spans="1:5">
       <c r="A97" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B97" t="s">
         <v>40</v>
       </c>
       <c r="C97" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="D97" t="s">
-        <v>285</v>
+        <v>287</v>
       </c>
       <c r="E97">
         <v>1</v>
@@ -3862,7 +3842,7 @@
     </row>
     <row r="98" spans="1:5">
       <c r="A98" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="B98" t="s">
         <v>40</v>
@@ -3871,7 +3851,7 @@
         <v>111</v>
       </c>
       <c r="D98" t="s">
-        <v>286</v>
+        <v>287</v>
       </c>
       <c r="E98">
         <v>1</v>
@@ -3879,16 +3859,16 @@
     </row>
     <row r="99" spans="1:5">
       <c r="A99" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B99" t="s">
         <v>40</v>
       </c>
       <c r="C99" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="D99" t="s">
-        <v>286</v>
+        <v>288</v>
       </c>
       <c r="E99">
         <v>1</v>
@@ -3896,7 +3876,7 @@
     </row>
     <row r="100" spans="1:5">
       <c r="A100" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="B100" t="s">
         <v>40</v>
@@ -3905,7 +3885,7 @@
         <v>112</v>
       </c>
       <c r="D100" t="s">
-        <v>287</v>
+        <v>288</v>
       </c>
       <c r="E100">
         <v>1</v>
@@ -3913,16 +3893,16 @@
     </row>
     <row r="101" spans="1:5">
       <c r="A101" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B101" t="s">
         <v>40</v>
       </c>
       <c r="C101" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="D101" t="s">
-        <v>287</v>
+        <v>289</v>
       </c>
       <c r="E101">
         <v>1</v>
@@ -3930,7 +3910,7 @@
     </row>
     <row r="102" spans="1:5">
       <c r="A102" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="B102" t="s">
         <v>40</v>
@@ -3939,7 +3919,7 @@
         <v>113</v>
       </c>
       <c r="D102" t="s">
-        <v>288</v>
+        <v>289</v>
       </c>
       <c r="E102">
         <v>1</v>
@@ -3947,16 +3927,16 @@
     </row>
     <row r="103" spans="1:5">
       <c r="A103" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B103" t="s">
         <v>40</v>
       </c>
       <c r="C103" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="D103" t="s">
-        <v>288</v>
+        <v>290</v>
       </c>
       <c r="E103">
         <v>1</v>
@@ -3964,16 +3944,16 @@
     </row>
     <row r="104" spans="1:5">
       <c r="A104" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="B104" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="C104" t="s">
         <v>114</v>
       </c>
       <c r="D104" t="s">
-        <v>289</v>
+        <v>290</v>
       </c>
       <c r="E104">
         <v>1</v>
@@ -3981,16 +3961,16 @@
     </row>
     <row r="105" spans="1:5">
       <c r="A105" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="B105" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C105" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="D105" t="s">
-        <v>289</v>
+        <v>291</v>
       </c>
       <c r="E105">
         <v>1</v>
@@ -3998,16 +3978,16 @@
     </row>
     <row r="106" spans="1:5">
       <c r="A106" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="B106" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="C106" t="s">
         <v>115</v>
       </c>
       <c r="D106" t="s">
-        <v>290</v>
+        <v>291</v>
       </c>
       <c r="E106">
         <v>1</v>
@@ -4015,16 +3995,16 @@
     </row>
     <row r="107" spans="1:5">
       <c r="A107" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="B107" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C107" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="D107" t="s">
-        <v>290</v>
+        <v>292</v>
       </c>
       <c r="E107">
         <v>1</v>
@@ -4038,10 +4018,10 @@
         <v>40</v>
       </c>
       <c r="C108" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="D108" t="s">
-        <v>291</v>
+        <v>293</v>
       </c>
       <c r="E108">
         <v>1</v>
@@ -4055,10 +4035,10 @@
         <v>40</v>
       </c>
       <c r="C109" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="D109" t="s">
-        <v>292</v>
+        <v>294</v>
       </c>
       <c r="E109">
         <v>1</v>
@@ -4072,10 +4052,10 @@
         <v>40</v>
       </c>
       <c r="C110" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="D110" t="s">
-        <v>293</v>
+        <v>295</v>
       </c>
       <c r="E110">
         <v>1</v>
@@ -4089,10 +4069,10 @@
         <v>40</v>
       </c>
       <c r="C111" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="D111" t="s">
-        <v>294</v>
+        <v>296</v>
       </c>
       <c r="E111">
         <v>1</v>
@@ -4106,10 +4086,10 @@
         <v>40</v>
       </c>
       <c r="C112" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="D112" t="s">
-        <v>295</v>
+        <v>297</v>
       </c>
       <c r="E112">
         <v>1</v>
@@ -4123,18 +4103,18 @@
         <v>40</v>
       </c>
       <c r="C113" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="D113" t="s">
-        <v>296</v>
+        <v>298</v>
       </c>
       <c r="E113">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="114" spans="1:5">
       <c r="A114" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="B114" t="s">
         <v>40</v>
@@ -4143,32 +4123,32 @@
         <v>122</v>
       </c>
       <c r="D114" t="s">
-        <v>297</v>
+        <v>298</v>
       </c>
       <c r="E114">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="115" spans="1:5">
       <c r="A115" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B115" t="s">
         <v>40</v>
       </c>
       <c r="C115" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="D115" t="s">
-        <v>297</v>
+        <v>299</v>
       </c>
       <c r="E115">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="116" spans="1:5">
       <c r="A116" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="B116" t="s">
         <v>40</v>
@@ -4177,7 +4157,7 @@
         <v>123</v>
       </c>
       <c r="D116" t="s">
-        <v>298</v>
+        <v>299</v>
       </c>
       <c r="E116">
         <v>2</v>
@@ -4185,16 +4165,16 @@
     </row>
     <row r="117" spans="1:5">
       <c r="A117" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="B117" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="C117" t="s">
         <v>123</v>
       </c>
       <c r="D117" t="s">
-        <v>298</v>
+        <v>299</v>
       </c>
       <c r="E117">
         <v>2</v>
@@ -4202,16 +4182,16 @@
     </row>
     <row r="118" spans="1:5">
       <c r="A118" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="B118" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C118" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="D118" t="s">
-        <v>298</v>
+        <v>300</v>
       </c>
       <c r="E118">
         <v>2</v>
@@ -4219,7 +4199,7 @@
     </row>
     <row r="119" spans="1:5">
       <c r="A119" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="B119" t="s">
         <v>40</v>
@@ -4228,7 +4208,7 @@
         <v>124</v>
       </c>
       <c r="D119" t="s">
-        <v>299</v>
+        <v>300</v>
       </c>
       <c r="E119">
         <v>2</v>
@@ -4236,16 +4216,16 @@
     </row>
     <row r="120" spans="1:5">
       <c r="A120" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="B120" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="C120" t="s">
         <v>124</v>
       </c>
       <c r="D120" t="s">
-        <v>299</v>
+        <v>300</v>
       </c>
       <c r="E120">
         <v>2</v>
@@ -4253,16 +4233,16 @@
     </row>
     <row r="121" spans="1:5">
       <c r="A121" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="B121" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C121" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="D121" t="s">
-        <v>299</v>
+        <v>301</v>
       </c>
       <c r="E121">
         <v>2</v>
@@ -4270,7 +4250,7 @@
     </row>
     <row r="122" spans="1:5">
       <c r="A122" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="B122" t="s">
         <v>40</v>
@@ -4279,7 +4259,7 @@
         <v>125</v>
       </c>
       <c r="D122" t="s">
-        <v>300</v>
+        <v>301</v>
       </c>
       <c r="E122">
         <v>2</v>
@@ -4287,16 +4267,16 @@
     </row>
     <row r="123" spans="1:5">
       <c r="A123" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B123" t="s">
         <v>40</v>
       </c>
       <c r="C123" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="D123" t="s">
-        <v>300</v>
+        <v>302</v>
       </c>
       <c r="E123">
         <v>2</v>
@@ -4304,7 +4284,7 @@
     </row>
     <row r="124" spans="1:5">
       <c r="A124" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="B124" t="s">
         <v>40</v>
@@ -4313,7 +4293,7 @@
         <v>126</v>
       </c>
       <c r="D124" t="s">
-        <v>301</v>
+        <v>302</v>
       </c>
       <c r="E124">
         <v>2</v>
@@ -4321,16 +4301,16 @@
     </row>
     <row r="125" spans="1:5">
       <c r="A125" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B125" t="s">
         <v>40</v>
       </c>
       <c r="C125" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="D125" t="s">
-        <v>301</v>
+        <v>282</v>
       </c>
       <c r="E125">
         <v>2</v>
@@ -4338,7 +4318,7 @@
     </row>
     <row r="126" spans="1:5">
       <c r="A126" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="B126" t="s">
         <v>40</v>
@@ -4347,24 +4327,24 @@
         <v>127</v>
       </c>
       <c r="D126" t="s">
-        <v>281</v>
+        <v>282</v>
       </c>
       <c r="E126">
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
     <row r="127" spans="1:5">
       <c r="A127" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="B127" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="C127" t="s">
         <v>127</v>
       </c>
       <c r="D127" t="s">
-        <v>281</v>
+        <v>282</v>
       </c>
       <c r="E127">
         <v>4</v>
@@ -4372,24 +4352,24 @@
     </row>
     <row r="128" spans="1:5">
       <c r="A128" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="B128" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C128" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="D128" t="s">
-        <v>281</v>
+        <v>303</v>
       </c>
       <c r="E128">
-        <v>4</v>
+        <v>2</v>
       </c>
     </row>
     <row r="129" spans="1:5">
       <c r="A129" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="B129" t="s">
         <v>40</v>
@@ -4398,27 +4378,27 @@
         <v>128</v>
       </c>
       <c r="D129" t="s">
-        <v>302</v>
+        <v>303</v>
       </c>
       <c r="E129">
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
     <row r="130" spans="1:5">
       <c r="A130" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B130" t="s">
         <v>40</v>
       </c>
       <c r="C130" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="D130" t="s">
-        <v>302</v>
+        <v>288</v>
       </c>
       <c r="E130">
-        <v>4</v>
+        <v>2</v>
       </c>
     </row>
     <row r="131" spans="1:5">
@@ -4429,10 +4409,10 @@
         <v>40</v>
       </c>
       <c r="C131" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="D131" t="s">
-        <v>287</v>
+        <v>304</v>
       </c>
       <c r="E131">
         <v>2</v>
@@ -4446,10 +4426,10 @@
         <v>40</v>
       </c>
       <c r="C132" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="D132" t="s">
-        <v>303</v>
+        <v>305</v>
       </c>
       <c r="E132">
         <v>2</v>
@@ -4463,18 +4443,18 @@
         <v>40</v>
       </c>
       <c r="C133" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="D133" t="s">
-        <v>304</v>
+        <v>306</v>
       </c>
       <c r="E133">
-        <v>2</v>
+        <v>5</v>
       </c>
     </row>
     <row r="134" spans="1:5">
       <c r="A134" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="B134" t="s">
         <v>40</v>
@@ -4483,7 +4463,7 @@
         <v>132</v>
       </c>
       <c r="D134" t="s">
-        <v>305</v>
+        <v>306</v>
       </c>
       <c r="E134">
         <v>5</v>
@@ -4491,19 +4471,19 @@
     </row>
     <row r="135" spans="1:5">
       <c r="A135" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B135" t="s">
         <v>40</v>
       </c>
       <c r="C135" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="D135" t="s">
-        <v>305</v>
+        <v>307</v>
       </c>
       <c r="E135">
-        <v>5</v>
+        <v>7</v>
       </c>
     </row>
     <row r="136" spans="1:5">
@@ -4514,13 +4494,13 @@
         <v>40</v>
       </c>
       <c r="C136" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="D136" t="s">
-        <v>306</v>
+        <v>308</v>
       </c>
       <c r="E136">
-        <v>7</v>
+        <v>10</v>
       </c>
     </row>
     <row r="137" spans="1:5">
@@ -4531,18 +4511,18 @@
         <v>40</v>
       </c>
       <c r="C137" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="D137" t="s">
-        <v>307</v>
+        <v>309</v>
       </c>
       <c r="E137">
-        <v>10</v>
+        <v>30</v>
       </c>
     </row>
     <row r="138" spans="1:5">
       <c r="A138" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="B138" t="s">
         <v>40</v>
@@ -4551,7 +4531,7 @@
         <v>135</v>
       </c>
       <c r="D138" t="s">
-        <v>308</v>
+        <v>309</v>
       </c>
       <c r="E138">
         <v>30</v>
@@ -4565,44 +4545,44 @@
         <v>40</v>
       </c>
       <c r="C139" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="D139" t="s">
-        <v>308</v>
+        <v>310</v>
       </c>
       <c r="E139">
-        <v>30</v>
+        <v>1</v>
       </c>
     </row>
     <row r="140" spans="1:5">
       <c r="A140" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="B140" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="C140" t="s">
         <v>136</v>
       </c>
       <c r="D140" t="s">
-        <v>309</v>
+        <v>310</v>
       </c>
       <c r="E140">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="141" spans="1:5">
       <c r="A141" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B141" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C141" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="D141" t="s">
-        <v>309</v>
+        <v>311</v>
       </c>
       <c r="E141">
         <v>1</v>
@@ -4616,10 +4596,10 @@
         <v>40</v>
       </c>
       <c r="C142" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="D142" t="s">
-        <v>310</v>
+        <v>312</v>
       </c>
       <c r="E142">
         <v>1</v>
@@ -4627,16 +4607,16 @@
     </row>
     <row r="143" spans="1:5">
       <c r="A143" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B143" t="s">
         <v>40</v>
       </c>
       <c r="C143" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="D143" t="s">
-        <v>311</v>
+        <v>313</v>
       </c>
       <c r="E143">
         <v>1</v>
@@ -4644,7 +4624,7 @@
     </row>
     <row r="144" spans="1:5">
       <c r="A144" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="B144" t="s">
         <v>40</v>
@@ -4653,7 +4633,7 @@
         <v>139</v>
       </c>
       <c r="D144" t="s">
-        <v>312</v>
+        <v>313</v>
       </c>
       <c r="E144">
         <v>1</v>
@@ -4667,10 +4647,10 @@
         <v>40</v>
       </c>
       <c r="C145" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="D145" t="s">
-        <v>312</v>
+        <v>314</v>
       </c>
       <c r="E145">
         <v>1</v>
@@ -4684,10 +4664,10 @@
         <v>40</v>
       </c>
       <c r="C146" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="D146" t="s">
-        <v>313</v>
+        <v>315</v>
       </c>
       <c r="E146">
         <v>1</v>
@@ -4701,10 +4681,10 @@
         <v>40</v>
       </c>
       <c r="C147" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="D147" t="s">
-        <v>314</v>
+        <v>316</v>
       </c>
       <c r="E147">
         <v>1</v>
@@ -4718,10 +4698,10 @@
         <v>40</v>
       </c>
       <c r="C148" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="D148" t="s">
-        <v>315</v>
+        <v>317</v>
       </c>
       <c r="E148">
         <v>1</v>
@@ -4735,10 +4715,10 @@
         <v>40</v>
       </c>
       <c r="C149" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="D149" t="s">
-        <v>316</v>
+        <v>318</v>
       </c>
       <c r="E149">
         <v>1</v>
@@ -4752,10 +4732,10 @@
         <v>40</v>
       </c>
       <c r="C150" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="D150" t="s">
-        <v>317</v>
+        <v>319</v>
       </c>
       <c r="E150">
         <v>1</v>
@@ -4769,10 +4749,10 @@
         <v>40</v>
       </c>
       <c r="C151" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="D151" t="s">
-        <v>318</v>
+        <v>320</v>
       </c>
       <c r="E151">
         <v>1</v>
@@ -4786,10 +4766,10 @@
         <v>40</v>
       </c>
       <c r="C152" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="D152" t="s">
-        <v>319</v>
+        <v>321</v>
       </c>
       <c r="E152">
         <v>1</v>
@@ -4803,10 +4783,10 @@
         <v>40</v>
       </c>
       <c r="C153" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="D153" t="s">
-        <v>320</v>
+        <v>322</v>
       </c>
       <c r="E153">
         <v>1</v>
@@ -4820,10 +4800,10 @@
         <v>40</v>
       </c>
       <c r="C154" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="D154" t="s">
-        <v>321</v>
+        <v>323</v>
       </c>
       <c r="E154">
         <v>1</v>
@@ -4837,10 +4817,10 @@
         <v>40</v>
       </c>
       <c r="C155" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="D155" t="s">
-        <v>322</v>
+        <v>324</v>
       </c>
       <c r="E155">
         <v>1</v>
@@ -4854,10 +4834,10 @@
         <v>40</v>
       </c>
       <c r="C156" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="D156" t="s">
-        <v>323</v>
+        <v>325</v>
       </c>
       <c r="E156">
         <v>1</v>
@@ -4871,10 +4851,10 @@
         <v>40</v>
       </c>
       <c r="C157" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="D157" t="s">
-        <v>324</v>
+        <v>326</v>
       </c>
       <c r="E157">
         <v>1</v>
@@ -4888,10 +4868,10 @@
         <v>40</v>
       </c>
       <c r="C158" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="D158" t="s">
-        <v>325</v>
+        <v>327</v>
       </c>
       <c r="E158">
         <v>1</v>
@@ -4905,10 +4885,10 @@
         <v>40</v>
       </c>
       <c r="C159" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="D159" t="s">
-        <v>326</v>
+        <v>328</v>
       </c>
       <c r="E159">
         <v>1</v>
@@ -4922,10 +4902,10 @@
         <v>40</v>
       </c>
       <c r="C160" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="D160" t="s">
-        <v>327</v>
+        <v>329</v>
       </c>
       <c r="E160">
         <v>1</v>
@@ -4939,10 +4919,10 @@
         <v>40</v>
       </c>
       <c r="C161" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="D161" t="s">
-        <v>328</v>
+        <v>330</v>
       </c>
       <c r="E161">
         <v>1</v>
@@ -4956,10 +4936,10 @@
         <v>40</v>
       </c>
       <c r="C162" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="D162" t="s">
-        <v>329</v>
+        <v>331</v>
       </c>
       <c r="E162">
         <v>1</v>
@@ -4973,10 +4953,10 @@
         <v>40</v>
       </c>
       <c r="C163" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="D163" t="s">
-        <v>330</v>
+        <v>332</v>
       </c>
       <c r="E163">
         <v>1</v>
@@ -4990,10 +4970,10 @@
         <v>40</v>
       </c>
       <c r="C164" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="D164" t="s">
-        <v>331</v>
+        <v>333</v>
       </c>
       <c r="E164">
         <v>1</v>
@@ -5007,10 +4987,10 @@
         <v>40</v>
       </c>
       <c r="C165" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="D165" t="s">
-        <v>332</v>
+        <v>334</v>
       </c>
       <c r="E165">
         <v>1</v>
@@ -5024,10 +5004,10 @@
         <v>40</v>
       </c>
       <c r="C166" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="D166" t="s">
-        <v>333</v>
+        <v>335</v>
       </c>
       <c r="E166">
         <v>1</v>
@@ -5041,10 +5021,10 @@
         <v>40</v>
       </c>
       <c r="C167" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="D167" t="s">
-        <v>334</v>
+        <v>336</v>
       </c>
       <c r="E167">
         <v>1</v>
@@ -5058,10 +5038,10 @@
         <v>40</v>
       </c>
       <c r="C168" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="D168" t="s">
-        <v>335</v>
+        <v>337</v>
       </c>
       <c r="E168">
         <v>1</v>
@@ -5075,10 +5055,10 @@
         <v>40</v>
       </c>
       <c r="C169" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="D169" t="s">
-        <v>336</v>
+        <v>338</v>
       </c>
       <c r="E169">
         <v>1</v>
@@ -5092,10 +5072,10 @@
         <v>40</v>
       </c>
       <c r="C170" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="D170" t="s">
-        <v>337</v>
+        <v>339</v>
       </c>
       <c r="E170">
         <v>1</v>
@@ -5109,10 +5089,10 @@
         <v>40</v>
       </c>
       <c r="C171" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="D171" t="s">
-        <v>338</v>
+        <v>340</v>
       </c>
       <c r="E171">
         <v>1</v>
@@ -5126,13 +5106,13 @@
         <v>40</v>
       </c>
       <c r="C172" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="D172" t="s">
-        <v>339</v>
+        <v>325</v>
       </c>
       <c r="E172">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="173" spans="1:5">
@@ -5143,10 +5123,10 @@
         <v>40</v>
       </c>
       <c r="C173" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="D173" t="s">
-        <v>324</v>
+        <v>341</v>
       </c>
       <c r="E173">
         <v>2</v>
@@ -5160,10 +5140,10 @@
         <v>40</v>
       </c>
       <c r="C174" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="D174" t="s">
-        <v>340</v>
+        <v>342</v>
       </c>
       <c r="E174">
         <v>2</v>
@@ -5177,10 +5157,10 @@
         <v>40</v>
       </c>
       <c r="C175" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="D175" t="s">
-        <v>341</v>
+        <v>343</v>
       </c>
       <c r="E175">
         <v>2</v>
@@ -5194,10 +5174,10 @@
         <v>40</v>
       </c>
       <c r="C176" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="D176" t="s">
-        <v>342</v>
+        <v>344</v>
       </c>
       <c r="E176">
         <v>2</v>
@@ -5211,13 +5191,13 @@
         <v>40</v>
       </c>
       <c r="C177" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="D177" t="s">
-        <v>343</v>
+        <v>345</v>
       </c>
       <c r="E177">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="178" spans="1:5">
@@ -5228,13 +5208,13 @@
         <v>40</v>
       </c>
       <c r="C178" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="D178" t="s">
-        <v>344</v>
+        <v>309</v>
       </c>
       <c r="E178">
-        <v>3</v>
+        <v>5</v>
       </c>
     </row>
     <row r="179" spans="1:5">
@@ -5245,13 +5225,13 @@
         <v>40</v>
       </c>
       <c r="C179" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="D179" t="s">
-        <v>308</v>
+        <v>346</v>
       </c>
       <c r="E179">
-        <v>5</v>
+        <v>8</v>
       </c>
     </row>
     <row r="180" spans="1:5">
@@ -5262,10 +5242,10 @@
         <v>40</v>
       </c>
       <c r="C180" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="D180" t="s">
-        <v>345</v>
+        <v>252</v>
       </c>
       <c r="E180">
         <v>8</v>
@@ -5279,30 +5259,30 @@
         <v>40</v>
       </c>
       <c r="C181" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="D181" t="s">
-        <v>252</v>
+        <v>347</v>
       </c>
       <c r="E181">
-        <v>8</v>
+        <v>10</v>
       </c>
     </row>
     <row r="182" spans="1:5">
       <c r="A182" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="B182" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="C182" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="D182" t="s">
-        <v>346</v>
+        <v>335</v>
       </c>
       <c r="E182">
-        <v>10</v>
+        <v>1</v>
       </c>
     </row>
     <row r="183" spans="1:5">
@@ -5313,10 +5293,10 @@
         <v>41</v>
       </c>
       <c r="C183" t="s">
-        <v>177</v>
+        <v>178</v>
       </c>
       <c r="D183" t="s">
-        <v>334</v>
+        <v>348</v>
       </c>
       <c r="E183">
         <v>1</v>
@@ -5330,10 +5310,10 @@
         <v>41</v>
       </c>
       <c r="C184" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="D184" t="s">
-        <v>347</v>
+        <v>349</v>
       </c>
       <c r="E184">
         <v>1</v>
@@ -5347,10 +5327,10 @@
         <v>41</v>
       </c>
       <c r="C185" t="s">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="D185" t="s">
-        <v>348</v>
+        <v>350</v>
       </c>
       <c r="E185">
         <v>1</v>
@@ -5364,10 +5344,10 @@
         <v>41</v>
       </c>
       <c r="C186" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="D186" t="s">
-        <v>349</v>
+        <v>351</v>
       </c>
       <c r="E186">
         <v>1</v>
@@ -5381,10 +5361,10 @@
         <v>41</v>
       </c>
       <c r="C187" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="D187" t="s">
-        <v>350</v>
+        <v>352</v>
       </c>
       <c r="E187">
         <v>1</v>
@@ -5398,10 +5378,10 @@
         <v>41</v>
       </c>
       <c r="C188" t="s">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="D188" t="s">
-        <v>351</v>
+        <v>271</v>
       </c>
       <c r="E188">
         <v>1</v>
@@ -5415,10 +5395,10 @@
         <v>41</v>
       </c>
       <c r="C189" t="s">
-        <v>183</v>
+        <v>184</v>
       </c>
       <c r="D189" t="s">
-        <v>270</v>
+        <v>353</v>
       </c>
       <c r="E189">
         <v>1</v>
@@ -5432,10 +5412,10 @@
         <v>41</v>
       </c>
       <c r="C190" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
       <c r="D190" t="s">
-        <v>352</v>
+        <v>354</v>
       </c>
       <c r="E190">
         <v>1</v>
@@ -5449,10 +5429,10 @@
         <v>41</v>
       </c>
       <c r="C191" t="s">
-        <v>185</v>
+        <v>186</v>
       </c>
       <c r="D191" t="s">
-        <v>353</v>
+        <v>355</v>
       </c>
       <c r="E191">
         <v>1</v>
@@ -5466,10 +5446,10 @@
         <v>41</v>
       </c>
       <c r="C192" t="s">
-        <v>186</v>
+        <v>187</v>
       </c>
       <c r="D192" t="s">
-        <v>354</v>
+        <v>356</v>
       </c>
       <c r="E192">
         <v>1</v>
@@ -5483,10 +5463,10 @@
         <v>41</v>
       </c>
       <c r="C193" t="s">
-        <v>187</v>
+        <v>188</v>
       </c>
       <c r="D193" t="s">
-        <v>355</v>
+        <v>357</v>
       </c>
       <c r="E193">
         <v>1</v>
@@ -5500,10 +5480,10 @@
         <v>41</v>
       </c>
       <c r="C194" t="s">
-        <v>188</v>
+        <v>189</v>
       </c>
       <c r="D194" t="s">
-        <v>356</v>
+        <v>358</v>
       </c>
       <c r="E194">
         <v>1</v>
@@ -5517,10 +5497,10 @@
         <v>41</v>
       </c>
       <c r="C195" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="D195" t="s">
-        <v>357</v>
+        <v>359</v>
       </c>
       <c r="E195">
         <v>1</v>
@@ -5534,10 +5514,10 @@
         <v>41</v>
       </c>
       <c r="C196" t="s">
-        <v>190</v>
+        <v>191</v>
       </c>
       <c r="D196" t="s">
-        <v>358</v>
+        <v>360</v>
       </c>
       <c r="E196">
         <v>1</v>
@@ -5551,10 +5531,10 @@
         <v>41</v>
       </c>
       <c r="C197" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="D197" t="s">
-        <v>359</v>
+        <v>361</v>
       </c>
       <c r="E197">
         <v>1</v>
@@ -5568,10 +5548,10 @@
         <v>41</v>
       </c>
       <c r="C198" t="s">
-        <v>192</v>
+        <v>193</v>
       </c>
       <c r="D198" t="s">
-        <v>360</v>
+        <v>362</v>
       </c>
       <c r="E198">
         <v>1</v>
@@ -5585,10 +5565,10 @@
         <v>41</v>
       </c>
       <c r="C199" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
       <c r="D199" t="s">
-        <v>361</v>
+        <v>363</v>
       </c>
       <c r="E199">
         <v>1</v>
@@ -5602,10 +5582,10 @@
         <v>41</v>
       </c>
       <c r="C200" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
       <c r="D200" t="s">
-        <v>362</v>
+        <v>364</v>
       </c>
       <c r="E200">
         <v>1</v>
@@ -5619,10 +5599,10 @@
         <v>41</v>
       </c>
       <c r="C201" t="s">
-        <v>195</v>
+        <v>196</v>
       </c>
       <c r="D201" t="s">
-        <v>363</v>
+        <v>365</v>
       </c>
       <c r="E201">
         <v>1</v>
@@ -5636,10 +5616,10 @@
         <v>41</v>
       </c>
       <c r="C202" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
       <c r="D202" t="s">
-        <v>364</v>
+        <v>366</v>
       </c>
       <c r="E202">
         <v>1</v>
@@ -5653,10 +5633,10 @@
         <v>41</v>
       </c>
       <c r="C203" t="s">
-        <v>197</v>
+        <v>198</v>
       </c>
       <c r="D203" t="s">
-        <v>365</v>
+        <v>367</v>
       </c>
       <c r="E203">
         <v>1</v>
@@ -5670,10 +5650,10 @@
         <v>41</v>
       </c>
       <c r="C204" t="s">
-        <v>198</v>
+        <v>199</v>
       </c>
       <c r="D204" t="s">
-        <v>366</v>
+        <v>368</v>
       </c>
       <c r="E204">
         <v>1</v>
@@ -5687,10 +5667,10 @@
         <v>41</v>
       </c>
       <c r="C205" t="s">
-        <v>199</v>
+        <v>200</v>
       </c>
       <c r="D205" t="s">
-        <v>367</v>
+        <v>369</v>
       </c>
       <c r="E205">
         <v>1</v>
@@ -5704,10 +5684,10 @@
         <v>41</v>
       </c>
       <c r="C206" t="s">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="D206" t="s">
-        <v>368</v>
+        <v>370</v>
       </c>
       <c r="E206">
         <v>1</v>
@@ -5721,10 +5701,10 @@
         <v>41</v>
       </c>
       <c r="C207" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
       <c r="D207" t="s">
-        <v>369</v>
+        <v>371</v>
       </c>
       <c r="E207">
         <v>1</v>
@@ -5738,10 +5718,10 @@
         <v>41</v>
       </c>
       <c r="C208" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="D208" t="s">
-        <v>370</v>
+        <v>372</v>
       </c>
       <c r="E208">
         <v>1</v>
@@ -5755,10 +5735,10 @@
         <v>41</v>
       </c>
       <c r="C209" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="D209" t="s">
-        <v>371</v>
+        <v>373</v>
       </c>
       <c r="E209">
         <v>1</v>
@@ -5772,10 +5752,10 @@
         <v>41</v>
       </c>
       <c r="C210" t="s">
-        <v>204</v>
+        <v>205</v>
       </c>
       <c r="D210" t="s">
-        <v>372</v>
+        <v>374</v>
       </c>
       <c r="E210">
         <v>1</v>
@@ -5789,10 +5769,10 @@
         <v>41</v>
       </c>
       <c r="C211" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
       <c r="D211" t="s">
-        <v>373</v>
+        <v>375</v>
       </c>
       <c r="E211">
         <v>1</v>
@@ -5806,10 +5786,10 @@
         <v>41</v>
       </c>
       <c r="C212" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="D212" t="s">
-        <v>374</v>
+        <v>376</v>
       </c>
       <c r="E212">
         <v>1</v>
@@ -5823,13 +5803,13 @@
         <v>41</v>
       </c>
       <c r="C213" t="s">
-        <v>207</v>
+        <v>208</v>
       </c>
       <c r="D213" t="s">
-        <v>375</v>
+        <v>377</v>
       </c>
       <c r="E213">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="214" spans="1:5">
@@ -5840,10 +5820,10 @@
         <v>41</v>
       </c>
       <c r="C214" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="D214" t="s">
-        <v>376</v>
+        <v>378</v>
       </c>
       <c r="E214">
         <v>2</v>
@@ -5857,10 +5837,10 @@
         <v>41</v>
       </c>
       <c r="C215" t="s">
-        <v>209</v>
+        <v>210</v>
       </c>
       <c r="D215" t="s">
-        <v>377</v>
+        <v>379</v>
       </c>
       <c r="E215">
         <v>2</v>
@@ -5874,10 +5854,10 @@
         <v>41</v>
       </c>
       <c r="C216" t="s">
-        <v>210</v>
+        <v>211</v>
       </c>
       <c r="D216" t="s">
-        <v>378</v>
+        <v>380</v>
       </c>
       <c r="E216">
         <v>2</v>
@@ -5891,10 +5871,10 @@
         <v>41</v>
       </c>
       <c r="C217" t="s">
-        <v>211</v>
+        <v>212</v>
       </c>
       <c r="D217" t="s">
-        <v>379</v>
+        <v>381</v>
       </c>
       <c r="E217">
         <v>2</v>
@@ -5908,10 +5888,10 @@
         <v>41</v>
       </c>
       <c r="C218" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="D218" t="s">
-        <v>380</v>
+        <v>382</v>
       </c>
       <c r="E218">
         <v>2</v>
@@ -5925,10 +5905,10 @@
         <v>41</v>
       </c>
       <c r="C219" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
       <c r="D219" t="s">
-        <v>381</v>
+        <v>383</v>
       </c>
       <c r="E219">
         <v>2</v>
@@ -5942,10 +5922,10 @@
         <v>41</v>
       </c>
       <c r="C220" t="s">
-        <v>214</v>
+        <v>215</v>
       </c>
       <c r="D220" t="s">
-        <v>382</v>
+        <v>384</v>
       </c>
       <c r="E220">
         <v>2</v>
@@ -5959,10 +5939,10 @@
         <v>41</v>
       </c>
       <c r="C221" t="s">
-        <v>215</v>
+        <v>216</v>
       </c>
       <c r="D221" t="s">
-        <v>383</v>
+        <v>385</v>
       </c>
       <c r="E221">
         <v>2</v>
@@ -5976,10 +5956,10 @@
         <v>41</v>
       </c>
       <c r="C222" t="s">
-        <v>216</v>
+        <v>217</v>
       </c>
       <c r="D222" t="s">
-        <v>384</v>
+        <v>385</v>
       </c>
       <c r="E222">
         <v>2</v>
@@ -5993,10 +5973,10 @@
         <v>41</v>
       </c>
       <c r="C223" t="s">
-        <v>217</v>
+        <v>218</v>
       </c>
       <c r="D223" t="s">
-        <v>384</v>
+        <v>386</v>
       </c>
       <c r="E223">
         <v>2</v>
@@ -6010,10 +5990,10 @@
         <v>41</v>
       </c>
       <c r="C224" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="D224" t="s">
-        <v>385</v>
+        <v>387</v>
       </c>
       <c r="E224">
         <v>2</v>
@@ -6027,13 +6007,13 @@
         <v>41</v>
       </c>
       <c r="C225" t="s">
-        <v>219</v>
+        <v>220</v>
       </c>
       <c r="D225" t="s">
-        <v>386</v>
+        <v>388</v>
       </c>
       <c r="E225">
-        <v>4</v>
+        <v>3</v>
       </c>
     </row>
     <row r="226" spans="1:5">
@@ -6044,10 +6024,10 @@
         <v>41</v>
       </c>
       <c r="C226" t="s">
-        <v>220</v>
+        <v>221</v>
       </c>
       <c r="D226" t="s">
-        <v>387</v>
+        <v>271</v>
       </c>
       <c r="E226">
         <v>3</v>
@@ -6061,13 +6041,13 @@
         <v>41</v>
       </c>
       <c r="C227" t="s">
-        <v>221</v>
+        <v>222</v>
       </c>
       <c r="D227" t="s">
-        <v>270</v>
+        <v>389</v>
       </c>
       <c r="E227">
-        <v>6</v>
+        <v>4</v>
       </c>
     </row>
     <row r="228" spans="1:5">
@@ -6078,10 +6058,10 @@
         <v>41</v>
       </c>
       <c r="C228" t="s">
-        <v>222</v>
+        <v>223</v>
       </c>
       <c r="D228" t="s">
-        <v>388</v>
+        <v>390</v>
       </c>
       <c r="E228">
         <v>4</v>
@@ -6095,10 +6075,10 @@
         <v>41</v>
       </c>
       <c r="C229" t="s">
-        <v>223</v>
+        <v>224</v>
       </c>
       <c r="D229" t="s">
-        <v>389</v>
+        <v>391</v>
       </c>
       <c r="E229">
         <v>4</v>
@@ -6112,10 +6092,10 @@
         <v>41</v>
       </c>
       <c r="C230" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
       <c r="D230" t="s">
-        <v>390</v>
+        <v>392</v>
       </c>
       <c r="E230">
         <v>4</v>
@@ -6129,10 +6109,10 @@
         <v>41</v>
       </c>
       <c r="C231" t="s">
-        <v>225</v>
+        <v>226</v>
       </c>
       <c r="D231" t="s">
-        <v>391</v>
+        <v>393</v>
       </c>
       <c r="E231">
         <v>4</v>
@@ -6146,13 +6126,13 @@
         <v>41</v>
       </c>
       <c r="C232" t="s">
-        <v>226</v>
+        <v>227</v>
       </c>
       <c r="D232" t="s">
-        <v>392</v>
+        <v>394</v>
       </c>
       <c r="E232">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="233" spans="1:5">
@@ -6163,10 +6143,10 @@
         <v>41</v>
       </c>
       <c r="C233" t="s">
-        <v>227</v>
+        <v>228</v>
       </c>
       <c r="D233" t="s">
-        <v>393</v>
+        <v>395</v>
       </c>
       <c r="E233">
         <v>5</v>
@@ -6180,13 +6160,13 @@
         <v>41</v>
       </c>
       <c r="C234" t="s">
-        <v>228</v>
+        <v>229</v>
       </c>
       <c r="D234" t="s">
-        <v>394</v>
+        <v>396</v>
       </c>
       <c r="E234">
-        <v>10</v>
+        <v>6</v>
       </c>
     </row>
     <row r="235" spans="1:5">
@@ -6197,13 +6177,13 @@
         <v>41</v>
       </c>
       <c r="C235" t="s">
-        <v>229</v>
+        <v>230</v>
       </c>
       <c r="D235" t="s">
-        <v>395</v>
+        <v>397</v>
       </c>
       <c r="E235">
-        <v>6</v>
+        <v>8</v>
       </c>
     </row>
     <row r="236" spans="1:5">
@@ -6214,13 +6194,13 @@
         <v>41</v>
       </c>
       <c r="C236" t="s">
-        <v>230</v>
+        <v>231</v>
       </c>
       <c r="D236" t="s">
-        <v>396</v>
+        <v>398</v>
       </c>
       <c r="E236">
-        <v>8</v>
+        <v>10</v>
       </c>
     </row>
     <row r="237" spans="1:5">
@@ -6231,10 +6211,10 @@
         <v>41</v>
       </c>
       <c r="C237" t="s">
-        <v>231</v>
+        <v>232</v>
       </c>
       <c r="D237" t="s">
-        <v>397</v>
+        <v>398</v>
       </c>
       <c r="E237">
         <v>10</v>
@@ -6248,13 +6228,13 @@
         <v>41</v>
       </c>
       <c r="C238" t="s">
-        <v>232</v>
+        <v>233</v>
       </c>
       <c r="D238" t="s">
-        <v>397</v>
+        <v>265</v>
       </c>
       <c r="E238">
-        <v>10</v>
+        <v>12</v>
       </c>
     </row>
     <row r="239" spans="1:5">
@@ -6265,10 +6245,10 @@
         <v>41</v>
       </c>
       <c r="C239" t="s">
-        <v>233</v>
+        <v>234</v>
       </c>
       <c r="D239" t="s">
-        <v>264</v>
+        <v>399</v>
       </c>
       <c r="E239">
         <v>12</v>
@@ -6282,13 +6262,13 @@
         <v>41</v>
       </c>
       <c r="C240" t="s">
-        <v>234</v>
+        <v>235</v>
       </c>
       <c r="D240" t="s">
-        <v>398</v>
+        <v>400</v>
       </c>
       <c r="E240">
-        <v>12</v>
+        <v>14</v>
       </c>
     </row>
     <row r="241" spans="1:5">
@@ -6299,13 +6279,13 @@
         <v>41</v>
       </c>
       <c r="C241" t="s">
-        <v>235</v>
+        <v>236</v>
       </c>
       <c r="D241" t="s">
-        <v>399</v>
+        <v>401</v>
       </c>
       <c r="E241">
-        <v>14</v>
+        <v>15</v>
       </c>
     </row>
     <row r="242" spans="1:5">
@@ -6316,30 +6296,30 @@
         <v>41</v>
       </c>
       <c r="C242" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
       <c r="D242" t="s">
-        <v>400</v>
+        <v>402</v>
       </c>
       <c r="E242">
-        <v>15</v>
+        <v>20</v>
       </c>
     </row>
     <row r="243" spans="1:5">
       <c r="A243" t="s">
-        <v>14</v>
+        <v>6</v>
       </c>
       <c r="B243" t="s">
-        <v>41</v>
+        <v>36</v>
       </c>
       <c r="C243" t="s">
-        <v>237</v>
+        <v>238</v>
       </c>
       <c r="D243" t="s">
-        <v>401</v>
+        <v>403</v>
       </c>
       <c r="E243">
-        <v>20</v>
+        <v>1</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Atualização automática: rac (23/10/2026 14:21)
</commit_message>
<xml_diff>
--- a/Coordenadoria/02_Dados_Tratados/base_rac_tratada.xlsx
+++ b/Coordenadoria/02_Dados_Tratados/base_rac_tratada.xlsx
@@ -1233,8 +1233,16 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <fonts count="1">
+  <fonts count="2">
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -1250,7 +1258,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -1258,12 +1266,30 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1562,22 +1588,22 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:6">
-      <c r="A1" t="s">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" t="s">
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" t="s">
+      <c r="F1" s="1" t="s">
         <v>5</v>
       </c>
     </row>
@@ -2192,19 +2218,19 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:5">
-      <c r="A1" t="s">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" t="s">
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
         <v>55</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>56</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="1" t="s">
         <v>57</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualização automática: rac (26/10/2026 14:17)
</commit_message>
<xml_diff>
--- a/Coordenadoria/02_Dados_Tratados/base_rac_tratada.xlsx
+++ b/Coordenadoria/02_Dados_Tratados/base_rac_tratada.xlsx
@@ -1233,16 +1233,8 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <fonts count="2">
+  <fonts count="1">
     <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -1258,7 +1250,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -1266,30 +1258,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color auto="1"/>
-      </left>
-      <right style="thin">
-        <color auto="1"/>
-      </right>
-      <top style="thin">
-        <color auto="1"/>
-      </top>
-      <bottom style="thin">
-        <color auto="1"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1588,22 +1562,22 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:6">
-      <c r="A1" s="1" t="s">
+      <c r="A1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" s="1" t="s">
+      <c r="B1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" t="s">
         <v>5</v>
       </c>
     </row>
@@ -2218,19 +2192,19 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:5">
-      <c r="A1" s="1" t="s">
+      <c r="A1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" s="1" t="s">
+      <c r="B1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" t="s">
         <v>55</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" t="s">
         <v>56</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" t="s">
         <v>57</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualização automática: rac (29/10/2026 14:23)
</commit_message>
<xml_diff>
--- a/Coordenadoria/02_Dados_Tratados/base_rac_tratada.xlsx
+++ b/Coordenadoria/02_Dados_Tratados/base_rac_tratada.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1099" uniqueCount="408">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1087" uniqueCount="408">
   <si>
     <t>matricula</t>
   </si>
@@ -215,7 +215,7 @@
     <t>2641014-5</t>
   </si>
   <si>
-    <t>MS21043-3</t>
+    <t>2643091-1</t>
   </si>
   <si>
     <t>NAS147-84</t>
@@ -764,7 +764,7 @@
     <t>SPRING-MAIN GEAR CEN</t>
   </si>
   <si>
-    <t>NUT,SELF-LOCKING,EXT</t>
+    <t>PIN ASSY-TORQUE LINK</t>
   </si>
   <si>
     <t>BOLT,INTERNAL WRENCHING</t>
@@ -1647,10 +1647,10 @@
         <v>53</v>
       </c>
       <c r="E4">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F4">
-        <v>4</v>
+        <v>3</v>
       </c>
     </row>
     <row r="5" spans="1:6">
@@ -1667,10 +1667,10 @@
         <v>53</v>
       </c>
       <c r="E5">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F5">
-        <v>13</v>
+        <v>1</v>
       </c>
     </row>
     <row r="6" spans="1:6">
@@ -1687,10 +1687,10 @@
         <v>53</v>
       </c>
       <c r="E6">
+        <v>1</v>
+      </c>
+      <c r="F6">
         <v>2</v>
-      </c>
-      <c r="F6">
-        <v>6</v>
       </c>
     </row>
     <row r="7" spans="1:6">
@@ -2200,7 +2200,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E243"/>
+  <dimension ref="A1:E240"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:5">
@@ -2290,10 +2290,10 @@
     </row>
     <row r="6" spans="1:5">
       <c r="A6" t="s">
-        <v>8</v>
+        <v>16</v>
       </c>
       <c r="B6" t="s">
-        <v>38</v>
+        <v>42</v>
       </c>
       <c r="C6" t="s">
         <v>61</v>
@@ -2307,16 +2307,16 @@
     </row>
     <row r="7" spans="1:5">
       <c r="A7" t="s">
-        <v>16</v>
+        <v>8</v>
       </c>
       <c r="B7" t="s">
-        <v>42</v>
+        <v>38</v>
       </c>
       <c r="C7" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="D7" t="s">
-        <v>244</v>
+        <v>245</v>
       </c>
       <c r="E7">
         <v>1</v>
@@ -2330,10 +2330,10 @@
         <v>38</v>
       </c>
       <c r="C8" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="D8" t="s">
-        <v>245</v>
+        <v>246</v>
       </c>
       <c r="E8">
         <v>1</v>
@@ -2347,10 +2347,10 @@
         <v>38</v>
       </c>
       <c r="C9" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="D9" t="s">
-        <v>246</v>
+        <v>247</v>
       </c>
       <c r="E9">
         <v>1</v>
@@ -2358,16 +2358,16 @@
     </row>
     <row r="10" spans="1:5">
       <c r="A10" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="B10" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="C10" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="D10" t="s">
-        <v>247</v>
+        <v>248</v>
       </c>
       <c r="E10">
         <v>1</v>
@@ -2375,10 +2375,10 @@
     </row>
     <row r="11" spans="1:5">
       <c r="A11" t="s">
-        <v>9</v>
+        <v>13</v>
       </c>
       <c r="B11" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="C11" t="s">
         <v>65</v>
@@ -2392,10 +2392,10 @@
     </row>
     <row r="12" spans="1:5">
       <c r="A12" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="B12" t="s">
-        <v>37</v>
+        <v>41</v>
       </c>
       <c r="C12" t="s">
         <v>65</v>
@@ -2409,10 +2409,10 @@
     </row>
     <row r="13" spans="1:5">
       <c r="A13" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="B13" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="C13" t="s">
         <v>65</v>
@@ -2426,50 +2426,50 @@
     </row>
     <row r="14" spans="1:5">
       <c r="A14" t="s">
-        <v>16</v>
+        <v>10</v>
       </c>
       <c r="B14" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="C14" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="D14" t="s">
-        <v>248</v>
+        <v>249</v>
       </c>
       <c r="E14">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="15" spans="1:5">
       <c r="A15" t="s">
-        <v>9</v>
+        <v>13</v>
       </c>
       <c r="B15" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="C15" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="D15" t="s">
-        <v>249</v>
+        <v>250</v>
       </c>
       <c r="E15">
-        <v>12</v>
+        <v>2</v>
       </c>
     </row>
     <row r="16" spans="1:5">
       <c r="A16" t="s">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="B16" t="s">
-        <v>40</v>
+        <v>37</v>
       </c>
       <c r="C16" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="D16" t="s">
-        <v>250</v>
+        <v>251</v>
       </c>
       <c r="E16">
         <v>2</v>
@@ -2477,53 +2477,53 @@
     </row>
     <row r="17" spans="1:5">
       <c r="A17" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="B17" t="s">
         <v>37</v>
       </c>
       <c r="C17" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="D17" t="s">
-        <v>250</v>
+        <v>252</v>
       </c>
       <c r="E17">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="18" spans="1:5">
       <c r="A18" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="B18" t="s">
-        <v>40</v>
+        <v>37</v>
       </c>
       <c r="C18" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="D18" t="s">
-        <v>251</v>
+        <v>253</v>
       </c>
       <c r="E18">
-        <v>4</v>
+        <v>1</v>
       </c>
     </row>
     <row r="19" spans="1:5">
       <c r="A19" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="B19" t="s">
         <v>37</v>
       </c>
       <c r="C19" t="s">
-        <v>68</v>
+        <v>71</v>
       </c>
       <c r="D19" t="s">
-        <v>251</v>
+        <v>254</v>
       </c>
       <c r="E19">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="20" spans="1:5">
@@ -2534,10 +2534,10 @@
         <v>37</v>
       </c>
       <c r="C20" t="s">
-        <v>69</v>
+        <v>72</v>
       </c>
       <c r="D20" t="s">
-        <v>252</v>
+        <v>255</v>
       </c>
       <c r="E20">
         <v>1</v>
@@ -2551,10 +2551,10 @@
         <v>37</v>
       </c>
       <c r="C21" t="s">
-        <v>70</v>
+        <v>73</v>
       </c>
       <c r="D21" t="s">
-        <v>253</v>
+        <v>256</v>
       </c>
       <c r="E21">
         <v>1</v>
@@ -2568,13 +2568,13 @@
         <v>37</v>
       </c>
       <c r="C22" t="s">
-        <v>71</v>
+        <v>74</v>
       </c>
       <c r="D22" t="s">
-        <v>254</v>
+        <v>257</v>
       </c>
       <c r="E22">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="23" spans="1:5">
@@ -2585,27 +2585,27 @@
         <v>37</v>
       </c>
       <c r="C23" t="s">
-        <v>72</v>
+        <v>75</v>
       </c>
       <c r="D23" t="s">
-        <v>255</v>
+        <v>258</v>
       </c>
       <c r="E23">
-        <v>1</v>
+        <v>12</v>
       </c>
     </row>
     <row r="24" spans="1:5">
       <c r="A24" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B24" t="s">
-        <v>37</v>
+        <v>41</v>
       </c>
       <c r="C24" t="s">
-        <v>73</v>
+        <v>76</v>
       </c>
       <c r="D24" t="s">
-        <v>256</v>
+        <v>259</v>
       </c>
       <c r="E24">
         <v>1</v>
@@ -2613,41 +2613,41 @@
     </row>
     <row r="25" spans="1:5">
       <c r="A25" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="B25" t="s">
         <v>37</v>
       </c>
       <c r="C25" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="D25" t="s">
-        <v>257</v>
+        <v>259</v>
       </c>
       <c r="E25">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="26" spans="1:5">
       <c r="A26" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="B26" t="s">
-        <v>37</v>
+        <v>41</v>
       </c>
       <c r="C26" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="D26" t="s">
-        <v>258</v>
+        <v>259</v>
       </c>
       <c r="E26">
-        <v>12</v>
+        <v>1</v>
       </c>
     </row>
     <row r="27" spans="1:5">
       <c r="A27" t="s">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="B27" t="s">
         <v>41</v>
@@ -2664,10 +2664,10 @@
     </row>
     <row r="28" spans="1:5">
       <c r="A28" t="s">
-        <v>13</v>
+        <v>16</v>
       </c>
       <c r="B28" t="s">
-        <v>37</v>
+        <v>42</v>
       </c>
       <c r="C28" t="s">
         <v>76</v>
@@ -2681,16 +2681,16 @@
     </row>
     <row r="29" spans="1:5">
       <c r="A29" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B29" t="s">
-        <v>41</v>
+        <v>37</v>
       </c>
       <c r="C29" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="D29" t="s">
-        <v>259</v>
+        <v>260</v>
       </c>
       <c r="E29">
         <v>1</v>
@@ -2698,16 +2698,16 @@
     </row>
     <row r="30" spans="1:5">
       <c r="A30" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B30" t="s">
         <v>41</v>
       </c>
       <c r="C30" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="D30" t="s">
-        <v>259</v>
+        <v>260</v>
       </c>
       <c r="E30">
         <v>1</v>
@@ -2715,16 +2715,16 @@
     </row>
     <row r="31" spans="1:5">
       <c r="A31" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="B31" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="C31" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="D31" t="s">
-        <v>259</v>
+        <v>260</v>
       </c>
       <c r="E31">
         <v>1</v>
@@ -2732,10 +2732,10 @@
     </row>
     <row r="32" spans="1:5">
       <c r="A32" t="s">
-        <v>13</v>
+        <v>16</v>
       </c>
       <c r="B32" t="s">
-        <v>37</v>
+        <v>42</v>
       </c>
       <c r="C32" t="s">
         <v>77</v>
@@ -2749,16 +2749,16 @@
     </row>
     <row r="33" spans="1:5">
       <c r="A33" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B33" t="s">
-        <v>41</v>
+        <v>37</v>
       </c>
       <c r="C33" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="D33" t="s">
-        <v>260</v>
+        <v>261</v>
       </c>
       <c r="E33">
         <v>1</v>
@@ -2766,16 +2766,16 @@
     </row>
     <row r="34" spans="1:5">
       <c r="A34" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B34" t="s">
         <v>41</v>
       </c>
       <c r="C34" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="D34" t="s">
-        <v>260</v>
+        <v>261</v>
       </c>
       <c r="E34">
         <v>1</v>
@@ -2783,16 +2783,16 @@
     </row>
     <row r="35" spans="1:5">
       <c r="A35" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="B35" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="C35" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="D35" t="s">
-        <v>260</v>
+        <v>261</v>
       </c>
       <c r="E35">
         <v>1</v>
@@ -2806,10 +2806,10 @@
         <v>37</v>
       </c>
       <c r="C36" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="D36" t="s">
-        <v>261</v>
+        <v>262</v>
       </c>
       <c r="E36">
         <v>1</v>
@@ -2823,10 +2823,10 @@
         <v>41</v>
       </c>
       <c r="C37" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="D37" t="s">
-        <v>261</v>
+        <v>262</v>
       </c>
       <c r="E37">
         <v>1</v>
@@ -2840,10 +2840,10 @@
         <v>41</v>
       </c>
       <c r="C38" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="D38" t="s">
-        <v>261</v>
+        <v>262</v>
       </c>
       <c r="E38">
         <v>1</v>
@@ -2857,10 +2857,10 @@
         <v>37</v>
       </c>
       <c r="C39" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="D39" t="s">
-        <v>262</v>
+        <v>263</v>
       </c>
       <c r="E39">
         <v>1</v>
@@ -2874,10 +2874,10 @@
         <v>41</v>
       </c>
       <c r="C40" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="D40" t="s">
-        <v>262</v>
+        <v>263</v>
       </c>
       <c r="E40">
         <v>1</v>
@@ -2885,16 +2885,16 @@
     </row>
     <row r="41" spans="1:5">
       <c r="A41" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="B41" t="s">
-        <v>41</v>
+        <v>37</v>
       </c>
       <c r="C41" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="D41" t="s">
-        <v>262</v>
+        <v>264</v>
       </c>
       <c r="E41">
         <v>1</v>
@@ -2902,16 +2902,16 @@
     </row>
     <row r="42" spans="1:5">
       <c r="A42" t="s">
-        <v>13</v>
+        <v>16</v>
       </c>
       <c r="B42" t="s">
-        <v>37</v>
+        <v>42</v>
       </c>
       <c r="C42" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="D42" t="s">
-        <v>263</v>
+        <v>264</v>
       </c>
       <c r="E42">
         <v>1</v>
@@ -2919,16 +2919,16 @@
     </row>
     <row r="43" spans="1:5">
       <c r="A43" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B43" t="s">
-        <v>41</v>
+        <v>37</v>
       </c>
       <c r="C43" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="D43" t="s">
-        <v>263</v>
+        <v>265</v>
       </c>
       <c r="E43">
         <v>1</v>
@@ -2936,33 +2936,33 @@
     </row>
     <row r="44" spans="1:5">
       <c r="A44" t="s">
-        <v>13</v>
+        <v>16</v>
       </c>
       <c r="B44" t="s">
-        <v>37</v>
+        <v>42</v>
       </c>
       <c r="C44" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="D44" t="s">
-        <v>264</v>
+        <v>265</v>
       </c>
       <c r="E44">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="45" spans="1:5">
       <c r="A45" t="s">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="B45" t="s">
-        <v>42</v>
+        <v>37</v>
       </c>
       <c r="C45" t="s">
-        <v>81</v>
+        <v>83</v>
       </c>
       <c r="D45" t="s">
-        <v>264</v>
+        <v>266</v>
       </c>
       <c r="E45">
         <v>1</v>
@@ -2976,10 +2976,10 @@
         <v>37</v>
       </c>
       <c r="C46" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="D46" t="s">
-        <v>265</v>
+        <v>267</v>
       </c>
       <c r="E46">
         <v>1</v>
@@ -2987,19 +2987,19 @@
     </row>
     <row r="47" spans="1:5">
       <c r="A47" t="s">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="B47" t="s">
-        <v>42</v>
+        <v>37</v>
       </c>
       <c r="C47" t="s">
-        <v>82</v>
+        <v>85</v>
       </c>
       <c r="D47" t="s">
-        <v>265</v>
+        <v>268</v>
       </c>
       <c r="E47">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="48" spans="1:5">
@@ -3010,10 +3010,10 @@
         <v>37</v>
       </c>
       <c r="C48" t="s">
-        <v>83</v>
+        <v>86</v>
       </c>
       <c r="D48" t="s">
-        <v>266</v>
+        <v>269</v>
       </c>
       <c r="E48">
         <v>1</v>
@@ -3027,10 +3027,10 @@
         <v>37</v>
       </c>
       <c r="C49" t="s">
-        <v>84</v>
+        <v>87</v>
       </c>
       <c r="D49" t="s">
-        <v>267</v>
+        <v>270</v>
       </c>
       <c r="E49">
         <v>1</v>
@@ -3044,10 +3044,10 @@
         <v>37</v>
       </c>
       <c r="C50" t="s">
-        <v>85</v>
+        <v>88</v>
       </c>
       <c r="D50" t="s">
-        <v>268</v>
+        <v>271</v>
       </c>
       <c r="E50">
         <v>1</v>
@@ -3061,10 +3061,10 @@
         <v>37</v>
       </c>
       <c r="C51" t="s">
-        <v>86</v>
+        <v>89</v>
       </c>
       <c r="D51" t="s">
-        <v>269</v>
+        <v>258</v>
       </c>
       <c r="E51">
         <v>1</v>
@@ -3078,55 +3078,55 @@
         <v>37</v>
       </c>
       <c r="C52" t="s">
-        <v>87</v>
+        <v>90</v>
       </c>
       <c r="D52" t="s">
-        <v>270</v>
+        <v>272</v>
       </c>
       <c r="E52">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="53" spans="1:5">
       <c r="A53" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="B53" t="s">
-        <v>37</v>
+        <v>41</v>
       </c>
       <c r="C53" t="s">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="D53" t="s">
-        <v>271</v>
+        <v>272</v>
       </c>
       <c r="E53">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="54" spans="1:5">
       <c r="A54" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="B54" t="s">
-        <v>37</v>
+        <v>41</v>
       </c>
       <c r="C54" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="D54" t="s">
-        <v>258</v>
+        <v>272</v>
       </c>
       <c r="E54">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="55" spans="1:5">
       <c r="A55" t="s">
-        <v>13</v>
+        <v>16</v>
       </c>
       <c r="B55" t="s">
-        <v>37</v>
+        <v>42</v>
       </c>
       <c r="C55" t="s">
         <v>90</v>
@@ -3140,19 +3140,19 @@
     </row>
     <row r="56" spans="1:5">
       <c r="A56" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B56" t="s">
-        <v>41</v>
+        <v>37</v>
       </c>
       <c r="C56" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="D56" t="s">
-        <v>272</v>
+        <v>273</v>
       </c>
       <c r="E56">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="57" spans="1:5">
@@ -3163,10 +3163,10 @@
         <v>41</v>
       </c>
       <c r="C57" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="D57" t="s">
-        <v>272</v>
+        <v>273</v>
       </c>
       <c r="E57">
         <v>2</v>
@@ -3180,13 +3180,13 @@
         <v>42</v>
       </c>
       <c r="C58" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="D58" t="s">
-        <v>272</v>
+        <v>273</v>
       </c>
       <c r="E58">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="59" spans="1:5">
@@ -3197,10 +3197,10 @@
         <v>37</v>
       </c>
       <c r="C59" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="D59" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
       <c r="E59">
         <v>2</v>
@@ -3214,13 +3214,13 @@
         <v>41</v>
       </c>
       <c r="C60" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="D60" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
       <c r="E60">
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
     <row r="61" spans="1:5">
@@ -3231,13 +3231,13 @@
         <v>42</v>
       </c>
       <c r="C61" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="D61" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
       <c r="E61">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="62" spans="1:5">
@@ -3248,10 +3248,10 @@
         <v>37</v>
       </c>
       <c r="C62" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="D62" t="s">
-        <v>274</v>
+        <v>275</v>
       </c>
       <c r="E62">
         <v>2</v>
@@ -3259,33 +3259,33 @@
     </row>
     <row r="63" spans="1:5">
       <c r="A63" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="B63" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="C63" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="D63" t="s">
-        <v>274</v>
+        <v>275</v>
       </c>
       <c r="E63">
-        <v>4</v>
+        <v>1</v>
       </c>
     </row>
     <row r="64" spans="1:5">
       <c r="A64" t="s">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="B64" t="s">
-        <v>42</v>
+        <v>37</v>
       </c>
       <c r="C64" t="s">
-        <v>92</v>
+        <v>94</v>
       </c>
       <c r="D64" t="s">
-        <v>274</v>
+        <v>276</v>
       </c>
       <c r="E64">
         <v>2</v>
@@ -3299,10 +3299,10 @@
         <v>37</v>
       </c>
       <c r="C65" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="D65" t="s">
-        <v>275</v>
+        <v>277</v>
       </c>
       <c r="E65">
         <v>2</v>
@@ -3310,19 +3310,19 @@
     </row>
     <row r="66" spans="1:5">
       <c r="A66" t="s">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="B66" t="s">
-        <v>42</v>
+        <v>37</v>
       </c>
       <c r="C66" t="s">
-        <v>93</v>
+        <v>96</v>
       </c>
       <c r="D66" t="s">
-        <v>275</v>
+        <v>278</v>
       </c>
       <c r="E66">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="67" spans="1:5">
@@ -3333,10 +3333,10 @@
         <v>37</v>
       </c>
       <c r="C67" t="s">
-        <v>94</v>
+        <v>97</v>
       </c>
       <c r="D67" t="s">
-        <v>276</v>
+        <v>279</v>
       </c>
       <c r="E67">
         <v>2</v>
@@ -3350,10 +3350,10 @@
         <v>37</v>
       </c>
       <c r="C68" t="s">
-        <v>95</v>
+        <v>98</v>
       </c>
       <c r="D68" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
       <c r="E68">
         <v>2</v>
@@ -3367,10 +3367,10 @@
         <v>37</v>
       </c>
       <c r="C69" t="s">
-        <v>96</v>
+        <v>99</v>
       </c>
       <c r="D69" t="s">
-        <v>278</v>
+        <v>280</v>
       </c>
       <c r="E69">
         <v>2</v>
@@ -3384,10 +3384,10 @@
         <v>37</v>
       </c>
       <c r="C70" t="s">
-        <v>97</v>
+        <v>100</v>
       </c>
       <c r="D70" t="s">
-        <v>279</v>
+        <v>272</v>
       </c>
       <c r="E70">
         <v>2</v>
@@ -3401,30 +3401,30 @@
         <v>37</v>
       </c>
       <c r="C71" t="s">
-        <v>98</v>
+        <v>101</v>
       </c>
       <c r="D71" t="s">
-        <v>276</v>
+        <v>270</v>
       </c>
       <c r="E71">
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
     <row r="72" spans="1:5">
       <c r="A72" t="s">
-        <v>13</v>
+        <v>16</v>
       </c>
       <c r="B72" t="s">
-        <v>37</v>
+        <v>42</v>
       </c>
       <c r="C72" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="D72" t="s">
-        <v>280</v>
+        <v>270</v>
       </c>
       <c r="E72">
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
     <row r="73" spans="1:5">
@@ -3435,13 +3435,13 @@
         <v>37</v>
       </c>
       <c r="C73" t="s">
-        <v>100</v>
+        <v>102</v>
       </c>
       <c r="D73" t="s">
-        <v>272</v>
+        <v>281</v>
       </c>
       <c r="E73">
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
     <row r="74" spans="1:5">
@@ -3452,10 +3452,10 @@
         <v>37</v>
       </c>
       <c r="C74" t="s">
-        <v>101</v>
+        <v>103</v>
       </c>
       <c r="D74" t="s">
-        <v>270</v>
+        <v>282</v>
       </c>
       <c r="E74">
         <v>4</v>
@@ -3463,16 +3463,16 @@
     </row>
     <row r="75" spans="1:5">
       <c r="A75" t="s">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="B75" t="s">
-        <v>42</v>
+        <v>37</v>
       </c>
       <c r="C75" t="s">
-        <v>101</v>
+        <v>104</v>
       </c>
       <c r="D75" t="s">
-        <v>270</v>
+        <v>258</v>
       </c>
       <c r="E75">
         <v>4</v>
@@ -3486,10 +3486,10 @@
         <v>37</v>
       </c>
       <c r="C76" t="s">
-        <v>102</v>
+        <v>105</v>
       </c>
       <c r="D76" t="s">
-        <v>281</v>
+        <v>283</v>
       </c>
       <c r="E76">
         <v>4</v>
@@ -3503,64 +3503,64 @@
         <v>37</v>
       </c>
       <c r="C77" t="s">
-        <v>103</v>
+        <v>106</v>
       </c>
       <c r="D77" t="s">
-        <v>282</v>
+        <v>284</v>
       </c>
       <c r="E77">
-        <v>4</v>
+        <v>40</v>
       </c>
     </row>
     <row r="78" spans="1:5">
       <c r="A78" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="B78" t="s">
-        <v>37</v>
+        <v>41</v>
       </c>
       <c r="C78" t="s">
-        <v>104</v>
+        <v>107</v>
       </c>
       <c r="D78" t="s">
-        <v>258</v>
+        <v>285</v>
       </c>
       <c r="E78">
-        <v>4</v>
+        <v>1</v>
       </c>
     </row>
     <row r="79" spans="1:5">
       <c r="A79" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="B79" t="s">
-        <v>37</v>
+        <v>41</v>
       </c>
       <c r="C79" t="s">
-        <v>105</v>
+        <v>107</v>
       </c>
       <c r="D79" t="s">
-        <v>283</v>
+        <v>285</v>
       </c>
       <c r="E79">
-        <v>4</v>
+        <v>1</v>
       </c>
     </row>
     <row r="80" spans="1:5">
       <c r="A80" t="s">
-        <v>13</v>
+        <v>16</v>
       </c>
       <c r="B80" t="s">
-        <v>37</v>
+        <v>42</v>
       </c>
       <c r="C80" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="D80" t="s">
-        <v>284</v>
+        <v>285</v>
       </c>
       <c r="E80">
-        <v>40</v>
+        <v>1</v>
       </c>
     </row>
     <row r="81" spans="1:5">
@@ -3571,10 +3571,10 @@
         <v>41</v>
       </c>
       <c r="C81" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="D81" t="s">
-        <v>285</v>
+        <v>286</v>
       </c>
       <c r="E81">
         <v>1</v>
@@ -3588,10 +3588,10 @@
         <v>41</v>
       </c>
       <c r="C82" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="D82" t="s">
-        <v>285</v>
+        <v>286</v>
       </c>
       <c r="E82">
         <v>1</v>
@@ -3605,13 +3605,13 @@
         <v>42</v>
       </c>
       <c r="C83" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="D83" t="s">
-        <v>285</v>
+        <v>286</v>
       </c>
       <c r="E83">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="84" spans="1:5">
@@ -3622,10 +3622,10 @@
         <v>41</v>
       </c>
       <c r="C84" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="D84" t="s">
-        <v>286</v>
+        <v>287</v>
       </c>
       <c r="E84">
         <v>1</v>
@@ -3639,10 +3639,10 @@
         <v>41</v>
       </c>
       <c r="C85" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="D85" t="s">
-        <v>286</v>
+        <v>287</v>
       </c>
       <c r="E85">
         <v>1</v>
@@ -3650,33 +3650,33 @@
     </row>
     <row r="86" spans="1:5">
       <c r="A86" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="B86" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="C86" t="s">
-        <v>108</v>
+        <v>110</v>
       </c>
       <c r="D86" t="s">
-        <v>286</v>
+        <v>288</v>
       </c>
       <c r="E86">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="87" spans="1:5">
       <c r="A87" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="B87" t="s">
         <v>41</v>
       </c>
       <c r="C87" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="D87" t="s">
-        <v>287</v>
+        <v>288</v>
       </c>
       <c r="E87">
         <v>1</v>
@@ -3684,16 +3684,16 @@
     </row>
     <row r="88" spans="1:5">
       <c r="A88" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B88" t="s">
         <v>41</v>
       </c>
       <c r="C88" t="s">
-        <v>109</v>
+        <v>111</v>
       </c>
       <c r="D88" t="s">
-        <v>287</v>
+        <v>289</v>
       </c>
       <c r="E88">
         <v>1</v>
@@ -3701,16 +3701,16 @@
     </row>
     <row r="89" spans="1:5">
       <c r="A89" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="B89" t="s">
         <v>41</v>
       </c>
       <c r="C89" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="D89" t="s">
-        <v>288</v>
+        <v>289</v>
       </c>
       <c r="E89">
         <v>1</v>
@@ -3718,16 +3718,16 @@
     </row>
     <row r="90" spans="1:5">
       <c r="A90" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B90" t="s">
         <v>41</v>
       </c>
       <c r="C90" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="D90" t="s">
-        <v>288</v>
+        <v>290</v>
       </c>
       <c r="E90">
         <v>1</v>
@@ -3735,16 +3735,16 @@
     </row>
     <row r="91" spans="1:5">
       <c r="A91" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="B91" t="s">
         <v>41</v>
       </c>
       <c r="C91" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="D91" t="s">
-        <v>289</v>
+        <v>290</v>
       </c>
       <c r="E91">
         <v>1</v>
@@ -3752,16 +3752,16 @@
     </row>
     <row r="92" spans="1:5">
       <c r="A92" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B92" t="s">
         <v>41</v>
       </c>
       <c r="C92" t="s">
-        <v>111</v>
+        <v>113</v>
       </c>
       <c r="D92" t="s">
-        <v>289</v>
+        <v>291</v>
       </c>
       <c r="E92">
         <v>1</v>
@@ -3769,16 +3769,16 @@
     </row>
     <row r="93" spans="1:5">
       <c r="A93" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="B93" t="s">
         <v>41</v>
       </c>
       <c r="C93" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="D93" t="s">
-        <v>290</v>
+        <v>291</v>
       </c>
       <c r="E93">
         <v>1</v>
@@ -3786,16 +3786,16 @@
     </row>
     <row r="94" spans="1:5">
       <c r="A94" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B94" t="s">
         <v>41</v>
       </c>
       <c r="C94" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
       <c r="D94" t="s">
-        <v>290</v>
+        <v>292</v>
       </c>
       <c r="E94">
         <v>1</v>
@@ -3803,16 +3803,16 @@
     </row>
     <row r="95" spans="1:5">
       <c r="A95" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="B95" t="s">
         <v>41</v>
       </c>
       <c r="C95" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="D95" t="s">
-        <v>291</v>
+        <v>292</v>
       </c>
       <c r="E95">
         <v>1</v>
@@ -3820,16 +3820,16 @@
     </row>
     <row r="96" spans="1:5">
       <c r="A96" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B96" t="s">
         <v>41</v>
       </c>
       <c r="C96" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="D96" t="s">
-        <v>291</v>
+        <v>293</v>
       </c>
       <c r="E96">
         <v>1</v>
@@ -3837,16 +3837,16 @@
     </row>
     <row r="97" spans="1:5">
       <c r="A97" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="B97" t="s">
         <v>41</v>
       </c>
       <c r="C97" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="D97" t="s">
-        <v>292</v>
+        <v>293</v>
       </c>
       <c r="E97">
         <v>1</v>
@@ -3854,16 +3854,16 @@
     </row>
     <row r="98" spans="1:5">
       <c r="A98" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B98" t="s">
         <v>41</v>
       </c>
       <c r="C98" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
       <c r="D98" t="s">
-        <v>292</v>
+        <v>294</v>
       </c>
       <c r="E98">
         <v>1</v>
@@ -3871,16 +3871,16 @@
     </row>
     <row r="99" spans="1:5">
       <c r="A99" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="B99" t="s">
         <v>41</v>
       </c>
       <c r="C99" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="D99" t="s">
-        <v>293</v>
+        <v>294</v>
       </c>
       <c r="E99">
         <v>1</v>
@@ -3888,16 +3888,16 @@
     </row>
     <row r="100" spans="1:5">
       <c r="A100" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B100" t="s">
         <v>41</v>
       </c>
       <c r="C100" t="s">
-        <v>115</v>
+        <v>117</v>
       </c>
       <c r="D100" t="s">
-        <v>293</v>
+        <v>295</v>
       </c>
       <c r="E100">
         <v>1</v>
@@ -3905,16 +3905,16 @@
     </row>
     <row r="101" spans="1:5">
       <c r="A101" t="s">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="B101" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="C101" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="D101" t="s">
-        <v>294</v>
+        <v>295</v>
       </c>
       <c r="E101">
         <v>1</v>
@@ -3922,16 +3922,16 @@
     </row>
     <row r="102" spans="1:5">
       <c r="A102" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B102" t="s">
         <v>41</v>
       </c>
       <c r="C102" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
       <c r="D102" t="s">
-        <v>294</v>
+        <v>296</v>
       </c>
       <c r="E102">
         <v>1</v>
@@ -3939,16 +3939,16 @@
     </row>
     <row r="103" spans="1:5">
       <c r="A103" t="s">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="B103" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="C103" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="D103" t="s">
-        <v>295</v>
+        <v>296</v>
       </c>
       <c r="E103">
         <v>1</v>
@@ -3956,16 +3956,16 @@
     </row>
     <row r="104" spans="1:5">
       <c r="A104" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="B104" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="C104" t="s">
-        <v>117</v>
+        <v>119</v>
       </c>
       <c r="D104" t="s">
-        <v>295</v>
+        <v>297</v>
       </c>
       <c r="E104">
         <v>1</v>
@@ -3973,16 +3973,16 @@
     </row>
     <row r="105" spans="1:5">
       <c r="A105" t="s">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="B105" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="C105" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="D105" t="s">
-        <v>296</v>
+        <v>297</v>
       </c>
       <c r="E105">
         <v>1</v>
@@ -3990,16 +3990,16 @@
     </row>
     <row r="106" spans="1:5">
       <c r="A106" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="B106" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="C106" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
       <c r="D106" t="s">
-        <v>296</v>
+        <v>298</v>
       </c>
       <c r="E106">
         <v>1</v>
@@ -4013,10 +4013,10 @@
         <v>41</v>
       </c>
       <c r="C107" t="s">
-        <v>119</v>
+        <v>121</v>
       </c>
       <c r="D107" t="s">
-        <v>297</v>
+        <v>299</v>
       </c>
       <c r="E107">
         <v>1</v>
@@ -4024,16 +4024,16 @@
     </row>
     <row r="108" spans="1:5">
       <c r="A108" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="B108" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="C108" t="s">
-        <v>119</v>
+        <v>122</v>
       </c>
       <c r="D108" t="s">
-        <v>297</v>
+        <v>300</v>
       </c>
       <c r="E108">
         <v>1</v>
@@ -4047,10 +4047,10 @@
         <v>41</v>
       </c>
       <c r="C109" t="s">
-        <v>120</v>
+        <v>123</v>
       </c>
       <c r="D109" t="s">
-        <v>298</v>
+        <v>301</v>
       </c>
       <c r="E109">
         <v>1</v>
@@ -4064,10 +4064,10 @@
         <v>41</v>
       </c>
       <c r="C110" t="s">
-        <v>121</v>
+        <v>124</v>
       </c>
       <c r="D110" t="s">
-        <v>299</v>
+        <v>302</v>
       </c>
       <c r="E110">
         <v>1</v>
@@ -4081,10 +4081,10 @@
         <v>41</v>
       </c>
       <c r="C111" t="s">
-        <v>122</v>
+        <v>125</v>
       </c>
       <c r="D111" t="s">
-        <v>300</v>
+        <v>303</v>
       </c>
       <c r="E111">
         <v>1</v>
@@ -4098,27 +4098,27 @@
         <v>41</v>
       </c>
       <c r="C112" t="s">
-        <v>123</v>
+        <v>126</v>
       </c>
       <c r="D112" t="s">
-        <v>301</v>
+        <v>304</v>
       </c>
       <c r="E112">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="113" spans="1:5">
       <c r="A113" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="B113" t="s">
         <v>41</v>
       </c>
       <c r="C113" t="s">
-        <v>124</v>
+        <v>126</v>
       </c>
       <c r="D113" t="s">
-        <v>302</v>
+        <v>304</v>
       </c>
       <c r="E113">
         <v>1</v>
@@ -4132,27 +4132,27 @@
         <v>41</v>
       </c>
       <c r="C114" t="s">
-        <v>125</v>
+        <v>127</v>
       </c>
       <c r="D114" t="s">
-        <v>303</v>
+        <v>305</v>
       </c>
       <c r="E114">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="115" spans="1:5">
       <c r="A115" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="B115" t="s">
         <v>41</v>
       </c>
       <c r="C115" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="D115" t="s">
-        <v>304</v>
+        <v>305</v>
       </c>
       <c r="E115">
         <v>2</v>
@@ -4160,19 +4160,19 @@
     </row>
     <row r="116" spans="1:5">
       <c r="A116" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="B116" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="C116" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="D116" t="s">
-        <v>304</v>
+        <v>305</v>
       </c>
       <c r="E116">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="117" spans="1:5">
@@ -4183,10 +4183,10 @@
         <v>41</v>
       </c>
       <c r="C117" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="D117" t="s">
-        <v>305</v>
+        <v>306</v>
       </c>
       <c r="E117">
         <v>2</v>
@@ -4200,10 +4200,10 @@
         <v>41</v>
       </c>
       <c r="C118" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="D118" t="s">
-        <v>305</v>
+        <v>306</v>
       </c>
       <c r="E118">
         <v>2</v>
@@ -4217,10 +4217,10 @@
         <v>42</v>
       </c>
       <c r="C119" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="D119" t="s">
-        <v>305</v>
+        <v>306</v>
       </c>
       <c r="E119">
         <v>2</v>
@@ -4234,10 +4234,10 @@
         <v>41</v>
       </c>
       <c r="C120" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="D120" t="s">
-        <v>306</v>
+        <v>307</v>
       </c>
       <c r="E120">
         <v>2</v>
@@ -4251,10 +4251,10 @@
         <v>41</v>
       </c>
       <c r="C121" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="D121" t="s">
-        <v>306</v>
+        <v>307</v>
       </c>
       <c r="E121">
         <v>2</v>
@@ -4262,16 +4262,16 @@
     </row>
     <row r="122" spans="1:5">
       <c r="A122" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="B122" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="C122" t="s">
-        <v>128</v>
+        <v>130</v>
       </c>
       <c r="D122" t="s">
-        <v>306</v>
+        <v>308</v>
       </c>
       <c r="E122">
         <v>2</v>
@@ -4279,16 +4279,16 @@
     </row>
     <row r="123" spans="1:5">
       <c r="A123" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="B123" t="s">
         <v>41</v>
       </c>
       <c r="C123" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="D123" t="s">
-        <v>307</v>
+        <v>308</v>
       </c>
       <c r="E123">
         <v>2</v>
@@ -4296,16 +4296,16 @@
     </row>
     <row r="124" spans="1:5">
       <c r="A124" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B124" t="s">
         <v>41</v>
       </c>
       <c r="C124" t="s">
-        <v>129</v>
+        <v>131</v>
       </c>
       <c r="D124" t="s">
-        <v>307</v>
+        <v>286</v>
       </c>
       <c r="E124">
         <v>2</v>
@@ -4313,36 +4313,36 @@
     </row>
     <row r="125" spans="1:5">
       <c r="A125" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="B125" t="s">
         <v>41</v>
       </c>
       <c r="C125" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="D125" t="s">
-        <v>308</v>
+        <v>286</v>
       </c>
       <c r="E125">
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
     <row r="126" spans="1:5">
       <c r="A126" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="B126" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="C126" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="D126" t="s">
-        <v>308</v>
+        <v>286</v>
       </c>
       <c r="E126">
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
     <row r="127" spans="1:5">
@@ -4353,10 +4353,10 @@
         <v>41</v>
       </c>
       <c r="C127" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="D127" t="s">
-        <v>286</v>
+        <v>309</v>
       </c>
       <c r="E127">
         <v>2</v>
@@ -4370,10 +4370,10 @@
         <v>41</v>
       </c>
       <c r="C128" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="D128" t="s">
-        <v>286</v>
+        <v>309</v>
       </c>
       <c r="E128">
         <v>4</v>
@@ -4381,19 +4381,19 @@
     </row>
     <row r="129" spans="1:5">
       <c r="A129" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="B129" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="C129" t="s">
-        <v>131</v>
+        <v>133</v>
       </c>
       <c r="D129" t="s">
-        <v>286</v>
+        <v>292</v>
       </c>
       <c r="E129">
-        <v>4</v>
+        <v>2</v>
       </c>
     </row>
     <row r="130" spans="1:5">
@@ -4404,10 +4404,10 @@
         <v>41</v>
       </c>
       <c r="C130" t="s">
-        <v>132</v>
+        <v>134</v>
       </c>
       <c r="D130" t="s">
-        <v>309</v>
+        <v>310</v>
       </c>
       <c r="E130">
         <v>2</v>
@@ -4415,19 +4415,19 @@
     </row>
     <row r="131" spans="1:5">
       <c r="A131" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B131" t="s">
         <v>41</v>
       </c>
       <c r="C131" t="s">
-        <v>132</v>
+        <v>135</v>
       </c>
       <c r="D131" t="s">
-        <v>309</v>
+        <v>311</v>
       </c>
       <c r="E131">
-        <v>4</v>
+        <v>2</v>
       </c>
     </row>
     <row r="132" spans="1:5">
@@ -4438,30 +4438,30 @@
         <v>41</v>
       </c>
       <c r="C132" t="s">
-        <v>133</v>
+        <v>136</v>
       </c>
       <c r="D132" t="s">
-        <v>292</v>
+        <v>312</v>
       </c>
       <c r="E132">
-        <v>2</v>
+        <v>5</v>
       </c>
     </row>
     <row r="133" spans="1:5">
       <c r="A133" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="B133" t="s">
         <v>41</v>
       </c>
       <c r="C133" t="s">
-        <v>134</v>
+        <v>136</v>
       </c>
       <c r="D133" t="s">
-        <v>310</v>
+        <v>312</v>
       </c>
       <c r="E133">
-        <v>2</v>
+        <v>5</v>
       </c>
     </row>
     <row r="134" spans="1:5">
@@ -4472,13 +4472,13 @@
         <v>41</v>
       </c>
       <c r="C134" t="s">
-        <v>135</v>
+        <v>137</v>
       </c>
       <c r="D134" t="s">
-        <v>311</v>
+        <v>313</v>
       </c>
       <c r="E134">
-        <v>2</v>
+        <v>7</v>
       </c>
     </row>
     <row r="135" spans="1:5">
@@ -4489,81 +4489,81 @@
         <v>41</v>
       </c>
       <c r="C135" t="s">
-        <v>136</v>
+        <v>138</v>
       </c>
       <c r="D135" t="s">
-        <v>312</v>
+        <v>314</v>
       </c>
       <c r="E135">
-        <v>5</v>
+        <v>10</v>
       </c>
     </row>
     <row r="136" spans="1:5">
       <c r="A136" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B136" t="s">
         <v>41</v>
       </c>
       <c r="C136" t="s">
-        <v>136</v>
+        <v>139</v>
       </c>
       <c r="D136" t="s">
-        <v>312</v>
+        <v>315</v>
       </c>
       <c r="E136">
-        <v>5</v>
+        <v>30</v>
       </c>
     </row>
     <row r="137" spans="1:5">
       <c r="A137" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="B137" t="s">
         <v>41</v>
       </c>
       <c r="C137" t="s">
-        <v>137</v>
+        <v>139</v>
       </c>
       <c r="D137" t="s">
-        <v>313</v>
+        <v>315</v>
       </c>
       <c r="E137">
-        <v>7</v>
+        <v>30</v>
       </c>
     </row>
     <row r="138" spans="1:5">
       <c r="A138" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="B138" t="s">
         <v>41</v>
       </c>
       <c r="C138" t="s">
-        <v>138</v>
+        <v>140</v>
       </c>
       <c r="D138" t="s">
-        <v>314</v>
+        <v>316</v>
       </c>
       <c r="E138">
-        <v>10</v>
+        <v>1</v>
       </c>
     </row>
     <row r="139" spans="1:5">
       <c r="A139" t="s">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="B139" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="C139" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="D139" t="s">
-        <v>315</v>
+        <v>316</v>
       </c>
       <c r="E139">
-        <v>30</v>
+        <v>1</v>
       </c>
     </row>
     <row r="140" spans="1:5">
@@ -4574,27 +4574,27 @@
         <v>41</v>
       </c>
       <c r="C140" t="s">
-        <v>139</v>
+        <v>141</v>
       </c>
       <c r="D140" t="s">
-        <v>315</v>
+        <v>317</v>
       </c>
       <c r="E140">
-        <v>30</v>
+        <v>1</v>
       </c>
     </row>
     <row r="141" spans="1:5">
       <c r="A141" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="B141" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="C141" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="D141" t="s">
-        <v>316</v>
+        <v>317</v>
       </c>
       <c r="E141">
         <v>1</v>
@@ -4602,16 +4602,16 @@
     </row>
     <row r="142" spans="1:5">
       <c r="A142" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="B142" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="C142" t="s">
-        <v>140</v>
+        <v>142</v>
       </c>
       <c r="D142" t="s">
-        <v>316</v>
+        <v>318</v>
       </c>
       <c r="E142">
         <v>1</v>
@@ -4625,10 +4625,10 @@
         <v>41</v>
       </c>
       <c r="C143" t="s">
-        <v>141</v>
+        <v>143</v>
       </c>
       <c r="D143" t="s">
-        <v>317</v>
+        <v>319</v>
       </c>
       <c r="E143">
         <v>1</v>
@@ -4636,16 +4636,16 @@
     </row>
     <row r="144" spans="1:5">
       <c r="A144" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="B144" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="C144" t="s">
-        <v>141</v>
+        <v>144</v>
       </c>
       <c r="D144" t="s">
-        <v>317</v>
+        <v>320</v>
       </c>
       <c r="E144">
         <v>1</v>
@@ -4659,10 +4659,10 @@
         <v>41</v>
       </c>
       <c r="C145" t="s">
-        <v>142</v>
+        <v>145</v>
       </c>
       <c r="D145" t="s">
-        <v>318</v>
+        <v>321</v>
       </c>
       <c r="E145">
         <v>1</v>
@@ -4676,10 +4676,10 @@
         <v>41</v>
       </c>
       <c r="C146" t="s">
-        <v>143</v>
+        <v>146</v>
       </c>
       <c r="D146" t="s">
-        <v>319</v>
+        <v>322</v>
       </c>
       <c r="E146">
         <v>1</v>
@@ -4693,10 +4693,10 @@
         <v>41</v>
       </c>
       <c r="C147" t="s">
-        <v>144</v>
+        <v>147</v>
       </c>
       <c r="D147" t="s">
-        <v>320</v>
+        <v>323</v>
       </c>
       <c r="E147">
         <v>1</v>
@@ -4710,10 +4710,10 @@
         <v>41</v>
       </c>
       <c r="C148" t="s">
-        <v>145</v>
+        <v>148</v>
       </c>
       <c r="D148" t="s">
-        <v>321</v>
+        <v>324</v>
       </c>
       <c r="E148">
         <v>1</v>
@@ -4727,10 +4727,10 @@
         <v>41</v>
       </c>
       <c r="C149" t="s">
-        <v>146</v>
+        <v>149</v>
       </c>
       <c r="D149" t="s">
-        <v>322</v>
+        <v>325</v>
       </c>
       <c r="E149">
         <v>1</v>
@@ -4744,10 +4744,10 @@
         <v>41</v>
       </c>
       <c r="C150" t="s">
-        <v>147</v>
+        <v>150</v>
       </c>
       <c r="D150" t="s">
-        <v>323</v>
+        <v>326</v>
       </c>
       <c r="E150">
         <v>1</v>
@@ -4761,10 +4761,10 @@
         <v>41</v>
       </c>
       <c r="C151" t="s">
-        <v>148</v>
+        <v>151</v>
       </c>
       <c r="D151" t="s">
-        <v>324</v>
+        <v>327</v>
       </c>
       <c r="E151">
         <v>1</v>
@@ -4778,10 +4778,10 @@
         <v>41</v>
       </c>
       <c r="C152" t="s">
-        <v>149</v>
+        <v>152</v>
       </c>
       <c r="D152" t="s">
-        <v>325</v>
+        <v>328</v>
       </c>
       <c r="E152">
         <v>1</v>
@@ -4795,10 +4795,10 @@
         <v>41</v>
       </c>
       <c r="C153" t="s">
-        <v>150</v>
+        <v>153</v>
       </c>
       <c r="D153" t="s">
-        <v>326</v>
+        <v>329</v>
       </c>
       <c r="E153">
         <v>1</v>
@@ -4812,10 +4812,10 @@
         <v>41</v>
       </c>
       <c r="C154" t="s">
-        <v>151</v>
+        <v>154</v>
       </c>
       <c r="D154" t="s">
-        <v>327</v>
+        <v>330</v>
       </c>
       <c r="E154">
         <v>1</v>
@@ -4829,10 +4829,10 @@
         <v>41</v>
       </c>
       <c r="C155" t="s">
-        <v>152</v>
+        <v>155</v>
       </c>
       <c r="D155" t="s">
-        <v>328</v>
+        <v>331</v>
       </c>
       <c r="E155">
         <v>1</v>
@@ -4846,10 +4846,10 @@
         <v>41</v>
       </c>
       <c r="C156" t="s">
-        <v>153</v>
+        <v>156</v>
       </c>
       <c r="D156" t="s">
-        <v>329</v>
+        <v>332</v>
       </c>
       <c r="E156">
         <v>1</v>
@@ -4863,10 +4863,10 @@
         <v>41</v>
       </c>
       <c r="C157" t="s">
-        <v>154</v>
+        <v>157</v>
       </c>
       <c r="D157" t="s">
-        <v>330</v>
+        <v>333</v>
       </c>
       <c r="E157">
         <v>1</v>
@@ -4880,10 +4880,10 @@
         <v>41</v>
       </c>
       <c r="C158" t="s">
-        <v>155</v>
+        <v>158</v>
       </c>
       <c r="D158" t="s">
-        <v>331</v>
+        <v>334</v>
       </c>
       <c r="E158">
         <v>1</v>
@@ -4897,10 +4897,10 @@
         <v>41</v>
       </c>
       <c r="C159" t="s">
-        <v>156</v>
+        <v>159</v>
       </c>
       <c r="D159" t="s">
-        <v>332</v>
+        <v>335</v>
       </c>
       <c r="E159">
         <v>1</v>
@@ -4914,10 +4914,10 @@
         <v>41</v>
       </c>
       <c r="C160" t="s">
-        <v>157</v>
+        <v>160</v>
       </c>
       <c r="D160" t="s">
-        <v>333</v>
+        <v>336</v>
       </c>
       <c r="E160">
         <v>1</v>
@@ -4931,10 +4931,10 @@
         <v>41</v>
       </c>
       <c r="C161" t="s">
-        <v>158</v>
+        <v>161</v>
       </c>
       <c r="D161" t="s">
-        <v>334</v>
+        <v>337</v>
       </c>
       <c r="E161">
         <v>1</v>
@@ -4948,10 +4948,10 @@
         <v>41</v>
       </c>
       <c r="C162" t="s">
-        <v>159</v>
+        <v>162</v>
       </c>
       <c r="D162" t="s">
-        <v>335</v>
+        <v>338</v>
       </c>
       <c r="E162">
         <v>1</v>
@@ -4965,10 +4965,10 @@
         <v>41</v>
       </c>
       <c r="C163" t="s">
-        <v>160</v>
+        <v>163</v>
       </c>
       <c r="D163" t="s">
-        <v>336</v>
+        <v>339</v>
       </c>
       <c r="E163">
         <v>1</v>
@@ -4982,10 +4982,10 @@
         <v>41</v>
       </c>
       <c r="C164" t="s">
-        <v>161</v>
+        <v>164</v>
       </c>
       <c r="D164" t="s">
-        <v>337</v>
+        <v>340</v>
       </c>
       <c r="E164">
         <v>1</v>
@@ -4999,10 +4999,10 @@
         <v>41</v>
       </c>
       <c r="C165" t="s">
-        <v>162</v>
+        <v>165</v>
       </c>
       <c r="D165" t="s">
-        <v>338</v>
+        <v>341</v>
       </c>
       <c r="E165">
         <v>1</v>
@@ -5016,10 +5016,10 @@
         <v>41</v>
       </c>
       <c r="C166" t="s">
-        <v>163</v>
+        <v>166</v>
       </c>
       <c r="D166" t="s">
-        <v>339</v>
+        <v>342</v>
       </c>
       <c r="E166">
         <v>1</v>
@@ -5033,10 +5033,10 @@
         <v>41</v>
       </c>
       <c r="C167" t="s">
-        <v>164</v>
+        <v>167</v>
       </c>
       <c r="D167" t="s">
-        <v>340</v>
+        <v>343</v>
       </c>
       <c r="E167">
         <v>1</v>
@@ -5050,10 +5050,10 @@
         <v>41</v>
       </c>
       <c r="C168" t="s">
-        <v>165</v>
+        <v>168</v>
       </c>
       <c r="D168" t="s">
-        <v>341</v>
+        <v>344</v>
       </c>
       <c r="E168">
         <v>1</v>
@@ -5067,10 +5067,10 @@
         <v>41</v>
       </c>
       <c r="C169" t="s">
-        <v>166</v>
+        <v>169</v>
       </c>
       <c r="D169" t="s">
-        <v>342</v>
+        <v>345</v>
       </c>
       <c r="E169">
         <v>1</v>
@@ -5084,10 +5084,10 @@
         <v>41</v>
       </c>
       <c r="C170" t="s">
-        <v>167</v>
+        <v>170</v>
       </c>
       <c r="D170" t="s">
-        <v>343</v>
+        <v>346</v>
       </c>
       <c r="E170">
         <v>1</v>
@@ -5101,10 +5101,10 @@
         <v>41</v>
       </c>
       <c r="C171" t="s">
-        <v>168</v>
+        <v>171</v>
       </c>
       <c r="D171" t="s">
-        <v>344</v>
+        <v>347</v>
       </c>
       <c r="E171">
         <v>1</v>
@@ -5118,13 +5118,13 @@
         <v>41</v>
       </c>
       <c r="C172" t="s">
-        <v>169</v>
+        <v>172</v>
       </c>
       <c r="D172" t="s">
-        <v>345</v>
+        <v>332</v>
       </c>
       <c r="E172">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="173" spans="1:5">
@@ -5135,13 +5135,13 @@
         <v>41</v>
       </c>
       <c r="C173" t="s">
-        <v>170</v>
+        <v>173</v>
       </c>
       <c r="D173" t="s">
-        <v>346</v>
+        <v>348</v>
       </c>
       <c r="E173">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="174" spans="1:5">
@@ -5152,13 +5152,13 @@
         <v>41</v>
       </c>
       <c r="C174" t="s">
-        <v>171</v>
+        <v>174</v>
       </c>
       <c r="D174" t="s">
-        <v>347</v>
+        <v>349</v>
       </c>
       <c r="E174">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="175" spans="1:5">
@@ -5169,10 +5169,10 @@
         <v>41</v>
       </c>
       <c r="C175" t="s">
-        <v>172</v>
+        <v>175</v>
       </c>
       <c r="D175" t="s">
-        <v>332</v>
+        <v>350</v>
       </c>
       <c r="E175">
         <v>2</v>
@@ -5186,10 +5186,10 @@
         <v>41</v>
       </c>
       <c r="C176" t="s">
-        <v>173</v>
+        <v>176</v>
       </c>
       <c r="D176" t="s">
-        <v>348</v>
+        <v>351</v>
       </c>
       <c r="E176">
         <v>2</v>
@@ -5203,13 +5203,13 @@
         <v>41</v>
       </c>
       <c r="C177" t="s">
-        <v>174</v>
+        <v>177</v>
       </c>
       <c r="D177" t="s">
-        <v>349</v>
+        <v>352</v>
       </c>
       <c r="E177">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="178" spans="1:5">
@@ -5220,13 +5220,13 @@
         <v>41</v>
       </c>
       <c r="C178" t="s">
-        <v>175</v>
+        <v>178</v>
       </c>
       <c r="D178" t="s">
-        <v>350</v>
+        <v>315</v>
       </c>
       <c r="E178">
-        <v>2</v>
+        <v>5</v>
       </c>
     </row>
     <row r="179" spans="1:5">
@@ -5237,13 +5237,13 @@
         <v>41</v>
       </c>
       <c r="C179" t="s">
-        <v>176</v>
+        <v>179</v>
       </c>
       <c r="D179" t="s">
-        <v>351</v>
+        <v>353</v>
       </c>
       <c r="E179">
-        <v>2</v>
+        <v>8</v>
       </c>
     </row>
     <row r="180" spans="1:5">
@@ -5254,13 +5254,13 @@
         <v>41</v>
       </c>
       <c r="C180" t="s">
-        <v>177</v>
+        <v>180</v>
       </c>
       <c r="D180" t="s">
-        <v>352</v>
+        <v>258</v>
       </c>
       <c r="E180">
-        <v>3</v>
+        <v>8</v>
       </c>
     </row>
     <row r="181" spans="1:5">
@@ -5271,64 +5271,64 @@
         <v>41</v>
       </c>
       <c r="C181" t="s">
-        <v>178</v>
+        <v>181</v>
       </c>
       <c r="D181" t="s">
-        <v>315</v>
+        <v>354</v>
       </c>
       <c r="E181">
-        <v>5</v>
+        <v>10</v>
       </c>
     </row>
     <row r="182" spans="1:5">
       <c r="A182" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="B182" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="C182" t="s">
-        <v>179</v>
+        <v>182</v>
       </c>
       <c r="D182" t="s">
-        <v>353</v>
+        <v>342</v>
       </c>
       <c r="E182">
-        <v>8</v>
+        <v>1</v>
       </c>
     </row>
     <row r="183" spans="1:5">
       <c r="A183" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="B183" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="C183" t="s">
-        <v>180</v>
+        <v>183</v>
       </c>
       <c r="D183" t="s">
-        <v>258</v>
+        <v>355</v>
       </c>
       <c r="E183">
-        <v>8</v>
+        <v>1</v>
       </c>
     </row>
     <row r="184" spans="1:5">
       <c r="A184" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="B184" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="C184" t="s">
-        <v>181</v>
+        <v>184</v>
       </c>
       <c r="D184" t="s">
-        <v>354</v>
+        <v>356</v>
       </c>
       <c r="E184">
-        <v>10</v>
+        <v>1</v>
       </c>
     </row>
     <row r="185" spans="1:5">
@@ -5339,10 +5339,10 @@
         <v>42</v>
       </c>
       <c r="C185" t="s">
-        <v>182</v>
+        <v>185</v>
       </c>
       <c r="D185" t="s">
-        <v>342</v>
+        <v>357</v>
       </c>
       <c r="E185">
         <v>1</v>
@@ -5356,10 +5356,10 @@
         <v>42</v>
       </c>
       <c r="C186" t="s">
-        <v>183</v>
+        <v>186</v>
       </c>
       <c r="D186" t="s">
-        <v>355</v>
+        <v>358</v>
       </c>
       <c r="E186">
         <v>1</v>
@@ -5373,10 +5373,10 @@
         <v>42</v>
       </c>
       <c r="C187" t="s">
-        <v>184</v>
+        <v>187</v>
       </c>
       <c r="D187" t="s">
-        <v>356</v>
+        <v>278</v>
       </c>
       <c r="E187">
         <v>1</v>
@@ -5390,10 +5390,10 @@
         <v>42</v>
       </c>
       <c r="C188" t="s">
-        <v>185</v>
+        <v>188</v>
       </c>
       <c r="D188" t="s">
-        <v>357</v>
+        <v>359</v>
       </c>
       <c r="E188">
         <v>1</v>
@@ -5407,10 +5407,10 @@
         <v>42</v>
       </c>
       <c r="C189" t="s">
-        <v>186</v>
+        <v>189</v>
       </c>
       <c r="D189" t="s">
-        <v>358</v>
+        <v>360</v>
       </c>
       <c r="E189">
         <v>1</v>
@@ -5424,10 +5424,10 @@
         <v>42</v>
       </c>
       <c r="C190" t="s">
-        <v>187</v>
+        <v>190</v>
       </c>
       <c r="D190" t="s">
-        <v>278</v>
+        <v>361</v>
       </c>
       <c r="E190">
         <v>1</v>
@@ -5441,10 +5441,10 @@
         <v>42</v>
       </c>
       <c r="C191" t="s">
-        <v>188</v>
+        <v>191</v>
       </c>
       <c r="D191" t="s">
-        <v>359</v>
+        <v>362</v>
       </c>
       <c r="E191">
         <v>1</v>
@@ -5458,10 +5458,10 @@
         <v>42</v>
       </c>
       <c r="C192" t="s">
-        <v>189</v>
+        <v>192</v>
       </c>
       <c r="D192" t="s">
-        <v>360</v>
+        <v>363</v>
       </c>
       <c r="E192">
         <v>1</v>
@@ -5475,10 +5475,10 @@
         <v>42</v>
       </c>
       <c r="C193" t="s">
-        <v>190</v>
+        <v>193</v>
       </c>
       <c r="D193" t="s">
-        <v>361</v>
+        <v>364</v>
       </c>
       <c r="E193">
         <v>1</v>
@@ -5492,10 +5492,10 @@
         <v>42</v>
       </c>
       <c r="C194" t="s">
-        <v>191</v>
+        <v>194</v>
       </c>
       <c r="D194" t="s">
-        <v>362</v>
+        <v>365</v>
       </c>
       <c r="E194">
         <v>1</v>
@@ -5509,10 +5509,10 @@
         <v>42</v>
       </c>
       <c r="C195" t="s">
-        <v>192</v>
+        <v>195</v>
       </c>
       <c r="D195" t="s">
-        <v>363</v>
+        <v>366</v>
       </c>
       <c r="E195">
         <v>1</v>
@@ -5526,10 +5526,10 @@
         <v>42</v>
       </c>
       <c r="C196" t="s">
-        <v>193</v>
+        <v>196</v>
       </c>
       <c r="D196" t="s">
-        <v>364</v>
+        <v>367</v>
       </c>
       <c r="E196">
         <v>1</v>
@@ -5543,10 +5543,10 @@
         <v>42</v>
       </c>
       <c r="C197" t="s">
-        <v>194</v>
+        <v>197</v>
       </c>
       <c r="D197" t="s">
-        <v>365</v>
+        <v>368</v>
       </c>
       <c r="E197">
         <v>1</v>
@@ -5560,10 +5560,10 @@
         <v>42</v>
       </c>
       <c r="C198" t="s">
-        <v>195</v>
+        <v>198</v>
       </c>
       <c r="D198" t="s">
-        <v>366</v>
+        <v>369</v>
       </c>
       <c r="E198">
         <v>1</v>
@@ -5577,10 +5577,10 @@
         <v>42</v>
       </c>
       <c r="C199" t="s">
-        <v>196</v>
+        <v>199</v>
       </c>
       <c r="D199" t="s">
-        <v>367</v>
+        <v>370</v>
       </c>
       <c r="E199">
         <v>1</v>
@@ -5594,10 +5594,10 @@
         <v>42</v>
       </c>
       <c r="C200" t="s">
-        <v>197</v>
+        <v>200</v>
       </c>
       <c r="D200" t="s">
-        <v>368</v>
+        <v>371</v>
       </c>
       <c r="E200">
         <v>1</v>
@@ -5611,10 +5611,10 @@
         <v>42</v>
       </c>
       <c r="C201" t="s">
-        <v>198</v>
+        <v>201</v>
       </c>
       <c r="D201" t="s">
-        <v>369</v>
+        <v>372</v>
       </c>
       <c r="E201">
         <v>1</v>
@@ -5628,10 +5628,10 @@
         <v>42</v>
       </c>
       <c r="C202" t="s">
-        <v>199</v>
+        <v>202</v>
       </c>
       <c r="D202" t="s">
-        <v>370</v>
+        <v>373</v>
       </c>
       <c r="E202">
         <v>1</v>
@@ -5645,10 +5645,10 @@
         <v>42</v>
       </c>
       <c r="C203" t="s">
-        <v>200</v>
+        <v>203</v>
       </c>
       <c r="D203" t="s">
-        <v>371</v>
+        <v>374</v>
       </c>
       <c r="E203">
         <v>1</v>
@@ -5662,10 +5662,10 @@
         <v>42</v>
       </c>
       <c r="C204" t="s">
-        <v>201</v>
+        <v>204</v>
       </c>
       <c r="D204" t="s">
-        <v>372</v>
+        <v>375</v>
       </c>
       <c r="E204">
         <v>1</v>
@@ -5679,10 +5679,10 @@
         <v>42</v>
       </c>
       <c r="C205" t="s">
-        <v>202</v>
+        <v>205</v>
       </c>
       <c r="D205" t="s">
-        <v>373</v>
+        <v>376</v>
       </c>
       <c r="E205">
         <v>1</v>
@@ -5696,10 +5696,10 @@
         <v>42</v>
       </c>
       <c r="C206" t="s">
-        <v>203</v>
+        <v>206</v>
       </c>
       <c r="D206" t="s">
-        <v>374</v>
+        <v>377</v>
       </c>
       <c r="E206">
         <v>1</v>
@@ -5713,10 +5713,10 @@
         <v>42</v>
       </c>
       <c r="C207" t="s">
-        <v>204</v>
+        <v>207</v>
       </c>
       <c r="D207" t="s">
-        <v>375</v>
+        <v>378</v>
       </c>
       <c r="E207">
         <v>1</v>
@@ -5730,10 +5730,10 @@
         <v>42</v>
       </c>
       <c r="C208" t="s">
-        <v>205</v>
+        <v>208</v>
       </c>
       <c r="D208" t="s">
-        <v>376</v>
+        <v>379</v>
       </c>
       <c r="E208">
         <v>1</v>
@@ -5747,10 +5747,10 @@
         <v>42</v>
       </c>
       <c r="C209" t="s">
-        <v>206</v>
+        <v>209</v>
       </c>
       <c r="D209" t="s">
-        <v>377</v>
+        <v>380</v>
       </c>
       <c r="E209">
         <v>1</v>
@@ -5764,10 +5764,10 @@
         <v>42</v>
       </c>
       <c r="C210" t="s">
-        <v>207</v>
+        <v>210</v>
       </c>
       <c r="D210" t="s">
-        <v>378</v>
+        <v>381</v>
       </c>
       <c r="E210">
         <v>1</v>
@@ -5781,13 +5781,13 @@
         <v>42</v>
       </c>
       <c r="C211" t="s">
-        <v>208</v>
+        <v>211</v>
       </c>
       <c r="D211" t="s">
-        <v>379</v>
+        <v>382</v>
       </c>
       <c r="E211">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="212" spans="1:5">
@@ -5798,13 +5798,13 @@
         <v>42</v>
       </c>
       <c r="C212" t="s">
-        <v>209</v>
+        <v>212</v>
       </c>
       <c r="D212" t="s">
-        <v>380</v>
+        <v>383</v>
       </c>
       <c r="E212">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="213" spans="1:5">
@@ -5815,13 +5815,13 @@
         <v>42</v>
       </c>
       <c r="C213" t="s">
-        <v>210</v>
+        <v>213</v>
       </c>
       <c r="D213" t="s">
-        <v>381</v>
+        <v>384</v>
       </c>
       <c r="E213">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="214" spans="1:5">
@@ -5832,10 +5832,10 @@
         <v>42</v>
       </c>
       <c r="C214" t="s">
-        <v>211</v>
+        <v>214</v>
       </c>
       <c r="D214" t="s">
-        <v>382</v>
+        <v>385</v>
       </c>
       <c r="E214">
         <v>2</v>
@@ -5849,10 +5849,10 @@
         <v>42</v>
       </c>
       <c r="C215" t="s">
-        <v>212</v>
+        <v>215</v>
       </c>
       <c r="D215" t="s">
-        <v>383</v>
+        <v>386</v>
       </c>
       <c r="E215">
         <v>2</v>
@@ -5866,10 +5866,10 @@
         <v>42</v>
       </c>
       <c r="C216" t="s">
-        <v>213</v>
+        <v>216</v>
       </c>
       <c r="D216" t="s">
-        <v>384</v>
+        <v>387</v>
       </c>
       <c r="E216">
         <v>2</v>
@@ -5883,10 +5883,10 @@
         <v>42</v>
       </c>
       <c r="C217" t="s">
-        <v>214</v>
+        <v>217</v>
       </c>
       <c r="D217" t="s">
-        <v>385</v>
+        <v>388</v>
       </c>
       <c r="E217">
         <v>2</v>
@@ -5900,10 +5900,10 @@
         <v>42</v>
       </c>
       <c r="C218" t="s">
-        <v>215</v>
+        <v>218</v>
       </c>
       <c r="D218" t="s">
-        <v>386</v>
+        <v>389</v>
       </c>
       <c r="E218">
         <v>2</v>
@@ -5917,10 +5917,10 @@
         <v>42</v>
       </c>
       <c r="C219" t="s">
-        <v>216</v>
+        <v>219</v>
       </c>
       <c r="D219" t="s">
-        <v>387</v>
+        <v>390</v>
       </c>
       <c r="E219">
         <v>2</v>
@@ -5934,10 +5934,10 @@
         <v>42</v>
       </c>
       <c r="C220" t="s">
-        <v>217</v>
+        <v>220</v>
       </c>
       <c r="D220" t="s">
-        <v>388</v>
+        <v>390</v>
       </c>
       <c r="E220">
         <v>2</v>
@@ -5951,10 +5951,10 @@
         <v>42</v>
       </c>
       <c r="C221" t="s">
-        <v>218</v>
+        <v>221</v>
       </c>
       <c r="D221" t="s">
-        <v>389</v>
+        <v>391</v>
       </c>
       <c r="E221">
         <v>2</v>
@@ -5968,10 +5968,10 @@
         <v>42</v>
       </c>
       <c r="C222" t="s">
-        <v>219</v>
+        <v>222</v>
       </c>
       <c r="D222" t="s">
-        <v>390</v>
+        <v>392</v>
       </c>
       <c r="E222">
         <v>2</v>
@@ -5985,13 +5985,13 @@
         <v>42</v>
       </c>
       <c r="C223" t="s">
-        <v>220</v>
+        <v>223</v>
       </c>
       <c r="D223" t="s">
-        <v>390</v>
+        <v>393</v>
       </c>
       <c r="E223">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="224" spans="1:5">
@@ -6002,13 +6002,13 @@
         <v>42</v>
       </c>
       <c r="C224" t="s">
-        <v>221</v>
+        <v>224</v>
       </c>
       <c r="D224" t="s">
-        <v>391</v>
+        <v>278</v>
       </c>
       <c r="E224">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="225" spans="1:5">
@@ -6019,13 +6019,13 @@
         <v>42</v>
       </c>
       <c r="C225" t="s">
-        <v>222</v>
+        <v>225</v>
       </c>
       <c r="D225" t="s">
-        <v>392</v>
+        <v>394</v>
       </c>
       <c r="E225">
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
     <row r="226" spans="1:5">
@@ -6036,13 +6036,13 @@
         <v>42</v>
       </c>
       <c r="C226" t="s">
-        <v>223</v>
+        <v>226</v>
       </c>
       <c r="D226" t="s">
-        <v>393</v>
+        <v>395</v>
       </c>
       <c r="E226">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="227" spans="1:5">
@@ -6053,13 +6053,13 @@
         <v>42</v>
       </c>
       <c r="C227" t="s">
-        <v>224</v>
+        <v>227</v>
       </c>
       <c r="D227" t="s">
-        <v>278</v>
+        <v>396</v>
       </c>
       <c r="E227">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="228" spans="1:5">
@@ -6070,10 +6070,10 @@
         <v>42</v>
       </c>
       <c r="C228" t="s">
-        <v>225</v>
+        <v>228</v>
       </c>
       <c r="D228" t="s">
-        <v>394</v>
+        <v>397</v>
       </c>
       <c r="E228">
         <v>4</v>
@@ -6087,10 +6087,10 @@
         <v>42</v>
       </c>
       <c r="C229" t="s">
-        <v>226</v>
+        <v>229</v>
       </c>
       <c r="D229" t="s">
-        <v>395</v>
+        <v>398</v>
       </c>
       <c r="E229">
         <v>4</v>
@@ -6104,13 +6104,13 @@
         <v>42</v>
       </c>
       <c r="C230" t="s">
-        <v>227</v>
+        <v>230</v>
       </c>
       <c r="D230" t="s">
-        <v>396</v>
+        <v>399</v>
       </c>
       <c r="E230">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="231" spans="1:5">
@@ -6121,13 +6121,13 @@
         <v>42</v>
       </c>
       <c r="C231" t="s">
-        <v>228</v>
+        <v>231</v>
       </c>
       <c r="D231" t="s">
-        <v>397</v>
+        <v>400</v>
       </c>
       <c r="E231">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="232" spans="1:5">
@@ -6138,13 +6138,13 @@
         <v>42</v>
       </c>
       <c r="C232" t="s">
-        <v>229</v>
+        <v>232</v>
       </c>
       <c r="D232" t="s">
-        <v>398</v>
+        <v>401</v>
       </c>
       <c r="E232">
-        <v>4</v>
+        <v>6</v>
       </c>
     </row>
     <row r="233" spans="1:5">
@@ -6155,13 +6155,13 @@
         <v>42</v>
       </c>
       <c r="C233" t="s">
-        <v>230</v>
+        <v>233</v>
       </c>
       <c r="D233" t="s">
-        <v>399</v>
+        <v>402</v>
       </c>
       <c r="E233">
-        <v>5</v>
+        <v>8</v>
       </c>
     </row>
     <row r="234" spans="1:5">
@@ -6172,13 +6172,13 @@
         <v>42</v>
       </c>
       <c r="C234" t="s">
-        <v>231</v>
+        <v>234</v>
       </c>
       <c r="D234" t="s">
-        <v>400</v>
+        <v>403</v>
       </c>
       <c r="E234">
-        <v>5</v>
+        <v>10</v>
       </c>
     </row>
     <row r="235" spans="1:5">
@@ -6189,13 +6189,13 @@
         <v>42</v>
       </c>
       <c r="C235" t="s">
-        <v>232</v>
+        <v>235</v>
       </c>
       <c r="D235" t="s">
-        <v>401</v>
+        <v>403</v>
       </c>
       <c r="E235">
-        <v>6</v>
+        <v>10</v>
       </c>
     </row>
     <row r="236" spans="1:5">
@@ -6206,13 +6206,13 @@
         <v>42</v>
       </c>
       <c r="C236" t="s">
-        <v>233</v>
+        <v>236</v>
       </c>
       <c r="D236" t="s">
-        <v>402</v>
+        <v>276</v>
       </c>
       <c r="E236">
-        <v>8</v>
+        <v>12</v>
       </c>
     </row>
     <row r="237" spans="1:5">
@@ -6223,13 +6223,13 @@
         <v>42</v>
       </c>
       <c r="C237" t="s">
-        <v>234</v>
+        <v>237</v>
       </c>
       <c r="D237" t="s">
-        <v>403</v>
+        <v>404</v>
       </c>
       <c r="E237">
-        <v>10</v>
+        <v>12</v>
       </c>
     </row>
     <row r="238" spans="1:5">
@@ -6240,13 +6240,13 @@
         <v>42</v>
       </c>
       <c r="C238" t="s">
-        <v>235</v>
+        <v>238</v>
       </c>
       <c r="D238" t="s">
-        <v>403</v>
+        <v>405</v>
       </c>
       <c r="E238">
-        <v>10</v>
+        <v>14</v>
       </c>
     </row>
     <row r="239" spans="1:5">
@@ -6257,13 +6257,13 @@
         <v>42</v>
       </c>
       <c r="C239" t="s">
-        <v>236</v>
+        <v>239</v>
       </c>
       <c r="D239" t="s">
-        <v>276</v>
+        <v>406</v>
       </c>
       <c r="E239">
-        <v>12</v>
+        <v>15</v>
       </c>
     </row>
     <row r="240" spans="1:5">
@@ -6274,63 +6274,12 @@
         <v>42</v>
       </c>
       <c r="C240" t="s">
-        <v>237</v>
+        <v>240</v>
       </c>
       <c r="D240" t="s">
-        <v>404</v>
+        <v>407</v>
       </c>
       <c r="E240">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="241" spans="1:5">
-      <c r="A241" t="s">
-        <v>16</v>
-      </c>
-      <c r="B241" t="s">
-        <v>42</v>
-      </c>
-      <c r="C241" t="s">
-        <v>238</v>
-      </c>
-      <c r="D241" t="s">
-        <v>405</v>
-      </c>
-      <c r="E241">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="242" spans="1:5">
-      <c r="A242" t="s">
-        <v>16</v>
-      </c>
-      <c r="B242" t="s">
-        <v>42</v>
-      </c>
-      <c r="C242" t="s">
-        <v>239</v>
-      </c>
-      <c r="D242" t="s">
-        <v>406</v>
-      </c>
-      <c r="E242">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="243" spans="1:5">
-      <c r="A243" t="s">
-        <v>16</v>
-      </c>
-      <c r="B243" t="s">
-        <v>42</v>
-      </c>
-      <c r="C243" t="s">
-        <v>240</v>
-      </c>
-      <c r="D243" t="s">
-        <v>407</v>
-      </c>
-      <c r="E243">
         <v>20</v>
       </c>
     </row>

</xml_diff>